<commit_message>
chore(data): batch update intraday televendas - 08:01:21
</commit_message>
<xml_diff>
--- a/data/dim_televendas.xlsx
+++ b/data/dim_televendas.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3465"/>
+  <dimension ref="A1:D3466"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -67614,20 +67614,20 @@
     <row r="3360">
       <c r="A3360" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3360" t="n">
-        <v>3337</v>
+        <v>3549</v>
       </c>
       <c r="C3360" t="inlineStr">
         <is>
-          <t>WESLEY FONTES DE ALMEIDA</t>
+          <t xml:space="preserve">FERNANDA CAROLINE E CESAR SOUSA </t>
         </is>
       </c>
       <c r="D3360" t="inlineStr">
         <is>
-          <t>WFALMEIDA</t>
+          <t>FCAROLINE</t>
         </is>
       </c>
     </row>
@@ -67638,16 +67638,16 @@
         </is>
       </c>
       <c r="B3361" t="n">
-        <v>3338</v>
+        <v>3337</v>
       </c>
       <c r="C3361" t="inlineStr">
         <is>
-          <t>FRANCISCA SAMARA MENDES DE OLIVEIRA C</t>
+          <t>WESLEY FONTES DE ALMEIDA</t>
         </is>
       </c>
       <c r="D3361" t="inlineStr">
         <is>
-          <t>FSCUNHA</t>
+          <t>WFALMEIDA</t>
         </is>
       </c>
     </row>
@@ -67658,176 +67658,176 @@
         </is>
       </c>
       <c r="B3362" t="n">
-        <v>3339</v>
+        <v>3338</v>
       </c>
       <c r="C3362" t="inlineStr">
         <is>
-          <t>MAYARA THALYA DIAS DE ANDRADE</t>
+          <t>FRANCISCA SAMARA MENDES DE OLIVEIRA C</t>
         </is>
       </c>
       <c r="D3362" t="inlineStr">
         <is>
-          <t>MTANDRADE</t>
+          <t>FSCUNHA</t>
         </is>
       </c>
     </row>
     <row r="3363">
       <c r="A3363" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3363" t="n">
-        <v>3359</v>
+        <v>3339</v>
       </c>
       <c r="C3363" t="inlineStr">
         <is>
-          <t xml:space="preserve">EVANESSA DA SILVA E SILVA </t>
+          <t>MAYARA THALYA DIAS DE ANDRADE</t>
         </is>
       </c>
       <c r="D3363" t="inlineStr">
         <is>
-          <t>EVANESSAS</t>
+          <t>MTANDRADE</t>
         </is>
       </c>
     </row>
     <row r="3364">
       <c r="A3364" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3364" t="n">
-        <v>3360</v>
+        <v>3359</v>
       </c>
       <c r="C3364" t="inlineStr">
         <is>
-          <t>THIAGO DE CARVALHO ARAUJO</t>
+          <t xml:space="preserve">EVANESSA DA SILVA E SILVA </t>
         </is>
       </c>
       <c r="D3364" t="inlineStr">
         <is>
-          <t>TCARAUJO</t>
+          <t>EVANESSAS</t>
         </is>
       </c>
     </row>
     <row r="3365">
       <c r="A3365" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3365" t="n">
-        <v>3481</v>
+        <v>3360</v>
       </c>
       <c r="C3365" t="inlineStr">
         <is>
-          <t xml:space="preserve">EDSON DA PAZ LIMA </t>
+          <t>THIAGO DE CARVALHO ARAUJO</t>
         </is>
       </c>
       <c r="D3365" t="inlineStr">
         <is>
-          <t>EDPAZ</t>
+          <t>TCARAUJO</t>
         </is>
       </c>
     </row>
     <row r="3366">
       <c r="A3366" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3366" t="n">
-        <v>3494</v>
+        <v>3481</v>
       </c>
       <c r="C3366" t="inlineStr">
         <is>
-          <t>ANTONIO CRISTINA BRITO GOMES</t>
+          <t xml:space="preserve">EDSON DA PAZ LIMA </t>
         </is>
       </c>
       <c r="D3366" t="inlineStr">
         <is>
-          <t>CRIS.GOMES</t>
+          <t>EDPAZ</t>
         </is>
       </c>
     </row>
     <row r="3367">
       <c r="A3367" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3367" t="n">
-        <v>3498</v>
+        <v>3494</v>
       </c>
       <c r="C3367" t="inlineStr">
         <is>
-          <t>SILVESTRA COSTA NUNES</t>
+          <t>ANTONIO CRISTINA BRITO GOMES</t>
         </is>
       </c>
       <c r="D3367" t="inlineStr">
         <is>
-          <t>SCNUNES</t>
+          <t>CRIS.GOMES</t>
         </is>
       </c>
     </row>
     <row r="3368">
       <c r="A3368" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3368" t="n">
-        <v>940562</v>
+        <v>3498</v>
       </c>
       <c r="C3368" t="inlineStr">
         <is>
-          <t>FRANCISCO DAVID ASSUNCAO ALVES</t>
+          <t>SILVESTRA COSTA NUNES</t>
         </is>
       </c>
       <c r="D3368" t="inlineStr">
         <is>
-          <t>ASSUNÇÃO</t>
+          <t>SCNUNES</t>
         </is>
       </c>
     </row>
     <row r="3369">
       <c r="A3369" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>99</t>
         </is>
       </c>
       <c r="B3369" t="n">
-        <v>3513</v>
+        <v>940562</v>
       </c>
       <c r="C3369" t="inlineStr">
         <is>
-          <t>RENARA ANDRADE MATIAS</t>
+          <t>FRANCISCO DAVID ASSUNCAO ALVES</t>
         </is>
       </c>
       <c r="D3369" t="inlineStr">
         <is>
-          <t>R.ANDRADE</t>
+          <t>ASSUNÇÃO</t>
         </is>
       </c>
     </row>
     <row r="3370">
       <c r="A3370" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3370" t="n">
-        <v>3275</v>
+        <v>3513</v>
       </c>
       <c r="C3370" t="inlineStr">
         <is>
-          <t>MARIA APARECIDA COELHO SILVA</t>
+          <t>RENARA ANDRADE MATIAS</t>
         </is>
       </c>
       <c r="D3370" t="inlineStr">
         <is>
-          <t>MCOELHO</t>
+          <t>R.ANDRADE</t>
         </is>
       </c>
     </row>
@@ -67838,96 +67838,96 @@
         </is>
       </c>
       <c r="B3371" t="n">
-        <v>3276</v>
+        <v>3275</v>
       </c>
       <c r="C3371" t="inlineStr">
         <is>
-          <t xml:space="preserve">PEROLA DE JESUS AMORIM SOUSA </t>
+          <t>MARIA APARECIDA COELHO SILVA</t>
         </is>
       </c>
       <c r="D3371" t="inlineStr">
         <is>
-          <t>PJESUS</t>
+          <t>MCOELHO</t>
         </is>
       </c>
     </row>
     <row r="3372">
       <c r="A3372" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3372" t="n">
-        <v>3526</v>
+        <v>3276</v>
       </c>
       <c r="C3372" t="inlineStr">
         <is>
-          <t>JOYCE NAZARE CORREA</t>
+          <t xml:space="preserve">PEROLA DE JESUS AMORIM SOUSA </t>
         </is>
       </c>
       <c r="D3372" t="inlineStr">
         <is>
-          <t>J.NAZARE</t>
+          <t>PJESUS</t>
         </is>
       </c>
     </row>
     <row r="3373">
       <c r="A3373" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3373" t="n">
-        <v>3527</v>
+        <v>3526</v>
       </c>
       <c r="C3373" t="inlineStr">
         <is>
-          <t>GILVANA DA SILVA MONTELES</t>
+          <t>JOYCE NAZARE CORREA</t>
         </is>
       </c>
       <c r="D3373" t="inlineStr">
         <is>
-          <t>GIL.SILVA</t>
+          <t>J.NAZARE</t>
         </is>
       </c>
     </row>
     <row r="3374">
       <c r="A3374" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3374" t="n">
-        <v>3548</v>
+        <v>3527</v>
       </c>
       <c r="C3374" t="inlineStr">
         <is>
-          <t>JAMILLY MARIA HENRIQUE ARAUJO</t>
+          <t>GILVANA DA SILVA MONTELES</t>
         </is>
       </c>
       <c r="D3374" t="inlineStr">
         <is>
-          <t>JAMILLY</t>
+          <t>GIL.SILVA</t>
         </is>
       </c>
     </row>
     <row r="3375">
       <c r="A3375" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3375" t="n">
-        <v>940525</v>
+        <v>3548</v>
       </c>
       <c r="C3375" t="inlineStr">
         <is>
-          <t>SANDUWELLINGTON</t>
+          <t>JAMILLY MARIA HENRIQUE ARAUJO</t>
         </is>
       </c>
       <c r="D3375" t="inlineStr">
         <is>
-          <t>SANDUWELLINGTON</t>
+          <t>JAMILLY</t>
         </is>
       </c>
     </row>
@@ -67938,36 +67938,36 @@
         </is>
       </c>
       <c r="B3376" t="n">
-        <v>3369</v>
+        <v>940525</v>
       </c>
       <c r="C3376" t="inlineStr">
         <is>
-          <t xml:space="preserve">PRISCILA DOS SANTOS LOPES </t>
+          <t>SANDUWELLINGTON</t>
         </is>
       </c>
       <c r="D3376" t="inlineStr">
         <is>
-          <t>PSLOPES</t>
+          <t>SANDUWELLINGTON</t>
         </is>
       </c>
     </row>
     <row r="3377">
       <c r="A3377" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3377" t="n">
-        <v>3433</v>
+        <v>3369</v>
       </c>
       <c r="C3377" t="inlineStr">
         <is>
-          <t>BRUNO NUNES CRUZ</t>
+          <t xml:space="preserve">PRISCILA DOS SANTOS LOPES </t>
         </is>
       </c>
       <c r="D3377" t="inlineStr">
         <is>
-          <t>BRUNOCRUZ</t>
+          <t>PSLOPES</t>
         </is>
       </c>
     </row>
@@ -67978,36 +67978,36 @@
         </is>
       </c>
       <c r="B3378" t="n">
-        <v>3434</v>
+        <v>3433</v>
       </c>
       <c r="C3378" t="inlineStr">
         <is>
-          <t>ANA TERCIA DE LIMA SA CARVALHO SERAFIM</t>
+          <t>BRUNO NUNES CRUZ</t>
         </is>
       </c>
       <c r="D3378" t="inlineStr">
         <is>
-          <t>ANATER</t>
+          <t>BRUNOCRUZ</t>
         </is>
       </c>
     </row>
     <row r="3379">
       <c r="A3379" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3379" t="n">
-        <v>3502</v>
+        <v>3434</v>
       </c>
       <c r="C3379" t="inlineStr">
         <is>
-          <t>LUIZ FELIPE MACHADO BARRETO</t>
+          <t>ANA TERCIA DE LIMA SA CARVALHO SERAFIM</t>
         </is>
       </c>
       <c r="D3379" t="inlineStr">
         <is>
-          <t>LUIZ.FELIPE</t>
+          <t>ANATER</t>
         </is>
       </c>
     </row>
@@ -68018,36 +68018,36 @@
         </is>
       </c>
       <c r="B3380" t="n">
-        <v>3503</v>
+        <v>3502</v>
       </c>
       <c r="C3380" t="inlineStr">
         <is>
-          <t>FABIO OLIVEIRA SILVA</t>
+          <t>LUIZ FELIPE MACHADO BARRETO</t>
         </is>
       </c>
       <c r="D3380" t="inlineStr">
         <is>
-          <t>FOSILVA</t>
+          <t>LUIZ.FELIPE</t>
         </is>
       </c>
     </row>
     <row r="3381">
       <c r="A3381" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3381" t="n">
-        <v>940549</v>
+        <v>3503</v>
       </c>
       <c r="C3381" t="inlineStr">
         <is>
-          <t>EDILSON ARAUJO - FL9</t>
+          <t>FABIO OLIVEIRA SILVA</t>
         </is>
       </c>
       <c r="D3381" t="inlineStr">
         <is>
-          <t>EDILSON</t>
+          <t>FOSILVA</t>
         </is>
       </c>
     </row>
@@ -68058,36 +68058,36 @@
         </is>
       </c>
       <c r="B3382" t="n">
-        <v>3470</v>
+        <v>940549</v>
       </c>
       <c r="C3382" t="inlineStr">
         <is>
-          <t>DEBORA ALVES CARVALHO</t>
+          <t>EDILSON ARAUJO - FL9</t>
         </is>
       </c>
       <c r="D3382" t="inlineStr">
         <is>
-          <t>DEBORA.ALVES</t>
+          <t>EDILSON</t>
         </is>
       </c>
     </row>
     <row r="3383">
       <c r="A3383" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3383" t="n">
-        <v>3510</v>
+        <v>3470</v>
       </c>
       <c r="C3383" t="inlineStr">
         <is>
-          <t>CAMILA RODIGUES PINTO</t>
+          <t>DEBORA ALVES CARVALHO</t>
         </is>
       </c>
       <c r="D3383" t="inlineStr">
         <is>
-          <t>MILA.PINTO</t>
+          <t>DEBORA.ALVES</t>
         </is>
       </c>
     </row>
@@ -68098,56 +68098,56 @@
         </is>
       </c>
       <c r="B3384" t="n">
-        <v>3511</v>
+        <v>3510</v>
       </c>
       <c r="C3384" t="inlineStr">
         <is>
-          <t>JORGE HENRIQUE DOS SANTOS RODRIGUES</t>
+          <t>CAMILA RODIGUES PINTO</t>
         </is>
       </c>
       <c r="D3384" t="inlineStr">
         <is>
-          <t>J.HENRIQUE</t>
+          <t>MILA.PINTO</t>
         </is>
       </c>
     </row>
     <row r="3385">
       <c r="A3385" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3385" t="n">
-        <v>3270</v>
+        <v>3511</v>
       </c>
       <c r="C3385" t="inlineStr">
         <is>
-          <t>ITANA NASCIMENTO SIMOES</t>
+          <t>JORGE HENRIQUE DOS SANTOS RODRIGUES</t>
         </is>
       </c>
       <c r="D3385" t="inlineStr">
         <is>
-          <t>ISIMOES</t>
+          <t>J.HENRIQUE</t>
         </is>
       </c>
     </row>
     <row r="3386">
       <c r="A3386" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3386" t="n">
-        <v>3318</v>
+        <v>3270</v>
       </c>
       <c r="C3386" t="inlineStr">
         <is>
-          <t>LUAN MONTEIRO COSTA</t>
+          <t>ITANA NASCIMENTO SIMOES</t>
         </is>
       </c>
       <c r="D3386" t="inlineStr">
         <is>
-          <t>LMONTEIRO</t>
+          <t>ISIMOES</t>
         </is>
       </c>
     </row>
@@ -68158,36 +68158,36 @@
         </is>
       </c>
       <c r="B3387" t="n">
-        <v>3319</v>
+        <v>3318</v>
       </c>
       <c r="C3387" t="inlineStr">
         <is>
-          <t>MARIANA MACEDA DOS SANTOS</t>
+          <t>LUAN MONTEIRO COSTA</t>
         </is>
       </c>
       <c r="D3387" t="inlineStr">
         <is>
-          <t>MMACEDA</t>
+          <t>LMONTEIRO</t>
         </is>
       </c>
     </row>
     <row r="3388">
       <c r="A3388" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3388" t="n">
-        <v>3389</v>
+        <v>3319</v>
       </c>
       <c r="C3388" t="inlineStr">
         <is>
-          <t>TAMILES DE SANTANA AMORIM BISPO</t>
+          <t>MARIANA MACEDA DOS SANTOS</t>
         </is>
       </c>
       <c r="D3388" t="inlineStr">
         <is>
-          <t>TAMILES</t>
+          <t>MMACEDA</t>
         </is>
       </c>
     </row>
@@ -68198,36 +68198,36 @@
         </is>
       </c>
       <c r="B3389" t="n">
-        <v>3390</v>
+        <v>3389</v>
       </c>
       <c r="C3389" t="inlineStr">
         <is>
-          <t>IRACEMA DE ALMEIDA MOURA</t>
+          <t>TAMILES DE SANTANA AMORIM BISPO</t>
         </is>
       </c>
       <c r="D3389" t="inlineStr">
         <is>
-          <t>IRACEMA</t>
+          <t>TAMILES</t>
         </is>
       </c>
     </row>
     <row r="3390">
       <c r="A3390" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3390" t="n">
-        <v>3286</v>
+        <v>3390</v>
       </c>
       <c r="C3390" t="inlineStr">
         <is>
-          <t>VALERIA MAIA DA SILVA</t>
+          <t>IRACEMA DE ALMEIDA MOURA</t>
         </is>
       </c>
       <c r="D3390" t="inlineStr">
         <is>
-          <t>VMAIAS</t>
+          <t>IRACEMA</t>
         </is>
       </c>
     </row>
@@ -68238,156 +68238,156 @@
         </is>
       </c>
       <c r="B3391" t="n">
-        <v>3287</v>
+        <v>3286</v>
       </c>
       <c r="C3391" t="inlineStr">
         <is>
-          <t>ERIVELTON DA SILVA OLIVEIRA</t>
+          <t>VALERIA MAIA DA SILVA</t>
         </is>
       </c>
       <c r="D3391" t="inlineStr">
         <is>
-          <t>ESOLIVEIRA</t>
+          <t>VMAIAS</t>
         </is>
       </c>
     </row>
     <row r="3392">
       <c r="A3392" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3392" t="n">
-        <v>3307</v>
+        <v>3287</v>
       </c>
       <c r="C3392" t="inlineStr">
         <is>
-          <t>ADRIEL XERES BARROS MARTINS</t>
+          <t>ERIVELTON DA SILVA OLIVEIRA</t>
         </is>
       </c>
       <c r="D3392" t="inlineStr">
         <is>
-          <t>AXERES</t>
+          <t>ESOLIVEIRA</t>
         </is>
       </c>
     </row>
     <row r="3393">
       <c r="A3393" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3393" t="n">
-        <v>3308</v>
+        <v>3307</v>
       </c>
       <c r="C3393" t="inlineStr">
         <is>
-          <t>ELKZIEL JUVINO DA SILVA</t>
+          <t>ADRIEL XERES BARROS MARTINS</t>
         </is>
       </c>
       <c r="D3393" t="inlineStr">
         <is>
-          <t>EJUVINO</t>
+          <t>AXERES</t>
         </is>
       </c>
     </row>
     <row r="3394">
       <c r="A3394" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3394" t="n">
-        <v>940539</v>
+        <v>3308</v>
       </c>
       <c r="C3394" t="inlineStr">
         <is>
-          <t>EDSON ARAUJO - FL9</t>
+          <t>ELKZIEL JUVINO DA SILVA</t>
         </is>
       </c>
       <c r="D3394" t="inlineStr">
         <is>
-          <t>EDS</t>
+          <t>EJUVINO</t>
         </is>
       </c>
     </row>
     <row r="3395">
       <c r="A3395" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3395" t="n">
-        <v>940540</v>
+        <v>940539</v>
       </c>
       <c r="C3395" t="inlineStr">
         <is>
-          <t>EDSON ARAUJO - FL8</t>
+          <t>EDSON ARAUJO - FL9</t>
         </is>
       </c>
       <c r="D3395" t="inlineStr">
         <is>
-          <t>EDS8</t>
+          <t>EDS</t>
         </is>
       </c>
     </row>
     <row r="3396">
       <c r="A3396" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B3396" t="n">
-        <v>3328</v>
+        <v>940540</v>
       </c>
       <c r="C3396" t="inlineStr">
         <is>
-          <t>ALAN ARAUJO DA SILVA</t>
+          <t>EDSON ARAUJO - FL8</t>
         </is>
       </c>
       <c r="D3396" t="inlineStr">
         <is>
-          <t>ARSILVA</t>
+          <t>EDS8</t>
         </is>
       </c>
     </row>
     <row r="3397">
       <c r="A3397" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3397" t="n">
-        <v>3350</v>
+        <v>3328</v>
       </c>
       <c r="C3397" t="inlineStr">
         <is>
-          <t xml:space="preserve">EDER RODRIGUES DA SILVA </t>
+          <t>ALAN ARAUJO DA SILVA</t>
         </is>
       </c>
       <c r="D3397" t="inlineStr">
         <is>
-          <t>EDERS</t>
+          <t>ARSILVA</t>
         </is>
       </c>
     </row>
     <row r="3398">
       <c r="A3398" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3398" t="n">
-        <v>3373</v>
+        <v>3350</v>
       </c>
       <c r="C3398" t="inlineStr">
         <is>
-          <t xml:space="preserve">NATANAEL TAVARES DE SOUSA </t>
+          <t xml:space="preserve">EDER RODRIGUES DA SILVA </t>
         </is>
       </c>
       <c r="D3398" t="inlineStr">
         <is>
-          <t>NTSOUSA</t>
+          <t>EDERS</t>
         </is>
       </c>
     </row>
@@ -68398,156 +68398,156 @@
         </is>
       </c>
       <c r="B3399" t="n">
-        <v>3374</v>
+        <v>3373</v>
       </c>
       <c r="C3399" t="inlineStr">
         <is>
-          <t>REINALDO DA SILVA COSTA</t>
+          <t xml:space="preserve">NATANAEL TAVARES DE SOUSA </t>
         </is>
       </c>
       <c r="D3399" t="inlineStr">
         <is>
-          <t>RSCOSTA</t>
+          <t>NTSOUSA</t>
         </is>
       </c>
     </row>
     <row r="3400">
       <c r="A3400" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3400" t="n">
-        <v>3399</v>
+        <v>3374</v>
       </c>
       <c r="C3400" t="inlineStr">
         <is>
-          <t xml:space="preserve">RICARDO BARBOSA DOS SANTOS </t>
+          <t>REINALDO DA SILVA COSTA</t>
         </is>
       </c>
       <c r="D3400" t="inlineStr">
         <is>
-          <t>RICARDOSAN</t>
+          <t>RSCOSTA</t>
         </is>
       </c>
     </row>
     <row r="3401">
       <c r="A3401" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3401" t="n">
-        <v>3427</v>
+        <v>3399</v>
       </c>
       <c r="C3401" t="inlineStr">
         <is>
-          <t>ROQUE COMERCIO TEMPORARIO</t>
+          <t xml:space="preserve">RICARDO BARBOSA DOS SANTOS </t>
         </is>
       </c>
       <c r="D3401" t="inlineStr">
         <is>
-          <t>ROQUECOM</t>
+          <t>RICARDOSAN</t>
         </is>
       </c>
     </row>
     <row r="3402">
       <c r="A3402" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3402" t="n">
-        <v>3428</v>
+        <v>3427</v>
       </c>
       <c r="C3402" t="inlineStr">
         <is>
-          <t>ROQUE PLUS TEMPORARIO</t>
+          <t>ROQUE COMERCIO TEMPORARIO</t>
         </is>
       </c>
       <c r="D3402" t="inlineStr">
         <is>
-          <t>ROQUEPLUS</t>
+          <t>ROQUECOM</t>
         </is>
       </c>
     </row>
     <row r="3403">
       <c r="A3403" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3403" t="n">
-        <v>3432</v>
+        <v>3428</v>
       </c>
       <c r="C3403" t="inlineStr">
         <is>
-          <t>PATRICIA DOS SANTOS NONATO OLIVEIRA</t>
+          <t>ROQUE PLUS TEMPORARIO</t>
         </is>
       </c>
       <c r="D3403" t="inlineStr">
         <is>
-          <t>PATRICIAD</t>
+          <t>ROQUEPLUS</t>
         </is>
       </c>
     </row>
     <row r="3404">
       <c r="A3404" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3404" t="n">
-        <v>3448</v>
+        <v>3432</v>
       </c>
       <c r="C3404" t="inlineStr">
         <is>
-          <t xml:space="preserve">GABRIEL SOUZA CARVALHO </t>
+          <t>PATRICIA DOS SANTOS NONATO OLIVEIRA</t>
         </is>
       </c>
       <c r="D3404" t="inlineStr">
         <is>
-          <t>GABRIEL20</t>
+          <t>PATRICIAD</t>
         </is>
       </c>
     </row>
     <row r="3405">
       <c r="A3405" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3405" t="n">
-        <v>3465</v>
+        <v>3448</v>
       </c>
       <c r="C3405" t="inlineStr">
         <is>
-          <t>LUIZA MARIA BARRETO BARBOSA</t>
+          <t xml:space="preserve">GABRIEL SOUZA CARVALHO </t>
         </is>
       </c>
       <c r="D3405" t="inlineStr">
         <is>
-          <t>LUIZA.MARIA</t>
+          <t>GABRIEL20</t>
         </is>
       </c>
     </row>
     <row r="3406">
       <c r="A3406" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3406" t="n">
-        <v>3468</v>
+        <v>3465</v>
       </c>
       <c r="C3406" t="inlineStr">
         <is>
-          <t>KAWA ALMEIDA CAMPOS</t>
+          <t>LUIZA MARIA BARRETO BARBOSA</t>
         </is>
       </c>
       <c r="D3406" t="inlineStr">
         <is>
-          <t>KAWA</t>
+          <t>LUIZA.MARIA</t>
         </is>
       </c>
     </row>
@@ -68558,16 +68558,16 @@
         </is>
       </c>
       <c r="B3407" t="n">
-        <v>3476</v>
+        <v>3468</v>
       </c>
       <c r="C3407" t="inlineStr">
         <is>
-          <t xml:space="preserve"> FRANCISCA LEIDIANE M. MENDES NASCIMENTO</t>
+          <t>KAWA ALMEIDA CAMPOS</t>
         </is>
       </c>
       <c r="D3407" t="inlineStr">
         <is>
-          <t>FLEIDIANE</t>
+          <t>KAWA</t>
         </is>
       </c>
     </row>
@@ -68578,76 +68578,76 @@
         </is>
       </c>
       <c r="B3408" t="n">
-        <v>3477</v>
+        <v>3476</v>
       </c>
       <c r="C3408" t="inlineStr">
         <is>
-          <t>MARIA THAIS MARTINS PEREIRA SILVA</t>
+          <t xml:space="preserve"> FRANCISCA LEIDIANE M. MENDES NASCIMENTO</t>
         </is>
       </c>
       <c r="D3408" t="inlineStr">
         <is>
-          <t>MTHAIS</t>
+          <t>FLEIDIANE</t>
         </is>
       </c>
     </row>
     <row r="3409">
       <c r="A3409" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3409" t="n">
-        <v>3271</v>
+        <v>3477</v>
       </c>
       <c r="C3409" t="inlineStr">
         <is>
-          <t>DIEGO DE ARAUJO CALÁBRIA</t>
+          <t>MARIA THAIS MARTINS PEREIRA SILVA</t>
         </is>
       </c>
       <c r="D3409" t="inlineStr">
         <is>
-          <t>ARAUJOC</t>
+          <t>MTHAIS</t>
         </is>
       </c>
     </row>
     <row r="3410">
       <c r="A3410" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3410" t="n">
-        <v>3272</v>
+        <v>3271</v>
       </c>
       <c r="C3410" t="inlineStr">
         <is>
-          <t>ANNE BEATRIZ SILVA VIRGINO</t>
+          <t>DIEGO DE ARAUJO CALÁBRIA</t>
         </is>
       </c>
       <c r="D3410" t="inlineStr">
         <is>
-          <t>ABVIRGINIO</t>
+          <t>ARAUJOC</t>
         </is>
       </c>
     </row>
     <row r="3411">
       <c r="A3411" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3411" t="n">
-        <v>3293</v>
+        <v>3272</v>
       </c>
       <c r="C3411" t="inlineStr">
         <is>
-          <t xml:space="preserve">CARLOS ALBERTO VIRIATO SANTOS </t>
+          <t>ANNE BEATRIZ SILVA VIRGINO</t>
         </is>
       </c>
       <c r="D3411" t="inlineStr">
         <is>
-          <t>CVIRIATO</t>
+          <t>ABVIRGINIO</t>
         </is>
       </c>
     </row>
@@ -68658,16 +68658,16 @@
         </is>
       </c>
       <c r="B3412" t="n">
-        <v>3381</v>
+        <v>3293</v>
       </c>
       <c r="C3412" t="inlineStr">
         <is>
-          <t>ALAN CAIQUE SANTOS E SANTOS</t>
+          <t xml:space="preserve">CARLOS ALBERTO VIRIATO SANTOS </t>
         </is>
       </c>
       <c r="D3412" t="inlineStr">
         <is>
-          <t>ALANSANTOS</t>
+          <t>CVIRIATO</t>
         </is>
       </c>
     </row>
@@ -68678,176 +68678,176 @@
         </is>
       </c>
       <c r="B3413" t="n">
-        <v>3443</v>
+        <v>3381</v>
       </c>
       <c r="C3413" t="inlineStr">
         <is>
-          <t>SANON MOREIRA SOUZA</t>
+          <t>ALAN CAIQUE SANTOS E SANTOS</t>
         </is>
       </c>
       <c r="D3413" t="inlineStr">
         <is>
-          <t>SANON</t>
+          <t>ALANSANTOS</t>
         </is>
       </c>
     </row>
     <row r="3414">
       <c r="A3414" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3414" t="n">
-        <v>3516</v>
+        <v>3443</v>
       </c>
       <c r="C3414" t="inlineStr">
         <is>
-          <t>FRANCISCO RILDER TELES DE OLIVEIRA</t>
+          <t>SANON MOREIRA SOUZA</t>
         </is>
       </c>
       <c r="D3414" t="inlineStr">
         <is>
-          <t>RILDER</t>
+          <t>SANON</t>
         </is>
       </c>
     </row>
     <row r="3415">
       <c r="A3415" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3415" t="n">
-        <v>3519</v>
+        <v>3516</v>
       </c>
       <c r="C3415" t="inlineStr">
         <is>
-          <t>MARIA LUANA DE ALMEIDA BATISTA</t>
+          <t>FRANCISCO RILDER TELES DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D3415" t="inlineStr">
         <is>
-          <t>M.LUANA</t>
+          <t>RILDER</t>
         </is>
       </c>
     </row>
     <row r="3416">
       <c r="A3416" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3416" t="n">
-        <v>3540</v>
+        <v>3519</v>
       </c>
       <c r="C3416" t="inlineStr">
         <is>
-          <t>HELEN VITORIA OLIVEIRA DA ROCHA</t>
+          <t>MARIA LUANA DE ALMEIDA BATISTA</t>
         </is>
       </c>
       <c r="D3416" t="inlineStr">
         <is>
-          <t>H.VITORIA</t>
+          <t>M.LUANA</t>
         </is>
       </c>
     </row>
     <row r="3417">
       <c r="A3417" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B3417" t="n">
-        <v>3331</v>
+        <v>3540</v>
       </c>
       <c r="C3417" t="inlineStr">
         <is>
-          <t>LOUIZE VANIELLE RODRIGUES FARIAS</t>
+          <t>HELEN VITORIA OLIVEIRA DA ROCHA</t>
         </is>
       </c>
       <c r="D3417" t="inlineStr">
         <is>
-          <t>LVFARIAS</t>
+          <t>H.VITORIA</t>
         </is>
       </c>
     </row>
     <row r="3418">
       <c r="A3418" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3418" t="n">
-        <v>3332</v>
+        <v>3331</v>
       </c>
       <c r="C3418" t="inlineStr">
         <is>
-          <t>ALEXSANDRO PEIXOTO DA VEIGA PACHECO</t>
+          <t>LOUIZE VANIELLE RODRIGUES FARIAS</t>
         </is>
       </c>
       <c r="D3418" t="inlineStr">
         <is>
-          <t>APVEIGA</t>
+          <t>LVFARIAS</t>
         </is>
       </c>
     </row>
     <row r="3419">
       <c r="A3419" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B3419" t="n">
-        <v>3334</v>
+        <v>3332</v>
       </c>
       <c r="C3419" t="inlineStr">
         <is>
-          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+          <t>ALEXSANDRO PEIXOTO DA VEIGA PACHECO</t>
         </is>
       </c>
       <c r="D3419" t="inlineStr">
         <is>
-          <t>MTGASPAR</t>
+          <t>APVEIGA</t>
         </is>
       </c>
     </row>
     <row r="3420">
       <c r="A3420" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3420" t="n">
-        <v>3345</v>
+        <v>3334</v>
       </c>
       <c r="C3420" t="inlineStr">
         <is>
-          <t>AURICÉLIA INACIO PEREIRA</t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
       <c r="D3420" t="inlineStr">
         <is>
-          <t>AIPEREIRA</t>
+          <t>MTGASPAR</t>
         </is>
       </c>
     </row>
     <row r="3421">
       <c r="A3421" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3421" t="n">
-        <v>3363</v>
+        <v>3345</v>
       </c>
       <c r="C3421" t="inlineStr">
         <is>
-          <t>IASMIN LEAL ALVES</t>
+          <t>AURICÉLIA INACIO PEREIRA</t>
         </is>
       </c>
       <c r="D3421" t="inlineStr">
         <is>
-          <t>ILALVES</t>
+          <t>AIPEREIRA</t>
         </is>
       </c>
     </row>
@@ -68858,196 +68858,196 @@
         </is>
       </c>
       <c r="B3422" t="n">
-        <v>3370</v>
+        <v>3363</v>
       </c>
       <c r="C3422" t="inlineStr">
         <is>
-          <t>CARLOS DIEGO ARAUJO ALMEIDA</t>
+          <t>IASMIN LEAL ALVES</t>
         </is>
       </c>
       <c r="D3422" t="inlineStr">
         <is>
-          <t>CDIEGO</t>
+          <t>ILALVES</t>
         </is>
       </c>
     </row>
     <row r="3423">
       <c r="A3423" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3423" t="n">
-        <v>3379</v>
+        <v>3370</v>
       </c>
       <c r="C3423" t="inlineStr">
         <is>
-          <t xml:space="preserve">MATHEUS EVANGELISTA FERREIRA </t>
+          <t>CARLOS DIEGO ARAUJO ALMEIDA</t>
         </is>
       </c>
       <c r="D3423" t="inlineStr">
         <is>
-          <t>MMFERREIRA</t>
+          <t>CDIEGO</t>
         </is>
       </c>
     </row>
     <row r="3424">
       <c r="A3424" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3424" t="n">
-        <v>3419</v>
+        <v>3379</v>
       </c>
       <c r="C3424" t="inlineStr">
         <is>
-          <t xml:space="preserve">DAVID EVANGELISTA SILVA </t>
+          <t xml:space="preserve">MATHEUS EVANGELISTA FERREIRA </t>
         </is>
       </c>
       <c r="D3424" t="inlineStr">
         <is>
-          <t>DAVID</t>
+          <t>MMFERREIRA</t>
         </is>
       </c>
     </row>
     <row r="3425">
       <c r="A3425" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3425" t="n">
-        <v>3423</v>
+        <v>3419</v>
       </c>
       <c r="C3425" t="inlineStr">
         <is>
-          <t>MARCIO JOSE TIAGO</t>
+          <t xml:space="preserve">DAVID EVANGELISTA SILVA </t>
         </is>
       </c>
       <c r="D3425" t="inlineStr">
         <is>
-          <t>MJTIAGO</t>
+          <t>DAVID</t>
         </is>
       </c>
     </row>
     <row r="3426">
       <c r="A3426" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3426" t="n">
-        <v>3453</v>
+        <v>3423</v>
       </c>
       <c r="C3426" t="inlineStr">
         <is>
-          <t xml:space="preserve">LAURIENE SILVA BARBOSA </t>
+          <t>MARCIO JOSE TIAGO</t>
         </is>
       </c>
       <c r="D3426" t="inlineStr">
         <is>
-          <t>LAURIENE</t>
+          <t>MJTIAGO</t>
         </is>
       </c>
     </row>
     <row r="3427">
       <c r="A3427" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3427" t="n">
-        <v>3478</v>
+        <v>3453</v>
       </c>
       <c r="C3427" t="inlineStr">
         <is>
-          <t>LEANDRO BRITO NOGUEIRA DE OLIVEIRA</t>
+          <t xml:space="preserve">LAURIENE SILVA BARBOSA </t>
         </is>
       </c>
       <c r="D3427" t="inlineStr">
         <is>
-          <t>LBNOGUEIRA</t>
+          <t>LAURIENE</t>
         </is>
       </c>
     </row>
     <row r="3428">
       <c r="A3428" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3428" t="n">
-        <v>3479</v>
+        <v>3478</v>
       </c>
       <c r="C3428" t="inlineStr">
         <is>
-          <t>ESDRAS ALESSANDRO SANTOS SANTANA</t>
+          <t>LEANDRO BRITO NOGUEIRA DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D3428" t="inlineStr">
         <is>
-          <t>EALESSANDRO</t>
+          <t>LBNOGUEIRA</t>
         </is>
       </c>
     </row>
     <row r="3429">
       <c r="A3429" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3429" t="n">
-        <v>3480</v>
+        <v>3479</v>
       </c>
       <c r="C3429" t="inlineStr">
         <is>
-          <t xml:space="preserve">LUCIMARA SOUSA LIMA </t>
+          <t>ESDRAS ALESSANDRO SANTOS SANTANA</t>
         </is>
       </c>
       <c r="D3429" t="inlineStr">
         <is>
-          <t>LUCIMARA</t>
+          <t>EALESSANDRO</t>
         </is>
       </c>
     </row>
     <row r="3430">
       <c r="A3430" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3430" t="n">
-        <v>3482</v>
+        <v>3480</v>
       </c>
       <c r="C3430" t="inlineStr">
         <is>
-          <t>DANIEL FERNANDES DINIZ HERACLIO</t>
+          <t xml:space="preserve">LUCIMARA SOUSA LIMA </t>
         </is>
       </c>
       <c r="D3430" t="inlineStr">
         <is>
-          <t>DFDINIZ</t>
+          <t>LUCIMARA</t>
         </is>
       </c>
     </row>
     <row r="3431">
       <c r="A3431" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3431" t="n">
-        <v>3518</v>
+        <v>3482</v>
       </c>
       <c r="C3431" t="inlineStr">
         <is>
-          <t>RAMYRA ALVES FELIX DA SILVA</t>
+          <t>DANIEL FERNANDES DINIZ HERACLIO</t>
         </is>
       </c>
       <c r="D3431" t="inlineStr">
         <is>
-          <t>RFELIX</t>
+          <t>DFDINIZ</t>
         </is>
       </c>
     </row>
@@ -69058,36 +69058,36 @@
         </is>
       </c>
       <c r="B3432" t="n">
-        <v>3534</v>
+        <v>3518</v>
       </c>
       <c r="C3432" t="inlineStr">
         <is>
-          <t xml:space="preserve">CAIO DE SOUZA VINHAS </t>
+          <t>RAMYRA ALVES FELIX DA SILVA</t>
         </is>
       </c>
       <c r="D3432" t="inlineStr">
         <is>
-          <t>CVINHAS</t>
+          <t>RFELIX</t>
         </is>
       </c>
     </row>
     <row r="3433">
       <c r="A3433" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3433" t="n">
-        <v>3535</v>
+        <v>3534</v>
       </c>
       <c r="C3433" t="inlineStr">
         <is>
-          <t>ROMARIO DE SOUSA SILVA</t>
+          <t xml:space="preserve">CAIO DE SOUZA VINHAS </t>
         </is>
       </c>
       <c r="D3433" t="inlineStr">
         <is>
-          <t>RSOUSAS</t>
+          <t>CVINHAS</t>
         </is>
       </c>
     </row>
@@ -69098,56 +69098,56 @@
         </is>
       </c>
       <c r="B3434" t="n">
-        <v>3536</v>
+        <v>3535</v>
       </c>
       <c r="C3434" t="inlineStr">
         <is>
-          <t>JHONATAS CARVALHO OLIVEIRA</t>
+          <t>ROMARIO DE SOUSA SILVA</t>
         </is>
       </c>
       <c r="D3434" t="inlineStr">
         <is>
-          <t>JHONATASC</t>
+          <t>RSOUSAS</t>
         </is>
       </c>
     </row>
     <row r="3435">
       <c r="A3435" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3435" t="n">
-        <v>940529</v>
+        <v>3536</v>
       </c>
       <c r="C3435" t="inlineStr">
         <is>
-          <t>EDGAR FELIX - FL9</t>
+          <t>JHONATAS CARVALHO OLIVEIRA</t>
         </is>
       </c>
       <c r="D3435" t="inlineStr">
         <is>
-          <t>EDGAR F</t>
+          <t>JHONATASC</t>
         </is>
       </c>
     </row>
     <row r="3436">
       <c r="A3436" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3436" t="n">
-        <v>3304</v>
+        <v>940529</v>
       </c>
       <c r="C3436" t="inlineStr">
         <is>
-          <t>JOACI GUILHERME GONÇALVES DA LUZ</t>
+          <t>EDGAR FELIX - FL9</t>
         </is>
       </c>
       <c r="D3436" t="inlineStr">
         <is>
-          <t>JLUZ</t>
+          <t>EDGAR F</t>
         </is>
       </c>
     </row>
@@ -69158,16 +69158,16 @@
         </is>
       </c>
       <c r="B3437" t="n">
-        <v>3305</v>
+        <v>3304</v>
       </c>
       <c r="C3437" t="inlineStr">
         <is>
-          <t>JOÃO VITOR DE ARAÚJO GONÇALVES</t>
+          <t>JOACI GUILHERME GONÇALVES DA LUZ</t>
         </is>
       </c>
       <c r="D3437" t="inlineStr">
         <is>
-          <t>JJVITOR</t>
+          <t>JLUZ</t>
         </is>
       </c>
     </row>
@@ -69178,36 +69178,36 @@
         </is>
       </c>
       <c r="B3438" t="n">
-        <v>3306</v>
+        <v>3305</v>
       </c>
       <c r="C3438" t="inlineStr">
         <is>
-          <t>WENDERSON MARCOS DOS SANTOS</t>
+          <t>JOÃO VITOR DE ARAÚJO GONÇALVES</t>
         </is>
       </c>
       <c r="D3438" t="inlineStr">
         <is>
-          <t>WWMARCOS</t>
+          <t>JJVITOR</t>
         </is>
       </c>
     </row>
     <row r="3439">
       <c r="A3439" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3439" t="n">
-        <v>3335</v>
+        <v>3306</v>
       </c>
       <c r="C3439" t="inlineStr">
         <is>
-          <t>EDILBERTO LEMOS DE LIMA</t>
+          <t>WENDERSON MARCOS DOS SANTOS</t>
         </is>
       </c>
       <c r="D3439" t="inlineStr">
         <is>
-          <t>ELEMOS</t>
+          <t>WWMARCOS</t>
         </is>
       </c>
     </row>
@@ -69218,116 +69218,116 @@
         </is>
       </c>
       <c r="B3440" t="n">
-        <v>3336</v>
+        <v>3335</v>
       </c>
       <c r="C3440" t="inlineStr">
         <is>
-          <t>EZEQUIEL SOUZA DO NASCIMENTO</t>
+          <t>EDILBERTO LEMOS DE LIMA</t>
         </is>
       </c>
       <c r="D3440" t="inlineStr">
         <is>
-          <t>ESNASCIMENTO</t>
+          <t>ELEMOS</t>
         </is>
       </c>
     </row>
     <row r="3441">
       <c r="A3441" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3441" t="n">
-        <v>3341</v>
+        <v>3336</v>
       </c>
       <c r="C3441" t="inlineStr">
         <is>
-          <t>ALCIONE MARIANO DE OLIVEIRA</t>
+          <t>EZEQUIEL SOUZA DO NASCIMENTO</t>
         </is>
       </c>
       <c r="D3441" t="inlineStr">
         <is>
-          <t>AMOLIVEIRA</t>
+          <t>ESNASCIMENTO</t>
         </is>
       </c>
     </row>
     <row r="3442">
       <c r="A3442" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3442" t="n">
-        <v>3401</v>
+        <v>3341</v>
       </c>
       <c r="C3442" t="inlineStr">
         <is>
-          <t xml:space="preserve">TULIO HENRIQUE DA SILVA CARVALHO </t>
+          <t>ALCIONE MARIANO DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D3442" t="inlineStr">
         <is>
-          <t>TULIO</t>
+          <t>AMOLIVEIRA</t>
         </is>
       </c>
     </row>
     <row r="3443">
       <c r="A3443" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3443" t="n">
-        <v>3411</v>
+        <v>3401</v>
       </c>
       <c r="C3443" t="inlineStr">
         <is>
-          <t>CONEXAO RUBYA DANILLA</t>
+          <t xml:space="preserve">TULIO HENRIQUE DA SILVA CARVALHO </t>
         </is>
       </c>
       <c r="D3443" t="inlineStr">
         <is>
-          <t>CONEXAORUBYA</t>
+          <t>TULIO</t>
         </is>
       </c>
     </row>
     <row r="3444">
       <c r="A3444" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3444" t="n">
-        <v>3412</v>
+        <v>3411</v>
       </c>
       <c r="C3444" t="inlineStr">
         <is>
-          <t>CONEXAO RAFAEL</t>
+          <t>CONEXAO RUBYA DANILLA</t>
         </is>
       </c>
       <c r="D3444" t="inlineStr">
         <is>
-          <t>CONEXAORAFAEL</t>
+          <t>CONEXAORUBYA</t>
         </is>
       </c>
     </row>
     <row r="3445">
       <c r="A3445" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3445" t="n">
-        <v>3264</v>
+        <v>3412</v>
       </c>
       <c r="C3445" t="inlineStr">
         <is>
-          <t xml:space="preserve">WILTON CARLOS MACIEL DE ASSIS </t>
+          <t>CONEXAO RAFAEL</t>
         </is>
       </c>
       <c r="D3445" t="inlineStr">
         <is>
-          <t>WCMACIEL</t>
+          <t>CONEXAORAFAEL</t>
         </is>
       </c>
     </row>
@@ -69338,56 +69338,56 @@
         </is>
       </c>
       <c r="B3446" t="n">
-        <v>3340</v>
+        <v>3264</v>
       </c>
       <c r="C3446" t="inlineStr">
         <is>
-          <t>ROGELENO FARIAS FEIJÃO FILHO</t>
+          <t xml:space="preserve">WILTON CARLOS MACIEL DE ASSIS </t>
         </is>
       </c>
       <c r="D3446" t="inlineStr">
         <is>
-          <t>RFEIJAO</t>
+          <t>WCMACIEL</t>
         </is>
       </c>
     </row>
     <row r="3447">
       <c r="A3447" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3447" t="n">
-        <v>940550</v>
+        <v>3340</v>
       </c>
       <c r="C3447" t="inlineStr">
         <is>
-          <t>RAFAELE RIBEIRO CARNEIRO</t>
+          <t>ROGELENO FARIAS FEIJÃO FILHO</t>
         </is>
       </c>
       <c r="D3447" t="inlineStr">
         <is>
-          <t>RAFAELE</t>
+          <t>RFEIJAO</t>
         </is>
       </c>
     </row>
     <row r="3448">
       <c r="A3448" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>99</t>
         </is>
       </c>
       <c r="B3448" t="n">
-        <v>3377</v>
+        <v>940550</v>
       </c>
       <c r="C3448" t="inlineStr">
         <is>
-          <t xml:space="preserve"> ISALTINO BISPO DE OLIVEIRA JUNIOR</t>
+          <t>RAFAELE RIBEIRO CARNEIRO</t>
         </is>
       </c>
       <c r="D3448" t="inlineStr">
         <is>
-          <t>BJUNIOR</t>
+          <t>RAFAELE</t>
         </is>
       </c>
     </row>
@@ -69398,56 +69398,56 @@
         </is>
       </c>
       <c r="B3449" t="n">
-        <v>3425</v>
+        <v>3377</v>
       </c>
       <c r="C3449" t="inlineStr">
         <is>
-          <t xml:space="preserve"> CIRLANE ARAUJO SOUZA </t>
+          <t xml:space="preserve"> ISALTINO BISPO DE OLIVEIRA JUNIOR</t>
         </is>
       </c>
       <c r="D3449" t="inlineStr">
         <is>
-          <t>CIRLANES</t>
+          <t>BJUNIOR</t>
         </is>
       </c>
     </row>
     <row r="3450">
       <c r="A3450" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3450" t="n">
-        <v>3454</v>
+        <v>3425</v>
       </c>
       <c r="C3450" t="inlineStr">
         <is>
-          <t>ANTONIA SAMARA DE SOUZA SOARES</t>
+          <t xml:space="preserve"> CIRLANE ARAUJO SOUZA </t>
         </is>
       </c>
       <c r="D3450" t="inlineStr">
         <is>
-          <t>ANTSAMARA</t>
+          <t>CIRLANES</t>
         </is>
       </c>
     </row>
     <row r="3451">
       <c r="A3451" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3451" t="n">
-        <v>3491</v>
+        <v>3454</v>
       </c>
       <c r="C3451" t="inlineStr">
         <is>
-          <t>PEDRO JOSE DO NASCIMENTO NETO</t>
+          <t>ANTONIA SAMARA DE SOUZA SOARES</t>
         </is>
       </c>
       <c r="D3451" t="inlineStr">
         <is>
-          <t>P.JOSE</t>
+          <t>ANTSAMARA</t>
         </is>
       </c>
     </row>
@@ -69458,36 +69458,36 @@
         </is>
       </c>
       <c r="B3452" t="n">
-        <v>3492</v>
+        <v>3491</v>
       </c>
       <c r="C3452" t="inlineStr">
         <is>
-          <t>PAULA CARLA CALDAS MOTA</t>
+          <t>PEDRO JOSE DO NASCIMENTO NETO</t>
         </is>
       </c>
       <c r="D3452" t="inlineStr">
         <is>
-          <t>P.CARLA</t>
+          <t>P.JOSE</t>
         </is>
       </c>
     </row>
     <row r="3453">
       <c r="A3453" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3453" t="n">
-        <v>3542</v>
+        <v>3492</v>
       </c>
       <c r="C3453" t="inlineStr">
         <is>
-          <t>ANTONIA MILENA SOUSA ANDRADE</t>
+          <t>PAULA CARLA CALDAS MOTA</t>
         </is>
       </c>
       <c r="D3453" t="inlineStr">
         <is>
-          <t>A.MILENA</t>
+          <t>P.CARLA</t>
         </is>
       </c>
     </row>
@@ -69498,16 +69498,16 @@
         </is>
       </c>
       <c r="B3454" t="n">
-        <v>3547</v>
+        <v>3542</v>
       </c>
       <c r="C3454" t="inlineStr">
         <is>
-          <t xml:space="preserve">DAVI PEREIRA DA SILVA </t>
+          <t>ANTONIA MILENA SOUSA ANDRADE</t>
         </is>
       </c>
       <c r="D3454" t="inlineStr">
         <is>
-          <t>DPSILVA</t>
+          <t>A.MILENA</t>
         </is>
       </c>
     </row>
@@ -69518,16 +69518,16 @@
         </is>
       </c>
       <c r="B3455" t="n">
-        <v>3294</v>
+        <v>3547</v>
       </c>
       <c r="C3455" t="inlineStr">
         <is>
-          <t>GLEICIANE MIRANDA DE MORAIS</t>
+          <t xml:space="preserve">DAVI PEREIRA DA SILVA </t>
         </is>
       </c>
       <c r="D3455" t="inlineStr">
         <is>
-          <t>GMIRANDA</t>
+          <t>DPSILVA</t>
         </is>
       </c>
     </row>
@@ -69538,176 +69538,176 @@
         </is>
       </c>
       <c r="B3456" t="n">
-        <v>3295</v>
+        <v>3294</v>
       </c>
       <c r="C3456" t="inlineStr">
         <is>
-          <t>MARIA ESTEFANNY DA SILVA MOURA</t>
+          <t>GLEICIANE MIRANDA DE MORAIS</t>
         </is>
       </c>
       <c r="D3456" t="inlineStr">
         <is>
-          <t>MESTEFANNY</t>
+          <t>GMIRANDA</t>
         </is>
       </c>
     </row>
     <row r="3457">
       <c r="A3457" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3457" t="n">
-        <v>3296</v>
+        <v>3295</v>
       </c>
       <c r="C3457" t="inlineStr">
         <is>
-          <t>PEDRO IAGO FONSECA EVANGELISTA</t>
+          <t>MARIA ESTEFANNY DA SILVA MOURA</t>
         </is>
       </c>
       <c r="D3457" t="inlineStr">
         <is>
-          <t>PIFONSECA</t>
+          <t>MESTEFANNY</t>
         </is>
       </c>
     </row>
     <row r="3458">
       <c r="A3458" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3458" t="n">
-        <v>940544</v>
+        <v>3296</v>
       </c>
       <c r="C3458" t="inlineStr">
         <is>
-          <t>LUTY LOG TRANSPORTES - FL8</t>
+          <t>PEDRO IAGO FONSECA EVANGELISTA</t>
         </is>
       </c>
       <c r="D3458" t="inlineStr">
         <is>
-          <t>LUTY LOG</t>
+          <t>PIFONSECA</t>
         </is>
       </c>
     </row>
     <row r="3459">
       <c r="A3459" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B3459" t="n">
-        <v>3380</v>
+        <v>940544</v>
       </c>
       <c r="C3459" t="inlineStr">
         <is>
-          <t>FRANCISCO MATHEUS RABELO DA COSTA</t>
+          <t>LUTY LOG TRANSPORTES - FL8</t>
         </is>
       </c>
       <c r="D3459" t="inlineStr">
         <is>
-          <t>FMATHEUS</t>
+          <t>LUTY LOG</t>
         </is>
       </c>
     </row>
     <row r="3460">
       <c r="A3460" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3460" t="n">
-        <v>3410</v>
+        <v>3380</v>
       </c>
       <c r="C3460" t="inlineStr">
         <is>
-          <t xml:space="preserve"> BRENO ALLAN DE JESUS</t>
+          <t>FRANCISCO MATHEUS RABELO DA COSTA</t>
         </is>
       </c>
       <c r="D3460" t="inlineStr">
         <is>
-          <t>JESUS</t>
+          <t>FMATHEUS</t>
         </is>
       </c>
     </row>
     <row r="3461">
       <c r="A3461" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3461" t="n">
-        <v>3444</v>
+        <v>3410</v>
       </c>
       <c r="C3461" t="inlineStr">
         <is>
-          <t>THIAGO COSTA SILVA</t>
+          <t xml:space="preserve"> BRENO ALLAN DE JESUS</t>
         </is>
       </c>
       <c r="D3461" t="inlineStr">
         <is>
-          <t>THIAGOC</t>
+          <t>JESUS</t>
         </is>
       </c>
     </row>
     <row r="3462">
       <c r="A3462" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3462" t="n">
-        <v>3456</v>
+        <v>3444</v>
       </c>
       <c r="C3462" t="inlineStr">
         <is>
-          <t>FELIPE BOTH MAZUCHINI</t>
+          <t>THIAGO COSTA SILVA</t>
         </is>
       </c>
       <c r="D3462" t="inlineStr">
         <is>
-          <t>FELIPEB</t>
+          <t>THIAGOC</t>
         </is>
       </c>
     </row>
     <row r="3463">
       <c r="A3463" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3463" t="n">
-        <v>3457</v>
+        <v>3456</v>
       </c>
       <c r="C3463" t="inlineStr">
         <is>
-          <t>FRANKLIN VIEIRA GOMES</t>
+          <t>FELIPE BOTH MAZUCHINI</t>
         </is>
       </c>
       <c r="D3463" t="inlineStr">
         <is>
-          <t>VIEIRAF</t>
+          <t>FELIPEB</t>
         </is>
       </c>
     </row>
     <row r="3464">
       <c r="A3464" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3464" t="n">
-        <v>3507</v>
+        <v>3457</v>
       </c>
       <c r="C3464" t="inlineStr">
         <is>
-          <t>KARINE TEODORA ALVES DE OLIVEIRA</t>
+          <t>FRANKLIN VIEIRA GOMES</t>
         </is>
       </c>
       <c r="D3464" t="inlineStr">
         <is>
-          <t>KOLIVEIRA</t>
+          <t>VIEIRAF</t>
         </is>
       </c>
     </row>
@@ -69718,14 +69718,34 @@
         </is>
       </c>
       <c r="B3465" t="n">
+        <v>3507</v>
+      </c>
+      <c r="C3465" t="inlineStr">
+        <is>
+          <t>KARINE TEODORA ALVES DE OLIVEIRA</t>
+        </is>
+      </c>
+      <c r="D3465" t="inlineStr">
+        <is>
+          <t>KOLIVEIRA</t>
+        </is>
+      </c>
+    </row>
+    <row r="3466">
+      <c r="A3466" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B3466" t="n">
         <v>3520</v>
       </c>
-      <c r="C3465" t="inlineStr">
+      <c r="C3466" t="inlineStr">
         <is>
           <t xml:space="preserve"> EMERSON FILIPE MELO DE AGUIAR</t>
         </is>
       </c>
-      <c r="D3465" t="inlineStr">
+      <c r="D3466" t="inlineStr">
         <is>
           <t>E.FILIPE</t>
         </is>

</xml_diff>

<commit_message>
chore(data): batch update intraday televendas - 10:03:44
</commit_message>
<xml_diff>
--- a/data/dim_televendas.xlsx
+++ b/data/dim_televendas.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3466"/>
+  <dimension ref="A1:D3468"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -67374,20 +67374,20 @@
     <row r="3348">
       <c r="A3348" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3348" t="n">
-        <v>3355</v>
+        <v>3550</v>
       </c>
       <c r="C3348" t="inlineStr">
         <is>
-          <t>HUGO MATHEUS DA COSTA FEITOSA</t>
+          <t>IARGO GABRIEL SANTOS DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D3348" t="inlineStr">
         <is>
-          <t>HMFEITOSA</t>
+          <t>IARGOG</t>
         </is>
       </c>
     </row>
@@ -67398,96 +67398,96 @@
         </is>
       </c>
       <c r="B3349" t="n">
-        <v>3356</v>
+        <v>3355</v>
       </c>
       <c r="C3349" t="inlineStr">
         <is>
-          <t>BRENDA LIMA DE OLIVEIRA CUNHA</t>
+          <t>HUGO MATHEUS DA COSTA FEITOSA</t>
         </is>
       </c>
       <c r="D3349" t="inlineStr">
         <is>
-          <t>BLCUNHA</t>
+          <t>HMFEITOSA</t>
         </is>
       </c>
     </row>
     <row r="3350">
       <c r="A3350" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3350" t="n">
-        <v>3361</v>
+        <v>3356</v>
       </c>
       <c r="C3350" t="inlineStr">
         <is>
-          <t>WLADIA DE ARAUJO BASTOS</t>
+          <t>BRENDA LIMA DE OLIVEIRA CUNHA</t>
         </is>
       </c>
       <c r="D3350" t="inlineStr">
         <is>
-          <t>WABASTOS</t>
+          <t>BLCUNHA</t>
         </is>
       </c>
     </row>
     <row r="3351">
       <c r="A3351" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3351" t="n">
-        <v>3362</v>
+        <v>3361</v>
       </c>
       <c r="C3351" t="inlineStr">
         <is>
-          <t>CARLOS HENRIQUE MELO DA SILVA</t>
+          <t>WLADIA DE ARAUJO BASTOS</t>
         </is>
       </c>
       <c r="D3351" t="inlineStr">
         <is>
-          <t>CHMELO</t>
+          <t>WABASTOS</t>
         </is>
       </c>
     </row>
     <row r="3352">
       <c r="A3352" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3352" t="n">
-        <v>3375</v>
+        <v>3362</v>
       </c>
       <c r="C3352" t="inlineStr">
         <is>
-          <t>AFONSO DE SOUSA RAMOS FILHO</t>
+          <t>CARLOS HENRIQUE MELO DA SILVA</t>
         </is>
       </c>
       <c r="D3352" t="inlineStr">
         <is>
-          <t>AFILHO</t>
+          <t>CHMELO</t>
         </is>
       </c>
     </row>
     <row r="3353">
       <c r="A3353" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3353" t="n">
-        <v>3404</v>
+        <v>3375</v>
       </c>
       <c r="C3353" t="inlineStr">
         <is>
-          <t>NOVATO 4 COM</t>
+          <t>AFONSO DE SOUSA RAMOS FILHO</t>
         </is>
       </c>
       <c r="D3353" t="inlineStr">
         <is>
-          <t>NOVATO4COM</t>
+          <t>AFILHO</t>
         </is>
       </c>
     </row>
@@ -67498,156 +67498,156 @@
         </is>
       </c>
       <c r="B3354" t="n">
-        <v>3405</v>
+        <v>3404</v>
       </c>
       <c r="C3354" t="inlineStr">
         <is>
-          <t>NOVATO 5 COM</t>
+          <t>NOVATO 4 COM</t>
         </is>
       </c>
       <c r="D3354" t="inlineStr">
         <is>
-          <t>NOVATO5COM</t>
+          <t>NOVATO4COM</t>
         </is>
       </c>
     </row>
     <row r="3355">
       <c r="A3355" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3355" t="n">
-        <v>3447</v>
+        <v>3405</v>
       </c>
       <c r="C3355" t="inlineStr">
         <is>
-          <t>RAYSSA KEYCE LINHARES AQUINO</t>
+          <t>NOVATO 5 COM</t>
         </is>
       </c>
       <c r="D3355" t="inlineStr">
         <is>
-          <t>RAYSSAK</t>
+          <t>NOVATO5COM</t>
         </is>
       </c>
     </row>
     <row r="3356">
       <c r="A3356" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3356" t="n">
-        <v>940559</v>
+        <v>3447</v>
       </c>
       <c r="C3356" t="inlineStr">
         <is>
-          <t>WALLEF DE OLIVEIRA</t>
+          <t>RAYSSA KEYCE LINHARES AQUINO</t>
         </is>
       </c>
       <c r="D3356" t="inlineStr">
         <is>
-          <t>WALLEF</t>
+          <t>RAYSSAK</t>
         </is>
       </c>
     </row>
     <row r="3357">
       <c r="A3357" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>99</t>
         </is>
       </c>
       <c r="B3357" t="n">
-        <v>3489</v>
+        <v>940559</v>
       </c>
       <c r="C3357" t="inlineStr">
         <is>
-          <t>MARCELA KARINA PEREIRA VELOSO</t>
+          <t>WALLEF DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D3357" t="inlineStr">
         <is>
-          <t>MKARINA</t>
+          <t>WALLEF</t>
         </is>
       </c>
     </row>
     <row r="3358">
       <c r="A3358" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3358" t="n">
-        <v>3490</v>
+        <v>3489</v>
       </c>
       <c r="C3358" t="inlineStr">
         <is>
-          <t>JOSE MAILSON GOMES NUNES</t>
+          <t>MARCELA KARINA PEREIRA VELOSO</t>
         </is>
       </c>
       <c r="D3358" t="inlineStr">
         <is>
-          <t>J.MAILSON</t>
+          <t>MKARINA</t>
         </is>
       </c>
     </row>
     <row r="3359">
       <c r="A3359" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3359" t="n">
-        <v>3537</v>
+        <v>3490</v>
       </c>
       <c r="C3359" t="inlineStr">
         <is>
-          <t>ALDAIR PEDRO DA SILVA</t>
+          <t>JOSE MAILSON GOMES NUNES</t>
         </is>
       </c>
       <c r="D3359" t="inlineStr">
         <is>
-          <t>A.PEDRO</t>
+          <t>J.MAILSON</t>
         </is>
       </c>
     </row>
     <row r="3360">
       <c r="A3360" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3360" t="n">
-        <v>3549</v>
+        <v>3537</v>
       </c>
       <c r="C3360" t="inlineStr">
         <is>
-          <t xml:space="preserve">FERNANDA CAROLINE E CESAR SOUSA </t>
+          <t>ALDAIR PEDRO DA SILVA</t>
         </is>
       </c>
       <c r="D3360" t="inlineStr">
         <is>
-          <t>FCAROLINE</t>
+          <t>A.PEDRO</t>
         </is>
       </c>
     </row>
     <row r="3361">
       <c r="A3361" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3361" t="n">
-        <v>3337</v>
+        <v>3549</v>
       </c>
       <c r="C3361" t="inlineStr">
         <is>
-          <t>WESLEY FONTES DE ALMEIDA</t>
+          <t xml:space="preserve">FERNANDA CAROLINE E CESAR SOUSA </t>
         </is>
       </c>
       <c r="D3361" t="inlineStr">
         <is>
-          <t>WFALMEIDA</t>
+          <t>FCAROLINE</t>
         </is>
       </c>
     </row>
@@ -67658,16 +67658,16 @@
         </is>
       </c>
       <c r="B3362" t="n">
-        <v>3338</v>
+        <v>3337</v>
       </c>
       <c r="C3362" t="inlineStr">
         <is>
-          <t>FRANCISCA SAMARA MENDES DE OLIVEIRA C</t>
+          <t>WESLEY FONTES DE ALMEIDA</t>
         </is>
       </c>
       <c r="D3362" t="inlineStr">
         <is>
-          <t>FSCUNHA</t>
+          <t>WFALMEIDA</t>
         </is>
       </c>
     </row>
@@ -67678,176 +67678,176 @@
         </is>
       </c>
       <c r="B3363" t="n">
-        <v>3339</v>
+        <v>3338</v>
       </c>
       <c r="C3363" t="inlineStr">
         <is>
-          <t>MAYARA THALYA DIAS DE ANDRADE</t>
+          <t>FRANCISCA SAMARA MENDES DE OLIVEIRA C</t>
         </is>
       </c>
       <c r="D3363" t="inlineStr">
         <is>
-          <t>MTANDRADE</t>
+          <t>FSCUNHA</t>
         </is>
       </c>
     </row>
     <row r="3364">
       <c r="A3364" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3364" t="n">
-        <v>3359</v>
+        <v>3339</v>
       </c>
       <c r="C3364" t="inlineStr">
         <is>
-          <t xml:space="preserve">EVANESSA DA SILVA E SILVA </t>
+          <t>MAYARA THALYA DIAS DE ANDRADE</t>
         </is>
       </c>
       <c r="D3364" t="inlineStr">
         <is>
-          <t>EVANESSAS</t>
+          <t>MTANDRADE</t>
         </is>
       </c>
     </row>
     <row r="3365">
       <c r="A3365" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3365" t="n">
-        <v>3360</v>
+        <v>3359</v>
       </c>
       <c r="C3365" t="inlineStr">
         <is>
-          <t>THIAGO DE CARVALHO ARAUJO</t>
+          <t xml:space="preserve">EVANESSA DA SILVA E SILVA </t>
         </is>
       </c>
       <c r="D3365" t="inlineStr">
         <is>
-          <t>TCARAUJO</t>
+          <t>EVANESSAS</t>
         </is>
       </c>
     </row>
     <row r="3366">
       <c r="A3366" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3366" t="n">
-        <v>3481</v>
+        <v>3360</v>
       </c>
       <c r="C3366" t="inlineStr">
         <is>
-          <t xml:space="preserve">EDSON DA PAZ LIMA </t>
+          <t>THIAGO DE CARVALHO ARAUJO</t>
         </is>
       </c>
       <c r="D3366" t="inlineStr">
         <is>
-          <t>EDPAZ</t>
+          <t>TCARAUJO</t>
         </is>
       </c>
     </row>
     <row r="3367">
       <c r="A3367" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3367" t="n">
-        <v>3494</v>
+        <v>3481</v>
       </c>
       <c r="C3367" t="inlineStr">
         <is>
-          <t>ANTONIO CRISTINA BRITO GOMES</t>
+          <t xml:space="preserve">EDSON DA PAZ LIMA </t>
         </is>
       </c>
       <c r="D3367" t="inlineStr">
         <is>
-          <t>CRIS.GOMES</t>
+          <t>EDPAZ</t>
         </is>
       </c>
     </row>
     <row r="3368">
       <c r="A3368" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3368" t="n">
-        <v>3498</v>
+        <v>3494</v>
       </c>
       <c r="C3368" t="inlineStr">
         <is>
-          <t>SILVESTRA COSTA NUNES</t>
+          <t>ANTONIO CRISTINA BRITO GOMES</t>
         </is>
       </c>
       <c r="D3368" t="inlineStr">
         <is>
-          <t>SCNUNES</t>
+          <t>CRIS.GOMES</t>
         </is>
       </c>
     </row>
     <row r="3369">
       <c r="A3369" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3369" t="n">
-        <v>940562</v>
+        <v>3498</v>
       </c>
       <c r="C3369" t="inlineStr">
         <is>
-          <t>FRANCISCO DAVID ASSUNCAO ALVES</t>
+          <t>SILVESTRA COSTA NUNES</t>
         </is>
       </c>
       <c r="D3369" t="inlineStr">
         <is>
-          <t>ASSUNÇÃO</t>
+          <t>SCNUNES</t>
         </is>
       </c>
     </row>
     <row r="3370">
       <c r="A3370" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>99</t>
         </is>
       </c>
       <c r="B3370" t="n">
-        <v>3513</v>
+        <v>940562</v>
       </c>
       <c r="C3370" t="inlineStr">
         <is>
-          <t>RENARA ANDRADE MATIAS</t>
+          <t>FRANCISCO DAVID ASSUNCAO ALVES</t>
         </is>
       </c>
       <c r="D3370" t="inlineStr">
         <is>
-          <t>R.ANDRADE</t>
+          <t>ASSUNÇÃO</t>
         </is>
       </c>
     </row>
     <row r="3371">
       <c r="A3371" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3371" t="n">
-        <v>3275</v>
+        <v>3513</v>
       </c>
       <c r="C3371" t="inlineStr">
         <is>
-          <t>MARIA APARECIDA COELHO SILVA</t>
+          <t>RENARA ANDRADE MATIAS</t>
         </is>
       </c>
       <c r="D3371" t="inlineStr">
         <is>
-          <t>MCOELHO</t>
+          <t>R.ANDRADE</t>
         </is>
       </c>
     </row>
@@ -67858,596 +67858,596 @@
         </is>
       </c>
       <c r="B3372" t="n">
-        <v>3276</v>
+        <v>3275</v>
       </c>
       <c r="C3372" t="inlineStr">
         <is>
-          <t xml:space="preserve">PEROLA DE JESUS AMORIM SOUSA </t>
+          <t>MARIA APARECIDA COELHO SILVA</t>
         </is>
       </c>
       <c r="D3372" t="inlineStr">
         <is>
-          <t>PJESUS</t>
+          <t>MCOELHO</t>
         </is>
       </c>
     </row>
     <row r="3373">
       <c r="A3373" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3373" t="n">
-        <v>3526</v>
+        <v>3276</v>
       </c>
       <c r="C3373" t="inlineStr">
         <is>
-          <t>JOYCE NAZARE CORREA</t>
+          <t xml:space="preserve">PEROLA DE JESUS AMORIM SOUSA </t>
         </is>
       </c>
       <c r="D3373" t="inlineStr">
         <is>
-          <t>J.NAZARE</t>
+          <t>PJESUS</t>
         </is>
       </c>
     </row>
     <row r="3374">
       <c r="A3374" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3374" t="n">
-        <v>3527</v>
+        <v>3526</v>
       </c>
       <c r="C3374" t="inlineStr">
         <is>
-          <t>GILVANA DA SILVA MONTELES</t>
+          <t>JOYCE NAZARE CORREA</t>
         </is>
       </c>
       <c r="D3374" t="inlineStr">
         <is>
-          <t>GIL.SILVA</t>
+          <t>J.NAZARE</t>
         </is>
       </c>
     </row>
     <row r="3375">
       <c r="A3375" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3375" t="n">
-        <v>3548</v>
+        <v>3527</v>
       </c>
       <c r="C3375" t="inlineStr">
         <is>
-          <t>JAMILLY MARIA HENRIQUE ARAUJO</t>
+          <t>GILVANA DA SILVA MONTELES</t>
         </is>
       </c>
       <c r="D3375" t="inlineStr">
         <is>
-          <t>JAMILLY</t>
+          <t>GIL.SILVA</t>
         </is>
       </c>
     </row>
     <row r="3376">
       <c r="A3376" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3376" t="n">
-        <v>940525</v>
+        <v>3548</v>
       </c>
       <c r="C3376" t="inlineStr">
         <is>
-          <t>SANDUWELLINGTON</t>
+          <t>JAMILLY MARIA HENRIQUE ARAUJO</t>
         </is>
       </c>
       <c r="D3376" t="inlineStr">
         <is>
-          <t>SANDUWELLINGTON</t>
+          <t>JAMILLY</t>
         </is>
       </c>
     </row>
     <row r="3377">
       <c r="A3377" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3377" t="n">
-        <v>3369</v>
+        <v>3551</v>
       </c>
       <c r="C3377" t="inlineStr">
         <is>
-          <t xml:space="preserve">PRISCILA DOS SANTOS LOPES </t>
+          <t xml:space="preserve">VITOR MANOEL DA SILVA BARBOSA </t>
         </is>
       </c>
       <c r="D3377" t="inlineStr">
         <is>
-          <t>PSLOPES</t>
+          <t>VMANOEL</t>
         </is>
       </c>
     </row>
     <row r="3378">
       <c r="A3378" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3378" t="n">
-        <v>3433</v>
+        <v>940525</v>
       </c>
       <c r="C3378" t="inlineStr">
         <is>
-          <t>BRUNO NUNES CRUZ</t>
+          <t>SANDUWELLINGTON</t>
         </is>
       </c>
       <c r="D3378" t="inlineStr">
         <is>
-          <t>BRUNOCRUZ</t>
+          <t>SANDUWELLINGTON</t>
         </is>
       </c>
     </row>
     <row r="3379">
       <c r="A3379" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3379" t="n">
-        <v>3434</v>
+        <v>3369</v>
       </c>
       <c r="C3379" t="inlineStr">
         <is>
-          <t>ANA TERCIA DE LIMA SA CARVALHO SERAFIM</t>
+          <t xml:space="preserve">PRISCILA DOS SANTOS LOPES </t>
         </is>
       </c>
       <c r="D3379" t="inlineStr">
         <is>
-          <t>ANATER</t>
+          <t>PSLOPES</t>
         </is>
       </c>
     </row>
     <row r="3380">
       <c r="A3380" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3380" t="n">
-        <v>3502</v>
+        <v>3433</v>
       </c>
       <c r="C3380" t="inlineStr">
         <is>
-          <t>LUIZ FELIPE MACHADO BARRETO</t>
+          <t>BRUNO NUNES CRUZ</t>
         </is>
       </c>
       <c r="D3380" t="inlineStr">
         <is>
-          <t>LUIZ.FELIPE</t>
+          <t>BRUNOCRUZ</t>
         </is>
       </c>
     </row>
     <row r="3381">
       <c r="A3381" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3381" t="n">
-        <v>3503</v>
+        <v>3434</v>
       </c>
       <c r="C3381" t="inlineStr">
         <is>
-          <t>FABIO OLIVEIRA SILVA</t>
+          <t>ANA TERCIA DE LIMA SA CARVALHO SERAFIM</t>
         </is>
       </c>
       <c r="D3381" t="inlineStr">
         <is>
-          <t>FOSILVA</t>
+          <t>ANATER</t>
         </is>
       </c>
     </row>
     <row r="3382">
       <c r="A3382" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3382" t="n">
-        <v>940549</v>
+        <v>3502</v>
       </c>
       <c r="C3382" t="inlineStr">
         <is>
-          <t>EDILSON ARAUJO - FL9</t>
+          <t>LUIZ FELIPE MACHADO BARRETO</t>
         </is>
       </c>
       <c r="D3382" t="inlineStr">
         <is>
-          <t>EDILSON</t>
+          <t>LUIZ.FELIPE</t>
         </is>
       </c>
     </row>
     <row r="3383">
       <c r="A3383" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3383" t="n">
-        <v>3470</v>
+        <v>3503</v>
       </c>
       <c r="C3383" t="inlineStr">
         <is>
-          <t>DEBORA ALVES CARVALHO</t>
+          <t>FABIO OLIVEIRA SILVA</t>
         </is>
       </c>
       <c r="D3383" t="inlineStr">
         <is>
-          <t>DEBORA.ALVES</t>
+          <t>FOSILVA</t>
         </is>
       </c>
     </row>
     <row r="3384">
       <c r="A3384" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3384" t="n">
-        <v>3510</v>
+        <v>940549</v>
       </c>
       <c r="C3384" t="inlineStr">
         <is>
-          <t>CAMILA RODIGUES PINTO</t>
+          <t>EDILSON ARAUJO - FL9</t>
         </is>
       </c>
       <c r="D3384" t="inlineStr">
         <is>
-          <t>MILA.PINTO</t>
+          <t>EDILSON</t>
         </is>
       </c>
     </row>
     <row r="3385">
       <c r="A3385" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3385" t="n">
-        <v>3511</v>
+        <v>3470</v>
       </c>
       <c r="C3385" t="inlineStr">
         <is>
-          <t>JORGE HENRIQUE DOS SANTOS RODRIGUES</t>
+          <t>DEBORA ALVES CARVALHO</t>
         </is>
       </c>
       <c r="D3385" t="inlineStr">
         <is>
-          <t>J.HENRIQUE</t>
+          <t>DEBORA.ALVES</t>
         </is>
       </c>
     </row>
     <row r="3386">
       <c r="A3386" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3386" t="n">
-        <v>3270</v>
+        <v>3510</v>
       </c>
       <c r="C3386" t="inlineStr">
         <is>
-          <t>ITANA NASCIMENTO SIMOES</t>
+          <t>CAMILA RODIGUES PINTO</t>
         </is>
       </c>
       <c r="D3386" t="inlineStr">
         <is>
-          <t>ISIMOES</t>
+          <t>MILA.PINTO</t>
         </is>
       </c>
     </row>
     <row r="3387">
       <c r="A3387" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3387" t="n">
-        <v>3318</v>
+        <v>3511</v>
       </c>
       <c r="C3387" t="inlineStr">
         <is>
-          <t>LUAN MONTEIRO COSTA</t>
+          <t>JORGE HENRIQUE DOS SANTOS RODRIGUES</t>
         </is>
       </c>
       <c r="D3387" t="inlineStr">
         <is>
-          <t>LMONTEIRO</t>
+          <t>J.HENRIQUE</t>
         </is>
       </c>
     </row>
     <row r="3388">
       <c r="A3388" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3388" t="n">
-        <v>3319</v>
+        <v>3270</v>
       </c>
       <c r="C3388" t="inlineStr">
         <is>
-          <t>MARIANA MACEDA DOS SANTOS</t>
+          <t>ITANA NASCIMENTO SIMOES</t>
         </is>
       </c>
       <c r="D3388" t="inlineStr">
         <is>
-          <t>MMACEDA</t>
+          <t>ISIMOES</t>
         </is>
       </c>
     </row>
     <row r="3389">
       <c r="A3389" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3389" t="n">
-        <v>3389</v>
+        <v>3318</v>
       </c>
       <c r="C3389" t="inlineStr">
         <is>
-          <t>TAMILES DE SANTANA AMORIM BISPO</t>
+          <t>LUAN MONTEIRO COSTA</t>
         </is>
       </c>
       <c r="D3389" t="inlineStr">
         <is>
-          <t>TAMILES</t>
+          <t>LMONTEIRO</t>
         </is>
       </c>
     </row>
     <row r="3390">
       <c r="A3390" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3390" t="n">
-        <v>3390</v>
+        <v>3319</v>
       </c>
       <c r="C3390" t="inlineStr">
         <is>
-          <t>IRACEMA DE ALMEIDA MOURA</t>
+          <t>MARIANA MACEDA DOS SANTOS</t>
         </is>
       </c>
       <c r="D3390" t="inlineStr">
         <is>
-          <t>IRACEMA</t>
+          <t>MMACEDA</t>
         </is>
       </c>
     </row>
     <row r="3391">
       <c r="A3391" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3391" t="n">
-        <v>3286</v>
+        <v>3389</v>
       </c>
       <c r="C3391" t="inlineStr">
         <is>
-          <t>VALERIA MAIA DA SILVA</t>
+          <t>TAMILES DE SANTANA AMORIM BISPO</t>
         </is>
       </c>
       <c r="D3391" t="inlineStr">
         <is>
-          <t>VMAIAS</t>
+          <t>TAMILES</t>
         </is>
       </c>
     </row>
     <row r="3392">
       <c r="A3392" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3392" t="n">
-        <v>3287</v>
+        <v>3390</v>
       </c>
       <c r="C3392" t="inlineStr">
         <is>
-          <t>ERIVELTON DA SILVA OLIVEIRA</t>
+          <t>IRACEMA DE ALMEIDA MOURA</t>
         </is>
       </c>
       <c r="D3392" t="inlineStr">
         <is>
-          <t>ESOLIVEIRA</t>
+          <t>IRACEMA</t>
         </is>
       </c>
     </row>
     <row r="3393">
       <c r="A3393" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3393" t="n">
-        <v>3307</v>
+        <v>3286</v>
       </c>
       <c r="C3393" t="inlineStr">
         <is>
-          <t>ADRIEL XERES BARROS MARTINS</t>
+          <t>VALERIA MAIA DA SILVA</t>
         </is>
       </c>
       <c r="D3393" t="inlineStr">
         <is>
-          <t>AXERES</t>
+          <t>VMAIAS</t>
         </is>
       </c>
     </row>
     <row r="3394">
       <c r="A3394" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3394" t="n">
-        <v>3308</v>
+        <v>3287</v>
       </c>
       <c r="C3394" t="inlineStr">
         <is>
-          <t>ELKZIEL JUVINO DA SILVA</t>
+          <t>ERIVELTON DA SILVA OLIVEIRA</t>
         </is>
       </c>
       <c r="D3394" t="inlineStr">
         <is>
-          <t>EJUVINO</t>
+          <t>ESOLIVEIRA</t>
         </is>
       </c>
     </row>
     <row r="3395">
       <c r="A3395" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3395" t="n">
-        <v>940539</v>
+        <v>3307</v>
       </c>
       <c r="C3395" t="inlineStr">
         <is>
-          <t>EDSON ARAUJO - FL9</t>
+          <t>ADRIEL XERES BARROS MARTINS</t>
         </is>
       </c>
       <c r="D3395" t="inlineStr">
         <is>
-          <t>EDS</t>
+          <t>AXERES</t>
         </is>
       </c>
     </row>
     <row r="3396">
       <c r="A3396" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3396" t="n">
-        <v>940540</v>
+        <v>3308</v>
       </c>
       <c r="C3396" t="inlineStr">
         <is>
-          <t>EDSON ARAUJO - FL8</t>
+          <t>ELKZIEL JUVINO DA SILVA</t>
         </is>
       </c>
       <c r="D3396" t="inlineStr">
         <is>
-          <t>EDS8</t>
+          <t>EJUVINO</t>
         </is>
       </c>
     </row>
     <row r="3397">
       <c r="A3397" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3397" t="n">
-        <v>3328</v>
+        <v>940539</v>
       </c>
       <c r="C3397" t="inlineStr">
         <is>
-          <t>ALAN ARAUJO DA SILVA</t>
+          <t>EDSON ARAUJO - FL9</t>
         </is>
       </c>
       <c r="D3397" t="inlineStr">
         <is>
-          <t>ARSILVA</t>
+          <t>EDS</t>
         </is>
       </c>
     </row>
     <row r="3398">
       <c r="A3398" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B3398" t="n">
-        <v>3350</v>
+        <v>940540</v>
       </c>
       <c r="C3398" t="inlineStr">
         <is>
-          <t xml:space="preserve">EDER RODRIGUES DA SILVA </t>
+          <t>EDSON ARAUJO - FL8</t>
         </is>
       </c>
       <c r="D3398" t="inlineStr">
         <is>
-          <t>EDERS</t>
+          <t>EDS8</t>
         </is>
       </c>
     </row>
     <row r="3399">
       <c r="A3399" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3399" t="n">
-        <v>3373</v>
+        <v>3328</v>
       </c>
       <c r="C3399" t="inlineStr">
         <is>
-          <t xml:space="preserve">NATANAEL TAVARES DE SOUSA </t>
+          <t>ALAN ARAUJO DA SILVA</t>
         </is>
       </c>
       <c r="D3399" t="inlineStr">
         <is>
-          <t>NTSOUSA</t>
+          <t>ARSILVA</t>
         </is>
       </c>
     </row>
     <row r="3400">
       <c r="A3400" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3400" t="n">
-        <v>3374</v>
+        <v>3350</v>
       </c>
       <c r="C3400" t="inlineStr">
         <is>
-          <t>REINALDO DA SILVA COSTA</t>
+          <t xml:space="preserve">EDER RODRIGUES DA SILVA </t>
         </is>
       </c>
       <c r="D3400" t="inlineStr">
         <is>
-          <t>RSCOSTA</t>
+          <t>EDERS</t>
         </is>
       </c>
     </row>
     <row r="3401">
       <c r="A3401" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3401" t="n">
-        <v>3399</v>
+        <v>3373</v>
       </c>
       <c r="C3401" t="inlineStr">
         <is>
-          <t xml:space="preserve">RICARDO BARBOSA DOS SANTOS </t>
+          <t xml:space="preserve">NATANAEL TAVARES DE SOUSA </t>
         </is>
       </c>
       <c r="D3401" t="inlineStr">
         <is>
-          <t>RICARDOSAN</t>
+          <t>NTSOUSA</t>
         </is>
       </c>
     </row>
@@ -68458,56 +68458,56 @@
         </is>
       </c>
       <c r="B3402" t="n">
-        <v>3427</v>
+        <v>3374</v>
       </c>
       <c r="C3402" t="inlineStr">
         <is>
-          <t>ROQUE COMERCIO TEMPORARIO</t>
+          <t>REINALDO DA SILVA COSTA</t>
         </is>
       </c>
       <c r="D3402" t="inlineStr">
         <is>
-          <t>ROQUECOM</t>
+          <t>RSCOSTA</t>
         </is>
       </c>
     </row>
     <row r="3403">
       <c r="A3403" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3403" t="n">
-        <v>3428</v>
+        <v>3399</v>
       </c>
       <c r="C3403" t="inlineStr">
         <is>
-          <t>ROQUE PLUS TEMPORARIO</t>
+          <t xml:space="preserve">RICARDO BARBOSA DOS SANTOS </t>
         </is>
       </c>
       <c r="D3403" t="inlineStr">
         <is>
-          <t>ROQUEPLUS</t>
+          <t>RICARDOSAN</t>
         </is>
       </c>
     </row>
     <row r="3404">
       <c r="A3404" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3404" t="n">
-        <v>3432</v>
+        <v>3427</v>
       </c>
       <c r="C3404" t="inlineStr">
         <is>
-          <t>PATRICIA DOS SANTOS NONATO OLIVEIRA</t>
+          <t>ROQUE COMERCIO TEMPORARIO</t>
         </is>
       </c>
       <c r="D3404" t="inlineStr">
         <is>
-          <t>PATRICIAD</t>
+          <t>ROQUECOM</t>
         </is>
       </c>
     </row>
@@ -68518,36 +68518,36 @@
         </is>
       </c>
       <c r="B3405" t="n">
-        <v>3448</v>
+        <v>3428</v>
       </c>
       <c r="C3405" t="inlineStr">
         <is>
-          <t xml:space="preserve">GABRIEL SOUZA CARVALHO </t>
+          <t>ROQUE PLUS TEMPORARIO</t>
         </is>
       </c>
       <c r="D3405" t="inlineStr">
         <is>
-          <t>GABRIEL20</t>
+          <t>ROQUEPLUS</t>
         </is>
       </c>
     </row>
     <row r="3406">
       <c r="A3406" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3406" t="n">
-        <v>3465</v>
+        <v>3432</v>
       </c>
       <c r="C3406" t="inlineStr">
         <is>
-          <t>LUIZA MARIA BARRETO BARBOSA</t>
+          <t>PATRICIA DOS SANTOS NONATO OLIVEIRA</t>
         </is>
       </c>
       <c r="D3406" t="inlineStr">
         <is>
-          <t>LUIZA.MARIA</t>
+          <t>PATRICIAD</t>
         </is>
       </c>
     </row>
@@ -68558,36 +68558,36 @@
         </is>
       </c>
       <c r="B3407" t="n">
-        <v>3468</v>
+        <v>3448</v>
       </c>
       <c r="C3407" t="inlineStr">
         <is>
-          <t>KAWA ALMEIDA CAMPOS</t>
+          <t xml:space="preserve">GABRIEL SOUZA CARVALHO </t>
         </is>
       </c>
       <c r="D3407" t="inlineStr">
         <is>
-          <t>KAWA</t>
+          <t>GABRIEL20</t>
         </is>
       </c>
     </row>
     <row r="3408">
       <c r="A3408" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3408" t="n">
-        <v>3476</v>
+        <v>3465</v>
       </c>
       <c r="C3408" t="inlineStr">
         <is>
-          <t xml:space="preserve"> FRANCISCA LEIDIANE M. MENDES NASCIMENTO</t>
+          <t>LUIZA MARIA BARRETO BARBOSA</t>
         </is>
       </c>
       <c r="D3408" t="inlineStr">
         <is>
-          <t>FLEIDIANE</t>
+          <t>LUIZA.MARIA</t>
         </is>
       </c>
     </row>
@@ -68598,96 +68598,96 @@
         </is>
       </c>
       <c r="B3409" t="n">
-        <v>3477</v>
+        <v>3468</v>
       </c>
       <c r="C3409" t="inlineStr">
         <is>
-          <t>MARIA THAIS MARTINS PEREIRA SILVA</t>
+          <t>KAWA ALMEIDA CAMPOS</t>
         </is>
       </c>
       <c r="D3409" t="inlineStr">
         <is>
-          <t>MTHAIS</t>
+          <t>KAWA</t>
         </is>
       </c>
     </row>
     <row r="3410">
       <c r="A3410" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3410" t="n">
-        <v>3271</v>
+        <v>3476</v>
       </c>
       <c r="C3410" t="inlineStr">
         <is>
-          <t>DIEGO DE ARAUJO CALÁBRIA</t>
+          <t xml:space="preserve"> FRANCISCA LEIDIANE M. MENDES NASCIMENTO</t>
         </is>
       </c>
       <c r="D3410" t="inlineStr">
         <is>
-          <t>ARAUJOC</t>
+          <t>FLEIDIANE</t>
         </is>
       </c>
     </row>
     <row r="3411">
       <c r="A3411" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3411" t="n">
-        <v>3272</v>
+        <v>3477</v>
       </c>
       <c r="C3411" t="inlineStr">
         <is>
-          <t>ANNE BEATRIZ SILVA VIRGINO</t>
+          <t>MARIA THAIS MARTINS PEREIRA SILVA</t>
         </is>
       </c>
       <c r="D3411" t="inlineStr">
         <is>
-          <t>ABVIRGINIO</t>
+          <t>MTHAIS</t>
         </is>
       </c>
     </row>
     <row r="3412">
       <c r="A3412" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3412" t="n">
-        <v>3293</v>
+        <v>3271</v>
       </c>
       <c r="C3412" t="inlineStr">
         <is>
-          <t xml:space="preserve">CARLOS ALBERTO VIRIATO SANTOS </t>
+          <t>DIEGO DE ARAUJO CALÁBRIA</t>
         </is>
       </c>
       <c r="D3412" t="inlineStr">
         <is>
-          <t>CVIRIATO</t>
+          <t>ARAUJOC</t>
         </is>
       </c>
     </row>
     <row r="3413">
       <c r="A3413" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3413" t="n">
-        <v>3381</v>
+        <v>3272</v>
       </c>
       <c r="C3413" t="inlineStr">
         <is>
-          <t>ALAN CAIQUE SANTOS E SANTOS</t>
+          <t>ANNE BEATRIZ SILVA VIRGINO</t>
         </is>
       </c>
       <c r="D3413" t="inlineStr">
         <is>
-          <t>ALANSANTOS</t>
+          <t>ABVIRGINIO</t>
         </is>
       </c>
     </row>
@@ -68698,496 +68698,496 @@
         </is>
       </c>
       <c r="B3414" t="n">
-        <v>3443</v>
+        <v>3293</v>
       </c>
       <c r="C3414" t="inlineStr">
         <is>
-          <t>SANON MOREIRA SOUZA</t>
+          <t xml:space="preserve">CARLOS ALBERTO VIRIATO SANTOS </t>
         </is>
       </c>
       <c r="D3414" t="inlineStr">
         <is>
-          <t>SANON</t>
+          <t>CVIRIATO</t>
         </is>
       </c>
     </row>
     <row r="3415">
       <c r="A3415" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3415" t="n">
-        <v>3516</v>
+        <v>3381</v>
       </c>
       <c r="C3415" t="inlineStr">
         <is>
-          <t>FRANCISCO RILDER TELES DE OLIVEIRA</t>
+          <t>ALAN CAIQUE SANTOS E SANTOS</t>
         </is>
       </c>
       <c r="D3415" t="inlineStr">
         <is>
-          <t>RILDER</t>
+          <t>ALANSANTOS</t>
         </is>
       </c>
     </row>
     <row r="3416">
       <c r="A3416" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3416" t="n">
-        <v>3519</v>
+        <v>3443</v>
       </c>
       <c r="C3416" t="inlineStr">
         <is>
-          <t>MARIA LUANA DE ALMEIDA BATISTA</t>
+          <t>SANON MOREIRA SOUZA</t>
         </is>
       </c>
       <c r="D3416" t="inlineStr">
         <is>
-          <t>M.LUANA</t>
+          <t>SANON</t>
         </is>
       </c>
     </row>
     <row r="3417">
       <c r="A3417" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3417" t="n">
-        <v>3540</v>
+        <v>3516</v>
       </c>
       <c r="C3417" t="inlineStr">
         <is>
-          <t>HELEN VITORIA OLIVEIRA DA ROCHA</t>
+          <t>FRANCISCO RILDER TELES DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D3417" t="inlineStr">
         <is>
-          <t>H.VITORIA</t>
+          <t>RILDER</t>
         </is>
       </c>
     </row>
     <row r="3418">
       <c r="A3418" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3418" t="n">
-        <v>3331</v>
+        <v>3519</v>
       </c>
       <c r="C3418" t="inlineStr">
         <is>
-          <t>LOUIZE VANIELLE RODRIGUES FARIAS</t>
+          <t>MARIA LUANA DE ALMEIDA BATISTA</t>
         </is>
       </c>
       <c r="D3418" t="inlineStr">
         <is>
-          <t>LVFARIAS</t>
+          <t>M.LUANA</t>
         </is>
       </c>
     </row>
     <row r="3419">
       <c r="A3419" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B3419" t="n">
-        <v>3332</v>
+        <v>3540</v>
       </c>
       <c r="C3419" t="inlineStr">
         <is>
-          <t>ALEXSANDRO PEIXOTO DA VEIGA PACHECO</t>
+          <t>HELEN VITORIA OLIVEIRA DA ROCHA</t>
         </is>
       </c>
       <c r="D3419" t="inlineStr">
         <is>
-          <t>APVEIGA</t>
+          <t>H.VITORIA</t>
         </is>
       </c>
     </row>
     <row r="3420">
       <c r="A3420" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3420" t="n">
-        <v>3334</v>
+        <v>3331</v>
       </c>
       <c r="C3420" t="inlineStr">
         <is>
-          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+          <t>LOUIZE VANIELLE RODRIGUES FARIAS</t>
         </is>
       </c>
       <c r="D3420" t="inlineStr">
         <is>
-          <t>MTGASPAR</t>
+          <t>LVFARIAS</t>
         </is>
       </c>
     </row>
     <row r="3421">
       <c r="A3421" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B3421" t="n">
-        <v>3345</v>
+        <v>3332</v>
       </c>
       <c r="C3421" t="inlineStr">
         <is>
-          <t>AURICÉLIA INACIO PEREIRA</t>
+          <t>ALEXSANDRO PEIXOTO DA VEIGA PACHECO</t>
         </is>
       </c>
       <c r="D3421" t="inlineStr">
         <is>
-          <t>AIPEREIRA</t>
+          <t>APVEIGA</t>
         </is>
       </c>
     </row>
     <row r="3422">
       <c r="A3422" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3422" t="n">
-        <v>3363</v>
+        <v>3334</v>
       </c>
       <c r="C3422" t="inlineStr">
         <is>
-          <t>IASMIN LEAL ALVES</t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
       <c r="D3422" t="inlineStr">
         <is>
-          <t>ILALVES</t>
+          <t>MTGASPAR</t>
         </is>
       </c>
     </row>
     <row r="3423">
       <c r="A3423" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3423" t="n">
-        <v>3370</v>
+        <v>3345</v>
       </c>
       <c r="C3423" t="inlineStr">
         <is>
-          <t>CARLOS DIEGO ARAUJO ALMEIDA</t>
+          <t>AURICÉLIA INACIO PEREIRA</t>
         </is>
       </c>
       <c r="D3423" t="inlineStr">
         <is>
-          <t>CDIEGO</t>
+          <t>AIPEREIRA</t>
         </is>
       </c>
     </row>
     <row r="3424">
       <c r="A3424" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3424" t="n">
-        <v>3379</v>
+        <v>3363</v>
       </c>
       <c r="C3424" t="inlineStr">
         <is>
-          <t xml:space="preserve">MATHEUS EVANGELISTA FERREIRA </t>
+          <t>IASMIN LEAL ALVES</t>
         </is>
       </c>
       <c r="D3424" t="inlineStr">
         <is>
-          <t>MMFERREIRA</t>
+          <t>ILALVES</t>
         </is>
       </c>
     </row>
     <row r="3425">
       <c r="A3425" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3425" t="n">
-        <v>3419</v>
+        <v>3370</v>
       </c>
       <c r="C3425" t="inlineStr">
         <is>
-          <t xml:space="preserve">DAVID EVANGELISTA SILVA </t>
+          <t>CARLOS DIEGO ARAUJO ALMEIDA</t>
         </is>
       </c>
       <c r="D3425" t="inlineStr">
         <is>
-          <t>DAVID</t>
+          <t>CDIEGO</t>
         </is>
       </c>
     </row>
     <row r="3426">
       <c r="A3426" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3426" t="n">
-        <v>3423</v>
+        <v>3379</v>
       </c>
       <c r="C3426" t="inlineStr">
         <is>
-          <t>MARCIO JOSE TIAGO</t>
+          <t xml:space="preserve">MATHEUS EVANGELISTA FERREIRA </t>
         </is>
       </c>
       <c r="D3426" t="inlineStr">
         <is>
-          <t>MJTIAGO</t>
+          <t>MMFERREIRA</t>
         </is>
       </c>
     </row>
     <row r="3427">
       <c r="A3427" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3427" t="n">
-        <v>3453</v>
+        <v>3419</v>
       </c>
       <c r="C3427" t="inlineStr">
         <is>
-          <t xml:space="preserve">LAURIENE SILVA BARBOSA </t>
+          <t xml:space="preserve">DAVID EVANGELISTA SILVA </t>
         </is>
       </c>
       <c r="D3427" t="inlineStr">
         <is>
-          <t>LAURIENE</t>
+          <t>DAVID</t>
         </is>
       </c>
     </row>
     <row r="3428">
       <c r="A3428" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3428" t="n">
-        <v>3478</v>
+        <v>3423</v>
       </c>
       <c r="C3428" t="inlineStr">
         <is>
-          <t>LEANDRO BRITO NOGUEIRA DE OLIVEIRA</t>
+          <t>MARCIO JOSE TIAGO</t>
         </is>
       </c>
       <c r="D3428" t="inlineStr">
         <is>
-          <t>LBNOGUEIRA</t>
+          <t>MJTIAGO</t>
         </is>
       </c>
     </row>
     <row r="3429">
       <c r="A3429" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3429" t="n">
-        <v>3479</v>
+        <v>3453</v>
       </c>
       <c r="C3429" t="inlineStr">
         <is>
-          <t>ESDRAS ALESSANDRO SANTOS SANTANA</t>
+          <t xml:space="preserve">LAURIENE SILVA BARBOSA </t>
         </is>
       </c>
       <c r="D3429" t="inlineStr">
         <is>
-          <t>EALESSANDRO</t>
+          <t>LAURIENE</t>
         </is>
       </c>
     </row>
     <row r="3430">
       <c r="A3430" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3430" t="n">
-        <v>3480</v>
+        <v>3478</v>
       </c>
       <c r="C3430" t="inlineStr">
         <is>
-          <t xml:space="preserve">LUCIMARA SOUSA LIMA </t>
+          <t>LEANDRO BRITO NOGUEIRA DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D3430" t="inlineStr">
         <is>
-          <t>LUCIMARA</t>
+          <t>LBNOGUEIRA</t>
         </is>
       </c>
     </row>
     <row r="3431">
       <c r="A3431" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3431" t="n">
-        <v>3482</v>
+        <v>3479</v>
       </c>
       <c r="C3431" t="inlineStr">
         <is>
-          <t>DANIEL FERNANDES DINIZ HERACLIO</t>
+          <t>ESDRAS ALESSANDRO SANTOS SANTANA</t>
         </is>
       </c>
       <c r="D3431" t="inlineStr">
         <is>
-          <t>DFDINIZ</t>
+          <t>EALESSANDRO</t>
         </is>
       </c>
     </row>
     <row r="3432">
       <c r="A3432" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3432" t="n">
-        <v>3518</v>
+        <v>3480</v>
       </c>
       <c r="C3432" t="inlineStr">
         <is>
-          <t>RAMYRA ALVES FELIX DA SILVA</t>
+          <t xml:space="preserve">LUCIMARA SOUSA LIMA </t>
         </is>
       </c>
       <c r="D3432" t="inlineStr">
         <is>
-          <t>RFELIX</t>
+          <t>LUCIMARA</t>
         </is>
       </c>
     </row>
     <row r="3433">
       <c r="A3433" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3433" t="n">
-        <v>3534</v>
+        <v>3482</v>
       </c>
       <c r="C3433" t="inlineStr">
         <is>
-          <t xml:space="preserve">CAIO DE SOUZA VINHAS </t>
+          <t>DANIEL FERNANDES DINIZ HERACLIO</t>
         </is>
       </c>
       <c r="D3433" t="inlineStr">
         <is>
-          <t>CVINHAS</t>
+          <t>DFDINIZ</t>
         </is>
       </c>
     </row>
     <row r="3434">
       <c r="A3434" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3434" t="n">
-        <v>3535</v>
+        <v>3518</v>
       </c>
       <c r="C3434" t="inlineStr">
         <is>
-          <t>ROMARIO DE SOUSA SILVA</t>
+          <t>RAMYRA ALVES FELIX DA SILVA</t>
         </is>
       </c>
       <c r="D3434" t="inlineStr">
         <is>
-          <t>RSOUSAS</t>
+          <t>RFELIX</t>
         </is>
       </c>
     </row>
     <row r="3435">
       <c r="A3435" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3435" t="n">
-        <v>3536</v>
+        <v>3534</v>
       </c>
       <c r="C3435" t="inlineStr">
         <is>
-          <t>JHONATAS CARVALHO OLIVEIRA</t>
+          <t xml:space="preserve">CAIO DE SOUZA VINHAS </t>
         </is>
       </c>
       <c r="D3435" t="inlineStr">
         <is>
-          <t>JHONATASC</t>
+          <t>CVINHAS</t>
         </is>
       </c>
     </row>
     <row r="3436">
       <c r="A3436" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3436" t="n">
-        <v>940529</v>
+        <v>3535</v>
       </c>
       <c r="C3436" t="inlineStr">
         <is>
-          <t>EDGAR FELIX - FL9</t>
+          <t>ROMARIO DE SOUSA SILVA</t>
         </is>
       </c>
       <c r="D3436" t="inlineStr">
         <is>
-          <t>EDGAR F</t>
+          <t>RSOUSAS</t>
         </is>
       </c>
     </row>
     <row r="3437">
       <c r="A3437" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3437" t="n">
-        <v>3304</v>
+        <v>3536</v>
       </c>
       <c r="C3437" t="inlineStr">
         <is>
-          <t>JOACI GUILHERME GONÇALVES DA LUZ</t>
+          <t>JHONATAS CARVALHO OLIVEIRA</t>
         </is>
       </c>
       <c r="D3437" t="inlineStr">
         <is>
-          <t>JLUZ</t>
+          <t>JHONATASC</t>
         </is>
       </c>
     </row>
     <row r="3438">
       <c r="A3438" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3438" t="n">
-        <v>3305</v>
+        <v>940529</v>
       </c>
       <c r="C3438" t="inlineStr">
         <is>
-          <t>JOÃO VITOR DE ARAÚJO GONÇALVES</t>
+          <t>EDGAR FELIX - FL9</t>
         </is>
       </c>
       <c r="D3438" t="inlineStr">
         <is>
-          <t>JJVITOR</t>
+          <t>EDGAR F</t>
         </is>
       </c>
     </row>
@@ -69198,256 +69198,256 @@
         </is>
       </c>
       <c r="B3439" t="n">
-        <v>3306</v>
+        <v>3304</v>
       </c>
       <c r="C3439" t="inlineStr">
         <is>
-          <t>WENDERSON MARCOS DOS SANTOS</t>
+          <t>JOACI GUILHERME GONÇALVES DA LUZ</t>
         </is>
       </c>
       <c r="D3439" t="inlineStr">
         <is>
-          <t>WWMARCOS</t>
+          <t>JLUZ</t>
         </is>
       </c>
     </row>
     <row r="3440">
       <c r="A3440" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3440" t="n">
-        <v>3335</v>
+        <v>3305</v>
       </c>
       <c r="C3440" t="inlineStr">
         <is>
-          <t>EDILBERTO LEMOS DE LIMA</t>
+          <t>JOÃO VITOR DE ARAÚJO GONÇALVES</t>
         </is>
       </c>
       <c r="D3440" t="inlineStr">
         <is>
-          <t>ELEMOS</t>
+          <t>JJVITOR</t>
         </is>
       </c>
     </row>
     <row r="3441">
       <c r="A3441" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3441" t="n">
-        <v>3336</v>
+        <v>3306</v>
       </c>
       <c r="C3441" t="inlineStr">
         <is>
-          <t>EZEQUIEL SOUZA DO NASCIMENTO</t>
+          <t>WENDERSON MARCOS DOS SANTOS</t>
         </is>
       </c>
       <c r="D3441" t="inlineStr">
         <is>
-          <t>ESNASCIMENTO</t>
+          <t>WWMARCOS</t>
         </is>
       </c>
     </row>
     <row r="3442">
       <c r="A3442" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3442" t="n">
-        <v>3341</v>
+        <v>3335</v>
       </c>
       <c r="C3442" t="inlineStr">
         <is>
-          <t>ALCIONE MARIANO DE OLIVEIRA</t>
+          <t>EDILBERTO LEMOS DE LIMA</t>
         </is>
       </c>
       <c r="D3442" t="inlineStr">
         <is>
-          <t>AMOLIVEIRA</t>
+          <t>ELEMOS</t>
         </is>
       </c>
     </row>
     <row r="3443">
       <c r="A3443" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3443" t="n">
-        <v>3401</v>
+        <v>3336</v>
       </c>
       <c r="C3443" t="inlineStr">
         <is>
-          <t xml:space="preserve">TULIO HENRIQUE DA SILVA CARVALHO </t>
+          <t>EZEQUIEL SOUZA DO NASCIMENTO</t>
         </is>
       </c>
       <c r="D3443" t="inlineStr">
         <is>
-          <t>TULIO</t>
+          <t>ESNASCIMENTO</t>
         </is>
       </c>
     </row>
     <row r="3444">
       <c r="A3444" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3444" t="n">
-        <v>3411</v>
+        <v>3341</v>
       </c>
       <c r="C3444" t="inlineStr">
         <is>
-          <t>CONEXAO RUBYA DANILLA</t>
+          <t>ALCIONE MARIANO DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D3444" t="inlineStr">
         <is>
-          <t>CONEXAORUBYA</t>
+          <t>AMOLIVEIRA</t>
         </is>
       </c>
     </row>
     <row r="3445">
       <c r="A3445" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3445" t="n">
-        <v>3412</v>
+        <v>3401</v>
       </c>
       <c r="C3445" t="inlineStr">
         <is>
-          <t>CONEXAO RAFAEL</t>
+          <t xml:space="preserve">TULIO HENRIQUE DA SILVA CARVALHO </t>
         </is>
       </c>
       <c r="D3445" t="inlineStr">
         <is>
-          <t>CONEXAORAFAEL</t>
+          <t>TULIO</t>
         </is>
       </c>
     </row>
     <row r="3446">
       <c r="A3446" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3446" t="n">
-        <v>3264</v>
+        <v>3411</v>
       </c>
       <c r="C3446" t="inlineStr">
         <is>
-          <t xml:space="preserve">WILTON CARLOS MACIEL DE ASSIS </t>
+          <t>CONEXAO RUBYA DANILLA</t>
         </is>
       </c>
       <c r="D3446" t="inlineStr">
         <is>
-          <t>WCMACIEL</t>
+          <t>CONEXAORUBYA</t>
         </is>
       </c>
     </row>
     <row r="3447">
       <c r="A3447" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3447" t="n">
-        <v>3340</v>
+        <v>3412</v>
       </c>
       <c r="C3447" t="inlineStr">
         <is>
-          <t>ROGELENO FARIAS FEIJÃO FILHO</t>
+          <t>CONEXAO RAFAEL</t>
         </is>
       </c>
       <c r="D3447" t="inlineStr">
         <is>
-          <t>RFEIJAO</t>
+          <t>CONEXAORAFAEL</t>
         </is>
       </c>
     </row>
     <row r="3448">
       <c r="A3448" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3448" t="n">
-        <v>940550</v>
+        <v>3264</v>
       </c>
       <c r="C3448" t="inlineStr">
         <is>
-          <t>RAFAELE RIBEIRO CARNEIRO</t>
+          <t xml:space="preserve">WILTON CARLOS MACIEL DE ASSIS </t>
         </is>
       </c>
       <c r="D3448" t="inlineStr">
         <is>
-          <t>RAFAELE</t>
+          <t>WCMACIEL</t>
         </is>
       </c>
     </row>
     <row r="3449">
       <c r="A3449" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3449" t="n">
-        <v>3377</v>
+        <v>3340</v>
       </c>
       <c r="C3449" t="inlineStr">
         <is>
-          <t xml:space="preserve"> ISALTINO BISPO DE OLIVEIRA JUNIOR</t>
+          <t>ROGELENO FARIAS FEIJÃO FILHO</t>
         </is>
       </c>
       <c r="D3449" t="inlineStr">
         <is>
-          <t>BJUNIOR</t>
+          <t>RFEIJAO</t>
         </is>
       </c>
     </row>
     <row r="3450">
       <c r="A3450" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>99</t>
         </is>
       </c>
       <c r="B3450" t="n">
-        <v>3425</v>
+        <v>940550</v>
       </c>
       <c r="C3450" t="inlineStr">
         <is>
-          <t xml:space="preserve"> CIRLANE ARAUJO SOUZA </t>
+          <t>RAFAELE RIBEIRO CARNEIRO</t>
         </is>
       </c>
       <c r="D3450" t="inlineStr">
         <is>
-          <t>CIRLANES</t>
+          <t>RAFAELE</t>
         </is>
       </c>
     </row>
     <row r="3451">
       <c r="A3451" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3451" t="n">
-        <v>3454</v>
+        <v>3377</v>
       </c>
       <c r="C3451" t="inlineStr">
         <is>
-          <t>ANTONIA SAMARA DE SOUZA SOARES</t>
+          <t xml:space="preserve"> ISALTINO BISPO DE OLIVEIRA JUNIOR</t>
         </is>
       </c>
       <c r="D3451" t="inlineStr">
         <is>
-          <t>ANTSAMARA</t>
+          <t>BJUNIOR</t>
         </is>
       </c>
     </row>
@@ -69458,76 +69458,76 @@
         </is>
       </c>
       <c r="B3452" t="n">
-        <v>3491</v>
+        <v>3425</v>
       </c>
       <c r="C3452" t="inlineStr">
         <is>
-          <t>PEDRO JOSE DO NASCIMENTO NETO</t>
+          <t xml:space="preserve"> CIRLANE ARAUJO SOUZA </t>
         </is>
       </c>
       <c r="D3452" t="inlineStr">
         <is>
-          <t>P.JOSE</t>
+          <t>CIRLANES</t>
         </is>
       </c>
     </row>
     <row r="3453">
       <c r="A3453" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3453" t="n">
-        <v>3492</v>
+        <v>3454</v>
       </c>
       <c r="C3453" t="inlineStr">
         <is>
-          <t>PAULA CARLA CALDAS MOTA</t>
+          <t>ANTONIA SAMARA DE SOUZA SOARES</t>
         </is>
       </c>
       <c r="D3453" t="inlineStr">
         <is>
-          <t>P.CARLA</t>
+          <t>ANTSAMARA</t>
         </is>
       </c>
     </row>
     <row r="3454">
       <c r="A3454" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3454" t="n">
-        <v>3542</v>
+        <v>3491</v>
       </c>
       <c r="C3454" t="inlineStr">
         <is>
-          <t>ANTONIA MILENA SOUSA ANDRADE</t>
+          <t>PEDRO JOSE DO NASCIMENTO NETO</t>
         </is>
       </c>
       <c r="D3454" t="inlineStr">
         <is>
-          <t>A.MILENA</t>
+          <t>P.JOSE</t>
         </is>
       </c>
     </row>
     <row r="3455">
       <c r="A3455" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3455" t="n">
-        <v>3547</v>
+        <v>3492</v>
       </c>
       <c r="C3455" t="inlineStr">
         <is>
-          <t xml:space="preserve">DAVI PEREIRA DA SILVA </t>
+          <t>PAULA CARLA CALDAS MOTA</t>
         </is>
       </c>
       <c r="D3455" t="inlineStr">
         <is>
-          <t>DPSILVA</t>
+          <t>P.CARLA</t>
         </is>
       </c>
     </row>
@@ -69538,16 +69538,16 @@
         </is>
       </c>
       <c r="B3456" t="n">
-        <v>3294</v>
+        <v>3542</v>
       </c>
       <c r="C3456" t="inlineStr">
         <is>
-          <t>GLEICIANE MIRANDA DE MORAIS</t>
+          <t>ANTONIA MILENA SOUSA ANDRADE</t>
         </is>
       </c>
       <c r="D3456" t="inlineStr">
         <is>
-          <t>GMIRANDA</t>
+          <t>A.MILENA</t>
         </is>
       </c>
     </row>
@@ -69558,194 +69558,234 @@
         </is>
       </c>
       <c r="B3457" t="n">
-        <v>3295</v>
+        <v>3547</v>
       </c>
       <c r="C3457" t="inlineStr">
         <is>
-          <t>MARIA ESTEFANNY DA SILVA MOURA</t>
+          <t xml:space="preserve">DAVI PEREIRA DA SILVA </t>
         </is>
       </c>
       <c r="D3457" t="inlineStr">
         <is>
-          <t>MESTEFANNY</t>
+          <t>DPSILVA</t>
         </is>
       </c>
     </row>
     <row r="3458">
       <c r="A3458" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3458" t="n">
-        <v>3296</v>
+        <v>3294</v>
       </c>
       <c r="C3458" t="inlineStr">
         <is>
-          <t>PEDRO IAGO FONSECA EVANGELISTA</t>
+          <t>GLEICIANE MIRANDA DE MORAIS</t>
         </is>
       </c>
       <c r="D3458" t="inlineStr">
         <is>
-          <t>PIFONSECA</t>
+          <t>GMIRANDA</t>
         </is>
       </c>
     </row>
     <row r="3459">
       <c r="A3459" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3459" t="n">
-        <v>940544</v>
+        <v>3295</v>
       </c>
       <c r="C3459" t="inlineStr">
         <is>
-          <t>LUTY LOG TRANSPORTES - FL8</t>
+          <t>MARIA ESTEFANNY DA SILVA MOURA</t>
         </is>
       </c>
       <c r="D3459" t="inlineStr">
         <is>
-          <t>LUTY LOG</t>
+          <t>MESTEFANNY</t>
         </is>
       </c>
     </row>
     <row r="3460">
       <c r="A3460" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3460" t="n">
-        <v>3380</v>
+        <v>3296</v>
       </c>
       <c r="C3460" t="inlineStr">
         <is>
-          <t>FRANCISCO MATHEUS RABELO DA COSTA</t>
+          <t>PEDRO IAGO FONSECA EVANGELISTA</t>
         </is>
       </c>
       <c r="D3460" t="inlineStr">
         <is>
-          <t>FMATHEUS</t>
+          <t>PIFONSECA</t>
         </is>
       </c>
     </row>
     <row r="3461">
       <c r="A3461" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B3461" t="n">
-        <v>3410</v>
+        <v>940544</v>
       </c>
       <c r="C3461" t="inlineStr">
         <is>
-          <t xml:space="preserve"> BRENO ALLAN DE JESUS</t>
+          <t>LUTY LOG TRANSPORTES - FL8</t>
         </is>
       </c>
       <c r="D3461" t="inlineStr">
         <is>
-          <t>JESUS</t>
+          <t>LUTY LOG</t>
         </is>
       </c>
     </row>
     <row r="3462">
       <c r="A3462" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3462" t="n">
-        <v>3444</v>
+        <v>3380</v>
       </c>
       <c r="C3462" t="inlineStr">
         <is>
-          <t>THIAGO COSTA SILVA</t>
+          <t>FRANCISCO MATHEUS RABELO DA COSTA</t>
         </is>
       </c>
       <c r="D3462" t="inlineStr">
         <is>
-          <t>THIAGOC</t>
+          <t>FMATHEUS</t>
         </is>
       </c>
     </row>
     <row r="3463">
       <c r="A3463" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3463" t="n">
-        <v>3456</v>
+        <v>3410</v>
       </c>
       <c r="C3463" t="inlineStr">
         <is>
-          <t>FELIPE BOTH MAZUCHINI</t>
+          <t xml:space="preserve"> BRENO ALLAN DE JESUS</t>
         </is>
       </c>
       <c r="D3463" t="inlineStr">
         <is>
-          <t>FELIPEB</t>
+          <t>JESUS</t>
         </is>
       </c>
     </row>
     <row r="3464">
       <c r="A3464" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3464" t="n">
-        <v>3457</v>
+        <v>3444</v>
       </c>
       <c r="C3464" t="inlineStr">
         <is>
-          <t>FRANKLIN VIEIRA GOMES</t>
+          <t>THIAGO COSTA SILVA</t>
         </is>
       </c>
       <c r="D3464" t="inlineStr">
         <is>
-          <t>VIEIRAF</t>
+          <t>THIAGOC</t>
         </is>
       </c>
     </row>
     <row r="3465">
       <c r="A3465" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3465" t="n">
-        <v>3507</v>
+        <v>3456</v>
       </c>
       <c r="C3465" t="inlineStr">
         <is>
-          <t>KARINE TEODORA ALVES DE OLIVEIRA</t>
+          <t>FELIPE BOTH MAZUCHINI</t>
         </is>
       </c>
       <c r="D3465" t="inlineStr">
         <is>
-          <t>KOLIVEIRA</t>
+          <t>FELIPEB</t>
         </is>
       </c>
     </row>
     <row r="3466">
       <c r="A3466" t="inlineStr">
         <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B3466" t="n">
+        <v>3457</v>
+      </c>
+      <c r="C3466" t="inlineStr">
+        <is>
+          <t>FRANKLIN VIEIRA GOMES</t>
+        </is>
+      </c>
+      <c r="D3466" t="inlineStr">
+        <is>
+          <t>VIEIRAF</t>
+        </is>
+      </c>
+    </row>
+    <row r="3467">
+      <c r="A3467" t="inlineStr">
+        <is>
           <t>5</t>
         </is>
       </c>
-      <c r="B3466" t="n">
+      <c r="B3467" t="n">
+        <v>3507</v>
+      </c>
+      <c r="C3467" t="inlineStr">
+        <is>
+          <t>KARINE TEODORA ALVES DE OLIVEIRA</t>
+        </is>
+      </c>
+      <c r="D3467" t="inlineStr">
+        <is>
+          <t>KOLIVEIRA</t>
+        </is>
+      </c>
+    </row>
+    <row r="3468">
+      <c r="A3468" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B3468" t="n">
         <v>3520</v>
       </c>
-      <c r="C3466" t="inlineStr">
+      <c r="C3468" t="inlineStr">
         <is>
           <t xml:space="preserve"> EMERSON FILIPE MELO DE AGUIAR</t>
         </is>
       </c>
-      <c r="D3466" t="inlineStr">
+      <c r="D3468" t="inlineStr">
         <is>
           <t>E.FILIPE</t>
         </is>

</xml_diff>

<commit_message>
chore(data): batch update intraday televendas - 08:03:05
</commit_message>
<xml_diff>
--- a/data/dim_televendas.xlsx
+++ b/data/dim_televendas.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3468"/>
+  <dimension ref="A1:D3470"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1026,7 +1026,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>1504</t>
+          <t>LEANDRA</t>
         </is>
       </c>
     </row>
@@ -1546,7 +1546,7 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>1507</t>
+          <t>TIAGO</t>
         </is>
       </c>
     </row>
@@ -1606,7 +1606,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>52</t>
+          <t>HELENA</t>
         </is>
       </c>
     </row>
@@ -3966,7 +3966,7 @@
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>1551</t>
+          <t>ROBSON</t>
         </is>
       </c>
     </row>
@@ -4246,7 +4246,7 @@
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>1524</t>
+          <t>RICARDO</t>
         </is>
       </c>
     </row>
@@ -65814,80 +65814,80 @@
     <row r="3270">
       <c r="A3270" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3270" t="n">
-        <v>3269</v>
+        <v>3553</v>
       </c>
       <c r="C3270" t="inlineStr">
         <is>
-          <t>MARCOS ANTONIO DOS SANTOS BARROS</t>
+          <t>CAIO LUA MENDES DE ARAUJO</t>
         </is>
       </c>
       <c r="D3270" t="inlineStr">
         <is>
-          <t>MABARROS</t>
+          <t>CAIO.LUA</t>
         </is>
       </c>
     </row>
     <row r="3271">
       <c r="A3271" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3271" t="n">
-        <v>3290</v>
+        <v>3269</v>
       </c>
       <c r="C3271" t="inlineStr">
         <is>
-          <t>ADRIANE DA SILVA ARAUJO</t>
+          <t>MARCOS ANTONIO DOS SANTOS BARROS</t>
         </is>
       </c>
       <c r="D3271" t="inlineStr">
         <is>
-          <t>ADRISILVA</t>
+          <t>MABARROS</t>
         </is>
       </c>
     </row>
     <row r="3272">
       <c r="A3272" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3272" t="n">
-        <v>3292</v>
+        <v>3290</v>
       </c>
       <c r="C3272" t="inlineStr">
         <is>
-          <t>GIOVANI BULHOES DE LIMA</t>
+          <t>ADRIANE DA SILVA ARAUJO</t>
         </is>
       </c>
       <c r="D3272" t="inlineStr">
         <is>
-          <t>GBULHOES</t>
+          <t>ADRISILVA</t>
         </is>
       </c>
     </row>
     <row r="3273">
       <c r="A3273" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3273" t="n">
-        <v>3322</v>
+        <v>3292</v>
       </c>
       <c r="C3273" t="inlineStr">
         <is>
-          <t>FRANCISCO ADRIANO DE OLIVEIRA</t>
+          <t>GIOVANI BULHOES DE LIMA</t>
         </is>
       </c>
       <c r="D3273" t="inlineStr">
         <is>
-          <t>FCOLIVEIRA</t>
+          <t>GBULHOES</t>
         </is>
       </c>
     </row>
@@ -65898,136 +65898,136 @@
         </is>
       </c>
       <c r="B3274" t="n">
-        <v>3323</v>
+        <v>3322</v>
       </c>
       <c r="C3274" t="inlineStr">
         <is>
-          <t>JOAO VICTOR MARTINS DE SOUSA</t>
+          <t>FRANCISCO ADRIANO DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D3274" t="inlineStr">
         <is>
-          <t>JVSOUSA</t>
+          <t>FCOLIVEIRA</t>
         </is>
       </c>
     </row>
     <row r="3275">
       <c r="A3275" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3275" t="n">
-        <v>940552</v>
+        <v>3323</v>
       </c>
       <c r="C3275" t="inlineStr">
         <is>
-          <t>ERASMO EDSON DOS ANJOS</t>
+          <t>JOAO VICTOR MARTINS DE SOUSA</t>
         </is>
       </c>
       <c r="D3275" t="inlineStr">
         <is>
-          <t>ERASMO</t>
+          <t>JVSOUSA</t>
         </is>
       </c>
     </row>
     <row r="3276">
       <c r="A3276" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3276" t="n">
-        <v>940557</v>
+        <v>940552</v>
       </c>
       <c r="C3276" t="inlineStr">
         <is>
-          <t>SEVERINO LUIZ - FL9</t>
+          <t>ERASMO EDSON DOS ANJOS</t>
         </is>
       </c>
       <c r="D3276" t="inlineStr">
         <is>
-          <t>LUIZ</t>
+          <t>ERASMO</t>
         </is>
       </c>
     </row>
     <row r="3277">
       <c r="A3277" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3277" t="n">
-        <v>3471</v>
+        <v>940557</v>
       </c>
       <c r="C3277" t="inlineStr">
         <is>
-          <t>KERLY VIEIRA DE OLIVEIRA VERAS</t>
+          <t>SEVERINO LUIZ - FL9</t>
         </is>
       </c>
       <c r="D3277" t="inlineStr">
         <is>
-          <t>KERLY.VERAS</t>
+          <t>LUIZ</t>
         </is>
       </c>
     </row>
     <row r="3278">
       <c r="A3278" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3278" t="n">
-        <v>3472</v>
+        <v>3471</v>
       </c>
       <c r="C3278" t="inlineStr">
         <is>
-          <t>SAVANA MARIA DE SANTANA</t>
+          <t>KERLY VIEIRA DE OLIVEIRA VERAS</t>
         </is>
       </c>
       <c r="D3278" t="inlineStr">
         <is>
-          <t>SAVANA</t>
+          <t>KERLY.VERAS</t>
         </is>
       </c>
     </row>
     <row r="3279">
       <c r="A3279" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B3279" t="n">
-        <v>3525</v>
+        <v>3472</v>
       </c>
       <c r="C3279" t="inlineStr">
         <is>
-          <t>JOAO VICTOR DE SOUSA SILVA</t>
+          <t>SAVANA MARIA DE SANTANA</t>
         </is>
       </c>
       <c r="D3279" t="inlineStr">
         <is>
-          <t>JVSILVA</t>
+          <t>SAVANA</t>
         </is>
       </c>
     </row>
     <row r="3280">
       <c r="A3280" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3280" t="n">
-        <v>3544</v>
+        <v>3525</v>
       </c>
       <c r="C3280" t="inlineStr">
         <is>
-          <t>ADEILZA PINTO DA SILVA</t>
+          <t>JOAO VICTOR DE SOUSA SILVA</t>
         </is>
       </c>
       <c r="D3280" t="inlineStr">
         <is>
-          <t>ADEILZA</t>
+          <t>JVSILVA</t>
         </is>
       </c>
     </row>
@@ -66038,36 +66038,36 @@
         </is>
       </c>
       <c r="B3281" t="n">
-        <v>3265</v>
+        <v>3544</v>
       </c>
       <c r="C3281" t="inlineStr">
         <is>
-          <t>ANAELSON FREITAS VIEIRA</t>
+          <t>ADEILZA PINTO DA SILVA</t>
         </is>
       </c>
       <c r="D3281" t="inlineStr">
         <is>
-          <t>AFVIEIRA</t>
+          <t>ADEILZA</t>
         </is>
       </c>
     </row>
     <row r="3282">
       <c r="A3282" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3282" t="n">
-        <v>3413</v>
+        <v>3265</v>
       </c>
       <c r="C3282" t="inlineStr">
         <is>
-          <t>CONEXAO THAMIRES MONTEIRO</t>
+          <t>ANAELSON FREITAS VIEIRA</t>
         </is>
       </c>
       <c r="D3282" t="inlineStr">
         <is>
-          <t>CONEXAOTHAMIRES</t>
+          <t>AFVIEIRA</t>
         </is>
       </c>
     </row>
@@ -66078,76 +66078,76 @@
         </is>
       </c>
       <c r="B3283" t="n">
-        <v>3431</v>
+        <v>3413</v>
       </c>
       <c r="C3283" t="inlineStr">
         <is>
-          <t>ALLYSSON PINHEIRO AGUIAR E SILVA</t>
+          <t>CONEXAO THAMIRES MONTEIRO</t>
         </is>
       </c>
       <c r="D3283" t="inlineStr">
         <is>
-          <t>ALYSSONP</t>
+          <t>CONEXAOTHAMIRES</t>
         </is>
       </c>
     </row>
     <row r="3284">
       <c r="A3284" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3284" t="n">
-        <v>3499</v>
+        <v>3431</v>
       </c>
       <c r="C3284" t="inlineStr">
         <is>
-          <t>JAIME VITORINO DE OLIVEIRA SOUSA</t>
+          <t>ALLYSSON PINHEIRO AGUIAR E SILVA</t>
         </is>
       </c>
       <c r="D3284" t="inlineStr">
         <is>
-          <t>JVITORINO</t>
+          <t>ALYSSONP</t>
         </is>
       </c>
     </row>
     <row r="3285">
       <c r="A3285" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3285" t="n">
-        <v>3500</v>
+        <v>3499</v>
       </c>
       <c r="C3285" t="inlineStr">
         <is>
-          <t>TACIANE DE HOLANDA MACIEL</t>
+          <t>JAIME VITORINO DE OLIVEIRA SOUSA</t>
         </is>
       </c>
       <c r="D3285" t="inlineStr">
         <is>
-          <t>TMACIEL</t>
+          <t>JVITORINO</t>
         </is>
       </c>
     </row>
     <row r="3286">
       <c r="A3286" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3286" t="n">
-        <v>3545</v>
+        <v>3500</v>
       </c>
       <c r="C3286" t="inlineStr">
         <is>
-          <t>FABIO JUNIOR DA SILVA FIGUEIRA</t>
+          <t>TACIANE DE HOLANDA MACIEL</t>
         </is>
       </c>
       <c r="D3286" t="inlineStr">
         <is>
-          <t>F.JUNIOR</t>
+          <t>TMACIEL</t>
         </is>
       </c>
     </row>
@@ -66158,76 +66158,76 @@
         </is>
       </c>
       <c r="B3287" t="n">
-        <v>3546</v>
+        <v>3545</v>
       </c>
       <c r="C3287" t="inlineStr">
         <is>
-          <t>GEREMIAS DA SILVA PEREIRA</t>
+          <t>FABIO JUNIOR DA SILVA FIGUEIRA</t>
         </is>
       </c>
       <c r="D3287" t="inlineStr">
         <is>
-          <t>G.SILVA</t>
+          <t>F.JUNIOR</t>
         </is>
       </c>
     </row>
     <row r="3288">
       <c r="A3288" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3288" t="n">
-        <v>3279</v>
+        <v>3546</v>
       </c>
       <c r="C3288" t="inlineStr">
         <is>
-          <t>IARGO GABRIEL SANTOS DE OLIVEIRA</t>
+          <t>GEREMIAS DA SILVA PEREIRA</t>
         </is>
       </c>
       <c r="D3288" t="inlineStr">
         <is>
-          <t>IARGOSANTOS</t>
+          <t>G.SILVA</t>
         </is>
       </c>
     </row>
     <row r="3289">
       <c r="A3289" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3289" t="n">
-        <v>3349</v>
+        <v>3279</v>
       </c>
       <c r="C3289" t="inlineStr">
         <is>
-          <t xml:space="preserve">ROBSON DE SOUZA LEITE </t>
+          <t>IARGO GABRIEL SANTOS DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D3289" t="inlineStr">
         <is>
-          <t>RLEITE</t>
+          <t>IARGOSANTOS</t>
         </is>
       </c>
     </row>
     <row r="3290">
       <c r="A3290" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3290" t="n">
-        <v>3367</v>
+        <v>3349</v>
       </c>
       <c r="C3290" t="inlineStr">
         <is>
-          <t>CARLOS JEANDERSON DA SILVA GUTERRES</t>
+          <t xml:space="preserve">ROBSON DE SOUZA LEITE </t>
         </is>
       </c>
       <c r="D3290" t="inlineStr">
         <is>
-          <t>CGUTERRES</t>
+          <t>RLEITE</t>
         </is>
       </c>
     </row>
@@ -66238,96 +66238,96 @@
         </is>
       </c>
       <c r="B3291" t="n">
-        <v>3392</v>
+        <v>3367</v>
       </c>
       <c r="C3291" t="inlineStr">
         <is>
-          <t xml:space="preserve">LAERCIA KARINE OLIVEIRA MORAIS </t>
+          <t>CARLOS JEANDERSON DA SILVA GUTERRES</t>
         </is>
       </c>
       <c r="D3291" t="inlineStr">
         <is>
-          <t>KARINE28</t>
+          <t>CGUTERRES</t>
         </is>
       </c>
     </row>
     <row r="3292">
       <c r="A3292" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3292" t="n">
-        <v>3446</v>
+        <v>3392</v>
       </c>
       <c r="C3292" t="inlineStr">
         <is>
-          <t>MARIA FERNANDA SOUSA DA CRUZ</t>
+          <t xml:space="preserve">LAERCIA KARINE OLIVEIRA MORAIS </t>
         </is>
       </c>
       <c r="D3292" t="inlineStr">
         <is>
-          <t>MSCRUZ</t>
+          <t>KARINE28</t>
         </is>
       </c>
     </row>
     <row r="3293">
       <c r="A3293" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3293" t="n">
-        <v>3256</v>
+        <v>3446</v>
       </c>
       <c r="C3293" t="inlineStr">
         <is>
-          <t>ANNE CAROLINE ALMEIDA DE MORAIS</t>
+          <t>MARIA FERNANDA SOUSA DA CRUZ</t>
         </is>
       </c>
       <c r="D3293" t="inlineStr">
         <is>
-          <t>ACMORAIS</t>
+          <t>MSCRUZ</t>
         </is>
       </c>
     </row>
     <row r="3294">
       <c r="A3294" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3294" t="n">
-        <v>3257</v>
+        <v>3256</v>
       </c>
       <c r="C3294" t="inlineStr">
         <is>
-          <t xml:space="preserve"> NARA RAIANE RABELO NOBRE</t>
+          <t>ANNE CAROLINE ALMEIDA DE MORAIS</t>
         </is>
       </c>
       <c r="D3294" t="inlineStr">
         <is>
-          <t>NRNOBRE</t>
+          <t>ACMORAIS</t>
         </is>
       </c>
     </row>
     <row r="3295">
       <c r="A3295" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3295" t="n">
-        <v>3268</v>
+        <v>3257</v>
       </c>
       <c r="C3295" t="inlineStr">
         <is>
-          <t>DANRLEY PEREIRA E PEREIRA</t>
+          <t xml:space="preserve"> NARA RAIANE RABELO NOBRE</t>
         </is>
       </c>
       <c r="D3295" t="inlineStr">
         <is>
-          <t>DPEREIRA</t>
+          <t>NRNOBRE</t>
         </is>
       </c>
     </row>
@@ -66338,16 +66338,16 @@
         </is>
       </c>
       <c r="B3296" t="n">
-        <v>3282</v>
+        <v>3268</v>
       </c>
       <c r="C3296" t="inlineStr">
         <is>
-          <t xml:space="preserve">JARDSON ROBERTH CUTRIM SOUZA </t>
+          <t>DANRLEY PEREIRA E PEREIRA</t>
         </is>
       </c>
       <c r="D3296" t="inlineStr">
         <is>
-          <t>JRCSOUZA</t>
+          <t>DPEREIRA</t>
         </is>
       </c>
     </row>
@@ -66358,156 +66358,156 @@
         </is>
       </c>
       <c r="B3297" t="n">
-        <v>3283</v>
+        <v>3282</v>
       </c>
       <c r="C3297" t="inlineStr">
         <is>
-          <t>JESOAIAS DOS SANTOS CABRAL</t>
+          <t xml:space="preserve">JARDSON ROBERTH CUTRIM SOUZA </t>
         </is>
       </c>
       <c r="D3297" t="inlineStr">
         <is>
-          <t>JSCABRAL</t>
+          <t>JRCSOUZA</t>
         </is>
       </c>
     </row>
     <row r="3298">
       <c r="A3298" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3298" t="n">
-        <v>3299</v>
+        <v>3283</v>
       </c>
       <c r="C3298" t="inlineStr">
         <is>
-          <t>CARLOS EDUARDO ANDRADE DE ASSIS</t>
+          <t>JESOAIAS DOS SANTOS CABRAL</t>
         </is>
       </c>
       <c r="D3298" t="inlineStr">
         <is>
-          <t>ANDRADE</t>
+          <t>JSCABRAL</t>
         </is>
       </c>
     </row>
     <row r="3299">
       <c r="A3299" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3299" t="n">
-        <v>3301</v>
+        <v>3299</v>
       </c>
       <c r="C3299" t="inlineStr">
         <is>
-          <t>DIANA KARINE VIANA DA SILVA</t>
+          <t>CARLOS EDUARDO ANDRADE DE ASSIS</t>
         </is>
       </c>
       <c r="D3299" t="inlineStr">
         <is>
-          <t>DKVIANA</t>
+          <t>ANDRADE</t>
         </is>
       </c>
     </row>
     <row r="3300">
       <c r="A3300" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3300" t="n">
-        <v>940537</v>
+        <v>3301</v>
       </c>
       <c r="C3300" t="inlineStr">
         <is>
-          <t xml:space="preserve">TGC TRANSPORTES </t>
+          <t>DIANA KARINE VIANA DA SILVA</t>
         </is>
       </c>
       <c r="D3300" t="inlineStr">
         <is>
-          <t>TGC</t>
+          <t>DKVIANA</t>
         </is>
       </c>
     </row>
     <row r="3301">
       <c r="A3301" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3301" t="n">
-        <v>3343</v>
+        <v>940537</v>
       </c>
       <c r="C3301" t="inlineStr">
         <is>
-          <t>REGINALDO FEITOSA DA SILVA JUNIOR</t>
+          <t xml:space="preserve">TGC TRANSPORTES </t>
         </is>
       </c>
       <c r="D3301" t="inlineStr">
         <is>
-          <t>RFJUNIOR</t>
+          <t>TGC</t>
         </is>
       </c>
     </row>
     <row r="3302">
       <c r="A3302" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3302" t="n">
-        <v>3344</v>
+        <v>3343</v>
       </c>
       <c r="C3302" t="inlineStr">
         <is>
-          <t>JOAO VICTOR MENDONCA DA SILVA</t>
+          <t>REGINALDO FEITOSA DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="D3302" t="inlineStr">
         <is>
-          <t>JVMENDONCA</t>
+          <t>RFJUNIOR</t>
         </is>
       </c>
     </row>
     <row r="3303">
       <c r="A3303" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3303" t="n">
-        <v>3352</v>
+        <v>3344</v>
       </c>
       <c r="C3303" t="inlineStr">
         <is>
-          <t>RICARDO MACAUBAS BOAVENTURA</t>
+          <t>JOAO VICTOR MENDONCA DA SILVA</t>
         </is>
       </c>
       <c r="D3303" t="inlineStr">
         <is>
-          <t>RMACAUBAS</t>
+          <t>JVMENDONCA</t>
         </is>
       </c>
     </row>
     <row r="3304">
       <c r="A3304" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3304" t="n">
-        <v>3364</v>
+        <v>3352</v>
       </c>
       <c r="C3304" t="inlineStr">
         <is>
-          <t>CLOVIS VIDAL DOS SANTOS NETO</t>
+          <t>RICARDO MACAUBAS BOAVENTURA</t>
         </is>
       </c>
       <c r="D3304" t="inlineStr">
         <is>
-          <t>CVNETO</t>
+          <t>RMACAUBAS</t>
         </is>
       </c>
     </row>
@@ -66518,156 +66518,156 @@
         </is>
       </c>
       <c r="B3305" t="n">
-        <v>3365</v>
+        <v>3364</v>
       </c>
       <c r="C3305" t="inlineStr">
         <is>
-          <t>CYNTIA RAFAELLA DE PONTES</t>
+          <t>CLOVIS VIDAL DOS SANTOS NETO</t>
         </is>
       </c>
       <c r="D3305" t="inlineStr">
         <is>
-          <t>CRPONTES</t>
+          <t>CVNETO</t>
         </is>
       </c>
     </row>
     <row r="3306">
       <c r="A3306" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3306" t="n">
-        <v>3387</v>
+        <v>3365</v>
       </c>
       <c r="C3306" t="inlineStr">
         <is>
-          <t>VALDECI NASCIMENTO DELGADO JUNIOR</t>
+          <t>CYNTIA RAFAELLA DE PONTES</t>
         </is>
       </c>
       <c r="D3306" t="inlineStr">
         <is>
-          <t>VALDECI05</t>
+          <t>CRPONTES</t>
         </is>
       </c>
     </row>
     <row r="3307">
       <c r="A3307" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3307" t="n">
-        <v>3458</v>
+        <v>3387</v>
       </c>
       <c r="C3307" t="inlineStr">
         <is>
-          <t>EDUARDO BEZERRA DE SOUSA</t>
+          <t>VALDECI NASCIMENTO DELGADO JUNIOR</t>
         </is>
       </c>
       <c r="D3307" t="inlineStr">
         <is>
-          <t>EDUARDOB</t>
+          <t>VALDECI05</t>
         </is>
       </c>
     </row>
     <row r="3308">
       <c r="A3308" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3308" t="n">
-        <v>940561</v>
+        <v>3458</v>
       </c>
       <c r="C3308" t="inlineStr">
         <is>
-          <t>NAIRTON DE ARAUJO MONTEIRO</t>
+          <t>EDUARDO BEZERRA DE SOUSA</t>
         </is>
       </c>
       <c r="D3308" t="inlineStr">
         <is>
-          <t>NAIRTON</t>
+          <t>EDUARDOB</t>
         </is>
       </c>
     </row>
     <row r="3309">
       <c r="A3309" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>99</t>
         </is>
       </c>
       <c r="B3309" t="n">
-        <v>3515</v>
+        <v>940561</v>
       </c>
       <c r="C3309" t="inlineStr">
         <is>
-          <t>DANIEL DOS SANTOS DE ALMEIDA</t>
+          <t>NAIRTON DE ARAUJO MONTEIRO</t>
         </is>
       </c>
       <c r="D3309" t="inlineStr">
         <is>
-          <t>DANIELSA</t>
+          <t>NAIRTON</t>
         </is>
       </c>
     </row>
     <row r="3310">
       <c r="A3310" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3310" t="n">
-        <v>3288</v>
+        <v>3515</v>
       </c>
       <c r="C3310" t="inlineStr">
         <is>
-          <t>ANA MARIA AMORIM MENDONÇA</t>
+          <t>DANIEL DOS SANTOS DE ALMEIDA</t>
         </is>
       </c>
       <c r="D3310" t="inlineStr">
         <is>
-          <t>AMENDONCA</t>
+          <t>DANIELSA</t>
         </is>
       </c>
     </row>
     <row r="3311">
       <c r="A3311" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3311" t="n">
-        <v>3312</v>
+        <v>3288</v>
       </c>
       <c r="C3311" t="inlineStr">
         <is>
-          <t>AURIANA LIMA DE MORAES</t>
+          <t>ANA MARIA AMORIM MENDONÇA</t>
         </is>
       </c>
       <c r="D3311" t="inlineStr">
         <is>
-          <t>ALM</t>
+          <t>AMENDONCA</t>
         </is>
       </c>
     </row>
     <row r="3312">
       <c r="A3312" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3312" t="n">
-        <v>940547</v>
+        <v>3312</v>
       </c>
       <c r="C3312" t="inlineStr">
         <is>
-          <t>JM EXPRESS - AGRESTE</t>
+          <t>AURIANA LIMA DE MORAES</t>
         </is>
       </c>
       <c r="D3312" t="inlineStr">
         <is>
-          <t>J M A</t>
+          <t>ALM</t>
         </is>
       </c>
     </row>
@@ -66678,76 +66678,76 @@
         </is>
       </c>
       <c r="B3313" t="n">
-        <v>940548</v>
+        <v>940547</v>
       </c>
       <c r="C3313" t="inlineStr">
         <is>
-          <t>JM EXPRESS - SERTAO</t>
+          <t>JM EXPRESS - AGRESTE</t>
         </is>
       </c>
       <c r="D3313" t="inlineStr">
         <is>
-          <t>J M S</t>
+          <t>J M A</t>
         </is>
       </c>
     </row>
     <row r="3314">
       <c r="A3314" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3314" t="n">
-        <v>940551</v>
+        <v>940548</v>
       </c>
       <c r="C3314" t="inlineStr">
         <is>
-          <t>LUCAS PONTES NOBRE</t>
+          <t>JM EXPRESS - SERTAO</t>
         </is>
       </c>
       <c r="D3314" t="inlineStr">
         <is>
-          <t>PONTES</t>
+          <t>J M S</t>
         </is>
       </c>
     </row>
     <row r="3315">
       <c r="A3315" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>99</t>
         </is>
       </c>
       <c r="B3315" t="n">
-        <v>3382</v>
+        <v>940551</v>
       </c>
       <c r="C3315" t="inlineStr">
         <is>
-          <t>MARIA CASSILANIA SOUSA DO NASCIMENTO</t>
+          <t>LUCAS PONTES NOBRE</t>
         </is>
       </c>
       <c r="D3315" t="inlineStr">
         <is>
-          <t>MCASSILANIA</t>
+          <t>PONTES</t>
         </is>
       </c>
     </row>
     <row r="3316">
       <c r="A3316" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3316" t="n">
-        <v>3474</v>
+        <v>3382</v>
       </c>
       <c r="C3316" t="inlineStr">
         <is>
-          <t>MARCOS VINICIUS GONCALVES MIRANDA</t>
+          <t>MARIA CASSILANIA SOUSA DO NASCIMENTO</t>
         </is>
       </c>
       <c r="D3316" t="inlineStr">
         <is>
-          <t>MARCOS.VINICIUS</t>
+          <t>MCASSILANIA</t>
         </is>
       </c>
     </row>
@@ -66758,136 +66758,136 @@
         </is>
       </c>
       <c r="B3317" t="n">
-        <v>3523</v>
+        <v>3474</v>
       </c>
       <c r="C3317" t="inlineStr">
         <is>
-          <t>ORLANDO RICARDO SANTOS ANDRADE</t>
+          <t>MARCOS VINICIUS GONCALVES MIRANDA</t>
         </is>
       </c>
       <c r="D3317" t="inlineStr">
         <is>
-          <t>ORLANDOR</t>
+          <t>MARCOS.VINICIUS</t>
         </is>
       </c>
     </row>
     <row r="3318">
       <c r="A3318" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3318" t="n">
-        <v>940541</v>
+        <v>3523</v>
       </c>
       <c r="C3318" t="inlineStr">
         <is>
-          <t>JOSE AMSTERDA TEIXEIRA DE MENEZES</t>
+          <t>ORLANDO RICARDO SANTOS ANDRADE</t>
         </is>
       </c>
       <c r="D3318" t="inlineStr">
         <is>
-          <t>AMSTERDA</t>
+          <t>ORLANDOR</t>
         </is>
       </c>
     </row>
     <row r="3319">
       <c r="A3319" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>99</t>
         </is>
       </c>
       <c r="B3319" t="n">
-        <v>940554</v>
+        <v>940541</v>
       </c>
       <c r="C3319" t="inlineStr">
         <is>
-          <t>ALEXANDRE ALVES DE FREITAS</t>
+          <t>JOSE AMSTERDA TEIXEIRA DE MENEZES</t>
         </is>
       </c>
       <c r="D3319" t="inlineStr">
         <is>
-          <t>ALEXANDRE</t>
+          <t>AMSTERDA</t>
         </is>
       </c>
     </row>
     <row r="3320">
       <c r="A3320" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3320" t="n">
-        <v>3402</v>
+        <v>940554</v>
       </c>
       <c r="C3320" t="inlineStr">
         <is>
-          <t xml:space="preserve">VINICIUS GUEDES DA SILVA </t>
+          <t>ALEXANDRE ALVES DE FREITAS</t>
         </is>
       </c>
       <c r="D3320" t="inlineStr">
         <is>
-          <t>GUEDES5</t>
+          <t>ALEXANDRE</t>
         </is>
       </c>
     </row>
     <row r="3321">
       <c r="A3321" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3321" t="n">
-        <v>3467</v>
+        <v>3402</v>
       </c>
       <c r="C3321" t="inlineStr">
         <is>
-          <t>CILENE FERREIRA DA SILVA</t>
+          <t xml:space="preserve">VINICIUS GUEDES DA SILVA </t>
         </is>
       </c>
       <c r="D3321" t="inlineStr">
         <is>
-          <t>CILENE</t>
+          <t>GUEDES5</t>
         </is>
       </c>
     </row>
     <row r="3322">
       <c r="A3322" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3322" t="n">
-        <v>3495</v>
+        <v>3467</v>
       </c>
       <c r="C3322" t="inlineStr">
         <is>
-          <t>LUCILENE SANTOS DE MELO DAMASCENA</t>
+          <t>CILENE FERREIRA DA SILVA</t>
         </is>
       </c>
       <c r="D3322" t="inlineStr">
         <is>
-          <t>LUCILENE21</t>
+          <t>CILENE</t>
         </is>
       </c>
     </row>
     <row r="3323">
       <c r="A3323" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3323" t="n">
-        <v>3496</v>
+        <v>3495</v>
       </c>
       <c r="C3323" t="inlineStr">
         <is>
-          <t>JOAO PEDRO HENRIQUE ALVES DE ARAUJO</t>
+          <t>LUCILENE SANTOS DE MELO DAMASCENA</t>
         </is>
       </c>
       <c r="D3323" t="inlineStr">
         <is>
-          <t>JOAO.PEDRO</t>
+          <t>LUCILENE21</t>
         </is>
       </c>
     </row>
@@ -66898,16 +66898,16 @@
         </is>
       </c>
       <c r="B3324" t="n">
-        <v>3497</v>
+        <v>3496</v>
       </c>
       <c r="C3324" t="inlineStr">
         <is>
-          <t>ORLANDO MONTEIRO DE AMORIM</t>
+          <t>JOAO PEDRO HENRIQUE ALVES DE ARAUJO</t>
         </is>
       </c>
       <c r="D3324" t="inlineStr">
         <is>
-          <t>ORLANDO</t>
+          <t>JOAO.PEDRO</t>
         </is>
       </c>
     </row>
@@ -66918,16 +66918,16 @@
         </is>
       </c>
       <c r="B3325" t="n">
-        <v>3538</v>
+        <v>3497</v>
       </c>
       <c r="C3325" t="inlineStr">
         <is>
-          <t>PAULO HENRIQUE BENTO DA SILVA</t>
+          <t>ORLANDO MONTEIRO DE AMORIM</t>
         </is>
       </c>
       <c r="D3325" t="inlineStr">
         <is>
-          <t>P.BENTO</t>
+          <t>ORLANDO</t>
         </is>
       </c>
     </row>
@@ -66938,96 +66938,96 @@
         </is>
       </c>
       <c r="B3326" t="n">
-        <v>3303</v>
+        <v>3538</v>
       </c>
       <c r="C3326" t="inlineStr">
         <is>
-          <t>DANIEL ALVES RODRIGUES</t>
+          <t>PAULO HENRIQUE BENTO DA SILVA</t>
         </is>
       </c>
       <c r="D3326" t="inlineStr">
         <is>
-          <t>DARODRIGUES</t>
+          <t>P.BENTO</t>
         </is>
       </c>
     </row>
     <row r="3327">
       <c r="A3327" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3327" t="n">
-        <v>3316</v>
+        <v>3303</v>
       </c>
       <c r="C3327" t="inlineStr">
         <is>
-          <t xml:space="preserve">MARCELO PEREIRA BASTOS </t>
+          <t>DANIEL ALVES RODRIGUES</t>
         </is>
       </c>
       <c r="D3327" t="inlineStr">
         <is>
-          <t>MBASTOS</t>
+          <t>DARODRIGUES</t>
         </is>
       </c>
     </row>
     <row r="3328">
       <c r="A3328" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3328" t="n">
-        <v>3366</v>
+        <v>3316</v>
       </c>
       <c r="C3328" t="inlineStr">
         <is>
-          <t>MATEUS TEIXEIRA DA PAZ SILVA</t>
+          <t xml:space="preserve">MARCELO PEREIRA BASTOS </t>
         </is>
       </c>
       <c r="D3328" t="inlineStr">
         <is>
-          <t>PAZSILVA</t>
+          <t>MBASTOS</t>
         </is>
       </c>
     </row>
     <row r="3329">
       <c r="A3329" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3329" t="n">
-        <v>3393</v>
+        <v>3366</v>
       </c>
       <c r="C3329" t="inlineStr">
         <is>
-          <t xml:space="preserve">DAVID LUCAS RIBEIRO DOS SANTOS </t>
+          <t>MATEUS TEIXEIRA DA PAZ SILVA</t>
         </is>
       </c>
       <c r="D3329" t="inlineStr">
         <is>
-          <t>DLUCAS</t>
+          <t>PAZSILVA</t>
         </is>
       </c>
     </row>
     <row r="3330">
       <c r="A3330" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3330" t="n">
-        <v>3420</v>
+        <v>3393</v>
       </c>
       <c r="C3330" t="inlineStr">
         <is>
-          <t xml:space="preserve">CLAUDIO ROBERTO SILVA SOUZA </t>
+          <t xml:space="preserve">DAVID LUCAS RIBEIRO DOS SANTOS </t>
         </is>
       </c>
       <c r="D3330" t="inlineStr">
         <is>
-          <t>CLAUDIO21</t>
+          <t>DLUCAS</t>
         </is>
       </c>
     </row>
@@ -67038,16 +67038,16 @@
         </is>
       </c>
       <c r="B3331" t="n">
-        <v>3421</v>
+        <v>3420</v>
       </c>
       <c r="C3331" t="inlineStr">
         <is>
-          <t>WILSON PORTUGAL AZEVEDO FILHO</t>
+          <t xml:space="preserve">CLAUDIO ROBERTO SILVA SOUZA </t>
         </is>
       </c>
       <c r="D3331" t="inlineStr">
         <is>
-          <t>WILSONF</t>
+          <t>CLAUDIO21</t>
         </is>
       </c>
     </row>
@@ -67058,156 +67058,156 @@
         </is>
       </c>
       <c r="B3332" t="n">
-        <v>3439</v>
+        <v>3421</v>
       </c>
       <c r="C3332" t="inlineStr">
         <is>
-          <t>FERNANDA MASCARENHAS CEDRAZ</t>
+          <t>WILSON PORTUGAL AZEVEDO FILHO</t>
         </is>
       </c>
       <c r="D3332" t="inlineStr">
         <is>
-          <t>FERNANDAM</t>
+          <t>WILSONF</t>
         </is>
       </c>
     </row>
     <row r="3333">
       <c r="A3333" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3333" t="n">
-        <v>3455</v>
+        <v>3439</v>
       </c>
       <c r="C3333" t="inlineStr">
         <is>
-          <t xml:space="preserve">MARDONIO CUNHA BASILIO </t>
+          <t>FERNANDA MASCARENHAS CEDRAZ</t>
         </is>
       </c>
       <c r="D3333" t="inlineStr">
         <is>
-          <t>MARDONIO1</t>
+          <t>FERNANDAM</t>
         </is>
       </c>
     </row>
     <row r="3334">
       <c r="A3334" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3334" t="n">
-        <v>3508</v>
+        <v>3455</v>
       </c>
       <c r="C3334" t="inlineStr">
         <is>
-          <t>REBECA PIRES DE SOUZA MELO</t>
+          <t xml:space="preserve">MARDONIO CUNHA BASILIO </t>
         </is>
       </c>
       <c r="D3334" t="inlineStr">
         <is>
-          <t>RPMELO</t>
+          <t>MARDONIO1</t>
         </is>
       </c>
     </row>
     <row r="3335">
       <c r="A3335" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3335" t="n">
-        <v>3543</v>
+        <v>3508</v>
       </c>
       <c r="C3335" t="inlineStr">
         <is>
-          <t>JOAO GABRIEL BARBOSA FIRMINO</t>
+          <t>REBECA PIRES DE SOUZA MELO</t>
         </is>
       </c>
       <c r="D3335" t="inlineStr">
         <is>
-          <t>JOAOG</t>
+          <t>RPMELO</t>
         </is>
       </c>
     </row>
     <row r="3336">
       <c r="A3336" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3336" t="n">
-        <v>3351</v>
+        <v>3543</v>
       </c>
       <c r="C3336" t="inlineStr">
         <is>
-          <t>HAWLLYSON DA SILVA COUTINHO</t>
+          <t>JOAO GABRIEL BARBOSA FIRMINO</t>
         </is>
       </c>
       <c r="D3336" t="inlineStr">
         <is>
-          <t>HCOUTINHO</t>
+          <t>JOAOG</t>
         </is>
       </c>
     </row>
     <row r="3337">
       <c r="A3337" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3337" t="n">
-        <v>940553</v>
+        <v>3351</v>
       </c>
       <c r="C3337" t="inlineStr">
         <is>
-          <t>LUTY TRANSPORTES- BA</t>
+          <t>HAWLLYSON DA SILVA COUTINHO</t>
         </is>
       </c>
       <c r="D3337" t="inlineStr">
         <is>
-          <t>LUTY TRANSPORTE</t>
+          <t>HCOUTINHO</t>
         </is>
       </c>
     </row>
     <row r="3338">
       <c r="A3338" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3338" t="n">
-        <v>3391</v>
+        <v>940553</v>
       </c>
       <c r="C3338" t="inlineStr">
         <is>
-          <t xml:space="preserve">NIKSON DA SILVA ALVES </t>
+          <t>LUTY TRANSPORTES- BA</t>
         </is>
       </c>
       <c r="D3338" t="inlineStr">
         <is>
-          <t>NIKSON</t>
+          <t>LUTY TRANSPORTE</t>
         </is>
       </c>
     </row>
     <row r="3339">
       <c r="A3339" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3339" t="n">
-        <v>3397</v>
+        <v>3391</v>
       </c>
       <c r="C3339" t="inlineStr">
         <is>
-          <t>EDILANE MENESES BALTAZAR</t>
+          <t xml:space="preserve">NIKSON DA SILVA ALVES </t>
         </is>
       </c>
       <c r="D3339" t="inlineStr">
         <is>
-          <t>EDILANE</t>
+          <t>NIKSON</t>
         </is>
       </c>
     </row>
@@ -67218,56 +67218,56 @@
         </is>
       </c>
       <c r="B3340" t="n">
-        <v>3398</v>
+        <v>3397</v>
       </c>
       <c r="C3340" t="inlineStr">
         <is>
-          <t>LUANA MARIA ROSIO DA SILVA</t>
+          <t>EDILANE MENESES BALTAZAR</t>
         </is>
       </c>
       <c r="D3340" t="inlineStr">
         <is>
-          <t>LUMARIA</t>
+          <t>EDILANE</t>
         </is>
       </c>
     </row>
     <row r="3341">
       <c r="A3341" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3341" t="n">
-        <v>3400</v>
+        <v>3398</v>
       </c>
       <c r="C3341" t="inlineStr">
         <is>
-          <t>ELILTON PINTO ROMEU</t>
+          <t>LUANA MARIA ROSIO DA SILVA</t>
         </is>
       </c>
       <c r="D3341" t="inlineStr">
         <is>
-          <t>ELILTON</t>
+          <t>LUMARIA</t>
         </is>
       </c>
     </row>
     <row r="3342">
       <c r="A3342" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3342" t="n">
-        <v>3406</v>
+        <v>3400</v>
       </c>
       <c r="C3342" t="inlineStr">
         <is>
-          <t>CONEXAO ALDA</t>
+          <t>ELILTON PINTO ROMEU</t>
         </is>
       </c>
       <c r="D3342" t="inlineStr">
         <is>
-          <t>CONEXAOALDA</t>
+          <t>ELILTON</t>
         </is>
       </c>
     </row>
@@ -67278,136 +67278,136 @@
         </is>
       </c>
       <c r="B3343" t="n">
-        <v>3407</v>
+        <v>3406</v>
       </c>
       <c r="C3343" t="inlineStr">
         <is>
-          <t>CONEXAO IRACEMA</t>
+          <t>CONEXAO ALDA</t>
         </is>
       </c>
       <c r="D3343" t="inlineStr">
         <is>
-          <t>CONEXAOIRACEMA</t>
+          <t>CONEXAOALDA</t>
         </is>
       </c>
     </row>
     <row r="3344">
       <c r="A3344" t="inlineStr">
         <is>
-          <t>9999</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3344" t="n">
-        <v>3408</v>
+        <v>3407</v>
       </c>
       <c r="C3344" t="inlineStr">
         <is>
-          <t>CONEXAO TAMILES</t>
+          <t>CONEXAO IRACEMA</t>
         </is>
       </c>
       <c r="D3344" t="inlineStr">
         <is>
-          <t>CONEXAOTAMILES</t>
+          <t>CONEXAOIRACEMA</t>
         </is>
       </c>
     </row>
     <row r="3345">
       <c r="A3345" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>9999</t>
         </is>
       </c>
       <c r="B3345" t="n">
-        <v>3414</v>
+        <v>3408</v>
       </c>
       <c r="C3345" t="inlineStr">
         <is>
-          <t>CONEXAO ADM PI MA</t>
+          <t>CONEXAO TAMILES</t>
         </is>
       </c>
       <c r="D3345" t="inlineStr">
         <is>
-          <t>CONEXAOPIMA</t>
+          <t>CONEXAOTAMILES</t>
         </is>
       </c>
     </row>
     <row r="3346">
       <c r="A3346" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3346" t="n">
-        <v>3524</v>
+        <v>3414</v>
       </c>
       <c r="C3346" t="inlineStr">
         <is>
-          <t>LUIS FELIPE DA SILVA SOUSA</t>
+          <t>CONEXAO ADM PI MA</t>
         </is>
       </c>
       <c r="D3346" t="inlineStr">
         <is>
-          <t>L.FELIPE</t>
+          <t>CONEXAOPIMA</t>
         </is>
       </c>
     </row>
     <row r="3347">
       <c r="A3347" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3347" t="n">
-        <v>3531</v>
+        <v>3524</v>
       </c>
       <c r="C3347" t="inlineStr">
         <is>
-          <t>LEICIANE COELHO SILVA</t>
+          <t>LUIS FELIPE DA SILVA SOUSA</t>
         </is>
       </c>
       <c r="D3347" t="inlineStr">
         <is>
-          <t>LEI.SILVA</t>
+          <t>L.FELIPE</t>
         </is>
       </c>
     </row>
     <row r="3348">
       <c r="A3348" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3348" t="n">
-        <v>3550</v>
+        <v>3531</v>
       </c>
       <c r="C3348" t="inlineStr">
         <is>
-          <t>IARGO GABRIEL SANTOS DE OLIVEIRA</t>
+          <t>LEICIANE COELHO SILVA</t>
         </is>
       </c>
       <c r="D3348" t="inlineStr">
         <is>
-          <t>IARGOG</t>
+          <t>LEI.SILVA</t>
         </is>
       </c>
     </row>
     <row r="3349">
       <c r="A3349" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3349" t="n">
-        <v>3355</v>
+        <v>3550</v>
       </c>
       <c r="C3349" t="inlineStr">
         <is>
-          <t>HUGO MATHEUS DA COSTA FEITOSA</t>
+          <t>IARGO GABRIEL SANTOS DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D3349" t="inlineStr">
         <is>
-          <t>HMFEITOSA</t>
+          <t>IARGOG</t>
         </is>
       </c>
     </row>
@@ -67418,96 +67418,96 @@
         </is>
       </c>
       <c r="B3350" t="n">
-        <v>3356</v>
+        <v>3355</v>
       </c>
       <c r="C3350" t="inlineStr">
         <is>
-          <t>BRENDA LIMA DE OLIVEIRA CUNHA</t>
+          <t>HUGO MATHEUS DA COSTA FEITOSA</t>
         </is>
       </c>
       <c r="D3350" t="inlineStr">
         <is>
-          <t>BLCUNHA</t>
+          <t>HMFEITOSA</t>
         </is>
       </c>
     </row>
     <row r="3351">
       <c r="A3351" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3351" t="n">
-        <v>3361</v>
+        <v>3356</v>
       </c>
       <c r="C3351" t="inlineStr">
         <is>
-          <t>WLADIA DE ARAUJO BASTOS</t>
+          <t>BRENDA LIMA DE OLIVEIRA CUNHA</t>
         </is>
       </c>
       <c r="D3351" t="inlineStr">
         <is>
-          <t>WABASTOS</t>
+          <t>BLCUNHA</t>
         </is>
       </c>
     </row>
     <row r="3352">
       <c r="A3352" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3352" t="n">
-        <v>3362</v>
+        <v>3361</v>
       </c>
       <c r="C3352" t="inlineStr">
         <is>
-          <t>CARLOS HENRIQUE MELO DA SILVA</t>
+          <t>WLADIA DE ARAUJO BASTOS</t>
         </is>
       </c>
       <c r="D3352" t="inlineStr">
         <is>
-          <t>CHMELO</t>
+          <t>WABASTOS</t>
         </is>
       </c>
     </row>
     <row r="3353">
       <c r="A3353" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3353" t="n">
-        <v>3375</v>
+        <v>3362</v>
       </c>
       <c r="C3353" t="inlineStr">
         <is>
-          <t>AFONSO DE SOUSA RAMOS FILHO</t>
+          <t>CARLOS HENRIQUE MELO DA SILVA</t>
         </is>
       </c>
       <c r="D3353" t="inlineStr">
         <is>
-          <t>AFILHO</t>
+          <t>CHMELO</t>
         </is>
       </c>
     </row>
     <row r="3354">
       <c r="A3354" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3354" t="n">
-        <v>3404</v>
+        <v>3375</v>
       </c>
       <c r="C3354" t="inlineStr">
         <is>
-          <t>NOVATO 4 COM</t>
+          <t>AFONSO DE SOUSA RAMOS FILHO</t>
         </is>
       </c>
       <c r="D3354" t="inlineStr">
         <is>
-          <t>NOVATO4COM</t>
+          <t>AFILHO</t>
         </is>
       </c>
     </row>
@@ -67518,156 +67518,156 @@
         </is>
       </c>
       <c r="B3355" t="n">
-        <v>3405</v>
+        <v>3404</v>
       </c>
       <c r="C3355" t="inlineStr">
         <is>
-          <t>NOVATO 5 COM</t>
+          <t>NOVATO 4 COM</t>
         </is>
       </c>
       <c r="D3355" t="inlineStr">
         <is>
-          <t>NOVATO5COM</t>
+          <t>NOVATO4COM</t>
         </is>
       </c>
     </row>
     <row r="3356">
       <c r="A3356" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3356" t="n">
-        <v>3447</v>
+        <v>3405</v>
       </c>
       <c r="C3356" t="inlineStr">
         <is>
-          <t>RAYSSA KEYCE LINHARES AQUINO</t>
+          <t>NOVATO 5 COM</t>
         </is>
       </c>
       <c r="D3356" t="inlineStr">
         <is>
-          <t>RAYSSAK</t>
+          <t>NOVATO5COM</t>
         </is>
       </c>
     </row>
     <row r="3357">
       <c r="A3357" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3357" t="n">
-        <v>940559</v>
+        <v>3447</v>
       </c>
       <c r="C3357" t="inlineStr">
         <is>
-          <t>WALLEF DE OLIVEIRA</t>
+          <t>RAYSSA KEYCE LINHARES AQUINO</t>
         </is>
       </c>
       <c r="D3357" t="inlineStr">
         <is>
-          <t>WALLEF</t>
+          <t>RAYSSAK</t>
         </is>
       </c>
     </row>
     <row r="3358">
       <c r="A3358" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>99</t>
         </is>
       </c>
       <c r="B3358" t="n">
-        <v>3489</v>
+        <v>940559</v>
       </c>
       <c r="C3358" t="inlineStr">
         <is>
-          <t>MARCELA KARINA PEREIRA VELOSO</t>
+          <t>WALLEF DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D3358" t="inlineStr">
         <is>
-          <t>MKARINA</t>
+          <t>WALLEF</t>
         </is>
       </c>
     </row>
     <row r="3359">
       <c r="A3359" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3359" t="n">
-        <v>3490</v>
+        <v>3489</v>
       </c>
       <c r="C3359" t="inlineStr">
         <is>
-          <t>JOSE MAILSON GOMES NUNES</t>
+          <t>MARCELA KARINA PEREIRA VELOSO</t>
         </is>
       </c>
       <c r="D3359" t="inlineStr">
         <is>
-          <t>J.MAILSON</t>
+          <t>MKARINA</t>
         </is>
       </c>
     </row>
     <row r="3360">
       <c r="A3360" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3360" t="n">
-        <v>3537</v>
+        <v>3490</v>
       </c>
       <c r="C3360" t="inlineStr">
         <is>
-          <t>ALDAIR PEDRO DA SILVA</t>
+          <t>JOSE MAILSON GOMES NUNES</t>
         </is>
       </c>
       <c r="D3360" t="inlineStr">
         <is>
-          <t>A.PEDRO</t>
+          <t>J.MAILSON</t>
         </is>
       </c>
     </row>
     <row r="3361">
       <c r="A3361" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3361" t="n">
-        <v>3549</v>
+        <v>3537</v>
       </c>
       <c r="C3361" t="inlineStr">
         <is>
-          <t xml:space="preserve">FERNANDA CAROLINE E CESAR SOUSA </t>
+          <t>ALDAIR PEDRO DA SILVA</t>
         </is>
       </c>
       <c r="D3361" t="inlineStr">
         <is>
-          <t>FCAROLINE</t>
+          <t>A.PEDRO</t>
         </is>
       </c>
     </row>
     <row r="3362">
       <c r="A3362" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3362" t="n">
-        <v>3337</v>
+        <v>3549</v>
       </c>
       <c r="C3362" t="inlineStr">
         <is>
-          <t>WESLEY FONTES DE ALMEIDA</t>
+          <t xml:space="preserve">FERNANDA CAROLINE E CESAR SOUSA </t>
         </is>
       </c>
       <c r="D3362" t="inlineStr">
         <is>
-          <t>WFALMEIDA</t>
+          <t>FCAROLINE</t>
         </is>
       </c>
     </row>
@@ -67678,16 +67678,16 @@
         </is>
       </c>
       <c r="B3363" t="n">
-        <v>3338</v>
+        <v>3337</v>
       </c>
       <c r="C3363" t="inlineStr">
         <is>
-          <t>FRANCISCA SAMARA MENDES DE OLIVEIRA C</t>
+          <t>WESLEY FONTES DE ALMEIDA</t>
         </is>
       </c>
       <c r="D3363" t="inlineStr">
         <is>
-          <t>FSCUNHA</t>
+          <t>WFALMEIDA</t>
         </is>
       </c>
     </row>
@@ -67698,176 +67698,176 @@
         </is>
       </c>
       <c r="B3364" t="n">
-        <v>3339</v>
+        <v>3338</v>
       </c>
       <c r="C3364" t="inlineStr">
         <is>
-          <t>MAYARA THALYA DIAS DE ANDRADE</t>
+          <t>FRANCISCA SAMARA MENDES DE OLIVEIRA C</t>
         </is>
       </c>
       <c r="D3364" t="inlineStr">
         <is>
-          <t>MTANDRADE</t>
+          <t>FSCUNHA</t>
         </is>
       </c>
     </row>
     <row r="3365">
       <c r="A3365" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3365" t="n">
-        <v>3359</v>
+        <v>3339</v>
       </c>
       <c r="C3365" t="inlineStr">
         <is>
-          <t xml:space="preserve">EVANESSA DA SILVA E SILVA </t>
+          <t>MAYARA THALYA DIAS DE ANDRADE</t>
         </is>
       </c>
       <c r="D3365" t="inlineStr">
         <is>
-          <t>EVANESSAS</t>
+          <t>MTANDRADE</t>
         </is>
       </c>
     </row>
     <row r="3366">
       <c r="A3366" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3366" t="n">
-        <v>3360</v>
+        <v>3359</v>
       </c>
       <c r="C3366" t="inlineStr">
         <is>
-          <t>THIAGO DE CARVALHO ARAUJO</t>
+          <t xml:space="preserve">EVANESSA DA SILVA E SILVA </t>
         </is>
       </c>
       <c r="D3366" t="inlineStr">
         <is>
-          <t>TCARAUJO</t>
+          <t>EVANESSAS</t>
         </is>
       </c>
     </row>
     <row r="3367">
       <c r="A3367" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3367" t="n">
-        <v>3481</v>
+        <v>3360</v>
       </c>
       <c r="C3367" t="inlineStr">
         <is>
-          <t xml:space="preserve">EDSON DA PAZ LIMA </t>
+          <t>THIAGO DE CARVALHO ARAUJO</t>
         </is>
       </c>
       <c r="D3367" t="inlineStr">
         <is>
-          <t>EDPAZ</t>
+          <t>TCARAUJO</t>
         </is>
       </c>
     </row>
     <row r="3368">
       <c r="A3368" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3368" t="n">
-        <v>3494</v>
+        <v>3481</v>
       </c>
       <c r="C3368" t="inlineStr">
         <is>
-          <t>ANTONIO CRISTINA BRITO GOMES</t>
+          <t xml:space="preserve">EDSON DA PAZ LIMA </t>
         </is>
       </c>
       <c r="D3368" t="inlineStr">
         <is>
-          <t>CRIS.GOMES</t>
+          <t>EDPAZ</t>
         </is>
       </c>
     </row>
     <row r="3369">
       <c r="A3369" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3369" t="n">
-        <v>3498</v>
+        <v>3494</v>
       </c>
       <c r="C3369" t="inlineStr">
         <is>
-          <t>SILVESTRA COSTA NUNES</t>
+          <t>ANTONIO CRISTINA BRITO GOMES</t>
         </is>
       </c>
       <c r="D3369" t="inlineStr">
         <is>
-          <t>SCNUNES</t>
+          <t>CRIS.GOMES</t>
         </is>
       </c>
     </row>
     <row r="3370">
       <c r="A3370" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3370" t="n">
-        <v>940562</v>
+        <v>3498</v>
       </c>
       <c r="C3370" t="inlineStr">
         <is>
-          <t>FRANCISCO DAVID ASSUNCAO ALVES</t>
+          <t>SILVESTRA COSTA NUNES</t>
         </is>
       </c>
       <c r="D3370" t="inlineStr">
         <is>
-          <t>ASSUNÇÃO</t>
+          <t>SCNUNES</t>
         </is>
       </c>
     </row>
     <row r="3371">
       <c r="A3371" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>99</t>
         </is>
       </c>
       <c r="B3371" t="n">
-        <v>3513</v>
+        <v>940562</v>
       </c>
       <c r="C3371" t="inlineStr">
         <is>
-          <t>RENARA ANDRADE MATIAS</t>
+          <t>FRANCISCO DAVID ASSUNCAO ALVES</t>
         </is>
       </c>
       <c r="D3371" t="inlineStr">
         <is>
-          <t>R.ANDRADE</t>
+          <t>ASSUNÇÃO</t>
         </is>
       </c>
     </row>
     <row r="3372">
       <c r="A3372" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3372" t="n">
-        <v>3275</v>
+        <v>3513</v>
       </c>
       <c r="C3372" t="inlineStr">
         <is>
-          <t>MARIA APARECIDA COELHO SILVA</t>
+          <t>RENARA ANDRADE MATIAS</t>
         </is>
       </c>
       <c r="D3372" t="inlineStr">
         <is>
-          <t>MCOELHO</t>
+          <t>R.ANDRADE</t>
         </is>
       </c>
     </row>
@@ -67878,116 +67878,116 @@
         </is>
       </c>
       <c r="B3373" t="n">
-        <v>3276</v>
+        <v>3275</v>
       </c>
       <c r="C3373" t="inlineStr">
         <is>
-          <t xml:space="preserve">PEROLA DE JESUS AMORIM SOUSA </t>
+          <t>MARIA APARECIDA COELHO SILVA</t>
         </is>
       </c>
       <c r="D3373" t="inlineStr">
         <is>
-          <t>PJESUS</t>
+          <t>MCOELHO</t>
         </is>
       </c>
     </row>
     <row r="3374">
       <c r="A3374" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3374" t="n">
-        <v>3526</v>
+        <v>3276</v>
       </c>
       <c r="C3374" t="inlineStr">
         <is>
-          <t>JOYCE NAZARE CORREA</t>
+          <t xml:space="preserve">PEROLA DE JESUS AMORIM SOUSA </t>
         </is>
       </c>
       <c r="D3374" t="inlineStr">
         <is>
-          <t>J.NAZARE</t>
+          <t>PJESUS</t>
         </is>
       </c>
     </row>
     <row r="3375">
       <c r="A3375" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3375" t="n">
-        <v>3527</v>
+        <v>3526</v>
       </c>
       <c r="C3375" t="inlineStr">
         <is>
-          <t>GILVANA DA SILVA MONTELES</t>
+          <t>JOYCE NAZARE CORREA</t>
         </is>
       </c>
       <c r="D3375" t="inlineStr">
         <is>
-          <t>GIL.SILVA</t>
+          <t>J.NAZARE</t>
         </is>
       </c>
     </row>
     <row r="3376">
       <c r="A3376" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3376" t="n">
-        <v>3548</v>
+        <v>3527</v>
       </c>
       <c r="C3376" t="inlineStr">
         <is>
-          <t>JAMILLY MARIA HENRIQUE ARAUJO</t>
+          <t>GILVANA DA SILVA MONTELES</t>
         </is>
       </c>
       <c r="D3376" t="inlineStr">
         <is>
-          <t>JAMILLY</t>
+          <t>GIL.SILVA</t>
         </is>
       </c>
     </row>
     <row r="3377">
       <c r="A3377" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3377" t="n">
-        <v>3551</v>
+        <v>3548</v>
       </c>
       <c r="C3377" t="inlineStr">
         <is>
-          <t xml:space="preserve">VITOR MANOEL DA SILVA BARBOSA </t>
+          <t>JAMILLY MARIA HENRIQUE ARAUJO</t>
         </is>
       </c>
       <c r="D3377" t="inlineStr">
         <is>
-          <t>VMANOEL</t>
+          <t>JAMILLY</t>
         </is>
       </c>
     </row>
     <row r="3378">
       <c r="A3378" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3378" t="n">
-        <v>940525</v>
+        <v>3551</v>
       </c>
       <c r="C3378" t="inlineStr">
         <is>
-          <t>SANDUWELLINGTON</t>
+          <t xml:space="preserve">VITOR MANOEL DA SILVA BARBOSA </t>
         </is>
       </c>
       <c r="D3378" t="inlineStr">
         <is>
-          <t>SANDUWELLINGTON</t>
+          <t>VMANOEL</t>
         </is>
       </c>
     </row>
@@ -67998,36 +67998,36 @@
         </is>
       </c>
       <c r="B3379" t="n">
-        <v>3369</v>
+        <v>940525</v>
       </c>
       <c r="C3379" t="inlineStr">
         <is>
-          <t xml:space="preserve">PRISCILA DOS SANTOS LOPES </t>
+          <t>SANDUWELLINGTON</t>
         </is>
       </c>
       <c r="D3379" t="inlineStr">
         <is>
-          <t>PSLOPES</t>
+          <t>SANDUWELLINGTON</t>
         </is>
       </c>
     </row>
     <row r="3380">
       <c r="A3380" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3380" t="n">
-        <v>3433</v>
+        <v>3369</v>
       </c>
       <c r="C3380" t="inlineStr">
         <is>
-          <t>BRUNO NUNES CRUZ</t>
+          <t xml:space="preserve">PRISCILA DOS SANTOS LOPES </t>
         </is>
       </c>
       <c r="D3380" t="inlineStr">
         <is>
-          <t>BRUNOCRUZ</t>
+          <t>PSLOPES</t>
         </is>
       </c>
     </row>
@@ -68038,36 +68038,36 @@
         </is>
       </c>
       <c r="B3381" t="n">
-        <v>3434</v>
+        <v>3433</v>
       </c>
       <c r="C3381" t="inlineStr">
         <is>
-          <t>ANA TERCIA DE LIMA SA CARVALHO SERAFIM</t>
+          <t>BRUNO NUNES CRUZ</t>
         </is>
       </c>
       <c r="D3381" t="inlineStr">
         <is>
-          <t>ANATER</t>
+          <t>BRUNOCRUZ</t>
         </is>
       </c>
     </row>
     <row r="3382">
       <c r="A3382" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3382" t="n">
-        <v>3502</v>
+        <v>3434</v>
       </c>
       <c r="C3382" t="inlineStr">
         <is>
-          <t>LUIZ FELIPE MACHADO BARRETO</t>
+          <t>ANA TERCIA DE LIMA SA CARVALHO SERAFIM</t>
         </is>
       </c>
       <c r="D3382" t="inlineStr">
         <is>
-          <t>LUIZ.FELIPE</t>
+          <t>ANATER</t>
         </is>
       </c>
     </row>
@@ -68078,36 +68078,36 @@
         </is>
       </c>
       <c r="B3383" t="n">
-        <v>3503</v>
+        <v>3502</v>
       </c>
       <c r="C3383" t="inlineStr">
         <is>
-          <t>FABIO OLIVEIRA SILVA</t>
+          <t>LUIZ FELIPE MACHADO BARRETO</t>
         </is>
       </c>
       <c r="D3383" t="inlineStr">
         <is>
-          <t>FOSILVA</t>
+          <t>LUIZ.FELIPE</t>
         </is>
       </c>
     </row>
     <row r="3384">
       <c r="A3384" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3384" t="n">
-        <v>940549</v>
+        <v>3503</v>
       </c>
       <c r="C3384" t="inlineStr">
         <is>
-          <t>EDILSON ARAUJO - FL9</t>
+          <t>FABIO OLIVEIRA SILVA</t>
         </is>
       </c>
       <c r="D3384" t="inlineStr">
         <is>
-          <t>EDILSON</t>
+          <t>FOSILVA</t>
         </is>
       </c>
     </row>
@@ -68118,36 +68118,36 @@
         </is>
       </c>
       <c r="B3385" t="n">
-        <v>3470</v>
+        <v>940549</v>
       </c>
       <c r="C3385" t="inlineStr">
         <is>
-          <t>DEBORA ALVES CARVALHO</t>
+          <t>EDILSON ARAUJO - FL9</t>
         </is>
       </c>
       <c r="D3385" t="inlineStr">
         <is>
-          <t>DEBORA.ALVES</t>
+          <t>EDILSON</t>
         </is>
       </c>
     </row>
     <row r="3386">
       <c r="A3386" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3386" t="n">
-        <v>3510</v>
+        <v>3470</v>
       </c>
       <c r="C3386" t="inlineStr">
         <is>
-          <t>CAMILA RODIGUES PINTO</t>
+          <t>DEBORA ALVES CARVALHO</t>
         </is>
       </c>
       <c r="D3386" t="inlineStr">
         <is>
-          <t>MILA.PINTO</t>
+          <t>DEBORA.ALVES</t>
         </is>
       </c>
     </row>
@@ -68158,56 +68158,56 @@
         </is>
       </c>
       <c r="B3387" t="n">
-        <v>3511</v>
+        <v>3510</v>
       </c>
       <c r="C3387" t="inlineStr">
         <is>
-          <t>JORGE HENRIQUE DOS SANTOS RODRIGUES</t>
+          <t>CAMILA RODIGUES PINTO</t>
         </is>
       </c>
       <c r="D3387" t="inlineStr">
         <is>
-          <t>J.HENRIQUE</t>
+          <t>MILA.PINTO</t>
         </is>
       </c>
     </row>
     <row r="3388">
       <c r="A3388" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3388" t="n">
-        <v>3270</v>
+        <v>3511</v>
       </c>
       <c r="C3388" t="inlineStr">
         <is>
-          <t>ITANA NASCIMENTO SIMOES</t>
+          <t>JORGE HENRIQUE DOS SANTOS RODRIGUES</t>
         </is>
       </c>
       <c r="D3388" t="inlineStr">
         <is>
-          <t>ISIMOES</t>
+          <t>J.HENRIQUE</t>
         </is>
       </c>
     </row>
     <row r="3389">
       <c r="A3389" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3389" t="n">
-        <v>3318</v>
+        <v>3270</v>
       </c>
       <c r="C3389" t="inlineStr">
         <is>
-          <t>LUAN MONTEIRO COSTA</t>
+          <t>ITANA NASCIMENTO SIMOES</t>
         </is>
       </c>
       <c r="D3389" t="inlineStr">
         <is>
-          <t>LMONTEIRO</t>
+          <t>ISIMOES</t>
         </is>
       </c>
     </row>
@@ -68218,36 +68218,36 @@
         </is>
       </c>
       <c r="B3390" t="n">
-        <v>3319</v>
+        <v>3318</v>
       </c>
       <c r="C3390" t="inlineStr">
         <is>
-          <t>MARIANA MACEDA DOS SANTOS</t>
+          <t>LUAN MONTEIRO COSTA</t>
         </is>
       </c>
       <c r="D3390" t="inlineStr">
         <is>
-          <t>MMACEDA</t>
+          <t>LMONTEIRO</t>
         </is>
       </c>
     </row>
     <row r="3391">
       <c r="A3391" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3391" t="n">
-        <v>3389</v>
+        <v>3319</v>
       </c>
       <c r="C3391" t="inlineStr">
         <is>
-          <t>TAMILES DE SANTANA AMORIM BISPO</t>
+          <t>MARIANA MACEDA DOS SANTOS</t>
         </is>
       </c>
       <c r="D3391" t="inlineStr">
         <is>
-          <t>TAMILES</t>
+          <t>MMACEDA</t>
         </is>
       </c>
     </row>
@@ -68258,36 +68258,36 @@
         </is>
       </c>
       <c r="B3392" t="n">
-        <v>3390</v>
+        <v>3389</v>
       </c>
       <c r="C3392" t="inlineStr">
         <is>
-          <t>IRACEMA DE ALMEIDA MOURA</t>
+          <t>TAMILES DE SANTANA AMORIM BISPO</t>
         </is>
       </c>
       <c r="D3392" t="inlineStr">
         <is>
-          <t>IRACEMA</t>
+          <t>TAMILES</t>
         </is>
       </c>
     </row>
     <row r="3393">
       <c r="A3393" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3393" t="n">
-        <v>3286</v>
+        <v>3390</v>
       </c>
       <c r="C3393" t="inlineStr">
         <is>
-          <t>VALERIA MAIA DA SILVA</t>
+          <t>IRACEMA DE ALMEIDA MOURA</t>
         </is>
       </c>
       <c r="D3393" t="inlineStr">
         <is>
-          <t>VMAIAS</t>
+          <t>IRACEMA</t>
         </is>
       </c>
     </row>
@@ -68298,156 +68298,156 @@
         </is>
       </c>
       <c r="B3394" t="n">
-        <v>3287</v>
+        <v>3286</v>
       </c>
       <c r="C3394" t="inlineStr">
         <is>
-          <t>ERIVELTON DA SILVA OLIVEIRA</t>
+          <t>VALERIA MAIA DA SILVA</t>
         </is>
       </c>
       <c r="D3394" t="inlineStr">
         <is>
-          <t>ESOLIVEIRA</t>
+          <t>VMAIAS</t>
         </is>
       </c>
     </row>
     <row r="3395">
       <c r="A3395" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3395" t="n">
-        <v>3307</v>
+        <v>3287</v>
       </c>
       <c r="C3395" t="inlineStr">
         <is>
-          <t>ADRIEL XERES BARROS MARTINS</t>
+          <t>ERIVELTON DA SILVA OLIVEIRA</t>
         </is>
       </c>
       <c r="D3395" t="inlineStr">
         <is>
-          <t>AXERES</t>
+          <t>ESOLIVEIRA</t>
         </is>
       </c>
     </row>
     <row r="3396">
       <c r="A3396" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3396" t="n">
-        <v>3308</v>
+        <v>3307</v>
       </c>
       <c r="C3396" t="inlineStr">
         <is>
-          <t>ELKZIEL JUVINO DA SILVA</t>
+          <t>ADRIEL XERES BARROS MARTINS</t>
         </is>
       </c>
       <c r="D3396" t="inlineStr">
         <is>
-          <t>EJUVINO</t>
+          <t>AXERES</t>
         </is>
       </c>
     </row>
     <row r="3397">
       <c r="A3397" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3397" t="n">
-        <v>940539</v>
+        <v>3308</v>
       </c>
       <c r="C3397" t="inlineStr">
         <is>
-          <t>EDSON ARAUJO - FL9</t>
+          <t>ELKZIEL JUVINO DA SILVA</t>
         </is>
       </c>
       <c r="D3397" t="inlineStr">
         <is>
-          <t>EDS</t>
+          <t>EJUVINO</t>
         </is>
       </c>
     </row>
     <row r="3398">
       <c r="A3398" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3398" t="n">
-        <v>940540</v>
+        <v>940539</v>
       </c>
       <c r="C3398" t="inlineStr">
         <is>
-          <t>EDSON ARAUJO - FL8</t>
+          <t>EDSON ARAUJO - FL9</t>
         </is>
       </c>
       <c r="D3398" t="inlineStr">
         <is>
-          <t>EDS8</t>
+          <t>EDS</t>
         </is>
       </c>
     </row>
     <row r="3399">
       <c r="A3399" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B3399" t="n">
-        <v>3328</v>
+        <v>940540</v>
       </c>
       <c r="C3399" t="inlineStr">
         <is>
-          <t>ALAN ARAUJO DA SILVA</t>
+          <t>EDSON ARAUJO - FL8</t>
         </is>
       </c>
       <c r="D3399" t="inlineStr">
         <is>
-          <t>ARSILVA</t>
+          <t>EDS8</t>
         </is>
       </c>
     </row>
     <row r="3400">
       <c r="A3400" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3400" t="n">
-        <v>3350</v>
+        <v>3328</v>
       </c>
       <c r="C3400" t="inlineStr">
         <is>
-          <t xml:space="preserve">EDER RODRIGUES DA SILVA </t>
+          <t>ALAN ARAUJO DA SILVA</t>
         </is>
       </c>
       <c r="D3400" t="inlineStr">
         <is>
-          <t>EDERS</t>
+          <t>ARSILVA</t>
         </is>
       </c>
     </row>
     <row r="3401">
       <c r="A3401" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3401" t="n">
-        <v>3373</v>
+        <v>3350</v>
       </c>
       <c r="C3401" t="inlineStr">
         <is>
-          <t xml:space="preserve">NATANAEL TAVARES DE SOUSA </t>
+          <t xml:space="preserve">EDER RODRIGUES DA SILVA </t>
         </is>
       </c>
       <c r="D3401" t="inlineStr">
         <is>
-          <t>NTSOUSA</t>
+          <t>EDERS</t>
         </is>
       </c>
     </row>
@@ -68458,156 +68458,156 @@
         </is>
       </c>
       <c r="B3402" t="n">
-        <v>3374</v>
+        <v>3373</v>
       </c>
       <c r="C3402" t="inlineStr">
         <is>
-          <t>REINALDO DA SILVA COSTA</t>
+          <t xml:space="preserve">NATANAEL TAVARES DE SOUSA </t>
         </is>
       </c>
       <c r="D3402" t="inlineStr">
         <is>
-          <t>RSCOSTA</t>
+          <t>NTSOUSA</t>
         </is>
       </c>
     </row>
     <row r="3403">
       <c r="A3403" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3403" t="n">
-        <v>3399</v>
+        <v>3374</v>
       </c>
       <c r="C3403" t="inlineStr">
         <is>
-          <t xml:space="preserve">RICARDO BARBOSA DOS SANTOS </t>
+          <t>REINALDO DA SILVA COSTA</t>
         </is>
       </c>
       <c r="D3403" t="inlineStr">
         <is>
-          <t>RICARDOSAN</t>
+          <t>RSCOSTA</t>
         </is>
       </c>
     </row>
     <row r="3404">
       <c r="A3404" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3404" t="n">
-        <v>3427</v>
+        <v>3399</v>
       </c>
       <c r="C3404" t="inlineStr">
         <is>
-          <t>ROQUE COMERCIO TEMPORARIO</t>
+          <t xml:space="preserve">RICARDO BARBOSA DOS SANTOS </t>
         </is>
       </c>
       <c r="D3404" t="inlineStr">
         <is>
-          <t>ROQUECOM</t>
+          <t>RICARDOSAN</t>
         </is>
       </c>
     </row>
     <row r="3405">
       <c r="A3405" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3405" t="n">
-        <v>3428</v>
+        <v>3427</v>
       </c>
       <c r="C3405" t="inlineStr">
         <is>
-          <t>ROQUE PLUS TEMPORARIO</t>
+          <t>ROQUE COMERCIO TEMPORARIO</t>
         </is>
       </c>
       <c r="D3405" t="inlineStr">
         <is>
-          <t>ROQUEPLUS</t>
+          <t>ROQUECOM</t>
         </is>
       </c>
     </row>
     <row r="3406">
       <c r="A3406" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3406" t="n">
-        <v>3432</v>
+        <v>3428</v>
       </c>
       <c r="C3406" t="inlineStr">
         <is>
-          <t>PATRICIA DOS SANTOS NONATO OLIVEIRA</t>
+          <t>ROQUE PLUS TEMPORARIO</t>
         </is>
       </c>
       <c r="D3406" t="inlineStr">
         <is>
-          <t>PATRICIAD</t>
+          <t>ROQUEPLUS</t>
         </is>
       </c>
     </row>
     <row r="3407">
       <c r="A3407" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3407" t="n">
-        <v>3448</v>
+        <v>3432</v>
       </c>
       <c r="C3407" t="inlineStr">
         <is>
-          <t xml:space="preserve">GABRIEL SOUZA CARVALHO </t>
+          <t>PATRICIA DOS SANTOS NONATO OLIVEIRA</t>
         </is>
       </c>
       <c r="D3407" t="inlineStr">
         <is>
-          <t>GABRIEL20</t>
+          <t>PATRICIAD</t>
         </is>
       </c>
     </row>
     <row r="3408">
       <c r="A3408" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3408" t="n">
-        <v>3465</v>
+        <v>3448</v>
       </c>
       <c r="C3408" t="inlineStr">
         <is>
-          <t>LUIZA MARIA BARRETO BARBOSA</t>
+          <t xml:space="preserve">GABRIEL SOUZA CARVALHO </t>
         </is>
       </c>
       <c r="D3408" t="inlineStr">
         <is>
-          <t>LUIZA.MARIA</t>
+          <t>GABRIEL20</t>
         </is>
       </c>
     </row>
     <row r="3409">
       <c r="A3409" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3409" t="n">
-        <v>3468</v>
+        <v>3465</v>
       </c>
       <c r="C3409" t="inlineStr">
         <is>
-          <t>KAWA ALMEIDA CAMPOS</t>
+          <t>LUIZA MARIA BARRETO BARBOSA</t>
         </is>
       </c>
       <c r="D3409" t="inlineStr">
         <is>
-          <t>KAWA</t>
+          <t>LUIZA.MARIA</t>
         </is>
       </c>
     </row>
@@ -68618,16 +68618,16 @@
         </is>
       </c>
       <c r="B3410" t="n">
-        <v>3476</v>
+        <v>3468</v>
       </c>
       <c r="C3410" t="inlineStr">
         <is>
-          <t xml:space="preserve"> FRANCISCA LEIDIANE M. MENDES NASCIMENTO</t>
+          <t>KAWA ALMEIDA CAMPOS</t>
         </is>
       </c>
       <c r="D3410" t="inlineStr">
         <is>
-          <t>FLEIDIANE</t>
+          <t>KAWA</t>
         </is>
       </c>
     </row>
@@ -68638,76 +68638,76 @@
         </is>
       </c>
       <c r="B3411" t="n">
-        <v>3477</v>
+        <v>3476</v>
       </c>
       <c r="C3411" t="inlineStr">
         <is>
-          <t>MARIA THAIS MARTINS PEREIRA SILVA</t>
+          <t xml:space="preserve"> FRANCISCA LEIDIANE M. MENDES NASCIMENTO</t>
         </is>
       </c>
       <c r="D3411" t="inlineStr">
         <is>
-          <t>MTHAIS</t>
+          <t>FLEIDIANE</t>
         </is>
       </c>
     </row>
     <row r="3412">
       <c r="A3412" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3412" t="n">
-        <v>3271</v>
+        <v>3477</v>
       </c>
       <c r="C3412" t="inlineStr">
         <is>
-          <t>DIEGO DE ARAUJO CALÁBRIA</t>
+          <t>MARIA THAIS MARTINS PEREIRA SILVA</t>
         </is>
       </c>
       <c r="D3412" t="inlineStr">
         <is>
-          <t>ARAUJOC</t>
+          <t>MTHAIS</t>
         </is>
       </c>
     </row>
     <row r="3413">
       <c r="A3413" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3413" t="n">
-        <v>3272</v>
+        <v>3271</v>
       </c>
       <c r="C3413" t="inlineStr">
         <is>
-          <t>ANNE BEATRIZ SILVA VIRGINO</t>
+          <t>DIEGO DE ARAUJO CALÁBRIA</t>
         </is>
       </c>
       <c r="D3413" t="inlineStr">
         <is>
-          <t>ABVIRGINIO</t>
+          <t>ARAUJOC</t>
         </is>
       </c>
     </row>
     <row r="3414">
       <c r="A3414" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3414" t="n">
-        <v>3293</v>
+        <v>3272</v>
       </c>
       <c r="C3414" t="inlineStr">
         <is>
-          <t xml:space="preserve">CARLOS ALBERTO VIRIATO SANTOS </t>
+          <t>ANNE BEATRIZ SILVA VIRGINO</t>
         </is>
       </c>
       <c r="D3414" t="inlineStr">
         <is>
-          <t>CVIRIATO</t>
+          <t>ABVIRGINIO</t>
         </is>
       </c>
     </row>
@@ -68718,16 +68718,16 @@
         </is>
       </c>
       <c r="B3415" t="n">
-        <v>3381</v>
+        <v>3293</v>
       </c>
       <c r="C3415" t="inlineStr">
         <is>
-          <t>ALAN CAIQUE SANTOS E SANTOS</t>
+          <t xml:space="preserve">CARLOS ALBERTO VIRIATO SANTOS </t>
         </is>
       </c>
       <c r="D3415" t="inlineStr">
         <is>
-          <t>ALANSANTOS</t>
+          <t>CVIRIATO</t>
         </is>
       </c>
     </row>
@@ -68738,176 +68738,176 @@
         </is>
       </c>
       <c r="B3416" t="n">
-        <v>3443</v>
+        <v>3381</v>
       </c>
       <c r="C3416" t="inlineStr">
         <is>
-          <t>SANON MOREIRA SOUZA</t>
+          <t>ALAN CAIQUE SANTOS E SANTOS</t>
         </is>
       </c>
       <c r="D3416" t="inlineStr">
         <is>
-          <t>SANON</t>
+          <t>ALANSANTOS</t>
         </is>
       </c>
     </row>
     <row r="3417">
       <c r="A3417" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3417" t="n">
-        <v>3516</v>
+        <v>3443</v>
       </c>
       <c r="C3417" t="inlineStr">
         <is>
-          <t>FRANCISCO RILDER TELES DE OLIVEIRA</t>
+          <t>SANON MOREIRA SOUZA</t>
         </is>
       </c>
       <c r="D3417" t="inlineStr">
         <is>
-          <t>RILDER</t>
+          <t>SANON</t>
         </is>
       </c>
     </row>
     <row r="3418">
       <c r="A3418" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3418" t="n">
-        <v>3519</v>
+        <v>3516</v>
       </c>
       <c r="C3418" t="inlineStr">
         <is>
-          <t>MARIA LUANA DE ALMEIDA BATISTA</t>
+          <t>FRANCISCO RILDER TELES DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D3418" t="inlineStr">
         <is>
-          <t>M.LUANA</t>
+          <t>RILDER</t>
         </is>
       </c>
     </row>
     <row r="3419">
       <c r="A3419" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3419" t="n">
-        <v>3540</v>
+        <v>3519</v>
       </c>
       <c r="C3419" t="inlineStr">
         <is>
-          <t>HELEN VITORIA OLIVEIRA DA ROCHA</t>
+          <t>MARIA LUANA DE ALMEIDA BATISTA</t>
         </is>
       </c>
       <c r="D3419" t="inlineStr">
         <is>
-          <t>H.VITORIA</t>
+          <t>M.LUANA</t>
         </is>
       </c>
     </row>
     <row r="3420">
       <c r="A3420" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B3420" t="n">
-        <v>3331</v>
+        <v>3540</v>
       </c>
       <c r="C3420" t="inlineStr">
         <is>
-          <t>LOUIZE VANIELLE RODRIGUES FARIAS</t>
+          <t>HELEN VITORIA OLIVEIRA DA ROCHA</t>
         </is>
       </c>
       <c r="D3420" t="inlineStr">
         <is>
-          <t>LVFARIAS</t>
+          <t>H.VITORIA</t>
         </is>
       </c>
     </row>
     <row r="3421">
       <c r="A3421" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3421" t="n">
-        <v>3332</v>
+        <v>3331</v>
       </c>
       <c r="C3421" t="inlineStr">
         <is>
-          <t>ALEXSANDRO PEIXOTO DA VEIGA PACHECO</t>
+          <t>LOUIZE VANIELLE RODRIGUES FARIAS</t>
         </is>
       </c>
       <c r="D3421" t="inlineStr">
         <is>
-          <t>APVEIGA</t>
+          <t>LVFARIAS</t>
         </is>
       </c>
     </row>
     <row r="3422">
       <c r="A3422" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B3422" t="n">
-        <v>3334</v>
+        <v>3332</v>
       </c>
       <c r="C3422" t="inlineStr">
         <is>
-          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+          <t>ALEXSANDRO PEIXOTO DA VEIGA PACHECO</t>
         </is>
       </c>
       <c r="D3422" t="inlineStr">
         <is>
-          <t>MTGASPAR</t>
+          <t>APVEIGA</t>
         </is>
       </c>
     </row>
     <row r="3423">
       <c r="A3423" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3423" t="n">
-        <v>3345</v>
+        <v>3334</v>
       </c>
       <c r="C3423" t="inlineStr">
         <is>
-          <t>AURICÉLIA INACIO PEREIRA</t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
       <c r="D3423" t="inlineStr">
         <is>
-          <t>AIPEREIRA</t>
+          <t>MTGASPAR</t>
         </is>
       </c>
     </row>
     <row r="3424">
       <c r="A3424" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3424" t="n">
-        <v>3363</v>
+        <v>3345</v>
       </c>
       <c r="C3424" t="inlineStr">
         <is>
-          <t>IASMIN LEAL ALVES</t>
+          <t>AURICÉLIA INACIO PEREIRA</t>
         </is>
       </c>
       <c r="D3424" t="inlineStr">
         <is>
-          <t>ILALVES</t>
+          <t>AIPEREIRA</t>
         </is>
       </c>
     </row>
@@ -68918,196 +68918,196 @@
         </is>
       </c>
       <c r="B3425" t="n">
-        <v>3370</v>
+        <v>3363</v>
       </c>
       <c r="C3425" t="inlineStr">
         <is>
-          <t>CARLOS DIEGO ARAUJO ALMEIDA</t>
+          <t>IASMIN LEAL ALVES</t>
         </is>
       </c>
       <c r="D3425" t="inlineStr">
         <is>
-          <t>CDIEGO</t>
+          <t>ILALVES</t>
         </is>
       </c>
     </row>
     <row r="3426">
       <c r="A3426" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3426" t="n">
-        <v>3379</v>
+        <v>3370</v>
       </c>
       <c r="C3426" t="inlineStr">
         <is>
-          <t xml:space="preserve">MATHEUS EVANGELISTA FERREIRA </t>
+          <t>CARLOS DIEGO ARAUJO ALMEIDA</t>
         </is>
       </c>
       <c r="D3426" t="inlineStr">
         <is>
-          <t>MMFERREIRA</t>
+          <t>CDIEGO</t>
         </is>
       </c>
     </row>
     <row r="3427">
       <c r="A3427" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3427" t="n">
-        <v>3419</v>
+        <v>3379</v>
       </c>
       <c r="C3427" t="inlineStr">
         <is>
-          <t xml:space="preserve">DAVID EVANGELISTA SILVA </t>
+          <t xml:space="preserve">MATHEUS EVANGELISTA FERREIRA </t>
         </is>
       </c>
       <c r="D3427" t="inlineStr">
         <is>
-          <t>DAVID</t>
+          <t>MMFERREIRA</t>
         </is>
       </c>
     </row>
     <row r="3428">
       <c r="A3428" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3428" t="n">
-        <v>3423</v>
+        <v>3419</v>
       </c>
       <c r="C3428" t="inlineStr">
         <is>
-          <t>MARCIO JOSE TIAGO</t>
+          <t xml:space="preserve">DAVID EVANGELISTA SILVA </t>
         </is>
       </c>
       <c r="D3428" t="inlineStr">
         <is>
-          <t>MJTIAGO</t>
+          <t>DAVID</t>
         </is>
       </c>
     </row>
     <row r="3429">
       <c r="A3429" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3429" t="n">
-        <v>3453</v>
+        <v>3423</v>
       </c>
       <c r="C3429" t="inlineStr">
         <is>
-          <t xml:space="preserve">LAURIENE SILVA BARBOSA </t>
+          <t>MARCIO JOSE TIAGO</t>
         </is>
       </c>
       <c r="D3429" t="inlineStr">
         <is>
-          <t>LAURIENE</t>
+          <t>MJTIAGO</t>
         </is>
       </c>
     </row>
     <row r="3430">
       <c r="A3430" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3430" t="n">
-        <v>3478</v>
+        <v>3453</v>
       </c>
       <c r="C3430" t="inlineStr">
         <is>
-          <t>LEANDRO BRITO NOGUEIRA DE OLIVEIRA</t>
+          <t xml:space="preserve">LAURIENE SILVA BARBOSA </t>
         </is>
       </c>
       <c r="D3430" t="inlineStr">
         <is>
-          <t>LBNOGUEIRA</t>
+          <t>LAURIENE</t>
         </is>
       </c>
     </row>
     <row r="3431">
       <c r="A3431" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3431" t="n">
-        <v>3479</v>
+        <v>3478</v>
       </c>
       <c r="C3431" t="inlineStr">
         <is>
-          <t>ESDRAS ALESSANDRO SANTOS SANTANA</t>
+          <t>LEANDRO BRITO NOGUEIRA DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D3431" t="inlineStr">
         <is>
-          <t>EALESSANDRO</t>
+          <t>LBNOGUEIRA</t>
         </is>
       </c>
     </row>
     <row r="3432">
       <c r="A3432" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3432" t="n">
-        <v>3480</v>
+        <v>3479</v>
       </c>
       <c r="C3432" t="inlineStr">
         <is>
-          <t xml:space="preserve">LUCIMARA SOUSA LIMA </t>
+          <t>ESDRAS ALESSANDRO SANTOS SANTANA</t>
         </is>
       </c>
       <c r="D3432" t="inlineStr">
         <is>
-          <t>LUCIMARA</t>
+          <t>EALESSANDRO</t>
         </is>
       </c>
     </row>
     <row r="3433">
       <c r="A3433" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3433" t="n">
-        <v>3482</v>
+        <v>3480</v>
       </c>
       <c r="C3433" t="inlineStr">
         <is>
-          <t>DANIEL FERNANDES DINIZ HERACLIO</t>
+          <t xml:space="preserve">LUCIMARA SOUSA LIMA </t>
         </is>
       </c>
       <c r="D3433" t="inlineStr">
         <is>
-          <t>DFDINIZ</t>
+          <t>LUCIMARA</t>
         </is>
       </c>
     </row>
     <row r="3434">
       <c r="A3434" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3434" t="n">
-        <v>3518</v>
+        <v>3482</v>
       </c>
       <c r="C3434" t="inlineStr">
         <is>
-          <t>RAMYRA ALVES FELIX DA SILVA</t>
+          <t>DANIEL FERNANDES DINIZ HERACLIO</t>
         </is>
       </c>
       <c r="D3434" t="inlineStr">
         <is>
-          <t>RFELIX</t>
+          <t>DFDINIZ</t>
         </is>
       </c>
     </row>
@@ -69118,36 +69118,36 @@
         </is>
       </c>
       <c r="B3435" t="n">
-        <v>3534</v>
+        <v>3518</v>
       </c>
       <c r="C3435" t="inlineStr">
         <is>
-          <t xml:space="preserve">CAIO DE SOUZA VINHAS </t>
+          <t>RAMYRA ALVES FELIX DA SILVA</t>
         </is>
       </c>
       <c r="D3435" t="inlineStr">
         <is>
-          <t>CVINHAS</t>
+          <t>RFELIX</t>
         </is>
       </c>
     </row>
     <row r="3436">
       <c r="A3436" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3436" t="n">
-        <v>3535</v>
+        <v>3534</v>
       </c>
       <c r="C3436" t="inlineStr">
         <is>
-          <t>ROMARIO DE SOUSA SILVA</t>
+          <t xml:space="preserve">CAIO DE SOUZA VINHAS </t>
         </is>
       </c>
       <c r="D3436" t="inlineStr">
         <is>
-          <t>RSOUSAS</t>
+          <t>CVINHAS</t>
         </is>
       </c>
     </row>
@@ -69158,56 +69158,56 @@
         </is>
       </c>
       <c r="B3437" t="n">
-        <v>3536</v>
+        <v>3535</v>
       </c>
       <c r="C3437" t="inlineStr">
         <is>
-          <t>JHONATAS CARVALHO OLIVEIRA</t>
+          <t>ROMARIO DE SOUSA SILVA</t>
         </is>
       </c>
       <c r="D3437" t="inlineStr">
         <is>
-          <t>JHONATASC</t>
+          <t>RSOUSAS</t>
         </is>
       </c>
     </row>
     <row r="3438">
       <c r="A3438" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3438" t="n">
-        <v>940529</v>
+        <v>3536</v>
       </c>
       <c r="C3438" t="inlineStr">
         <is>
-          <t>EDGAR FELIX - FL9</t>
+          <t>JHONATAS CARVALHO OLIVEIRA</t>
         </is>
       </c>
       <c r="D3438" t="inlineStr">
         <is>
-          <t>EDGAR F</t>
+          <t>JHONATASC</t>
         </is>
       </c>
     </row>
     <row r="3439">
       <c r="A3439" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3439" t="n">
-        <v>3304</v>
+        <v>940529</v>
       </c>
       <c r="C3439" t="inlineStr">
         <is>
-          <t>JOACI GUILHERME GONÇALVES DA LUZ</t>
+          <t>EDGAR FELIX - FL9</t>
         </is>
       </c>
       <c r="D3439" t="inlineStr">
         <is>
-          <t>JLUZ</t>
+          <t>EDGAR F</t>
         </is>
       </c>
     </row>
@@ -69218,16 +69218,16 @@
         </is>
       </c>
       <c r="B3440" t="n">
-        <v>3305</v>
+        <v>3304</v>
       </c>
       <c r="C3440" t="inlineStr">
         <is>
-          <t>JOÃO VITOR DE ARAÚJO GONÇALVES</t>
+          <t>JOACI GUILHERME GONÇALVES DA LUZ</t>
         </is>
       </c>
       <c r="D3440" t="inlineStr">
         <is>
-          <t>JJVITOR</t>
+          <t>JLUZ</t>
         </is>
       </c>
     </row>
@@ -69238,36 +69238,36 @@
         </is>
       </c>
       <c r="B3441" t="n">
-        <v>3306</v>
+        <v>3305</v>
       </c>
       <c r="C3441" t="inlineStr">
         <is>
-          <t>WENDERSON MARCOS DOS SANTOS</t>
+          <t>JOÃO VITOR DE ARAÚJO GONÇALVES</t>
         </is>
       </c>
       <c r="D3441" t="inlineStr">
         <is>
-          <t>WWMARCOS</t>
+          <t>JJVITOR</t>
         </is>
       </c>
     </row>
     <row r="3442">
       <c r="A3442" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3442" t="n">
-        <v>3335</v>
+        <v>3306</v>
       </c>
       <c r="C3442" t="inlineStr">
         <is>
-          <t>EDILBERTO LEMOS DE LIMA</t>
+          <t>WENDERSON MARCOS DOS SANTOS</t>
         </is>
       </c>
       <c r="D3442" t="inlineStr">
         <is>
-          <t>ELEMOS</t>
+          <t>WWMARCOS</t>
         </is>
       </c>
     </row>
@@ -69278,116 +69278,116 @@
         </is>
       </c>
       <c r="B3443" t="n">
-        <v>3336</v>
+        <v>3335</v>
       </c>
       <c r="C3443" t="inlineStr">
         <is>
-          <t>EZEQUIEL SOUZA DO NASCIMENTO</t>
+          <t>EDILBERTO LEMOS DE LIMA</t>
         </is>
       </c>
       <c r="D3443" t="inlineStr">
         <is>
-          <t>ESNASCIMENTO</t>
+          <t>ELEMOS</t>
         </is>
       </c>
     </row>
     <row r="3444">
       <c r="A3444" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3444" t="n">
-        <v>3341</v>
+        <v>3336</v>
       </c>
       <c r="C3444" t="inlineStr">
         <is>
-          <t>ALCIONE MARIANO DE OLIVEIRA</t>
+          <t>EZEQUIEL SOUZA DO NASCIMENTO</t>
         </is>
       </c>
       <c r="D3444" t="inlineStr">
         <is>
-          <t>AMOLIVEIRA</t>
+          <t>ESNASCIMENTO</t>
         </is>
       </c>
     </row>
     <row r="3445">
       <c r="A3445" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3445" t="n">
-        <v>3401</v>
+        <v>3341</v>
       </c>
       <c r="C3445" t="inlineStr">
         <is>
-          <t xml:space="preserve">TULIO HENRIQUE DA SILVA CARVALHO </t>
+          <t>ALCIONE MARIANO DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D3445" t="inlineStr">
         <is>
-          <t>TULIO</t>
+          <t>AMOLIVEIRA</t>
         </is>
       </c>
     </row>
     <row r="3446">
       <c r="A3446" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3446" t="n">
-        <v>3411</v>
+        <v>3401</v>
       </c>
       <c r="C3446" t="inlineStr">
         <is>
-          <t>CONEXAO RUBYA DANILLA</t>
+          <t xml:space="preserve">TULIO HENRIQUE DA SILVA CARVALHO </t>
         </is>
       </c>
       <c r="D3446" t="inlineStr">
         <is>
-          <t>CONEXAORUBYA</t>
+          <t>TULIO</t>
         </is>
       </c>
     </row>
     <row r="3447">
       <c r="A3447" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3447" t="n">
-        <v>3412</v>
+        <v>3411</v>
       </c>
       <c r="C3447" t="inlineStr">
         <is>
-          <t>CONEXAO RAFAEL</t>
+          <t>CONEXAO RUBYA DANILLA</t>
         </is>
       </c>
       <c r="D3447" t="inlineStr">
         <is>
-          <t>CONEXAORAFAEL</t>
+          <t>CONEXAORUBYA</t>
         </is>
       </c>
     </row>
     <row r="3448">
       <c r="A3448" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3448" t="n">
-        <v>3264</v>
+        <v>3412</v>
       </c>
       <c r="C3448" t="inlineStr">
         <is>
-          <t xml:space="preserve">WILTON CARLOS MACIEL DE ASSIS </t>
+          <t>CONEXAO RAFAEL</t>
         </is>
       </c>
       <c r="D3448" t="inlineStr">
         <is>
-          <t>WCMACIEL</t>
+          <t>CONEXAORAFAEL</t>
         </is>
       </c>
     </row>
@@ -69398,56 +69398,56 @@
         </is>
       </c>
       <c r="B3449" t="n">
-        <v>3340</v>
+        <v>3264</v>
       </c>
       <c r="C3449" t="inlineStr">
         <is>
-          <t>ROGELENO FARIAS FEIJÃO FILHO</t>
+          <t xml:space="preserve">WILTON CARLOS MACIEL DE ASSIS </t>
         </is>
       </c>
       <c r="D3449" t="inlineStr">
         <is>
-          <t>RFEIJAO</t>
+          <t>WCMACIEL</t>
         </is>
       </c>
     </row>
     <row r="3450">
       <c r="A3450" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3450" t="n">
-        <v>940550</v>
+        <v>3340</v>
       </c>
       <c r="C3450" t="inlineStr">
         <is>
-          <t>RAFAELE RIBEIRO CARNEIRO</t>
+          <t>ROGELENO FARIAS FEIJÃO FILHO</t>
         </is>
       </c>
       <c r="D3450" t="inlineStr">
         <is>
-          <t>RAFAELE</t>
+          <t>RFEIJAO</t>
         </is>
       </c>
     </row>
     <row r="3451">
       <c r="A3451" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>99</t>
         </is>
       </c>
       <c r="B3451" t="n">
-        <v>3377</v>
+        <v>940550</v>
       </c>
       <c r="C3451" t="inlineStr">
         <is>
-          <t xml:space="preserve"> ISALTINO BISPO DE OLIVEIRA JUNIOR</t>
+          <t>RAFAELE RIBEIRO CARNEIRO</t>
         </is>
       </c>
       <c r="D3451" t="inlineStr">
         <is>
-          <t>BJUNIOR</t>
+          <t>RAFAELE</t>
         </is>
       </c>
     </row>
@@ -69458,56 +69458,56 @@
         </is>
       </c>
       <c r="B3452" t="n">
-        <v>3425</v>
+        <v>3377</v>
       </c>
       <c r="C3452" t="inlineStr">
         <is>
-          <t xml:space="preserve"> CIRLANE ARAUJO SOUZA </t>
+          <t xml:space="preserve"> ISALTINO BISPO DE OLIVEIRA JUNIOR</t>
         </is>
       </c>
       <c r="D3452" t="inlineStr">
         <is>
-          <t>CIRLANES</t>
+          <t>BJUNIOR</t>
         </is>
       </c>
     </row>
     <row r="3453">
       <c r="A3453" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3453" t="n">
-        <v>3454</v>
+        <v>3425</v>
       </c>
       <c r="C3453" t="inlineStr">
         <is>
-          <t>ANTONIA SAMARA DE SOUZA SOARES</t>
+          <t xml:space="preserve"> CIRLANE ARAUJO SOUZA </t>
         </is>
       </c>
       <c r="D3453" t="inlineStr">
         <is>
-          <t>ANTSAMARA</t>
+          <t>CIRLANES</t>
         </is>
       </c>
     </row>
     <row r="3454">
       <c r="A3454" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3454" t="n">
-        <v>3491</v>
+        <v>3454</v>
       </c>
       <c r="C3454" t="inlineStr">
         <is>
-          <t>PEDRO JOSE DO NASCIMENTO NETO</t>
+          <t>ANTONIA SAMARA DE SOUZA SOARES</t>
         </is>
       </c>
       <c r="D3454" t="inlineStr">
         <is>
-          <t>P.JOSE</t>
+          <t>ANTSAMARA</t>
         </is>
       </c>
     </row>
@@ -69518,36 +69518,36 @@
         </is>
       </c>
       <c r="B3455" t="n">
-        <v>3492</v>
+        <v>3491</v>
       </c>
       <c r="C3455" t="inlineStr">
         <is>
-          <t>PAULA CARLA CALDAS MOTA</t>
+          <t>PEDRO JOSE DO NASCIMENTO NETO</t>
         </is>
       </c>
       <c r="D3455" t="inlineStr">
         <is>
-          <t>P.CARLA</t>
+          <t>P.JOSE</t>
         </is>
       </c>
     </row>
     <row r="3456">
       <c r="A3456" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3456" t="n">
-        <v>3542</v>
+        <v>3492</v>
       </c>
       <c r="C3456" t="inlineStr">
         <is>
-          <t>ANTONIA MILENA SOUSA ANDRADE</t>
+          <t>PAULA CARLA CALDAS MOTA</t>
         </is>
       </c>
       <c r="D3456" t="inlineStr">
         <is>
-          <t>A.MILENA</t>
+          <t>P.CARLA</t>
         </is>
       </c>
     </row>
@@ -69558,16 +69558,16 @@
         </is>
       </c>
       <c r="B3457" t="n">
-        <v>3547</v>
+        <v>3542</v>
       </c>
       <c r="C3457" t="inlineStr">
         <is>
-          <t xml:space="preserve">DAVI PEREIRA DA SILVA </t>
+          <t>ANTONIA MILENA SOUSA ANDRADE</t>
         </is>
       </c>
       <c r="D3457" t="inlineStr">
         <is>
-          <t>DPSILVA</t>
+          <t>A.MILENA</t>
         </is>
       </c>
     </row>
@@ -69578,214 +69578,254 @@
         </is>
       </c>
       <c r="B3458" t="n">
-        <v>3294</v>
+        <v>3547</v>
       </c>
       <c r="C3458" t="inlineStr">
         <is>
-          <t>GLEICIANE MIRANDA DE MORAIS</t>
+          <t xml:space="preserve">DAVI PEREIRA DA SILVA </t>
         </is>
       </c>
       <c r="D3458" t="inlineStr">
         <is>
-          <t>GMIRANDA</t>
+          <t>DPSILVA</t>
         </is>
       </c>
     </row>
     <row r="3459">
       <c r="A3459" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3459" t="n">
-        <v>3295</v>
+        <v>3552</v>
       </c>
       <c r="C3459" t="inlineStr">
         <is>
-          <t>MARIA ESTEFANNY DA SILVA MOURA</t>
+          <t>PAULO SERGIO MENDES DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D3459" t="inlineStr">
         <is>
-          <t>MESTEFANNY</t>
+          <t>PSMENDES</t>
         </is>
       </c>
     </row>
     <row r="3460">
       <c r="A3460" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3460" t="n">
-        <v>3296</v>
+        <v>3294</v>
       </c>
       <c r="C3460" t="inlineStr">
         <is>
-          <t>PEDRO IAGO FONSECA EVANGELISTA</t>
+          <t>GLEICIANE MIRANDA DE MORAIS</t>
         </is>
       </c>
       <c r="D3460" t="inlineStr">
         <is>
-          <t>PIFONSECA</t>
+          <t>GMIRANDA</t>
         </is>
       </c>
     </row>
     <row r="3461">
       <c r="A3461" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3461" t="n">
-        <v>940544</v>
+        <v>3295</v>
       </c>
       <c r="C3461" t="inlineStr">
         <is>
-          <t>LUTY LOG TRANSPORTES - FL8</t>
+          <t>MARIA ESTEFANNY DA SILVA MOURA</t>
         </is>
       </c>
       <c r="D3461" t="inlineStr">
         <is>
-          <t>LUTY LOG</t>
+          <t>MESTEFANNY</t>
         </is>
       </c>
     </row>
     <row r="3462">
       <c r="A3462" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3462" t="n">
-        <v>3380</v>
+        <v>3296</v>
       </c>
       <c r="C3462" t="inlineStr">
         <is>
-          <t>FRANCISCO MATHEUS RABELO DA COSTA</t>
+          <t>PEDRO IAGO FONSECA EVANGELISTA</t>
         </is>
       </c>
       <c r="D3462" t="inlineStr">
         <is>
-          <t>FMATHEUS</t>
+          <t>PIFONSECA</t>
         </is>
       </c>
     </row>
     <row r="3463">
       <c r="A3463" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B3463" t="n">
-        <v>3410</v>
+        <v>940544</v>
       </c>
       <c r="C3463" t="inlineStr">
         <is>
-          <t xml:space="preserve"> BRENO ALLAN DE JESUS</t>
+          <t>LUTY LOG TRANSPORTES - FL8</t>
         </is>
       </c>
       <c r="D3463" t="inlineStr">
         <is>
-          <t>JESUS</t>
+          <t>LUTY LOG</t>
         </is>
       </c>
     </row>
     <row r="3464">
       <c r="A3464" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3464" t="n">
-        <v>3444</v>
+        <v>3380</v>
       </c>
       <c r="C3464" t="inlineStr">
         <is>
-          <t>THIAGO COSTA SILVA</t>
+          <t>FRANCISCO MATHEUS RABELO DA COSTA</t>
         </is>
       </c>
       <c r="D3464" t="inlineStr">
         <is>
-          <t>THIAGOC</t>
+          <t>FMATHEUS</t>
         </is>
       </c>
     </row>
     <row r="3465">
       <c r="A3465" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3465" t="n">
-        <v>3456</v>
+        <v>3410</v>
       </c>
       <c r="C3465" t="inlineStr">
         <is>
-          <t>FELIPE BOTH MAZUCHINI</t>
+          <t xml:space="preserve"> BRENO ALLAN DE JESUS</t>
         </is>
       </c>
       <c r="D3465" t="inlineStr">
         <is>
-          <t>FELIPEB</t>
+          <t>JESUS</t>
         </is>
       </c>
     </row>
     <row r="3466">
       <c r="A3466" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3466" t="n">
-        <v>3457</v>
+        <v>3444</v>
       </c>
       <c r="C3466" t="inlineStr">
         <is>
-          <t>FRANKLIN VIEIRA GOMES</t>
+          <t>THIAGO COSTA SILVA</t>
         </is>
       </c>
       <c r="D3466" t="inlineStr">
         <is>
-          <t>VIEIRAF</t>
+          <t>THIAGOC</t>
         </is>
       </c>
     </row>
     <row r="3467">
       <c r="A3467" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3467" t="n">
-        <v>3507</v>
+        <v>3456</v>
       </c>
       <c r="C3467" t="inlineStr">
         <is>
-          <t>KARINE TEODORA ALVES DE OLIVEIRA</t>
+          <t>FELIPE BOTH MAZUCHINI</t>
         </is>
       </c>
       <c r="D3467" t="inlineStr">
         <is>
-          <t>KOLIVEIRA</t>
+          <t>FELIPEB</t>
         </is>
       </c>
     </row>
     <row r="3468">
       <c r="A3468" t="inlineStr">
         <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B3468" t="n">
+        <v>3457</v>
+      </c>
+      <c r="C3468" t="inlineStr">
+        <is>
+          <t>FRANKLIN VIEIRA GOMES</t>
+        </is>
+      </c>
+      <c r="D3468" t="inlineStr">
+        <is>
+          <t>VIEIRAF</t>
+        </is>
+      </c>
+    </row>
+    <row r="3469">
+      <c r="A3469" t="inlineStr">
+        <is>
           <t>5</t>
         </is>
       </c>
-      <c r="B3468" t="n">
+      <c r="B3469" t="n">
+        <v>3507</v>
+      </c>
+      <c r="C3469" t="inlineStr">
+        <is>
+          <t>KARINE TEODORA ALVES DE OLIVEIRA</t>
+        </is>
+      </c>
+      <c r="D3469" t="inlineStr">
+        <is>
+          <t>KOLIVEIRA</t>
+        </is>
+      </c>
+    </row>
+    <row r="3470">
+      <c r="A3470" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B3470" t="n">
         <v>3520</v>
       </c>
-      <c r="C3468" t="inlineStr">
+      <c r="C3470" t="inlineStr">
         <is>
           <t xml:space="preserve"> EMERSON FILIPE MELO DE AGUIAR</t>
         </is>
       </c>
-      <c r="D3468" t="inlineStr">
+      <c r="D3470" t="inlineStr">
         <is>
           <t>E.FILIPE</t>
         </is>

</xml_diff>

<commit_message>
chore(data): batch update intraday televendas - 08:03:00
</commit_message>
<xml_diff>
--- a/data/dim_televendas.xlsx
+++ b/data/dim_televendas.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3473"/>
+  <dimension ref="A1:D3476"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -67434,20 +67434,20 @@
     <row r="3351">
       <c r="A3351" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3351" t="n">
-        <v>3355</v>
+        <v>3560</v>
       </c>
       <c r="C3351" t="inlineStr">
         <is>
-          <t>HUGO MATHEUS DA COSTA FEITOSA</t>
+          <t>MARIA EDUARDA MELO DOS SANTOS</t>
         </is>
       </c>
       <c r="D3351" t="inlineStr">
         <is>
-          <t>HMFEITOSA</t>
+          <t>EDU.MELO</t>
         </is>
       </c>
     </row>
@@ -67458,96 +67458,96 @@
         </is>
       </c>
       <c r="B3352" t="n">
-        <v>3356</v>
+        <v>3355</v>
       </c>
       <c r="C3352" t="inlineStr">
         <is>
-          <t>BRENDA LIMA DE OLIVEIRA CUNHA</t>
+          <t>HUGO MATHEUS DA COSTA FEITOSA</t>
         </is>
       </c>
       <c r="D3352" t="inlineStr">
         <is>
-          <t>BLCUNHA</t>
+          <t>HMFEITOSA</t>
         </is>
       </c>
     </row>
     <row r="3353">
       <c r="A3353" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3353" t="n">
-        <v>3361</v>
+        <v>3356</v>
       </c>
       <c r="C3353" t="inlineStr">
         <is>
-          <t>WLADIA DE ARAUJO BASTOS</t>
+          <t>BRENDA LIMA DE OLIVEIRA CUNHA</t>
         </is>
       </c>
       <c r="D3353" t="inlineStr">
         <is>
-          <t>WABASTOS</t>
+          <t>BLCUNHA</t>
         </is>
       </c>
     </row>
     <row r="3354">
       <c r="A3354" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3354" t="n">
-        <v>3362</v>
+        <v>3361</v>
       </c>
       <c r="C3354" t="inlineStr">
         <is>
-          <t>CARLOS HENRIQUE MELO DA SILVA</t>
+          <t>WLADIA DE ARAUJO BASTOS</t>
         </is>
       </c>
       <c r="D3354" t="inlineStr">
         <is>
-          <t>CHMELO</t>
+          <t>WABASTOS</t>
         </is>
       </c>
     </row>
     <row r="3355">
       <c r="A3355" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3355" t="n">
-        <v>3375</v>
+        <v>3362</v>
       </c>
       <c r="C3355" t="inlineStr">
         <is>
-          <t>AFONSO DE SOUSA RAMOS FILHO</t>
+          <t>CARLOS HENRIQUE MELO DA SILVA</t>
         </is>
       </c>
       <c r="D3355" t="inlineStr">
         <is>
-          <t>AFILHO</t>
+          <t>CHMELO</t>
         </is>
       </c>
     </row>
     <row r="3356">
       <c r="A3356" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3356" t="n">
-        <v>3404</v>
+        <v>3375</v>
       </c>
       <c r="C3356" t="inlineStr">
         <is>
-          <t>NOVATO 4 COM</t>
+          <t>AFONSO DE SOUSA RAMOS FILHO</t>
         </is>
       </c>
       <c r="D3356" t="inlineStr">
         <is>
-          <t>NOVATO4COM</t>
+          <t>AFILHO</t>
         </is>
       </c>
     </row>
@@ -67558,156 +67558,156 @@
         </is>
       </c>
       <c r="B3357" t="n">
-        <v>3405</v>
+        <v>3404</v>
       </c>
       <c r="C3357" t="inlineStr">
         <is>
-          <t>NOVATO 5 COM</t>
+          <t>NOVATO 4 COM</t>
         </is>
       </c>
       <c r="D3357" t="inlineStr">
         <is>
-          <t>NOVATO5COM</t>
+          <t>NOVATO4COM</t>
         </is>
       </c>
     </row>
     <row r="3358">
       <c r="A3358" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3358" t="n">
-        <v>3447</v>
+        <v>3405</v>
       </c>
       <c r="C3358" t="inlineStr">
         <is>
-          <t>RAYSSA KEYCE LINHARES AQUINO</t>
+          <t>NOVATO 5 COM</t>
         </is>
       </c>
       <c r="D3358" t="inlineStr">
         <is>
-          <t>RAYSSAK</t>
+          <t>NOVATO5COM</t>
         </is>
       </c>
     </row>
     <row r="3359">
       <c r="A3359" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3359" t="n">
-        <v>940559</v>
+        <v>3447</v>
       </c>
       <c r="C3359" t="inlineStr">
         <is>
-          <t>WALLEF DE OLIVEIRA</t>
+          <t>RAYSSA KEYCE LINHARES AQUINO</t>
         </is>
       </c>
       <c r="D3359" t="inlineStr">
         <is>
-          <t>WALLEF</t>
+          <t>RAYSSAK</t>
         </is>
       </c>
     </row>
     <row r="3360">
       <c r="A3360" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>99</t>
         </is>
       </c>
       <c r="B3360" t="n">
-        <v>3489</v>
+        <v>940559</v>
       </c>
       <c r="C3360" t="inlineStr">
         <is>
-          <t>MARCELA KARINA PEREIRA VELOSO</t>
+          <t>WALLEF DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D3360" t="inlineStr">
         <is>
-          <t>MKARINA</t>
+          <t>WALLEF</t>
         </is>
       </c>
     </row>
     <row r="3361">
       <c r="A3361" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3361" t="n">
-        <v>3490</v>
+        <v>3489</v>
       </c>
       <c r="C3361" t="inlineStr">
         <is>
-          <t>JOSE MAILSON GOMES NUNES</t>
+          <t>MARCELA KARINA PEREIRA VELOSO</t>
         </is>
       </c>
       <c r="D3361" t="inlineStr">
         <is>
-          <t>J.MAILSON</t>
+          <t>MKARINA</t>
         </is>
       </c>
     </row>
     <row r="3362">
       <c r="A3362" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3362" t="n">
-        <v>3537</v>
+        <v>3490</v>
       </c>
       <c r="C3362" t="inlineStr">
         <is>
-          <t>ALDAIR PEDRO DA SILVA</t>
+          <t>JOSE MAILSON GOMES NUNES</t>
         </is>
       </c>
       <c r="D3362" t="inlineStr">
         <is>
-          <t>A.PEDRO</t>
+          <t>J.MAILSON</t>
         </is>
       </c>
     </row>
     <row r="3363">
       <c r="A3363" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3363" t="n">
-        <v>3549</v>
+        <v>3537</v>
       </c>
       <c r="C3363" t="inlineStr">
         <is>
-          <t xml:space="preserve">FERNANDA CAROLINE E CESAR SOUSA </t>
+          <t>ALDAIR PEDRO DA SILVA</t>
         </is>
       </c>
       <c r="D3363" t="inlineStr">
         <is>
-          <t>FCAROLINE</t>
+          <t>A.PEDRO</t>
         </is>
       </c>
     </row>
     <row r="3364">
       <c r="A3364" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3364" t="n">
-        <v>3337</v>
+        <v>3549</v>
       </c>
       <c r="C3364" t="inlineStr">
         <is>
-          <t>WESLEY FONTES DE ALMEIDA</t>
+          <t xml:space="preserve">FERNANDA CAROLINE E CESAR SOUSA </t>
         </is>
       </c>
       <c r="D3364" t="inlineStr">
         <is>
-          <t>WFALMEIDA</t>
+          <t>FCAROLINE</t>
         </is>
       </c>
     </row>
@@ -67718,16 +67718,16 @@
         </is>
       </c>
       <c r="B3365" t="n">
-        <v>3338</v>
+        <v>3337</v>
       </c>
       <c r="C3365" t="inlineStr">
         <is>
-          <t>FRANCISCA SAMARA MENDES DE OLIVEIRA C</t>
+          <t>WESLEY FONTES DE ALMEIDA</t>
         </is>
       </c>
       <c r="D3365" t="inlineStr">
         <is>
-          <t>FSCUNHA</t>
+          <t>WFALMEIDA</t>
         </is>
       </c>
     </row>
@@ -67738,176 +67738,176 @@
         </is>
       </c>
       <c r="B3366" t="n">
-        <v>3339</v>
+        <v>3338</v>
       </c>
       <c r="C3366" t="inlineStr">
         <is>
-          <t>MAYARA THALYA DIAS DE ANDRADE</t>
+          <t>FRANCISCA SAMARA MENDES DE OLIVEIRA C</t>
         </is>
       </c>
       <c r="D3366" t="inlineStr">
         <is>
-          <t>MTANDRADE</t>
+          <t>FSCUNHA</t>
         </is>
       </c>
     </row>
     <row r="3367">
       <c r="A3367" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3367" t="n">
-        <v>3359</v>
+        <v>3339</v>
       </c>
       <c r="C3367" t="inlineStr">
         <is>
-          <t xml:space="preserve">EVANESSA DA SILVA E SILVA </t>
+          <t>MAYARA THALYA DIAS DE ANDRADE</t>
         </is>
       </c>
       <c r="D3367" t="inlineStr">
         <is>
-          <t>EVANESSAS</t>
+          <t>MTANDRADE</t>
         </is>
       </c>
     </row>
     <row r="3368">
       <c r="A3368" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3368" t="n">
-        <v>3360</v>
+        <v>3359</v>
       </c>
       <c r="C3368" t="inlineStr">
         <is>
-          <t>THIAGO DE CARVALHO ARAUJO</t>
+          <t xml:space="preserve">EVANESSA DA SILVA E SILVA </t>
         </is>
       </c>
       <c r="D3368" t="inlineStr">
         <is>
-          <t>TCARAUJO</t>
+          <t>EVANESSAS</t>
         </is>
       </c>
     </row>
     <row r="3369">
       <c r="A3369" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3369" t="n">
-        <v>3481</v>
+        <v>3360</v>
       </c>
       <c r="C3369" t="inlineStr">
         <is>
-          <t xml:space="preserve">EDSON DA PAZ LIMA </t>
+          <t>THIAGO DE CARVALHO ARAUJO</t>
         </is>
       </c>
       <c r="D3369" t="inlineStr">
         <is>
-          <t>EDPAZ</t>
+          <t>TCARAUJO</t>
         </is>
       </c>
     </row>
     <row r="3370">
       <c r="A3370" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3370" t="n">
-        <v>3494</v>
+        <v>3481</v>
       </c>
       <c r="C3370" t="inlineStr">
         <is>
-          <t>ANTONIO CRISTINA BRITO GOMES</t>
+          <t xml:space="preserve">EDSON DA PAZ LIMA </t>
         </is>
       </c>
       <c r="D3370" t="inlineStr">
         <is>
-          <t>CRIS.GOMES</t>
+          <t>EDPAZ</t>
         </is>
       </c>
     </row>
     <row r="3371">
       <c r="A3371" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3371" t="n">
-        <v>3498</v>
+        <v>3494</v>
       </c>
       <c r="C3371" t="inlineStr">
         <is>
-          <t>SILVESTRA COSTA NUNES</t>
+          <t>ANTONIO CRISTINA BRITO GOMES</t>
         </is>
       </c>
       <c r="D3371" t="inlineStr">
         <is>
-          <t>SCNUNES</t>
+          <t>CRIS.GOMES</t>
         </is>
       </c>
     </row>
     <row r="3372">
       <c r="A3372" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3372" t="n">
-        <v>940562</v>
+        <v>3498</v>
       </c>
       <c r="C3372" t="inlineStr">
         <is>
-          <t>FRANCISCO DAVID ASSUNCAO ALVES</t>
+          <t>SILVESTRA COSTA NUNES</t>
         </is>
       </c>
       <c r="D3372" t="inlineStr">
         <is>
-          <t>ASSUNÇÃO</t>
+          <t>SCNUNES</t>
         </is>
       </c>
     </row>
     <row r="3373">
       <c r="A3373" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>99</t>
         </is>
       </c>
       <c r="B3373" t="n">
-        <v>3513</v>
+        <v>940562</v>
       </c>
       <c r="C3373" t="inlineStr">
         <is>
-          <t>RENARA ANDRADE MATIAS</t>
+          <t>FRANCISCO DAVID ASSUNCAO ALVES</t>
         </is>
       </c>
       <c r="D3373" t="inlineStr">
         <is>
-          <t>R.ANDRADE</t>
+          <t>ASSUNÇÃO</t>
         </is>
       </c>
     </row>
     <row r="3374">
       <c r="A3374" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3374" t="n">
-        <v>3275</v>
+        <v>3513</v>
       </c>
       <c r="C3374" t="inlineStr">
         <is>
-          <t>MARIA APARECIDA COELHO SILVA</t>
+          <t>RENARA ANDRADE MATIAS</t>
         </is>
       </c>
       <c r="D3374" t="inlineStr">
         <is>
-          <t>MCOELHO</t>
+          <t>R.ANDRADE</t>
         </is>
       </c>
     </row>
@@ -67918,116 +67918,116 @@
         </is>
       </c>
       <c r="B3375" t="n">
-        <v>3276</v>
+        <v>3275</v>
       </c>
       <c r="C3375" t="inlineStr">
         <is>
-          <t xml:space="preserve">PEROLA DE JESUS AMORIM SOUSA </t>
+          <t>MARIA APARECIDA COELHO SILVA</t>
         </is>
       </c>
       <c r="D3375" t="inlineStr">
         <is>
-          <t>PJESUS</t>
+          <t>MCOELHO</t>
         </is>
       </c>
     </row>
     <row r="3376">
       <c r="A3376" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3376" t="n">
-        <v>3526</v>
+        <v>3276</v>
       </c>
       <c r="C3376" t="inlineStr">
         <is>
-          <t>JOYCE NAZARE CORREA</t>
+          <t xml:space="preserve">PEROLA DE JESUS AMORIM SOUSA </t>
         </is>
       </c>
       <c r="D3376" t="inlineStr">
         <is>
-          <t>J.NAZARE</t>
+          <t>PJESUS</t>
         </is>
       </c>
     </row>
     <row r="3377">
       <c r="A3377" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3377" t="n">
-        <v>3527</v>
+        <v>3526</v>
       </c>
       <c r="C3377" t="inlineStr">
         <is>
-          <t>GILVANA DA SILVA MONTELES</t>
+          <t>JOYCE NAZARE CORREA</t>
         </is>
       </c>
       <c r="D3377" t="inlineStr">
         <is>
-          <t>GIL.SILVA</t>
+          <t>J.NAZARE</t>
         </is>
       </c>
     </row>
     <row r="3378">
       <c r="A3378" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3378" t="n">
-        <v>3548</v>
+        <v>3527</v>
       </c>
       <c r="C3378" t="inlineStr">
         <is>
-          <t>JAMILLY MARIA HENRIQUE ARAUJO</t>
+          <t>GILVANA DA SILVA MONTELES</t>
         </is>
       </c>
       <c r="D3378" t="inlineStr">
         <is>
-          <t>JAMILLY</t>
+          <t>GIL.SILVA</t>
         </is>
       </c>
     </row>
     <row r="3379">
       <c r="A3379" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3379" t="n">
-        <v>3551</v>
+        <v>3548</v>
       </c>
       <c r="C3379" t="inlineStr">
         <is>
-          <t xml:space="preserve">VITOR MANOEL DA SILVA BARBOSA </t>
+          <t>JAMILLY MARIA HENRIQUE ARAUJO</t>
         </is>
       </c>
       <c r="D3379" t="inlineStr">
         <is>
-          <t>VMANOEL</t>
+          <t>JAMILLY</t>
         </is>
       </c>
     </row>
     <row r="3380">
       <c r="A3380" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3380" t="n">
-        <v>940525</v>
+        <v>3551</v>
       </c>
       <c r="C3380" t="inlineStr">
         <is>
-          <t>SANDUWELLINGTON</t>
+          <t xml:space="preserve">VITOR MANOEL DA SILVA BARBOSA </t>
         </is>
       </c>
       <c r="D3380" t="inlineStr">
         <is>
-          <t>SANDUWELLINGTON</t>
+          <t>VMANOEL</t>
         </is>
       </c>
     </row>
@@ -68038,36 +68038,36 @@
         </is>
       </c>
       <c r="B3381" t="n">
-        <v>3369</v>
+        <v>940525</v>
       </c>
       <c r="C3381" t="inlineStr">
         <is>
-          <t xml:space="preserve">PRISCILA DOS SANTOS LOPES </t>
+          <t>SANDUWELLINGTON</t>
         </is>
       </c>
       <c r="D3381" t="inlineStr">
         <is>
-          <t>PSLOPES</t>
+          <t>SANDUWELLINGTON</t>
         </is>
       </c>
     </row>
     <row r="3382">
       <c r="A3382" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3382" t="n">
-        <v>3433</v>
+        <v>3369</v>
       </c>
       <c r="C3382" t="inlineStr">
         <is>
-          <t>BRUNO NUNES CRUZ</t>
+          <t xml:space="preserve">PRISCILA DOS SANTOS LOPES </t>
         </is>
       </c>
       <c r="D3382" t="inlineStr">
         <is>
-          <t>BRUNOCRUZ</t>
+          <t>PSLOPES</t>
         </is>
       </c>
     </row>
@@ -68078,36 +68078,36 @@
         </is>
       </c>
       <c r="B3383" t="n">
-        <v>3434</v>
+        <v>3433</v>
       </c>
       <c r="C3383" t="inlineStr">
         <is>
-          <t>ANA TERCIA DE LIMA SA CARVALHO SERAFIM</t>
+          <t>BRUNO NUNES CRUZ</t>
         </is>
       </c>
       <c r="D3383" t="inlineStr">
         <is>
-          <t>ANATER</t>
+          <t>BRUNOCRUZ</t>
         </is>
       </c>
     </row>
     <row r="3384">
       <c r="A3384" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3384" t="n">
-        <v>3502</v>
+        <v>3434</v>
       </c>
       <c r="C3384" t="inlineStr">
         <is>
-          <t>LUIZ FELIPE MACHADO BARRETO</t>
+          <t>ANA TERCIA DE LIMA SA CARVALHO SERAFIM</t>
         </is>
       </c>
       <c r="D3384" t="inlineStr">
         <is>
-          <t>LUIZ.FELIPE</t>
+          <t>ANATER</t>
         </is>
       </c>
     </row>
@@ -68118,56 +68118,56 @@
         </is>
       </c>
       <c r="B3385" t="n">
-        <v>3503</v>
+        <v>3502</v>
       </c>
       <c r="C3385" t="inlineStr">
         <is>
-          <t>FABIO OLIVEIRA SILVA</t>
+          <t>LUIZ FELIPE MACHADO BARRETO</t>
         </is>
       </c>
       <c r="D3385" t="inlineStr">
         <is>
-          <t>FOSILVA</t>
+          <t>LUIZ.FELIPE</t>
         </is>
       </c>
     </row>
     <row r="3386">
       <c r="A3386" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3386" t="n">
-        <v>3554</v>
+        <v>3503</v>
       </c>
       <c r="C3386" t="inlineStr">
         <is>
-          <t xml:space="preserve">MANOEL RIBEIRO DE SOUZA JUNIOR </t>
+          <t>FABIO OLIVEIRA SILVA</t>
         </is>
       </c>
       <c r="D3386" t="inlineStr">
         <is>
-          <t>MRJUNIOR</t>
+          <t>FOSILVA</t>
         </is>
       </c>
     </row>
     <row r="3387">
       <c r="A3387" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3387" t="n">
-        <v>940549</v>
+        <v>3554</v>
       </c>
       <c r="C3387" t="inlineStr">
         <is>
-          <t>EDILSON ARAUJO - FL9</t>
+          <t xml:space="preserve">MANOEL RIBEIRO DE SOUZA JUNIOR </t>
         </is>
       </c>
       <c r="D3387" t="inlineStr">
         <is>
-          <t>EDILSON</t>
+          <t>MRJUNIOR</t>
         </is>
       </c>
     </row>
@@ -68178,36 +68178,36 @@
         </is>
       </c>
       <c r="B3388" t="n">
-        <v>3470</v>
+        <v>940549</v>
       </c>
       <c r="C3388" t="inlineStr">
         <is>
-          <t>DEBORA ALVES CARVALHO</t>
+          <t>EDILSON ARAUJO - FL9</t>
         </is>
       </c>
       <c r="D3388" t="inlineStr">
         <is>
-          <t>DEBORA.ALVES</t>
+          <t>EDILSON</t>
         </is>
       </c>
     </row>
     <row r="3389">
       <c r="A3389" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3389" t="n">
-        <v>3510</v>
+        <v>3470</v>
       </c>
       <c r="C3389" t="inlineStr">
         <is>
-          <t>CAMILA RODIGUES PINTO</t>
+          <t>DEBORA ALVES CARVALHO</t>
         </is>
       </c>
       <c r="D3389" t="inlineStr">
         <is>
-          <t>MILA.PINTO</t>
+          <t>DEBORA.ALVES</t>
         </is>
       </c>
     </row>
@@ -68218,76 +68218,76 @@
         </is>
       </c>
       <c r="B3390" t="n">
-        <v>3511</v>
+        <v>3510</v>
       </c>
       <c r="C3390" t="inlineStr">
         <is>
-          <t>JORGE HENRIQUE DOS SANTOS RODRIGUES</t>
+          <t>CAMILA RODIGUES PINTO</t>
         </is>
       </c>
       <c r="D3390" t="inlineStr">
         <is>
-          <t>J.HENRIQUE</t>
+          <t>MILA.PINTO</t>
         </is>
       </c>
     </row>
     <row r="3391">
       <c r="A3391" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3391" t="n">
-        <v>3270</v>
+        <v>3511</v>
       </c>
       <c r="C3391" t="inlineStr">
         <is>
-          <t>ITANA NASCIMENTO SIMOES</t>
+          <t>JORGE HENRIQUE DOS SANTOS RODRIGUES</t>
         </is>
       </c>
       <c r="D3391" t="inlineStr">
         <is>
-          <t>ISIMOES</t>
+          <t>J.HENRIQUE</t>
         </is>
       </c>
     </row>
     <row r="3392">
       <c r="A3392" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3392" t="n">
-        <v>3318</v>
+        <v>3561</v>
       </c>
       <c r="C3392" t="inlineStr">
         <is>
-          <t>LUAN MONTEIRO COSTA</t>
+          <t>RONARIA PATRICIA VILARINDO DE ALMEIDA</t>
         </is>
       </c>
       <c r="D3392" t="inlineStr">
         <is>
-          <t>LMONTEIRO</t>
+          <t>RPATRICIA</t>
         </is>
       </c>
     </row>
     <row r="3393">
       <c r="A3393" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3393" t="n">
-        <v>3319</v>
+        <v>3562</v>
       </c>
       <c r="C3393" t="inlineStr">
         <is>
-          <t>MARIANA MACEDA DOS SANTOS</t>
+          <t>LETICIA MARIA BENTO NOGUEIRA</t>
         </is>
       </c>
       <c r="D3393" t="inlineStr">
         <is>
-          <t>MMACEDA</t>
+          <t>LBENTO</t>
         </is>
       </c>
     </row>
@@ -68298,256 +68298,256 @@
         </is>
       </c>
       <c r="B3394" t="n">
-        <v>3389</v>
+        <v>3270</v>
       </c>
       <c r="C3394" t="inlineStr">
         <is>
-          <t>TAMILES DE SANTANA AMORIM BISPO</t>
+          <t>ITANA NASCIMENTO SIMOES</t>
         </is>
       </c>
       <c r="D3394" t="inlineStr">
         <is>
-          <t>TAMILES</t>
+          <t>ISIMOES</t>
         </is>
       </c>
     </row>
     <row r="3395">
       <c r="A3395" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3395" t="n">
-        <v>3390</v>
+        <v>3318</v>
       </c>
       <c r="C3395" t="inlineStr">
         <is>
-          <t>IRACEMA DE ALMEIDA MOURA</t>
+          <t>LUAN MONTEIRO COSTA</t>
         </is>
       </c>
       <c r="D3395" t="inlineStr">
         <is>
-          <t>IRACEMA</t>
+          <t>LMONTEIRO</t>
         </is>
       </c>
     </row>
     <row r="3396">
       <c r="A3396" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3396" t="n">
-        <v>3286</v>
+        <v>3319</v>
       </c>
       <c r="C3396" t="inlineStr">
         <is>
-          <t>VALERIA MAIA DA SILVA</t>
+          <t>MARIANA MACEDA DOS SANTOS</t>
         </is>
       </c>
       <c r="D3396" t="inlineStr">
         <is>
-          <t>VMAIAS</t>
+          <t>MMACEDA</t>
         </is>
       </c>
     </row>
     <row r="3397">
       <c r="A3397" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3397" t="n">
-        <v>3287</v>
+        <v>3389</v>
       </c>
       <c r="C3397" t="inlineStr">
         <is>
-          <t>ERIVELTON DA SILVA OLIVEIRA</t>
+          <t>TAMILES DE SANTANA AMORIM BISPO</t>
         </is>
       </c>
       <c r="D3397" t="inlineStr">
         <is>
-          <t>ESOLIVEIRA</t>
+          <t>TAMILES</t>
         </is>
       </c>
     </row>
     <row r="3398">
       <c r="A3398" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3398" t="n">
-        <v>3307</v>
+        <v>3390</v>
       </c>
       <c r="C3398" t="inlineStr">
         <is>
-          <t>ADRIEL XERES BARROS MARTINS</t>
+          <t>IRACEMA DE ALMEIDA MOURA</t>
         </is>
       </c>
       <c r="D3398" t="inlineStr">
         <is>
-          <t>AXERES</t>
+          <t>IRACEMA</t>
         </is>
       </c>
     </row>
     <row r="3399">
       <c r="A3399" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3399" t="n">
-        <v>3308</v>
+        <v>3286</v>
       </c>
       <c r="C3399" t="inlineStr">
         <is>
-          <t>ELKZIEL JUVINO DA SILVA</t>
+          <t>VALERIA MAIA DA SILVA</t>
         </is>
       </c>
       <c r="D3399" t="inlineStr">
         <is>
-          <t>EJUVINO</t>
+          <t>VMAIAS</t>
         </is>
       </c>
     </row>
     <row r="3400">
       <c r="A3400" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3400" t="n">
-        <v>940539</v>
+        <v>3287</v>
       </c>
       <c r="C3400" t="inlineStr">
         <is>
-          <t>EDSON ARAUJO - FL9</t>
+          <t>ERIVELTON DA SILVA OLIVEIRA</t>
         </is>
       </c>
       <c r="D3400" t="inlineStr">
         <is>
-          <t>EDS</t>
+          <t>ESOLIVEIRA</t>
         </is>
       </c>
     </row>
     <row r="3401">
       <c r="A3401" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3401" t="n">
-        <v>940540</v>
+        <v>3307</v>
       </c>
       <c r="C3401" t="inlineStr">
         <is>
-          <t>EDSON ARAUJO - FL8</t>
+          <t>ADRIEL XERES BARROS MARTINS</t>
         </is>
       </c>
       <c r="D3401" t="inlineStr">
         <is>
-          <t>EDS8</t>
+          <t>AXERES</t>
         </is>
       </c>
     </row>
     <row r="3402">
       <c r="A3402" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3402" t="n">
-        <v>3328</v>
+        <v>3308</v>
       </c>
       <c r="C3402" t="inlineStr">
         <is>
-          <t>ALAN ARAUJO DA SILVA</t>
+          <t>ELKZIEL JUVINO DA SILVA</t>
         </is>
       </c>
       <c r="D3402" t="inlineStr">
         <is>
-          <t>ARSILVA</t>
+          <t>EJUVINO</t>
         </is>
       </c>
     </row>
     <row r="3403">
       <c r="A3403" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3403" t="n">
-        <v>3350</v>
+        <v>940539</v>
       </c>
       <c r="C3403" t="inlineStr">
         <is>
-          <t xml:space="preserve">EDER RODRIGUES DA SILVA </t>
+          <t>EDSON ARAUJO - FL9</t>
         </is>
       </c>
       <c r="D3403" t="inlineStr">
         <is>
-          <t>EDERS</t>
+          <t>EDS</t>
         </is>
       </c>
     </row>
     <row r="3404">
       <c r="A3404" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B3404" t="n">
-        <v>3373</v>
+        <v>940540</v>
       </c>
       <c r="C3404" t="inlineStr">
         <is>
-          <t xml:space="preserve">NATANAEL TAVARES DE SOUSA </t>
+          <t>EDSON ARAUJO - FL8</t>
         </is>
       </c>
       <c r="D3404" t="inlineStr">
         <is>
-          <t>NTSOUSA</t>
+          <t>EDS8</t>
         </is>
       </c>
     </row>
     <row r="3405">
       <c r="A3405" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3405" t="n">
-        <v>3374</v>
+        <v>3328</v>
       </c>
       <c r="C3405" t="inlineStr">
         <is>
-          <t>REINALDO DA SILVA COSTA</t>
+          <t>ALAN ARAUJO DA SILVA</t>
         </is>
       </c>
       <c r="D3405" t="inlineStr">
         <is>
-          <t>RSCOSTA</t>
+          <t>ARSILVA</t>
         </is>
       </c>
     </row>
     <row r="3406">
       <c r="A3406" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3406" t="n">
-        <v>3399</v>
+        <v>3350</v>
       </c>
       <c r="C3406" t="inlineStr">
         <is>
-          <t xml:space="preserve">RICARDO BARBOSA DOS SANTOS </t>
+          <t xml:space="preserve">EDER RODRIGUES DA SILVA </t>
         </is>
       </c>
       <c r="D3406" t="inlineStr">
         <is>
-          <t>RICARDOSAN</t>
+          <t>EDERS</t>
         </is>
       </c>
     </row>
@@ -68558,36 +68558,36 @@
         </is>
       </c>
       <c r="B3407" t="n">
-        <v>3427</v>
+        <v>3373</v>
       </c>
       <c r="C3407" t="inlineStr">
         <is>
-          <t>ROQUE COMERCIO TEMPORARIO</t>
+          <t xml:space="preserve">NATANAEL TAVARES DE SOUSA </t>
         </is>
       </c>
       <c r="D3407" t="inlineStr">
         <is>
-          <t>ROQUECOM</t>
+          <t>NTSOUSA</t>
         </is>
       </c>
     </row>
     <row r="3408">
       <c r="A3408" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3408" t="n">
-        <v>3428</v>
+        <v>3374</v>
       </c>
       <c r="C3408" t="inlineStr">
         <is>
-          <t>ROQUE PLUS TEMPORARIO</t>
+          <t>REINALDO DA SILVA COSTA</t>
         </is>
       </c>
       <c r="D3408" t="inlineStr">
         <is>
-          <t>ROQUEPLUS</t>
+          <t>RSCOSTA</t>
         </is>
       </c>
     </row>
@@ -68598,76 +68598,76 @@
         </is>
       </c>
       <c r="B3409" t="n">
-        <v>3432</v>
+        <v>3399</v>
       </c>
       <c r="C3409" t="inlineStr">
         <is>
-          <t>PATRICIA DOS SANTOS NONATO OLIVEIRA</t>
+          <t xml:space="preserve">RICARDO BARBOSA DOS SANTOS </t>
         </is>
       </c>
       <c r="D3409" t="inlineStr">
         <is>
-          <t>PATRICIAD</t>
+          <t>RICARDOSAN</t>
         </is>
       </c>
     </row>
     <row r="3410">
       <c r="A3410" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3410" t="n">
-        <v>3448</v>
+        <v>3427</v>
       </c>
       <c r="C3410" t="inlineStr">
         <is>
-          <t xml:space="preserve">GABRIEL SOUZA CARVALHO </t>
+          <t>ROQUE COMERCIO TEMPORARIO</t>
         </is>
       </c>
       <c r="D3410" t="inlineStr">
         <is>
-          <t>GABRIEL20</t>
+          <t>ROQUECOM</t>
         </is>
       </c>
     </row>
     <row r="3411">
       <c r="A3411" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3411" t="n">
-        <v>3465</v>
+        <v>3428</v>
       </c>
       <c r="C3411" t="inlineStr">
         <is>
-          <t>LUIZA MARIA BARRETO BARBOSA</t>
+          <t>ROQUE PLUS TEMPORARIO</t>
         </is>
       </c>
       <c r="D3411" t="inlineStr">
         <is>
-          <t>LUIZA.MARIA</t>
+          <t>ROQUEPLUS</t>
         </is>
       </c>
     </row>
     <row r="3412">
       <c r="A3412" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3412" t="n">
-        <v>3468</v>
+        <v>3432</v>
       </c>
       <c r="C3412" t="inlineStr">
         <is>
-          <t>KAWA ALMEIDA CAMPOS</t>
+          <t>PATRICIA DOS SANTOS NONATO OLIVEIRA</t>
         </is>
       </c>
       <c r="D3412" t="inlineStr">
         <is>
-          <t>KAWA</t>
+          <t>PATRICIAD</t>
         </is>
       </c>
     </row>
@@ -68678,436 +68678,436 @@
         </is>
       </c>
       <c r="B3413" t="n">
-        <v>3476</v>
+        <v>3448</v>
       </c>
       <c r="C3413" t="inlineStr">
         <is>
-          <t xml:space="preserve"> FRANCISCA LEIDIANE M. MENDES NASCIMENTO</t>
+          <t xml:space="preserve">GABRIEL SOUZA CARVALHO </t>
         </is>
       </c>
       <c r="D3413" t="inlineStr">
         <is>
-          <t>FLEIDIANE</t>
+          <t>GABRIEL20</t>
         </is>
       </c>
     </row>
     <row r="3414">
       <c r="A3414" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3414" t="n">
-        <v>3477</v>
+        <v>3465</v>
       </c>
       <c r="C3414" t="inlineStr">
         <is>
-          <t>MARIA THAIS MARTINS PEREIRA SILVA</t>
+          <t>LUIZA MARIA BARRETO BARBOSA</t>
         </is>
       </c>
       <c r="D3414" t="inlineStr">
         <is>
-          <t>MTHAIS</t>
+          <t>LUIZA.MARIA</t>
         </is>
       </c>
     </row>
     <row r="3415">
       <c r="A3415" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3415" t="n">
-        <v>3271</v>
+        <v>3468</v>
       </c>
       <c r="C3415" t="inlineStr">
         <is>
-          <t>DIEGO DE ARAUJO CALÁBRIA</t>
+          <t>KAWA ALMEIDA CAMPOS</t>
         </is>
       </c>
       <c r="D3415" t="inlineStr">
         <is>
-          <t>ARAUJOC</t>
+          <t>KAWA</t>
         </is>
       </c>
     </row>
     <row r="3416">
       <c r="A3416" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3416" t="n">
-        <v>3272</v>
+        <v>3476</v>
       </c>
       <c r="C3416" t="inlineStr">
         <is>
-          <t>ANNE BEATRIZ SILVA VIRGINO</t>
+          <t xml:space="preserve"> FRANCISCA LEIDIANE M. MENDES NASCIMENTO</t>
         </is>
       </c>
       <c r="D3416" t="inlineStr">
         <is>
-          <t>ABVIRGINIO</t>
+          <t>FLEIDIANE</t>
         </is>
       </c>
     </row>
     <row r="3417">
       <c r="A3417" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3417" t="n">
-        <v>3293</v>
+        <v>3477</v>
       </c>
       <c r="C3417" t="inlineStr">
         <is>
-          <t xml:space="preserve">CARLOS ALBERTO VIRIATO SANTOS </t>
+          <t>MARIA THAIS MARTINS PEREIRA SILVA</t>
         </is>
       </c>
       <c r="D3417" t="inlineStr">
         <is>
-          <t>CVIRIATO</t>
+          <t>MTHAIS</t>
         </is>
       </c>
     </row>
     <row r="3418">
       <c r="A3418" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3418" t="n">
-        <v>3381</v>
+        <v>3271</v>
       </c>
       <c r="C3418" t="inlineStr">
         <is>
-          <t>ALAN CAIQUE SANTOS E SANTOS</t>
+          <t>DIEGO DE ARAUJO CALÁBRIA</t>
         </is>
       </c>
       <c r="D3418" t="inlineStr">
         <is>
-          <t>ALANSANTOS</t>
+          <t>ARAUJOC</t>
         </is>
       </c>
     </row>
     <row r="3419">
       <c r="A3419" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3419" t="n">
-        <v>3443</v>
+        <v>3272</v>
       </c>
       <c r="C3419" t="inlineStr">
         <is>
-          <t>SANON MOREIRA SOUZA</t>
+          <t>ANNE BEATRIZ SILVA VIRGINO</t>
         </is>
       </c>
       <c r="D3419" t="inlineStr">
         <is>
-          <t>SANON</t>
+          <t>ABVIRGINIO</t>
         </is>
       </c>
     </row>
     <row r="3420">
       <c r="A3420" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3420" t="n">
-        <v>3516</v>
+        <v>3293</v>
       </c>
       <c r="C3420" t="inlineStr">
         <is>
-          <t>FRANCISCO RILDER TELES DE OLIVEIRA</t>
+          <t xml:space="preserve">CARLOS ALBERTO VIRIATO SANTOS </t>
         </is>
       </c>
       <c r="D3420" t="inlineStr">
         <is>
-          <t>RILDER</t>
+          <t>CVIRIATO</t>
         </is>
       </c>
     </row>
     <row r="3421">
       <c r="A3421" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3421" t="n">
-        <v>3519</v>
+        <v>3381</v>
       </c>
       <c r="C3421" t="inlineStr">
         <is>
-          <t>MARIA LUANA DE ALMEIDA BATISTA</t>
+          <t>ALAN CAIQUE SANTOS E SANTOS</t>
         </is>
       </c>
       <c r="D3421" t="inlineStr">
         <is>
-          <t>M.LUANA</t>
+          <t>ALANSANTOS</t>
         </is>
       </c>
     </row>
     <row r="3422">
       <c r="A3422" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3422" t="n">
-        <v>3540</v>
+        <v>3443</v>
       </c>
       <c r="C3422" t="inlineStr">
         <is>
-          <t>HELEN VITORIA OLIVEIRA DA ROCHA</t>
+          <t>SANON MOREIRA SOUZA</t>
         </is>
       </c>
       <c r="D3422" t="inlineStr">
         <is>
-          <t>H.VITORIA</t>
+          <t>SANON</t>
         </is>
       </c>
     </row>
     <row r="3423">
       <c r="A3423" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3423" t="n">
-        <v>3331</v>
+        <v>3516</v>
       </c>
       <c r="C3423" t="inlineStr">
         <is>
-          <t>LOUIZE VANIELLE RODRIGUES FARIAS</t>
+          <t>FRANCISCO RILDER TELES DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D3423" t="inlineStr">
         <is>
-          <t>LVFARIAS</t>
+          <t>RILDER</t>
         </is>
       </c>
     </row>
     <row r="3424">
       <c r="A3424" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3424" t="n">
-        <v>3332</v>
+        <v>3519</v>
       </c>
       <c r="C3424" t="inlineStr">
         <is>
-          <t>ALEXSANDRO PEIXOTO DA VEIGA PACHECO</t>
+          <t>MARIA LUANA DE ALMEIDA BATISTA</t>
         </is>
       </c>
       <c r="D3424" t="inlineStr">
         <is>
-          <t>APVEIGA</t>
+          <t>M.LUANA</t>
         </is>
       </c>
     </row>
     <row r="3425">
       <c r="A3425" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B3425" t="n">
-        <v>3334</v>
+        <v>3540</v>
       </c>
       <c r="C3425" t="inlineStr">
         <is>
-          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+          <t>HELEN VITORIA OLIVEIRA DA ROCHA</t>
         </is>
       </c>
       <c r="D3425" t="inlineStr">
         <is>
-          <t>MTGASPAR</t>
+          <t>H.VITORIA</t>
         </is>
       </c>
     </row>
     <row r="3426">
       <c r="A3426" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3426" t="n">
-        <v>3345</v>
+        <v>3559</v>
       </c>
       <c r="C3426" t="inlineStr">
         <is>
-          <t>AURICÉLIA INACIO PEREIRA</t>
+          <t>ARKBERYS TELES DE SOUSA</t>
         </is>
       </c>
       <c r="D3426" t="inlineStr">
         <is>
-          <t>AIPEREIRA</t>
+          <t>ARKBERYS</t>
         </is>
       </c>
     </row>
     <row r="3427">
       <c r="A3427" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3427" t="n">
-        <v>3363</v>
+        <v>3331</v>
       </c>
       <c r="C3427" t="inlineStr">
         <is>
-          <t>IASMIN LEAL ALVES</t>
+          <t>LOUIZE VANIELLE RODRIGUES FARIAS</t>
         </is>
       </c>
       <c r="D3427" t="inlineStr">
         <is>
-          <t>ILALVES</t>
+          <t>LVFARIAS</t>
         </is>
       </c>
     </row>
     <row r="3428">
       <c r="A3428" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3428" t="n">
-        <v>3370</v>
+        <v>3334</v>
       </c>
       <c r="C3428" t="inlineStr">
         <is>
-          <t>CARLOS DIEGO ARAUJO ALMEIDA</t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
       <c r="D3428" t="inlineStr">
         <is>
-          <t>CDIEGO</t>
+          <t>MTGASPAR</t>
         </is>
       </c>
     </row>
     <row r="3429">
       <c r="A3429" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3429" t="n">
-        <v>3379</v>
+        <v>3345</v>
       </c>
       <c r="C3429" t="inlineStr">
         <is>
-          <t xml:space="preserve">MATHEUS EVANGELISTA FERREIRA </t>
+          <t>AURICÉLIA INACIO PEREIRA</t>
         </is>
       </c>
       <c r="D3429" t="inlineStr">
         <is>
-          <t>MMFERREIRA</t>
+          <t>AIPEREIRA</t>
         </is>
       </c>
     </row>
     <row r="3430">
       <c r="A3430" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3430" t="n">
-        <v>3419</v>
+        <v>3363</v>
       </c>
       <c r="C3430" t="inlineStr">
         <is>
-          <t xml:space="preserve">DAVID EVANGELISTA SILVA </t>
+          <t>IASMIN LEAL ALVES</t>
         </is>
       </c>
       <c r="D3430" t="inlineStr">
         <is>
-          <t>DAVID</t>
+          <t>ILALVES</t>
         </is>
       </c>
     </row>
     <row r="3431">
       <c r="A3431" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3431" t="n">
-        <v>3423</v>
+        <v>3370</v>
       </c>
       <c r="C3431" t="inlineStr">
         <is>
-          <t>MARCIO JOSE TIAGO</t>
+          <t>CARLOS DIEGO ARAUJO ALMEIDA</t>
         </is>
       </c>
       <c r="D3431" t="inlineStr">
         <is>
-          <t>MJTIAGO</t>
+          <t>CDIEGO</t>
         </is>
       </c>
     </row>
     <row r="3432">
       <c r="A3432" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3432" t="n">
-        <v>3453</v>
+        <v>3379</v>
       </c>
       <c r="C3432" t="inlineStr">
         <is>
-          <t xml:space="preserve">LAURIENE SILVA BARBOSA </t>
+          <t xml:space="preserve">MATHEUS EVANGELISTA FERREIRA </t>
         </is>
       </c>
       <c r="D3432" t="inlineStr">
         <is>
-          <t>LAURIENE</t>
+          <t>MMFERREIRA</t>
         </is>
       </c>
     </row>
     <row r="3433">
       <c r="A3433" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3433" t="n">
-        <v>3478</v>
+        <v>3419</v>
       </c>
       <c r="C3433" t="inlineStr">
         <is>
-          <t>LEANDRO BRITO NOGUEIRA DE OLIVEIRA</t>
+          <t xml:space="preserve">DAVID EVANGELISTA SILVA </t>
         </is>
       </c>
       <c r="D3433" t="inlineStr">
         <is>
-          <t>LBNOGUEIRA</t>
+          <t>DAVID</t>
         </is>
       </c>
     </row>
     <row r="3434">
       <c r="A3434" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3434" t="n">
-        <v>3479</v>
+        <v>3423</v>
       </c>
       <c r="C3434" t="inlineStr">
         <is>
-          <t>ESDRAS ALESSANDRO SANTOS SANTANA</t>
+          <t>MARCIO JOSE TIAGO</t>
         </is>
       </c>
       <c r="D3434" t="inlineStr">
         <is>
-          <t>EALESSANDRO</t>
+          <t>MJTIAGO</t>
         </is>
       </c>
     </row>
@@ -69118,456 +69118,456 @@
         </is>
       </c>
       <c r="B3435" t="n">
-        <v>3480</v>
+        <v>3453</v>
       </c>
       <c r="C3435" t="inlineStr">
         <is>
-          <t xml:space="preserve">LUCIMARA SOUSA LIMA </t>
+          <t xml:space="preserve">LAURIENE SILVA BARBOSA </t>
         </is>
       </c>
       <c r="D3435" t="inlineStr">
         <is>
-          <t>LUCIMARA</t>
+          <t>LAURIENE</t>
         </is>
       </c>
     </row>
     <row r="3436">
       <c r="A3436" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3436" t="n">
-        <v>3482</v>
+        <v>3478</v>
       </c>
       <c r="C3436" t="inlineStr">
         <is>
-          <t>DANIEL FERNANDES DINIZ HERACLIO</t>
+          <t>LEANDRO BRITO NOGUEIRA DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D3436" t="inlineStr">
         <is>
-          <t>DFDINIZ</t>
+          <t>LBNOGUEIRA</t>
         </is>
       </c>
     </row>
     <row r="3437">
       <c r="A3437" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3437" t="n">
-        <v>3518</v>
+        <v>3479</v>
       </c>
       <c r="C3437" t="inlineStr">
         <is>
-          <t>RAMYRA ALVES FELIX DA SILVA</t>
+          <t>ESDRAS ALESSANDRO SANTOS SANTANA</t>
         </is>
       </c>
       <c r="D3437" t="inlineStr">
         <is>
-          <t>RFELIX</t>
+          <t>EALESSANDRO</t>
         </is>
       </c>
     </row>
     <row r="3438">
       <c r="A3438" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3438" t="n">
-        <v>3534</v>
+        <v>3480</v>
       </c>
       <c r="C3438" t="inlineStr">
         <is>
-          <t xml:space="preserve">CAIO DE SOUZA VINHAS </t>
+          <t xml:space="preserve">LUCIMARA SOUSA LIMA </t>
         </is>
       </c>
       <c r="D3438" t="inlineStr">
         <is>
-          <t>CVINHAS</t>
+          <t>LUCIMARA</t>
         </is>
       </c>
     </row>
     <row r="3439">
       <c r="A3439" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3439" t="n">
-        <v>3535</v>
+        <v>3482</v>
       </c>
       <c r="C3439" t="inlineStr">
         <is>
-          <t>ROMARIO DE SOUSA SILVA</t>
+          <t>DANIEL FERNANDES DINIZ HERACLIO</t>
         </is>
       </c>
       <c r="D3439" t="inlineStr">
         <is>
-          <t>RSOUSAS</t>
+          <t>DFDINIZ</t>
         </is>
       </c>
     </row>
     <row r="3440">
       <c r="A3440" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3440" t="n">
-        <v>3536</v>
+        <v>3518</v>
       </c>
       <c r="C3440" t="inlineStr">
         <is>
-          <t>JHONATAS CARVALHO OLIVEIRA</t>
+          <t>RAMYRA ALVES FELIX DA SILVA</t>
         </is>
       </c>
       <c r="D3440" t="inlineStr">
         <is>
-          <t>JHONATASC</t>
+          <t>RFELIX</t>
         </is>
       </c>
     </row>
     <row r="3441">
       <c r="A3441" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3441" t="n">
-        <v>940529</v>
+        <v>3534</v>
       </c>
       <c r="C3441" t="inlineStr">
         <is>
-          <t>EDGAR FELIX - FL9</t>
+          <t xml:space="preserve">CAIO DE SOUZA VINHAS </t>
         </is>
       </c>
       <c r="D3441" t="inlineStr">
         <is>
-          <t>EDGAR F</t>
+          <t>CVINHAS</t>
         </is>
       </c>
     </row>
     <row r="3442">
       <c r="A3442" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3442" t="n">
-        <v>3304</v>
+        <v>3535</v>
       </c>
       <c r="C3442" t="inlineStr">
         <is>
-          <t>JOACI GUILHERME GONÇALVES DA LUZ</t>
+          <t>ROMARIO DE SOUSA SILVA</t>
         </is>
       </c>
       <c r="D3442" t="inlineStr">
         <is>
-          <t>JLUZ</t>
+          <t>RSOUSAS</t>
         </is>
       </c>
     </row>
     <row r="3443">
       <c r="A3443" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3443" t="n">
-        <v>3305</v>
+        <v>3536</v>
       </c>
       <c r="C3443" t="inlineStr">
         <is>
-          <t>JOÃO VITOR DE ARAÚJO GONÇALVES</t>
+          <t>JHONATAS CARVALHO OLIVEIRA</t>
         </is>
       </c>
       <c r="D3443" t="inlineStr">
         <is>
-          <t>JJVITOR</t>
+          <t>JHONATASC</t>
         </is>
       </c>
     </row>
     <row r="3444">
       <c r="A3444" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3444" t="n">
-        <v>3306</v>
+        <v>940529</v>
       </c>
       <c r="C3444" t="inlineStr">
         <is>
-          <t>WENDERSON MARCOS DOS SANTOS</t>
+          <t>EDGAR FELIX - FL9</t>
         </is>
       </c>
       <c r="D3444" t="inlineStr">
         <is>
-          <t>WWMARCOS</t>
+          <t>EDGAR F</t>
         </is>
       </c>
     </row>
     <row r="3445">
       <c r="A3445" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3445" t="n">
-        <v>3335</v>
+        <v>3304</v>
       </c>
       <c r="C3445" t="inlineStr">
         <is>
-          <t>EDILBERTO LEMOS DE LIMA</t>
+          <t>JOACI GUILHERME GONÇALVES DA LUZ</t>
         </is>
       </c>
       <c r="D3445" t="inlineStr">
         <is>
-          <t>ELEMOS</t>
+          <t>JLUZ</t>
         </is>
       </c>
     </row>
     <row r="3446">
       <c r="A3446" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3446" t="n">
-        <v>3336</v>
+        <v>3305</v>
       </c>
       <c r="C3446" t="inlineStr">
         <is>
-          <t>EZEQUIEL SOUZA DO NASCIMENTO</t>
+          <t>JOÃO VITOR DE ARAÚJO GONÇALVES</t>
         </is>
       </c>
       <c r="D3446" t="inlineStr">
         <is>
-          <t>ESNASCIMENTO</t>
+          <t>JJVITOR</t>
         </is>
       </c>
     </row>
     <row r="3447">
       <c r="A3447" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3447" t="n">
-        <v>3341</v>
+        <v>3306</v>
       </c>
       <c r="C3447" t="inlineStr">
         <is>
-          <t>ALCIONE MARIANO DE OLIVEIRA</t>
+          <t>WENDERSON MARCOS DOS SANTOS</t>
         </is>
       </c>
       <c r="D3447" t="inlineStr">
         <is>
-          <t>AMOLIVEIRA</t>
+          <t>WWMARCOS</t>
         </is>
       </c>
     </row>
     <row r="3448">
       <c r="A3448" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3448" t="n">
-        <v>3401</v>
+        <v>3335</v>
       </c>
       <c r="C3448" t="inlineStr">
         <is>
-          <t xml:space="preserve">TULIO HENRIQUE DA SILVA CARVALHO </t>
+          <t>EDILBERTO LEMOS DE LIMA</t>
         </is>
       </c>
       <c r="D3448" t="inlineStr">
         <is>
-          <t>TULIO</t>
+          <t>ELEMOS</t>
         </is>
       </c>
     </row>
     <row r="3449">
       <c r="A3449" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3449" t="n">
-        <v>3411</v>
+        <v>3336</v>
       </c>
       <c r="C3449" t="inlineStr">
         <is>
-          <t>CONEXAO RUBYA DANILLA</t>
+          <t>EZEQUIEL SOUZA DO NASCIMENTO</t>
         </is>
       </c>
       <c r="D3449" t="inlineStr">
         <is>
-          <t>CONEXAORUBYA</t>
+          <t>ESNASCIMENTO</t>
         </is>
       </c>
     </row>
     <row r="3450">
       <c r="A3450" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3450" t="n">
-        <v>3412</v>
+        <v>3341</v>
       </c>
       <c r="C3450" t="inlineStr">
         <is>
-          <t>CONEXAO RAFAEL</t>
+          <t>ALCIONE MARIANO DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D3450" t="inlineStr">
         <is>
-          <t>CONEXAORAFAEL</t>
+          <t>AMOLIVEIRA</t>
         </is>
       </c>
     </row>
     <row r="3451">
       <c r="A3451" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3451" t="n">
-        <v>3558</v>
+        <v>3401</v>
       </c>
       <c r="C3451" t="inlineStr">
         <is>
-          <t>WALLYS QUEIROZ VIANA</t>
+          <t xml:space="preserve">TULIO HENRIQUE DA SILVA CARVALHO </t>
         </is>
       </c>
       <c r="D3451" t="inlineStr">
         <is>
-          <t>WALLYS</t>
+          <t>TULIO</t>
         </is>
       </c>
     </row>
     <row r="3452">
       <c r="A3452" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3452" t="n">
-        <v>3264</v>
+        <v>3411</v>
       </c>
       <c r="C3452" t="inlineStr">
         <is>
-          <t xml:space="preserve">WILTON CARLOS MACIEL DE ASSIS </t>
+          <t>CONEXAO RUBYA DANILLA</t>
         </is>
       </c>
       <c r="D3452" t="inlineStr">
         <is>
-          <t>WCMACIEL</t>
+          <t>CONEXAORUBYA</t>
         </is>
       </c>
     </row>
     <row r="3453">
       <c r="A3453" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3453" t="n">
-        <v>3340</v>
+        <v>3412</v>
       </c>
       <c r="C3453" t="inlineStr">
         <is>
-          <t>ROGELENO FARIAS FEIJÃO FILHO</t>
+          <t>CONEXAO RAFAEL</t>
         </is>
       </c>
       <c r="D3453" t="inlineStr">
         <is>
-          <t>RFEIJAO</t>
+          <t>CONEXAORAFAEL</t>
         </is>
       </c>
     </row>
     <row r="3454">
       <c r="A3454" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3454" t="n">
-        <v>940550</v>
+        <v>3558</v>
       </c>
       <c r="C3454" t="inlineStr">
         <is>
-          <t>RAFAELE RIBEIRO CARNEIRO</t>
+          <t>WALLYS QUEIROZ VIANA</t>
         </is>
       </c>
       <c r="D3454" t="inlineStr">
         <is>
-          <t>RAFAELE</t>
+          <t>WALLYS</t>
         </is>
       </c>
     </row>
     <row r="3455">
       <c r="A3455" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3455" t="n">
-        <v>3377</v>
+        <v>3264</v>
       </c>
       <c r="C3455" t="inlineStr">
         <is>
-          <t xml:space="preserve"> ISALTINO BISPO DE OLIVEIRA JUNIOR</t>
+          <t xml:space="preserve">WILTON CARLOS MACIEL DE ASSIS </t>
         </is>
       </c>
       <c r="D3455" t="inlineStr">
         <is>
-          <t>BJUNIOR</t>
+          <t>WCMACIEL</t>
         </is>
       </c>
     </row>
     <row r="3456">
       <c r="A3456" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3456" t="n">
-        <v>3425</v>
+        <v>3340</v>
       </c>
       <c r="C3456" t="inlineStr">
         <is>
-          <t xml:space="preserve"> CIRLANE ARAUJO SOUZA </t>
+          <t>ROGELENO FARIAS FEIJÃO FILHO</t>
         </is>
       </c>
       <c r="D3456" t="inlineStr">
         <is>
-          <t>CIRLANES</t>
+          <t>RFEIJAO</t>
         </is>
       </c>
     </row>
     <row r="3457">
       <c r="A3457" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>99</t>
         </is>
       </c>
       <c r="B3457" t="n">
-        <v>3454</v>
+        <v>940550</v>
       </c>
       <c r="C3457" t="inlineStr">
         <is>
-          <t>ANTONIA SAMARA DE SOUZA SOARES</t>
+          <t>RAFAELE RIBEIRO CARNEIRO</t>
         </is>
       </c>
       <c r="D3457" t="inlineStr">
         <is>
-          <t>ANTSAMARA</t>
+          <t>RAFAELE</t>
         </is>
       </c>
     </row>
@@ -69578,16 +69578,16 @@
         </is>
       </c>
       <c r="B3458" t="n">
-        <v>3491</v>
+        <v>3377</v>
       </c>
       <c r="C3458" t="inlineStr">
         <is>
-          <t>PEDRO JOSE DO NASCIMENTO NETO</t>
+          <t xml:space="preserve"> ISALTINO BISPO DE OLIVEIRA JUNIOR</t>
         </is>
       </c>
       <c r="D3458" t="inlineStr">
         <is>
-          <t>P.JOSE</t>
+          <t>BJUNIOR</t>
         </is>
       </c>
     </row>
@@ -69598,76 +69598,76 @@
         </is>
       </c>
       <c r="B3459" t="n">
-        <v>3492</v>
+        <v>3425</v>
       </c>
       <c r="C3459" t="inlineStr">
         <is>
-          <t>PAULA CARLA CALDAS MOTA</t>
+          <t xml:space="preserve"> CIRLANE ARAUJO SOUZA </t>
         </is>
       </c>
       <c r="D3459" t="inlineStr">
         <is>
-          <t>P.CARLA</t>
+          <t>CIRLANES</t>
         </is>
       </c>
     </row>
     <row r="3460">
       <c r="A3460" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3460" t="n">
-        <v>3542</v>
+        <v>3454</v>
       </c>
       <c r="C3460" t="inlineStr">
         <is>
-          <t>ANTONIA MILENA SOUSA ANDRADE</t>
+          <t>ANTONIA SAMARA DE SOUZA SOARES</t>
         </is>
       </c>
       <c r="D3460" t="inlineStr">
         <is>
-          <t>A.MILENA</t>
+          <t>ANTSAMARA</t>
         </is>
       </c>
     </row>
     <row r="3461">
       <c r="A3461" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3461" t="n">
-        <v>3547</v>
+        <v>3491</v>
       </c>
       <c r="C3461" t="inlineStr">
         <is>
-          <t xml:space="preserve">DAVI PEREIRA DA SILVA </t>
+          <t>PEDRO JOSE DO NASCIMENTO NETO</t>
         </is>
       </c>
       <c r="D3461" t="inlineStr">
         <is>
-          <t>DPSILVA</t>
+          <t>P.JOSE</t>
         </is>
       </c>
     </row>
     <row r="3462">
       <c r="A3462" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3462" t="n">
-        <v>3552</v>
+        <v>3492</v>
       </c>
       <c r="C3462" t="inlineStr">
         <is>
-          <t>PAULO SERGIO MENDES DE OLIVEIRA</t>
+          <t>PAULA CARLA CALDAS MOTA</t>
         </is>
       </c>
       <c r="D3462" t="inlineStr">
         <is>
-          <t>PSMENDES</t>
+          <t>P.CARLA</t>
         </is>
       </c>
     </row>
@@ -69678,16 +69678,16 @@
         </is>
       </c>
       <c r="B3463" t="n">
-        <v>3294</v>
+        <v>3542</v>
       </c>
       <c r="C3463" t="inlineStr">
         <is>
-          <t>GLEICIANE MIRANDA DE MORAIS</t>
+          <t>ANTONIA MILENA SOUSA ANDRADE</t>
         </is>
       </c>
       <c r="D3463" t="inlineStr">
         <is>
-          <t>GMIRANDA</t>
+          <t>A.MILENA</t>
         </is>
       </c>
     </row>
@@ -69698,16 +69698,16 @@
         </is>
       </c>
       <c r="B3464" t="n">
-        <v>3295</v>
+        <v>3547</v>
       </c>
       <c r="C3464" t="inlineStr">
         <is>
-          <t>MARIA ESTEFANNY DA SILVA MOURA</t>
+          <t xml:space="preserve">DAVI PEREIRA DA SILVA </t>
         </is>
       </c>
       <c r="D3464" t="inlineStr">
         <is>
-          <t>MESTEFANNY</t>
+          <t>DPSILVA</t>
         </is>
       </c>
     </row>
@@ -69718,36 +69718,36 @@
         </is>
       </c>
       <c r="B3465" t="n">
-        <v>3296</v>
+        <v>3552</v>
       </c>
       <c r="C3465" t="inlineStr">
         <is>
-          <t>PEDRO IAGO FONSECA EVANGELISTA</t>
+          <t>PAULO SERGIO MENDES DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D3465" t="inlineStr">
         <is>
-          <t>PIFONSECA</t>
+          <t>PSMENDES</t>
         </is>
       </c>
     </row>
     <row r="3466">
       <c r="A3466" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3466" t="n">
-        <v>940544</v>
+        <v>3294</v>
       </c>
       <c r="C3466" t="inlineStr">
         <is>
-          <t>LUTY LOG TRANSPORTES - FL8</t>
+          <t>GLEICIANE MIRANDA DE MORAIS</t>
         </is>
       </c>
       <c r="D3466" t="inlineStr">
         <is>
-          <t>LUTY LOG</t>
+          <t>GMIRANDA</t>
         </is>
       </c>
     </row>
@@ -69758,96 +69758,96 @@
         </is>
       </c>
       <c r="B3467" t="n">
-        <v>3380</v>
+        <v>3295</v>
       </c>
       <c r="C3467" t="inlineStr">
         <is>
-          <t>FRANCISCO MATHEUS RABELO DA COSTA</t>
+          <t>MARIA ESTEFANNY DA SILVA MOURA</t>
         </is>
       </c>
       <c r="D3467" t="inlineStr">
         <is>
-          <t>FMATHEUS</t>
+          <t>MESTEFANNY</t>
         </is>
       </c>
     </row>
     <row r="3468">
       <c r="A3468" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3468" t="n">
-        <v>3410</v>
+        <v>3296</v>
       </c>
       <c r="C3468" t="inlineStr">
         <is>
-          <t xml:space="preserve"> BRENO ALLAN DE JESUS</t>
+          <t>PEDRO IAGO FONSECA EVANGELISTA</t>
         </is>
       </c>
       <c r="D3468" t="inlineStr">
         <is>
-          <t>JESUS</t>
+          <t>PIFONSECA</t>
         </is>
       </c>
     </row>
     <row r="3469">
       <c r="A3469" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B3469" t="n">
-        <v>3444</v>
+        <v>940544</v>
       </c>
       <c r="C3469" t="inlineStr">
         <is>
-          <t>THIAGO COSTA SILVA</t>
+          <t>LUTY LOG TRANSPORTES - FL8</t>
         </is>
       </c>
       <c r="D3469" t="inlineStr">
         <is>
-          <t>THIAGOC</t>
+          <t>LUTY LOG</t>
         </is>
       </c>
     </row>
     <row r="3470">
       <c r="A3470" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3470" t="n">
-        <v>3456</v>
+        <v>3380</v>
       </c>
       <c r="C3470" t="inlineStr">
         <is>
-          <t>FELIPE BOTH MAZUCHINI</t>
+          <t>FRANCISCO MATHEUS RABELO DA COSTA</t>
         </is>
       </c>
       <c r="D3470" t="inlineStr">
         <is>
-          <t>FELIPEB</t>
+          <t>FMATHEUS</t>
         </is>
       </c>
     </row>
     <row r="3471">
       <c r="A3471" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3471" t="n">
-        <v>3457</v>
+        <v>3410</v>
       </c>
       <c r="C3471" t="inlineStr">
         <is>
-          <t>FRANKLIN VIEIRA GOMES</t>
+          <t xml:space="preserve"> BRENO ALLAN DE JESUS</t>
         </is>
       </c>
       <c r="D3471" t="inlineStr">
         <is>
-          <t>VIEIRAF</t>
+          <t>JESUS</t>
         </is>
       </c>
     </row>
@@ -69858,34 +69858,94 @@
         </is>
       </c>
       <c r="B3472" t="n">
-        <v>3507</v>
+        <v>3444</v>
       </c>
       <c r="C3472" t="inlineStr">
         <is>
-          <t>KARINE TEODORA ALVES DE OLIVEIRA</t>
+          <t>THIAGO COSTA SILVA</t>
         </is>
       </c>
       <c r="D3472" t="inlineStr">
         <is>
-          <t>KOLIVEIRA</t>
+          <t>THIAGOC</t>
         </is>
       </c>
     </row>
     <row r="3473">
       <c r="A3473" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B3473" t="n">
+        <v>3456</v>
+      </c>
+      <c r="C3473" t="inlineStr">
+        <is>
+          <t>FELIPE BOTH MAZUCHINI</t>
+        </is>
+      </c>
+      <c r="D3473" t="inlineStr">
+        <is>
+          <t>FELIPEB</t>
+        </is>
+      </c>
+    </row>
+    <row r="3474">
+      <c r="A3474" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B3474" t="n">
+        <v>3457</v>
+      </c>
+      <c r="C3474" t="inlineStr">
+        <is>
+          <t>FRANKLIN VIEIRA GOMES</t>
+        </is>
+      </c>
+      <c r="D3474" t="inlineStr">
+        <is>
+          <t>VIEIRAF</t>
+        </is>
+      </c>
+    </row>
+    <row r="3475">
+      <c r="A3475" t="inlineStr">
+        <is>
           <t>5</t>
         </is>
       </c>
-      <c r="B3473" t="n">
+      <c r="B3475" t="n">
+        <v>3507</v>
+      </c>
+      <c r="C3475" t="inlineStr">
+        <is>
+          <t>KARINE TEODORA ALVES DE OLIVEIRA</t>
+        </is>
+      </c>
+      <c r="D3475" t="inlineStr">
+        <is>
+          <t>KOLIVEIRA</t>
+        </is>
+      </c>
+    </row>
+    <row r="3476">
+      <c r="A3476" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B3476" t="n">
         <v>3520</v>
       </c>
-      <c r="C3473" t="inlineStr">
+      <c r="C3476" t="inlineStr">
         <is>
           <t xml:space="preserve"> EMERSON FILIPE MELO DE AGUIAR</t>
         </is>
       </c>
-      <c r="D3473" t="inlineStr">
+      <c r="D3476" t="inlineStr">
         <is>
           <t>E.FILIPE</t>
         </is>

</xml_diff>

<commit_message>
chore(data): batch update intraday televendas - 08:01:28
</commit_message>
<xml_diff>
--- a/data/dim_televendas.xlsx
+++ b/data/dim_televendas.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3479"/>
+  <dimension ref="A1:D3481"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23054,7 +23054,7 @@
     <row r="1132">
       <c r="A1132" t="inlineStr">
         <is>
-          <t>9999</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B1132" t="n">
@@ -66854,120 +66854,120 @@
     <row r="3322">
       <c r="A3322" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3322" t="n">
-        <v>940541</v>
+        <v>3566</v>
       </c>
       <c r="C3322" t="inlineStr">
         <is>
-          <t>JOSE AMSTERDA TEIXEIRA DE MENEZES</t>
+          <t xml:space="preserve">WESLEY HENRIQUE ALVES DOS SANTOS </t>
         </is>
       </c>
       <c r="D3322" t="inlineStr">
         <is>
-          <t>AMSTERDA</t>
+          <t>W.ALVES</t>
         </is>
       </c>
     </row>
     <row r="3323">
       <c r="A3323" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>99</t>
         </is>
       </c>
       <c r="B3323" t="n">
-        <v>940554</v>
+        <v>940541</v>
       </c>
       <c r="C3323" t="inlineStr">
         <is>
-          <t>ALEXANDRE ALVES DE FREITAS</t>
+          <t>JOSE AMSTERDA TEIXEIRA DE MENEZES</t>
         </is>
       </c>
       <c r="D3323" t="inlineStr">
         <is>
-          <t>ALEXANDRE</t>
+          <t>AMSTERDA</t>
         </is>
       </c>
     </row>
     <row r="3324">
       <c r="A3324" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3324" t="n">
-        <v>3402</v>
+        <v>940554</v>
       </c>
       <c r="C3324" t="inlineStr">
         <is>
-          <t xml:space="preserve">VINICIUS GUEDES DA SILVA </t>
+          <t>ALEXANDRE ALVES DE FREITAS</t>
         </is>
       </c>
       <c r="D3324" t="inlineStr">
         <is>
-          <t>GUEDES5</t>
+          <t>ALEXANDRE</t>
         </is>
       </c>
     </row>
     <row r="3325">
       <c r="A3325" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3325" t="n">
-        <v>3467</v>
+        <v>3402</v>
       </c>
       <c r="C3325" t="inlineStr">
         <is>
-          <t>CILENE FERREIRA DA SILVA</t>
+          <t xml:space="preserve">VINICIUS GUEDES DA SILVA </t>
         </is>
       </c>
       <c r="D3325" t="inlineStr">
         <is>
-          <t>CILENE</t>
+          <t>GUEDES5</t>
         </is>
       </c>
     </row>
     <row r="3326">
       <c r="A3326" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3326" t="n">
-        <v>3495</v>
+        <v>3467</v>
       </c>
       <c r="C3326" t="inlineStr">
         <is>
-          <t>LUCILENE SANTOS DE MELO DAMASCENA</t>
+          <t>CILENE FERREIRA DA SILVA</t>
         </is>
       </c>
       <c r="D3326" t="inlineStr">
         <is>
-          <t>LUCILENE21</t>
+          <t>CILENE</t>
         </is>
       </c>
     </row>
     <row r="3327">
       <c r="A3327" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3327" t="n">
-        <v>3496</v>
+        <v>3495</v>
       </c>
       <c r="C3327" t="inlineStr">
         <is>
-          <t>JOAO PEDRO HENRIQUE ALVES DE ARAUJO</t>
+          <t>LUCILENE SANTOS DE MELO DAMASCENA</t>
         </is>
       </c>
       <c r="D3327" t="inlineStr">
         <is>
-          <t>JOAO.PEDRO</t>
+          <t>LUCILENE21</t>
         </is>
       </c>
     </row>
@@ -66978,16 +66978,16 @@
         </is>
       </c>
       <c r="B3328" t="n">
-        <v>3497</v>
+        <v>3496</v>
       </c>
       <c r="C3328" t="inlineStr">
         <is>
-          <t>ORLANDO MONTEIRO DE AMORIM</t>
+          <t>JOAO PEDRO HENRIQUE ALVES DE ARAUJO</t>
         </is>
       </c>
       <c r="D3328" t="inlineStr">
         <is>
-          <t>ORLANDO</t>
+          <t>JOAO.PEDRO</t>
         </is>
       </c>
     </row>
@@ -66998,16 +66998,16 @@
         </is>
       </c>
       <c r="B3329" t="n">
-        <v>3538</v>
+        <v>3497</v>
       </c>
       <c r="C3329" t="inlineStr">
         <is>
-          <t>PAULO HENRIQUE BENTO DA SILVA</t>
+          <t>ORLANDO MONTEIRO DE AMORIM</t>
         </is>
       </c>
       <c r="D3329" t="inlineStr">
         <is>
-          <t>P.BENTO</t>
+          <t>ORLANDO</t>
         </is>
       </c>
     </row>
@@ -67018,96 +67018,96 @@
         </is>
       </c>
       <c r="B3330" t="n">
-        <v>3303</v>
+        <v>3538</v>
       </c>
       <c r="C3330" t="inlineStr">
         <is>
-          <t>DANIEL ALVES RODRIGUES</t>
+          <t>PAULO HENRIQUE BENTO DA SILVA</t>
         </is>
       </c>
       <c r="D3330" t="inlineStr">
         <is>
-          <t>DARODRIGUES</t>
+          <t>P.BENTO</t>
         </is>
       </c>
     </row>
     <row r="3331">
       <c r="A3331" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3331" t="n">
-        <v>3316</v>
+        <v>3303</v>
       </c>
       <c r="C3331" t="inlineStr">
         <is>
-          <t xml:space="preserve">MARCELO PEREIRA BASTOS </t>
+          <t>DANIEL ALVES RODRIGUES</t>
         </is>
       </c>
       <c r="D3331" t="inlineStr">
         <is>
-          <t>MBASTOS</t>
+          <t>DARODRIGUES</t>
         </is>
       </c>
     </row>
     <row r="3332">
       <c r="A3332" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3332" t="n">
-        <v>3366</v>
+        <v>3316</v>
       </c>
       <c r="C3332" t="inlineStr">
         <is>
-          <t>MATEUS TEIXEIRA DA PAZ SILVA</t>
+          <t xml:space="preserve">MARCELO PEREIRA BASTOS </t>
         </is>
       </c>
       <c r="D3332" t="inlineStr">
         <is>
-          <t>PAZSILVA</t>
+          <t>MBASTOS</t>
         </is>
       </c>
     </row>
     <row r="3333">
       <c r="A3333" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3333" t="n">
-        <v>3393</v>
+        <v>3366</v>
       </c>
       <c r="C3333" t="inlineStr">
         <is>
-          <t xml:space="preserve">DAVID LUCAS RIBEIRO DOS SANTOS </t>
+          <t>MATEUS TEIXEIRA DA PAZ SILVA</t>
         </is>
       </c>
       <c r="D3333" t="inlineStr">
         <is>
-          <t>DLUCAS</t>
+          <t>PAZSILVA</t>
         </is>
       </c>
     </row>
     <row r="3334">
       <c r="A3334" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3334" t="n">
-        <v>3420</v>
+        <v>3393</v>
       </c>
       <c r="C3334" t="inlineStr">
         <is>
-          <t xml:space="preserve">CLAUDIO ROBERTO SILVA SOUZA </t>
+          <t xml:space="preserve">DAVID LUCAS RIBEIRO DOS SANTOS </t>
         </is>
       </c>
       <c r="D3334" t="inlineStr">
         <is>
-          <t>CLAUDIO21</t>
+          <t>DLUCAS</t>
         </is>
       </c>
     </row>
@@ -67118,16 +67118,16 @@
         </is>
       </c>
       <c r="B3335" t="n">
-        <v>3421</v>
+        <v>3420</v>
       </c>
       <c r="C3335" t="inlineStr">
         <is>
-          <t>WILSON PORTUGAL AZEVEDO FILHO</t>
+          <t xml:space="preserve">CLAUDIO ROBERTO SILVA SOUZA </t>
         </is>
       </c>
       <c r="D3335" t="inlineStr">
         <is>
-          <t>WILSONF</t>
+          <t>CLAUDIO21</t>
         </is>
       </c>
     </row>
@@ -67138,156 +67138,156 @@
         </is>
       </c>
       <c r="B3336" t="n">
-        <v>3439</v>
+        <v>3421</v>
       </c>
       <c r="C3336" t="inlineStr">
         <is>
-          <t>FERNANDA MASCARENHAS CEDRAZ</t>
+          <t>WILSON PORTUGAL AZEVEDO FILHO</t>
         </is>
       </c>
       <c r="D3336" t="inlineStr">
         <is>
-          <t>FERNANDAM</t>
+          <t>WILSONF</t>
         </is>
       </c>
     </row>
     <row r="3337">
       <c r="A3337" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3337" t="n">
-        <v>3455</v>
+        <v>3439</v>
       </c>
       <c r="C3337" t="inlineStr">
         <is>
-          <t xml:space="preserve">MARDONIO CUNHA BASILIO </t>
+          <t>FERNANDA MASCARENHAS CEDRAZ</t>
         </is>
       </c>
       <c r="D3337" t="inlineStr">
         <is>
-          <t>MARDONIO1</t>
+          <t>FERNANDAM</t>
         </is>
       </c>
     </row>
     <row r="3338">
       <c r="A3338" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3338" t="n">
-        <v>3508</v>
+        <v>3455</v>
       </c>
       <c r="C3338" t="inlineStr">
         <is>
-          <t>REBECA PIRES DE SOUZA MELO</t>
+          <t xml:space="preserve">MARDONIO CUNHA BASILIO </t>
         </is>
       </c>
       <c r="D3338" t="inlineStr">
         <is>
-          <t>RPMELO</t>
+          <t>MARDONIO1</t>
         </is>
       </c>
     </row>
     <row r="3339">
       <c r="A3339" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3339" t="n">
-        <v>3543</v>
+        <v>3508</v>
       </c>
       <c r="C3339" t="inlineStr">
         <is>
-          <t>JOAO GABRIEL BARBOSA FIRMINO</t>
+          <t>REBECA PIRES DE SOUZA MELO</t>
         </is>
       </c>
       <c r="D3339" t="inlineStr">
         <is>
-          <t>JOAOG</t>
+          <t>RPMELO</t>
         </is>
       </c>
     </row>
     <row r="3340">
       <c r="A3340" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3340" t="n">
-        <v>3351</v>
+        <v>3543</v>
       </c>
       <c r="C3340" t="inlineStr">
         <is>
-          <t>HAWLLYSON DA SILVA COUTINHO</t>
+          <t>JOAO GABRIEL BARBOSA FIRMINO</t>
         </is>
       </c>
       <c r="D3340" t="inlineStr">
         <is>
-          <t>HCOUTINHO</t>
+          <t>JOAOG</t>
         </is>
       </c>
     </row>
     <row r="3341">
       <c r="A3341" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3341" t="n">
-        <v>940553</v>
+        <v>3351</v>
       </c>
       <c r="C3341" t="inlineStr">
         <is>
-          <t>LUTY TRANSPORTES- BA</t>
+          <t>HAWLLYSON DA SILVA COUTINHO</t>
         </is>
       </c>
       <c r="D3341" t="inlineStr">
         <is>
-          <t>LUTY TRANSPORTE</t>
+          <t>HCOUTINHO</t>
         </is>
       </c>
     </row>
     <row r="3342">
       <c r="A3342" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3342" t="n">
-        <v>3391</v>
+        <v>940553</v>
       </c>
       <c r="C3342" t="inlineStr">
         <is>
-          <t xml:space="preserve">NIKSON DA SILVA ALVES </t>
+          <t>LUTY TRANSPORTES- BA</t>
         </is>
       </c>
       <c r="D3342" t="inlineStr">
         <is>
-          <t>NIKSON</t>
+          <t>LUTY TRANSPORTE</t>
         </is>
       </c>
     </row>
     <row r="3343">
       <c r="A3343" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3343" t="n">
-        <v>3397</v>
+        <v>3391</v>
       </c>
       <c r="C3343" t="inlineStr">
         <is>
-          <t>EDILANE MENESES BALTAZAR</t>
+          <t xml:space="preserve">NIKSON DA SILVA ALVES </t>
         </is>
       </c>
       <c r="D3343" t="inlineStr">
         <is>
-          <t>EDILANE</t>
+          <t>NIKSON</t>
         </is>
       </c>
     </row>
@@ -67298,56 +67298,56 @@
         </is>
       </c>
       <c r="B3344" t="n">
-        <v>3398</v>
+        <v>3397</v>
       </c>
       <c r="C3344" t="inlineStr">
         <is>
-          <t>LUANA MARIA ROSIO DA SILVA</t>
+          <t>EDILANE MENESES BALTAZAR</t>
         </is>
       </c>
       <c r="D3344" t="inlineStr">
         <is>
-          <t>LUMARIA</t>
+          <t>EDILANE</t>
         </is>
       </c>
     </row>
     <row r="3345">
       <c r="A3345" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3345" t="n">
-        <v>3400</v>
+        <v>3398</v>
       </c>
       <c r="C3345" t="inlineStr">
         <is>
-          <t>ELILTON PINTO ROMEU</t>
+          <t>LUANA MARIA ROSIO DA SILVA</t>
         </is>
       </c>
       <c r="D3345" t="inlineStr">
         <is>
-          <t>ELILTON</t>
+          <t>LUMARIA</t>
         </is>
       </c>
     </row>
     <row r="3346">
       <c r="A3346" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3346" t="n">
-        <v>3406</v>
+        <v>3400</v>
       </c>
       <c r="C3346" t="inlineStr">
         <is>
-          <t>CONEXAO ALDA</t>
+          <t>ELILTON PINTO ROMEU</t>
         </is>
       </c>
       <c r="D3346" t="inlineStr">
         <is>
-          <t>CONEXAOALDA</t>
+          <t>ELILTON</t>
         </is>
       </c>
     </row>
@@ -67358,176 +67358,176 @@
         </is>
       </c>
       <c r="B3347" t="n">
-        <v>3407</v>
+        <v>3406</v>
       </c>
       <c r="C3347" t="inlineStr">
         <is>
-          <t>CONEXAO IRACEMA</t>
+          <t>CONEXAO ALDA</t>
         </is>
       </c>
       <c r="D3347" t="inlineStr">
         <is>
-          <t>CONEXAOIRACEMA</t>
+          <t>CONEXAOALDA</t>
         </is>
       </c>
     </row>
     <row r="3348">
       <c r="A3348" t="inlineStr">
         <is>
-          <t>9999</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3348" t="n">
-        <v>3408</v>
+        <v>3407</v>
       </c>
       <c r="C3348" t="inlineStr">
         <is>
-          <t>CONEXAO TAMILES</t>
+          <t>CONEXAO IRACEMA</t>
         </is>
       </c>
       <c r="D3348" t="inlineStr">
         <is>
-          <t>CONEXAOTAMILES</t>
+          <t>CONEXAOIRACEMA</t>
         </is>
       </c>
     </row>
     <row r="3349">
       <c r="A3349" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>9999</t>
         </is>
       </c>
       <c r="B3349" t="n">
-        <v>3414</v>
+        <v>3408</v>
       </c>
       <c r="C3349" t="inlineStr">
         <is>
-          <t>CONEXAO ADM PI MA</t>
+          <t>CONEXAO TAMILES</t>
         </is>
       </c>
       <c r="D3349" t="inlineStr">
         <is>
-          <t>CONEXAOPIMA</t>
+          <t>CONEXAOTAMILES</t>
         </is>
       </c>
     </row>
     <row r="3350">
       <c r="A3350" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3350" t="n">
-        <v>3524</v>
+        <v>3414</v>
       </c>
       <c r="C3350" t="inlineStr">
         <is>
-          <t>LUIS FELIPE DA SILVA SOUSA</t>
+          <t>CONEXAO ADM PI MA</t>
         </is>
       </c>
       <c r="D3350" t="inlineStr">
         <is>
-          <t>L.FELIPE</t>
+          <t>CONEXAOPIMA</t>
         </is>
       </c>
     </row>
     <row r="3351">
       <c r="A3351" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3351" t="n">
-        <v>3531</v>
+        <v>3524</v>
       </c>
       <c r="C3351" t="inlineStr">
         <is>
-          <t>LEICIANE COELHO SILVA</t>
+          <t>LUIS FELIPE DA SILVA SOUSA</t>
         </is>
       </c>
       <c r="D3351" t="inlineStr">
         <is>
-          <t>LEI.SILVA</t>
+          <t>L.FELIPE</t>
         </is>
       </c>
     </row>
     <row r="3352">
       <c r="A3352" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3352" t="n">
-        <v>3550</v>
+        <v>3531</v>
       </c>
       <c r="C3352" t="inlineStr">
         <is>
-          <t>IARGO GABRIEL SANTOS DE OLIVEIRA</t>
+          <t>LEICIANE COELHO SILVA</t>
         </is>
       </c>
       <c r="D3352" t="inlineStr">
         <is>
-          <t>IARGOG</t>
+          <t>LEI.SILVA</t>
         </is>
       </c>
     </row>
     <row r="3353">
       <c r="A3353" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3353" t="n">
-        <v>940567</v>
+        <v>3550</v>
       </c>
       <c r="C3353" t="inlineStr">
         <is>
-          <t>MS CARGAS E TRANSPORTES</t>
+          <t>IARGO GABRIEL SANTOS DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D3353" t="inlineStr">
         <is>
-          <t>ALAN BARBOSA</t>
+          <t>IARGOG</t>
         </is>
       </c>
     </row>
     <row r="3354">
       <c r="A3354" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3354" t="n">
-        <v>3560</v>
+        <v>940567</v>
       </c>
       <c r="C3354" t="inlineStr">
         <is>
-          <t>MARIA EDUARDA MELO DOS SANTOS</t>
+          <t>MS CARGAS E TRANSPORTES</t>
         </is>
       </c>
       <c r="D3354" t="inlineStr">
         <is>
-          <t>EDU.MELO</t>
+          <t>ALAN BARBOSA</t>
         </is>
       </c>
     </row>
     <row r="3355">
       <c r="A3355" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3355" t="n">
-        <v>3355</v>
+        <v>3560</v>
       </c>
       <c r="C3355" t="inlineStr">
         <is>
-          <t>HUGO MATHEUS DA COSTA FEITOSA</t>
+          <t>MARIA EDUARDA MELO DOS SANTOS</t>
         </is>
       </c>
       <c r="D3355" t="inlineStr">
         <is>
-          <t>HMFEITOSA</t>
+          <t>EDU.MELO</t>
         </is>
       </c>
     </row>
@@ -67538,96 +67538,96 @@
         </is>
       </c>
       <c r="B3356" t="n">
-        <v>3356</v>
+        <v>3355</v>
       </c>
       <c r="C3356" t="inlineStr">
         <is>
-          <t>BRENDA LIMA DE OLIVEIRA CUNHA</t>
+          <t>HUGO MATHEUS DA COSTA FEITOSA</t>
         </is>
       </c>
       <c r="D3356" t="inlineStr">
         <is>
-          <t>BLCUNHA</t>
+          <t>HMFEITOSA</t>
         </is>
       </c>
     </row>
     <row r="3357">
       <c r="A3357" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3357" t="n">
-        <v>3361</v>
+        <v>3356</v>
       </c>
       <c r="C3357" t="inlineStr">
         <is>
-          <t>WLADIA DE ARAUJO BASTOS</t>
+          <t>BRENDA LIMA DE OLIVEIRA CUNHA</t>
         </is>
       </c>
       <c r="D3357" t="inlineStr">
         <is>
-          <t>WABASTOS</t>
+          <t>BLCUNHA</t>
         </is>
       </c>
     </row>
     <row r="3358">
       <c r="A3358" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3358" t="n">
-        <v>3362</v>
+        <v>3361</v>
       </c>
       <c r="C3358" t="inlineStr">
         <is>
-          <t>CARLOS HENRIQUE MELO DA SILVA</t>
+          <t>WLADIA DE ARAUJO BASTOS</t>
         </is>
       </c>
       <c r="D3358" t="inlineStr">
         <is>
-          <t>CHMELO</t>
+          <t>WABASTOS</t>
         </is>
       </c>
     </row>
     <row r="3359">
       <c r="A3359" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3359" t="n">
-        <v>3375</v>
+        <v>3362</v>
       </c>
       <c r="C3359" t="inlineStr">
         <is>
-          <t>AFONSO DE SOUSA RAMOS FILHO</t>
+          <t>CARLOS HENRIQUE MELO DA SILVA</t>
         </is>
       </c>
       <c r="D3359" t="inlineStr">
         <is>
-          <t>AFILHO</t>
+          <t>CHMELO</t>
         </is>
       </c>
     </row>
     <row r="3360">
       <c r="A3360" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3360" t="n">
-        <v>3404</v>
+        <v>3375</v>
       </c>
       <c r="C3360" t="inlineStr">
         <is>
-          <t>NOVATO 4 COM</t>
+          <t>AFONSO DE SOUSA RAMOS FILHO</t>
         </is>
       </c>
       <c r="D3360" t="inlineStr">
         <is>
-          <t>NOVATO4COM</t>
+          <t>AFILHO</t>
         </is>
       </c>
     </row>
@@ -67638,156 +67638,156 @@
         </is>
       </c>
       <c r="B3361" t="n">
-        <v>3405</v>
+        <v>3404</v>
       </c>
       <c r="C3361" t="inlineStr">
         <is>
-          <t>NOVATO 5 COM</t>
+          <t>NOVATO 4 COM</t>
         </is>
       </c>
       <c r="D3361" t="inlineStr">
         <is>
-          <t>NOVATO5COM</t>
+          <t>NOVATO4COM</t>
         </is>
       </c>
     </row>
     <row r="3362">
       <c r="A3362" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3362" t="n">
-        <v>3447</v>
+        <v>3405</v>
       </c>
       <c r="C3362" t="inlineStr">
         <is>
-          <t>RAYSSA KEYCE LINHARES AQUINO</t>
+          <t>NOVATO 5 COM</t>
         </is>
       </c>
       <c r="D3362" t="inlineStr">
         <is>
-          <t>RAYSSAK</t>
+          <t>NOVATO5COM</t>
         </is>
       </c>
     </row>
     <row r="3363">
       <c r="A3363" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3363" t="n">
-        <v>940559</v>
+        <v>3447</v>
       </c>
       <c r="C3363" t="inlineStr">
         <is>
-          <t>WALLEF DE OLIVEIRA</t>
+          <t>RAYSSA KEYCE LINHARES AQUINO</t>
         </is>
       </c>
       <c r="D3363" t="inlineStr">
         <is>
-          <t>WALLEF</t>
+          <t>RAYSSAK</t>
         </is>
       </c>
     </row>
     <row r="3364">
       <c r="A3364" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>99</t>
         </is>
       </c>
       <c r="B3364" t="n">
-        <v>3489</v>
+        <v>940559</v>
       </c>
       <c r="C3364" t="inlineStr">
         <is>
-          <t>MARCELA KARINA PEREIRA VELOSO</t>
+          <t>WALLEF DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D3364" t="inlineStr">
         <is>
-          <t>MKARINA</t>
+          <t>WALLEF</t>
         </is>
       </c>
     </row>
     <row r="3365">
       <c r="A3365" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3365" t="n">
-        <v>3490</v>
+        <v>3489</v>
       </c>
       <c r="C3365" t="inlineStr">
         <is>
-          <t>JOSE MAILSON GOMES NUNES</t>
+          <t>MARCELA KARINA PEREIRA VELOSO</t>
         </is>
       </c>
       <c r="D3365" t="inlineStr">
         <is>
-          <t>J.MAILSON</t>
+          <t>MKARINA</t>
         </is>
       </c>
     </row>
     <row r="3366">
       <c r="A3366" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3366" t="n">
-        <v>3537</v>
+        <v>3490</v>
       </c>
       <c r="C3366" t="inlineStr">
         <is>
-          <t>ALDAIR PEDRO DA SILVA</t>
+          <t>JOSE MAILSON GOMES NUNES</t>
         </is>
       </c>
       <c r="D3366" t="inlineStr">
         <is>
-          <t>A.PEDRO</t>
+          <t>J.MAILSON</t>
         </is>
       </c>
     </row>
     <row r="3367">
       <c r="A3367" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3367" t="n">
-        <v>3549</v>
+        <v>3537</v>
       </c>
       <c r="C3367" t="inlineStr">
         <is>
-          <t xml:space="preserve">FERNANDA CAROLINE E CESAR SOUSA </t>
+          <t>ALDAIR PEDRO DA SILVA</t>
         </is>
       </c>
       <c r="D3367" t="inlineStr">
         <is>
-          <t>FCAROLINE</t>
+          <t>A.PEDRO</t>
         </is>
       </c>
     </row>
     <row r="3368">
       <c r="A3368" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3368" t="n">
-        <v>3337</v>
+        <v>3549</v>
       </c>
       <c r="C3368" t="inlineStr">
         <is>
-          <t>WESLEY FONTES DE ALMEIDA</t>
+          <t xml:space="preserve">FERNANDA CAROLINE E CESAR SOUSA </t>
         </is>
       </c>
       <c r="D3368" t="inlineStr">
         <is>
-          <t>WFALMEIDA</t>
+          <t>FCAROLINE</t>
         </is>
       </c>
     </row>
@@ -67798,16 +67798,16 @@
         </is>
       </c>
       <c r="B3369" t="n">
-        <v>3338</v>
+        <v>3337</v>
       </c>
       <c r="C3369" t="inlineStr">
         <is>
-          <t>FRANCISCA SAMARA MENDES DE OLIVEIRA C</t>
+          <t>WESLEY FONTES DE ALMEIDA</t>
         </is>
       </c>
       <c r="D3369" t="inlineStr">
         <is>
-          <t>FSCUNHA</t>
+          <t>WFALMEIDA</t>
         </is>
       </c>
     </row>
@@ -67818,176 +67818,176 @@
         </is>
       </c>
       <c r="B3370" t="n">
-        <v>3339</v>
+        <v>3338</v>
       </c>
       <c r="C3370" t="inlineStr">
         <is>
-          <t>MAYARA THALYA DIAS DE ANDRADE</t>
+          <t>FRANCISCA SAMARA MENDES DE OLIVEIRA C</t>
         </is>
       </c>
       <c r="D3370" t="inlineStr">
         <is>
-          <t>MTANDRADE</t>
+          <t>FSCUNHA</t>
         </is>
       </c>
     </row>
     <row r="3371">
       <c r="A3371" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3371" t="n">
-        <v>3359</v>
+        <v>3339</v>
       </c>
       <c r="C3371" t="inlineStr">
         <is>
-          <t xml:space="preserve">EVANESSA DA SILVA E SILVA </t>
+          <t>MAYARA THALYA DIAS DE ANDRADE</t>
         </is>
       </c>
       <c r="D3371" t="inlineStr">
         <is>
-          <t>EVANESSAS</t>
+          <t>MTANDRADE</t>
         </is>
       </c>
     </row>
     <row r="3372">
       <c r="A3372" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3372" t="n">
-        <v>3360</v>
+        <v>3359</v>
       </c>
       <c r="C3372" t="inlineStr">
         <is>
-          <t>THIAGO DE CARVALHO ARAUJO</t>
+          <t xml:space="preserve">EVANESSA DA SILVA E SILVA </t>
         </is>
       </c>
       <c r="D3372" t="inlineStr">
         <is>
-          <t>TCARAUJO</t>
+          <t>EVANESSAS</t>
         </is>
       </c>
     </row>
     <row r="3373">
       <c r="A3373" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3373" t="n">
-        <v>3481</v>
+        <v>3360</v>
       </c>
       <c r="C3373" t="inlineStr">
         <is>
-          <t xml:space="preserve">EDSON DA PAZ LIMA </t>
+          <t>THIAGO DE CARVALHO ARAUJO</t>
         </is>
       </c>
       <c r="D3373" t="inlineStr">
         <is>
-          <t>EDPAZ</t>
+          <t>TCARAUJO</t>
         </is>
       </c>
     </row>
     <row r="3374">
       <c r="A3374" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3374" t="n">
-        <v>3494</v>
+        <v>3481</v>
       </c>
       <c r="C3374" t="inlineStr">
         <is>
-          <t>ANTONIO CRISTINA BRITO GOMES</t>
+          <t xml:space="preserve">EDSON DA PAZ LIMA </t>
         </is>
       </c>
       <c r="D3374" t="inlineStr">
         <is>
-          <t>CRIS.GOMES</t>
+          <t>EDPAZ</t>
         </is>
       </c>
     </row>
     <row r="3375">
       <c r="A3375" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3375" t="n">
-        <v>3498</v>
+        <v>3494</v>
       </c>
       <c r="C3375" t="inlineStr">
         <is>
-          <t>SILVESTRA COSTA NUNES</t>
+          <t>ANTONIO CRISTINA BRITO GOMES</t>
         </is>
       </c>
       <c r="D3375" t="inlineStr">
         <is>
-          <t>SCNUNES</t>
+          <t>CRIS.GOMES</t>
         </is>
       </c>
     </row>
     <row r="3376">
       <c r="A3376" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3376" t="n">
-        <v>940562</v>
+        <v>3498</v>
       </c>
       <c r="C3376" t="inlineStr">
         <is>
-          <t>FRANCISCO DAVID ASSUNCAO ALVES</t>
+          <t>SILVESTRA COSTA NUNES</t>
         </is>
       </c>
       <c r="D3376" t="inlineStr">
         <is>
-          <t>ASSUNÇÃO</t>
+          <t>SCNUNES</t>
         </is>
       </c>
     </row>
     <row r="3377">
       <c r="A3377" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>99</t>
         </is>
       </c>
       <c r="B3377" t="n">
-        <v>3513</v>
+        <v>940562</v>
       </c>
       <c r="C3377" t="inlineStr">
         <is>
-          <t>RENARA ANDRADE MATIAS</t>
+          <t>FRANCISCO DAVID ASSUNCAO ALVES</t>
         </is>
       </c>
       <c r="D3377" t="inlineStr">
         <is>
-          <t>R.ANDRADE</t>
+          <t>ASSUNÇÃO</t>
         </is>
       </c>
     </row>
     <row r="3378">
       <c r="A3378" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3378" t="n">
-        <v>3275</v>
+        <v>3513</v>
       </c>
       <c r="C3378" t="inlineStr">
         <is>
-          <t>MARIA APARECIDA COELHO SILVA</t>
+          <t>RENARA ANDRADE MATIAS</t>
         </is>
       </c>
       <c r="D3378" t="inlineStr">
         <is>
-          <t>MCOELHO</t>
+          <t>R.ANDRADE</t>
         </is>
       </c>
     </row>
@@ -67998,116 +67998,116 @@
         </is>
       </c>
       <c r="B3379" t="n">
-        <v>3276</v>
+        <v>3275</v>
       </c>
       <c r="C3379" t="inlineStr">
         <is>
-          <t xml:space="preserve">PEROLA DE JESUS AMORIM SOUSA </t>
+          <t>MARIA APARECIDA COELHO SILVA</t>
         </is>
       </c>
       <c r="D3379" t="inlineStr">
         <is>
-          <t>PJESUS</t>
+          <t>MCOELHO</t>
         </is>
       </c>
     </row>
     <row r="3380">
       <c r="A3380" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3380" t="n">
-        <v>3526</v>
+        <v>3276</v>
       </c>
       <c r="C3380" t="inlineStr">
         <is>
-          <t>JOYCE NAZARE CORREA</t>
+          <t xml:space="preserve">PEROLA DE JESUS AMORIM SOUSA </t>
         </is>
       </c>
       <c r="D3380" t="inlineStr">
         <is>
-          <t>J.NAZARE</t>
+          <t>PJESUS</t>
         </is>
       </c>
     </row>
     <row r="3381">
       <c r="A3381" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3381" t="n">
-        <v>3527</v>
+        <v>3526</v>
       </c>
       <c r="C3381" t="inlineStr">
         <is>
-          <t>GILVANA DA SILVA MONTELES</t>
+          <t>JOYCE NAZARE CORREA</t>
         </is>
       </c>
       <c r="D3381" t="inlineStr">
         <is>
-          <t>GIL.SILVA</t>
+          <t>J.NAZARE</t>
         </is>
       </c>
     </row>
     <row r="3382">
       <c r="A3382" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3382" t="n">
-        <v>3548</v>
+        <v>3527</v>
       </c>
       <c r="C3382" t="inlineStr">
         <is>
-          <t>JAMILLY MARIA HENRIQUE ARAUJO</t>
+          <t>GILVANA DA SILVA MONTELES</t>
         </is>
       </c>
       <c r="D3382" t="inlineStr">
         <is>
-          <t>JAMILLY</t>
+          <t>GIL.SILVA</t>
         </is>
       </c>
     </row>
     <row r="3383">
       <c r="A3383" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3383" t="n">
-        <v>3551</v>
+        <v>3548</v>
       </c>
       <c r="C3383" t="inlineStr">
         <is>
-          <t xml:space="preserve">VITOR MANOEL DA SILVA BARBOSA </t>
+          <t>JAMILLY MARIA HENRIQUE ARAUJO</t>
         </is>
       </c>
       <c r="D3383" t="inlineStr">
         <is>
-          <t>VMANOEL</t>
+          <t>JAMILLY</t>
         </is>
       </c>
     </row>
     <row r="3384">
       <c r="A3384" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3384" t="n">
-        <v>940525</v>
+        <v>3551</v>
       </c>
       <c r="C3384" t="inlineStr">
         <is>
-          <t>SANDUWELLINGTON</t>
+          <t xml:space="preserve">VITOR MANOEL DA SILVA BARBOSA </t>
         </is>
       </c>
       <c r="D3384" t="inlineStr">
         <is>
-          <t>SANDUWELLINGTON</t>
+          <t>VMANOEL</t>
         </is>
       </c>
     </row>
@@ -68118,36 +68118,36 @@
         </is>
       </c>
       <c r="B3385" t="n">
-        <v>3369</v>
+        <v>940525</v>
       </c>
       <c r="C3385" t="inlineStr">
         <is>
-          <t xml:space="preserve">PRISCILA DOS SANTOS LOPES </t>
+          <t>SANDUWELLINGTON</t>
         </is>
       </c>
       <c r="D3385" t="inlineStr">
         <is>
-          <t>PSLOPES</t>
+          <t>SANDUWELLINGTON</t>
         </is>
       </c>
     </row>
     <row r="3386">
       <c r="A3386" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3386" t="n">
-        <v>3433</v>
+        <v>3369</v>
       </c>
       <c r="C3386" t="inlineStr">
         <is>
-          <t>BRUNO NUNES CRUZ</t>
+          <t xml:space="preserve">PRISCILA DOS SANTOS LOPES </t>
         </is>
       </c>
       <c r="D3386" t="inlineStr">
         <is>
-          <t>BRUNOCRUZ</t>
+          <t>PSLOPES</t>
         </is>
       </c>
     </row>
@@ -68158,36 +68158,36 @@
         </is>
       </c>
       <c r="B3387" t="n">
-        <v>3434</v>
+        <v>3433</v>
       </c>
       <c r="C3387" t="inlineStr">
         <is>
-          <t>ANA TERCIA DE LIMA SA CARVALHO SERAFIM</t>
+          <t>BRUNO NUNES CRUZ</t>
         </is>
       </c>
       <c r="D3387" t="inlineStr">
         <is>
-          <t>ANATER</t>
+          <t>BRUNOCRUZ</t>
         </is>
       </c>
     </row>
     <row r="3388">
       <c r="A3388" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3388" t="n">
-        <v>3502</v>
+        <v>3434</v>
       </c>
       <c r="C3388" t="inlineStr">
         <is>
-          <t>LUIZ FELIPE MACHADO BARRETO</t>
+          <t>ANA TERCIA DE LIMA SA CARVALHO SERAFIM</t>
         </is>
       </c>
       <c r="D3388" t="inlineStr">
         <is>
-          <t>LUIZ.FELIPE</t>
+          <t>ANATER</t>
         </is>
       </c>
     </row>
@@ -68198,56 +68198,56 @@
         </is>
       </c>
       <c r="B3389" t="n">
-        <v>3503</v>
+        <v>3502</v>
       </c>
       <c r="C3389" t="inlineStr">
         <is>
-          <t>FABIO OLIVEIRA SILVA</t>
+          <t>LUIZ FELIPE MACHADO BARRETO</t>
         </is>
       </c>
       <c r="D3389" t="inlineStr">
         <is>
-          <t>FOSILVA</t>
+          <t>LUIZ.FELIPE</t>
         </is>
       </c>
     </row>
     <row r="3390">
       <c r="A3390" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3390" t="n">
-        <v>3554</v>
+        <v>3503</v>
       </c>
       <c r="C3390" t="inlineStr">
         <is>
-          <t xml:space="preserve">MANOEL RIBEIRO DE SOUZA JUNIOR </t>
+          <t>FABIO OLIVEIRA SILVA</t>
         </is>
       </c>
       <c r="D3390" t="inlineStr">
         <is>
-          <t>MRJUNIOR</t>
+          <t>FOSILVA</t>
         </is>
       </c>
     </row>
     <row r="3391">
       <c r="A3391" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3391" t="n">
-        <v>940549</v>
+        <v>3554</v>
       </c>
       <c r="C3391" t="inlineStr">
         <is>
-          <t>EDILSON ARAUJO - FL9</t>
+          <t xml:space="preserve">MANOEL RIBEIRO DE SOUZA JUNIOR </t>
         </is>
       </c>
       <c r="D3391" t="inlineStr">
         <is>
-          <t>EDILSON</t>
+          <t>MRJUNIOR</t>
         </is>
       </c>
     </row>
@@ -68258,36 +68258,36 @@
         </is>
       </c>
       <c r="B3392" t="n">
-        <v>3470</v>
+        <v>940549</v>
       </c>
       <c r="C3392" t="inlineStr">
         <is>
-          <t>DEBORA ALVES CARVALHO</t>
+          <t>EDILSON ARAUJO - FL9</t>
         </is>
       </c>
       <c r="D3392" t="inlineStr">
         <is>
-          <t>DEBORA.ALVES</t>
+          <t>EDILSON</t>
         </is>
       </c>
     </row>
     <row r="3393">
       <c r="A3393" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3393" t="n">
-        <v>3510</v>
+        <v>3470</v>
       </c>
       <c r="C3393" t="inlineStr">
         <is>
-          <t>CAMILA RODIGUES PINTO</t>
+          <t>DEBORA ALVES CARVALHO</t>
         </is>
       </c>
       <c r="D3393" t="inlineStr">
         <is>
-          <t>MILA.PINTO</t>
+          <t>DEBORA.ALVES</t>
         </is>
       </c>
     </row>
@@ -68298,96 +68298,96 @@
         </is>
       </c>
       <c r="B3394" t="n">
-        <v>3511</v>
+        <v>3510</v>
       </c>
       <c r="C3394" t="inlineStr">
         <is>
-          <t>JORGE HENRIQUE DOS SANTOS RODRIGUES</t>
+          <t>CAMILA RODIGUES PINTO</t>
         </is>
       </c>
       <c r="D3394" t="inlineStr">
         <is>
-          <t>J.HENRIQUE</t>
+          <t>MILA.PINTO</t>
         </is>
       </c>
     </row>
     <row r="3395">
       <c r="A3395" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3395" t="n">
-        <v>3561</v>
+        <v>3511</v>
       </c>
       <c r="C3395" t="inlineStr">
         <is>
-          <t>RONARIA PATRICIA VILARINDO DE ALMEIDA</t>
+          <t>JORGE HENRIQUE DOS SANTOS RODRIGUES</t>
         </is>
       </c>
       <c r="D3395" t="inlineStr">
         <is>
-          <t>RPATRICIA</t>
+          <t>J.HENRIQUE</t>
         </is>
       </c>
     </row>
     <row r="3396">
       <c r="A3396" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3396" t="n">
-        <v>3562</v>
+        <v>3561</v>
       </c>
       <c r="C3396" t="inlineStr">
         <is>
-          <t>LETICIA MARIA BENTO NOGUEIRA</t>
+          <t>RONARIA PATRICIA VILARINDO DE ALMEIDA</t>
         </is>
       </c>
       <c r="D3396" t="inlineStr">
         <is>
-          <t>LBENTO</t>
+          <t>RPATRICIA</t>
         </is>
       </c>
     </row>
     <row r="3397">
       <c r="A3397" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3397" t="n">
-        <v>3270</v>
+        <v>3562</v>
       </c>
       <c r="C3397" t="inlineStr">
         <is>
-          <t>ITANA NASCIMENTO SIMOES</t>
+          <t>LETICIA MARIA BENTO NOGUEIRA</t>
         </is>
       </c>
       <c r="D3397" t="inlineStr">
         <is>
-          <t>ISIMOES</t>
+          <t>LBENTO</t>
         </is>
       </c>
     </row>
     <row r="3398">
       <c r="A3398" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3398" t="n">
-        <v>3318</v>
+        <v>3270</v>
       </c>
       <c r="C3398" t="inlineStr">
         <is>
-          <t>LUAN MONTEIRO COSTA</t>
+          <t>ITANA NASCIMENTO SIMOES</t>
         </is>
       </c>
       <c r="D3398" t="inlineStr">
         <is>
-          <t>LMONTEIRO</t>
+          <t>ISIMOES</t>
         </is>
       </c>
     </row>
@@ -68398,36 +68398,36 @@
         </is>
       </c>
       <c r="B3399" t="n">
-        <v>3319</v>
+        <v>3318</v>
       </c>
       <c r="C3399" t="inlineStr">
         <is>
-          <t>MARIANA MACEDA DOS SANTOS</t>
+          <t>LUAN MONTEIRO COSTA</t>
         </is>
       </c>
       <c r="D3399" t="inlineStr">
         <is>
-          <t>MMACEDA</t>
+          <t>LMONTEIRO</t>
         </is>
       </c>
     </row>
     <row r="3400">
       <c r="A3400" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3400" t="n">
-        <v>3389</v>
+        <v>3319</v>
       </c>
       <c r="C3400" t="inlineStr">
         <is>
-          <t>TAMILES DE SANTANA AMORIM BISPO</t>
+          <t>MARIANA MACEDA DOS SANTOS</t>
         </is>
       </c>
       <c r="D3400" t="inlineStr">
         <is>
-          <t>TAMILES</t>
+          <t>MMACEDA</t>
         </is>
       </c>
     </row>
@@ -68438,36 +68438,36 @@
         </is>
       </c>
       <c r="B3401" t="n">
-        <v>3390</v>
+        <v>3389</v>
       </c>
       <c r="C3401" t="inlineStr">
         <is>
-          <t>IRACEMA DE ALMEIDA MOURA</t>
+          <t>TAMILES DE SANTANA AMORIM BISPO</t>
         </is>
       </c>
       <c r="D3401" t="inlineStr">
         <is>
-          <t>IRACEMA</t>
+          <t>TAMILES</t>
         </is>
       </c>
     </row>
     <row r="3402">
       <c r="A3402" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3402" t="n">
-        <v>3286</v>
+        <v>3390</v>
       </c>
       <c r="C3402" t="inlineStr">
         <is>
-          <t>VALERIA MAIA DA SILVA</t>
+          <t>IRACEMA DE ALMEIDA MOURA</t>
         </is>
       </c>
       <c r="D3402" t="inlineStr">
         <is>
-          <t>VMAIAS</t>
+          <t>IRACEMA</t>
         </is>
       </c>
     </row>
@@ -68478,156 +68478,156 @@
         </is>
       </c>
       <c r="B3403" t="n">
-        <v>3287</v>
+        <v>3286</v>
       </c>
       <c r="C3403" t="inlineStr">
         <is>
-          <t>ERIVELTON DA SILVA OLIVEIRA</t>
+          <t>VALERIA MAIA DA SILVA</t>
         </is>
       </c>
       <c r="D3403" t="inlineStr">
         <is>
-          <t>ESOLIVEIRA</t>
+          <t>VMAIAS</t>
         </is>
       </c>
     </row>
     <row r="3404">
       <c r="A3404" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3404" t="n">
-        <v>3307</v>
+        <v>3287</v>
       </c>
       <c r="C3404" t="inlineStr">
         <is>
-          <t>ADRIEL XERES BARROS MARTINS</t>
+          <t>ERIVELTON DA SILVA OLIVEIRA</t>
         </is>
       </c>
       <c r="D3404" t="inlineStr">
         <is>
-          <t>AXERES</t>
+          <t>ESOLIVEIRA</t>
         </is>
       </c>
     </row>
     <row r="3405">
       <c r="A3405" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3405" t="n">
-        <v>3308</v>
+        <v>3307</v>
       </c>
       <c r="C3405" t="inlineStr">
         <is>
-          <t>ELKZIEL JUVINO DA SILVA</t>
+          <t>ADRIEL XERES BARROS MARTINS</t>
         </is>
       </c>
       <c r="D3405" t="inlineStr">
         <is>
-          <t>EJUVINO</t>
+          <t>AXERES</t>
         </is>
       </c>
     </row>
     <row r="3406">
       <c r="A3406" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3406" t="n">
-        <v>940539</v>
+        <v>3308</v>
       </c>
       <c r="C3406" t="inlineStr">
         <is>
-          <t>EDSON ARAUJO - FL9</t>
+          <t>ELKZIEL JUVINO DA SILVA</t>
         </is>
       </c>
       <c r="D3406" t="inlineStr">
         <is>
-          <t>EDS</t>
+          <t>EJUVINO</t>
         </is>
       </c>
     </row>
     <row r="3407">
       <c r="A3407" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3407" t="n">
-        <v>940540</v>
+        <v>940539</v>
       </c>
       <c r="C3407" t="inlineStr">
         <is>
-          <t>EDSON ARAUJO - FL8</t>
+          <t>EDSON ARAUJO - FL9</t>
         </is>
       </c>
       <c r="D3407" t="inlineStr">
         <is>
-          <t>EDS8</t>
+          <t>EDS</t>
         </is>
       </c>
     </row>
     <row r="3408">
       <c r="A3408" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B3408" t="n">
-        <v>3328</v>
+        <v>940540</v>
       </c>
       <c r="C3408" t="inlineStr">
         <is>
-          <t>ALAN ARAUJO DA SILVA</t>
+          <t>EDSON ARAUJO - FL8</t>
         </is>
       </c>
       <c r="D3408" t="inlineStr">
         <is>
-          <t>ARSILVA</t>
+          <t>EDS8</t>
         </is>
       </c>
     </row>
     <row r="3409">
       <c r="A3409" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3409" t="n">
-        <v>3350</v>
+        <v>3328</v>
       </c>
       <c r="C3409" t="inlineStr">
         <is>
-          <t xml:space="preserve">EDER RODRIGUES DA SILVA </t>
+          <t>ALAN ARAUJO DA SILVA</t>
         </is>
       </c>
       <c r="D3409" t="inlineStr">
         <is>
-          <t>EDERS</t>
+          <t>ARSILVA</t>
         </is>
       </c>
     </row>
     <row r="3410">
       <c r="A3410" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3410" t="n">
-        <v>3373</v>
+        <v>3350</v>
       </c>
       <c r="C3410" t="inlineStr">
         <is>
-          <t xml:space="preserve">NATANAEL TAVARES DE SOUSA </t>
+          <t xml:space="preserve">EDER RODRIGUES DA SILVA </t>
         </is>
       </c>
       <c r="D3410" t="inlineStr">
         <is>
-          <t>NTSOUSA</t>
+          <t>EDERS</t>
         </is>
       </c>
     </row>
@@ -68638,156 +68638,156 @@
         </is>
       </c>
       <c r="B3411" t="n">
-        <v>3374</v>
+        <v>3373</v>
       </c>
       <c r="C3411" t="inlineStr">
         <is>
-          <t>REINALDO DA SILVA COSTA</t>
+          <t xml:space="preserve">NATANAEL TAVARES DE SOUSA </t>
         </is>
       </c>
       <c r="D3411" t="inlineStr">
         <is>
-          <t>RSCOSTA</t>
+          <t>NTSOUSA</t>
         </is>
       </c>
     </row>
     <row r="3412">
       <c r="A3412" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3412" t="n">
-        <v>3399</v>
+        <v>3374</v>
       </c>
       <c r="C3412" t="inlineStr">
         <is>
-          <t xml:space="preserve">RICARDO BARBOSA DOS SANTOS </t>
+          <t>REINALDO DA SILVA COSTA</t>
         </is>
       </c>
       <c r="D3412" t="inlineStr">
         <is>
-          <t>RICARDOSAN</t>
+          <t>RSCOSTA</t>
         </is>
       </c>
     </row>
     <row r="3413">
       <c r="A3413" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3413" t="n">
-        <v>3427</v>
+        <v>3399</v>
       </c>
       <c r="C3413" t="inlineStr">
         <is>
-          <t>ROQUE COMERCIO TEMPORARIO</t>
+          <t xml:space="preserve">RICARDO BARBOSA DOS SANTOS </t>
         </is>
       </c>
       <c r="D3413" t="inlineStr">
         <is>
-          <t>ROQUECOM</t>
+          <t>RICARDOSAN</t>
         </is>
       </c>
     </row>
     <row r="3414">
       <c r="A3414" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3414" t="n">
-        <v>3428</v>
+        <v>3427</v>
       </c>
       <c r="C3414" t="inlineStr">
         <is>
-          <t>ROQUE PLUS TEMPORARIO</t>
+          <t>ROQUE COMERCIO TEMPORARIO</t>
         </is>
       </c>
       <c r="D3414" t="inlineStr">
         <is>
-          <t>ROQUEPLUS</t>
+          <t>ROQUECOM</t>
         </is>
       </c>
     </row>
     <row r="3415">
       <c r="A3415" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3415" t="n">
-        <v>3432</v>
+        <v>3428</v>
       </c>
       <c r="C3415" t="inlineStr">
         <is>
-          <t>PATRICIA DOS SANTOS NONATO OLIVEIRA</t>
+          <t>ROQUE PLUS TEMPORARIO</t>
         </is>
       </c>
       <c r="D3415" t="inlineStr">
         <is>
-          <t>PATRICIAD</t>
+          <t>ROQUEPLUS</t>
         </is>
       </c>
     </row>
     <row r="3416">
       <c r="A3416" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3416" t="n">
-        <v>3448</v>
+        <v>3432</v>
       </c>
       <c r="C3416" t="inlineStr">
         <is>
-          <t xml:space="preserve">GABRIEL SOUZA CARVALHO </t>
+          <t>PATRICIA DOS SANTOS NONATO OLIVEIRA</t>
         </is>
       </c>
       <c r="D3416" t="inlineStr">
         <is>
-          <t>GABRIEL20</t>
+          <t>PATRICIAD</t>
         </is>
       </c>
     </row>
     <row r="3417">
       <c r="A3417" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3417" t="n">
-        <v>3465</v>
+        <v>3448</v>
       </c>
       <c r="C3417" t="inlineStr">
         <is>
-          <t>LUIZA MARIA BARRETO BARBOSA</t>
+          <t xml:space="preserve">GABRIEL SOUZA CARVALHO </t>
         </is>
       </c>
       <c r="D3417" t="inlineStr">
         <is>
-          <t>LUIZA.MARIA</t>
+          <t>GABRIEL20</t>
         </is>
       </c>
     </row>
     <row r="3418">
       <c r="A3418" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3418" t="n">
-        <v>3468</v>
+        <v>3465</v>
       </c>
       <c r="C3418" t="inlineStr">
         <is>
-          <t>KAWA ALMEIDA CAMPOS</t>
+          <t>LUIZA MARIA BARRETO BARBOSA</t>
         </is>
       </c>
       <c r="D3418" t="inlineStr">
         <is>
-          <t>KAWA</t>
+          <t>LUIZA.MARIA</t>
         </is>
       </c>
     </row>
@@ -68798,16 +68798,16 @@
         </is>
       </c>
       <c r="B3419" t="n">
-        <v>3476</v>
+        <v>3468</v>
       </c>
       <c r="C3419" t="inlineStr">
         <is>
-          <t xml:space="preserve"> FRANCISCA LEIDIANE M. MENDES NASCIMENTO</t>
+          <t>KAWA ALMEIDA CAMPOS</t>
         </is>
       </c>
       <c r="D3419" t="inlineStr">
         <is>
-          <t>FLEIDIANE</t>
+          <t>KAWA</t>
         </is>
       </c>
     </row>
@@ -68818,76 +68818,76 @@
         </is>
       </c>
       <c r="B3420" t="n">
-        <v>3477</v>
+        <v>3476</v>
       </c>
       <c r="C3420" t="inlineStr">
         <is>
-          <t>MARIA THAIS MARTINS PEREIRA SILVA</t>
+          <t xml:space="preserve"> FRANCISCA LEIDIANE M. MENDES NASCIMENTO</t>
         </is>
       </c>
       <c r="D3420" t="inlineStr">
         <is>
-          <t>MTHAIS</t>
+          <t>FLEIDIANE</t>
         </is>
       </c>
     </row>
     <row r="3421">
       <c r="A3421" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3421" t="n">
-        <v>3271</v>
+        <v>3477</v>
       </c>
       <c r="C3421" t="inlineStr">
         <is>
-          <t>DIEGO DE ARAUJO CALÁBRIA</t>
+          <t>MARIA THAIS MARTINS PEREIRA SILVA</t>
         </is>
       </c>
       <c r="D3421" t="inlineStr">
         <is>
-          <t>ARAUJOC</t>
+          <t>MTHAIS</t>
         </is>
       </c>
     </row>
     <row r="3422">
       <c r="A3422" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3422" t="n">
-        <v>3272</v>
+        <v>3271</v>
       </c>
       <c r="C3422" t="inlineStr">
         <is>
-          <t>ANNE BEATRIZ SILVA VIRGINO</t>
+          <t>DIEGO DE ARAUJO CALÁBRIA</t>
         </is>
       </c>
       <c r="D3422" t="inlineStr">
         <is>
-          <t>ABVIRGINIO</t>
+          <t>ARAUJOC</t>
         </is>
       </c>
     </row>
     <row r="3423">
       <c r="A3423" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3423" t="n">
-        <v>3293</v>
+        <v>3272</v>
       </c>
       <c r="C3423" t="inlineStr">
         <is>
-          <t xml:space="preserve">CARLOS ALBERTO VIRIATO SANTOS </t>
+          <t>ANNE BEATRIZ SILVA VIRGINO</t>
         </is>
       </c>
       <c r="D3423" t="inlineStr">
         <is>
-          <t>CVIRIATO</t>
+          <t>ABVIRGINIO</t>
         </is>
       </c>
     </row>
@@ -68898,16 +68898,16 @@
         </is>
       </c>
       <c r="B3424" t="n">
-        <v>3381</v>
+        <v>3293</v>
       </c>
       <c r="C3424" t="inlineStr">
         <is>
-          <t>ALAN CAIQUE SANTOS E SANTOS</t>
+          <t xml:space="preserve">CARLOS ALBERTO VIRIATO SANTOS </t>
         </is>
       </c>
       <c r="D3424" t="inlineStr">
         <is>
-          <t>ALANSANTOS</t>
+          <t>CVIRIATO</t>
         </is>
       </c>
     </row>
@@ -68918,136 +68918,136 @@
         </is>
       </c>
       <c r="B3425" t="n">
-        <v>3443</v>
+        <v>3381</v>
       </c>
       <c r="C3425" t="inlineStr">
         <is>
-          <t>SANON MOREIRA SOUZA</t>
+          <t>ALAN CAIQUE SANTOS E SANTOS</t>
         </is>
       </c>
       <c r="D3425" t="inlineStr">
         <is>
-          <t>SANON</t>
+          <t>ALANSANTOS</t>
         </is>
       </c>
     </row>
     <row r="3426">
       <c r="A3426" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3426" t="n">
-        <v>3516</v>
+        <v>3443</v>
       </c>
       <c r="C3426" t="inlineStr">
         <is>
-          <t>FRANCISCO RILDER TELES DE OLIVEIRA</t>
+          <t>SANON MOREIRA SOUZA</t>
         </is>
       </c>
       <c r="D3426" t="inlineStr">
         <is>
-          <t>RILDER</t>
+          <t>SANON</t>
         </is>
       </c>
     </row>
     <row r="3427">
       <c r="A3427" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3427" t="n">
-        <v>3519</v>
+        <v>3516</v>
       </c>
       <c r="C3427" t="inlineStr">
         <is>
-          <t>MARIA LUANA DE ALMEIDA BATISTA</t>
+          <t>FRANCISCO RILDER TELES DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D3427" t="inlineStr">
         <is>
-          <t>M.LUANA</t>
+          <t>RILDER</t>
         </is>
       </c>
     </row>
     <row r="3428">
       <c r="A3428" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3428" t="n">
-        <v>3540</v>
+        <v>3519</v>
       </c>
       <c r="C3428" t="inlineStr">
         <is>
-          <t>HELEN VITORIA OLIVEIRA DA ROCHA</t>
+          <t>MARIA LUANA DE ALMEIDA BATISTA</t>
         </is>
       </c>
       <c r="D3428" t="inlineStr">
         <is>
-          <t>H.VITORIA</t>
+          <t>M.LUANA</t>
         </is>
       </c>
     </row>
     <row r="3429">
       <c r="A3429" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B3429" t="n">
-        <v>3559</v>
+        <v>3540</v>
       </c>
       <c r="C3429" t="inlineStr">
         <is>
-          <t>ARKBERYS TELES DE SOUSA</t>
+          <t>HELEN VITORIA OLIVEIRA DA ROCHA</t>
         </is>
       </c>
       <c r="D3429" t="inlineStr">
         <is>
-          <t>ARKBERYS</t>
+          <t>H.VITORIA</t>
         </is>
       </c>
     </row>
     <row r="3430">
       <c r="A3430" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3430" t="n">
-        <v>3331</v>
+        <v>3559</v>
       </c>
       <c r="C3430" t="inlineStr">
         <is>
-          <t>LOUIZE VANIELLE RODRIGUES FARIAS</t>
+          <t>ARKBERYS TELES DE SOUSA</t>
         </is>
       </c>
       <c r="D3430" t="inlineStr">
         <is>
-          <t>LVFARIAS</t>
+          <t>ARKBERYS</t>
         </is>
       </c>
     </row>
     <row r="3431">
       <c r="A3431" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3431" t="n">
-        <v>3334</v>
+        <v>3567</v>
       </c>
       <c r="C3431" t="inlineStr">
         <is>
-          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+          <t>PEDRO HENRIQUE VIEIRA DE LIMA</t>
         </is>
       </c>
       <c r="D3431" t="inlineStr">
         <is>
-          <t>MTGASPAR</t>
+          <t>P.LIMA</t>
         </is>
       </c>
     </row>
@@ -69058,356 +69058,356 @@
         </is>
       </c>
       <c r="B3432" t="n">
-        <v>3345</v>
+        <v>3331</v>
       </c>
       <c r="C3432" t="inlineStr">
         <is>
-          <t>AURICÉLIA INACIO PEREIRA</t>
+          <t>LOUIZE VANIELLE RODRIGUES FARIAS</t>
         </is>
       </c>
       <c r="D3432" t="inlineStr">
         <is>
-          <t>AIPEREIRA</t>
+          <t>LVFARIAS</t>
         </is>
       </c>
     </row>
     <row r="3433">
       <c r="A3433" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3433" t="n">
-        <v>3363</v>
+        <v>3334</v>
       </c>
       <c r="C3433" t="inlineStr">
         <is>
-          <t>IASMIN LEAL ALVES</t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
       <c r="D3433" t="inlineStr">
         <is>
-          <t>ILALVES</t>
+          <t>MTGASPAR</t>
         </is>
       </c>
     </row>
     <row r="3434">
       <c r="A3434" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3434" t="n">
-        <v>3370</v>
+        <v>3345</v>
       </c>
       <c r="C3434" t="inlineStr">
         <is>
-          <t>CARLOS DIEGO ARAUJO ALMEIDA</t>
+          <t>AURICÉLIA INACIO PEREIRA</t>
         </is>
       </c>
       <c r="D3434" t="inlineStr">
         <is>
-          <t>CDIEGO</t>
+          <t>AIPEREIRA</t>
         </is>
       </c>
     </row>
     <row r="3435">
       <c r="A3435" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3435" t="n">
-        <v>3379</v>
+        <v>3363</v>
       </c>
       <c r="C3435" t="inlineStr">
         <is>
-          <t xml:space="preserve">MATHEUS EVANGELISTA FERREIRA </t>
+          <t>IASMIN LEAL ALVES</t>
         </is>
       </c>
       <c r="D3435" t="inlineStr">
         <is>
-          <t>MMFERREIRA</t>
+          <t>ILALVES</t>
         </is>
       </c>
     </row>
     <row r="3436">
       <c r="A3436" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3436" t="n">
-        <v>3419</v>
+        <v>3370</v>
       </c>
       <c r="C3436" t="inlineStr">
         <is>
-          <t xml:space="preserve">DAVID EVANGELISTA SILVA </t>
+          <t>CARLOS DIEGO ARAUJO ALMEIDA</t>
         </is>
       </c>
       <c r="D3436" t="inlineStr">
         <is>
-          <t>DAVID</t>
+          <t>CDIEGO</t>
         </is>
       </c>
     </row>
     <row r="3437">
       <c r="A3437" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3437" t="n">
-        <v>3423</v>
+        <v>3379</v>
       </c>
       <c r="C3437" t="inlineStr">
         <is>
-          <t>MARCIO JOSE TIAGO</t>
+          <t xml:space="preserve">MATHEUS EVANGELISTA FERREIRA </t>
         </is>
       </c>
       <c r="D3437" t="inlineStr">
         <is>
-          <t>MJTIAGO</t>
+          <t>MMFERREIRA</t>
         </is>
       </c>
     </row>
     <row r="3438">
       <c r="A3438" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3438" t="n">
-        <v>3453</v>
+        <v>3419</v>
       </c>
       <c r="C3438" t="inlineStr">
         <is>
-          <t xml:space="preserve">LAURIENE SILVA BARBOSA </t>
+          <t xml:space="preserve">DAVID EVANGELISTA SILVA </t>
         </is>
       </c>
       <c r="D3438" t="inlineStr">
         <is>
-          <t>LAURIENE</t>
+          <t>DAVID</t>
         </is>
       </c>
     </row>
     <row r="3439">
       <c r="A3439" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3439" t="n">
-        <v>3478</v>
+        <v>3423</v>
       </c>
       <c r="C3439" t="inlineStr">
         <is>
-          <t>LEANDRO BRITO NOGUEIRA DE OLIVEIRA</t>
+          <t>MARCIO JOSE TIAGO</t>
         </is>
       </c>
       <c r="D3439" t="inlineStr">
         <is>
-          <t>LBNOGUEIRA</t>
+          <t>MJTIAGO</t>
         </is>
       </c>
     </row>
     <row r="3440">
       <c r="A3440" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3440" t="n">
-        <v>3479</v>
+        <v>3453</v>
       </c>
       <c r="C3440" t="inlineStr">
         <is>
-          <t>ESDRAS ALESSANDRO SANTOS SANTANA</t>
+          <t xml:space="preserve">LAURIENE SILVA BARBOSA </t>
         </is>
       </c>
       <c r="D3440" t="inlineStr">
         <is>
-          <t>EALESSANDRO</t>
+          <t>LAURIENE</t>
         </is>
       </c>
     </row>
     <row r="3441">
       <c r="A3441" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3441" t="n">
-        <v>3480</v>
+        <v>3478</v>
       </c>
       <c r="C3441" t="inlineStr">
         <is>
-          <t xml:space="preserve">LUCIMARA SOUSA LIMA </t>
+          <t>LEANDRO BRITO NOGUEIRA DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D3441" t="inlineStr">
         <is>
-          <t>LUCIMARA</t>
+          <t>LBNOGUEIRA</t>
         </is>
       </c>
     </row>
     <row r="3442">
       <c r="A3442" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3442" t="n">
-        <v>3482</v>
+        <v>3479</v>
       </c>
       <c r="C3442" t="inlineStr">
         <is>
-          <t>DANIEL FERNANDES DINIZ HERACLIO</t>
+          <t>ESDRAS ALESSANDRO SANTOS SANTANA</t>
         </is>
       </c>
       <c r="D3442" t="inlineStr">
         <is>
-          <t>DFDINIZ</t>
+          <t>EALESSANDRO</t>
         </is>
       </c>
     </row>
     <row r="3443">
       <c r="A3443" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3443" t="n">
-        <v>3518</v>
+        <v>3480</v>
       </c>
       <c r="C3443" t="inlineStr">
         <is>
-          <t>RAMYRA ALVES FELIX DA SILVA</t>
+          <t xml:space="preserve">LUCIMARA SOUSA LIMA </t>
         </is>
       </c>
       <c r="D3443" t="inlineStr">
         <is>
-          <t>RFELIX</t>
+          <t>LUCIMARA</t>
         </is>
       </c>
     </row>
     <row r="3444">
       <c r="A3444" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3444" t="n">
-        <v>3534</v>
+        <v>3482</v>
       </c>
       <c r="C3444" t="inlineStr">
         <is>
-          <t xml:space="preserve">CAIO DE SOUZA VINHAS </t>
+          <t>DANIEL FERNANDES DINIZ HERACLIO</t>
         </is>
       </c>
       <c r="D3444" t="inlineStr">
         <is>
-          <t>CVINHAS</t>
+          <t>DFDINIZ</t>
         </is>
       </c>
     </row>
     <row r="3445">
       <c r="A3445" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3445" t="n">
-        <v>3535</v>
+        <v>3518</v>
       </c>
       <c r="C3445" t="inlineStr">
         <is>
-          <t>ROMARIO DE SOUSA SILVA</t>
+          <t>RAMYRA ALVES FELIX DA SILVA</t>
         </is>
       </c>
       <c r="D3445" t="inlineStr">
         <is>
-          <t>RSOUSAS</t>
+          <t>RFELIX</t>
         </is>
       </c>
     </row>
     <row r="3446">
       <c r="A3446" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3446" t="n">
-        <v>3536</v>
+        <v>3534</v>
       </c>
       <c r="C3446" t="inlineStr">
         <is>
-          <t>JHONATAS CARVALHO OLIVEIRA</t>
+          <t xml:space="preserve">CAIO DE SOUZA VINHAS </t>
         </is>
       </c>
       <c r="D3446" t="inlineStr">
         <is>
-          <t>JHONATASC</t>
+          <t>CVINHAS</t>
         </is>
       </c>
     </row>
     <row r="3447">
       <c r="A3447" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3447" t="n">
-        <v>940529</v>
+        <v>3535</v>
       </c>
       <c r="C3447" t="inlineStr">
         <is>
-          <t>EDGAR FELIX - FL9</t>
+          <t>ROMARIO DE SOUSA SILVA</t>
         </is>
       </c>
       <c r="D3447" t="inlineStr">
         <is>
-          <t>EDGAR F</t>
+          <t>RSOUSAS</t>
         </is>
       </c>
     </row>
     <row r="3448">
       <c r="A3448" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3448" t="n">
-        <v>3304</v>
+        <v>3536</v>
       </c>
       <c r="C3448" t="inlineStr">
         <is>
-          <t>JOACI GUILHERME GONÇALVES DA LUZ</t>
+          <t>JHONATAS CARVALHO OLIVEIRA</t>
         </is>
       </c>
       <c r="D3448" t="inlineStr">
         <is>
-          <t>JLUZ</t>
+          <t>JHONATASC</t>
         </is>
       </c>
     </row>
     <row r="3449">
       <c r="A3449" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3449" t="n">
-        <v>3305</v>
+        <v>940529</v>
       </c>
       <c r="C3449" t="inlineStr">
         <is>
-          <t>JOÃO VITOR DE ARAÚJO GONÇALVES</t>
+          <t>EDGAR FELIX - FL9</t>
         </is>
       </c>
       <c r="D3449" t="inlineStr">
         <is>
-          <t>JJVITOR</t>
+          <t>EDGAR F</t>
         </is>
       </c>
     </row>
@@ -69418,276 +69418,276 @@
         </is>
       </c>
       <c r="B3450" t="n">
-        <v>3306</v>
+        <v>3304</v>
       </c>
       <c r="C3450" t="inlineStr">
         <is>
-          <t>WENDERSON MARCOS DOS SANTOS</t>
+          <t>JOACI GUILHERME GONÇALVES DA LUZ</t>
         </is>
       </c>
       <c r="D3450" t="inlineStr">
         <is>
-          <t>WWMARCOS</t>
+          <t>JLUZ</t>
         </is>
       </c>
     </row>
     <row r="3451">
       <c r="A3451" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3451" t="n">
-        <v>3335</v>
+        <v>3305</v>
       </c>
       <c r="C3451" t="inlineStr">
         <is>
-          <t>EDILBERTO LEMOS DE LIMA</t>
+          <t>JOÃO VITOR DE ARAÚJO GONÇALVES</t>
         </is>
       </c>
       <c r="D3451" t="inlineStr">
         <is>
-          <t>ELEMOS</t>
+          <t>JJVITOR</t>
         </is>
       </c>
     </row>
     <row r="3452">
       <c r="A3452" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3452" t="n">
-        <v>3336</v>
+        <v>3306</v>
       </c>
       <c r="C3452" t="inlineStr">
         <is>
-          <t>EZEQUIEL SOUZA DO NASCIMENTO</t>
+          <t>WENDERSON MARCOS DOS SANTOS</t>
         </is>
       </c>
       <c r="D3452" t="inlineStr">
         <is>
-          <t>ESNASCIMENTO</t>
+          <t>WWMARCOS</t>
         </is>
       </c>
     </row>
     <row r="3453">
       <c r="A3453" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3453" t="n">
-        <v>3341</v>
+        <v>3335</v>
       </c>
       <c r="C3453" t="inlineStr">
         <is>
-          <t>ALCIONE MARIANO DE OLIVEIRA</t>
+          <t>EDILBERTO LEMOS DE LIMA</t>
         </is>
       </c>
       <c r="D3453" t="inlineStr">
         <is>
-          <t>AMOLIVEIRA</t>
+          <t>ELEMOS</t>
         </is>
       </c>
     </row>
     <row r="3454">
       <c r="A3454" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3454" t="n">
-        <v>3401</v>
+        <v>3336</v>
       </c>
       <c r="C3454" t="inlineStr">
         <is>
-          <t xml:space="preserve">TULIO HENRIQUE DA SILVA CARVALHO </t>
+          <t>EZEQUIEL SOUZA DO NASCIMENTO</t>
         </is>
       </c>
       <c r="D3454" t="inlineStr">
         <is>
-          <t>TULIO</t>
+          <t>ESNASCIMENTO</t>
         </is>
       </c>
     </row>
     <row r="3455">
       <c r="A3455" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3455" t="n">
-        <v>3411</v>
+        <v>3341</v>
       </c>
       <c r="C3455" t="inlineStr">
         <is>
-          <t>CONEXAO RUBYA DANILLA</t>
+          <t>ALCIONE MARIANO DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D3455" t="inlineStr">
         <is>
-          <t>CONEXAORUBYA</t>
+          <t>AMOLIVEIRA</t>
         </is>
       </c>
     </row>
     <row r="3456">
       <c r="A3456" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3456" t="n">
-        <v>3412</v>
+        <v>3401</v>
       </c>
       <c r="C3456" t="inlineStr">
         <is>
-          <t>CONEXAO RAFAEL</t>
+          <t xml:space="preserve">TULIO HENRIQUE DA SILVA CARVALHO </t>
         </is>
       </c>
       <c r="D3456" t="inlineStr">
         <is>
-          <t>CONEXAORAFAEL</t>
+          <t>TULIO</t>
         </is>
       </c>
     </row>
     <row r="3457">
       <c r="A3457" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3457" t="n">
-        <v>3558</v>
+        <v>3411</v>
       </c>
       <c r="C3457" t="inlineStr">
         <is>
-          <t>WALLYS QUEIROZ VIANA</t>
+          <t>CONEXAO RUBYA DANILLA</t>
         </is>
       </c>
       <c r="D3457" t="inlineStr">
         <is>
-          <t>WALLYS</t>
+          <t>CONEXAORUBYA</t>
         </is>
       </c>
     </row>
     <row r="3458">
       <c r="A3458" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3458" t="n">
-        <v>3264</v>
+        <v>3412</v>
       </c>
       <c r="C3458" t="inlineStr">
         <is>
-          <t xml:space="preserve">WILTON CARLOS MACIEL DE ASSIS </t>
+          <t>CONEXAO RAFAEL</t>
         </is>
       </c>
       <c r="D3458" t="inlineStr">
         <is>
-          <t>WCMACIEL</t>
+          <t>CONEXAORAFAEL</t>
         </is>
       </c>
     </row>
     <row r="3459">
       <c r="A3459" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3459" t="n">
-        <v>3340</v>
+        <v>3558</v>
       </c>
       <c r="C3459" t="inlineStr">
         <is>
-          <t>ROGELENO FARIAS FEIJÃO FILHO</t>
+          <t>WALLYS QUEIROZ VIANA</t>
         </is>
       </c>
       <c r="D3459" t="inlineStr">
         <is>
-          <t>RFEIJAO</t>
+          <t>WALLYS</t>
         </is>
       </c>
     </row>
     <row r="3460">
       <c r="A3460" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3460" t="n">
-        <v>940550</v>
+        <v>3264</v>
       </c>
       <c r="C3460" t="inlineStr">
         <is>
-          <t>RAFAELE RIBEIRO CARNEIRO</t>
+          <t xml:space="preserve">WILTON CARLOS MACIEL DE ASSIS </t>
         </is>
       </c>
       <c r="D3460" t="inlineStr">
         <is>
-          <t>RAFAELE</t>
+          <t>WCMACIEL</t>
         </is>
       </c>
     </row>
     <row r="3461">
       <c r="A3461" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3461" t="n">
-        <v>3377</v>
+        <v>3340</v>
       </c>
       <c r="C3461" t="inlineStr">
         <is>
-          <t xml:space="preserve"> ISALTINO BISPO DE OLIVEIRA JUNIOR</t>
+          <t>ROGELENO FARIAS FEIJÃO FILHO</t>
         </is>
       </c>
       <c r="D3461" t="inlineStr">
         <is>
-          <t>BJUNIOR</t>
+          <t>RFEIJAO</t>
         </is>
       </c>
     </row>
     <row r="3462">
       <c r="A3462" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>99</t>
         </is>
       </c>
       <c r="B3462" t="n">
-        <v>3425</v>
+        <v>940550</v>
       </c>
       <c r="C3462" t="inlineStr">
         <is>
-          <t xml:space="preserve"> CIRLANE ARAUJO SOUZA </t>
+          <t>RAFAELE RIBEIRO CARNEIRO</t>
         </is>
       </c>
       <c r="D3462" t="inlineStr">
         <is>
-          <t>CIRLANES</t>
+          <t>RAFAELE</t>
         </is>
       </c>
     </row>
     <row r="3463">
       <c r="A3463" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3463" t="n">
-        <v>3454</v>
+        <v>3377</v>
       </c>
       <c r="C3463" t="inlineStr">
         <is>
-          <t>ANTONIA SAMARA DE SOUZA SOARES</t>
+          <t xml:space="preserve"> ISALTINO BISPO DE OLIVEIRA JUNIOR</t>
         </is>
       </c>
       <c r="D3463" t="inlineStr">
         <is>
-          <t>ANTSAMARA</t>
+          <t>BJUNIOR</t>
         </is>
       </c>
     </row>
@@ -69698,96 +69698,96 @@
         </is>
       </c>
       <c r="B3464" t="n">
-        <v>3491</v>
+        <v>3425</v>
       </c>
       <c r="C3464" t="inlineStr">
         <is>
-          <t>PEDRO JOSE DO NASCIMENTO NETO</t>
+          <t xml:space="preserve"> CIRLANE ARAUJO SOUZA </t>
         </is>
       </c>
       <c r="D3464" t="inlineStr">
         <is>
-          <t>P.JOSE</t>
+          <t>CIRLANES</t>
         </is>
       </c>
     </row>
     <row r="3465">
       <c r="A3465" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3465" t="n">
-        <v>3492</v>
+        <v>3454</v>
       </c>
       <c r="C3465" t="inlineStr">
         <is>
-          <t>PAULA CARLA CALDAS MOTA</t>
+          <t>ANTONIA SAMARA DE SOUZA SOARES</t>
         </is>
       </c>
       <c r="D3465" t="inlineStr">
         <is>
-          <t>P.CARLA</t>
+          <t>ANTSAMARA</t>
         </is>
       </c>
     </row>
     <row r="3466">
       <c r="A3466" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3466" t="n">
-        <v>3542</v>
+        <v>3491</v>
       </c>
       <c r="C3466" t="inlineStr">
         <is>
-          <t>ANTONIA MILENA SOUSA ANDRADE</t>
+          <t>PEDRO JOSE DO NASCIMENTO NETO</t>
         </is>
       </c>
       <c r="D3466" t="inlineStr">
         <is>
-          <t>A.MILENA</t>
+          <t>P.JOSE</t>
         </is>
       </c>
     </row>
     <row r="3467">
       <c r="A3467" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3467" t="n">
-        <v>3547</v>
+        <v>3492</v>
       </c>
       <c r="C3467" t="inlineStr">
         <is>
-          <t xml:space="preserve">DAVI PEREIRA DA SILVA </t>
+          <t>PAULA CARLA CALDAS MOTA</t>
         </is>
       </c>
       <c r="D3467" t="inlineStr">
         <is>
-          <t>DPSILVA</t>
+          <t>P.CARLA</t>
         </is>
       </c>
     </row>
     <row r="3468">
       <c r="A3468" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3468" t="n">
-        <v>3552</v>
+        <v>3542</v>
       </c>
       <c r="C3468" t="inlineStr">
         <is>
-          <t>PAULO SERGIO MENDES DE OLIVEIRA</t>
+          <t>ANTONIA MILENA SOUSA ANDRADE</t>
         </is>
       </c>
       <c r="D3468" t="inlineStr">
         <is>
-          <t>PSMENDES</t>
+          <t>A.MILENA</t>
         </is>
       </c>
     </row>
@@ -69798,214 +69798,254 @@
         </is>
       </c>
       <c r="B3469" t="n">
-        <v>3294</v>
+        <v>3547</v>
       </c>
       <c r="C3469" t="inlineStr">
         <is>
-          <t>GLEICIANE MIRANDA DE MORAIS</t>
+          <t xml:space="preserve">DAVI PEREIRA DA SILVA </t>
         </is>
       </c>
       <c r="D3469" t="inlineStr">
         <is>
-          <t>GMIRANDA</t>
+          <t>DPSILVA</t>
         </is>
       </c>
     </row>
     <row r="3470">
       <c r="A3470" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3470" t="n">
-        <v>3295</v>
+        <v>3552</v>
       </c>
       <c r="C3470" t="inlineStr">
         <is>
-          <t>MARIA ESTEFANNY DA SILVA MOURA</t>
+          <t>PAULO SERGIO MENDES DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D3470" t="inlineStr">
         <is>
-          <t>MESTEFANNY</t>
+          <t>PSMENDES</t>
         </is>
       </c>
     </row>
     <row r="3471">
       <c r="A3471" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3471" t="n">
-        <v>3296</v>
+        <v>3294</v>
       </c>
       <c r="C3471" t="inlineStr">
         <is>
-          <t>PEDRO IAGO FONSECA EVANGELISTA</t>
+          <t>GLEICIANE MIRANDA DE MORAIS</t>
         </is>
       </c>
       <c r="D3471" t="inlineStr">
         <is>
-          <t>PIFONSECA</t>
+          <t>GMIRANDA</t>
         </is>
       </c>
     </row>
     <row r="3472">
       <c r="A3472" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3472" t="n">
-        <v>940544</v>
+        <v>3295</v>
       </c>
       <c r="C3472" t="inlineStr">
         <is>
-          <t>LUTY LOG TRANSPORTES - FL8</t>
+          <t>MARIA ESTEFANNY DA SILVA MOURA</t>
         </is>
       </c>
       <c r="D3472" t="inlineStr">
         <is>
-          <t>LUTY LOG</t>
+          <t>MESTEFANNY</t>
         </is>
       </c>
     </row>
     <row r="3473">
       <c r="A3473" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3473" t="n">
-        <v>3380</v>
+        <v>3296</v>
       </c>
       <c r="C3473" t="inlineStr">
         <is>
-          <t>FRANCISCO MATHEUS RABELO DA COSTA</t>
+          <t>PEDRO IAGO FONSECA EVANGELISTA</t>
         </is>
       </c>
       <c r="D3473" t="inlineStr">
         <is>
-          <t>FMATHEUS</t>
+          <t>PIFONSECA</t>
         </is>
       </c>
     </row>
     <row r="3474">
       <c r="A3474" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B3474" t="n">
-        <v>3410</v>
+        <v>940544</v>
       </c>
       <c r="C3474" t="inlineStr">
         <is>
-          <t xml:space="preserve"> BRENO ALLAN DE JESUS</t>
+          <t>LUTY LOG TRANSPORTES - FL8</t>
         </is>
       </c>
       <c r="D3474" t="inlineStr">
         <is>
-          <t>JESUS</t>
+          <t>LUTY LOG</t>
         </is>
       </c>
     </row>
     <row r="3475">
       <c r="A3475" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3475" t="n">
-        <v>3444</v>
+        <v>3380</v>
       </c>
       <c r="C3475" t="inlineStr">
         <is>
-          <t>THIAGO COSTA SILVA</t>
+          <t>FRANCISCO MATHEUS RABELO DA COSTA</t>
         </is>
       </c>
       <c r="D3475" t="inlineStr">
         <is>
-          <t>THIAGOC</t>
+          <t>FMATHEUS</t>
         </is>
       </c>
     </row>
     <row r="3476">
       <c r="A3476" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3476" t="n">
-        <v>3456</v>
+        <v>3410</v>
       </c>
       <c r="C3476" t="inlineStr">
         <is>
-          <t>FELIPE BOTH MAZUCHINI</t>
+          <t xml:space="preserve"> BRENO ALLAN DE JESUS</t>
         </is>
       </c>
       <c r="D3476" t="inlineStr">
         <is>
-          <t>FELIPEB</t>
+          <t>JESUS</t>
         </is>
       </c>
     </row>
     <row r="3477">
       <c r="A3477" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3477" t="n">
-        <v>3457</v>
+        <v>3444</v>
       </c>
       <c r="C3477" t="inlineStr">
         <is>
-          <t>FRANKLIN VIEIRA GOMES</t>
+          <t>THIAGO COSTA SILVA</t>
         </is>
       </c>
       <c r="D3477" t="inlineStr">
         <is>
-          <t>VIEIRAF</t>
+          <t>THIAGOC</t>
         </is>
       </c>
     </row>
     <row r="3478">
       <c r="A3478" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3478" t="n">
-        <v>3507</v>
+        <v>3456</v>
       </c>
       <c r="C3478" t="inlineStr">
         <is>
-          <t>KARINE TEODORA ALVES DE OLIVEIRA</t>
+          <t>FELIPE BOTH MAZUCHINI</t>
         </is>
       </c>
       <c r="D3478" t="inlineStr">
         <is>
-          <t>KOLIVEIRA</t>
+          <t>FELIPEB</t>
         </is>
       </c>
     </row>
     <row r="3479">
       <c r="A3479" t="inlineStr">
         <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B3479" t="n">
+        <v>3457</v>
+      </c>
+      <c r="C3479" t="inlineStr">
+        <is>
+          <t>FRANKLIN VIEIRA GOMES</t>
+        </is>
+      </c>
+      <c r="D3479" t="inlineStr">
+        <is>
+          <t>VIEIRAF</t>
+        </is>
+      </c>
+    </row>
+    <row r="3480">
+      <c r="A3480" t="inlineStr">
+        <is>
           <t>5</t>
         </is>
       </c>
-      <c r="B3479" t="n">
+      <c r="B3480" t="n">
+        <v>3507</v>
+      </c>
+      <c r="C3480" t="inlineStr">
+        <is>
+          <t>KARINE TEODORA ALVES DE OLIVEIRA</t>
+        </is>
+      </c>
+      <c r="D3480" t="inlineStr">
+        <is>
+          <t>KOLIVEIRA</t>
+        </is>
+      </c>
+    </row>
+    <row r="3481">
+      <c r="A3481" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B3481" t="n">
         <v>3520</v>
       </c>
-      <c r="C3479" t="inlineStr">
+      <c r="C3481" t="inlineStr">
         <is>
           <t xml:space="preserve"> EMERSON FILIPE MELO DE AGUIAR</t>
         </is>
       </c>
-      <c r="D3479" t="inlineStr">
+      <c r="D3481" t="inlineStr">
         <is>
           <t>E.FILIPE</t>
         </is>

</xml_diff>

<commit_message>
chore(data): batch update intraday televendas - 08:01:33
</commit_message>
<xml_diff>
--- a/data/dim_televendas.xlsx
+++ b/data/dim_televendas.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3489"/>
+  <dimension ref="A1:D3490"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -41587,7 +41587,7 @@
       </c>
       <c r="D2058" t="inlineStr">
         <is>
-          <t>DEBARROS</t>
+          <t>DE.BARROS</t>
         </is>
       </c>
     </row>
@@ -59674,7 +59674,7 @@
     <row r="2963">
       <c r="A2963" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B2963" t="n">
@@ -60774,7 +60774,7 @@
     <row r="3018">
       <c r="A3018" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3018" t="n">
@@ -68394,20 +68394,20 @@
     <row r="3399">
       <c r="A3399" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3399" t="n">
-        <v>940549</v>
+        <v>3576</v>
       </c>
       <c r="C3399" t="inlineStr">
         <is>
-          <t>EDILSON ARAUJO - FL9</t>
+          <t>ANA BEATRIZ PARENTE CAVALCANTE</t>
         </is>
       </c>
       <c r="D3399" t="inlineStr">
         <is>
-          <t>EDILSON</t>
+          <t>A.BEATRIZ</t>
         </is>
       </c>
     </row>
@@ -68418,36 +68418,36 @@
         </is>
       </c>
       <c r="B3400" t="n">
-        <v>3470</v>
+        <v>940549</v>
       </c>
       <c r="C3400" t="inlineStr">
         <is>
-          <t>DEBORA ALVES CARVALHO</t>
+          <t>EDILSON ARAUJO - FL9</t>
         </is>
       </c>
       <c r="D3400" t="inlineStr">
         <is>
-          <t>DEBORA.ALVES</t>
+          <t>EDILSON</t>
         </is>
       </c>
     </row>
     <row r="3401">
       <c r="A3401" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3401" t="n">
-        <v>3510</v>
+        <v>3470</v>
       </c>
       <c r="C3401" t="inlineStr">
         <is>
-          <t>CAMILA RODIGUES PINTO</t>
+          <t>DEBORA ALVES CARVALHO</t>
         </is>
       </c>
       <c r="D3401" t="inlineStr">
         <is>
-          <t>MILA.PINTO</t>
+          <t>DEBORA.ALVES</t>
         </is>
       </c>
     </row>
@@ -68458,96 +68458,96 @@
         </is>
       </c>
       <c r="B3402" t="n">
-        <v>3511</v>
+        <v>3510</v>
       </c>
       <c r="C3402" t="inlineStr">
         <is>
-          <t>JORGE HENRIQUE DOS SANTOS RODRIGUES</t>
+          <t>CAMILA RODIGUES PINTO</t>
         </is>
       </c>
       <c r="D3402" t="inlineStr">
         <is>
-          <t>J.HENRIQUE</t>
+          <t>MILA.PINTO</t>
         </is>
       </c>
     </row>
     <row r="3403">
       <c r="A3403" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3403" t="n">
-        <v>3561</v>
+        <v>3511</v>
       </c>
       <c r="C3403" t="inlineStr">
         <is>
-          <t>RONARIA PATRICIA VILARINDO DE ALMEIDA</t>
+          <t>JORGE HENRIQUE DOS SANTOS RODRIGUES</t>
         </is>
       </c>
       <c r="D3403" t="inlineStr">
         <is>
-          <t>RPATRICIA</t>
+          <t>J.HENRIQUE</t>
         </is>
       </c>
     </row>
     <row r="3404">
       <c r="A3404" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3404" t="n">
-        <v>3562</v>
+        <v>3561</v>
       </c>
       <c r="C3404" t="inlineStr">
         <is>
-          <t>LETICIA MARIA BENTO NOGUEIRA</t>
+          <t>RONARIA PATRICIA VILARINDO DE ALMEIDA</t>
         </is>
       </c>
       <c r="D3404" t="inlineStr">
         <is>
-          <t>LBENTO</t>
+          <t>RPATRICIA</t>
         </is>
       </c>
     </row>
     <row r="3405">
       <c r="A3405" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3405" t="n">
-        <v>3270</v>
+        <v>3562</v>
       </c>
       <c r="C3405" t="inlineStr">
         <is>
-          <t>ITANA NASCIMENTO SIMOES</t>
+          <t>LETICIA MARIA BENTO NOGUEIRA</t>
         </is>
       </c>
       <c r="D3405" t="inlineStr">
         <is>
-          <t>ISIMOES</t>
+          <t>LBENTO</t>
         </is>
       </c>
     </row>
     <row r="3406">
       <c r="A3406" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3406" t="n">
-        <v>3318</v>
+        <v>3270</v>
       </c>
       <c r="C3406" t="inlineStr">
         <is>
-          <t>LUAN MONTEIRO COSTA</t>
+          <t>ITANA NASCIMENTO SIMOES</t>
         </is>
       </c>
       <c r="D3406" t="inlineStr">
         <is>
-          <t>LMONTEIRO</t>
+          <t>ISIMOES</t>
         </is>
       </c>
     </row>
@@ -68558,36 +68558,36 @@
         </is>
       </c>
       <c r="B3407" t="n">
-        <v>3319</v>
+        <v>3318</v>
       </c>
       <c r="C3407" t="inlineStr">
         <is>
-          <t>MARIANA MACEDA DOS SANTOS</t>
+          <t>LUAN MONTEIRO COSTA</t>
         </is>
       </c>
       <c r="D3407" t="inlineStr">
         <is>
-          <t>MMACEDA</t>
+          <t>LMONTEIRO</t>
         </is>
       </c>
     </row>
     <row r="3408">
       <c r="A3408" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3408" t="n">
-        <v>3389</v>
+        <v>3319</v>
       </c>
       <c r="C3408" t="inlineStr">
         <is>
-          <t>TAMILES DE SANTANA AMORIM BISPO</t>
+          <t>MARIANA MACEDA DOS SANTOS</t>
         </is>
       </c>
       <c r="D3408" t="inlineStr">
         <is>
-          <t>TAMILES</t>
+          <t>MMACEDA</t>
         </is>
       </c>
     </row>
@@ -68598,36 +68598,36 @@
         </is>
       </c>
       <c r="B3409" t="n">
-        <v>3390</v>
+        <v>3389</v>
       </c>
       <c r="C3409" t="inlineStr">
         <is>
-          <t>IRACEMA DE ALMEIDA MOURA</t>
+          <t>TAMILES DE SANTANA AMORIM BISPO</t>
         </is>
       </c>
       <c r="D3409" t="inlineStr">
         <is>
-          <t>IRACEMA</t>
+          <t>TAMILES</t>
         </is>
       </c>
     </row>
     <row r="3410">
       <c r="A3410" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3410" t="n">
-        <v>3575</v>
+        <v>3390</v>
       </c>
       <c r="C3410" t="inlineStr">
         <is>
-          <t>SAMARA ALVES DA SILVA</t>
+          <t>IRACEMA DE ALMEIDA MOURA</t>
         </is>
       </c>
       <c r="D3410" t="inlineStr">
         <is>
-          <t>S.ALVES</t>
+          <t>IRACEMA</t>
         </is>
       </c>
     </row>
@@ -68638,16 +68638,16 @@
         </is>
       </c>
       <c r="B3411" t="n">
-        <v>3286</v>
+        <v>3575</v>
       </c>
       <c r="C3411" t="inlineStr">
         <is>
-          <t>VALERIA MAIA DA SILVA</t>
+          <t>SAMARA ALVES DA SILVA</t>
         </is>
       </c>
       <c r="D3411" t="inlineStr">
         <is>
-          <t>VMAIAS</t>
+          <t>S.ALVES</t>
         </is>
       </c>
     </row>
@@ -68658,156 +68658,156 @@
         </is>
       </c>
       <c r="B3412" t="n">
-        <v>3287</v>
+        <v>3286</v>
       </c>
       <c r="C3412" t="inlineStr">
         <is>
-          <t>ERIVELTON DA SILVA OLIVEIRA</t>
+          <t>VALERIA MAIA DA SILVA</t>
         </is>
       </c>
       <c r="D3412" t="inlineStr">
         <is>
-          <t>ESOLIVEIRA</t>
+          <t>VMAIAS</t>
         </is>
       </c>
     </row>
     <row r="3413">
       <c r="A3413" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3413" t="n">
-        <v>3307</v>
+        <v>3287</v>
       </c>
       <c r="C3413" t="inlineStr">
         <is>
-          <t>ADRIEL XERES BARROS MARTINS</t>
+          <t>ERIVELTON DA SILVA OLIVEIRA</t>
         </is>
       </c>
       <c r="D3413" t="inlineStr">
         <is>
-          <t>AXERES</t>
+          <t>ESOLIVEIRA</t>
         </is>
       </c>
     </row>
     <row r="3414">
       <c r="A3414" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3414" t="n">
-        <v>3308</v>
+        <v>3307</v>
       </c>
       <c r="C3414" t="inlineStr">
         <is>
-          <t>ELKZIEL JUVINO DA SILVA</t>
+          <t>ADRIEL XERES BARROS MARTINS</t>
         </is>
       </c>
       <c r="D3414" t="inlineStr">
         <is>
-          <t>EJUVINO</t>
+          <t>AXERES</t>
         </is>
       </c>
     </row>
     <row r="3415">
       <c r="A3415" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3415" t="n">
-        <v>940539</v>
+        <v>3308</v>
       </c>
       <c r="C3415" t="inlineStr">
         <is>
-          <t>EDSON ARAUJO - FL9</t>
+          <t>ELKZIEL JUVINO DA SILVA</t>
         </is>
       </c>
       <c r="D3415" t="inlineStr">
         <is>
-          <t>EDS</t>
+          <t>EJUVINO</t>
         </is>
       </c>
     </row>
     <row r="3416">
       <c r="A3416" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3416" t="n">
-        <v>940540</v>
+        <v>940539</v>
       </c>
       <c r="C3416" t="inlineStr">
         <is>
-          <t>EDSON ARAUJO - FL8</t>
+          <t>EDSON ARAUJO - FL9</t>
         </is>
       </c>
       <c r="D3416" t="inlineStr">
         <is>
-          <t>EDS8</t>
+          <t>EDS</t>
         </is>
       </c>
     </row>
     <row r="3417">
       <c r="A3417" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B3417" t="n">
-        <v>3328</v>
+        <v>940540</v>
       </c>
       <c r="C3417" t="inlineStr">
         <is>
-          <t>ALAN ARAUJO DA SILVA</t>
+          <t>EDSON ARAUJO - FL8</t>
         </is>
       </c>
       <c r="D3417" t="inlineStr">
         <is>
-          <t>ARSILVA</t>
+          <t>EDS8</t>
         </is>
       </c>
     </row>
     <row r="3418">
       <c r="A3418" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3418" t="n">
-        <v>3350</v>
+        <v>3328</v>
       </c>
       <c r="C3418" t="inlineStr">
         <is>
-          <t xml:space="preserve">EDER RODRIGUES DA SILVA </t>
+          <t>ALAN ARAUJO DA SILVA</t>
         </is>
       </c>
       <c r="D3418" t="inlineStr">
         <is>
-          <t>EDERS</t>
+          <t>ARSILVA</t>
         </is>
       </c>
     </row>
     <row r="3419">
       <c r="A3419" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3419" t="n">
-        <v>3373</v>
+        <v>3350</v>
       </c>
       <c r="C3419" t="inlineStr">
         <is>
-          <t xml:space="preserve">NATANAEL TAVARES DE SOUSA </t>
+          <t xml:space="preserve">EDER RODRIGUES DA SILVA </t>
         </is>
       </c>
       <c r="D3419" t="inlineStr">
         <is>
-          <t>NTSOUSA</t>
+          <t>EDERS</t>
         </is>
       </c>
     </row>
@@ -68818,156 +68818,156 @@
         </is>
       </c>
       <c r="B3420" t="n">
-        <v>3374</v>
+        <v>3373</v>
       </c>
       <c r="C3420" t="inlineStr">
         <is>
-          <t>REINALDO DA SILVA COSTA</t>
+          <t xml:space="preserve">NATANAEL TAVARES DE SOUSA </t>
         </is>
       </c>
       <c r="D3420" t="inlineStr">
         <is>
-          <t>RSCOSTA</t>
+          <t>NTSOUSA</t>
         </is>
       </c>
     </row>
     <row r="3421">
       <c r="A3421" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3421" t="n">
-        <v>3399</v>
+        <v>3374</v>
       </c>
       <c r="C3421" t="inlineStr">
         <is>
-          <t xml:space="preserve">RICARDO BARBOSA DOS SANTOS </t>
+          <t>REINALDO DA SILVA COSTA</t>
         </is>
       </c>
       <c r="D3421" t="inlineStr">
         <is>
-          <t>RICARDOSAN</t>
+          <t>RSCOSTA</t>
         </is>
       </c>
     </row>
     <row r="3422">
       <c r="A3422" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3422" t="n">
-        <v>3427</v>
+        <v>3399</v>
       </c>
       <c r="C3422" t="inlineStr">
         <is>
-          <t>ROQUE COMERCIO TEMPORARIO</t>
+          <t xml:space="preserve">RICARDO BARBOSA DOS SANTOS </t>
         </is>
       </c>
       <c r="D3422" t="inlineStr">
         <is>
-          <t>ROQUECOM</t>
+          <t>RICARDOSAN</t>
         </is>
       </c>
     </row>
     <row r="3423">
       <c r="A3423" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3423" t="n">
-        <v>3428</v>
+        <v>3427</v>
       </c>
       <c r="C3423" t="inlineStr">
         <is>
-          <t>ROQUE PLUS TEMPORARIO</t>
+          <t>ROQUE COMERCIO TEMPORARIO</t>
         </is>
       </c>
       <c r="D3423" t="inlineStr">
         <is>
-          <t>ROQUEPLUS</t>
+          <t>ROQUECOM</t>
         </is>
       </c>
     </row>
     <row r="3424">
       <c r="A3424" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3424" t="n">
-        <v>3432</v>
+        <v>3428</v>
       </c>
       <c r="C3424" t="inlineStr">
         <is>
-          <t>PATRICIA DOS SANTOS NONATO OLIVEIRA</t>
+          <t>ROQUE PLUS TEMPORARIO</t>
         </is>
       </c>
       <c r="D3424" t="inlineStr">
         <is>
-          <t>PATRICIAD</t>
+          <t>ROQUEPLUS</t>
         </is>
       </c>
     </row>
     <row r="3425">
       <c r="A3425" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3425" t="n">
-        <v>3448</v>
+        <v>3432</v>
       </c>
       <c r="C3425" t="inlineStr">
         <is>
-          <t xml:space="preserve">GABRIEL SOUZA CARVALHO </t>
+          <t>PATRICIA DOS SANTOS NONATO OLIVEIRA</t>
         </is>
       </c>
       <c r="D3425" t="inlineStr">
         <is>
-          <t>GABRIEL20</t>
+          <t>PATRICIAD</t>
         </is>
       </c>
     </row>
     <row r="3426">
       <c r="A3426" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3426" t="n">
-        <v>3465</v>
+        <v>3448</v>
       </c>
       <c r="C3426" t="inlineStr">
         <is>
-          <t>LUIZA MARIA BARRETO BARBOSA</t>
+          <t xml:space="preserve">GABRIEL SOUZA CARVALHO </t>
         </is>
       </c>
       <c r="D3426" t="inlineStr">
         <is>
-          <t>LUIZA.MARIA</t>
+          <t>GABRIEL20</t>
         </is>
       </c>
     </row>
     <row r="3427">
       <c r="A3427" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3427" t="n">
-        <v>3468</v>
+        <v>3465</v>
       </c>
       <c r="C3427" t="inlineStr">
         <is>
-          <t>KAWA ALMEIDA CAMPOS</t>
+          <t>LUIZA MARIA BARRETO BARBOSA</t>
         </is>
       </c>
       <c r="D3427" t="inlineStr">
         <is>
-          <t>KAWA</t>
+          <t>LUIZA.MARIA</t>
         </is>
       </c>
     </row>
@@ -68978,16 +68978,16 @@
         </is>
       </c>
       <c r="B3428" t="n">
-        <v>3476</v>
+        <v>3468</v>
       </c>
       <c r="C3428" t="inlineStr">
         <is>
-          <t xml:space="preserve"> FRANCISCA LEIDIANE M. MENDES NASCIMENTO</t>
+          <t>KAWA ALMEIDA CAMPOS</t>
         </is>
       </c>
       <c r="D3428" t="inlineStr">
         <is>
-          <t>FLEIDIANE</t>
+          <t>KAWA</t>
         </is>
       </c>
     </row>
@@ -68998,76 +68998,76 @@
         </is>
       </c>
       <c r="B3429" t="n">
-        <v>3477</v>
+        <v>3476</v>
       </c>
       <c r="C3429" t="inlineStr">
         <is>
-          <t>MARIA THAIS MARTINS PEREIRA SILVA</t>
+          <t xml:space="preserve"> FRANCISCA LEIDIANE M. MENDES NASCIMENTO</t>
         </is>
       </c>
       <c r="D3429" t="inlineStr">
         <is>
-          <t>MTHAIS</t>
+          <t>FLEIDIANE</t>
         </is>
       </c>
     </row>
     <row r="3430">
       <c r="A3430" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3430" t="n">
-        <v>3271</v>
+        <v>3477</v>
       </c>
       <c r="C3430" t="inlineStr">
         <is>
-          <t>DIEGO DE ARAUJO CALÁBRIA</t>
+          <t>MARIA THAIS MARTINS PEREIRA SILVA</t>
         </is>
       </c>
       <c r="D3430" t="inlineStr">
         <is>
-          <t>ARAUJOC</t>
+          <t>MTHAIS</t>
         </is>
       </c>
     </row>
     <row r="3431">
       <c r="A3431" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3431" t="n">
-        <v>3272</v>
+        <v>3271</v>
       </c>
       <c r="C3431" t="inlineStr">
         <is>
-          <t>ANNE BEATRIZ SILVA VIRGINO</t>
+          <t>DIEGO DE ARAUJO CALÁBRIA</t>
         </is>
       </c>
       <c r="D3431" t="inlineStr">
         <is>
-          <t>ABVIRGINIO</t>
+          <t>ARAUJOC</t>
         </is>
       </c>
     </row>
     <row r="3432">
       <c r="A3432" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3432" t="n">
-        <v>3293</v>
+        <v>3272</v>
       </c>
       <c r="C3432" t="inlineStr">
         <is>
-          <t xml:space="preserve">CARLOS ALBERTO VIRIATO SANTOS </t>
+          <t>ANNE BEATRIZ SILVA VIRGINO</t>
         </is>
       </c>
       <c r="D3432" t="inlineStr">
         <is>
-          <t>CVIRIATO</t>
+          <t>ABVIRGINIO</t>
         </is>
       </c>
     </row>
@@ -69078,16 +69078,16 @@
         </is>
       </c>
       <c r="B3433" t="n">
-        <v>3381</v>
+        <v>3293</v>
       </c>
       <c r="C3433" t="inlineStr">
         <is>
-          <t>ALAN CAIQUE SANTOS E SANTOS</t>
+          <t xml:space="preserve">CARLOS ALBERTO VIRIATO SANTOS </t>
         </is>
       </c>
       <c r="D3433" t="inlineStr">
         <is>
-          <t>ALANSANTOS</t>
+          <t>CVIRIATO</t>
         </is>
       </c>
     </row>
@@ -69098,116 +69098,116 @@
         </is>
       </c>
       <c r="B3434" t="n">
-        <v>3443</v>
+        <v>3381</v>
       </c>
       <c r="C3434" t="inlineStr">
         <is>
-          <t>SANON MOREIRA SOUZA</t>
+          <t>ALAN CAIQUE SANTOS E SANTOS</t>
         </is>
       </c>
       <c r="D3434" t="inlineStr">
         <is>
-          <t>SANON</t>
+          <t>ALANSANTOS</t>
         </is>
       </c>
     </row>
     <row r="3435">
       <c r="A3435" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3435" t="n">
-        <v>3516</v>
+        <v>3443</v>
       </c>
       <c r="C3435" t="inlineStr">
         <is>
-          <t>FRANCISCO RILDER TELES DE OLIVEIRA</t>
+          <t>SANON MOREIRA SOUZA</t>
         </is>
       </c>
       <c r="D3435" t="inlineStr">
         <is>
-          <t>RILDER</t>
+          <t>SANON</t>
         </is>
       </c>
     </row>
     <row r="3436">
       <c r="A3436" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3436" t="n">
-        <v>3519</v>
+        <v>3516</v>
       </c>
       <c r="C3436" t="inlineStr">
         <is>
-          <t>MARIA LUANA DE ALMEIDA BATISTA</t>
+          <t>FRANCISCO RILDER TELES DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D3436" t="inlineStr">
         <is>
-          <t>M.LUANA</t>
+          <t>RILDER</t>
         </is>
       </c>
     </row>
     <row r="3437">
       <c r="A3437" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3437" t="n">
-        <v>3540</v>
+        <v>3519</v>
       </c>
       <c r="C3437" t="inlineStr">
         <is>
-          <t>HELEN VITORIA OLIVEIRA DA ROCHA</t>
+          <t>MARIA LUANA DE ALMEIDA BATISTA</t>
         </is>
       </c>
       <c r="D3437" t="inlineStr">
         <is>
-          <t>H.VITORIA</t>
+          <t>M.LUANA</t>
         </is>
       </c>
     </row>
     <row r="3438">
       <c r="A3438" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B3438" t="n">
-        <v>3559</v>
+        <v>3540</v>
       </c>
       <c r="C3438" t="inlineStr">
         <is>
-          <t>ARKBERYS TELES DE SOUSA</t>
+          <t>HELEN VITORIA OLIVEIRA DA ROCHA</t>
         </is>
       </c>
       <c r="D3438" t="inlineStr">
         <is>
-          <t>ARKBERYS</t>
+          <t>H.VITORIA</t>
         </is>
       </c>
     </row>
     <row r="3439">
       <c r="A3439" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3439" t="n">
-        <v>3567</v>
+        <v>3559</v>
       </c>
       <c r="C3439" t="inlineStr">
         <is>
-          <t>PEDRO HENRIQUE VIEIRA DE LIMA</t>
+          <t>ARKBERYS TELES DE SOUSA</t>
         </is>
       </c>
       <c r="D3439" t="inlineStr">
         <is>
-          <t>P.LIMA</t>
+          <t>ARKBERYS</t>
         </is>
       </c>
     </row>
@@ -69218,76 +69218,76 @@
         </is>
       </c>
       <c r="B3440" t="n">
-        <v>3331</v>
+        <v>3567</v>
       </c>
       <c r="C3440" t="inlineStr">
         <is>
-          <t>LOUIZE VANIELLE RODRIGUES FARIAS</t>
+          <t>PEDRO HENRIQUE VIEIRA DE LIMA</t>
         </is>
       </c>
       <c r="D3440" t="inlineStr">
         <is>
-          <t>LVFARIAS</t>
+          <t>P.LIMA</t>
         </is>
       </c>
     </row>
     <row r="3441">
       <c r="A3441" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3441" t="n">
-        <v>3334</v>
+        <v>3331</v>
       </c>
       <c r="C3441" t="inlineStr">
         <is>
-          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+          <t>LOUIZE VANIELLE RODRIGUES FARIAS</t>
         </is>
       </c>
       <c r="D3441" t="inlineStr">
         <is>
-          <t>MTGASPAR</t>
+          <t>LVFARIAS</t>
         </is>
       </c>
     </row>
     <row r="3442">
       <c r="A3442" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3442" t="n">
-        <v>3345</v>
+        <v>3334</v>
       </c>
       <c r="C3442" t="inlineStr">
         <is>
-          <t>AURICÉLIA INACIO PEREIRA</t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
       <c r="D3442" t="inlineStr">
         <is>
-          <t>AIPEREIRA</t>
+          <t>MTGASPAR</t>
         </is>
       </c>
     </row>
     <row r="3443">
       <c r="A3443" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3443" t="n">
-        <v>3363</v>
+        <v>3345</v>
       </c>
       <c r="C3443" t="inlineStr">
         <is>
-          <t>IASMIN LEAL ALVES</t>
+          <t>AURICÉLIA INACIO PEREIRA</t>
         </is>
       </c>
       <c r="D3443" t="inlineStr">
         <is>
-          <t>ILALVES</t>
+          <t>AIPEREIRA</t>
         </is>
       </c>
     </row>
@@ -69298,196 +69298,196 @@
         </is>
       </c>
       <c r="B3444" t="n">
-        <v>3370</v>
+        <v>3363</v>
       </c>
       <c r="C3444" t="inlineStr">
         <is>
-          <t>CARLOS DIEGO ARAUJO ALMEIDA</t>
+          <t>IASMIN LEAL ALVES</t>
         </is>
       </c>
       <c r="D3444" t="inlineStr">
         <is>
-          <t>CDIEGO</t>
+          <t>ILALVES</t>
         </is>
       </c>
     </row>
     <row r="3445">
       <c r="A3445" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3445" t="n">
-        <v>3379</v>
+        <v>3370</v>
       </c>
       <c r="C3445" t="inlineStr">
         <is>
-          <t xml:space="preserve">MATHEUS EVANGELISTA FERREIRA </t>
+          <t>CARLOS DIEGO ARAUJO ALMEIDA</t>
         </is>
       </c>
       <c r="D3445" t="inlineStr">
         <is>
-          <t>MMFERREIRA</t>
+          <t>CDIEGO</t>
         </is>
       </c>
     </row>
     <row r="3446">
       <c r="A3446" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3446" t="n">
-        <v>3419</v>
+        <v>3379</v>
       </c>
       <c r="C3446" t="inlineStr">
         <is>
-          <t xml:space="preserve">DAVID EVANGELISTA SILVA </t>
+          <t xml:space="preserve">MATHEUS EVANGELISTA FERREIRA </t>
         </is>
       </c>
       <c r="D3446" t="inlineStr">
         <is>
-          <t>DAVID</t>
+          <t>MMFERREIRA</t>
         </is>
       </c>
     </row>
     <row r="3447">
       <c r="A3447" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3447" t="n">
-        <v>3423</v>
+        <v>3419</v>
       </c>
       <c r="C3447" t="inlineStr">
         <is>
-          <t>MARCIO JOSE TIAGO</t>
+          <t xml:space="preserve">DAVID EVANGELISTA SILVA </t>
         </is>
       </c>
       <c r="D3447" t="inlineStr">
         <is>
-          <t>MJTIAGO</t>
+          <t>DAVID</t>
         </is>
       </c>
     </row>
     <row r="3448">
       <c r="A3448" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3448" t="n">
-        <v>3453</v>
+        <v>3423</v>
       </c>
       <c r="C3448" t="inlineStr">
         <is>
-          <t xml:space="preserve">LAURIENE SILVA BARBOSA </t>
+          <t>MARCIO JOSE TIAGO</t>
         </is>
       </c>
       <c r="D3448" t="inlineStr">
         <is>
-          <t>LAURIENE</t>
+          <t>MJTIAGO</t>
         </is>
       </c>
     </row>
     <row r="3449">
       <c r="A3449" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3449" t="n">
-        <v>3478</v>
+        <v>3453</v>
       </c>
       <c r="C3449" t="inlineStr">
         <is>
-          <t>LEANDRO BRITO NOGUEIRA DE OLIVEIRA</t>
+          <t xml:space="preserve">LAURIENE SILVA BARBOSA </t>
         </is>
       </c>
       <c r="D3449" t="inlineStr">
         <is>
-          <t>LBNOGUEIRA</t>
+          <t>LAURIENE</t>
         </is>
       </c>
     </row>
     <row r="3450">
       <c r="A3450" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3450" t="n">
-        <v>3479</v>
+        <v>3478</v>
       </c>
       <c r="C3450" t="inlineStr">
         <is>
-          <t>ESDRAS ALESSANDRO SANTOS SANTANA</t>
+          <t>LEANDRO BRITO NOGUEIRA DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D3450" t="inlineStr">
         <is>
-          <t>EALESSANDRO</t>
+          <t>LBNOGUEIRA</t>
         </is>
       </c>
     </row>
     <row r="3451">
       <c r="A3451" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3451" t="n">
-        <v>3480</v>
+        <v>3479</v>
       </c>
       <c r="C3451" t="inlineStr">
         <is>
-          <t xml:space="preserve">LUCIMARA SOUSA LIMA </t>
+          <t>ESDRAS ALESSANDRO SANTOS SANTANA</t>
         </is>
       </c>
       <c r="D3451" t="inlineStr">
         <is>
-          <t>LUCIMARA</t>
+          <t>EALESSANDRO</t>
         </is>
       </c>
     </row>
     <row r="3452">
       <c r="A3452" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3452" t="n">
-        <v>3482</v>
+        <v>3480</v>
       </c>
       <c r="C3452" t="inlineStr">
         <is>
-          <t>DANIEL FERNANDES DINIZ HERACLIO</t>
+          <t xml:space="preserve">LUCIMARA SOUSA LIMA </t>
         </is>
       </c>
       <c r="D3452" t="inlineStr">
         <is>
-          <t>DFDINIZ</t>
+          <t>LUCIMARA</t>
         </is>
       </c>
     </row>
     <row r="3453">
       <c r="A3453" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3453" t="n">
-        <v>3518</v>
+        <v>3482</v>
       </c>
       <c r="C3453" t="inlineStr">
         <is>
-          <t>RAMYRA ALVES FELIX DA SILVA</t>
+          <t>DANIEL FERNANDES DINIZ HERACLIO</t>
         </is>
       </c>
       <c r="D3453" t="inlineStr">
         <is>
-          <t>RFELIX</t>
+          <t>DFDINIZ</t>
         </is>
       </c>
     </row>
@@ -69498,36 +69498,36 @@
         </is>
       </c>
       <c r="B3454" t="n">
-        <v>3534</v>
+        <v>3518</v>
       </c>
       <c r="C3454" t="inlineStr">
         <is>
-          <t xml:space="preserve">CAIO DE SOUZA VINHAS </t>
+          <t>RAMYRA ALVES FELIX DA SILVA</t>
         </is>
       </c>
       <c r="D3454" t="inlineStr">
         <is>
-          <t>CVINHAS</t>
+          <t>RFELIX</t>
         </is>
       </c>
     </row>
     <row r="3455">
       <c r="A3455" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3455" t="n">
-        <v>3535</v>
+        <v>3534</v>
       </c>
       <c r="C3455" t="inlineStr">
         <is>
-          <t>ROMARIO DE SOUSA SILVA</t>
+          <t xml:space="preserve">CAIO DE SOUZA VINHAS </t>
         </is>
       </c>
       <c r="D3455" t="inlineStr">
         <is>
-          <t>RSOUSAS</t>
+          <t>CVINHAS</t>
         </is>
       </c>
     </row>
@@ -69538,56 +69538,56 @@
         </is>
       </c>
       <c r="B3456" t="n">
-        <v>3536</v>
+        <v>3535</v>
       </c>
       <c r="C3456" t="inlineStr">
         <is>
-          <t>JHONATAS CARVALHO OLIVEIRA</t>
+          <t>ROMARIO DE SOUSA SILVA</t>
         </is>
       </c>
       <c r="D3456" t="inlineStr">
         <is>
-          <t>JHONATASC</t>
+          <t>RSOUSAS</t>
         </is>
       </c>
     </row>
     <row r="3457">
       <c r="A3457" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3457" t="n">
-        <v>940529</v>
+        <v>3536</v>
       </c>
       <c r="C3457" t="inlineStr">
         <is>
-          <t>EDGAR FELIX - FL9</t>
+          <t>JHONATAS CARVALHO OLIVEIRA</t>
         </is>
       </c>
       <c r="D3457" t="inlineStr">
         <is>
-          <t>EDGAR F</t>
+          <t>JHONATASC</t>
         </is>
       </c>
     </row>
     <row r="3458">
       <c r="A3458" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3458" t="n">
-        <v>3304</v>
+        <v>940529</v>
       </c>
       <c r="C3458" t="inlineStr">
         <is>
-          <t>JOACI GUILHERME GONÇALVES DA LUZ</t>
+          <t>EDGAR FELIX - FL9</t>
         </is>
       </c>
       <c r="D3458" t="inlineStr">
         <is>
-          <t>JLUZ</t>
+          <t>EDGAR F</t>
         </is>
       </c>
     </row>
@@ -69598,16 +69598,16 @@
         </is>
       </c>
       <c r="B3459" t="n">
-        <v>3305</v>
+        <v>3304</v>
       </c>
       <c r="C3459" t="inlineStr">
         <is>
-          <t>JOÃO VITOR DE ARAÚJO GONÇALVES</t>
+          <t>JOACI GUILHERME GONÇALVES DA LUZ</t>
         </is>
       </c>
       <c r="D3459" t="inlineStr">
         <is>
-          <t>JJVITOR</t>
+          <t>JLUZ</t>
         </is>
       </c>
     </row>
@@ -69618,36 +69618,36 @@
         </is>
       </c>
       <c r="B3460" t="n">
-        <v>3306</v>
+        <v>3305</v>
       </c>
       <c r="C3460" t="inlineStr">
         <is>
-          <t>WENDERSON MARCOS DOS SANTOS</t>
+          <t>JOÃO VITOR DE ARAÚJO GONÇALVES</t>
         </is>
       </c>
       <c r="D3460" t="inlineStr">
         <is>
-          <t>WWMARCOS</t>
+          <t>JJVITOR</t>
         </is>
       </c>
     </row>
     <row r="3461">
       <c r="A3461" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3461" t="n">
-        <v>3335</v>
+        <v>3306</v>
       </c>
       <c r="C3461" t="inlineStr">
         <is>
-          <t>EDILBERTO LEMOS DE LIMA</t>
+          <t>WENDERSON MARCOS DOS SANTOS</t>
         </is>
       </c>
       <c r="D3461" t="inlineStr">
         <is>
-          <t>ELEMOS</t>
+          <t>WWMARCOS</t>
         </is>
       </c>
     </row>
@@ -69658,136 +69658,136 @@
         </is>
       </c>
       <c r="B3462" t="n">
-        <v>3336</v>
+        <v>3335</v>
       </c>
       <c r="C3462" t="inlineStr">
         <is>
-          <t>EZEQUIEL SOUZA DO NASCIMENTO</t>
+          <t>EDILBERTO LEMOS DE LIMA</t>
         </is>
       </c>
       <c r="D3462" t="inlineStr">
         <is>
-          <t>ESNASCIMENTO</t>
+          <t>ELEMOS</t>
         </is>
       </c>
     </row>
     <row r="3463">
       <c r="A3463" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3463" t="n">
-        <v>3341</v>
+        <v>3336</v>
       </c>
       <c r="C3463" t="inlineStr">
         <is>
-          <t>ALCIONE MARIANO DE OLIVEIRA</t>
+          <t>EZEQUIEL SOUZA DO NASCIMENTO</t>
         </is>
       </c>
       <c r="D3463" t="inlineStr">
         <is>
-          <t>AMOLIVEIRA</t>
+          <t>ESNASCIMENTO</t>
         </is>
       </c>
     </row>
     <row r="3464">
       <c r="A3464" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3464" t="n">
-        <v>3401</v>
+        <v>3341</v>
       </c>
       <c r="C3464" t="inlineStr">
         <is>
-          <t xml:space="preserve">TULIO HENRIQUE DA SILVA CARVALHO </t>
+          <t>ALCIONE MARIANO DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D3464" t="inlineStr">
         <is>
-          <t>TULIO</t>
+          <t>AMOLIVEIRA</t>
         </is>
       </c>
     </row>
     <row r="3465">
       <c r="A3465" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3465" t="n">
-        <v>3411</v>
+        <v>3401</v>
       </c>
       <c r="C3465" t="inlineStr">
         <is>
-          <t>CONEXAO RUBYA DANILLA</t>
+          <t xml:space="preserve">TULIO HENRIQUE DA SILVA CARVALHO </t>
         </is>
       </c>
       <c r="D3465" t="inlineStr">
         <is>
-          <t>CONEXAORUBYA</t>
+          <t>TULIO</t>
         </is>
       </c>
     </row>
     <row r="3466">
       <c r="A3466" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3466" t="n">
-        <v>3412</v>
+        <v>3411</v>
       </c>
       <c r="C3466" t="inlineStr">
         <is>
-          <t>CONEXAO RAFAEL</t>
+          <t>CONEXAO RUBYA DANILLA</t>
         </is>
       </c>
       <c r="D3466" t="inlineStr">
         <is>
-          <t>CONEXAORAFAEL</t>
+          <t>CONEXAORUBYA</t>
         </is>
       </c>
     </row>
     <row r="3467">
       <c r="A3467" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3467" t="n">
-        <v>3558</v>
+        <v>3412</v>
       </c>
       <c r="C3467" t="inlineStr">
         <is>
-          <t>WALLYS QUEIROZ VIANA</t>
+          <t>CONEXAO RAFAEL</t>
         </is>
       </c>
       <c r="D3467" t="inlineStr">
         <is>
-          <t>WALLYS</t>
+          <t>CONEXAORAFAEL</t>
         </is>
       </c>
     </row>
     <row r="3468">
       <c r="A3468" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3468" t="n">
-        <v>3264</v>
+        <v>3558</v>
       </c>
       <c r="C3468" t="inlineStr">
         <is>
-          <t xml:space="preserve">WILTON CARLOS MACIEL DE ASSIS </t>
+          <t>WALLYS QUEIROZ VIANA</t>
         </is>
       </c>
       <c r="D3468" t="inlineStr">
         <is>
-          <t>WCMACIEL</t>
+          <t>WALLYS</t>
         </is>
       </c>
     </row>
@@ -69798,56 +69798,56 @@
         </is>
       </c>
       <c r="B3469" t="n">
-        <v>3340</v>
+        <v>3264</v>
       </c>
       <c r="C3469" t="inlineStr">
         <is>
-          <t>ROGELENO FARIAS FEIJÃO FILHO</t>
+          <t xml:space="preserve">WILTON CARLOS MACIEL DE ASSIS </t>
         </is>
       </c>
       <c r="D3469" t="inlineStr">
         <is>
-          <t>RFEIJAO</t>
+          <t>WCMACIEL</t>
         </is>
       </c>
     </row>
     <row r="3470">
       <c r="A3470" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3470" t="n">
-        <v>940550</v>
+        <v>3340</v>
       </c>
       <c r="C3470" t="inlineStr">
         <is>
-          <t>RAFAELE RIBEIRO CARNEIRO</t>
+          <t>ROGELENO FARIAS FEIJÃO FILHO</t>
         </is>
       </c>
       <c r="D3470" t="inlineStr">
         <is>
-          <t>RAFAELE</t>
+          <t>RFEIJAO</t>
         </is>
       </c>
     </row>
     <row r="3471">
       <c r="A3471" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>99</t>
         </is>
       </c>
       <c r="B3471" t="n">
-        <v>3377</v>
+        <v>940550</v>
       </c>
       <c r="C3471" t="inlineStr">
         <is>
-          <t xml:space="preserve"> ISALTINO BISPO DE OLIVEIRA JUNIOR</t>
+          <t>RAFAELE RIBEIRO CARNEIRO</t>
         </is>
       </c>
       <c r="D3471" t="inlineStr">
         <is>
-          <t>BJUNIOR</t>
+          <t>RAFAELE</t>
         </is>
       </c>
     </row>
@@ -69858,56 +69858,56 @@
         </is>
       </c>
       <c r="B3472" t="n">
-        <v>3425</v>
+        <v>3377</v>
       </c>
       <c r="C3472" t="inlineStr">
         <is>
-          <t xml:space="preserve"> CIRLANE ARAUJO SOUZA </t>
+          <t xml:space="preserve"> ISALTINO BISPO DE OLIVEIRA JUNIOR</t>
         </is>
       </c>
       <c r="D3472" t="inlineStr">
         <is>
-          <t>CIRLANES</t>
+          <t>BJUNIOR</t>
         </is>
       </c>
     </row>
     <row r="3473">
       <c r="A3473" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3473" t="n">
-        <v>3454</v>
+        <v>3425</v>
       </c>
       <c r="C3473" t="inlineStr">
         <is>
-          <t>ANTONIA SAMARA DE SOUZA SOARES</t>
+          <t xml:space="preserve"> CIRLANE ARAUJO SOUZA </t>
         </is>
       </c>
       <c r="D3473" t="inlineStr">
         <is>
-          <t>ANTSAMARA</t>
+          <t>CIRLANES</t>
         </is>
       </c>
     </row>
     <row r="3474">
       <c r="A3474" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3474" t="n">
-        <v>3491</v>
+        <v>3454</v>
       </c>
       <c r="C3474" t="inlineStr">
         <is>
-          <t>PEDRO JOSE DO NASCIMENTO NETO</t>
+          <t>ANTONIA SAMARA DE SOUZA SOARES</t>
         </is>
       </c>
       <c r="D3474" t="inlineStr">
         <is>
-          <t>P.JOSE</t>
+          <t>ANTSAMARA</t>
         </is>
       </c>
     </row>
@@ -69918,36 +69918,36 @@
         </is>
       </c>
       <c r="B3475" t="n">
-        <v>3492</v>
+        <v>3491</v>
       </c>
       <c r="C3475" t="inlineStr">
         <is>
-          <t>PAULA CARLA CALDAS MOTA</t>
+          <t>PEDRO JOSE DO NASCIMENTO NETO</t>
         </is>
       </c>
       <c r="D3475" t="inlineStr">
         <is>
-          <t>P.CARLA</t>
+          <t>P.JOSE</t>
         </is>
       </c>
     </row>
     <row r="3476">
       <c r="A3476" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3476" t="n">
-        <v>3542</v>
+        <v>3492</v>
       </c>
       <c r="C3476" t="inlineStr">
         <is>
-          <t>ANTONIA MILENA SOUSA ANDRADE</t>
+          <t>PAULA CARLA CALDAS MOTA</t>
         </is>
       </c>
       <c r="D3476" t="inlineStr">
         <is>
-          <t>A.MILENA</t>
+          <t>P.CARLA</t>
         </is>
       </c>
     </row>
@@ -69958,56 +69958,56 @@
         </is>
       </c>
       <c r="B3477" t="n">
-        <v>3547</v>
+        <v>3542</v>
       </c>
       <c r="C3477" t="inlineStr">
         <is>
-          <t xml:space="preserve">DAVI PEREIRA DA SILVA </t>
+          <t>ANTONIA MILENA SOUSA ANDRADE</t>
         </is>
       </c>
       <c r="D3477" t="inlineStr">
         <is>
-          <t>DPSILVA</t>
+          <t>A.MILENA</t>
         </is>
       </c>
     </row>
     <row r="3478">
       <c r="A3478" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3478" t="n">
-        <v>3552</v>
+        <v>3547</v>
       </c>
       <c r="C3478" t="inlineStr">
         <is>
-          <t>PAULO SERGIO MENDES DE OLIVEIRA</t>
+          <t xml:space="preserve">DAVI PEREIRA DA SILVA </t>
         </is>
       </c>
       <c r="D3478" t="inlineStr">
         <is>
-          <t>PSMENDES</t>
+          <t>DPSILVA</t>
         </is>
       </c>
     </row>
     <row r="3479">
       <c r="A3479" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3479" t="n">
-        <v>3294</v>
+        <v>3552</v>
       </c>
       <c r="C3479" t="inlineStr">
         <is>
-          <t>GLEICIANE MIRANDA DE MORAIS</t>
+          <t>PAULO SERGIO MENDES DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D3479" t="inlineStr">
         <is>
-          <t>GMIRANDA</t>
+          <t>PSMENDES</t>
         </is>
       </c>
     </row>
@@ -70018,176 +70018,176 @@
         </is>
       </c>
       <c r="B3480" t="n">
-        <v>3295</v>
+        <v>3294</v>
       </c>
       <c r="C3480" t="inlineStr">
         <is>
-          <t>MARIA ESTEFANNY DA SILVA MOURA</t>
+          <t>GLEICIANE MIRANDA DE MORAIS</t>
         </is>
       </c>
       <c r="D3480" t="inlineStr">
         <is>
-          <t>MESTEFANNY</t>
+          <t>GMIRANDA</t>
         </is>
       </c>
     </row>
     <row r="3481">
       <c r="A3481" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3481" t="n">
-        <v>3296</v>
+        <v>3295</v>
       </c>
       <c r="C3481" t="inlineStr">
         <is>
-          <t>PEDRO IAGO FONSECA EVANGELISTA</t>
+          <t>MARIA ESTEFANNY DA SILVA MOURA</t>
         </is>
       </c>
       <c r="D3481" t="inlineStr">
         <is>
-          <t>PIFONSECA</t>
+          <t>MESTEFANNY</t>
         </is>
       </c>
     </row>
     <row r="3482">
       <c r="A3482" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3482" t="n">
-        <v>940544</v>
+        <v>3296</v>
       </c>
       <c r="C3482" t="inlineStr">
         <is>
-          <t>LUTY LOG TRANSPORTES - FL8</t>
+          <t>PEDRO IAGO FONSECA EVANGELISTA</t>
         </is>
       </c>
       <c r="D3482" t="inlineStr">
         <is>
-          <t>LUTY LOG</t>
+          <t>PIFONSECA</t>
         </is>
       </c>
     </row>
     <row r="3483">
       <c r="A3483" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B3483" t="n">
-        <v>3380</v>
+        <v>940544</v>
       </c>
       <c r="C3483" t="inlineStr">
         <is>
-          <t>FRANCISCO MATHEUS RABELO DA COSTA</t>
+          <t>LUTY LOG TRANSPORTES - FL8</t>
         </is>
       </c>
       <c r="D3483" t="inlineStr">
         <is>
-          <t>FMATHEUS</t>
+          <t>LUTY LOG</t>
         </is>
       </c>
     </row>
     <row r="3484">
       <c r="A3484" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3484" t="n">
-        <v>3410</v>
+        <v>3380</v>
       </c>
       <c r="C3484" t="inlineStr">
         <is>
-          <t xml:space="preserve"> BRENO ALLAN DE JESUS</t>
+          <t>FRANCISCO MATHEUS RABELO DA COSTA</t>
         </is>
       </c>
       <c r="D3484" t="inlineStr">
         <is>
-          <t>JESUS</t>
+          <t>FMATHEUS</t>
         </is>
       </c>
     </row>
     <row r="3485">
       <c r="A3485" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3485" t="n">
-        <v>3444</v>
+        <v>3410</v>
       </c>
       <c r="C3485" t="inlineStr">
         <is>
-          <t>THIAGO COSTA SILVA</t>
+          <t xml:space="preserve"> BRENO ALLAN DE JESUS</t>
         </is>
       </c>
       <c r="D3485" t="inlineStr">
         <is>
-          <t>THIAGOC</t>
+          <t>JESUS</t>
         </is>
       </c>
     </row>
     <row r="3486">
       <c r="A3486" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3486" t="n">
-        <v>3456</v>
+        <v>3444</v>
       </c>
       <c r="C3486" t="inlineStr">
         <is>
-          <t>FELIPE BOTH MAZUCHINI</t>
+          <t>THIAGO COSTA SILVA</t>
         </is>
       </c>
       <c r="D3486" t="inlineStr">
         <is>
-          <t>FELIPEB</t>
+          <t>THIAGOC</t>
         </is>
       </c>
     </row>
     <row r="3487">
       <c r="A3487" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3487" t="n">
-        <v>3457</v>
+        <v>3456</v>
       </c>
       <c r="C3487" t="inlineStr">
         <is>
-          <t>FRANKLIN VIEIRA GOMES</t>
+          <t>FELIPE BOTH MAZUCHINI</t>
         </is>
       </c>
       <c r="D3487" t="inlineStr">
         <is>
-          <t>VIEIRAF</t>
+          <t>FELIPEB</t>
         </is>
       </c>
     </row>
     <row r="3488">
       <c r="A3488" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3488" t="n">
-        <v>3507</v>
+        <v>3457</v>
       </c>
       <c r="C3488" t="inlineStr">
         <is>
-          <t>KARINE TEODORA ALVES DE OLIVEIRA</t>
+          <t>FRANKLIN VIEIRA GOMES</t>
         </is>
       </c>
       <c r="D3488" t="inlineStr">
         <is>
-          <t>KOLIVEIRA</t>
+          <t>VIEIRAF</t>
         </is>
       </c>
     </row>
@@ -70198,14 +70198,34 @@
         </is>
       </c>
       <c r="B3489" t="n">
+        <v>3507</v>
+      </c>
+      <c r="C3489" t="inlineStr">
+        <is>
+          <t>KARINE TEODORA ALVES DE OLIVEIRA</t>
+        </is>
+      </c>
+      <c r="D3489" t="inlineStr">
+        <is>
+          <t>KOLIVEIRA</t>
+        </is>
+      </c>
+    </row>
+    <row r="3490">
+      <c r="A3490" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B3490" t="n">
         <v>3520</v>
       </c>
-      <c r="C3489" t="inlineStr">
+      <c r="C3490" t="inlineStr">
         <is>
           <t xml:space="preserve"> EMERSON FILIPE MELO DE AGUIAR</t>
         </is>
       </c>
-      <c r="D3489" t="inlineStr">
+      <c r="D3490" t="inlineStr">
         <is>
           <t>E.FILIPE</t>
         </is>

</xml_diff>

<commit_message>
chore(data): batch update intraday televendas - 08:02:02
</commit_message>
<xml_diff>
--- a/data/dim_televendas.xlsx
+++ b/data/dim_televendas.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3493"/>
+  <dimension ref="A1:D3494"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -67394,80 +67394,80 @@
     <row r="3349">
       <c r="A3349" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3349" t="n">
-        <v>3351</v>
+        <v>3580</v>
       </c>
       <c r="C3349" t="inlineStr">
         <is>
-          <t>HAWLLYSON DA SILVA COUTINHO</t>
+          <t>ALEXANDRE MARTINS CHAVES</t>
         </is>
       </c>
       <c r="D3349" t="inlineStr">
         <is>
-          <t>HCOUTINHO</t>
+          <t>MARTINS</t>
         </is>
       </c>
     </row>
     <row r="3350">
       <c r="A3350" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3350" t="n">
-        <v>940553</v>
+        <v>3351</v>
       </c>
       <c r="C3350" t="inlineStr">
         <is>
-          <t>LUTY TRANSPORTES- BA</t>
+          <t>HAWLLYSON DA SILVA COUTINHO</t>
         </is>
       </c>
       <c r="D3350" t="inlineStr">
         <is>
-          <t>LUTY TRANSPORTE</t>
+          <t>HCOUTINHO</t>
         </is>
       </c>
     </row>
     <row r="3351">
       <c r="A3351" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3351" t="n">
-        <v>3391</v>
+        <v>940553</v>
       </c>
       <c r="C3351" t="inlineStr">
         <is>
-          <t xml:space="preserve">NIKSON DA SILVA ALVES </t>
+          <t>LUTY TRANSPORTES- BA</t>
         </is>
       </c>
       <c r="D3351" t="inlineStr">
         <is>
-          <t>NIKSON</t>
+          <t>LUTY TRANSPORTE</t>
         </is>
       </c>
     </row>
     <row r="3352">
       <c r="A3352" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3352" t="n">
-        <v>3397</v>
+        <v>3391</v>
       </c>
       <c r="C3352" t="inlineStr">
         <is>
-          <t>EDILANE MENESES BALTAZAR</t>
+          <t xml:space="preserve">NIKSON DA SILVA ALVES </t>
         </is>
       </c>
       <c r="D3352" t="inlineStr">
         <is>
-          <t>EDILANE</t>
+          <t>NIKSON</t>
         </is>
       </c>
     </row>
@@ -67478,56 +67478,56 @@
         </is>
       </c>
       <c r="B3353" t="n">
-        <v>3398</v>
+        <v>3397</v>
       </c>
       <c r="C3353" t="inlineStr">
         <is>
-          <t>LUANA MARIA ROSIO DA SILVA</t>
+          <t>EDILANE MENESES BALTAZAR</t>
         </is>
       </c>
       <c r="D3353" t="inlineStr">
         <is>
-          <t>LUMARIA</t>
+          <t>EDILANE</t>
         </is>
       </c>
     </row>
     <row r="3354">
       <c r="A3354" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3354" t="n">
-        <v>3400</v>
+        <v>3398</v>
       </c>
       <c r="C3354" t="inlineStr">
         <is>
-          <t>ELILTON PINTO ROMEU</t>
+          <t>LUANA MARIA ROSIO DA SILVA</t>
         </is>
       </c>
       <c r="D3354" t="inlineStr">
         <is>
-          <t>ELILTON</t>
+          <t>LUMARIA</t>
         </is>
       </c>
     </row>
     <row r="3355">
       <c r="A3355" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3355" t="n">
-        <v>3406</v>
+        <v>3400</v>
       </c>
       <c r="C3355" t="inlineStr">
         <is>
-          <t>CONEXAO ALDA</t>
+          <t>ELILTON PINTO ROMEU</t>
         </is>
       </c>
       <c r="D3355" t="inlineStr">
         <is>
-          <t>CONEXAOALDA</t>
+          <t>ELILTON</t>
         </is>
       </c>
     </row>
@@ -67538,176 +67538,176 @@
         </is>
       </c>
       <c r="B3356" t="n">
-        <v>3407</v>
+        <v>3406</v>
       </c>
       <c r="C3356" t="inlineStr">
         <is>
-          <t>CONEXAO IRACEMA</t>
+          <t>CONEXAO ALDA</t>
         </is>
       </c>
       <c r="D3356" t="inlineStr">
         <is>
-          <t>CONEXAOIRACEMA</t>
+          <t>CONEXAOALDA</t>
         </is>
       </c>
     </row>
     <row r="3357">
       <c r="A3357" t="inlineStr">
         <is>
-          <t>9999</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3357" t="n">
-        <v>3408</v>
+        <v>3407</v>
       </c>
       <c r="C3357" t="inlineStr">
         <is>
-          <t>CONEXAO TAMILES</t>
+          <t>CONEXAO IRACEMA</t>
         </is>
       </c>
       <c r="D3357" t="inlineStr">
         <is>
-          <t>CONEXAOTAMILES</t>
+          <t>CONEXAOIRACEMA</t>
         </is>
       </c>
     </row>
     <row r="3358">
       <c r="A3358" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>9999</t>
         </is>
       </c>
       <c r="B3358" t="n">
-        <v>3414</v>
+        <v>3408</v>
       </c>
       <c r="C3358" t="inlineStr">
         <is>
-          <t>CONEXAO ADM PI MA</t>
+          <t>CONEXAO TAMILES</t>
         </is>
       </c>
       <c r="D3358" t="inlineStr">
         <is>
-          <t>CONEXAOPIMA</t>
+          <t>CONEXAOTAMILES</t>
         </is>
       </c>
     </row>
     <row r="3359">
       <c r="A3359" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3359" t="n">
-        <v>3524</v>
+        <v>3414</v>
       </c>
       <c r="C3359" t="inlineStr">
         <is>
-          <t>LUIS FELIPE DA SILVA SOUSA</t>
+          <t>CONEXAO ADM PI MA</t>
         </is>
       </c>
       <c r="D3359" t="inlineStr">
         <is>
-          <t>L.FELIPE</t>
+          <t>CONEXAOPIMA</t>
         </is>
       </c>
     </row>
     <row r="3360">
       <c r="A3360" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3360" t="n">
-        <v>3531</v>
+        <v>3524</v>
       </c>
       <c r="C3360" t="inlineStr">
         <is>
-          <t>LEICIANE COELHO SILVA</t>
+          <t>LUIS FELIPE DA SILVA SOUSA</t>
         </is>
       </c>
       <c r="D3360" t="inlineStr">
         <is>
-          <t>LEI.SILVA</t>
+          <t>L.FELIPE</t>
         </is>
       </c>
     </row>
     <row r="3361">
       <c r="A3361" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3361" t="n">
-        <v>3550</v>
+        <v>3531</v>
       </c>
       <c r="C3361" t="inlineStr">
         <is>
-          <t>IARGO GABRIEL SANTOS DE OLIVEIRA</t>
+          <t>LEICIANE COELHO SILVA</t>
         </is>
       </c>
       <c r="D3361" t="inlineStr">
         <is>
-          <t>IARGOG</t>
+          <t>LEI.SILVA</t>
         </is>
       </c>
     </row>
     <row r="3362">
       <c r="A3362" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3362" t="n">
-        <v>940567</v>
+        <v>3550</v>
       </c>
       <c r="C3362" t="inlineStr">
         <is>
-          <t>MS CARGAS E TRANSPORTES</t>
+          <t>IARGO GABRIEL SANTOS DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D3362" t="inlineStr">
         <is>
-          <t>ALAN BARBOSA</t>
+          <t>IARGOG</t>
         </is>
       </c>
     </row>
     <row r="3363">
       <c r="A3363" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3363" t="n">
-        <v>3560</v>
+        <v>940567</v>
       </c>
       <c r="C3363" t="inlineStr">
         <is>
-          <t>MARIA EDUARDA MELO DOS SANTOS</t>
+          <t>MS CARGAS E TRANSPORTES</t>
         </is>
       </c>
       <c r="D3363" t="inlineStr">
         <is>
-          <t>EDU.MELO</t>
+          <t>ALAN BARBOSA</t>
         </is>
       </c>
     </row>
     <row r="3364">
       <c r="A3364" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3364" t="n">
-        <v>3355</v>
+        <v>3560</v>
       </c>
       <c r="C3364" t="inlineStr">
         <is>
-          <t>HUGO MATHEUS DA COSTA FEITOSA</t>
+          <t>MARIA EDUARDA MELO DOS SANTOS</t>
         </is>
       </c>
       <c r="D3364" t="inlineStr">
         <is>
-          <t>HMFEITOSA</t>
+          <t>EDU.MELO</t>
         </is>
       </c>
     </row>
@@ -67718,96 +67718,96 @@
         </is>
       </c>
       <c r="B3365" t="n">
-        <v>3356</v>
+        <v>3355</v>
       </c>
       <c r="C3365" t="inlineStr">
         <is>
-          <t>BRENDA LIMA DE OLIVEIRA CUNHA</t>
+          <t>HUGO MATHEUS DA COSTA FEITOSA</t>
         </is>
       </c>
       <c r="D3365" t="inlineStr">
         <is>
-          <t>BLCUNHA</t>
+          <t>HMFEITOSA</t>
         </is>
       </c>
     </row>
     <row r="3366">
       <c r="A3366" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3366" t="n">
-        <v>3361</v>
+        <v>3356</v>
       </c>
       <c r="C3366" t="inlineStr">
         <is>
-          <t>WLADIA DE ARAUJO BASTOS</t>
+          <t>BRENDA LIMA DE OLIVEIRA CUNHA</t>
         </is>
       </c>
       <c r="D3366" t="inlineStr">
         <is>
-          <t>WABASTOS</t>
+          <t>BLCUNHA</t>
         </is>
       </c>
     </row>
     <row r="3367">
       <c r="A3367" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3367" t="n">
-        <v>3362</v>
+        <v>3361</v>
       </c>
       <c r="C3367" t="inlineStr">
         <is>
-          <t>CARLOS HENRIQUE MELO DA SILVA</t>
+          <t>WLADIA DE ARAUJO BASTOS</t>
         </is>
       </c>
       <c r="D3367" t="inlineStr">
         <is>
-          <t>CHMELO</t>
+          <t>WABASTOS</t>
         </is>
       </c>
     </row>
     <row r="3368">
       <c r="A3368" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3368" t="n">
-        <v>3375</v>
+        <v>3362</v>
       </c>
       <c r="C3368" t="inlineStr">
         <is>
-          <t>AFONSO DE SOUSA RAMOS FILHO</t>
+          <t>CARLOS HENRIQUE MELO DA SILVA</t>
         </is>
       </c>
       <c r="D3368" t="inlineStr">
         <is>
-          <t>AFILHO</t>
+          <t>CHMELO</t>
         </is>
       </c>
     </row>
     <row r="3369">
       <c r="A3369" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3369" t="n">
-        <v>3404</v>
+        <v>3375</v>
       </c>
       <c r="C3369" t="inlineStr">
         <is>
-          <t>NOVATO 4 COM</t>
+          <t>AFONSO DE SOUSA RAMOS FILHO</t>
         </is>
       </c>
       <c r="D3369" t="inlineStr">
         <is>
-          <t>NOVATO4COM</t>
+          <t>AFILHO</t>
         </is>
       </c>
     </row>
@@ -67818,156 +67818,156 @@
         </is>
       </c>
       <c r="B3370" t="n">
-        <v>3405</v>
+        <v>3404</v>
       </c>
       <c r="C3370" t="inlineStr">
         <is>
-          <t>NOVATO 5 COM</t>
+          <t>NOVATO 4 COM</t>
         </is>
       </c>
       <c r="D3370" t="inlineStr">
         <is>
-          <t>NOVATO5COM</t>
+          <t>NOVATO4COM</t>
         </is>
       </c>
     </row>
     <row r="3371">
       <c r="A3371" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3371" t="n">
-        <v>3447</v>
+        <v>3405</v>
       </c>
       <c r="C3371" t="inlineStr">
         <is>
-          <t>RAYSSA KEYCE LINHARES AQUINO</t>
+          <t>NOVATO 5 COM</t>
         </is>
       </c>
       <c r="D3371" t="inlineStr">
         <is>
-          <t>RAYSSAK</t>
+          <t>NOVATO5COM</t>
         </is>
       </c>
     </row>
     <row r="3372">
       <c r="A3372" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3372" t="n">
-        <v>940559</v>
+        <v>3447</v>
       </c>
       <c r="C3372" t="inlineStr">
         <is>
-          <t>WALLEF DE OLIVEIRA</t>
+          <t>RAYSSA KEYCE LINHARES AQUINO</t>
         </is>
       </c>
       <c r="D3372" t="inlineStr">
         <is>
-          <t>WALLEF</t>
+          <t>RAYSSAK</t>
         </is>
       </c>
     </row>
     <row r="3373">
       <c r="A3373" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>99</t>
         </is>
       </c>
       <c r="B3373" t="n">
-        <v>3489</v>
+        <v>940559</v>
       </c>
       <c r="C3373" t="inlineStr">
         <is>
-          <t>MARCELA KARINA PEREIRA VELOSO</t>
+          <t>WALLEF DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D3373" t="inlineStr">
         <is>
-          <t>MKARINA</t>
+          <t>WALLEF</t>
         </is>
       </c>
     </row>
     <row r="3374">
       <c r="A3374" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3374" t="n">
-        <v>3490</v>
+        <v>3489</v>
       </c>
       <c r="C3374" t="inlineStr">
         <is>
-          <t>JOSE MAILSON GOMES NUNES</t>
+          <t>MARCELA KARINA PEREIRA VELOSO</t>
         </is>
       </c>
       <c r="D3374" t="inlineStr">
         <is>
-          <t>J.MAILSON</t>
+          <t>MKARINA</t>
         </is>
       </c>
     </row>
     <row r="3375">
       <c r="A3375" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3375" t="n">
-        <v>3537</v>
+        <v>3490</v>
       </c>
       <c r="C3375" t="inlineStr">
         <is>
-          <t>ALDAIR PEDRO DA SILVA</t>
+          <t>JOSE MAILSON GOMES NUNES</t>
         </is>
       </c>
       <c r="D3375" t="inlineStr">
         <is>
-          <t>A.PEDRO</t>
+          <t>J.MAILSON</t>
         </is>
       </c>
     </row>
     <row r="3376">
       <c r="A3376" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3376" t="n">
-        <v>3549</v>
+        <v>3537</v>
       </c>
       <c r="C3376" t="inlineStr">
         <is>
-          <t xml:space="preserve">FERNANDA CAROLINE E CESAR SOUSA </t>
+          <t>ALDAIR PEDRO DA SILVA</t>
         </is>
       </c>
       <c r="D3376" t="inlineStr">
         <is>
-          <t>FCAROLINE</t>
+          <t>A.PEDRO</t>
         </is>
       </c>
     </row>
     <row r="3377">
       <c r="A3377" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3377" t="n">
-        <v>3337</v>
+        <v>3549</v>
       </c>
       <c r="C3377" t="inlineStr">
         <is>
-          <t>WESLEY FONTES DE ALMEIDA</t>
+          <t xml:space="preserve">FERNANDA CAROLINE E CESAR SOUSA </t>
         </is>
       </c>
       <c r="D3377" t="inlineStr">
         <is>
-          <t>WFALMEIDA</t>
+          <t>FCAROLINE</t>
         </is>
       </c>
     </row>
@@ -67978,16 +67978,16 @@
         </is>
       </c>
       <c r="B3378" t="n">
-        <v>3338</v>
+        <v>3337</v>
       </c>
       <c r="C3378" t="inlineStr">
         <is>
-          <t>FRANCISCA SAMARA MENDES DE OLIVEIRA C</t>
+          <t>WESLEY FONTES DE ALMEIDA</t>
         </is>
       </c>
       <c r="D3378" t="inlineStr">
         <is>
-          <t>FSCUNHA</t>
+          <t>WFALMEIDA</t>
         </is>
       </c>
     </row>
@@ -67998,176 +67998,176 @@
         </is>
       </c>
       <c r="B3379" t="n">
-        <v>3339</v>
+        <v>3338</v>
       </c>
       <c r="C3379" t="inlineStr">
         <is>
-          <t>MAYARA THALYA DIAS DE ANDRADE</t>
+          <t>FRANCISCA SAMARA MENDES DE OLIVEIRA C</t>
         </is>
       </c>
       <c r="D3379" t="inlineStr">
         <is>
-          <t>MTANDRADE</t>
+          <t>FSCUNHA</t>
         </is>
       </c>
     </row>
     <row r="3380">
       <c r="A3380" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3380" t="n">
-        <v>3359</v>
+        <v>3339</v>
       </c>
       <c r="C3380" t="inlineStr">
         <is>
-          <t xml:space="preserve">EVANESSA DA SILVA E SILVA </t>
+          <t>MAYARA THALYA DIAS DE ANDRADE</t>
         </is>
       </c>
       <c r="D3380" t="inlineStr">
         <is>
-          <t>EVANESSAS</t>
+          <t>MTANDRADE</t>
         </is>
       </c>
     </row>
     <row r="3381">
       <c r="A3381" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3381" t="n">
-        <v>3360</v>
+        <v>3359</v>
       </c>
       <c r="C3381" t="inlineStr">
         <is>
-          <t>THIAGO DE CARVALHO ARAUJO</t>
+          <t xml:space="preserve">EVANESSA DA SILVA E SILVA </t>
         </is>
       </c>
       <c r="D3381" t="inlineStr">
         <is>
-          <t>TCARAUJO</t>
+          <t>EVANESSAS</t>
         </is>
       </c>
     </row>
     <row r="3382">
       <c r="A3382" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3382" t="n">
-        <v>3481</v>
+        <v>3360</v>
       </c>
       <c r="C3382" t="inlineStr">
         <is>
-          <t xml:space="preserve">EDSON DA PAZ LIMA </t>
+          <t>THIAGO DE CARVALHO ARAUJO</t>
         </is>
       </c>
       <c r="D3382" t="inlineStr">
         <is>
-          <t>EDPAZ</t>
+          <t>TCARAUJO</t>
         </is>
       </c>
     </row>
     <row r="3383">
       <c r="A3383" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3383" t="n">
-        <v>3494</v>
+        <v>3481</v>
       </c>
       <c r="C3383" t="inlineStr">
         <is>
-          <t>ANTONIO CRISTINA BRITO GOMES</t>
+          <t xml:space="preserve">EDSON DA PAZ LIMA </t>
         </is>
       </c>
       <c r="D3383" t="inlineStr">
         <is>
-          <t>CRIS.GOMES</t>
+          <t>EDPAZ</t>
         </is>
       </c>
     </row>
     <row r="3384">
       <c r="A3384" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3384" t="n">
-        <v>3498</v>
+        <v>3494</v>
       </c>
       <c r="C3384" t="inlineStr">
         <is>
-          <t>SILVESTRA COSTA NUNES</t>
+          <t>ANTONIO CRISTINA BRITO GOMES</t>
         </is>
       </c>
       <c r="D3384" t="inlineStr">
         <is>
-          <t>SCNUNES</t>
+          <t>CRIS.GOMES</t>
         </is>
       </c>
     </row>
     <row r="3385">
       <c r="A3385" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3385" t="n">
-        <v>940562</v>
+        <v>3498</v>
       </c>
       <c r="C3385" t="inlineStr">
         <is>
-          <t>FRANCISCO DAVID ASSUNCAO ALVES</t>
+          <t>SILVESTRA COSTA NUNES</t>
         </is>
       </c>
       <c r="D3385" t="inlineStr">
         <is>
-          <t>ASSUNÇÃO</t>
+          <t>SCNUNES</t>
         </is>
       </c>
     </row>
     <row r="3386">
       <c r="A3386" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>99</t>
         </is>
       </c>
       <c r="B3386" t="n">
-        <v>3513</v>
+        <v>940562</v>
       </c>
       <c r="C3386" t="inlineStr">
         <is>
-          <t>RENARA ANDRADE MATIAS</t>
+          <t>FRANCISCO DAVID ASSUNCAO ALVES</t>
         </is>
       </c>
       <c r="D3386" t="inlineStr">
         <is>
-          <t>R.ANDRADE</t>
+          <t>ASSUNÇÃO</t>
         </is>
       </c>
     </row>
     <row r="3387">
       <c r="A3387" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3387" t="n">
-        <v>3275</v>
+        <v>3513</v>
       </c>
       <c r="C3387" t="inlineStr">
         <is>
-          <t>MARIA APARECIDA COELHO SILVA</t>
+          <t>RENARA ANDRADE MATIAS</t>
         </is>
       </c>
       <c r="D3387" t="inlineStr">
         <is>
-          <t>MCOELHO</t>
+          <t>R.ANDRADE</t>
         </is>
       </c>
     </row>
@@ -68178,116 +68178,116 @@
         </is>
       </c>
       <c r="B3388" t="n">
-        <v>3276</v>
+        <v>3275</v>
       </c>
       <c r="C3388" t="inlineStr">
         <is>
-          <t xml:space="preserve">PEROLA DE JESUS AMORIM SOUSA </t>
+          <t>MARIA APARECIDA COELHO SILVA</t>
         </is>
       </c>
       <c r="D3388" t="inlineStr">
         <is>
-          <t>PJESUS</t>
+          <t>MCOELHO</t>
         </is>
       </c>
     </row>
     <row r="3389">
       <c r="A3389" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3389" t="n">
-        <v>3526</v>
+        <v>3276</v>
       </c>
       <c r="C3389" t="inlineStr">
         <is>
-          <t>JOYCE NAZARE CORREA</t>
+          <t xml:space="preserve">PEROLA DE JESUS AMORIM SOUSA </t>
         </is>
       </c>
       <c r="D3389" t="inlineStr">
         <is>
-          <t>J.NAZARE</t>
+          <t>PJESUS</t>
         </is>
       </c>
     </row>
     <row r="3390">
       <c r="A3390" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3390" t="n">
-        <v>3527</v>
+        <v>3526</v>
       </c>
       <c r="C3390" t="inlineStr">
         <is>
-          <t>GILVANA DA SILVA MONTELES</t>
+          <t>JOYCE NAZARE CORREA</t>
         </is>
       </c>
       <c r="D3390" t="inlineStr">
         <is>
-          <t>GIL.SILVA</t>
+          <t>J.NAZARE</t>
         </is>
       </c>
     </row>
     <row r="3391">
       <c r="A3391" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3391" t="n">
-        <v>3548</v>
+        <v>3527</v>
       </c>
       <c r="C3391" t="inlineStr">
         <is>
-          <t>JAMILLY MARIA HENRIQUE ARAUJO</t>
+          <t>GILVANA DA SILVA MONTELES</t>
         </is>
       </c>
       <c r="D3391" t="inlineStr">
         <is>
-          <t>JAMILLY</t>
+          <t>GIL.SILVA</t>
         </is>
       </c>
     </row>
     <row r="3392">
       <c r="A3392" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3392" t="n">
-        <v>3551</v>
+        <v>3548</v>
       </c>
       <c r="C3392" t="inlineStr">
         <is>
-          <t xml:space="preserve">VITOR MANOEL DA SILVA BARBOSA </t>
+          <t>JAMILLY MARIA HENRIQUE ARAUJO</t>
         </is>
       </c>
       <c r="D3392" t="inlineStr">
         <is>
-          <t>VMANOEL</t>
+          <t>JAMILLY</t>
         </is>
       </c>
     </row>
     <row r="3393">
       <c r="A3393" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3393" t="n">
-        <v>940525</v>
+        <v>3551</v>
       </c>
       <c r="C3393" t="inlineStr">
         <is>
-          <t>SANDUWELLINGTON</t>
+          <t xml:space="preserve">VITOR MANOEL DA SILVA BARBOSA </t>
         </is>
       </c>
       <c r="D3393" t="inlineStr">
         <is>
-          <t>SANDUWELLINGTON</t>
+          <t>VMANOEL</t>
         </is>
       </c>
     </row>
@@ -68298,36 +68298,36 @@
         </is>
       </c>
       <c r="B3394" t="n">
-        <v>3369</v>
+        <v>940525</v>
       </c>
       <c r="C3394" t="inlineStr">
         <is>
-          <t xml:space="preserve">PRISCILA DOS SANTOS LOPES </t>
+          <t>SANDUWELLINGTON</t>
         </is>
       </c>
       <c r="D3394" t="inlineStr">
         <is>
-          <t>PSLOPES</t>
+          <t>SANDUWELLINGTON</t>
         </is>
       </c>
     </row>
     <row r="3395">
       <c r="A3395" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3395" t="n">
-        <v>3433</v>
+        <v>3369</v>
       </c>
       <c r="C3395" t="inlineStr">
         <is>
-          <t>BRUNO NUNES CRUZ</t>
+          <t xml:space="preserve">PRISCILA DOS SANTOS LOPES </t>
         </is>
       </c>
       <c r="D3395" t="inlineStr">
         <is>
-          <t>BRUNOCRUZ</t>
+          <t>PSLOPES</t>
         </is>
       </c>
     </row>
@@ -68338,36 +68338,36 @@
         </is>
       </c>
       <c r="B3396" t="n">
-        <v>3434</v>
+        <v>3433</v>
       </c>
       <c r="C3396" t="inlineStr">
         <is>
-          <t>ANA TERCIA DE LIMA SA CARVALHO SERAFIM</t>
+          <t>BRUNO NUNES CRUZ</t>
         </is>
       </c>
       <c r="D3396" t="inlineStr">
         <is>
-          <t>ANATER</t>
+          <t>BRUNOCRUZ</t>
         </is>
       </c>
     </row>
     <row r="3397">
       <c r="A3397" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3397" t="n">
-        <v>3502</v>
+        <v>3434</v>
       </c>
       <c r="C3397" t="inlineStr">
         <is>
-          <t>LUIZ FELIPE MACHADO BARRETO</t>
+          <t>ANA TERCIA DE LIMA SA CARVALHO SERAFIM</t>
         </is>
       </c>
       <c r="D3397" t="inlineStr">
         <is>
-          <t>LUIZ.FELIPE</t>
+          <t>ANATER</t>
         </is>
       </c>
     </row>
@@ -68378,36 +68378,36 @@
         </is>
       </c>
       <c r="B3398" t="n">
-        <v>3503</v>
+        <v>3502</v>
       </c>
       <c r="C3398" t="inlineStr">
         <is>
-          <t>FABIO OLIVEIRA SILVA</t>
+          <t>LUIZ FELIPE MACHADO BARRETO</t>
         </is>
       </c>
       <c r="D3398" t="inlineStr">
         <is>
-          <t>FOSILVA</t>
+          <t>LUIZ.FELIPE</t>
         </is>
       </c>
     </row>
     <row r="3399">
       <c r="A3399" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3399" t="n">
-        <v>3554</v>
+        <v>3503</v>
       </c>
       <c r="C3399" t="inlineStr">
         <is>
-          <t xml:space="preserve">MANOEL RIBEIRO DE SOUZA JUNIOR </t>
+          <t>FABIO OLIVEIRA SILVA</t>
         </is>
       </c>
       <c r="D3399" t="inlineStr">
         <is>
-          <t>MRJUNIOR</t>
+          <t>FOSILVA</t>
         </is>
       </c>
     </row>
@@ -68418,16 +68418,16 @@
         </is>
       </c>
       <c r="B3400" t="n">
-        <v>3568</v>
+        <v>3554</v>
       </c>
       <c r="C3400" t="inlineStr">
         <is>
-          <t xml:space="preserve">ANGELICA TORRES DA SILVA </t>
+          <t xml:space="preserve">MANOEL RIBEIRO DE SOUZA JUNIOR </t>
         </is>
       </c>
       <c r="D3400" t="inlineStr">
         <is>
-          <t>ANGEL.TORRES</t>
+          <t>MRJUNIOR</t>
         </is>
       </c>
     </row>
@@ -68438,56 +68438,56 @@
         </is>
       </c>
       <c r="B3401" t="n">
-        <v>3569</v>
+        <v>3568</v>
       </c>
       <c r="C3401" t="inlineStr">
         <is>
-          <t>LORENA DE LIMA MATOS</t>
+          <t xml:space="preserve">ANGELICA TORRES DA SILVA </t>
         </is>
       </c>
       <c r="D3401" t="inlineStr">
         <is>
-          <t>LORE.LIMA</t>
+          <t>ANGEL.TORRES</t>
         </is>
       </c>
     </row>
     <row r="3402">
       <c r="A3402" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3402" t="n">
-        <v>3576</v>
+        <v>3569</v>
       </c>
       <c r="C3402" t="inlineStr">
         <is>
-          <t>ANA BEATRIZ PARENTE CAVALCANTE</t>
+          <t>LORENA DE LIMA MATOS</t>
         </is>
       </c>
       <c r="D3402" t="inlineStr">
         <is>
-          <t>A.BEATRIZ</t>
+          <t>LORE.LIMA</t>
         </is>
       </c>
     </row>
     <row r="3403">
       <c r="A3403" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3403" t="n">
-        <v>940549</v>
+        <v>3576</v>
       </c>
       <c r="C3403" t="inlineStr">
         <is>
-          <t>EDILSON ARAUJO - FL9</t>
+          <t>ANA BEATRIZ PARENTE CAVALCANTE</t>
         </is>
       </c>
       <c r="D3403" t="inlineStr">
         <is>
-          <t>EDILSON</t>
+          <t>A.BEATRIZ</t>
         </is>
       </c>
     </row>
@@ -68498,36 +68498,36 @@
         </is>
       </c>
       <c r="B3404" t="n">
-        <v>3470</v>
+        <v>940549</v>
       </c>
       <c r="C3404" t="inlineStr">
         <is>
-          <t>DEBORA ALVES CARVALHO</t>
+          <t>EDILSON ARAUJO - FL9</t>
         </is>
       </c>
       <c r="D3404" t="inlineStr">
         <is>
-          <t>DEBORA.ALVES</t>
+          <t>EDILSON</t>
         </is>
       </c>
     </row>
     <row r="3405">
       <c r="A3405" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3405" t="n">
-        <v>3510</v>
+        <v>3470</v>
       </c>
       <c r="C3405" t="inlineStr">
         <is>
-          <t>CAMILA RODIGUES PINTO</t>
+          <t>DEBORA ALVES CARVALHO</t>
         </is>
       </c>
       <c r="D3405" t="inlineStr">
         <is>
-          <t>MILA.PINTO</t>
+          <t>DEBORA.ALVES</t>
         </is>
       </c>
     </row>
@@ -68538,96 +68538,96 @@
         </is>
       </c>
       <c r="B3406" t="n">
-        <v>3511</v>
+        <v>3510</v>
       </c>
       <c r="C3406" t="inlineStr">
         <is>
-          <t>JORGE HENRIQUE DOS SANTOS RODRIGUES</t>
+          <t>CAMILA RODIGUES PINTO</t>
         </is>
       </c>
       <c r="D3406" t="inlineStr">
         <is>
-          <t>J.HENRIQUE</t>
+          <t>MILA.PINTO</t>
         </is>
       </c>
     </row>
     <row r="3407">
       <c r="A3407" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3407" t="n">
-        <v>3561</v>
+        <v>3511</v>
       </c>
       <c r="C3407" t="inlineStr">
         <is>
-          <t>RONARIA PATRICIA VILARINDO DE ALMEIDA</t>
+          <t>JORGE HENRIQUE DOS SANTOS RODRIGUES</t>
         </is>
       </c>
       <c r="D3407" t="inlineStr">
         <is>
-          <t>RPATRICIA</t>
+          <t>J.HENRIQUE</t>
         </is>
       </c>
     </row>
     <row r="3408">
       <c r="A3408" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3408" t="n">
-        <v>3562</v>
+        <v>3561</v>
       </c>
       <c r="C3408" t="inlineStr">
         <is>
-          <t>LETICIA MARIA BENTO NOGUEIRA</t>
+          <t>RONARIA PATRICIA VILARINDO DE ALMEIDA</t>
         </is>
       </c>
       <c r="D3408" t="inlineStr">
         <is>
-          <t>LBENTO</t>
+          <t>RPATRICIA</t>
         </is>
       </c>
     </row>
     <row r="3409">
       <c r="A3409" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3409" t="n">
-        <v>3270</v>
+        <v>3562</v>
       </c>
       <c r="C3409" t="inlineStr">
         <is>
-          <t>ITANA NASCIMENTO SIMOES</t>
+          <t>LETICIA MARIA BENTO NOGUEIRA</t>
         </is>
       </c>
       <c r="D3409" t="inlineStr">
         <is>
-          <t>ISIMOES</t>
+          <t>LBENTO</t>
         </is>
       </c>
     </row>
     <row r="3410">
       <c r="A3410" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3410" t="n">
-        <v>3318</v>
+        <v>3270</v>
       </c>
       <c r="C3410" t="inlineStr">
         <is>
-          <t>LUAN MONTEIRO COSTA</t>
+          <t>ITANA NASCIMENTO SIMOES</t>
         </is>
       </c>
       <c r="D3410" t="inlineStr">
         <is>
-          <t>LMONTEIRO</t>
+          <t>ISIMOES</t>
         </is>
       </c>
     </row>
@@ -68638,36 +68638,36 @@
         </is>
       </c>
       <c r="B3411" t="n">
-        <v>3319</v>
+        <v>3318</v>
       </c>
       <c r="C3411" t="inlineStr">
         <is>
-          <t>MARIANA MACEDA DOS SANTOS</t>
+          <t>LUAN MONTEIRO COSTA</t>
         </is>
       </c>
       <c r="D3411" t="inlineStr">
         <is>
-          <t>MMACEDA</t>
+          <t>LMONTEIRO</t>
         </is>
       </c>
     </row>
     <row r="3412">
       <c r="A3412" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3412" t="n">
-        <v>3389</v>
+        <v>3319</v>
       </c>
       <c r="C3412" t="inlineStr">
         <is>
-          <t>TAMILES DE SANTANA AMORIM BISPO</t>
+          <t>MARIANA MACEDA DOS SANTOS</t>
         </is>
       </c>
       <c r="D3412" t="inlineStr">
         <is>
-          <t>TAMILES</t>
+          <t>MMACEDA</t>
         </is>
       </c>
     </row>
@@ -68678,36 +68678,36 @@
         </is>
       </c>
       <c r="B3413" t="n">
-        <v>3390</v>
+        <v>3389</v>
       </c>
       <c r="C3413" t="inlineStr">
         <is>
-          <t>IRACEMA DE ALMEIDA MOURA</t>
+          <t>TAMILES DE SANTANA AMORIM BISPO</t>
         </is>
       </c>
       <c r="D3413" t="inlineStr">
         <is>
-          <t>IRACEMA</t>
+          <t>TAMILES</t>
         </is>
       </c>
     </row>
     <row r="3414">
       <c r="A3414" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3414" t="n">
-        <v>3575</v>
+        <v>3390</v>
       </c>
       <c r="C3414" t="inlineStr">
         <is>
-          <t>SAMARA ALVES DA SILVA</t>
+          <t>IRACEMA DE ALMEIDA MOURA</t>
         </is>
       </c>
       <c r="D3414" t="inlineStr">
         <is>
-          <t>S.ALVES</t>
+          <t>IRACEMA</t>
         </is>
       </c>
     </row>
@@ -68718,16 +68718,16 @@
         </is>
       </c>
       <c r="B3415" t="n">
-        <v>3286</v>
+        <v>3575</v>
       </c>
       <c r="C3415" t="inlineStr">
         <is>
-          <t>VALERIA MAIA DA SILVA</t>
+          <t>SAMARA ALVES DA SILVA</t>
         </is>
       </c>
       <c r="D3415" t="inlineStr">
         <is>
-          <t>VMAIAS</t>
+          <t>S.ALVES</t>
         </is>
       </c>
     </row>
@@ -68738,156 +68738,156 @@
         </is>
       </c>
       <c r="B3416" t="n">
-        <v>3287</v>
+        <v>3286</v>
       </c>
       <c r="C3416" t="inlineStr">
         <is>
-          <t>ERIVELTON DA SILVA OLIVEIRA</t>
+          <t>VALERIA MAIA DA SILVA</t>
         </is>
       </c>
       <c r="D3416" t="inlineStr">
         <is>
-          <t>ESOLIVEIRA</t>
+          <t>VMAIAS</t>
         </is>
       </c>
     </row>
     <row r="3417">
       <c r="A3417" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3417" t="n">
-        <v>3307</v>
+        <v>3287</v>
       </c>
       <c r="C3417" t="inlineStr">
         <is>
-          <t>ADRIEL XERES BARROS MARTINS</t>
+          <t>ERIVELTON DA SILVA OLIVEIRA</t>
         </is>
       </c>
       <c r="D3417" t="inlineStr">
         <is>
-          <t>AXERES</t>
+          <t>ESOLIVEIRA</t>
         </is>
       </c>
     </row>
     <row r="3418">
       <c r="A3418" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3418" t="n">
-        <v>3308</v>
+        <v>3307</v>
       </c>
       <c r="C3418" t="inlineStr">
         <is>
-          <t>ELKZIEL JUVINO DA SILVA</t>
+          <t>ADRIEL XERES BARROS MARTINS</t>
         </is>
       </c>
       <c r="D3418" t="inlineStr">
         <is>
-          <t>EJUVINO</t>
+          <t>AXERES</t>
         </is>
       </c>
     </row>
     <row r="3419">
       <c r="A3419" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3419" t="n">
-        <v>940539</v>
+        <v>3308</v>
       </c>
       <c r="C3419" t="inlineStr">
         <is>
-          <t>EDSON ARAUJO - FL9</t>
+          <t>ELKZIEL JUVINO DA SILVA</t>
         </is>
       </c>
       <c r="D3419" t="inlineStr">
         <is>
-          <t>EDS</t>
+          <t>EJUVINO</t>
         </is>
       </c>
     </row>
     <row r="3420">
       <c r="A3420" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3420" t="n">
-        <v>940540</v>
+        <v>940539</v>
       </c>
       <c r="C3420" t="inlineStr">
         <is>
-          <t>EDSON ARAUJO - FL8</t>
+          <t>EDSON ARAUJO - FL9</t>
         </is>
       </c>
       <c r="D3420" t="inlineStr">
         <is>
-          <t>EDS8</t>
+          <t>EDS</t>
         </is>
       </c>
     </row>
     <row r="3421">
       <c r="A3421" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B3421" t="n">
-        <v>3328</v>
+        <v>940540</v>
       </c>
       <c r="C3421" t="inlineStr">
         <is>
-          <t>ALAN ARAUJO DA SILVA</t>
+          <t>EDSON ARAUJO - FL8</t>
         </is>
       </c>
       <c r="D3421" t="inlineStr">
         <is>
-          <t>ARSILVA</t>
+          <t>EDS8</t>
         </is>
       </c>
     </row>
     <row r="3422">
       <c r="A3422" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3422" t="n">
-        <v>3350</v>
+        <v>3328</v>
       </c>
       <c r="C3422" t="inlineStr">
         <is>
-          <t xml:space="preserve">EDER RODRIGUES DA SILVA </t>
+          <t>ALAN ARAUJO DA SILVA</t>
         </is>
       </c>
       <c r="D3422" t="inlineStr">
         <is>
-          <t>EDERS</t>
+          <t>ARSILVA</t>
         </is>
       </c>
     </row>
     <row r="3423">
       <c r="A3423" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3423" t="n">
-        <v>3373</v>
+        <v>3350</v>
       </c>
       <c r="C3423" t="inlineStr">
         <is>
-          <t xml:space="preserve">NATANAEL TAVARES DE SOUSA </t>
+          <t xml:space="preserve">EDER RODRIGUES DA SILVA </t>
         </is>
       </c>
       <c r="D3423" t="inlineStr">
         <is>
-          <t>NTSOUSA</t>
+          <t>EDERS</t>
         </is>
       </c>
     </row>
@@ -68898,156 +68898,156 @@
         </is>
       </c>
       <c r="B3424" t="n">
-        <v>3374</v>
+        <v>3373</v>
       </c>
       <c r="C3424" t="inlineStr">
         <is>
-          <t>REINALDO DA SILVA COSTA</t>
+          <t xml:space="preserve">NATANAEL TAVARES DE SOUSA </t>
         </is>
       </c>
       <c r="D3424" t="inlineStr">
         <is>
-          <t>RSCOSTA</t>
+          <t>NTSOUSA</t>
         </is>
       </c>
     </row>
     <row r="3425">
       <c r="A3425" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3425" t="n">
-        <v>3399</v>
+        <v>3374</v>
       </c>
       <c r="C3425" t="inlineStr">
         <is>
-          <t xml:space="preserve">RICARDO BARBOSA DOS SANTOS </t>
+          <t>REINALDO DA SILVA COSTA</t>
         </is>
       </c>
       <c r="D3425" t="inlineStr">
         <is>
-          <t>RICARDOSAN</t>
+          <t>RSCOSTA</t>
         </is>
       </c>
     </row>
     <row r="3426">
       <c r="A3426" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3426" t="n">
-        <v>3427</v>
+        <v>3399</v>
       </c>
       <c r="C3426" t="inlineStr">
         <is>
-          <t>ROQUE COMERCIO TEMPORARIO</t>
+          <t xml:space="preserve">RICARDO BARBOSA DOS SANTOS </t>
         </is>
       </c>
       <c r="D3426" t="inlineStr">
         <is>
-          <t>ROQUECOM</t>
+          <t>RICARDOSAN</t>
         </is>
       </c>
     </row>
     <row r="3427">
       <c r="A3427" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3427" t="n">
-        <v>3428</v>
+        <v>3427</v>
       </c>
       <c r="C3427" t="inlineStr">
         <is>
-          <t>ROQUE PLUS TEMPORARIO</t>
+          <t>ROQUE COMERCIO TEMPORARIO</t>
         </is>
       </c>
       <c r="D3427" t="inlineStr">
         <is>
-          <t>ROQUEPLUS</t>
+          <t>ROQUECOM</t>
         </is>
       </c>
     </row>
     <row r="3428">
       <c r="A3428" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3428" t="n">
-        <v>3432</v>
+        <v>3428</v>
       </c>
       <c r="C3428" t="inlineStr">
         <is>
-          <t>PATRICIA DOS SANTOS NONATO OLIVEIRA</t>
+          <t>ROQUE PLUS TEMPORARIO</t>
         </is>
       </c>
       <c r="D3428" t="inlineStr">
         <is>
-          <t>PATRICIAD</t>
+          <t>ROQUEPLUS</t>
         </is>
       </c>
     </row>
     <row r="3429">
       <c r="A3429" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3429" t="n">
-        <v>3448</v>
+        <v>3432</v>
       </c>
       <c r="C3429" t="inlineStr">
         <is>
-          <t xml:space="preserve">GABRIEL SOUZA CARVALHO </t>
+          <t>PATRICIA DOS SANTOS NONATO OLIVEIRA</t>
         </is>
       </c>
       <c r="D3429" t="inlineStr">
         <is>
-          <t>GABRIEL20</t>
+          <t>PATRICIAD</t>
         </is>
       </c>
     </row>
     <row r="3430">
       <c r="A3430" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3430" t="n">
-        <v>3465</v>
+        <v>3448</v>
       </c>
       <c r="C3430" t="inlineStr">
         <is>
-          <t>LUIZA MARIA BARRETO BARBOSA</t>
+          <t xml:space="preserve">GABRIEL SOUZA CARVALHO </t>
         </is>
       </c>
       <c r="D3430" t="inlineStr">
         <is>
-          <t>LUIZA.MARIA</t>
+          <t>GABRIEL20</t>
         </is>
       </c>
     </row>
     <row r="3431">
       <c r="A3431" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3431" t="n">
-        <v>3468</v>
+        <v>3465</v>
       </c>
       <c r="C3431" t="inlineStr">
         <is>
-          <t>KAWA ALMEIDA CAMPOS</t>
+          <t>LUIZA MARIA BARRETO BARBOSA</t>
         </is>
       </c>
       <c r="D3431" t="inlineStr">
         <is>
-          <t>KAWA</t>
+          <t>LUIZA.MARIA</t>
         </is>
       </c>
     </row>
@@ -69058,16 +69058,16 @@
         </is>
       </c>
       <c r="B3432" t="n">
-        <v>3476</v>
+        <v>3468</v>
       </c>
       <c r="C3432" t="inlineStr">
         <is>
-          <t xml:space="preserve"> FRANCISCA LEIDIANE M. MENDES NASCIMENTO</t>
+          <t>KAWA ALMEIDA CAMPOS</t>
         </is>
       </c>
       <c r="D3432" t="inlineStr">
         <is>
-          <t>FLEIDIANE</t>
+          <t>KAWA</t>
         </is>
       </c>
     </row>
@@ -69078,76 +69078,76 @@
         </is>
       </c>
       <c r="B3433" t="n">
-        <v>3477</v>
+        <v>3476</v>
       </c>
       <c r="C3433" t="inlineStr">
         <is>
-          <t>MARIA THAIS MARTINS PEREIRA SILVA</t>
+          <t xml:space="preserve"> FRANCISCA LEIDIANE M. MENDES NASCIMENTO</t>
         </is>
       </c>
       <c r="D3433" t="inlineStr">
         <is>
-          <t>MTHAIS</t>
+          <t>FLEIDIANE</t>
         </is>
       </c>
     </row>
     <row r="3434">
       <c r="A3434" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3434" t="n">
-        <v>3271</v>
+        <v>3477</v>
       </c>
       <c r="C3434" t="inlineStr">
         <is>
-          <t>DIEGO DE ARAUJO CALÁBRIA</t>
+          <t>MARIA THAIS MARTINS PEREIRA SILVA</t>
         </is>
       </c>
       <c r="D3434" t="inlineStr">
         <is>
-          <t>ARAUJOC</t>
+          <t>MTHAIS</t>
         </is>
       </c>
     </row>
     <row r="3435">
       <c r="A3435" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3435" t="n">
-        <v>3272</v>
+        <v>3271</v>
       </c>
       <c r="C3435" t="inlineStr">
         <is>
-          <t>ANNE BEATRIZ SILVA VIRGINO</t>
+          <t>DIEGO DE ARAUJO CALÁBRIA</t>
         </is>
       </c>
       <c r="D3435" t="inlineStr">
         <is>
-          <t>ABVIRGINIO</t>
+          <t>ARAUJOC</t>
         </is>
       </c>
     </row>
     <row r="3436">
       <c r="A3436" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3436" t="n">
-        <v>3293</v>
+        <v>3272</v>
       </c>
       <c r="C3436" t="inlineStr">
         <is>
-          <t xml:space="preserve">CARLOS ALBERTO VIRIATO SANTOS </t>
+          <t>ANNE BEATRIZ SILVA VIRGINO</t>
         </is>
       </c>
       <c r="D3436" t="inlineStr">
         <is>
-          <t>CVIRIATO</t>
+          <t>ABVIRGINIO</t>
         </is>
       </c>
     </row>
@@ -69158,16 +69158,16 @@
         </is>
       </c>
       <c r="B3437" t="n">
-        <v>3381</v>
+        <v>3293</v>
       </c>
       <c r="C3437" t="inlineStr">
         <is>
-          <t>ALAN CAIQUE SANTOS E SANTOS</t>
+          <t xml:space="preserve">CARLOS ALBERTO VIRIATO SANTOS </t>
         </is>
       </c>
       <c r="D3437" t="inlineStr">
         <is>
-          <t>ALANSANTOS</t>
+          <t>CVIRIATO</t>
         </is>
       </c>
     </row>
@@ -69178,116 +69178,116 @@
         </is>
       </c>
       <c r="B3438" t="n">
-        <v>3443</v>
+        <v>3381</v>
       </c>
       <c r="C3438" t="inlineStr">
         <is>
-          <t>SANON MOREIRA SOUZA</t>
+          <t>ALAN CAIQUE SANTOS E SANTOS</t>
         </is>
       </c>
       <c r="D3438" t="inlineStr">
         <is>
-          <t>SANON</t>
+          <t>ALANSANTOS</t>
         </is>
       </c>
     </row>
     <row r="3439">
       <c r="A3439" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3439" t="n">
-        <v>3516</v>
+        <v>3443</v>
       </c>
       <c r="C3439" t="inlineStr">
         <is>
-          <t>FRANCISCO RILDER TELES DE OLIVEIRA</t>
+          <t>SANON MOREIRA SOUZA</t>
         </is>
       </c>
       <c r="D3439" t="inlineStr">
         <is>
-          <t>RILDER</t>
+          <t>SANON</t>
         </is>
       </c>
     </row>
     <row r="3440">
       <c r="A3440" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3440" t="n">
-        <v>3519</v>
+        <v>3516</v>
       </c>
       <c r="C3440" t="inlineStr">
         <is>
-          <t>MARIA LUANA DE ALMEIDA BATISTA</t>
+          <t>FRANCISCO RILDER TELES DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D3440" t="inlineStr">
         <is>
-          <t>M.LUANA</t>
+          <t>RILDER</t>
         </is>
       </c>
     </row>
     <row r="3441">
       <c r="A3441" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3441" t="n">
-        <v>3540</v>
+        <v>3519</v>
       </c>
       <c r="C3441" t="inlineStr">
         <is>
-          <t>HELEN VITORIA OLIVEIRA DA ROCHA</t>
+          <t>MARIA LUANA DE ALMEIDA BATISTA</t>
         </is>
       </c>
       <c r="D3441" t="inlineStr">
         <is>
-          <t>H.VITORIA</t>
+          <t>M.LUANA</t>
         </is>
       </c>
     </row>
     <row r="3442">
       <c r="A3442" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B3442" t="n">
-        <v>3559</v>
+        <v>3540</v>
       </c>
       <c r="C3442" t="inlineStr">
         <is>
-          <t>ARKBERYS TELES DE SOUSA</t>
+          <t>HELEN VITORIA OLIVEIRA DA ROCHA</t>
         </is>
       </c>
       <c r="D3442" t="inlineStr">
         <is>
-          <t>ARKBERYS</t>
+          <t>H.VITORIA</t>
         </is>
       </c>
     </row>
     <row r="3443">
       <c r="A3443" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3443" t="n">
-        <v>3567</v>
+        <v>3559</v>
       </c>
       <c r="C3443" t="inlineStr">
         <is>
-          <t>PEDRO HENRIQUE VIEIRA DE LIMA</t>
+          <t>ARKBERYS TELES DE SOUSA</t>
         </is>
       </c>
       <c r="D3443" t="inlineStr">
         <is>
-          <t>P.LIMA</t>
+          <t>ARKBERYS</t>
         </is>
       </c>
     </row>
@@ -69298,76 +69298,76 @@
         </is>
       </c>
       <c r="B3444" t="n">
-        <v>3331</v>
+        <v>3567</v>
       </c>
       <c r="C3444" t="inlineStr">
         <is>
-          <t>LOUIZE VANIELLE RODRIGUES FARIAS</t>
+          <t>PEDRO HENRIQUE VIEIRA DE LIMA</t>
         </is>
       </c>
       <c r="D3444" t="inlineStr">
         <is>
-          <t>LVFARIAS</t>
+          <t>P.LIMA</t>
         </is>
       </c>
     </row>
     <row r="3445">
       <c r="A3445" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3445" t="n">
-        <v>3334</v>
+        <v>3331</v>
       </c>
       <c r="C3445" t="inlineStr">
         <is>
-          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+          <t>LOUIZE VANIELLE RODRIGUES FARIAS</t>
         </is>
       </c>
       <c r="D3445" t="inlineStr">
         <is>
-          <t>MTGASPAR</t>
+          <t>LVFARIAS</t>
         </is>
       </c>
     </row>
     <row r="3446">
       <c r="A3446" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3446" t="n">
-        <v>3345</v>
+        <v>3334</v>
       </c>
       <c r="C3446" t="inlineStr">
         <is>
-          <t>AURICÉLIA INACIO PEREIRA</t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
       <c r="D3446" t="inlineStr">
         <is>
-          <t>AIPEREIRA</t>
+          <t>MTGASPAR</t>
         </is>
       </c>
     </row>
     <row r="3447">
       <c r="A3447" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3447" t="n">
-        <v>3363</v>
+        <v>3345</v>
       </c>
       <c r="C3447" t="inlineStr">
         <is>
-          <t>IASMIN LEAL ALVES</t>
+          <t>AURICÉLIA INACIO PEREIRA</t>
         </is>
       </c>
       <c r="D3447" t="inlineStr">
         <is>
-          <t>ILALVES</t>
+          <t>AIPEREIRA</t>
         </is>
       </c>
     </row>
@@ -69378,196 +69378,196 @@
         </is>
       </c>
       <c r="B3448" t="n">
-        <v>3370</v>
+        <v>3363</v>
       </c>
       <c r="C3448" t="inlineStr">
         <is>
-          <t>CARLOS DIEGO ARAUJO ALMEIDA</t>
+          <t>IASMIN LEAL ALVES</t>
         </is>
       </c>
       <c r="D3448" t="inlineStr">
         <is>
-          <t>CDIEGO</t>
+          <t>ILALVES</t>
         </is>
       </c>
     </row>
     <row r="3449">
       <c r="A3449" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3449" t="n">
-        <v>3379</v>
+        <v>3370</v>
       </c>
       <c r="C3449" t="inlineStr">
         <is>
-          <t xml:space="preserve">MATHEUS EVANGELISTA FERREIRA </t>
+          <t>CARLOS DIEGO ARAUJO ALMEIDA</t>
         </is>
       </c>
       <c r="D3449" t="inlineStr">
         <is>
-          <t>MMFERREIRA</t>
+          <t>CDIEGO</t>
         </is>
       </c>
     </row>
     <row r="3450">
       <c r="A3450" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3450" t="n">
-        <v>3419</v>
+        <v>3379</v>
       </c>
       <c r="C3450" t="inlineStr">
         <is>
-          <t xml:space="preserve">DAVID EVANGELISTA SILVA </t>
+          <t xml:space="preserve">MATHEUS EVANGELISTA FERREIRA </t>
         </is>
       </c>
       <c r="D3450" t="inlineStr">
         <is>
-          <t>DAVID</t>
+          <t>MMFERREIRA</t>
         </is>
       </c>
     </row>
     <row r="3451">
       <c r="A3451" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3451" t="n">
-        <v>3423</v>
+        <v>3419</v>
       </c>
       <c r="C3451" t="inlineStr">
         <is>
-          <t>MARCIO JOSE TIAGO</t>
+          <t xml:space="preserve">DAVID EVANGELISTA SILVA </t>
         </is>
       </c>
       <c r="D3451" t="inlineStr">
         <is>
-          <t>MJTIAGO</t>
+          <t>DAVID</t>
         </is>
       </c>
     </row>
     <row r="3452">
       <c r="A3452" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3452" t="n">
-        <v>3453</v>
+        <v>3423</v>
       </c>
       <c r="C3452" t="inlineStr">
         <is>
-          <t xml:space="preserve">LAURIENE SILVA BARBOSA </t>
+          <t>MARCIO JOSE TIAGO</t>
         </is>
       </c>
       <c r="D3452" t="inlineStr">
         <is>
-          <t>LAURIENE</t>
+          <t>MJTIAGO</t>
         </is>
       </c>
     </row>
     <row r="3453">
       <c r="A3453" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3453" t="n">
-        <v>3478</v>
+        <v>3453</v>
       </c>
       <c r="C3453" t="inlineStr">
         <is>
-          <t>LEANDRO BRITO NOGUEIRA DE OLIVEIRA</t>
+          <t xml:space="preserve">LAURIENE SILVA BARBOSA </t>
         </is>
       </c>
       <c r="D3453" t="inlineStr">
         <is>
-          <t>LBNOGUEIRA</t>
+          <t>LAURIENE</t>
         </is>
       </c>
     </row>
     <row r="3454">
       <c r="A3454" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3454" t="n">
-        <v>3479</v>
+        <v>3478</v>
       </c>
       <c r="C3454" t="inlineStr">
         <is>
-          <t>ESDRAS ALESSANDRO SANTOS SANTANA</t>
+          <t>LEANDRO BRITO NOGUEIRA DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D3454" t="inlineStr">
         <is>
-          <t>EALESSANDRO</t>
+          <t>LBNOGUEIRA</t>
         </is>
       </c>
     </row>
     <row r="3455">
       <c r="A3455" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3455" t="n">
-        <v>3480</v>
+        <v>3479</v>
       </c>
       <c r="C3455" t="inlineStr">
         <is>
-          <t xml:space="preserve">LUCIMARA SOUSA LIMA </t>
+          <t>ESDRAS ALESSANDRO SANTOS SANTANA</t>
         </is>
       </c>
       <c r="D3455" t="inlineStr">
         <is>
-          <t>LUCIMARA</t>
+          <t>EALESSANDRO</t>
         </is>
       </c>
     </row>
     <row r="3456">
       <c r="A3456" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3456" t="n">
-        <v>3482</v>
+        <v>3480</v>
       </c>
       <c r="C3456" t="inlineStr">
         <is>
-          <t>DANIEL FERNANDES DINIZ HERACLIO</t>
+          <t xml:space="preserve">LUCIMARA SOUSA LIMA </t>
         </is>
       </c>
       <c r="D3456" t="inlineStr">
         <is>
-          <t>DFDINIZ</t>
+          <t>LUCIMARA</t>
         </is>
       </c>
     </row>
     <row r="3457">
       <c r="A3457" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3457" t="n">
-        <v>3518</v>
+        <v>3482</v>
       </c>
       <c r="C3457" t="inlineStr">
         <is>
-          <t>RAMYRA ALVES FELIX DA SILVA</t>
+          <t>DANIEL FERNANDES DINIZ HERACLIO</t>
         </is>
       </c>
       <c r="D3457" t="inlineStr">
         <is>
-          <t>RFELIX</t>
+          <t>DFDINIZ</t>
         </is>
       </c>
     </row>
@@ -69578,36 +69578,36 @@
         </is>
       </c>
       <c r="B3458" t="n">
-        <v>3534</v>
+        <v>3518</v>
       </c>
       <c r="C3458" t="inlineStr">
         <is>
-          <t xml:space="preserve">CAIO DE SOUZA VINHAS </t>
+          <t>RAMYRA ALVES FELIX DA SILVA</t>
         </is>
       </c>
       <c r="D3458" t="inlineStr">
         <is>
-          <t>CVINHAS</t>
+          <t>RFELIX</t>
         </is>
       </c>
     </row>
     <row r="3459">
       <c r="A3459" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3459" t="n">
-        <v>3535</v>
+        <v>3534</v>
       </c>
       <c r="C3459" t="inlineStr">
         <is>
-          <t>ROMARIO DE SOUSA SILVA</t>
+          <t xml:space="preserve">CAIO DE SOUZA VINHAS </t>
         </is>
       </c>
       <c r="D3459" t="inlineStr">
         <is>
-          <t>RSOUSAS</t>
+          <t>CVINHAS</t>
         </is>
       </c>
     </row>
@@ -69618,56 +69618,56 @@
         </is>
       </c>
       <c r="B3460" t="n">
-        <v>3536</v>
+        <v>3535</v>
       </c>
       <c r="C3460" t="inlineStr">
         <is>
-          <t>JHONATAS CARVALHO OLIVEIRA</t>
+          <t>ROMARIO DE SOUSA SILVA</t>
         </is>
       </c>
       <c r="D3460" t="inlineStr">
         <is>
-          <t>JHONATASC</t>
+          <t>RSOUSAS</t>
         </is>
       </c>
     </row>
     <row r="3461">
       <c r="A3461" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3461" t="n">
-        <v>940529</v>
+        <v>3536</v>
       </c>
       <c r="C3461" t="inlineStr">
         <is>
-          <t>EDGAR FELIX - FL9</t>
+          <t>JHONATAS CARVALHO OLIVEIRA</t>
         </is>
       </c>
       <c r="D3461" t="inlineStr">
         <is>
-          <t>EDGAR F</t>
+          <t>JHONATASC</t>
         </is>
       </c>
     </row>
     <row r="3462">
       <c r="A3462" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3462" t="n">
-        <v>3304</v>
+        <v>940529</v>
       </c>
       <c r="C3462" t="inlineStr">
         <is>
-          <t>JOACI GUILHERME GONÇALVES DA LUZ</t>
+          <t>EDGAR FELIX - FL9</t>
         </is>
       </c>
       <c r="D3462" t="inlineStr">
         <is>
-          <t>JLUZ</t>
+          <t>EDGAR F</t>
         </is>
       </c>
     </row>
@@ -69678,16 +69678,16 @@
         </is>
       </c>
       <c r="B3463" t="n">
-        <v>3305</v>
+        <v>3304</v>
       </c>
       <c r="C3463" t="inlineStr">
         <is>
-          <t>JOÃO VITOR DE ARAÚJO GONÇALVES</t>
+          <t>JOACI GUILHERME GONÇALVES DA LUZ</t>
         </is>
       </c>
       <c r="D3463" t="inlineStr">
         <is>
-          <t>JJVITOR</t>
+          <t>JLUZ</t>
         </is>
       </c>
     </row>
@@ -69698,36 +69698,36 @@
         </is>
       </c>
       <c r="B3464" t="n">
-        <v>3306</v>
+        <v>3305</v>
       </c>
       <c r="C3464" t="inlineStr">
         <is>
-          <t>WENDERSON MARCOS DOS SANTOS</t>
+          <t>JOÃO VITOR DE ARAÚJO GONÇALVES</t>
         </is>
       </c>
       <c r="D3464" t="inlineStr">
         <is>
-          <t>WWMARCOS</t>
+          <t>JJVITOR</t>
         </is>
       </c>
     </row>
     <row r="3465">
       <c r="A3465" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3465" t="n">
-        <v>3335</v>
+        <v>3306</v>
       </c>
       <c r="C3465" t="inlineStr">
         <is>
-          <t>EDILBERTO LEMOS DE LIMA</t>
+          <t>WENDERSON MARCOS DOS SANTOS</t>
         </is>
       </c>
       <c r="D3465" t="inlineStr">
         <is>
-          <t>ELEMOS</t>
+          <t>WWMARCOS</t>
         </is>
       </c>
     </row>
@@ -69738,136 +69738,136 @@
         </is>
       </c>
       <c r="B3466" t="n">
-        <v>3336</v>
+        <v>3335</v>
       </c>
       <c r="C3466" t="inlineStr">
         <is>
-          <t>EZEQUIEL SOUZA DO NASCIMENTO</t>
+          <t>EDILBERTO LEMOS DE LIMA</t>
         </is>
       </c>
       <c r="D3466" t="inlineStr">
         <is>
-          <t>ESNASCIMENTO</t>
+          <t>ELEMOS</t>
         </is>
       </c>
     </row>
     <row r="3467">
       <c r="A3467" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3467" t="n">
-        <v>3341</v>
+        <v>3336</v>
       </c>
       <c r="C3467" t="inlineStr">
         <is>
-          <t>ALCIONE MARIANO DE OLIVEIRA</t>
+          <t>EZEQUIEL SOUZA DO NASCIMENTO</t>
         </is>
       </c>
       <c r="D3467" t="inlineStr">
         <is>
-          <t>AMOLIVEIRA</t>
+          <t>ESNASCIMENTO</t>
         </is>
       </c>
     </row>
     <row r="3468">
       <c r="A3468" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3468" t="n">
-        <v>3401</v>
+        <v>3341</v>
       </c>
       <c r="C3468" t="inlineStr">
         <is>
-          <t xml:space="preserve">TULIO HENRIQUE DA SILVA CARVALHO </t>
+          <t>ALCIONE MARIANO DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D3468" t="inlineStr">
         <is>
-          <t>TULIO</t>
+          <t>AMOLIVEIRA</t>
         </is>
       </c>
     </row>
     <row r="3469">
       <c r="A3469" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3469" t="n">
-        <v>3411</v>
+        <v>3401</v>
       </c>
       <c r="C3469" t="inlineStr">
         <is>
-          <t>CONEXAO RUBYA DANILLA</t>
+          <t xml:space="preserve">TULIO HENRIQUE DA SILVA CARVALHO </t>
         </is>
       </c>
       <c r="D3469" t="inlineStr">
         <is>
-          <t>CONEXAORUBYA</t>
+          <t>TULIO</t>
         </is>
       </c>
     </row>
     <row r="3470">
       <c r="A3470" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3470" t="n">
-        <v>3412</v>
+        <v>3411</v>
       </c>
       <c r="C3470" t="inlineStr">
         <is>
-          <t>CONEXAO RAFAEL</t>
+          <t>CONEXAO RUBYA DANILLA</t>
         </is>
       </c>
       <c r="D3470" t="inlineStr">
         <is>
-          <t>CONEXAORAFAEL</t>
+          <t>CONEXAORUBYA</t>
         </is>
       </c>
     </row>
     <row r="3471">
       <c r="A3471" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3471" t="n">
-        <v>3558</v>
+        <v>3412</v>
       </c>
       <c r="C3471" t="inlineStr">
         <is>
-          <t>WALLYS QUEIROZ VIANA</t>
+          <t>CONEXAO RAFAEL</t>
         </is>
       </c>
       <c r="D3471" t="inlineStr">
         <is>
-          <t>WALLYS</t>
+          <t>CONEXAORAFAEL</t>
         </is>
       </c>
     </row>
     <row r="3472">
       <c r="A3472" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3472" t="n">
-        <v>3264</v>
+        <v>3558</v>
       </c>
       <c r="C3472" t="inlineStr">
         <is>
-          <t xml:space="preserve">WILTON CARLOS MACIEL DE ASSIS </t>
+          <t>WALLYS QUEIROZ VIANA</t>
         </is>
       </c>
       <c r="D3472" t="inlineStr">
         <is>
-          <t>WCMACIEL</t>
+          <t>WALLYS</t>
         </is>
       </c>
     </row>
@@ -69878,56 +69878,56 @@
         </is>
       </c>
       <c r="B3473" t="n">
-        <v>3340</v>
+        <v>3264</v>
       </c>
       <c r="C3473" t="inlineStr">
         <is>
-          <t>ROGELENO FARIAS FEIJÃO FILHO</t>
+          <t xml:space="preserve">WILTON CARLOS MACIEL DE ASSIS </t>
         </is>
       </c>
       <c r="D3473" t="inlineStr">
         <is>
-          <t>RFEIJAO</t>
+          <t>WCMACIEL</t>
         </is>
       </c>
     </row>
     <row r="3474">
       <c r="A3474" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3474" t="n">
-        <v>940550</v>
+        <v>3340</v>
       </c>
       <c r="C3474" t="inlineStr">
         <is>
-          <t>RAFAELE RIBEIRO CARNEIRO</t>
+          <t>ROGELENO FARIAS FEIJÃO FILHO</t>
         </is>
       </c>
       <c r="D3474" t="inlineStr">
         <is>
-          <t>RAFAELE</t>
+          <t>RFEIJAO</t>
         </is>
       </c>
     </row>
     <row r="3475">
       <c r="A3475" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>99</t>
         </is>
       </c>
       <c r="B3475" t="n">
-        <v>3377</v>
+        <v>940550</v>
       </c>
       <c r="C3475" t="inlineStr">
         <is>
-          <t xml:space="preserve"> ISALTINO BISPO DE OLIVEIRA JUNIOR</t>
+          <t>RAFAELE RIBEIRO CARNEIRO</t>
         </is>
       </c>
       <c r="D3475" t="inlineStr">
         <is>
-          <t>BJUNIOR</t>
+          <t>RAFAELE</t>
         </is>
       </c>
     </row>
@@ -69938,56 +69938,56 @@
         </is>
       </c>
       <c r="B3476" t="n">
-        <v>3425</v>
+        <v>3377</v>
       </c>
       <c r="C3476" t="inlineStr">
         <is>
-          <t xml:space="preserve"> CIRLANE ARAUJO SOUZA </t>
+          <t xml:space="preserve"> ISALTINO BISPO DE OLIVEIRA JUNIOR</t>
         </is>
       </c>
       <c r="D3476" t="inlineStr">
         <is>
-          <t>CIRLANES</t>
+          <t>BJUNIOR</t>
         </is>
       </c>
     </row>
     <row r="3477">
       <c r="A3477" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3477" t="n">
-        <v>3454</v>
+        <v>3425</v>
       </c>
       <c r="C3477" t="inlineStr">
         <is>
-          <t>ANTONIA SAMARA DE SOUZA SOARES</t>
+          <t xml:space="preserve"> CIRLANE ARAUJO SOUZA </t>
         </is>
       </c>
       <c r="D3477" t="inlineStr">
         <is>
-          <t>ANTSAMARA</t>
+          <t>CIRLANES</t>
         </is>
       </c>
     </row>
     <row r="3478">
       <c r="A3478" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3478" t="n">
-        <v>3491</v>
+        <v>3454</v>
       </c>
       <c r="C3478" t="inlineStr">
         <is>
-          <t>PEDRO JOSE DO NASCIMENTO NETO</t>
+          <t>ANTONIA SAMARA DE SOUZA SOARES</t>
         </is>
       </c>
       <c r="D3478" t="inlineStr">
         <is>
-          <t>P.JOSE</t>
+          <t>ANTSAMARA</t>
         </is>
       </c>
     </row>
@@ -69998,36 +69998,36 @@
         </is>
       </c>
       <c r="B3479" t="n">
-        <v>3492</v>
+        <v>3491</v>
       </c>
       <c r="C3479" t="inlineStr">
         <is>
-          <t>PAULA CARLA CALDAS MOTA</t>
+          <t>PEDRO JOSE DO NASCIMENTO NETO</t>
         </is>
       </c>
       <c r="D3479" t="inlineStr">
         <is>
-          <t>P.CARLA</t>
+          <t>P.JOSE</t>
         </is>
       </c>
     </row>
     <row r="3480">
       <c r="A3480" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3480" t="n">
-        <v>3542</v>
+        <v>3492</v>
       </c>
       <c r="C3480" t="inlineStr">
         <is>
-          <t>ANTONIA MILENA SOUSA ANDRADE</t>
+          <t>PAULA CARLA CALDAS MOTA</t>
         </is>
       </c>
       <c r="D3480" t="inlineStr">
         <is>
-          <t>A.MILENA</t>
+          <t>P.CARLA</t>
         </is>
       </c>
     </row>
@@ -70038,56 +70038,56 @@
         </is>
       </c>
       <c r="B3481" t="n">
-        <v>3547</v>
+        <v>3542</v>
       </c>
       <c r="C3481" t="inlineStr">
         <is>
-          <t xml:space="preserve">DAVI PEREIRA DA SILVA </t>
+          <t>ANTONIA MILENA SOUSA ANDRADE</t>
         </is>
       </c>
       <c r="D3481" t="inlineStr">
         <is>
-          <t>DPSILVA</t>
+          <t>A.MILENA</t>
         </is>
       </c>
     </row>
     <row r="3482">
       <c r="A3482" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3482" t="n">
-        <v>3552</v>
+        <v>3547</v>
       </c>
       <c r="C3482" t="inlineStr">
         <is>
-          <t>PAULO SERGIO MENDES DE OLIVEIRA</t>
+          <t xml:space="preserve">DAVI PEREIRA DA SILVA </t>
         </is>
       </c>
       <c r="D3482" t="inlineStr">
         <is>
-          <t>PSMENDES</t>
+          <t>DPSILVA</t>
         </is>
       </c>
     </row>
     <row r="3483">
       <c r="A3483" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3483" t="n">
-        <v>3294</v>
+        <v>3552</v>
       </c>
       <c r="C3483" t="inlineStr">
         <is>
-          <t>GLEICIANE MIRANDA DE MORAIS</t>
+          <t>PAULO SERGIO MENDES DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D3483" t="inlineStr">
         <is>
-          <t>GMIRANDA</t>
+          <t>PSMENDES</t>
         </is>
       </c>
     </row>
@@ -70098,176 +70098,176 @@
         </is>
       </c>
       <c r="B3484" t="n">
-        <v>3295</v>
+        <v>3294</v>
       </c>
       <c r="C3484" t="inlineStr">
         <is>
-          <t>MARIA ESTEFANNY DA SILVA MOURA</t>
+          <t>GLEICIANE MIRANDA DE MORAIS</t>
         </is>
       </c>
       <c r="D3484" t="inlineStr">
         <is>
-          <t>MESTEFANNY</t>
+          <t>GMIRANDA</t>
         </is>
       </c>
     </row>
     <row r="3485">
       <c r="A3485" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3485" t="n">
-        <v>3296</v>
+        <v>3295</v>
       </c>
       <c r="C3485" t="inlineStr">
         <is>
-          <t>PEDRO IAGO FONSECA EVANGELISTA</t>
+          <t>MARIA ESTEFANNY DA SILVA MOURA</t>
         </is>
       </c>
       <c r="D3485" t="inlineStr">
         <is>
-          <t>PIFONSECA</t>
+          <t>MESTEFANNY</t>
         </is>
       </c>
     </row>
     <row r="3486">
       <c r="A3486" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3486" t="n">
-        <v>940544</v>
+        <v>3296</v>
       </c>
       <c r="C3486" t="inlineStr">
         <is>
-          <t>LUTY LOG TRANSPORTES - FL8</t>
+          <t>PEDRO IAGO FONSECA EVANGELISTA</t>
         </is>
       </c>
       <c r="D3486" t="inlineStr">
         <is>
-          <t>LUTY LOG</t>
+          <t>PIFONSECA</t>
         </is>
       </c>
     </row>
     <row r="3487">
       <c r="A3487" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B3487" t="n">
-        <v>3380</v>
+        <v>940544</v>
       </c>
       <c r="C3487" t="inlineStr">
         <is>
-          <t>FRANCISCO MATHEUS RABELO DA COSTA</t>
+          <t>LUTY LOG TRANSPORTES - FL8</t>
         </is>
       </c>
       <c r="D3487" t="inlineStr">
         <is>
-          <t>FMATHEUS</t>
+          <t>LUTY LOG</t>
         </is>
       </c>
     </row>
     <row r="3488">
       <c r="A3488" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3488" t="n">
-        <v>3410</v>
+        <v>3380</v>
       </c>
       <c r="C3488" t="inlineStr">
         <is>
-          <t xml:space="preserve"> BRENO ALLAN DE JESUS</t>
+          <t>FRANCISCO MATHEUS RABELO DA COSTA</t>
         </is>
       </c>
       <c r="D3488" t="inlineStr">
         <is>
-          <t>JESUS</t>
+          <t>FMATHEUS</t>
         </is>
       </c>
     </row>
     <row r="3489">
       <c r="A3489" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3489" t="n">
-        <v>3444</v>
+        <v>3410</v>
       </c>
       <c r="C3489" t="inlineStr">
         <is>
-          <t>THIAGO COSTA SILVA</t>
+          <t xml:space="preserve"> BRENO ALLAN DE JESUS</t>
         </is>
       </c>
       <c r="D3489" t="inlineStr">
         <is>
-          <t>THIAGOC</t>
+          <t>JESUS</t>
         </is>
       </c>
     </row>
     <row r="3490">
       <c r="A3490" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3490" t="n">
-        <v>3456</v>
+        <v>3444</v>
       </c>
       <c r="C3490" t="inlineStr">
         <is>
-          <t>FELIPE BOTH MAZUCHINI</t>
+          <t>THIAGO COSTA SILVA</t>
         </is>
       </c>
       <c r="D3490" t="inlineStr">
         <is>
-          <t>FELIPEB</t>
+          <t>THIAGOC</t>
         </is>
       </c>
     </row>
     <row r="3491">
       <c r="A3491" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3491" t="n">
-        <v>3457</v>
+        <v>3456</v>
       </c>
       <c r="C3491" t="inlineStr">
         <is>
-          <t>FRANKLIN VIEIRA GOMES</t>
+          <t>FELIPE BOTH MAZUCHINI</t>
         </is>
       </c>
       <c r="D3491" t="inlineStr">
         <is>
-          <t>VIEIRAF</t>
+          <t>FELIPEB</t>
         </is>
       </c>
     </row>
     <row r="3492">
       <c r="A3492" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3492" t="n">
-        <v>3507</v>
+        <v>3457</v>
       </c>
       <c r="C3492" t="inlineStr">
         <is>
-          <t>KARINE TEODORA ALVES DE OLIVEIRA</t>
+          <t>FRANKLIN VIEIRA GOMES</t>
         </is>
       </c>
       <c r="D3492" t="inlineStr">
         <is>
-          <t>KOLIVEIRA</t>
+          <t>VIEIRAF</t>
         </is>
       </c>
     </row>
@@ -70278,14 +70278,34 @@
         </is>
       </c>
       <c r="B3493" t="n">
+        <v>3507</v>
+      </c>
+      <c r="C3493" t="inlineStr">
+        <is>
+          <t>KARINE TEODORA ALVES DE OLIVEIRA</t>
+        </is>
+      </c>
+      <c r="D3493" t="inlineStr">
+        <is>
+          <t>KOLIVEIRA</t>
+        </is>
+      </c>
+    </row>
+    <row r="3494">
+      <c r="A3494" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B3494" t="n">
         <v>3520</v>
       </c>
-      <c r="C3493" t="inlineStr">
+      <c r="C3494" t="inlineStr">
         <is>
           <t xml:space="preserve"> EMERSON FILIPE MELO DE AGUIAR</t>
         </is>
       </c>
-      <c r="D3493" t="inlineStr">
+      <c r="D3494" t="inlineStr">
         <is>
           <t>E.FILIPE</t>
         </is>

</xml_diff>

<commit_message>
chore(data): batch update intraday televendas - 08:01:34
</commit_message>
<xml_diff>
--- a/data/dim_televendas.xlsx
+++ b/data/dim_televendas.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3494"/>
+  <dimension ref="A1:D3496"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -52542,7 +52542,7 @@
       </c>
       <c r="C2606" t="inlineStr">
         <is>
-          <t>MARLY DARLY DE ARAUJO</t>
+          <t>MARY DARLY DE ARAUJO</t>
         </is>
       </c>
       <c r="D2606" t="inlineStr">
@@ -66358,56 +66358,56 @@
         </is>
       </c>
       <c r="B3297" t="n">
-        <v>3279</v>
+        <v>3582</v>
       </c>
       <c r="C3297" t="inlineStr">
         <is>
-          <t>IARGO GABRIEL SANTOS DE OLIVEIRA</t>
+          <t>MARCOS SERGIO DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D3297" t="inlineStr">
         <is>
-          <t>IARGOSANTOS</t>
+          <t>MARCOS.S</t>
         </is>
       </c>
     </row>
     <row r="3298">
       <c r="A3298" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3298" t="n">
-        <v>3349</v>
+        <v>3279</v>
       </c>
       <c r="C3298" t="inlineStr">
         <is>
-          <t xml:space="preserve">ROBSON DE SOUZA LEITE </t>
+          <t>IARGO GABRIEL SANTOS DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D3298" t="inlineStr">
         <is>
-          <t>RLEITE</t>
+          <t>IARGOSANTOS</t>
         </is>
       </c>
     </row>
     <row r="3299">
       <c r="A3299" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3299" t="n">
-        <v>3367</v>
+        <v>3349</v>
       </c>
       <c r="C3299" t="inlineStr">
         <is>
-          <t>CARLOS JEANDERSON DA SILVA GUTERRES</t>
+          <t xml:space="preserve">ROBSON DE SOUZA LEITE </t>
         </is>
       </c>
       <c r="D3299" t="inlineStr">
         <is>
-          <t>CGUTERRES</t>
+          <t>RLEITE</t>
         </is>
       </c>
     </row>
@@ -66418,96 +66418,96 @@
         </is>
       </c>
       <c r="B3300" t="n">
-        <v>3392</v>
+        <v>3367</v>
       </c>
       <c r="C3300" t="inlineStr">
         <is>
-          <t xml:space="preserve">LAERCIA KARINE OLIVEIRA MORAIS </t>
+          <t>CARLOS JEANDERSON DA SILVA GUTERRES</t>
         </is>
       </c>
       <c r="D3300" t="inlineStr">
         <is>
-          <t>KARINE28</t>
+          <t>CGUTERRES</t>
         </is>
       </c>
     </row>
     <row r="3301">
       <c r="A3301" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3301" t="n">
-        <v>3446</v>
+        <v>3392</v>
       </c>
       <c r="C3301" t="inlineStr">
         <is>
-          <t>MARIA FERNANDA SOUSA DA CRUZ</t>
+          <t xml:space="preserve">LAERCIA KARINE OLIVEIRA MORAIS </t>
         </is>
       </c>
       <c r="D3301" t="inlineStr">
         <is>
-          <t>MSCRUZ</t>
+          <t>KARINE28</t>
         </is>
       </c>
     </row>
     <row r="3302">
       <c r="A3302" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3302" t="n">
-        <v>3256</v>
+        <v>3446</v>
       </c>
       <c r="C3302" t="inlineStr">
         <is>
-          <t>ANNE CAROLINE ALMEIDA DE MORAIS</t>
+          <t>MARIA FERNANDA SOUSA DA CRUZ</t>
         </is>
       </c>
       <c r="D3302" t="inlineStr">
         <is>
-          <t>ACMORAIS</t>
+          <t>MSCRUZ</t>
         </is>
       </c>
     </row>
     <row r="3303">
       <c r="A3303" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3303" t="n">
-        <v>3257</v>
+        <v>3256</v>
       </c>
       <c r="C3303" t="inlineStr">
         <is>
-          <t xml:space="preserve"> NARA RAIANE RABELO NOBRE</t>
+          <t>ANNE CAROLINE ALMEIDA DE MORAIS</t>
         </is>
       </c>
       <c r="D3303" t="inlineStr">
         <is>
-          <t>NRNOBRE</t>
+          <t>ACMORAIS</t>
         </is>
       </c>
     </row>
     <row r="3304">
       <c r="A3304" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3304" t="n">
-        <v>3268</v>
+        <v>3257</v>
       </c>
       <c r="C3304" t="inlineStr">
         <is>
-          <t>DANRLEY PEREIRA E PEREIRA</t>
+          <t xml:space="preserve"> NARA RAIANE RABELO NOBRE</t>
         </is>
       </c>
       <c r="D3304" t="inlineStr">
         <is>
-          <t>DPEREIRA</t>
+          <t>NRNOBRE</t>
         </is>
       </c>
     </row>
@@ -66518,16 +66518,16 @@
         </is>
       </c>
       <c r="B3305" t="n">
-        <v>3282</v>
+        <v>3268</v>
       </c>
       <c r="C3305" t="inlineStr">
         <is>
-          <t xml:space="preserve">JARDSON ROBERTH CUTRIM SOUZA </t>
+          <t>DANRLEY PEREIRA E PEREIRA</t>
         </is>
       </c>
       <c r="D3305" t="inlineStr">
         <is>
-          <t>JRCSOUZA</t>
+          <t>DPEREIRA</t>
         </is>
       </c>
     </row>
@@ -66538,156 +66538,156 @@
         </is>
       </c>
       <c r="B3306" t="n">
-        <v>3283</v>
+        <v>3282</v>
       </c>
       <c r="C3306" t="inlineStr">
         <is>
-          <t>JESOAIAS DOS SANTOS CABRAL</t>
+          <t xml:space="preserve">JARDSON ROBERTH CUTRIM SOUZA </t>
         </is>
       </c>
       <c r="D3306" t="inlineStr">
         <is>
-          <t>JSCABRAL</t>
+          <t>JRCSOUZA</t>
         </is>
       </c>
     </row>
     <row r="3307">
       <c r="A3307" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3307" t="n">
-        <v>3299</v>
+        <v>3283</v>
       </c>
       <c r="C3307" t="inlineStr">
         <is>
-          <t>CARLOS EDUARDO ANDRADE DE ASSIS</t>
+          <t>JESOAIAS DOS SANTOS CABRAL</t>
         </is>
       </c>
       <c r="D3307" t="inlineStr">
         <is>
-          <t>ANDRADE</t>
+          <t>JSCABRAL</t>
         </is>
       </c>
     </row>
     <row r="3308">
       <c r="A3308" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3308" t="n">
-        <v>3301</v>
+        <v>3299</v>
       </c>
       <c r="C3308" t="inlineStr">
         <is>
-          <t>DIANA KARINE VIANA DA SILVA</t>
+          <t>CARLOS EDUARDO ANDRADE DE ASSIS</t>
         </is>
       </c>
       <c r="D3308" t="inlineStr">
         <is>
-          <t>DKVIANA</t>
+          <t>ANDRADE</t>
         </is>
       </c>
     </row>
     <row r="3309">
       <c r="A3309" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3309" t="n">
-        <v>940537</v>
+        <v>3301</v>
       </c>
       <c r="C3309" t="inlineStr">
         <is>
-          <t xml:space="preserve">TGC TRANSPORTES </t>
+          <t>DIANA KARINE VIANA DA SILVA</t>
         </is>
       </c>
       <c r="D3309" t="inlineStr">
         <is>
-          <t>TGC</t>
+          <t>DKVIANA</t>
         </is>
       </c>
     </row>
     <row r="3310">
       <c r="A3310" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3310" t="n">
-        <v>3343</v>
+        <v>940537</v>
       </c>
       <c r="C3310" t="inlineStr">
         <is>
-          <t>REGINALDO FEITOSA DA SILVA JUNIOR</t>
+          <t xml:space="preserve">TGC TRANSPORTES </t>
         </is>
       </c>
       <c r="D3310" t="inlineStr">
         <is>
-          <t>RFJUNIOR</t>
+          <t>TGC</t>
         </is>
       </c>
     </row>
     <row r="3311">
       <c r="A3311" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3311" t="n">
-        <v>3344</v>
+        <v>3343</v>
       </c>
       <c r="C3311" t="inlineStr">
         <is>
-          <t>JOAO VICTOR MENDONCA DA SILVA</t>
+          <t>REGINALDO FEITOSA DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="D3311" t="inlineStr">
         <is>
-          <t>JVMENDONCA</t>
+          <t>RFJUNIOR</t>
         </is>
       </c>
     </row>
     <row r="3312">
       <c r="A3312" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3312" t="n">
-        <v>3352</v>
+        <v>3344</v>
       </c>
       <c r="C3312" t="inlineStr">
         <is>
-          <t>RICARDO MACAUBAS BOAVENTURA</t>
+          <t>JOAO VICTOR MENDONCA DA SILVA</t>
         </is>
       </c>
       <c r="D3312" t="inlineStr">
         <is>
-          <t>RMACAUBAS</t>
+          <t>JVMENDONCA</t>
         </is>
       </c>
     </row>
     <row r="3313">
       <c r="A3313" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3313" t="n">
-        <v>3364</v>
+        <v>3352</v>
       </c>
       <c r="C3313" t="inlineStr">
         <is>
-          <t>CLOVIS VIDAL DOS SANTOS NETO</t>
+          <t>RICARDO MACAUBAS BOAVENTURA</t>
         </is>
       </c>
       <c r="D3313" t="inlineStr">
         <is>
-          <t>CVNETO</t>
+          <t>RMACAUBAS</t>
         </is>
       </c>
     </row>
@@ -66698,156 +66698,156 @@
         </is>
       </c>
       <c r="B3314" t="n">
-        <v>3365</v>
+        <v>3364</v>
       </c>
       <c r="C3314" t="inlineStr">
         <is>
-          <t>CYNTIA RAFAELLA DE PONTES</t>
+          <t>CLOVIS VIDAL DOS SANTOS NETO</t>
         </is>
       </c>
       <c r="D3314" t="inlineStr">
         <is>
-          <t>CRPONTES</t>
+          <t>CVNETO</t>
         </is>
       </c>
     </row>
     <row r="3315">
       <c r="A3315" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3315" t="n">
-        <v>3387</v>
+        <v>3365</v>
       </c>
       <c r="C3315" t="inlineStr">
         <is>
-          <t>VALDECI NASCIMENTO DELGADO JUNIOR</t>
+          <t>CYNTIA RAFAELLA DE PONTES</t>
         </is>
       </c>
       <c r="D3315" t="inlineStr">
         <is>
-          <t>VALDECI05</t>
+          <t>CRPONTES</t>
         </is>
       </c>
     </row>
     <row r="3316">
       <c r="A3316" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3316" t="n">
-        <v>3458</v>
+        <v>3387</v>
       </c>
       <c r="C3316" t="inlineStr">
         <is>
-          <t>EDUARDO BEZERRA DE SOUSA</t>
+          <t>VALDECI NASCIMENTO DELGADO JUNIOR</t>
         </is>
       </c>
       <c r="D3316" t="inlineStr">
         <is>
-          <t>EDUARDOB</t>
+          <t>VALDECI05</t>
         </is>
       </c>
     </row>
     <row r="3317">
       <c r="A3317" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3317" t="n">
-        <v>940561</v>
+        <v>3458</v>
       </c>
       <c r="C3317" t="inlineStr">
         <is>
-          <t>NAIRTON DE ARAUJO MONTEIRO</t>
+          <t>EDUARDO BEZERRA DE SOUSA</t>
         </is>
       </c>
       <c r="D3317" t="inlineStr">
         <is>
-          <t>NAIRTON</t>
+          <t>EDUARDOB</t>
         </is>
       </c>
     </row>
     <row r="3318">
       <c r="A3318" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>99</t>
         </is>
       </c>
       <c r="B3318" t="n">
-        <v>3515</v>
+        <v>940561</v>
       </c>
       <c r="C3318" t="inlineStr">
         <is>
-          <t>DANIEL DOS SANTOS DE ALMEIDA</t>
+          <t>NAIRTON DE ARAUJO MONTEIRO</t>
         </is>
       </c>
       <c r="D3318" t="inlineStr">
         <is>
-          <t>DANIELSA</t>
+          <t>NAIRTON</t>
         </is>
       </c>
     </row>
     <row r="3319">
       <c r="A3319" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3319" t="n">
-        <v>3288</v>
+        <v>3515</v>
       </c>
       <c r="C3319" t="inlineStr">
         <is>
-          <t>ANA MARIA AMORIM MENDONÇA</t>
+          <t>DANIEL DOS SANTOS DE ALMEIDA</t>
         </is>
       </c>
       <c r="D3319" t="inlineStr">
         <is>
-          <t>AMENDONCA</t>
+          <t>DANIELSA</t>
         </is>
       </c>
     </row>
     <row r="3320">
       <c r="A3320" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3320" t="n">
-        <v>3312</v>
+        <v>3288</v>
       </c>
       <c r="C3320" t="inlineStr">
         <is>
-          <t>AURIANA LIMA DE MORAES</t>
+          <t>ANA MARIA AMORIM MENDONÇA</t>
         </is>
       </c>
       <c r="D3320" t="inlineStr">
         <is>
-          <t>ALM</t>
+          <t>AMENDONCA</t>
         </is>
       </c>
     </row>
     <row r="3321">
       <c r="A3321" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3321" t="n">
-        <v>940547</v>
+        <v>3312</v>
       </c>
       <c r="C3321" t="inlineStr">
         <is>
-          <t>JM EXPRESS - AGRESTE</t>
+          <t>AURIANA LIMA DE MORAES</t>
         </is>
       </c>
       <c r="D3321" t="inlineStr">
         <is>
-          <t>J M A</t>
+          <t>ALM</t>
         </is>
       </c>
     </row>
@@ -66858,76 +66858,76 @@
         </is>
       </c>
       <c r="B3322" t="n">
-        <v>940548</v>
+        <v>940547</v>
       </c>
       <c r="C3322" t="inlineStr">
         <is>
-          <t>JM EXPRESS - SERTAO</t>
+          <t>JM EXPRESS - AGRESTE</t>
         </is>
       </c>
       <c r="D3322" t="inlineStr">
         <is>
-          <t>J M S</t>
+          <t>J M A</t>
         </is>
       </c>
     </row>
     <row r="3323">
       <c r="A3323" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3323" t="n">
-        <v>940551</v>
+        <v>940548</v>
       </c>
       <c r="C3323" t="inlineStr">
         <is>
-          <t>LUCAS PONTES NOBRE</t>
+          <t>JM EXPRESS - SERTAO</t>
         </is>
       </c>
       <c r="D3323" t="inlineStr">
         <is>
-          <t>PONTES</t>
+          <t>J M S</t>
         </is>
       </c>
     </row>
     <row r="3324">
       <c r="A3324" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>99</t>
         </is>
       </c>
       <c r="B3324" t="n">
-        <v>3382</v>
+        <v>940551</v>
       </c>
       <c r="C3324" t="inlineStr">
         <is>
-          <t>MARIA CASSILANIA SOUSA DO NASCIMENTO</t>
+          <t>LUCAS PONTES NOBRE</t>
         </is>
       </c>
       <c r="D3324" t="inlineStr">
         <is>
-          <t>MCASSILANIA</t>
+          <t>PONTES</t>
         </is>
       </c>
     </row>
     <row r="3325">
       <c r="A3325" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3325" t="n">
-        <v>3474</v>
+        <v>3382</v>
       </c>
       <c r="C3325" t="inlineStr">
         <is>
-          <t>MARCOS VINICIUS GONCALVES MIRANDA</t>
+          <t>MARIA CASSILANIA SOUSA DO NASCIMENTO</t>
         </is>
       </c>
       <c r="D3325" t="inlineStr">
         <is>
-          <t>MARCOS.VINICIUS</t>
+          <t>MCASSILANIA</t>
         </is>
       </c>
     </row>
@@ -66938,176 +66938,176 @@
         </is>
       </c>
       <c r="B3326" t="n">
-        <v>3523</v>
+        <v>3474</v>
       </c>
       <c r="C3326" t="inlineStr">
         <is>
-          <t>ORLANDO RICARDO SANTOS ANDRADE</t>
+          <t>MARCOS VINICIUS GONCALVES MIRANDA</t>
         </is>
       </c>
       <c r="D3326" t="inlineStr">
         <is>
-          <t>ORLANDOR</t>
+          <t>MARCOS.VINICIUS</t>
         </is>
       </c>
     </row>
     <row r="3327">
       <c r="A3327" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3327" t="n">
-        <v>3566</v>
+        <v>3523</v>
       </c>
       <c r="C3327" t="inlineStr">
         <is>
-          <t xml:space="preserve">WESLEY HENRIQUE ALVES DOS SANTOS </t>
+          <t>ORLANDO RICARDO SANTOS ANDRADE</t>
         </is>
       </c>
       <c r="D3327" t="inlineStr">
         <is>
-          <t>W.ALVES</t>
+          <t>ORLANDOR</t>
         </is>
       </c>
     </row>
     <row r="3328">
       <c r="A3328" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3328" t="n">
-        <v>3573</v>
+        <v>3566</v>
       </c>
       <c r="C3328" t="inlineStr">
         <is>
-          <t>GABRIEL DA SILVA MENDES</t>
+          <t xml:space="preserve">WESLEY HENRIQUE ALVES DOS SANTOS </t>
         </is>
       </c>
       <c r="D3328" t="inlineStr">
         <is>
-          <t>GMENDES</t>
+          <t>W.ALVES</t>
         </is>
       </c>
     </row>
     <row r="3329">
       <c r="A3329" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3329" t="n">
-        <v>940541</v>
+        <v>3573</v>
       </c>
       <c r="C3329" t="inlineStr">
         <is>
-          <t>JOSE AMSTERDA TEIXEIRA DE MENEZES</t>
+          <t>GABRIEL DA SILVA MENDES</t>
         </is>
       </c>
       <c r="D3329" t="inlineStr">
         <is>
-          <t>AMSTERDA</t>
+          <t>GMENDES</t>
         </is>
       </c>
     </row>
     <row r="3330">
       <c r="A3330" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>99</t>
         </is>
       </c>
       <c r="B3330" t="n">
-        <v>940554</v>
+        <v>940541</v>
       </c>
       <c r="C3330" t="inlineStr">
         <is>
-          <t>ALEXANDRE ALVES DE FREITAS</t>
+          <t>JOSE AMSTERDA TEIXEIRA DE MENEZES</t>
         </is>
       </c>
       <c r="D3330" t="inlineStr">
         <is>
-          <t>ALEXANDRE</t>
+          <t>AMSTERDA</t>
         </is>
       </c>
     </row>
     <row r="3331">
       <c r="A3331" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3331" t="n">
-        <v>3402</v>
+        <v>940554</v>
       </c>
       <c r="C3331" t="inlineStr">
         <is>
-          <t xml:space="preserve">VINICIUS GUEDES DA SILVA </t>
+          <t>ALEXANDRE ALVES DE FREITAS</t>
         </is>
       </c>
       <c r="D3331" t="inlineStr">
         <is>
-          <t>GUEDES5</t>
+          <t>ALEXANDRE</t>
         </is>
       </c>
     </row>
     <row r="3332">
       <c r="A3332" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3332" t="n">
-        <v>3467</v>
+        <v>3402</v>
       </c>
       <c r="C3332" t="inlineStr">
         <is>
-          <t>CILENE FERREIRA DA SILVA</t>
+          <t xml:space="preserve">VINICIUS GUEDES DA SILVA </t>
         </is>
       </c>
       <c r="D3332" t="inlineStr">
         <is>
-          <t>CILENE</t>
+          <t>GUEDES5</t>
         </is>
       </c>
     </row>
     <row r="3333">
       <c r="A3333" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3333" t="n">
-        <v>3495</v>
+        <v>3467</v>
       </c>
       <c r="C3333" t="inlineStr">
         <is>
-          <t>LUCILENE SANTOS DE MELO DAMASCENA</t>
+          <t>CILENE FERREIRA DA SILVA</t>
         </is>
       </c>
       <c r="D3333" t="inlineStr">
         <is>
-          <t>LUCILENE21</t>
+          <t>CILENE</t>
         </is>
       </c>
     </row>
     <row r="3334">
       <c r="A3334" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3334" t="n">
-        <v>3496</v>
+        <v>3495</v>
       </c>
       <c r="C3334" t="inlineStr">
         <is>
-          <t>JOAO PEDRO HENRIQUE ALVES DE ARAUJO</t>
+          <t>LUCILENE SANTOS DE MELO DAMASCENA</t>
         </is>
       </c>
       <c r="D3334" t="inlineStr">
         <is>
-          <t>JOAO.PEDRO</t>
+          <t>LUCILENE21</t>
         </is>
       </c>
     </row>
@@ -67118,16 +67118,16 @@
         </is>
       </c>
       <c r="B3335" t="n">
-        <v>3497</v>
+        <v>3496</v>
       </c>
       <c r="C3335" t="inlineStr">
         <is>
-          <t>ORLANDO MONTEIRO DE AMORIM</t>
+          <t>JOAO PEDRO HENRIQUE ALVES DE ARAUJO</t>
         </is>
       </c>
       <c r="D3335" t="inlineStr">
         <is>
-          <t>ORLANDO</t>
+          <t>JOAO.PEDRO</t>
         </is>
       </c>
     </row>
@@ -67138,156 +67138,156 @@
         </is>
       </c>
       <c r="B3336" t="n">
-        <v>3538</v>
+        <v>3497</v>
       </c>
       <c r="C3336" t="inlineStr">
         <is>
-          <t>PAULO HENRIQUE BENTO DA SILVA</t>
+          <t>ORLANDO MONTEIRO DE AMORIM</t>
         </is>
       </c>
       <c r="D3336" t="inlineStr">
         <is>
-          <t>P.BENTO</t>
+          <t>ORLANDO</t>
         </is>
       </c>
     </row>
     <row r="3337">
       <c r="A3337" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3337" t="n">
-        <v>3577</v>
+        <v>3538</v>
       </c>
       <c r="C3337" t="inlineStr">
         <is>
-          <t>NEGOCIACAO PI</t>
+          <t>PAULO HENRIQUE BENTO DA SILVA</t>
         </is>
       </c>
       <c r="D3337" t="inlineStr">
         <is>
-          <t>NEGOCIACAOPI</t>
+          <t>P.BENTO</t>
         </is>
       </c>
     </row>
     <row r="3338">
       <c r="A3338" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3338" t="n">
-        <v>3578</v>
+        <v>3577</v>
       </c>
       <c r="C3338" t="inlineStr">
         <is>
-          <t>NEGOCIACAO MA</t>
+          <t>NEGOCIACAO PI</t>
         </is>
       </c>
       <c r="D3338" t="inlineStr">
         <is>
-          <t>NEGOCIACAOMA</t>
+          <t>NEGOCIACAOPI</t>
         </is>
       </c>
     </row>
     <row r="3339">
       <c r="A3339" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3339" t="n">
-        <v>3303</v>
+        <v>3578</v>
       </c>
       <c r="C3339" t="inlineStr">
         <is>
-          <t>DANIEL ALVES RODRIGUES</t>
+          <t>NEGOCIACAO MA</t>
         </is>
       </c>
       <c r="D3339" t="inlineStr">
         <is>
-          <t>DARODRIGUES</t>
+          <t>NEGOCIACAOMA</t>
         </is>
       </c>
     </row>
     <row r="3340">
       <c r="A3340" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3340" t="n">
-        <v>3316</v>
+        <v>3303</v>
       </c>
       <c r="C3340" t="inlineStr">
         <is>
-          <t xml:space="preserve">MARCELO PEREIRA BASTOS </t>
+          <t>DANIEL ALVES RODRIGUES</t>
         </is>
       </c>
       <c r="D3340" t="inlineStr">
         <is>
-          <t>MBASTOS</t>
+          <t>DARODRIGUES</t>
         </is>
       </c>
     </row>
     <row r="3341">
       <c r="A3341" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3341" t="n">
-        <v>3366</v>
+        <v>3316</v>
       </c>
       <c r="C3341" t="inlineStr">
         <is>
-          <t>MATEUS TEIXEIRA DA PAZ SILVA</t>
+          <t xml:space="preserve">MARCELO PEREIRA BASTOS </t>
         </is>
       </c>
       <c r="D3341" t="inlineStr">
         <is>
-          <t>PAZSILVA</t>
+          <t>MBASTOS</t>
         </is>
       </c>
     </row>
     <row r="3342">
       <c r="A3342" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3342" t="n">
-        <v>3393</v>
+        <v>3366</v>
       </c>
       <c r="C3342" t="inlineStr">
         <is>
-          <t xml:space="preserve">DAVID LUCAS RIBEIRO DOS SANTOS </t>
+          <t>MATEUS TEIXEIRA DA PAZ SILVA</t>
         </is>
       </c>
       <c r="D3342" t="inlineStr">
         <is>
-          <t>DLUCAS</t>
+          <t>PAZSILVA</t>
         </is>
       </c>
     </row>
     <row r="3343">
       <c r="A3343" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3343" t="n">
-        <v>3420</v>
+        <v>3393</v>
       </c>
       <c r="C3343" t="inlineStr">
         <is>
-          <t xml:space="preserve">CLAUDIO ROBERTO SILVA SOUZA </t>
+          <t xml:space="preserve">DAVID LUCAS RIBEIRO DOS SANTOS </t>
         </is>
       </c>
       <c r="D3343" t="inlineStr">
         <is>
-          <t>CLAUDIO21</t>
+          <t>DLUCAS</t>
         </is>
       </c>
     </row>
@@ -67298,16 +67298,16 @@
         </is>
       </c>
       <c r="B3344" t="n">
-        <v>3421</v>
+        <v>3420</v>
       </c>
       <c r="C3344" t="inlineStr">
         <is>
-          <t>WILSON PORTUGAL AZEVEDO FILHO</t>
+          <t xml:space="preserve">CLAUDIO ROBERTO SILVA SOUZA </t>
         </is>
       </c>
       <c r="D3344" t="inlineStr">
         <is>
-          <t>WILSONF</t>
+          <t>CLAUDIO21</t>
         </is>
       </c>
     </row>
@@ -67318,176 +67318,176 @@
         </is>
       </c>
       <c r="B3345" t="n">
-        <v>3439</v>
+        <v>3421</v>
       </c>
       <c r="C3345" t="inlineStr">
         <is>
-          <t>FERNANDA MASCARENHAS CEDRAZ</t>
+          <t>WILSON PORTUGAL AZEVEDO FILHO</t>
         </is>
       </c>
       <c r="D3345" t="inlineStr">
         <is>
-          <t>FERNANDAM</t>
+          <t>WILSONF</t>
         </is>
       </c>
     </row>
     <row r="3346">
       <c r="A3346" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3346" t="n">
-        <v>3455</v>
+        <v>3439</v>
       </c>
       <c r="C3346" t="inlineStr">
         <is>
-          <t xml:space="preserve">MARDONIO CUNHA BASILIO </t>
+          <t>FERNANDA MASCARENHAS CEDRAZ</t>
         </is>
       </c>
       <c r="D3346" t="inlineStr">
         <is>
-          <t>MARDONIO1</t>
+          <t>FERNANDAM</t>
         </is>
       </c>
     </row>
     <row r="3347">
       <c r="A3347" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3347" t="n">
-        <v>3508</v>
+        <v>3455</v>
       </c>
       <c r="C3347" t="inlineStr">
         <is>
-          <t>REBECA PIRES DE SOUZA MELO</t>
+          <t xml:space="preserve">MARDONIO CUNHA BASILIO </t>
         </is>
       </c>
       <c r="D3347" t="inlineStr">
         <is>
-          <t>RPMELO</t>
+          <t>MARDONIO1</t>
         </is>
       </c>
     </row>
     <row r="3348">
       <c r="A3348" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3348" t="n">
-        <v>3543</v>
+        <v>3508</v>
       </c>
       <c r="C3348" t="inlineStr">
         <is>
-          <t>JOAO GABRIEL BARBOSA FIRMINO</t>
+          <t>REBECA PIRES DE SOUZA MELO</t>
         </is>
       </c>
       <c r="D3348" t="inlineStr">
         <is>
-          <t>JOAOG</t>
+          <t>RPMELO</t>
         </is>
       </c>
     </row>
     <row r="3349">
       <c r="A3349" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3349" t="n">
-        <v>3580</v>
+        <v>3543</v>
       </c>
       <c r="C3349" t="inlineStr">
         <is>
-          <t>ALEXANDRE MARTINS CHAVES</t>
+          <t>JOAO GABRIEL BARBOSA FIRMINO</t>
         </is>
       </c>
       <c r="D3349" t="inlineStr">
         <is>
-          <t>MARTINS</t>
+          <t>JOAOG</t>
         </is>
       </c>
     </row>
     <row r="3350">
       <c r="A3350" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3350" t="n">
-        <v>3351</v>
+        <v>3580</v>
       </c>
       <c r="C3350" t="inlineStr">
         <is>
-          <t>HAWLLYSON DA SILVA COUTINHO</t>
+          <t>ALEXANDRE MARTINS CHAVES</t>
         </is>
       </c>
       <c r="D3350" t="inlineStr">
         <is>
-          <t>HCOUTINHO</t>
+          <t>MARTINS</t>
         </is>
       </c>
     </row>
     <row r="3351">
       <c r="A3351" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3351" t="n">
-        <v>940553</v>
+        <v>3351</v>
       </c>
       <c r="C3351" t="inlineStr">
         <is>
-          <t>LUTY TRANSPORTES- BA</t>
+          <t>HAWLLYSON DA SILVA COUTINHO</t>
         </is>
       </c>
       <c r="D3351" t="inlineStr">
         <is>
-          <t>LUTY TRANSPORTE</t>
+          <t>HCOUTINHO</t>
         </is>
       </c>
     </row>
     <row r="3352">
       <c r="A3352" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3352" t="n">
-        <v>3391</v>
+        <v>940553</v>
       </c>
       <c r="C3352" t="inlineStr">
         <is>
-          <t xml:space="preserve">NIKSON DA SILVA ALVES </t>
+          <t>LUTY TRANSPORTES- BA</t>
         </is>
       </c>
       <c r="D3352" t="inlineStr">
         <is>
-          <t>NIKSON</t>
+          <t>LUTY TRANSPORTE</t>
         </is>
       </c>
     </row>
     <row r="3353">
       <c r="A3353" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3353" t="n">
-        <v>3397</v>
+        <v>3391</v>
       </c>
       <c r="C3353" t="inlineStr">
         <is>
-          <t>EDILANE MENESES BALTAZAR</t>
+          <t xml:space="preserve">NIKSON DA SILVA ALVES </t>
         </is>
       </c>
       <c r="D3353" t="inlineStr">
         <is>
-          <t>EDILANE</t>
+          <t>NIKSON</t>
         </is>
       </c>
     </row>
@@ -67498,56 +67498,56 @@
         </is>
       </c>
       <c r="B3354" t="n">
-        <v>3398</v>
+        <v>3397</v>
       </c>
       <c r="C3354" t="inlineStr">
         <is>
-          <t>LUANA MARIA ROSIO DA SILVA</t>
+          <t>EDILANE MENESES BALTAZAR</t>
         </is>
       </c>
       <c r="D3354" t="inlineStr">
         <is>
-          <t>LUMARIA</t>
+          <t>EDILANE</t>
         </is>
       </c>
     </row>
     <row r="3355">
       <c r="A3355" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3355" t="n">
-        <v>3400</v>
+        <v>3398</v>
       </c>
       <c r="C3355" t="inlineStr">
         <is>
-          <t>ELILTON PINTO ROMEU</t>
+          <t>LUANA MARIA ROSIO DA SILVA</t>
         </is>
       </c>
       <c r="D3355" t="inlineStr">
         <is>
-          <t>ELILTON</t>
+          <t>LUMARIA</t>
         </is>
       </c>
     </row>
     <row r="3356">
       <c r="A3356" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3356" t="n">
-        <v>3406</v>
+        <v>3400</v>
       </c>
       <c r="C3356" t="inlineStr">
         <is>
-          <t>CONEXAO ALDA</t>
+          <t>ELILTON PINTO ROMEU</t>
         </is>
       </c>
       <c r="D3356" t="inlineStr">
         <is>
-          <t>CONEXAOALDA</t>
+          <t>ELILTON</t>
         </is>
       </c>
     </row>
@@ -67558,176 +67558,176 @@
         </is>
       </c>
       <c r="B3357" t="n">
-        <v>3407</v>
+        <v>3406</v>
       </c>
       <c r="C3357" t="inlineStr">
         <is>
-          <t>CONEXAO IRACEMA</t>
+          <t>CONEXAO ALDA</t>
         </is>
       </c>
       <c r="D3357" t="inlineStr">
         <is>
-          <t>CONEXAOIRACEMA</t>
+          <t>CONEXAOALDA</t>
         </is>
       </c>
     </row>
     <row r="3358">
       <c r="A3358" t="inlineStr">
         <is>
-          <t>9999</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3358" t="n">
-        <v>3408</v>
+        <v>3407</v>
       </c>
       <c r="C3358" t="inlineStr">
         <is>
-          <t>CONEXAO TAMILES</t>
+          <t>CONEXAO IRACEMA</t>
         </is>
       </c>
       <c r="D3358" t="inlineStr">
         <is>
-          <t>CONEXAOTAMILES</t>
+          <t>CONEXAOIRACEMA</t>
         </is>
       </c>
     </row>
     <row r="3359">
       <c r="A3359" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>9999</t>
         </is>
       </c>
       <c r="B3359" t="n">
-        <v>3414</v>
+        <v>3408</v>
       </c>
       <c r="C3359" t="inlineStr">
         <is>
-          <t>CONEXAO ADM PI MA</t>
+          <t>CONEXAO TAMILES</t>
         </is>
       </c>
       <c r="D3359" t="inlineStr">
         <is>
-          <t>CONEXAOPIMA</t>
+          <t>CONEXAOTAMILES</t>
         </is>
       </c>
     </row>
     <row r="3360">
       <c r="A3360" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3360" t="n">
-        <v>3524</v>
+        <v>3414</v>
       </c>
       <c r="C3360" t="inlineStr">
         <is>
-          <t>LUIS FELIPE DA SILVA SOUSA</t>
+          <t>CONEXAO ADM PI MA</t>
         </is>
       </c>
       <c r="D3360" t="inlineStr">
         <is>
-          <t>L.FELIPE</t>
+          <t>CONEXAOPIMA</t>
         </is>
       </c>
     </row>
     <row r="3361">
       <c r="A3361" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3361" t="n">
-        <v>3531</v>
+        <v>3524</v>
       </c>
       <c r="C3361" t="inlineStr">
         <is>
-          <t>LEICIANE COELHO SILVA</t>
+          <t>LUIS FELIPE DA SILVA SOUSA</t>
         </is>
       </c>
       <c r="D3361" t="inlineStr">
         <is>
-          <t>LEI.SILVA</t>
+          <t>L.FELIPE</t>
         </is>
       </c>
     </row>
     <row r="3362">
       <c r="A3362" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3362" t="n">
-        <v>3550</v>
+        <v>3531</v>
       </c>
       <c r="C3362" t="inlineStr">
         <is>
-          <t>IARGO GABRIEL SANTOS DE OLIVEIRA</t>
+          <t>LEICIANE COELHO SILVA</t>
         </is>
       </c>
       <c r="D3362" t="inlineStr">
         <is>
-          <t>IARGOG</t>
+          <t>LEI.SILVA</t>
         </is>
       </c>
     </row>
     <row r="3363">
       <c r="A3363" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3363" t="n">
-        <v>940567</v>
+        <v>3550</v>
       </c>
       <c r="C3363" t="inlineStr">
         <is>
-          <t>MS CARGAS E TRANSPORTES</t>
+          <t>IARGO GABRIEL SANTOS DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D3363" t="inlineStr">
         <is>
-          <t>ALAN BARBOSA</t>
+          <t>IARGOG</t>
         </is>
       </c>
     </row>
     <row r="3364">
       <c r="A3364" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3364" t="n">
-        <v>3560</v>
+        <v>940567</v>
       </c>
       <c r="C3364" t="inlineStr">
         <is>
-          <t>MARIA EDUARDA MELO DOS SANTOS</t>
+          <t>MS CARGAS E TRANSPORTES</t>
         </is>
       </c>
       <c r="D3364" t="inlineStr">
         <is>
-          <t>EDU.MELO</t>
+          <t>ALAN BARBOSA</t>
         </is>
       </c>
     </row>
     <row r="3365">
       <c r="A3365" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3365" t="n">
-        <v>3355</v>
+        <v>3560</v>
       </c>
       <c r="C3365" t="inlineStr">
         <is>
-          <t>HUGO MATHEUS DA COSTA FEITOSA</t>
+          <t>MARIA EDUARDA MELO DOS SANTOS</t>
         </is>
       </c>
       <c r="D3365" t="inlineStr">
         <is>
-          <t>HMFEITOSA</t>
+          <t>EDU.MELO</t>
         </is>
       </c>
     </row>
@@ -67738,96 +67738,96 @@
         </is>
       </c>
       <c r="B3366" t="n">
-        <v>3356</v>
+        <v>3355</v>
       </c>
       <c r="C3366" t="inlineStr">
         <is>
-          <t>BRENDA LIMA DE OLIVEIRA CUNHA</t>
+          <t>HUGO MATHEUS DA COSTA FEITOSA</t>
         </is>
       </c>
       <c r="D3366" t="inlineStr">
         <is>
-          <t>BLCUNHA</t>
+          <t>HMFEITOSA</t>
         </is>
       </c>
     </row>
     <row r="3367">
       <c r="A3367" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3367" t="n">
-        <v>3361</v>
+        <v>3356</v>
       </c>
       <c r="C3367" t="inlineStr">
         <is>
-          <t>WLADIA DE ARAUJO BASTOS</t>
+          <t>BRENDA LIMA DE OLIVEIRA CUNHA</t>
         </is>
       </c>
       <c r="D3367" t="inlineStr">
         <is>
-          <t>WABASTOS</t>
+          <t>BLCUNHA</t>
         </is>
       </c>
     </row>
     <row r="3368">
       <c r="A3368" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3368" t="n">
-        <v>3362</v>
+        <v>3361</v>
       </c>
       <c r="C3368" t="inlineStr">
         <is>
-          <t>CARLOS HENRIQUE MELO DA SILVA</t>
+          <t>WLADIA DE ARAUJO BASTOS</t>
         </is>
       </c>
       <c r="D3368" t="inlineStr">
         <is>
-          <t>CHMELO</t>
+          <t>WABASTOS</t>
         </is>
       </c>
     </row>
     <row r="3369">
       <c r="A3369" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3369" t="n">
-        <v>3375</v>
+        <v>3362</v>
       </c>
       <c r="C3369" t="inlineStr">
         <is>
-          <t>AFONSO DE SOUSA RAMOS FILHO</t>
+          <t>CARLOS HENRIQUE MELO DA SILVA</t>
         </is>
       </c>
       <c r="D3369" t="inlineStr">
         <is>
-          <t>AFILHO</t>
+          <t>CHMELO</t>
         </is>
       </c>
     </row>
     <row r="3370">
       <c r="A3370" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3370" t="n">
-        <v>3404</v>
+        <v>3375</v>
       </c>
       <c r="C3370" t="inlineStr">
         <is>
-          <t>NOVATO 4 COM</t>
+          <t>AFONSO DE SOUSA RAMOS FILHO</t>
         </is>
       </c>
       <c r="D3370" t="inlineStr">
         <is>
-          <t>NOVATO4COM</t>
+          <t>AFILHO</t>
         </is>
       </c>
     </row>
@@ -67838,176 +67838,176 @@
         </is>
       </c>
       <c r="B3371" t="n">
-        <v>3405</v>
+        <v>3404</v>
       </c>
       <c r="C3371" t="inlineStr">
         <is>
-          <t>NOVATO 5 COM</t>
+          <t>NOVATO 4 COM</t>
         </is>
       </c>
       <c r="D3371" t="inlineStr">
         <is>
-          <t>NOVATO5COM</t>
+          <t>NOVATO4COM</t>
         </is>
       </c>
     </row>
     <row r="3372">
       <c r="A3372" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3372" t="n">
-        <v>3447</v>
+        <v>3405</v>
       </c>
       <c r="C3372" t="inlineStr">
         <is>
-          <t>RAYSSA KEYCE LINHARES AQUINO</t>
+          <t>NOVATO 5 COM</t>
         </is>
       </c>
       <c r="D3372" t="inlineStr">
         <is>
-          <t>RAYSSAK</t>
+          <t>NOVATO5COM</t>
         </is>
       </c>
     </row>
     <row r="3373">
       <c r="A3373" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3373" t="n">
-        <v>940559</v>
+        <v>3447</v>
       </c>
       <c r="C3373" t="inlineStr">
         <is>
-          <t>WALLEF DE OLIVEIRA</t>
+          <t>RAYSSA KEYCE LINHARES AQUINO</t>
         </is>
       </c>
       <c r="D3373" t="inlineStr">
         <is>
-          <t>WALLEF</t>
+          <t>RAYSSAK</t>
         </is>
       </c>
     </row>
     <row r="3374">
       <c r="A3374" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>99</t>
         </is>
       </c>
       <c r="B3374" t="n">
-        <v>3489</v>
+        <v>940559</v>
       </c>
       <c r="C3374" t="inlineStr">
         <is>
-          <t>MARCELA KARINA PEREIRA VELOSO</t>
+          <t>WALLEF DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D3374" t="inlineStr">
         <is>
-          <t>MKARINA</t>
+          <t>WALLEF</t>
         </is>
       </c>
     </row>
     <row r="3375">
       <c r="A3375" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3375" t="n">
-        <v>3490</v>
+        <v>3489</v>
       </c>
       <c r="C3375" t="inlineStr">
         <is>
-          <t>JOSE MAILSON GOMES NUNES</t>
+          <t>MARCELA KARINA PEREIRA VELOSO</t>
         </is>
       </c>
       <c r="D3375" t="inlineStr">
         <is>
-          <t>J.MAILSON</t>
+          <t>MKARINA</t>
         </is>
       </c>
     </row>
     <row r="3376">
       <c r="A3376" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3376" t="n">
-        <v>3537</v>
+        <v>3490</v>
       </c>
       <c r="C3376" t="inlineStr">
         <is>
-          <t>ALDAIR PEDRO DA SILVA</t>
+          <t>JOSE MAILSON GOMES NUNES</t>
         </is>
       </c>
       <c r="D3376" t="inlineStr">
         <is>
-          <t>A.PEDRO</t>
+          <t>J.MAILSON</t>
         </is>
       </c>
     </row>
     <row r="3377">
       <c r="A3377" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3377" t="n">
-        <v>3549</v>
+        <v>3537</v>
       </c>
       <c r="C3377" t="inlineStr">
         <is>
-          <t xml:space="preserve">FERNANDA CAROLINE E CESAR SOUSA </t>
+          <t>ALDAIR PEDRO DA SILVA</t>
         </is>
       </c>
       <c r="D3377" t="inlineStr">
         <is>
-          <t>FCAROLINE</t>
+          <t>A.PEDRO</t>
         </is>
       </c>
     </row>
     <row r="3378">
       <c r="A3378" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3378" t="n">
-        <v>3337</v>
+        <v>3549</v>
       </c>
       <c r="C3378" t="inlineStr">
         <is>
-          <t>WESLEY FONTES DE ALMEIDA</t>
+          <t xml:space="preserve">FERNANDA CAROLINE E CESAR SOUSA </t>
         </is>
       </c>
       <c r="D3378" t="inlineStr">
         <is>
-          <t>WFALMEIDA</t>
+          <t>FCAROLINE</t>
         </is>
       </c>
     </row>
     <row r="3379">
       <c r="A3379" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3379" t="n">
-        <v>3338</v>
+        <v>3581</v>
       </c>
       <c r="C3379" t="inlineStr">
         <is>
-          <t>FRANCISCA SAMARA MENDES DE OLIVEIRA C</t>
+          <t xml:space="preserve">VALQUIRIO OLIVEIRA SOUSA </t>
         </is>
       </c>
       <c r="D3379" t="inlineStr">
         <is>
-          <t>FSCUNHA</t>
+          <t>VALQUIRIO</t>
         </is>
       </c>
     </row>
@@ -68018,216 +68018,216 @@
         </is>
       </c>
       <c r="B3380" t="n">
-        <v>3339</v>
+        <v>3337</v>
       </c>
       <c r="C3380" t="inlineStr">
         <is>
-          <t>MAYARA THALYA DIAS DE ANDRADE</t>
+          <t>WESLEY FONTES DE ALMEIDA</t>
         </is>
       </c>
       <c r="D3380" t="inlineStr">
         <is>
-          <t>MTANDRADE</t>
+          <t>WFALMEIDA</t>
         </is>
       </c>
     </row>
     <row r="3381">
       <c r="A3381" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3381" t="n">
-        <v>3359</v>
+        <v>3338</v>
       </c>
       <c r="C3381" t="inlineStr">
         <is>
-          <t xml:space="preserve">EVANESSA DA SILVA E SILVA </t>
+          <t>FRANCISCA SAMARA MENDES DE OLIVEIRA C</t>
         </is>
       </c>
       <c r="D3381" t="inlineStr">
         <is>
-          <t>EVANESSAS</t>
+          <t>FSCUNHA</t>
         </is>
       </c>
     </row>
     <row r="3382">
       <c r="A3382" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3382" t="n">
-        <v>3360</v>
+        <v>3339</v>
       </c>
       <c r="C3382" t="inlineStr">
         <is>
-          <t>THIAGO DE CARVALHO ARAUJO</t>
+          <t>MAYARA THALYA DIAS DE ANDRADE</t>
         </is>
       </c>
       <c r="D3382" t="inlineStr">
         <is>
-          <t>TCARAUJO</t>
+          <t>MTANDRADE</t>
         </is>
       </c>
     </row>
     <row r="3383">
       <c r="A3383" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3383" t="n">
-        <v>3481</v>
+        <v>3359</v>
       </c>
       <c r="C3383" t="inlineStr">
         <is>
-          <t xml:space="preserve">EDSON DA PAZ LIMA </t>
+          <t xml:space="preserve">EVANESSA DA SILVA E SILVA </t>
         </is>
       </c>
       <c r="D3383" t="inlineStr">
         <is>
-          <t>EDPAZ</t>
+          <t>EVANESSAS</t>
         </is>
       </c>
     </row>
     <row r="3384">
       <c r="A3384" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3384" t="n">
-        <v>3494</v>
+        <v>3360</v>
       </c>
       <c r="C3384" t="inlineStr">
         <is>
-          <t>ANTONIO CRISTINA BRITO GOMES</t>
+          <t>THIAGO DE CARVALHO ARAUJO</t>
         </is>
       </c>
       <c r="D3384" t="inlineStr">
         <is>
-          <t>CRIS.GOMES</t>
+          <t>TCARAUJO</t>
         </is>
       </c>
     </row>
     <row r="3385">
       <c r="A3385" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3385" t="n">
-        <v>3498</v>
+        <v>3481</v>
       </c>
       <c r="C3385" t="inlineStr">
         <is>
-          <t>SILVESTRA COSTA NUNES</t>
+          <t xml:space="preserve">EDSON DA PAZ LIMA </t>
         </is>
       </c>
       <c r="D3385" t="inlineStr">
         <is>
-          <t>SCNUNES</t>
+          <t>EDPAZ</t>
         </is>
       </c>
     </row>
     <row r="3386">
       <c r="A3386" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3386" t="n">
-        <v>940562</v>
+        <v>3494</v>
       </c>
       <c r="C3386" t="inlineStr">
         <is>
-          <t>FRANCISCO DAVID ASSUNCAO ALVES</t>
+          <t>ANTONIO CRISTINA BRITO GOMES</t>
         </is>
       </c>
       <c r="D3386" t="inlineStr">
         <is>
-          <t>ASSUNÇÃO</t>
+          <t>CRIS.GOMES</t>
         </is>
       </c>
     </row>
     <row r="3387">
       <c r="A3387" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3387" t="n">
-        <v>3513</v>
+        <v>3498</v>
       </c>
       <c r="C3387" t="inlineStr">
         <is>
-          <t>RENARA ANDRADE MATIAS</t>
+          <t>SILVESTRA COSTA NUNES</t>
         </is>
       </c>
       <c r="D3387" t="inlineStr">
         <is>
-          <t>R.ANDRADE</t>
+          <t>SCNUNES</t>
         </is>
       </c>
     </row>
     <row r="3388">
       <c r="A3388" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>99</t>
         </is>
       </c>
       <c r="B3388" t="n">
-        <v>3275</v>
+        <v>940562</v>
       </c>
       <c r="C3388" t="inlineStr">
         <is>
-          <t>MARIA APARECIDA COELHO SILVA</t>
+          <t>FRANCISCO DAVID ASSUNCAO ALVES</t>
         </is>
       </c>
       <c r="D3388" t="inlineStr">
         <is>
-          <t>MCOELHO</t>
+          <t>ASSUNÇÃO</t>
         </is>
       </c>
     </row>
     <row r="3389">
       <c r="A3389" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3389" t="n">
-        <v>3276</v>
+        <v>3513</v>
       </c>
       <c r="C3389" t="inlineStr">
         <is>
-          <t xml:space="preserve">PEROLA DE JESUS AMORIM SOUSA </t>
+          <t>RENARA ANDRADE MATIAS</t>
         </is>
       </c>
       <c r="D3389" t="inlineStr">
         <is>
-          <t>PJESUS</t>
+          <t>R.ANDRADE</t>
         </is>
       </c>
     </row>
     <row r="3390">
       <c r="A3390" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3390" t="n">
-        <v>3526</v>
+        <v>3275</v>
       </c>
       <c r="C3390" t="inlineStr">
         <is>
-          <t>JOYCE NAZARE CORREA</t>
+          <t>MARIA APARECIDA COELHO SILVA</t>
         </is>
       </c>
       <c r="D3390" t="inlineStr">
         <is>
-          <t>J.NAZARE</t>
+          <t>MCOELHO</t>
         </is>
       </c>
     </row>
@@ -68238,216 +68238,216 @@
         </is>
       </c>
       <c r="B3391" t="n">
-        <v>3527</v>
+        <v>3276</v>
       </c>
       <c r="C3391" t="inlineStr">
         <is>
-          <t>GILVANA DA SILVA MONTELES</t>
+          <t xml:space="preserve">PEROLA DE JESUS AMORIM SOUSA </t>
         </is>
       </c>
       <c r="D3391" t="inlineStr">
         <is>
-          <t>GIL.SILVA</t>
+          <t>PJESUS</t>
         </is>
       </c>
     </row>
     <row r="3392">
       <c r="A3392" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3392" t="n">
-        <v>3548</v>
+        <v>3526</v>
       </c>
       <c r="C3392" t="inlineStr">
         <is>
-          <t>JAMILLY MARIA HENRIQUE ARAUJO</t>
+          <t>JOYCE NAZARE CORREA</t>
         </is>
       </c>
       <c r="D3392" t="inlineStr">
         <is>
-          <t>JAMILLY</t>
+          <t>J.NAZARE</t>
         </is>
       </c>
     </row>
     <row r="3393">
       <c r="A3393" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3393" t="n">
-        <v>3551</v>
+        <v>3527</v>
       </c>
       <c r="C3393" t="inlineStr">
         <is>
-          <t xml:space="preserve">VITOR MANOEL DA SILVA BARBOSA </t>
+          <t>GILVANA DA SILVA MONTELES</t>
         </is>
       </c>
       <c r="D3393" t="inlineStr">
         <is>
-          <t>VMANOEL</t>
+          <t>GIL.SILVA</t>
         </is>
       </c>
     </row>
     <row r="3394">
       <c r="A3394" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3394" t="n">
-        <v>940525</v>
+        <v>3548</v>
       </c>
       <c r="C3394" t="inlineStr">
         <is>
-          <t>SANDUWELLINGTON</t>
+          <t>JAMILLY MARIA HENRIQUE ARAUJO</t>
         </is>
       </c>
       <c r="D3394" t="inlineStr">
         <is>
-          <t>SANDUWELLINGTON</t>
+          <t>JAMILLY</t>
         </is>
       </c>
     </row>
     <row r="3395">
       <c r="A3395" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3395" t="n">
-        <v>3369</v>
+        <v>3551</v>
       </c>
       <c r="C3395" t="inlineStr">
         <is>
-          <t xml:space="preserve">PRISCILA DOS SANTOS LOPES </t>
+          <t xml:space="preserve">VITOR MANOEL DA SILVA BARBOSA </t>
         </is>
       </c>
       <c r="D3395" t="inlineStr">
         <is>
-          <t>PSLOPES</t>
+          <t>VMANOEL</t>
         </is>
       </c>
     </row>
     <row r="3396">
       <c r="A3396" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3396" t="n">
-        <v>3433</v>
+        <v>940525</v>
       </c>
       <c r="C3396" t="inlineStr">
         <is>
-          <t>BRUNO NUNES CRUZ</t>
+          <t>SANDUWELLINGTON</t>
         </is>
       </c>
       <c r="D3396" t="inlineStr">
         <is>
-          <t>BRUNOCRUZ</t>
+          <t>SANDUWELLINGTON</t>
         </is>
       </c>
     </row>
     <row r="3397">
       <c r="A3397" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3397" t="n">
-        <v>3434</v>
+        <v>3369</v>
       </c>
       <c r="C3397" t="inlineStr">
         <is>
-          <t>ANA TERCIA DE LIMA SA CARVALHO SERAFIM</t>
+          <t xml:space="preserve">PRISCILA DOS SANTOS LOPES </t>
         </is>
       </c>
       <c r="D3397" t="inlineStr">
         <is>
-          <t>ANATER</t>
+          <t>PSLOPES</t>
         </is>
       </c>
     </row>
     <row r="3398">
       <c r="A3398" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3398" t="n">
-        <v>3502</v>
+        <v>3433</v>
       </c>
       <c r="C3398" t="inlineStr">
         <is>
-          <t>LUIZ FELIPE MACHADO BARRETO</t>
+          <t>BRUNO NUNES CRUZ</t>
         </is>
       </c>
       <c r="D3398" t="inlineStr">
         <is>
-          <t>LUIZ.FELIPE</t>
+          <t>BRUNOCRUZ</t>
         </is>
       </c>
     </row>
     <row r="3399">
       <c r="A3399" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3399" t="n">
-        <v>3503</v>
+        <v>3434</v>
       </c>
       <c r="C3399" t="inlineStr">
         <is>
-          <t>FABIO OLIVEIRA SILVA</t>
+          <t>ANA TERCIA DE LIMA SA CARVALHO SERAFIM</t>
         </is>
       </c>
       <c r="D3399" t="inlineStr">
         <is>
-          <t>FOSILVA</t>
+          <t>ANATER</t>
         </is>
       </c>
     </row>
     <row r="3400">
       <c r="A3400" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3400" t="n">
-        <v>3554</v>
+        <v>3502</v>
       </c>
       <c r="C3400" t="inlineStr">
         <is>
-          <t xml:space="preserve">MANOEL RIBEIRO DE SOUZA JUNIOR </t>
+          <t>LUIZ FELIPE MACHADO BARRETO</t>
         </is>
       </c>
       <c r="D3400" t="inlineStr">
         <is>
-          <t>MRJUNIOR</t>
+          <t>LUIZ.FELIPE</t>
         </is>
       </c>
     </row>
     <row r="3401">
       <c r="A3401" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3401" t="n">
-        <v>3568</v>
+        <v>3503</v>
       </c>
       <c r="C3401" t="inlineStr">
         <is>
-          <t xml:space="preserve">ANGELICA TORRES DA SILVA </t>
+          <t>FABIO OLIVEIRA SILVA</t>
         </is>
       </c>
       <c r="D3401" t="inlineStr">
         <is>
-          <t>ANGEL.TORRES</t>
+          <t>FOSILVA</t>
         </is>
       </c>
     </row>
@@ -68458,136 +68458,136 @@
         </is>
       </c>
       <c r="B3402" t="n">
-        <v>3569</v>
+        <v>3554</v>
       </c>
       <c r="C3402" t="inlineStr">
         <is>
-          <t>LORENA DE LIMA MATOS</t>
+          <t xml:space="preserve">MANOEL RIBEIRO DE SOUZA JUNIOR </t>
         </is>
       </c>
       <c r="D3402" t="inlineStr">
         <is>
-          <t>LORE.LIMA</t>
+          <t>MRJUNIOR</t>
         </is>
       </c>
     </row>
     <row r="3403">
       <c r="A3403" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3403" t="n">
-        <v>3576</v>
+        <v>3568</v>
       </c>
       <c r="C3403" t="inlineStr">
         <is>
-          <t>ANA BEATRIZ PARENTE CAVALCANTE</t>
+          <t xml:space="preserve">ANGELICA TORRES DA SILVA </t>
         </is>
       </c>
       <c r="D3403" t="inlineStr">
         <is>
-          <t>A.BEATRIZ</t>
+          <t>ANGEL.TORRES</t>
         </is>
       </c>
     </row>
     <row r="3404">
       <c r="A3404" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3404" t="n">
-        <v>940549</v>
+        <v>3569</v>
       </c>
       <c r="C3404" t="inlineStr">
         <is>
-          <t>EDILSON ARAUJO - FL9</t>
+          <t>LORENA DE LIMA MATOS</t>
         </is>
       </c>
       <c r="D3404" t="inlineStr">
         <is>
-          <t>EDILSON</t>
+          <t>LORE.LIMA</t>
         </is>
       </c>
     </row>
     <row r="3405">
       <c r="A3405" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3405" t="n">
-        <v>3470</v>
+        <v>3576</v>
       </c>
       <c r="C3405" t="inlineStr">
         <is>
-          <t>DEBORA ALVES CARVALHO</t>
+          <t>ANA BEATRIZ PARENTE CAVALCANTE</t>
         </is>
       </c>
       <c r="D3405" t="inlineStr">
         <is>
-          <t>DEBORA.ALVES</t>
+          <t>A.BEATRIZ</t>
         </is>
       </c>
     </row>
     <row r="3406">
       <c r="A3406" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3406" t="n">
-        <v>3510</v>
+        <v>940549</v>
       </c>
       <c r="C3406" t="inlineStr">
         <is>
-          <t>CAMILA RODIGUES PINTO</t>
+          <t>EDILSON ARAUJO - FL9</t>
         </is>
       </c>
       <c r="D3406" t="inlineStr">
         <is>
-          <t>MILA.PINTO</t>
+          <t>EDILSON</t>
         </is>
       </c>
     </row>
     <row r="3407">
       <c r="A3407" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3407" t="n">
-        <v>3511</v>
+        <v>3470</v>
       </c>
       <c r="C3407" t="inlineStr">
         <is>
-          <t>JORGE HENRIQUE DOS SANTOS RODRIGUES</t>
+          <t>DEBORA ALVES CARVALHO</t>
         </is>
       </c>
       <c r="D3407" t="inlineStr">
         <is>
-          <t>J.HENRIQUE</t>
+          <t>DEBORA.ALVES</t>
         </is>
       </c>
     </row>
     <row r="3408">
       <c r="A3408" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3408" t="n">
-        <v>3561</v>
+        <v>3510</v>
       </c>
       <c r="C3408" t="inlineStr">
         <is>
-          <t>RONARIA PATRICIA VILARINDO DE ALMEIDA</t>
+          <t>CAMILA RODIGUES PINTO</t>
         </is>
       </c>
       <c r="D3408" t="inlineStr">
         <is>
-          <t>RPATRICIA</t>
+          <t>MILA.PINTO</t>
         </is>
       </c>
     </row>
@@ -68598,156 +68598,156 @@
         </is>
       </c>
       <c r="B3409" t="n">
-        <v>3562</v>
+        <v>3511</v>
       </c>
       <c r="C3409" t="inlineStr">
         <is>
-          <t>LETICIA MARIA BENTO NOGUEIRA</t>
+          <t>JORGE HENRIQUE DOS SANTOS RODRIGUES</t>
         </is>
       </c>
       <c r="D3409" t="inlineStr">
         <is>
-          <t>LBENTO</t>
+          <t>J.HENRIQUE</t>
         </is>
       </c>
     </row>
     <row r="3410">
       <c r="A3410" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3410" t="n">
-        <v>3270</v>
+        <v>3561</v>
       </c>
       <c r="C3410" t="inlineStr">
         <is>
-          <t>ITANA NASCIMENTO SIMOES</t>
+          <t>RONARIA PATRICIA VILARINDO DE ALMEIDA</t>
         </is>
       </c>
       <c r="D3410" t="inlineStr">
         <is>
-          <t>ISIMOES</t>
+          <t>RPATRICIA</t>
         </is>
       </c>
     </row>
     <row r="3411">
       <c r="A3411" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3411" t="n">
-        <v>3318</v>
+        <v>3562</v>
       </c>
       <c r="C3411" t="inlineStr">
         <is>
-          <t>LUAN MONTEIRO COSTA</t>
+          <t>LETICIA MARIA BENTO NOGUEIRA</t>
         </is>
       </c>
       <c r="D3411" t="inlineStr">
         <is>
-          <t>LMONTEIRO</t>
+          <t>LBENTO</t>
         </is>
       </c>
     </row>
     <row r="3412">
       <c r="A3412" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3412" t="n">
-        <v>3319</v>
+        <v>3270</v>
       </c>
       <c r="C3412" t="inlineStr">
         <is>
-          <t>MARIANA MACEDA DOS SANTOS</t>
+          <t>ITANA NASCIMENTO SIMOES</t>
         </is>
       </c>
       <c r="D3412" t="inlineStr">
         <is>
-          <t>MMACEDA</t>
+          <t>ISIMOES</t>
         </is>
       </c>
     </row>
     <row r="3413">
       <c r="A3413" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3413" t="n">
-        <v>3389</v>
+        <v>3318</v>
       </c>
       <c r="C3413" t="inlineStr">
         <is>
-          <t>TAMILES DE SANTANA AMORIM BISPO</t>
+          <t>LUAN MONTEIRO COSTA</t>
         </is>
       </c>
       <c r="D3413" t="inlineStr">
         <is>
-          <t>TAMILES</t>
+          <t>LMONTEIRO</t>
         </is>
       </c>
     </row>
     <row r="3414">
       <c r="A3414" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3414" t="n">
-        <v>3390</v>
+        <v>3319</v>
       </c>
       <c r="C3414" t="inlineStr">
         <is>
-          <t>IRACEMA DE ALMEIDA MOURA</t>
+          <t>MARIANA MACEDA DOS SANTOS</t>
         </is>
       </c>
       <c r="D3414" t="inlineStr">
         <is>
-          <t>IRACEMA</t>
+          <t>MMACEDA</t>
         </is>
       </c>
     </row>
     <row r="3415">
       <c r="A3415" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3415" t="n">
-        <v>3575</v>
+        <v>3389</v>
       </c>
       <c r="C3415" t="inlineStr">
         <is>
-          <t>SAMARA ALVES DA SILVA</t>
+          <t>TAMILES DE SANTANA AMORIM BISPO</t>
         </is>
       </c>
       <c r="D3415" t="inlineStr">
         <is>
-          <t>S.ALVES</t>
+          <t>TAMILES</t>
         </is>
       </c>
     </row>
     <row r="3416">
       <c r="A3416" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3416" t="n">
-        <v>3286</v>
+        <v>3390</v>
       </c>
       <c r="C3416" t="inlineStr">
         <is>
-          <t>VALERIA MAIA DA SILVA</t>
+          <t>IRACEMA DE ALMEIDA MOURA</t>
         </is>
       </c>
       <c r="D3416" t="inlineStr">
         <is>
-          <t>VMAIAS</t>
+          <t>IRACEMA</t>
         </is>
       </c>
     </row>
@@ -68758,196 +68758,196 @@
         </is>
       </c>
       <c r="B3417" t="n">
-        <v>3287</v>
+        <v>3575</v>
       </c>
       <c r="C3417" t="inlineStr">
         <is>
-          <t>ERIVELTON DA SILVA OLIVEIRA</t>
+          <t>SAMARA ALVES DA SILVA</t>
         </is>
       </c>
       <c r="D3417" t="inlineStr">
         <is>
-          <t>ESOLIVEIRA</t>
+          <t>S.ALVES</t>
         </is>
       </c>
     </row>
     <row r="3418">
       <c r="A3418" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3418" t="n">
-        <v>3307</v>
+        <v>3286</v>
       </c>
       <c r="C3418" t="inlineStr">
         <is>
-          <t>ADRIEL XERES BARROS MARTINS</t>
+          <t>VALERIA MAIA DA SILVA</t>
         </is>
       </c>
       <c r="D3418" t="inlineStr">
         <is>
-          <t>AXERES</t>
+          <t>VMAIAS</t>
         </is>
       </c>
     </row>
     <row r="3419">
       <c r="A3419" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3419" t="n">
-        <v>3308</v>
+        <v>3287</v>
       </c>
       <c r="C3419" t="inlineStr">
         <is>
-          <t>ELKZIEL JUVINO DA SILVA</t>
+          <t>ERIVELTON DA SILVA OLIVEIRA</t>
         </is>
       </c>
       <c r="D3419" t="inlineStr">
         <is>
-          <t>EJUVINO</t>
+          <t>ESOLIVEIRA</t>
         </is>
       </c>
     </row>
     <row r="3420">
       <c r="A3420" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3420" t="n">
-        <v>940539</v>
+        <v>3307</v>
       </c>
       <c r="C3420" t="inlineStr">
         <is>
-          <t>EDSON ARAUJO - FL9</t>
+          <t>ADRIEL XERES BARROS MARTINS</t>
         </is>
       </c>
       <c r="D3420" t="inlineStr">
         <is>
-          <t>EDS</t>
+          <t>AXERES</t>
         </is>
       </c>
     </row>
     <row r="3421">
       <c r="A3421" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3421" t="n">
-        <v>940540</v>
+        <v>3308</v>
       </c>
       <c r="C3421" t="inlineStr">
         <is>
-          <t>EDSON ARAUJO - FL8</t>
+          <t>ELKZIEL JUVINO DA SILVA</t>
         </is>
       </c>
       <c r="D3421" t="inlineStr">
         <is>
-          <t>EDS8</t>
+          <t>EJUVINO</t>
         </is>
       </c>
     </row>
     <row r="3422">
       <c r="A3422" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3422" t="n">
-        <v>3328</v>
+        <v>940539</v>
       </c>
       <c r="C3422" t="inlineStr">
         <is>
-          <t>ALAN ARAUJO DA SILVA</t>
+          <t>EDSON ARAUJO - FL9</t>
         </is>
       </c>
       <c r="D3422" t="inlineStr">
         <is>
-          <t>ARSILVA</t>
+          <t>EDS</t>
         </is>
       </c>
     </row>
     <row r="3423">
       <c r="A3423" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B3423" t="n">
-        <v>3350</v>
+        <v>940540</v>
       </c>
       <c r="C3423" t="inlineStr">
         <is>
-          <t xml:space="preserve">EDER RODRIGUES DA SILVA </t>
+          <t>EDSON ARAUJO - FL8</t>
         </is>
       </c>
       <c r="D3423" t="inlineStr">
         <is>
-          <t>EDERS</t>
+          <t>EDS8</t>
         </is>
       </c>
     </row>
     <row r="3424">
       <c r="A3424" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3424" t="n">
-        <v>3373</v>
+        <v>3328</v>
       </c>
       <c r="C3424" t="inlineStr">
         <is>
-          <t xml:space="preserve">NATANAEL TAVARES DE SOUSA </t>
+          <t>ALAN ARAUJO DA SILVA</t>
         </is>
       </c>
       <c r="D3424" t="inlineStr">
         <is>
-          <t>NTSOUSA</t>
+          <t>ARSILVA</t>
         </is>
       </c>
     </row>
     <row r="3425">
       <c r="A3425" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3425" t="n">
-        <v>3374</v>
+        <v>3350</v>
       </c>
       <c r="C3425" t="inlineStr">
         <is>
-          <t>REINALDO DA SILVA COSTA</t>
+          <t xml:space="preserve">EDER RODRIGUES DA SILVA </t>
         </is>
       </c>
       <c r="D3425" t="inlineStr">
         <is>
-          <t>RSCOSTA</t>
+          <t>EDERS</t>
         </is>
       </c>
     </row>
     <row r="3426">
       <c r="A3426" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3426" t="n">
-        <v>3399</v>
+        <v>3373</v>
       </c>
       <c r="C3426" t="inlineStr">
         <is>
-          <t xml:space="preserve">RICARDO BARBOSA DOS SANTOS </t>
+          <t xml:space="preserve">NATANAEL TAVARES DE SOUSA </t>
         </is>
       </c>
       <c r="D3426" t="inlineStr">
         <is>
-          <t>RICARDOSAN</t>
+          <t>NTSOUSA</t>
         </is>
       </c>
     </row>
@@ -68958,56 +68958,56 @@
         </is>
       </c>
       <c r="B3427" t="n">
-        <v>3427</v>
+        <v>3374</v>
       </c>
       <c r="C3427" t="inlineStr">
         <is>
-          <t>ROQUE COMERCIO TEMPORARIO</t>
+          <t>REINALDO DA SILVA COSTA</t>
         </is>
       </c>
       <c r="D3427" t="inlineStr">
         <is>
-          <t>ROQUECOM</t>
+          <t>RSCOSTA</t>
         </is>
       </c>
     </row>
     <row r="3428">
       <c r="A3428" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3428" t="n">
-        <v>3428</v>
+        <v>3399</v>
       </c>
       <c r="C3428" t="inlineStr">
         <is>
-          <t>ROQUE PLUS TEMPORARIO</t>
+          <t xml:space="preserve">RICARDO BARBOSA DOS SANTOS </t>
         </is>
       </c>
       <c r="D3428" t="inlineStr">
         <is>
-          <t>ROQUEPLUS</t>
+          <t>RICARDOSAN</t>
         </is>
       </c>
     </row>
     <row r="3429">
       <c r="A3429" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3429" t="n">
-        <v>3432</v>
+        <v>3427</v>
       </c>
       <c r="C3429" t="inlineStr">
         <is>
-          <t>PATRICIA DOS SANTOS NONATO OLIVEIRA</t>
+          <t>ROQUE COMERCIO TEMPORARIO</t>
         </is>
       </c>
       <c r="D3429" t="inlineStr">
         <is>
-          <t>PATRICIAD</t>
+          <t>ROQUECOM</t>
         </is>
       </c>
     </row>
@@ -69018,36 +69018,36 @@
         </is>
       </c>
       <c r="B3430" t="n">
-        <v>3448</v>
+        <v>3428</v>
       </c>
       <c r="C3430" t="inlineStr">
         <is>
-          <t xml:space="preserve">GABRIEL SOUZA CARVALHO </t>
+          <t>ROQUE PLUS TEMPORARIO</t>
         </is>
       </c>
       <c r="D3430" t="inlineStr">
         <is>
-          <t>GABRIEL20</t>
+          <t>ROQUEPLUS</t>
         </is>
       </c>
     </row>
     <row r="3431">
       <c r="A3431" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3431" t="n">
-        <v>3465</v>
+        <v>3432</v>
       </c>
       <c r="C3431" t="inlineStr">
         <is>
-          <t>LUIZA MARIA BARRETO BARBOSA</t>
+          <t>PATRICIA DOS SANTOS NONATO OLIVEIRA</t>
         </is>
       </c>
       <c r="D3431" t="inlineStr">
         <is>
-          <t>LUIZA.MARIA</t>
+          <t>PATRICIAD</t>
         </is>
       </c>
     </row>
@@ -69058,36 +69058,36 @@
         </is>
       </c>
       <c r="B3432" t="n">
-        <v>3468</v>
+        <v>3448</v>
       </c>
       <c r="C3432" t="inlineStr">
         <is>
-          <t>KAWA ALMEIDA CAMPOS</t>
+          <t xml:space="preserve">GABRIEL SOUZA CARVALHO </t>
         </is>
       </c>
       <c r="D3432" t="inlineStr">
         <is>
-          <t>KAWA</t>
+          <t>GABRIEL20</t>
         </is>
       </c>
     </row>
     <row r="3433">
       <c r="A3433" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3433" t="n">
-        <v>3476</v>
+        <v>3465</v>
       </c>
       <c r="C3433" t="inlineStr">
         <is>
-          <t xml:space="preserve"> FRANCISCA LEIDIANE M. MENDES NASCIMENTO</t>
+          <t>LUIZA MARIA BARRETO BARBOSA</t>
         </is>
       </c>
       <c r="D3433" t="inlineStr">
         <is>
-          <t>FLEIDIANE</t>
+          <t>LUIZA.MARIA</t>
         </is>
       </c>
     </row>
@@ -69098,96 +69098,96 @@
         </is>
       </c>
       <c r="B3434" t="n">
-        <v>3477</v>
+        <v>3468</v>
       </c>
       <c r="C3434" t="inlineStr">
         <is>
-          <t>MARIA THAIS MARTINS PEREIRA SILVA</t>
+          <t>KAWA ALMEIDA CAMPOS</t>
         </is>
       </c>
       <c r="D3434" t="inlineStr">
         <is>
-          <t>MTHAIS</t>
+          <t>KAWA</t>
         </is>
       </c>
     </row>
     <row r="3435">
       <c r="A3435" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3435" t="n">
-        <v>3271</v>
+        <v>3476</v>
       </c>
       <c r="C3435" t="inlineStr">
         <is>
-          <t>DIEGO DE ARAUJO CALÁBRIA</t>
+          <t xml:space="preserve"> FRANCISCA LEIDIANE M. MENDES NASCIMENTO</t>
         </is>
       </c>
       <c r="D3435" t="inlineStr">
         <is>
-          <t>ARAUJOC</t>
+          <t>FLEIDIANE</t>
         </is>
       </c>
     </row>
     <row r="3436">
       <c r="A3436" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3436" t="n">
-        <v>3272</v>
+        <v>3477</v>
       </c>
       <c r="C3436" t="inlineStr">
         <is>
-          <t>ANNE BEATRIZ SILVA VIRGINO</t>
+          <t>MARIA THAIS MARTINS PEREIRA SILVA</t>
         </is>
       </c>
       <c r="D3436" t="inlineStr">
         <is>
-          <t>ABVIRGINIO</t>
+          <t>MTHAIS</t>
         </is>
       </c>
     </row>
     <row r="3437">
       <c r="A3437" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3437" t="n">
-        <v>3293</v>
+        <v>3271</v>
       </c>
       <c r="C3437" t="inlineStr">
         <is>
-          <t xml:space="preserve">CARLOS ALBERTO VIRIATO SANTOS </t>
+          <t>DIEGO DE ARAUJO CALÁBRIA</t>
         </is>
       </c>
       <c r="D3437" t="inlineStr">
         <is>
-          <t>CVIRIATO</t>
+          <t>ARAUJOC</t>
         </is>
       </c>
     </row>
     <row r="3438">
       <c r="A3438" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3438" t="n">
-        <v>3381</v>
+        <v>3272</v>
       </c>
       <c r="C3438" t="inlineStr">
         <is>
-          <t>ALAN CAIQUE SANTOS E SANTOS</t>
+          <t>ANNE BEATRIZ SILVA VIRGINO</t>
         </is>
       </c>
       <c r="D3438" t="inlineStr">
         <is>
-          <t>ALANSANTOS</t>
+          <t>ABVIRGINIO</t>
         </is>
       </c>
     </row>
@@ -69198,76 +69198,76 @@
         </is>
       </c>
       <c r="B3439" t="n">
-        <v>3443</v>
+        <v>3293</v>
       </c>
       <c r="C3439" t="inlineStr">
         <is>
-          <t>SANON MOREIRA SOUZA</t>
+          <t xml:space="preserve">CARLOS ALBERTO VIRIATO SANTOS </t>
         </is>
       </c>
       <c r="D3439" t="inlineStr">
         <is>
-          <t>SANON</t>
+          <t>CVIRIATO</t>
         </is>
       </c>
     </row>
     <row r="3440">
       <c r="A3440" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3440" t="n">
-        <v>3516</v>
+        <v>3381</v>
       </c>
       <c r="C3440" t="inlineStr">
         <is>
-          <t>FRANCISCO RILDER TELES DE OLIVEIRA</t>
+          <t>ALAN CAIQUE SANTOS E SANTOS</t>
         </is>
       </c>
       <c r="D3440" t="inlineStr">
         <is>
-          <t>RILDER</t>
+          <t>ALANSANTOS</t>
         </is>
       </c>
     </row>
     <row r="3441">
       <c r="A3441" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3441" t="n">
-        <v>3519</v>
+        <v>3443</v>
       </c>
       <c r="C3441" t="inlineStr">
         <is>
-          <t>MARIA LUANA DE ALMEIDA BATISTA</t>
+          <t>SANON MOREIRA SOUZA</t>
         </is>
       </c>
       <c r="D3441" t="inlineStr">
         <is>
-          <t>M.LUANA</t>
+          <t>SANON</t>
         </is>
       </c>
     </row>
     <row r="3442">
       <c r="A3442" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3442" t="n">
-        <v>3540</v>
+        <v>3516</v>
       </c>
       <c r="C3442" t="inlineStr">
         <is>
-          <t>HELEN VITORIA OLIVEIRA DA ROCHA</t>
+          <t>FRANCISCO RILDER TELES DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D3442" t="inlineStr">
         <is>
-          <t>H.VITORIA</t>
+          <t>RILDER</t>
         </is>
       </c>
     </row>
@@ -69278,76 +69278,76 @@
         </is>
       </c>
       <c r="B3443" t="n">
-        <v>3559</v>
+        <v>3519</v>
       </c>
       <c r="C3443" t="inlineStr">
         <is>
-          <t>ARKBERYS TELES DE SOUSA</t>
+          <t>MARIA LUANA DE ALMEIDA BATISTA</t>
         </is>
       </c>
       <c r="D3443" t="inlineStr">
         <is>
-          <t>ARKBERYS</t>
+          <t>M.LUANA</t>
         </is>
       </c>
     </row>
     <row r="3444">
       <c r="A3444" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B3444" t="n">
-        <v>3567</v>
+        <v>3540</v>
       </c>
       <c r="C3444" t="inlineStr">
         <is>
-          <t>PEDRO HENRIQUE VIEIRA DE LIMA</t>
+          <t>HELEN VITORIA OLIVEIRA DA ROCHA</t>
         </is>
       </c>
       <c r="D3444" t="inlineStr">
         <is>
-          <t>P.LIMA</t>
+          <t>H.VITORIA</t>
         </is>
       </c>
     </row>
     <row r="3445">
       <c r="A3445" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3445" t="n">
-        <v>3331</v>
+        <v>3559</v>
       </c>
       <c r="C3445" t="inlineStr">
         <is>
-          <t>LOUIZE VANIELLE RODRIGUES FARIAS</t>
+          <t>ARKBERYS TELES DE SOUSA</t>
         </is>
       </c>
       <c r="D3445" t="inlineStr">
         <is>
-          <t>LVFARIAS</t>
+          <t>ARKBERYS</t>
         </is>
       </c>
     </row>
     <row r="3446">
       <c r="A3446" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3446" t="n">
-        <v>3334</v>
+        <v>3567</v>
       </c>
       <c r="C3446" t="inlineStr">
         <is>
-          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+          <t>PEDRO HENRIQUE VIEIRA DE LIMA</t>
         </is>
       </c>
       <c r="D3446" t="inlineStr">
         <is>
-          <t>MTGASPAR</t>
+          <t>P.LIMA</t>
         </is>
       </c>
     </row>
@@ -69358,356 +69358,356 @@
         </is>
       </c>
       <c r="B3447" t="n">
-        <v>3345</v>
+        <v>3331</v>
       </c>
       <c r="C3447" t="inlineStr">
         <is>
-          <t>AURICÉLIA INACIO PEREIRA</t>
+          <t>LOUIZE VANIELLE RODRIGUES FARIAS</t>
         </is>
       </c>
       <c r="D3447" t="inlineStr">
         <is>
-          <t>AIPEREIRA</t>
+          <t>LVFARIAS</t>
         </is>
       </c>
     </row>
     <row r="3448">
       <c r="A3448" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3448" t="n">
-        <v>3363</v>
+        <v>3334</v>
       </c>
       <c r="C3448" t="inlineStr">
         <is>
-          <t>IASMIN LEAL ALVES</t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
       <c r="D3448" t="inlineStr">
         <is>
-          <t>ILALVES</t>
+          <t>MTGASPAR</t>
         </is>
       </c>
     </row>
     <row r="3449">
       <c r="A3449" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3449" t="n">
-        <v>3370</v>
+        <v>3345</v>
       </c>
       <c r="C3449" t="inlineStr">
         <is>
-          <t>CARLOS DIEGO ARAUJO ALMEIDA</t>
+          <t>AURICÉLIA INACIO PEREIRA</t>
         </is>
       </c>
       <c r="D3449" t="inlineStr">
         <is>
-          <t>CDIEGO</t>
+          <t>AIPEREIRA</t>
         </is>
       </c>
     </row>
     <row r="3450">
       <c r="A3450" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3450" t="n">
-        <v>3379</v>
+        <v>3363</v>
       </c>
       <c r="C3450" t="inlineStr">
         <is>
-          <t xml:space="preserve">MATHEUS EVANGELISTA FERREIRA </t>
+          <t>IASMIN LEAL ALVES</t>
         </is>
       </c>
       <c r="D3450" t="inlineStr">
         <is>
-          <t>MMFERREIRA</t>
+          <t>ILALVES</t>
         </is>
       </c>
     </row>
     <row r="3451">
       <c r="A3451" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3451" t="n">
-        <v>3419</v>
+        <v>3370</v>
       </c>
       <c r="C3451" t="inlineStr">
         <is>
-          <t xml:space="preserve">DAVID EVANGELISTA SILVA </t>
+          <t>CARLOS DIEGO ARAUJO ALMEIDA</t>
         </is>
       </c>
       <c r="D3451" t="inlineStr">
         <is>
-          <t>DAVID</t>
+          <t>CDIEGO</t>
         </is>
       </c>
     </row>
     <row r="3452">
       <c r="A3452" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3452" t="n">
-        <v>3423</v>
+        <v>3379</v>
       </c>
       <c r="C3452" t="inlineStr">
         <is>
-          <t>MARCIO JOSE TIAGO</t>
+          <t xml:space="preserve">MATHEUS EVANGELISTA FERREIRA </t>
         </is>
       </c>
       <c r="D3452" t="inlineStr">
         <is>
-          <t>MJTIAGO</t>
+          <t>MMFERREIRA</t>
         </is>
       </c>
     </row>
     <row r="3453">
       <c r="A3453" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3453" t="n">
-        <v>3453</v>
+        <v>3419</v>
       </c>
       <c r="C3453" t="inlineStr">
         <is>
-          <t xml:space="preserve">LAURIENE SILVA BARBOSA </t>
+          <t xml:space="preserve">DAVID EVANGELISTA SILVA </t>
         </is>
       </c>
       <c r="D3453" t="inlineStr">
         <is>
-          <t>LAURIENE</t>
+          <t>DAVID</t>
         </is>
       </c>
     </row>
     <row r="3454">
       <c r="A3454" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3454" t="n">
-        <v>3478</v>
+        <v>3423</v>
       </c>
       <c r="C3454" t="inlineStr">
         <is>
-          <t>LEANDRO BRITO NOGUEIRA DE OLIVEIRA</t>
+          <t>MARCIO JOSE TIAGO</t>
         </is>
       </c>
       <c r="D3454" t="inlineStr">
         <is>
-          <t>LBNOGUEIRA</t>
+          <t>MJTIAGO</t>
         </is>
       </c>
     </row>
     <row r="3455">
       <c r="A3455" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3455" t="n">
-        <v>3479</v>
+        <v>3453</v>
       </c>
       <c r="C3455" t="inlineStr">
         <is>
-          <t>ESDRAS ALESSANDRO SANTOS SANTANA</t>
+          <t xml:space="preserve">LAURIENE SILVA BARBOSA </t>
         </is>
       </c>
       <c r="D3455" t="inlineStr">
         <is>
-          <t>EALESSANDRO</t>
+          <t>LAURIENE</t>
         </is>
       </c>
     </row>
     <row r="3456">
       <c r="A3456" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3456" t="n">
-        <v>3480</v>
+        <v>3478</v>
       </c>
       <c r="C3456" t="inlineStr">
         <is>
-          <t xml:space="preserve">LUCIMARA SOUSA LIMA </t>
+          <t>LEANDRO BRITO NOGUEIRA DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D3456" t="inlineStr">
         <is>
-          <t>LUCIMARA</t>
+          <t>LBNOGUEIRA</t>
         </is>
       </c>
     </row>
     <row r="3457">
       <c r="A3457" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3457" t="n">
-        <v>3482</v>
+        <v>3479</v>
       </c>
       <c r="C3457" t="inlineStr">
         <is>
-          <t>DANIEL FERNANDES DINIZ HERACLIO</t>
+          <t>ESDRAS ALESSANDRO SANTOS SANTANA</t>
         </is>
       </c>
       <c r="D3457" t="inlineStr">
         <is>
-          <t>DFDINIZ</t>
+          <t>EALESSANDRO</t>
         </is>
       </c>
     </row>
     <row r="3458">
       <c r="A3458" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3458" t="n">
-        <v>3518</v>
+        <v>3480</v>
       </c>
       <c r="C3458" t="inlineStr">
         <is>
-          <t>RAMYRA ALVES FELIX DA SILVA</t>
+          <t xml:space="preserve">LUCIMARA SOUSA LIMA </t>
         </is>
       </c>
       <c r="D3458" t="inlineStr">
         <is>
-          <t>RFELIX</t>
+          <t>LUCIMARA</t>
         </is>
       </c>
     </row>
     <row r="3459">
       <c r="A3459" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3459" t="n">
-        <v>3534</v>
+        <v>3482</v>
       </c>
       <c r="C3459" t="inlineStr">
         <is>
-          <t xml:space="preserve">CAIO DE SOUZA VINHAS </t>
+          <t>DANIEL FERNANDES DINIZ HERACLIO</t>
         </is>
       </c>
       <c r="D3459" t="inlineStr">
         <is>
-          <t>CVINHAS</t>
+          <t>DFDINIZ</t>
         </is>
       </c>
     </row>
     <row r="3460">
       <c r="A3460" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3460" t="n">
-        <v>3535</v>
+        <v>3518</v>
       </c>
       <c r="C3460" t="inlineStr">
         <is>
-          <t>ROMARIO DE SOUSA SILVA</t>
+          <t>RAMYRA ALVES FELIX DA SILVA</t>
         </is>
       </c>
       <c r="D3460" t="inlineStr">
         <is>
-          <t>RSOUSAS</t>
+          <t>RFELIX</t>
         </is>
       </c>
     </row>
     <row r="3461">
       <c r="A3461" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3461" t="n">
-        <v>3536</v>
+        <v>3534</v>
       </c>
       <c r="C3461" t="inlineStr">
         <is>
-          <t>JHONATAS CARVALHO OLIVEIRA</t>
+          <t xml:space="preserve">CAIO DE SOUZA VINHAS </t>
         </is>
       </c>
       <c r="D3461" t="inlineStr">
         <is>
-          <t>JHONATASC</t>
+          <t>CVINHAS</t>
         </is>
       </c>
     </row>
     <row r="3462">
       <c r="A3462" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3462" t="n">
-        <v>940529</v>
+        <v>3535</v>
       </c>
       <c r="C3462" t="inlineStr">
         <is>
-          <t>EDGAR FELIX - FL9</t>
+          <t>ROMARIO DE SOUSA SILVA</t>
         </is>
       </c>
       <c r="D3462" t="inlineStr">
         <is>
-          <t>EDGAR F</t>
+          <t>RSOUSAS</t>
         </is>
       </c>
     </row>
     <row r="3463">
       <c r="A3463" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3463" t="n">
-        <v>3304</v>
+        <v>3536</v>
       </c>
       <c r="C3463" t="inlineStr">
         <is>
-          <t>JOACI GUILHERME GONÇALVES DA LUZ</t>
+          <t>JHONATAS CARVALHO OLIVEIRA</t>
         </is>
       </c>
       <c r="D3463" t="inlineStr">
         <is>
-          <t>JLUZ</t>
+          <t>JHONATASC</t>
         </is>
       </c>
     </row>
     <row r="3464">
       <c r="A3464" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3464" t="n">
-        <v>3305</v>
+        <v>940529</v>
       </c>
       <c r="C3464" t="inlineStr">
         <is>
-          <t>JOÃO VITOR DE ARAÚJO GONÇALVES</t>
+          <t>EDGAR FELIX - FL9</t>
         </is>
       </c>
       <c r="D3464" t="inlineStr">
         <is>
-          <t>JJVITOR</t>
+          <t>EDGAR F</t>
         </is>
       </c>
     </row>
@@ -69718,276 +69718,276 @@
         </is>
       </c>
       <c r="B3465" t="n">
-        <v>3306</v>
+        <v>3304</v>
       </c>
       <c r="C3465" t="inlineStr">
         <is>
-          <t>WENDERSON MARCOS DOS SANTOS</t>
+          <t>JOACI GUILHERME GONÇALVES DA LUZ</t>
         </is>
       </c>
       <c r="D3465" t="inlineStr">
         <is>
-          <t>WWMARCOS</t>
+          <t>JLUZ</t>
         </is>
       </c>
     </row>
     <row r="3466">
       <c r="A3466" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3466" t="n">
-        <v>3335</v>
+        <v>3305</v>
       </c>
       <c r="C3466" t="inlineStr">
         <is>
-          <t>EDILBERTO LEMOS DE LIMA</t>
+          <t>JOÃO VITOR DE ARAÚJO GONÇALVES</t>
         </is>
       </c>
       <c r="D3466" t="inlineStr">
         <is>
-          <t>ELEMOS</t>
+          <t>JJVITOR</t>
         </is>
       </c>
     </row>
     <row r="3467">
       <c r="A3467" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3467" t="n">
-        <v>3336</v>
+        <v>3306</v>
       </c>
       <c r="C3467" t="inlineStr">
         <is>
-          <t>EZEQUIEL SOUZA DO NASCIMENTO</t>
+          <t>WENDERSON MARCOS DOS SANTOS</t>
         </is>
       </c>
       <c r="D3467" t="inlineStr">
         <is>
-          <t>ESNASCIMENTO</t>
+          <t>WWMARCOS</t>
         </is>
       </c>
     </row>
     <row r="3468">
       <c r="A3468" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3468" t="n">
-        <v>3341</v>
+        <v>3335</v>
       </c>
       <c r="C3468" t="inlineStr">
         <is>
-          <t>ALCIONE MARIANO DE OLIVEIRA</t>
+          <t>EDILBERTO LEMOS DE LIMA</t>
         </is>
       </c>
       <c r="D3468" t="inlineStr">
         <is>
-          <t>AMOLIVEIRA</t>
+          <t>ELEMOS</t>
         </is>
       </c>
     </row>
     <row r="3469">
       <c r="A3469" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3469" t="n">
-        <v>3401</v>
+        <v>3336</v>
       </c>
       <c r="C3469" t="inlineStr">
         <is>
-          <t xml:space="preserve">TULIO HENRIQUE DA SILVA CARVALHO </t>
+          <t>EZEQUIEL SOUZA DO NASCIMENTO</t>
         </is>
       </c>
       <c r="D3469" t="inlineStr">
         <is>
-          <t>TULIO</t>
+          <t>ESNASCIMENTO</t>
         </is>
       </c>
     </row>
     <row r="3470">
       <c r="A3470" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3470" t="n">
-        <v>3411</v>
+        <v>3341</v>
       </c>
       <c r="C3470" t="inlineStr">
         <is>
-          <t>CONEXAO RUBYA DANILLA</t>
+          <t>ALCIONE MARIANO DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D3470" t="inlineStr">
         <is>
-          <t>CONEXAORUBYA</t>
+          <t>AMOLIVEIRA</t>
         </is>
       </c>
     </row>
     <row r="3471">
       <c r="A3471" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3471" t="n">
-        <v>3412</v>
+        <v>3401</v>
       </c>
       <c r="C3471" t="inlineStr">
         <is>
-          <t>CONEXAO RAFAEL</t>
+          <t xml:space="preserve">TULIO HENRIQUE DA SILVA CARVALHO </t>
         </is>
       </c>
       <c r="D3471" t="inlineStr">
         <is>
-          <t>CONEXAORAFAEL</t>
+          <t>TULIO</t>
         </is>
       </c>
     </row>
     <row r="3472">
       <c r="A3472" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3472" t="n">
-        <v>3558</v>
+        <v>3411</v>
       </c>
       <c r="C3472" t="inlineStr">
         <is>
-          <t>WALLYS QUEIROZ VIANA</t>
+          <t>CONEXAO RUBYA DANILLA</t>
         </is>
       </c>
       <c r="D3472" t="inlineStr">
         <is>
-          <t>WALLYS</t>
+          <t>CONEXAORUBYA</t>
         </is>
       </c>
     </row>
     <row r="3473">
       <c r="A3473" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3473" t="n">
-        <v>3264</v>
+        <v>3412</v>
       </c>
       <c r="C3473" t="inlineStr">
         <is>
-          <t xml:space="preserve">WILTON CARLOS MACIEL DE ASSIS </t>
+          <t>CONEXAO RAFAEL</t>
         </is>
       </c>
       <c r="D3473" t="inlineStr">
         <is>
-          <t>WCMACIEL</t>
+          <t>CONEXAORAFAEL</t>
         </is>
       </c>
     </row>
     <row r="3474">
       <c r="A3474" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3474" t="n">
-        <v>3340</v>
+        <v>3558</v>
       </c>
       <c r="C3474" t="inlineStr">
         <is>
-          <t>ROGELENO FARIAS FEIJÃO FILHO</t>
+          <t>WALLYS QUEIROZ VIANA</t>
         </is>
       </c>
       <c r="D3474" t="inlineStr">
         <is>
-          <t>RFEIJAO</t>
+          <t>WALLYS</t>
         </is>
       </c>
     </row>
     <row r="3475">
       <c r="A3475" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3475" t="n">
-        <v>940550</v>
+        <v>3264</v>
       </c>
       <c r="C3475" t="inlineStr">
         <is>
-          <t>RAFAELE RIBEIRO CARNEIRO</t>
+          <t xml:space="preserve">WILTON CARLOS MACIEL DE ASSIS </t>
         </is>
       </c>
       <c r="D3475" t="inlineStr">
         <is>
-          <t>RAFAELE</t>
+          <t>WCMACIEL</t>
         </is>
       </c>
     </row>
     <row r="3476">
       <c r="A3476" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3476" t="n">
-        <v>3377</v>
+        <v>3340</v>
       </c>
       <c r="C3476" t="inlineStr">
         <is>
-          <t xml:space="preserve"> ISALTINO BISPO DE OLIVEIRA JUNIOR</t>
+          <t>ROGELENO FARIAS FEIJÃO FILHO</t>
         </is>
       </c>
       <c r="D3476" t="inlineStr">
         <is>
-          <t>BJUNIOR</t>
+          <t>RFEIJAO</t>
         </is>
       </c>
     </row>
     <row r="3477">
       <c r="A3477" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>99</t>
         </is>
       </c>
       <c r="B3477" t="n">
-        <v>3425</v>
+        <v>940550</v>
       </c>
       <c r="C3477" t="inlineStr">
         <is>
-          <t xml:space="preserve"> CIRLANE ARAUJO SOUZA </t>
+          <t>RAFAELE RIBEIRO CARNEIRO</t>
         </is>
       </c>
       <c r="D3477" t="inlineStr">
         <is>
-          <t>CIRLANES</t>
+          <t>RAFAELE</t>
         </is>
       </c>
     </row>
     <row r="3478">
       <c r="A3478" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3478" t="n">
-        <v>3454</v>
+        <v>3377</v>
       </c>
       <c r="C3478" t="inlineStr">
         <is>
-          <t>ANTONIA SAMARA DE SOUZA SOARES</t>
+          <t xml:space="preserve"> ISALTINO BISPO DE OLIVEIRA JUNIOR</t>
         </is>
       </c>
       <c r="D3478" t="inlineStr">
         <is>
-          <t>ANTSAMARA</t>
+          <t>BJUNIOR</t>
         </is>
       </c>
     </row>
@@ -69998,96 +69998,96 @@
         </is>
       </c>
       <c r="B3479" t="n">
-        <v>3491</v>
+        <v>3425</v>
       </c>
       <c r="C3479" t="inlineStr">
         <is>
-          <t>PEDRO JOSE DO NASCIMENTO NETO</t>
+          <t xml:space="preserve"> CIRLANE ARAUJO SOUZA </t>
         </is>
       </c>
       <c r="D3479" t="inlineStr">
         <is>
-          <t>P.JOSE</t>
+          <t>CIRLANES</t>
         </is>
       </c>
     </row>
     <row r="3480">
       <c r="A3480" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3480" t="n">
-        <v>3492</v>
+        <v>3454</v>
       </c>
       <c r="C3480" t="inlineStr">
         <is>
-          <t>PAULA CARLA CALDAS MOTA</t>
+          <t>ANTONIA SAMARA DE SOUZA SOARES</t>
         </is>
       </c>
       <c r="D3480" t="inlineStr">
         <is>
-          <t>P.CARLA</t>
+          <t>ANTSAMARA</t>
         </is>
       </c>
     </row>
     <row r="3481">
       <c r="A3481" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3481" t="n">
-        <v>3542</v>
+        <v>3491</v>
       </c>
       <c r="C3481" t="inlineStr">
         <is>
-          <t>ANTONIA MILENA SOUSA ANDRADE</t>
+          <t>PEDRO JOSE DO NASCIMENTO NETO</t>
         </is>
       </c>
       <c r="D3481" t="inlineStr">
         <is>
-          <t>A.MILENA</t>
+          <t>P.JOSE</t>
         </is>
       </c>
     </row>
     <row r="3482">
       <c r="A3482" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3482" t="n">
-        <v>3547</v>
+        <v>3492</v>
       </c>
       <c r="C3482" t="inlineStr">
         <is>
-          <t xml:space="preserve">DAVI PEREIRA DA SILVA </t>
+          <t>PAULA CARLA CALDAS MOTA</t>
         </is>
       </c>
       <c r="D3482" t="inlineStr">
         <is>
-          <t>DPSILVA</t>
+          <t>P.CARLA</t>
         </is>
       </c>
     </row>
     <row r="3483">
       <c r="A3483" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3483" t="n">
-        <v>3552</v>
+        <v>3542</v>
       </c>
       <c r="C3483" t="inlineStr">
         <is>
-          <t>PAULO SERGIO MENDES DE OLIVEIRA</t>
+          <t>ANTONIA MILENA SOUSA ANDRADE</t>
         </is>
       </c>
       <c r="D3483" t="inlineStr">
         <is>
-          <t>PSMENDES</t>
+          <t>A.MILENA</t>
         </is>
       </c>
     </row>
@@ -70098,214 +70098,254 @@
         </is>
       </c>
       <c r="B3484" t="n">
-        <v>3294</v>
+        <v>3547</v>
       </c>
       <c r="C3484" t="inlineStr">
         <is>
-          <t>GLEICIANE MIRANDA DE MORAIS</t>
+          <t xml:space="preserve">DAVI PEREIRA DA SILVA </t>
         </is>
       </c>
       <c r="D3484" t="inlineStr">
         <is>
-          <t>GMIRANDA</t>
+          <t>DPSILVA</t>
         </is>
       </c>
     </row>
     <row r="3485">
       <c r="A3485" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3485" t="n">
-        <v>3295</v>
+        <v>3552</v>
       </c>
       <c r="C3485" t="inlineStr">
         <is>
-          <t>MARIA ESTEFANNY DA SILVA MOURA</t>
+          <t>PAULO SERGIO MENDES DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D3485" t="inlineStr">
         <is>
-          <t>MESTEFANNY</t>
+          <t>PSMENDES</t>
         </is>
       </c>
     </row>
     <row r="3486">
       <c r="A3486" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3486" t="n">
-        <v>3296</v>
+        <v>3294</v>
       </c>
       <c r="C3486" t="inlineStr">
         <is>
-          <t>PEDRO IAGO FONSECA EVANGELISTA</t>
+          <t>GLEICIANE MIRANDA DE MORAIS</t>
         </is>
       </c>
       <c r="D3486" t="inlineStr">
         <is>
-          <t>PIFONSECA</t>
+          <t>GMIRANDA</t>
         </is>
       </c>
     </row>
     <row r="3487">
       <c r="A3487" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3487" t="n">
-        <v>940544</v>
+        <v>3295</v>
       </c>
       <c r="C3487" t="inlineStr">
         <is>
-          <t>LUTY LOG TRANSPORTES - FL8</t>
+          <t>MARIA ESTEFANNY DA SILVA MOURA</t>
         </is>
       </c>
       <c r="D3487" t="inlineStr">
         <is>
-          <t>LUTY LOG</t>
+          <t>MESTEFANNY</t>
         </is>
       </c>
     </row>
     <row r="3488">
       <c r="A3488" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3488" t="n">
-        <v>3380</v>
+        <v>3296</v>
       </c>
       <c r="C3488" t="inlineStr">
         <is>
-          <t>FRANCISCO MATHEUS RABELO DA COSTA</t>
+          <t>PEDRO IAGO FONSECA EVANGELISTA</t>
         </is>
       </c>
       <c r="D3488" t="inlineStr">
         <is>
-          <t>FMATHEUS</t>
+          <t>PIFONSECA</t>
         </is>
       </c>
     </row>
     <row r="3489">
       <c r="A3489" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B3489" t="n">
-        <v>3410</v>
+        <v>940544</v>
       </c>
       <c r="C3489" t="inlineStr">
         <is>
-          <t xml:space="preserve"> BRENO ALLAN DE JESUS</t>
+          <t>LUTY LOG TRANSPORTES - FL8</t>
         </is>
       </c>
       <c r="D3489" t="inlineStr">
         <is>
-          <t>JESUS</t>
+          <t>LUTY LOG</t>
         </is>
       </c>
     </row>
     <row r="3490">
       <c r="A3490" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3490" t="n">
-        <v>3444</v>
+        <v>3380</v>
       </c>
       <c r="C3490" t="inlineStr">
         <is>
-          <t>THIAGO COSTA SILVA</t>
+          <t>FRANCISCO MATHEUS RABELO DA COSTA</t>
         </is>
       </c>
       <c r="D3490" t="inlineStr">
         <is>
-          <t>THIAGOC</t>
+          <t>FMATHEUS</t>
         </is>
       </c>
     </row>
     <row r="3491">
       <c r="A3491" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3491" t="n">
-        <v>3456</v>
+        <v>3410</v>
       </c>
       <c r="C3491" t="inlineStr">
         <is>
-          <t>FELIPE BOTH MAZUCHINI</t>
+          <t xml:space="preserve"> BRENO ALLAN DE JESUS</t>
         </is>
       </c>
       <c r="D3491" t="inlineStr">
         <is>
-          <t>FELIPEB</t>
+          <t>JESUS</t>
         </is>
       </c>
     </row>
     <row r="3492">
       <c r="A3492" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3492" t="n">
-        <v>3457</v>
+        <v>3444</v>
       </c>
       <c r="C3492" t="inlineStr">
         <is>
-          <t>FRANKLIN VIEIRA GOMES</t>
+          <t>THIAGO COSTA SILVA</t>
         </is>
       </c>
       <c r="D3492" t="inlineStr">
         <is>
-          <t>VIEIRAF</t>
+          <t>THIAGOC</t>
         </is>
       </c>
     </row>
     <row r="3493">
       <c r="A3493" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3493" t="n">
-        <v>3507</v>
+        <v>3456</v>
       </c>
       <c r="C3493" t="inlineStr">
         <is>
-          <t>KARINE TEODORA ALVES DE OLIVEIRA</t>
+          <t>FELIPE BOTH MAZUCHINI</t>
         </is>
       </c>
       <c r="D3493" t="inlineStr">
         <is>
-          <t>KOLIVEIRA</t>
+          <t>FELIPEB</t>
         </is>
       </c>
     </row>
     <row r="3494">
       <c r="A3494" t="inlineStr">
         <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B3494" t="n">
+        <v>3457</v>
+      </c>
+      <c r="C3494" t="inlineStr">
+        <is>
+          <t>FRANKLIN VIEIRA GOMES</t>
+        </is>
+      </c>
+      <c r="D3494" t="inlineStr">
+        <is>
+          <t>VIEIRAF</t>
+        </is>
+      </c>
+    </row>
+    <row r="3495">
+      <c r="A3495" t="inlineStr">
+        <is>
           <t>5</t>
         </is>
       </c>
-      <c r="B3494" t="n">
+      <c r="B3495" t="n">
+        <v>3507</v>
+      </c>
+      <c r="C3495" t="inlineStr">
+        <is>
+          <t>KARINE TEODORA ALVES DE OLIVEIRA</t>
+        </is>
+      </c>
+      <c r="D3495" t="inlineStr">
+        <is>
+          <t>KOLIVEIRA</t>
+        </is>
+      </c>
+    </row>
+    <row r="3496">
+      <c r="A3496" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B3496" t="n">
         <v>3520</v>
       </c>
-      <c r="C3494" t="inlineStr">
+      <c r="C3496" t="inlineStr">
         <is>
           <t xml:space="preserve"> EMERSON FILIPE MELO DE AGUIAR</t>
         </is>
       </c>
-      <c r="D3494" t="inlineStr">
+      <c r="D3496" t="inlineStr">
         <is>
           <t>E.FILIPE</t>
         </is>

</xml_diff>

<commit_message>
chore(data): batch update intraday televendas - 08:02:23
</commit_message>
<xml_diff>
--- a/data/dim_televendas.xlsx
+++ b/data/dim_televendas.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3506"/>
+  <dimension ref="A1:D3507"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16254,7 +16254,7 @@
     <row r="792">
       <c r="A792" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B792" t="n">
@@ -66374,40 +66374,40 @@
     <row r="3298">
       <c r="A3298" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3298" t="n">
-        <v>3265</v>
+        <v>3594</v>
       </c>
       <c r="C3298" t="inlineStr">
         <is>
-          <t>ANAELSON FREITAS VIEIRA</t>
+          <t>TESTE9</t>
         </is>
       </c>
       <c r="D3298" t="inlineStr">
         <is>
-          <t>AFVIEIRA</t>
+          <t>TESTE9</t>
         </is>
       </c>
     </row>
     <row r="3299">
       <c r="A3299" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3299" t="n">
-        <v>3413</v>
+        <v>3265</v>
       </c>
       <c r="C3299" t="inlineStr">
         <is>
-          <t>CONEXAO THAMIRES MONTEIRO</t>
+          <t>ANAELSON FREITAS VIEIRA</t>
         </is>
       </c>
       <c r="D3299" t="inlineStr">
         <is>
-          <t>CONEXAOTHAMIRES</t>
+          <t>AFVIEIRA</t>
         </is>
       </c>
     </row>
@@ -66418,76 +66418,76 @@
         </is>
       </c>
       <c r="B3300" t="n">
-        <v>3431</v>
+        <v>3413</v>
       </c>
       <c r="C3300" t="inlineStr">
         <is>
-          <t>ALLYSSON PINHEIRO AGUIAR E SILVA</t>
+          <t>CONEXAO THAMIRES MONTEIRO</t>
         </is>
       </c>
       <c r="D3300" t="inlineStr">
         <is>
-          <t>ALYSSONP</t>
+          <t>CONEXAOTHAMIRES</t>
         </is>
       </c>
     </row>
     <row r="3301">
       <c r="A3301" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3301" t="n">
-        <v>3499</v>
+        <v>3431</v>
       </c>
       <c r="C3301" t="inlineStr">
         <is>
-          <t>JAIME VITORINO DE OLIVEIRA SOUSA</t>
+          <t>ALLYSSON PINHEIRO AGUIAR E SILVA</t>
         </is>
       </c>
       <c r="D3301" t="inlineStr">
         <is>
-          <t>JVITORINO</t>
+          <t>ALYSSONP</t>
         </is>
       </c>
     </row>
     <row r="3302">
       <c r="A3302" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3302" t="n">
-        <v>3500</v>
+        <v>3499</v>
       </c>
       <c r="C3302" t="inlineStr">
         <is>
-          <t>TACIANE DE HOLANDA MACIEL</t>
+          <t>JAIME VITORINO DE OLIVEIRA SOUSA</t>
         </is>
       </c>
       <c r="D3302" t="inlineStr">
         <is>
-          <t>TMACIEL</t>
+          <t>JVITORINO</t>
         </is>
       </c>
     </row>
     <row r="3303">
       <c r="A3303" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3303" t="n">
-        <v>3545</v>
+        <v>3500</v>
       </c>
       <c r="C3303" t="inlineStr">
         <is>
-          <t>FABIO JUNIOR DA SILVA FIGUEIRA</t>
+          <t>TACIANE DE HOLANDA MACIEL</t>
         </is>
       </c>
       <c r="D3303" t="inlineStr">
         <is>
-          <t>F.JUNIOR</t>
+          <t>TMACIEL</t>
         </is>
       </c>
     </row>
@@ -66498,36 +66498,36 @@
         </is>
       </c>
       <c r="B3304" t="n">
-        <v>3546</v>
+        <v>3545</v>
       </c>
       <c r="C3304" t="inlineStr">
         <is>
-          <t>GEREMIAS DA SILVA PEREIRA</t>
+          <t>FABIO JUNIOR DA SILVA FIGUEIRA</t>
         </is>
       </c>
       <c r="D3304" t="inlineStr">
         <is>
-          <t>G.SILVA</t>
+          <t>F.JUNIOR</t>
         </is>
       </c>
     </row>
     <row r="3305">
       <c r="A3305" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3305" t="n">
-        <v>3582</v>
+        <v>3546</v>
       </c>
       <c r="C3305" t="inlineStr">
         <is>
-          <t>MARCOS SERGIO DE OLIVEIRA</t>
+          <t>GEREMIAS DA SILVA PEREIRA</t>
         </is>
       </c>
       <c r="D3305" t="inlineStr">
         <is>
-          <t>MARCOS.S</t>
+          <t>G.SILVA</t>
         </is>
       </c>
     </row>
@@ -66538,56 +66538,56 @@
         </is>
       </c>
       <c r="B3306" t="n">
-        <v>3279</v>
+        <v>3582</v>
       </c>
       <c r="C3306" t="inlineStr">
         <is>
-          <t>IARGO GABRIEL SANTOS DE OLIVEIRA</t>
+          <t>MARCOS SERGIO DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D3306" t="inlineStr">
         <is>
-          <t>IARGOSANTOS</t>
+          <t>MARCOS.S</t>
         </is>
       </c>
     </row>
     <row r="3307">
       <c r="A3307" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3307" t="n">
-        <v>3349</v>
+        <v>3279</v>
       </c>
       <c r="C3307" t="inlineStr">
         <is>
-          <t xml:space="preserve">ROBSON DE SOUZA LEITE </t>
+          <t>IARGO GABRIEL SANTOS DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D3307" t="inlineStr">
         <is>
-          <t>RLEITE</t>
+          <t>IARGOSANTOS</t>
         </is>
       </c>
     </row>
     <row r="3308">
       <c r="A3308" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3308" t="n">
-        <v>3367</v>
+        <v>3349</v>
       </c>
       <c r="C3308" t="inlineStr">
         <is>
-          <t>CARLOS JEANDERSON DA SILVA GUTERRES</t>
+          <t xml:space="preserve">ROBSON DE SOUZA LEITE </t>
         </is>
       </c>
       <c r="D3308" t="inlineStr">
         <is>
-          <t>CGUTERRES</t>
+          <t>RLEITE</t>
         </is>
       </c>
     </row>
@@ -66598,96 +66598,96 @@
         </is>
       </c>
       <c r="B3309" t="n">
-        <v>3392</v>
+        <v>3367</v>
       </c>
       <c r="C3309" t="inlineStr">
         <is>
-          <t xml:space="preserve">LAERCIA KARINE OLIVEIRA MORAIS </t>
+          <t>CARLOS JEANDERSON DA SILVA GUTERRES</t>
         </is>
       </c>
       <c r="D3309" t="inlineStr">
         <is>
-          <t>KARINE28</t>
+          <t>CGUTERRES</t>
         </is>
       </c>
     </row>
     <row r="3310">
       <c r="A3310" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3310" t="n">
-        <v>3446</v>
+        <v>3392</v>
       </c>
       <c r="C3310" t="inlineStr">
         <is>
-          <t>MARIA FERNANDA SOUSA DA CRUZ</t>
+          <t xml:space="preserve">LAERCIA KARINE OLIVEIRA MORAIS </t>
         </is>
       </c>
       <c r="D3310" t="inlineStr">
         <is>
-          <t>MSCRUZ</t>
+          <t>KARINE28</t>
         </is>
       </c>
     </row>
     <row r="3311">
       <c r="A3311" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3311" t="n">
-        <v>3256</v>
+        <v>3446</v>
       </c>
       <c r="C3311" t="inlineStr">
         <is>
-          <t>ANNE CAROLINE ALMEIDA DE MORAIS</t>
+          <t>MARIA FERNANDA SOUSA DA CRUZ</t>
         </is>
       </c>
       <c r="D3311" t="inlineStr">
         <is>
-          <t>ACMORAIS</t>
+          <t>MSCRUZ</t>
         </is>
       </c>
     </row>
     <row r="3312">
       <c r="A3312" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3312" t="n">
-        <v>3257</v>
+        <v>3256</v>
       </c>
       <c r="C3312" t="inlineStr">
         <is>
-          <t xml:space="preserve"> NARA RAIANE RABELO NOBRE</t>
+          <t>ANNE CAROLINE ALMEIDA DE MORAIS</t>
         </is>
       </c>
       <c r="D3312" t="inlineStr">
         <is>
-          <t>NRNOBRE</t>
+          <t>ACMORAIS</t>
         </is>
       </c>
     </row>
     <row r="3313">
       <c r="A3313" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3313" t="n">
-        <v>3268</v>
+        <v>3257</v>
       </c>
       <c r="C3313" t="inlineStr">
         <is>
-          <t>DANRLEY PEREIRA E PEREIRA</t>
+          <t xml:space="preserve"> NARA RAIANE RABELO NOBRE</t>
         </is>
       </c>
       <c r="D3313" t="inlineStr">
         <is>
-          <t>DPEREIRA</t>
+          <t>NRNOBRE</t>
         </is>
       </c>
     </row>
@@ -66698,16 +66698,16 @@
         </is>
       </c>
       <c r="B3314" t="n">
-        <v>3282</v>
+        <v>3268</v>
       </c>
       <c r="C3314" t="inlineStr">
         <is>
-          <t xml:space="preserve">JARDSON ROBERTH CUTRIM SOUZA </t>
+          <t>DANRLEY PEREIRA E PEREIRA</t>
         </is>
       </c>
       <c r="D3314" t="inlineStr">
         <is>
-          <t>JRCSOUZA</t>
+          <t>DPEREIRA</t>
         </is>
       </c>
     </row>
@@ -66718,156 +66718,156 @@
         </is>
       </c>
       <c r="B3315" t="n">
-        <v>3283</v>
+        <v>3282</v>
       </c>
       <c r="C3315" t="inlineStr">
         <is>
-          <t>JESOAIAS DOS SANTOS CABRAL</t>
+          <t xml:space="preserve">JARDSON ROBERTH CUTRIM SOUZA </t>
         </is>
       </c>
       <c r="D3315" t="inlineStr">
         <is>
-          <t>JSCABRAL</t>
+          <t>JRCSOUZA</t>
         </is>
       </c>
     </row>
     <row r="3316">
       <c r="A3316" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3316" t="n">
-        <v>3299</v>
+        <v>3283</v>
       </c>
       <c r="C3316" t="inlineStr">
         <is>
-          <t>CARLOS EDUARDO ANDRADE DE ASSIS</t>
+          <t>JESOAIAS DOS SANTOS CABRAL</t>
         </is>
       </c>
       <c r="D3316" t="inlineStr">
         <is>
-          <t>ANDRADE</t>
+          <t>JSCABRAL</t>
         </is>
       </c>
     </row>
     <row r="3317">
       <c r="A3317" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3317" t="n">
-        <v>3301</v>
+        <v>3299</v>
       </c>
       <c r="C3317" t="inlineStr">
         <is>
-          <t>DIANA KARINE VIANA DA SILVA</t>
+          <t>CARLOS EDUARDO ANDRADE DE ASSIS</t>
         </is>
       </c>
       <c r="D3317" t="inlineStr">
         <is>
-          <t>DKVIANA</t>
+          <t>ANDRADE</t>
         </is>
       </c>
     </row>
     <row r="3318">
       <c r="A3318" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3318" t="n">
-        <v>940537</v>
+        <v>3301</v>
       </c>
       <c r="C3318" t="inlineStr">
         <is>
-          <t xml:space="preserve">TGC TRANSPORTES </t>
+          <t>DIANA KARINE VIANA DA SILVA</t>
         </is>
       </c>
       <c r="D3318" t="inlineStr">
         <is>
-          <t>TGC</t>
+          <t>DKVIANA</t>
         </is>
       </c>
     </row>
     <row r="3319">
       <c r="A3319" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3319" t="n">
-        <v>3343</v>
+        <v>940537</v>
       </c>
       <c r="C3319" t="inlineStr">
         <is>
-          <t>REGINALDO FEITOSA DA SILVA JUNIOR</t>
+          <t xml:space="preserve">TGC TRANSPORTES </t>
         </is>
       </c>
       <c r="D3319" t="inlineStr">
         <is>
-          <t>RFJUNIOR</t>
+          <t>TGC</t>
         </is>
       </c>
     </row>
     <row r="3320">
       <c r="A3320" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3320" t="n">
-        <v>3344</v>
+        <v>3343</v>
       </c>
       <c r="C3320" t="inlineStr">
         <is>
-          <t>JOAO VICTOR MENDONCA DA SILVA</t>
+          <t>REGINALDO FEITOSA DA SILVA JUNIOR</t>
         </is>
       </c>
       <c r="D3320" t="inlineStr">
         <is>
-          <t>JVMENDONCA</t>
+          <t>RFJUNIOR</t>
         </is>
       </c>
     </row>
     <row r="3321">
       <c r="A3321" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3321" t="n">
-        <v>3352</v>
+        <v>3344</v>
       </c>
       <c r="C3321" t="inlineStr">
         <is>
-          <t>RICARDO MACAUBAS BOAVENTURA</t>
+          <t>JOAO VICTOR MENDONCA DA SILVA</t>
         </is>
       </c>
       <c r="D3321" t="inlineStr">
         <is>
-          <t>RMACAUBAS</t>
+          <t>JVMENDONCA</t>
         </is>
       </c>
     </row>
     <row r="3322">
       <c r="A3322" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3322" t="n">
-        <v>3364</v>
+        <v>3352</v>
       </c>
       <c r="C3322" t="inlineStr">
         <is>
-          <t>CLOVIS VIDAL DOS SANTOS NETO</t>
+          <t>RICARDO MACAUBAS BOAVENTURA</t>
         </is>
       </c>
       <c r="D3322" t="inlineStr">
         <is>
-          <t>CVNETO</t>
+          <t>RMACAUBAS</t>
         </is>
       </c>
     </row>
@@ -66878,156 +66878,156 @@
         </is>
       </c>
       <c r="B3323" t="n">
-        <v>3365</v>
+        <v>3364</v>
       </c>
       <c r="C3323" t="inlineStr">
         <is>
-          <t>CYNTIA RAFAELLA DE PONTES</t>
+          <t>CLOVIS VIDAL DOS SANTOS NETO</t>
         </is>
       </c>
       <c r="D3323" t="inlineStr">
         <is>
-          <t>CRPONTES</t>
+          <t>CVNETO</t>
         </is>
       </c>
     </row>
     <row r="3324">
       <c r="A3324" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3324" t="n">
-        <v>3387</v>
+        <v>3365</v>
       </c>
       <c r="C3324" t="inlineStr">
         <is>
-          <t>VALDECI NASCIMENTO DELGADO JUNIOR</t>
+          <t>CYNTIA RAFAELLA DE PONTES</t>
         </is>
       </c>
       <c r="D3324" t="inlineStr">
         <is>
-          <t>VALDECI05</t>
+          <t>CRPONTES</t>
         </is>
       </c>
     </row>
     <row r="3325">
       <c r="A3325" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3325" t="n">
-        <v>3458</v>
+        <v>3387</v>
       </c>
       <c r="C3325" t="inlineStr">
         <is>
-          <t>EDUARDO BEZERRA DE SOUSA</t>
+          <t>VALDECI NASCIMENTO DELGADO JUNIOR</t>
         </is>
       </c>
       <c r="D3325" t="inlineStr">
         <is>
-          <t>EDUARDOB</t>
+          <t>VALDECI05</t>
         </is>
       </c>
     </row>
     <row r="3326">
       <c r="A3326" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3326" t="n">
-        <v>940561</v>
+        <v>3458</v>
       </c>
       <c r="C3326" t="inlineStr">
         <is>
-          <t>NAIRTON DE ARAUJO MONTEIRO</t>
+          <t>EDUARDO BEZERRA DE SOUSA</t>
         </is>
       </c>
       <c r="D3326" t="inlineStr">
         <is>
-          <t>NAIRTON</t>
+          <t>EDUARDOB</t>
         </is>
       </c>
     </row>
     <row r="3327">
       <c r="A3327" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>99</t>
         </is>
       </c>
       <c r="B3327" t="n">
-        <v>3515</v>
+        <v>940561</v>
       </c>
       <c r="C3327" t="inlineStr">
         <is>
-          <t>DANIEL DOS SANTOS DE ALMEIDA</t>
+          <t>NAIRTON DE ARAUJO MONTEIRO</t>
         </is>
       </c>
       <c r="D3327" t="inlineStr">
         <is>
-          <t>DANIELSA</t>
+          <t>NAIRTON</t>
         </is>
       </c>
     </row>
     <row r="3328">
       <c r="A3328" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3328" t="n">
-        <v>3288</v>
+        <v>3515</v>
       </c>
       <c r="C3328" t="inlineStr">
         <is>
-          <t>ANA MARIA AMORIM MENDONÇA</t>
+          <t>DANIEL DOS SANTOS DE ALMEIDA</t>
         </is>
       </c>
       <c r="D3328" t="inlineStr">
         <is>
-          <t>AMENDONCA</t>
+          <t>DANIELSA</t>
         </is>
       </c>
     </row>
     <row r="3329">
       <c r="A3329" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3329" t="n">
-        <v>3312</v>
+        <v>3288</v>
       </c>
       <c r="C3329" t="inlineStr">
         <is>
-          <t>AURIANA LIMA DE MORAES</t>
+          <t>ANA MARIA AMORIM MENDONÇA</t>
         </is>
       </c>
       <c r="D3329" t="inlineStr">
         <is>
-          <t>ALM</t>
+          <t>AMENDONCA</t>
         </is>
       </c>
     </row>
     <row r="3330">
       <c r="A3330" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3330" t="n">
-        <v>940547</v>
+        <v>3312</v>
       </c>
       <c r="C3330" t="inlineStr">
         <is>
-          <t>JM EXPRESS - AGRESTE</t>
+          <t>AURIANA LIMA DE MORAES</t>
         </is>
       </c>
       <c r="D3330" t="inlineStr">
         <is>
-          <t>J M A</t>
+          <t>ALM</t>
         </is>
       </c>
     </row>
@@ -67038,76 +67038,76 @@
         </is>
       </c>
       <c r="B3331" t="n">
-        <v>940548</v>
+        <v>940547</v>
       </c>
       <c r="C3331" t="inlineStr">
         <is>
-          <t>JM EXPRESS - SERTAO</t>
+          <t>JM EXPRESS - AGRESTE</t>
         </is>
       </c>
       <c r="D3331" t="inlineStr">
         <is>
-          <t>J M S</t>
+          <t>J M A</t>
         </is>
       </c>
     </row>
     <row r="3332">
       <c r="A3332" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3332" t="n">
-        <v>940551</v>
+        <v>940548</v>
       </c>
       <c r="C3332" t="inlineStr">
         <is>
-          <t>LUCAS PONTES NOBRE</t>
+          <t>JM EXPRESS - SERTAO</t>
         </is>
       </c>
       <c r="D3332" t="inlineStr">
         <is>
-          <t>PONTES</t>
+          <t>J M S</t>
         </is>
       </c>
     </row>
     <row r="3333">
       <c r="A3333" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>99</t>
         </is>
       </c>
       <c r="B3333" t="n">
-        <v>3382</v>
+        <v>940551</v>
       </c>
       <c r="C3333" t="inlineStr">
         <is>
-          <t>MARIA CASSILANIA SOUSA DO NASCIMENTO</t>
+          <t>LUCAS PONTES NOBRE</t>
         </is>
       </c>
       <c r="D3333" t="inlineStr">
         <is>
-          <t>MCASSILANIA</t>
+          <t>PONTES</t>
         </is>
       </c>
     </row>
     <row r="3334">
       <c r="A3334" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3334" t="n">
-        <v>3474</v>
+        <v>3382</v>
       </c>
       <c r="C3334" t="inlineStr">
         <is>
-          <t>MARCOS VINICIUS GONCALVES MIRANDA</t>
+          <t>MARIA CASSILANIA SOUSA DO NASCIMENTO</t>
         </is>
       </c>
       <c r="D3334" t="inlineStr">
         <is>
-          <t>MARCOS.VINICIUS</t>
+          <t>MCASSILANIA</t>
         </is>
       </c>
     </row>
@@ -67118,176 +67118,176 @@
         </is>
       </c>
       <c r="B3335" t="n">
-        <v>3523</v>
+        <v>3474</v>
       </c>
       <c r="C3335" t="inlineStr">
         <is>
-          <t>ORLANDO RICARDO SANTOS ANDRADE</t>
+          <t>MARCOS VINICIUS GONCALVES MIRANDA</t>
         </is>
       </c>
       <c r="D3335" t="inlineStr">
         <is>
-          <t>ORLANDOR</t>
+          <t>MARCOS.VINICIUS</t>
         </is>
       </c>
     </row>
     <row r="3336">
       <c r="A3336" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3336" t="n">
-        <v>3566</v>
+        <v>3523</v>
       </c>
       <c r="C3336" t="inlineStr">
         <is>
-          <t xml:space="preserve">WESLEY HENRIQUE ALVES DOS SANTOS </t>
+          <t>ORLANDO RICARDO SANTOS ANDRADE</t>
         </is>
       </c>
       <c r="D3336" t="inlineStr">
         <is>
-          <t>W.ALVES</t>
+          <t>ORLANDOR</t>
         </is>
       </c>
     </row>
     <row r="3337">
       <c r="A3337" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3337" t="n">
-        <v>3573</v>
+        <v>3566</v>
       </c>
       <c r="C3337" t="inlineStr">
         <is>
-          <t>GABRIEL DA SILVA MENDES</t>
+          <t xml:space="preserve">WESLEY HENRIQUE ALVES DOS SANTOS </t>
         </is>
       </c>
       <c r="D3337" t="inlineStr">
         <is>
-          <t>GMENDES</t>
+          <t>W.ALVES</t>
         </is>
       </c>
     </row>
     <row r="3338">
       <c r="A3338" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3338" t="n">
-        <v>940541</v>
+        <v>3573</v>
       </c>
       <c r="C3338" t="inlineStr">
         <is>
-          <t>JOSE AMSTERDA TEIXEIRA DE MENEZES</t>
+          <t>GABRIEL DA SILVA MENDES</t>
         </is>
       </c>
       <c r="D3338" t="inlineStr">
         <is>
-          <t>AMSTERDA</t>
+          <t>GMENDES</t>
         </is>
       </c>
     </row>
     <row r="3339">
       <c r="A3339" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>99</t>
         </is>
       </c>
       <c r="B3339" t="n">
-        <v>940554</v>
+        <v>940541</v>
       </c>
       <c r="C3339" t="inlineStr">
         <is>
-          <t>ALEXANDRE ALVES DE FREITAS</t>
+          <t>JOSE AMSTERDA TEIXEIRA DE MENEZES</t>
         </is>
       </c>
       <c r="D3339" t="inlineStr">
         <is>
-          <t>ALEXANDRE</t>
+          <t>AMSTERDA</t>
         </is>
       </c>
     </row>
     <row r="3340">
       <c r="A3340" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3340" t="n">
-        <v>3402</v>
+        <v>940554</v>
       </c>
       <c r="C3340" t="inlineStr">
         <is>
-          <t xml:space="preserve">VINICIUS GUEDES DA SILVA </t>
+          <t>ALEXANDRE ALVES DE FREITAS</t>
         </is>
       </c>
       <c r="D3340" t="inlineStr">
         <is>
-          <t>GUEDES5</t>
+          <t>ALEXANDRE</t>
         </is>
       </c>
     </row>
     <row r="3341">
       <c r="A3341" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3341" t="n">
-        <v>3467</v>
+        <v>3402</v>
       </c>
       <c r="C3341" t="inlineStr">
         <is>
-          <t>CILENE FERREIRA DA SILVA</t>
+          <t xml:space="preserve">VINICIUS GUEDES DA SILVA </t>
         </is>
       </c>
       <c r="D3341" t="inlineStr">
         <is>
-          <t>CILENE</t>
+          <t>GUEDES5</t>
         </is>
       </c>
     </row>
     <row r="3342">
       <c r="A3342" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3342" t="n">
-        <v>3495</v>
+        <v>3467</v>
       </c>
       <c r="C3342" t="inlineStr">
         <is>
-          <t>LUCILENE SANTOS DE MELO DAMASCENA</t>
+          <t>CILENE FERREIRA DA SILVA</t>
         </is>
       </c>
       <c r="D3342" t="inlineStr">
         <is>
-          <t>LUCILENE21</t>
+          <t>CILENE</t>
         </is>
       </c>
     </row>
     <row r="3343">
       <c r="A3343" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3343" t="n">
-        <v>3496</v>
+        <v>3495</v>
       </c>
       <c r="C3343" t="inlineStr">
         <is>
-          <t>JOAO PEDRO HENRIQUE ALVES DE ARAUJO</t>
+          <t>LUCILENE SANTOS DE MELO DAMASCENA</t>
         </is>
       </c>
       <c r="D3343" t="inlineStr">
         <is>
-          <t>JOAO.PEDRO</t>
+          <t>LUCILENE21</t>
         </is>
       </c>
     </row>
@@ -67298,16 +67298,16 @@
         </is>
       </c>
       <c r="B3344" t="n">
-        <v>3497</v>
+        <v>3496</v>
       </c>
       <c r="C3344" t="inlineStr">
         <is>
-          <t>ORLANDO MONTEIRO DE AMORIM</t>
+          <t>JOAO PEDRO HENRIQUE ALVES DE ARAUJO</t>
         </is>
       </c>
       <c r="D3344" t="inlineStr">
         <is>
-          <t>ORLANDO</t>
+          <t>JOAO.PEDRO</t>
         </is>
       </c>
     </row>
@@ -67318,156 +67318,156 @@
         </is>
       </c>
       <c r="B3345" t="n">
-        <v>3538</v>
+        <v>3497</v>
       </c>
       <c r="C3345" t="inlineStr">
         <is>
-          <t>PAULO HENRIQUE BENTO DA SILVA</t>
+          <t>ORLANDO MONTEIRO DE AMORIM</t>
         </is>
       </c>
       <c r="D3345" t="inlineStr">
         <is>
-          <t>P.BENTO</t>
+          <t>ORLANDO</t>
         </is>
       </c>
     </row>
     <row r="3346">
       <c r="A3346" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3346" t="n">
-        <v>3577</v>
+        <v>3538</v>
       </c>
       <c r="C3346" t="inlineStr">
         <is>
-          <t>NEGOCIACAO PI</t>
+          <t>PAULO HENRIQUE BENTO DA SILVA</t>
         </is>
       </c>
       <c r="D3346" t="inlineStr">
         <is>
-          <t>NEGOCIACAOPI</t>
+          <t>P.BENTO</t>
         </is>
       </c>
     </row>
     <row r="3347">
       <c r="A3347" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3347" t="n">
-        <v>3578</v>
+        <v>3577</v>
       </c>
       <c r="C3347" t="inlineStr">
         <is>
-          <t>NEGOCIACAO MA</t>
+          <t>NEGOCIACAO PI</t>
         </is>
       </c>
       <c r="D3347" t="inlineStr">
         <is>
-          <t>NEGOCIACAOMA</t>
+          <t>NEGOCIACAOPI</t>
         </is>
       </c>
     </row>
     <row r="3348">
       <c r="A3348" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3348" t="n">
-        <v>3303</v>
+        <v>3578</v>
       </c>
       <c r="C3348" t="inlineStr">
         <is>
-          <t>DANIEL ALVES RODRIGUES</t>
+          <t>NEGOCIACAO MA</t>
         </is>
       </c>
       <c r="D3348" t="inlineStr">
         <is>
-          <t>DARODRIGUES</t>
+          <t>NEGOCIACAOMA</t>
         </is>
       </c>
     </row>
     <row r="3349">
       <c r="A3349" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3349" t="n">
-        <v>3316</v>
+        <v>3303</v>
       </c>
       <c r="C3349" t="inlineStr">
         <is>
-          <t xml:space="preserve">MARCELO PEREIRA BASTOS </t>
+          <t>DANIEL ALVES RODRIGUES</t>
         </is>
       </c>
       <c r="D3349" t="inlineStr">
         <is>
-          <t>MBASTOS</t>
+          <t>DARODRIGUES</t>
         </is>
       </c>
     </row>
     <row r="3350">
       <c r="A3350" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3350" t="n">
-        <v>3366</v>
+        <v>3316</v>
       </c>
       <c r="C3350" t="inlineStr">
         <is>
-          <t>MATEUS TEIXEIRA DA PAZ SILVA</t>
+          <t xml:space="preserve">MARCELO PEREIRA BASTOS </t>
         </is>
       </c>
       <c r="D3350" t="inlineStr">
         <is>
-          <t>PAZSILVA</t>
+          <t>MBASTOS</t>
         </is>
       </c>
     </row>
     <row r="3351">
       <c r="A3351" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3351" t="n">
-        <v>3393</v>
+        <v>3366</v>
       </c>
       <c r="C3351" t="inlineStr">
         <is>
-          <t xml:space="preserve">DAVID LUCAS RIBEIRO DOS SANTOS </t>
+          <t>MATEUS TEIXEIRA DA PAZ SILVA</t>
         </is>
       </c>
       <c r="D3351" t="inlineStr">
         <is>
-          <t>DLUCAS</t>
+          <t>PAZSILVA</t>
         </is>
       </c>
     </row>
     <row r="3352">
       <c r="A3352" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3352" t="n">
-        <v>3420</v>
+        <v>3393</v>
       </c>
       <c r="C3352" t="inlineStr">
         <is>
-          <t xml:space="preserve">CLAUDIO ROBERTO SILVA SOUZA </t>
+          <t xml:space="preserve">DAVID LUCAS RIBEIRO DOS SANTOS </t>
         </is>
       </c>
       <c r="D3352" t="inlineStr">
         <is>
-          <t>CLAUDIO21</t>
+          <t>DLUCAS</t>
         </is>
       </c>
     </row>
@@ -67478,16 +67478,16 @@
         </is>
       </c>
       <c r="B3353" t="n">
-        <v>3421</v>
+        <v>3420</v>
       </c>
       <c r="C3353" t="inlineStr">
         <is>
-          <t>WILSON PORTUGAL AZEVEDO FILHO</t>
+          <t xml:space="preserve">CLAUDIO ROBERTO SILVA SOUZA </t>
         </is>
       </c>
       <c r="D3353" t="inlineStr">
         <is>
-          <t>WILSONF</t>
+          <t>CLAUDIO21</t>
         </is>
       </c>
     </row>
@@ -67498,176 +67498,176 @@
         </is>
       </c>
       <c r="B3354" t="n">
-        <v>3439</v>
+        <v>3421</v>
       </c>
       <c r="C3354" t="inlineStr">
         <is>
-          <t>FERNANDA MASCARENHAS CEDRAZ</t>
+          <t>WILSON PORTUGAL AZEVEDO FILHO</t>
         </is>
       </c>
       <c r="D3354" t="inlineStr">
         <is>
-          <t>FERNANDAM</t>
+          <t>WILSONF</t>
         </is>
       </c>
     </row>
     <row r="3355">
       <c r="A3355" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3355" t="n">
-        <v>3455</v>
+        <v>3439</v>
       </c>
       <c r="C3355" t="inlineStr">
         <is>
-          <t xml:space="preserve">MARDONIO CUNHA BASILIO </t>
+          <t>FERNANDA MASCARENHAS CEDRAZ</t>
         </is>
       </c>
       <c r="D3355" t="inlineStr">
         <is>
-          <t>MARDONIO1</t>
+          <t>FERNANDAM</t>
         </is>
       </c>
     </row>
     <row r="3356">
       <c r="A3356" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3356" t="n">
-        <v>3508</v>
+        <v>3455</v>
       </c>
       <c r="C3356" t="inlineStr">
         <is>
-          <t>REBECA PIRES DE SOUZA MELO</t>
+          <t xml:space="preserve">MARDONIO CUNHA BASILIO </t>
         </is>
       </c>
       <c r="D3356" t="inlineStr">
         <is>
-          <t>RPMELO</t>
+          <t>MARDONIO1</t>
         </is>
       </c>
     </row>
     <row r="3357">
       <c r="A3357" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3357" t="n">
-        <v>3543</v>
+        <v>3508</v>
       </c>
       <c r="C3357" t="inlineStr">
         <is>
-          <t>JOAO GABRIEL BARBOSA FIRMINO</t>
+          <t>REBECA PIRES DE SOUZA MELO</t>
         </is>
       </c>
       <c r="D3357" t="inlineStr">
         <is>
-          <t>JOAOG</t>
+          <t>RPMELO</t>
         </is>
       </c>
     </row>
     <row r="3358">
       <c r="A3358" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3358" t="n">
-        <v>3580</v>
+        <v>3543</v>
       </c>
       <c r="C3358" t="inlineStr">
         <is>
-          <t>ALEXANDRE MARTINS CHAVES</t>
+          <t>JOAO GABRIEL BARBOSA FIRMINO</t>
         </is>
       </c>
       <c r="D3358" t="inlineStr">
         <is>
-          <t>MARTINS</t>
+          <t>JOAOG</t>
         </is>
       </c>
     </row>
     <row r="3359">
       <c r="A3359" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3359" t="n">
-        <v>3351</v>
+        <v>3580</v>
       </c>
       <c r="C3359" t="inlineStr">
         <is>
-          <t>HAWLLYSON DA SILVA COUTINHO</t>
+          <t>ALEXANDRE MARTINS CHAVES</t>
         </is>
       </c>
       <c r="D3359" t="inlineStr">
         <is>
-          <t>HCOUTINHO</t>
+          <t>MARTINS</t>
         </is>
       </c>
     </row>
     <row r="3360">
       <c r="A3360" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3360" t="n">
-        <v>940553</v>
+        <v>3351</v>
       </c>
       <c r="C3360" t="inlineStr">
         <is>
-          <t>LUTY TRANSPORTES- BA</t>
+          <t>HAWLLYSON DA SILVA COUTINHO</t>
         </is>
       </c>
       <c r="D3360" t="inlineStr">
         <is>
-          <t>LUTY TRANSPORTE</t>
+          <t>HCOUTINHO</t>
         </is>
       </c>
     </row>
     <row r="3361">
       <c r="A3361" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3361" t="n">
-        <v>3391</v>
+        <v>940553</v>
       </c>
       <c r="C3361" t="inlineStr">
         <is>
-          <t xml:space="preserve">NIKSON DA SILVA ALVES </t>
+          <t>LUTY TRANSPORTES- BA</t>
         </is>
       </c>
       <c r="D3361" t="inlineStr">
         <is>
-          <t>NIKSON</t>
+          <t>LUTY TRANSPORTE</t>
         </is>
       </c>
     </row>
     <row r="3362">
       <c r="A3362" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3362" t="n">
-        <v>3397</v>
+        <v>3391</v>
       </c>
       <c r="C3362" t="inlineStr">
         <is>
-          <t>EDILANE MENESES BALTAZAR</t>
+          <t xml:space="preserve">NIKSON DA SILVA ALVES </t>
         </is>
       </c>
       <c r="D3362" t="inlineStr">
         <is>
-          <t>EDILANE</t>
+          <t>NIKSON</t>
         </is>
       </c>
     </row>
@@ -67678,56 +67678,56 @@
         </is>
       </c>
       <c r="B3363" t="n">
-        <v>3398</v>
+        <v>3397</v>
       </c>
       <c r="C3363" t="inlineStr">
         <is>
-          <t>LUANA MARIA ROSIO DA SILVA</t>
+          <t>EDILANE MENESES BALTAZAR</t>
         </is>
       </c>
       <c r="D3363" t="inlineStr">
         <is>
-          <t>LUMARIA</t>
+          <t>EDILANE</t>
         </is>
       </c>
     </row>
     <row r="3364">
       <c r="A3364" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3364" t="n">
-        <v>3400</v>
+        <v>3398</v>
       </c>
       <c r="C3364" t="inlineStr">
         <is>
-          <t>ELILTON PINTO ROMEU</t>
+          <t>LUANA MARIA ROSIO DA SILVA</t>
         </is>
       </c>
       <c r="D3364" t="inlineStr">
         <is>
-          <t>ELILTON</t>
+          <t>LUMARIA</t>
         </is>
       </c>
     </row>
     <row r="3365">
       <c r="A3365" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3365" t="n">
-        <v>3406</v>
+        <v>3400</v>
       </c>
       <c r="C3365" t="inlineStr">
         <is>
-          <t>CONEXAO ALDA</t>
+          <t>ELILTON PINTO ROMEU</t>
         </is>
       </c>
       <c r="D3365" t="inlineStr">
         <is>
-          <t>CONEXAOALDA</t>
+          <t>ELILTON</t>
         </is>
       </c>
     </row>
@@ -67738,176 +67738,176 @@
         </is>
       </c>
       <c r="B3366" t="n">
-        <v>3407</v>
+        <v>3406</v>
       </c>
       <c r="C3366" t="inlineStr">
         <is>
-          <t>CONEXAO IRACEMA</t>
+          <t>CONEXAO ALDA</t>
         </is>
       </c>
       <c r="D3366" t="inlineStr">
         <is>
-          <t>CONEXAOIRACEMA</t>
+          <t>CONEXAOALDA</t>
         </is>
       </c>
     </row>
     <row r="3367">
       <c r="A3367" t="inlineStr">
         <is>
-          <t>9999</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3367" t="n">
-        <v>3408</v>
+        <v>3407</v>
       </c>
       <c r="C3367" t="inlineStr">
         <is>
-          <t>CONEXAO TAMILES</t>
+          <t>CONEXAO IRACEMA</t>
         </is>
       </c>
       <c r="D3367" t="inlineStr">
         <is>
-          <t>CONEXAOTAMILES</t>
+          <t>CONEXAOIRACEMA</t>
         </is>
       </c>
     </row>
     <row r="3368">
       <c r="A3368" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>9999</t>
         </is>
       </c>
       <c r="B3368" t="n">
-        <v>3414</v>
+        <v>3408</v>
       </c>
       <c r="C3368" t="inlineStr">
         <is>
-          <t>CONEXAO ADM PI MA</t>
+          <t>CONEXAO TAMILES</t>
         </is>
       </c>
       <c r="D3368" t="inlineStr">
         <is>
-          <t>CONEXAOPIMA</t>
+          <t>CONEXAOTAMILES</t>
         </is>
       </c>
     </row>
     <row r="3369">
       <c r="A3369" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3369" t="n">
-        <v>3524</v>
+        <v>3414</v>
       </c>
       <c r="C3369" t="inlineStr">
         <is>
-          <t>LUIS FELIPE DA SILVA SOUSA</t>
+          <t>CONEXAO ADM PI MA</t>
         </is>
       </c>
       <c r="D3369" t="inlineStr">
         <is>
-          <t>L.FELIPE</t>
+          <t>CONEXAOPIMA</t>
         </is>
       </c>
     </row>
     <row r="3370">
       <c r="A3370" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3370" t="n">
-        <v>3531</v>
+        <v>3524</v>
       </c>
       <c r="C3370" t="inlineStr">
         <is>
-          <t>LEICIANE COELHO SILVA</t>
+          <t>LUIS FELIPE DA SILVA SOUSA</t>
         </is>
       </c>
       <c r="D3370" t="inlineStr">
         <is>
-          <t>LEI.SILVA</t>
+          <t>L.FELIPE</t>
         </is>
       </c>
     </row>
     <row r="3371">
       <c r="A3371" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3371" t="n">
-        <v>3550</v>
+        <v>3531</v>
       </c>
       <c r="C3371" t="inlineStr">
         <is>
-          <t>IARGO GABRIEL SANTOS DE OLIVEIRA</t>
+          <t>LEICIANE COELHO SILVA</t>
         </is>
       </c>
       <c r="D3371" t="inlineStr">
         <is>
-          <t>IARGOG</t>
+          <t>LEI.SILVA</t>
         </is>
       </c>
     </row>
     <row r="3372">
       <c r="A3372" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3372" t="n">
-        <v>940567</v>
+        <v>3550</v>
       </c>
       <c r="C3372" t="inlineStr">
         <is>
-          <t>MS CARGAS E TRANSPORTES</t>
+          <t>IARGO GABRIEL SANTOS DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D3372" t="inlineStr">
         <is>
-          <t>ALAN BARBOSA</t>
+          <t>IARGOG</t>
         </is>
       </c>
     </row>
     <row r="3373">
       <c r="A3373" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3373" t="n">
-        <v>3560</v>
+        <v>940567</v>
       </c>
       <c r="C3373" t="inlineStr">
         <is>
-          <t>MARIA EDUARDA MELO DOS SANTOS</t>
+          <t>MS CARGAS E TRANSPORTES</t>
         </is>
       </c>
       <c r="D3373" t="inlineStr">
         <is>
-          <t>EDU.MELO</t>
+          <t>ALAN BARBOSA</t>
         </is>
       </c>
     </row>
     <row r="3374">
       <c r="A3374" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3374" t="n">
-        <v>3355</v>
+        <v>3560</v>
       </c>
       <c r="C3374" t="inlineStr">
         <is>
-          <t>HUGO MATHEUS DA COSTA FEITOSA</t>
+          <t>MARIA EDUARDA MELO DOS SANTOS</t>
         </is>
       </c>
       <c r="D3374" t="inlineStr">
         <is>
-          <t>HMFEITOSA</t>
+          <t>EDU.MELO</t>
         </is>
       </c>
     </row>
@@ -67918,96 +67918,96 @@
         </is>
       </c>
       <c r="B3375" t="n">
-        <v>3356</v>
+        <v>3355</v>
       </c>
       <c r="C3375" t="inlineStr">
         <is>
-          <t>BRENDA LIMA DE OLIVEIRA CUNHA</t>
+          <t>HUGO MATHEUS DA COSTA FEITOSA</t>
         </is>
       </c>
       <c r="D3375" t="inlineStr">
         <is>
-          <t>BLCUNHA</t>
+          <t>HMFEITOSA</t>
         </is>
       </c>
     </row>
     <row r="3376">
       <c r="A3376" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3376" t="n">
-        <v>3361</v>
+        <v>3356</v>
       </c>
       <c r="C3376" t="inlineStr">
         <is>
-          <t>WLADIA DE ARAUJO BASTOS</t>
+          <t>BRENDA LIMA DE OLIVEIRA CUNHA</t>
         </is>
       </c>
       <c r="D3376" t="inlineStr">
         <is>
-          <t>WABASTOS</t>
+          <t>BLCUNHA</t>
         </is>
       </c>
     </row>
     <row r="3377">
       <c r="A3377" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3377" t="n">
-        <v>3362</v>
+        <v>3361</v>
       </c>
       <c r="C3377" t="inlineStr">
         <is>
-          <t>CARLOS HENRIQUE MELO DA SILVA</t>
+          <t>WLADIA DE ARAUJO BASTOS</t>
         </is>
       </c>
       <c r="D3377" t="inlineStr">
         <is>
-          <t>CHMELO</t>
+          <t>WABASTOS</t>
         </is>
       </c>
     </row>
     <row r="3378">
       <c r="A3378" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3378" t="n">
-        <v>3375</v>
+        <v>3362</v>
       </c>
       <c r="C3378" t="inlineStr">
         <is>
-          <t>AFONSO DE SOUSA RAMOS FILHO</t>
+          <t>CARLOS HENRIQUE MELO DA SILVA</t>
         </is>
       </c>
       <c r="D3378" t="inlineStr">
         <is>
-          <t>AFILHO</t>
+          <t>CHMELO</t>
         </is>
       </c>
     </row>
     <row r="3379">
       <c r="A3379" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3379" t="n">
-        <v>3404</v>
+        <v>3375</v>
       </c>
       <c r="C3379" t="inlineStr">
         <is>
-          <t>NOVATO 4 COM</t>
+          <t>AFONSO DE SOUSA RAMOS FILHO</t>
         </is>
       </c>
       <c r="D3379" t="inlineStr">
         <is>
-          <t>NOVATO4COM</t>
+          <t>AFILHO</t>
         </is>
       </c>
     </row>
@@ -68018,176 +68018,176 @@
         </is>
       </c>
       <c r="B3380" t="n">
-        <v>3405</v>
+        <v>3404</v>
       </c>
       <c r="C3380" t="inlineStr">
         <is>
-          <t>NOVATO 5 COM</t>
+          <t>NOVATO 4 COM</t>
         </is>
       </c>
       <c r="D3380" t="inlineStr">
         <is>
-          <t>NOVATO5COM</t>
+          <t>NOVATO4COM</t>
         </is>
       </c>
     </row>
     <row r="3381">
       <c r="A3381" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3381" t="n">
-        <v>3447</v>
+        <v>3405</v>
       </c>
       <c r="C3381" t="inlineStr">
         <is>
-          <t>RAYSSA KEYCE LINHARES AQUINO</t>
+          <t>NOVATO 5 COM</t>
         </is>
       </c>
       <c r="D3381" t="inlineStr">
         <is>
-          <t>RAYSSAK</t>
+          <t>NOVATO5COM</t>
         </is>
       </c>
     </row>
     <row r="3382">
       <c r="A3382" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3382" t="n">
-        <v>940559</v>
+        <v>3447</v>
       </c>
       <c r="C3382" t="inlineStr">
         <is>
-          <t>WALLEF DE OLIVEIRA</t>
+          <t>RAYSSA KEYCE LINHARES AQUINO</t>
         </is>
       </c>
       <c r="D3382" t="inlineStr">
         <is>
-          <t>WALLEF</t>
+          <t>RAYSSAK</t>
         </is>
       </c>
     </row>
     <row r="3383">
       <c r="A3383" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>99</t>
         </is>
       </c>
       <c r="B3383" t="n">
-        <v>3489</v>
+        <v>940559</v>
       </c>
       <c r="C3383" t="inlineStr">
         <is>
-          <t>MARCELA KARINA PEREIRA VELOSO</t>
+          <t>WALLEF DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D3383" t="inlineStr">
         <is>
-          <t>MKARINA</t>
+          <t>WALLEF</t>
         </is>
       </c>
     </row>
     <row r="3384">
       <c r="A3384" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3384" t="n">
-        <v>3490</v>
+        <v>3489</v>
       </c>
       <c r="C3384" t="inlineStr">
         <is>
-          <t>JOSE MAILSON GOMES NUNES</t>
+          <t>MARCELA KARINA PEREIRA VELOSO</t>
         </is>
       </c>
       <c r="D3384" t="inlineStr">
         <is>
-          <t>J.MAILSON</t>
+          <t>MKARINA</t>
         </is>
       </c>
     </row>
     <row r="3385">
       <c r="A3385" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3385" t="n">
-        <v>3537</v>
+        <v>3490</v>
       </c>
       <c r="C3385" t="inlineStr">
         <is>
-          <t>ALDAIR PEDRO DA SILVA</t>
+          <t>JOSE MAILSON GOMES NUNES</t>
         </is>
       </c>
       <c r="D3385" t="inlineStr">
         <is>
-          <t>A.PEDRO</t>
+          <t>J.MAILSON</t>
         </is>
       </c>
     </row>
     <row r="3386">
       <c r="A3386" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3386" t="n">
-        <v>3549</v>
+        <v>3537</v>
       </c>
       <c r="C3386" t="inlineStr">
         <is>
-          <t xml:space="preserve">FERNANDA CAROLINE E CESAR SOUSA </t>
+          <t>ALDAIR PEDRO DA SILVA</t>
         </is>
       </c>
       <c r="D3386" t="inlineStr">
         <is>
-          <t>FCAROLINE</t>
+          <t>A.PEDRO</t>
         </is>
       </c>
     </row>
     <row r="3387">
       <c r="A3387" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3387" t="n">
-        <v>3581</v>
+        <v>3549</v>
       </c>
       <c r="C3387" t="inlineStr">
         <is>
-          <t xml:space="preserve">VALQUIRIO OLIVEIRA SOUSA </t>
+          <t xml:space="preserve">FERNANDA CAROLINE E CESAR SOUSA </t>
         </is>
       </c>
       <c r="D3387" t="inlineStr">
         <is>
-          <t>VALQUIRIO</t>
+          <t>FCAROLINE</t>
         </is>
       </c>
     </row>
     <row r="3388">
       <c r="A3388" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3388" t="n">
-        <v>3337</v>
+        <v>3581</v>
       </c>
       <c r="C3388" t="inlineStr">
         <is>
-          <t>WESLEY FONTES DE ALMEIDA</t>
+          <t xml:space="preserve">VALQUIRIO OLIVEIRA SOUSA </t>
         </is>
       </c>
       <c r="D3388" t="inlineStr">
         <is>
-          <t>WFALMEIDA</t>
+          <t>VALQUIRIO</t>
         </is>
       </c>
     </row>
@@ -68198,16 +68198,16 @@
         </is>
       </c>
       <c r="B3389" t="n">
-        <v>3338</v>
+        <v>3337</v>
       </c>
       <c r="C3389" t="inlineStr">
         <is>
-          <t>FRANCISCA SAMARA MENDES DE OLIVEIRA C</t>
+          <t>WESLEY FONTES DE ALMEIDA</t>
         </is>
       </c>
       <c r="D3389" t="inlineStr">
         <is>
-          <t>FSCUNHA</t>
+          <t>WFALMEIDA</t>
         </is>
       </c>
     </row>
@@ -68218,176 +68218,176 @@
         </is>
       </c>
       <c r="B3390" t="n">
-        <v>3339</v>
+        <v>3338</v>
       </c>
       <c r="C3390" t="inlineStr">
         <is>
-          <t>MAYARA THALYA DIAS DE ANDRADE</t>
+          <t>FRANCISCA SAMARA MENDES DE OLIVEIRA C</t>
         </is>
       </c>
       <c r="D3390" t="inlineStr">
         <is>
-          <t>MTANDRADE</t>
+          <t>FSCUNHA</t>
         </is>
       </c>
     </row>
     <row r="3391">
       <c r="A3391" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3391" t="n">
-        <v>3359</v>
+        <v>3339</v>
       </c>
       <c r="C3391" t="inlineStr">
         <is>
-          <t xml:space="preserve">EVANESSA DA SILVA E SILVA </t>
+          <t>MAYARA THALYA DIAS DE ANDRADE</t>
         </is>
       </c>
       <c r="D3391" t="inlineStr">
         <is>
-          <t>EVANESSAS</t>
+          <t>MTANDRADE</t>
         </is>
       </c>
     </row>
     <row r="3392">
       <c r="A3392" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3392" t="n">
-        <v>3360</v>
+        <v>3359</v>
       </c>
       <c r="C3392" t="inlineStr">
         <is>
-          <t>THIAGO DE CARVALHO ARAUJO</t>
+          <t xml:space="preserve">EVANESSA DA SILVA E SILVA </t>
         </is>
       </c>
       <c r="D3392" t="inlineStr">
         <is>
-          <t>TCARAUJO</t>
+          <t>EVANESSAS</t>
         </is>
       </c>
     </row>
     <row r="3393">
       <c r="A3393" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3393" t="n">
-        <v>3481</v>
+        <v>3360</v>
       </c>
       <c r="C3393" t="inlineStr">
         <is>
-          <t xml:space="preserve">EDSON DA PAZ LIMA </t>
+          <t>THIAGO DE CARVALHO ARAUJO</t>
         </is>
       </c>
       <c r="D3393" t="inlineStr">
         <is>
-          <t>EDPAZ</t>
+          <t>TCARAUJO</t>
         </is>
       </c>
     </row>
     <row r="3394">
       <c r="A3394" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3394" t="n">
-        <v>3494</v>
+        <v>3481</v>
       </c>
       <c r="C3394" t="inlineStr">
         <is>
-          <t>ANTONIO CRISTINA BRITO GOMES</t>
+          <t xml:space="preserve">EDSON DA PAZ LIMA </t>
         </is>
       </c>
       <c r="D3394" t="inlineStr">
         <is>
-          <t>CRIS.GOMES</t>
+          <t>EDPAZ</t>
         </is>
       </c>
     </row>
     <row r="3395">
       <c r="A3395" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3395" t="n">
-        <v>3498</v>
+        <v>3494</v>
       </c>
       <c r="C3395" t="inlineStr">
         <is>
-          <t>SILVESTRA COSTA NUNES</t>
+          <t>ANTONIO CRISTINA BRITO GOMES</t>
         </is>
       </c>
       <c r="D3395" t="inlineStr">
         <is>
-          <t>SCNUNES</t>
+          <t>CRIS.GOMES</t>
         </is>
       </c>
     </row>
     <row r="3396">
       <c r="A3396" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3396" t="n">
-        <v>940562</v>
+        <v>3498</v>
       </c>
       <c r="C3396" t="inlineStr">
         <is>
-          <t>FRANCISCO DAVID ASSUNCAO ALVES</t>
+          <t>SILVESTRA COSTA NUNES</t>
         </is>
       </c>
       <c r="D3396" t="inlineStr">
         <is>
-          <t>ASSUNÇÃO</t>
+          <t>SCNUNES</t>
         </is>
       </c>
     </row>
     <row r="3397">
       <c r="A3397" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>99</t>
         </is>
       </c>
       <c r="B3397" t="n">
-        <v>3513</v>
+        <v>940562</v>
       </c>
       <c r="C3397" t="inlineStr">
         <is>
-          <t>RENARA ANDRADE MATIAS</t>
+          <t>FRANCISCO DAVID ASSUNCAO ALVES</t>
         </is>
       </c>
       <c r="D3397" t="inlineStr">
         <is>
-          <t>R.ANDRADE</t>
+          <t>ASSUNÇÃO</t>
         </is>
       </c>
     </row>
     <row r="3398">
       <c r="A3398" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3398" t="n">
-        <v>3275</v>
+        <v>3513</v>
       </c>
       <c r="C3398" t="inlineStr">
         <is>
-          <t>MARIA APARECIDA COELHO SILVA</t>
+          <t>RENARA ANDRADE MATIAS</t>
         </is>
       </c>
       <c r="D3398" t="inlineStr">
         <is>
-          <t>MCOELHO</t>
+          <t>R.ANDRADE</t>
         </is>
       </c>
     </row>
@@ -68398,136 +68398,136 @@
         </is>
       </c>
       <c r="B3399" t="n">
-        <v>3276</v>
+        <v>3275</v>
       </c>
       <c r="C3399" t="inlineStr">
         <is>
-          <t xml:space="preserve">PEROLA DE JESUS AMORIM SOUSA </t>
+          <t>MARIA APARECIDA COELHO SILVA</t>
         </is>
       </c>
       <c r="D3399" t="inlineStr">
         <is>
-          <t>PJESUS</t>
+          <t>MCOELHO</t>
         </is>
       </c>
     </row>
     <row r="3400">
       <c r="A3400" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3400" t="n">
-        <v>3526</v>
+        <v>3276</v>
       </c>
       <c r="C3400" t="inlineStr">
         <is>
-          <t>JOYCE NAZARE CORREA</t>
+          <t xml:space="preserve">PEROLA DE JESUS AMORIM SOUSA </t>
         </is>
       </c>
       <c r="D3400" t="inlineStr">
         <is>
-          <t>J.NAZARE</t>
+          <t>PJESUS</t>
         </is>
       </c>
     </row>
     <row r="3401">
       <c r="A3401" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3401" t="n">
-        <v>3527</v>
+        <v>3526</v>
       </c>
       <c r="C3401" t="inlineStr">
         <is>
-          <t>GILVANA DA SILVA MONTELES</t>
+          <t>JOYCE NAZARE CORREA</t>
         </is>
       </c>
       <c r="D3401" t="inlineStr">
         <is>
-          <t>GIL.SILVA</t>
+          <t>J.NAZARE</t>
         </is>
       </c>
     </row>
     <row r="3402">
       <c r="A3402" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3402" t="n">
-        <v>3548</v>
+        <v>3527</v>
       </c>
       <c r="C3402" t="inlineStr">
         <is>
-          <t>JAMILLY MARIA HENRIQUE ARAUJO</t>
+          <t>GILVANA DA SILVA MONTELES</t>
         </is>
       </c>
       <c r="D3402" t="inlineStr">
         <is>
-          <t>JAMILLY</t>
+          <t>GIL.SILVA</t>
         </is>
       </c>
     </row>
     <row r="3403">
       <c r="A3403" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3403" t="n">
-        <v>3551</v>
+        <v>3548</v>
       </c>
       <c r="C3403" t="inlineStr">
         <is>
-          <t xml:space="preserve">VITOR MANOEL DA SILVA BARBOSA </t>
+          <t>JAMILLY MARIA HENRIQUE ARAUJO</t>
         </is>
       </c>
       <c r="D3403" t="inlineStr">
         <is>
-          <t>VMANOEL</t>
+          <t>JAMILLY</t>
         </is>
       </c>
     </row>
     <row r="3404">
       <c r="A3404" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3404" t="n">
-        <v>3588</v>
+        <v>3551</v>
       </c>
       <c r="C3404" t="inlineStr">
         <is>
-          <t>BRUNA RAISEYLLA SANTOS DE SALES</t>
+          <t xml:space="preserve">VITOR MANOEL DA SILVA BARBOSA </t>
         </is>
       </c>
       <c r="D3404" t="inlineStr">
         <is>
-          <t>BRU.SALES</t>
+          <t>VMANOEL</t>
         </is>
       </c>
     </row>
     <row r="3405">
       <c r="A3405" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3405" t="n">
-        <v>940525</v>
+        <v>3588</v>
       </c>
       <c r="C3405" t="inlineStr">
         <is>
-          <t>SANDUWELLINGTON</t>
+          <t>BRUNA RAISEYLLA SANTOS DE SALES</t>
         </is>
       </c>
       <c r="D3405" t="inlineStr">
         <is>
-          <t>SANDUWELLINGTON</t>
+          <t>BRU.SALES</t>
         </is>
       </c>
     </row>
@@ -68538,36 +68538,36 @@
         </is>
       </c>
       <c r="B3406" t="n">
-        <v>3369</v>
+        <v>940525</v>
       </c>
       <c r="C3406" t="inlineStr">
         <is>
-          <t xml:space="preserve">PRISCILA DOS SANTOS LOPES </t>
+          <t>SANDUWELLINGTON</t>
         </is>
       </c>
       <c r="D3406" t="inlineStr">
         <is>
-          <t>PSLOPES</t>
+          <t>SANDUWELLINGTON</t>
         </is>
       </c>
     </row>
     <row r="3407">
       <c r="A3407" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3407" t="n">
-        <v>3433</v>
+        <v>3369</v>
       </c>
       <c r="C3407" t="inlineStr">
         <is>
-          <t>BRUNO NUNES CRUZ</t>
+          <t xml:space="preserve">PRISCILA DOS SANTOS LOPES </t>
         </is>
       </c>
       <c r="D3407" t="inlineStr">
         <is>
-          <t>BRUNOCRUZ</t>
+          <t>PSLOPES</t>
         </is>
       </c>
     </row>
@@ -68578,36 +68578,36 @@
         </is>
       </c>
       <c r="B3408" t="n">
-        <v>3434</v>
+        <v>3433</v>
       </c>
       <c r="C3408" t="inlineStr">
         <is>
-          <t>ANA TERCIA DE LIMA SA CARVALHO SERAFIM</t>
+          <t>BRUNO NUNES CRUZ</t>
         </is>
       </c>
       <c r="D3408" t="inlineStr">
         <is>
-          <t>ANATER</t>
+          <t>BRUNOCRUZ</t>
         </is>
       </c>
     </row>
     <row r="3409">
       <c r="A3409" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3409" t="n">
-        <v>3502</v>
+        <v>3434</v>
       </c>
       <c r="C3409" t="inlineStr">
         <is>
-          <t>LUIZ FELIPE MACHADO BARRETO</t>
+          <t>ANA TERCIA DE LIMA SA CARVALHO SERAFIM</t>
         </is>
       </c>
       <c r="D3409" t="inlineStr">
         <is>
-          <t>LUIZ.FELIPE</t>
+          <t>ANATER</t>
         </is>
       </c>
     </row>
@@ -68618,36 +68618,36 @@
         </is>
       </c>
       <c r="B3410" t="n">
-        <v>3503</v>
+        <v>3502</v>
       </c>
       <c r="C3410" t="inlineStr">
         <is>
-          <t>FABIO OLIVEIRA SILVA</t>
+          <t>LUIZ FELIPE MACHADO BARRETO</t>
         </is>
       </c>
       <c r="D3410" t="inlineStr">
         <is>
-          <t>FOSILVA</t>
+          <t>LUIZ.FELIPE</t>
         </is>
       </c>
     </row>
     <row r="3411">
       <c r="A3411" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3411" t="n">
-        <v>3554</v>
+        <v>3503</v>
       </c>
       <c r="C3411" t="inlineStr">
         <is>
-          <t xml:space="preserve">MANOEL RIBEIRO DE SOUZA JUNIOR </t>
+          <t>FABIO OLIVEIRA SILVA</t>
         </is>
       </c>
       <c r="D3411" t="inlineStr">
         <is>
-          <t>MRJUNIOR</t>
+          <t>FOSILVA</t>
         </is>
       </c>
     </row>
@@ -68658,16 +68658,16 @@
         </is>
       </c>
       <c r="B3412" t="n">
-        <v>3568</v>
+        <v>3554</v>
       </c>
       <c r="C3412" t="inlineStr">
         <is>
-          <t xml:space="preserve">ANGELICA TORRES DA SILVA </t>
+          <t xml:space="preserve">MANOEL RIBEIRO DE SOUZA JUNIOR </t>
         </is>
       </c>
       <c r="D3412" t="inlineStr">
         <is>
-          <t>ANGEL.TORRES</t>
+          <t>MRJUNIOR</t>
         </is>
       </c>
     </row>
@@ -68678,56 +68678,56 @@
         </is>
       </c>
       <c r="B3413" t="n">
-        <v>3569</v>
+        <v>3568</v>
       </c>
       <c r="C3413" t="inlineStr">
         <is>
-          <t>LORENA DE LIMA MATOS</t>
+          <t xml:space="preserve">ANGELICA TORRES DA SILVA </t>
         </is>
       </c>
       <c r="D3413" t="inlineStr">
         <is>
-          <t>LORE.LIMA</t>
+          <t>ANGEL.TORRES</t>
         </is>
       </c>
     </row>
     <row r="3414">
       <c r="A3414" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3414" t="n">
-        <v>3576</v>
+        <v>3569</v>
       </c>
       <c r="C3414" t="inlineStr">
         <is>
-          <t>ANA BEATRIZ PARENTE CAVALCANTE</t>
+          <t>LORENA DE LIMA MATOS</t>
         </is>
       </c>
       <c r="D3414" t="inlineStr">
         <is>
-          <t>A.BEATRIZ</t>
+          <t>LORE.LIMA</t>
         </is>
       </c>
     </row>
     <row r="3415">
       <c r="A3415" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3415" t="n">
-        <v>940549</v>
+        <v>3576</v>
       </c>
       <c r="C3415" t="inlineStr">
         <is>
-          <t>EDILSON ARAUJO - FL9</t>
+          <t>ANA BEATRIZ PARENTE CAVALCANTE</t>
         </is>
       </c>
       <c r="D3415" t="inlineStr">
         <is>
-          <t>EDILSON</t>
+          <t>A.BEATRIZ</t>
         </is>
       </c>
     </row>
@@ -68738,36 +68738,36 @@
         </is>
       </c>
       <c r="B3416" t="n">
-        <v>3470</v>
+        <v>940549</v>
       </c>
       <c r="C3416" t="inlineStr">
         <is>
-          <t>DEBORA ALVES CARVALHO</t>
+          <t>EDILSON ARAUJO - FL9</t>
         </is>
       </c>
       <c r="D3416" t="inlineStr">
         <is>
-          <t>DEBORA.ALVES</t>
+          <t>EDILSON</t>
         </is>
       </c>
     </row>
     <row r="3417">
       <c r="A3417" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3417" t="n">
-        <v>3510</v>
+        <v>3470</v>
       </c>
       <c r="C3417" t="inlineStr">
         <is>
-          <t>CAMILA RODIGUES PINTO</t>
+          <t>DEBORA ALVES CARVALHO</t>
         </is>
       </c>
       <c r="D3417" t="inlineStr">
         <is>
-          <t>MILA.PINTO</t>
+          <t>DEBORA.ALVES</t>
         </is>
       </c>
     </row>
@@ -68778,96 +68778,96 @@
         </is>
       </c>
       <c r="B3418" t="n">
-        <v>3511</v>
+        <v>3510</v>
       </c>
       <c r="C3418" t="inlineStr">
         <is>
-          <t>JORGE HENRIQUE DOS SANTOS RODRIGUES</t>
+          <t>CAMILA RODIGUES PINTO</t>
         </is>
       </c>
       <c r="D3418" t="inlineStr">
         <is>
-          <t>J.HENRIQUE</t>
+          <t>MILA.PINTO</t>
         </is>
       </c>
     </row>
     <row r="3419">
       <c r="A3419" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3419" t="n">
-        <v>3561</v>
+        <v>3511</v>
       </c>
       <c r="C3419" t="inlineStr">
         <is>
-          <t>RONARIA PATRICIA VILARINDO DE ALMEIDA</t>
+          <t>JORGE HENRIQUE DOS SANTOS RODRIGUES</t>
         </is>
       </c>
       <c r="D3419" t="inlineStr">
         <is>
-          <t>RPATRICIA</t>
+          <t>J.HENRIQUE</t>
         </is>
       </c>
     </row>
     <row r="3420">
       <c r="A3420" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3420" t="n">
-        <v>3562</v>
+        <v>3561</v>
       </c>
       <c r="C3420" t="inlineStr">
         <is>
-          <t>LETICIA MARIA BENTO NOGUEIRA</t>
+          <t>RONARIA PATRICIA VILARINDO DE ALMEIDA</t>
         </is>
       </c>
       <c r="D3420" t="inlineStr">
         <is>
-          <t>LBENTO</t>
+          <t>RPATRICIA</t>
         </is>
       </c>
     </row>
     <row r="3421">
       <c r="A3421" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3421" t="n">
-        <v>3270</v>
+        <v>3562</v>
       </c>
       <c r="C3421" t="inlineStr">
         <is>
-          <t>ITANA NASCIMENTO SIMOES</t>
+          <t>LETICIA MARIA BENTO NOGUEIRA</t>
         </is>
       </c>
       <c r="D3421" t="inlineStr">
         <is>
-          <t>ISIMOES</t>
+          <t>LBENTO</t>
         </is>
       </c>
     </row>
     <row r="3422">
       <c r="A3422" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3422" t="n">
-        <v>3318</v>
+        <v>3270</v>
       </c>
       <c r="C3422" t="inlineStr">
         <is>
-          <t>LUAN MONTEIRO COSTA</t>
+          <t>ITANA NASCIMENTO SIMOES</t>
         </is>
       </c>
       <c r="D3422" t="inlineStr">
         <is>
-          <t>LMONTEIRO</t>
+          <t>ISIMOES</t>
         </is>
       </c>
     </row>
@@ -68878,36 +68878,36 @@
         </is>
       </c>
       <c r="B3423" t="n">
-        <v>3319</v>
+        <v>3318</v>
       </c>
       <c r="C3423" t="inlineStr">
         <is>
-          <t>MARIANA MACEDA DOS SANTOS</t>
+          <t>LUAN MONTEIRO COSTA</t>
         </is>
       </c>
       <c r="D3423" t="inlineStr">
         <is>
-          <t>MMACEDA</t>
+          <t>LMONTEIRO</t>
         </is>
       </c>
     </row>
     <row r="3424">
       <c r="A3424" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3424" t="n">
-        <v>3389</v>
+        <v>3319</v>
       </c>
       <c r="C3424" t="inlineStr">
         <is>
-          <t>TAMILES DE SANTANA AMORIM BISPO</t>
+          <t>MARIANA MACEDA DOS SANTOS</t>
         </is>
       </c>
       <c r="D3424" t="inlineStr">
         <is>
-          <t>TAMILES</t>
+          <t>MMACEDA</t>
         </is>
       </c>
     </row>
@@ -68918,76 +68918,76 @@
         </is>
       </c>
       <c r="B3425" t="n">
-        <v>3390</v>
+        <v>3389</v>
       </c>
       <c r="C3425" t="inlineStr">
         <is>
-          <t>IRACEMA DE ALMEIDA MOURA</t>
+          <t>TAMILES DE SANTANA AMORIM BISPO</t>
         </is>
       </c>
       <c r="D3425" t="inlineStr">
         <is>
-          <t>IRACEMA</t>
+          <t>TAMILES</t>
         </is>
       </c>
     </row>
     <row r="3426">
       <c r="A3426" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3426" t="n">
-        <v>3575</v>
+        <v>3390</v>
       </c>
       <c r="C3426" t="inlineStr">
         <is>
-          <t>SAMARA ALVES DA SILVA</t>
+          <t>IRACEMA DE ALMEIDA MOURA</t>
         </is>
       </c>
       <c r="D3426" t="inlineStr">
         <is>
-          <t>S.ALVES</t>
+          <t>IRACEMA</t>
         </is>
       </c>
     </row>
     <row r="3427">
       <c r="A3427" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3427" t="n">
-        <v>3583</v>
+        <v>3575</v>
       </c>
       <c r="C3427" t="inlineStr">
         <is>
-          <t>TALLIS GUTTEMBERG GUIMARES BATISTA</t>
+          <t>SAMARA ALVES DA SILVA</t>
         </is>
       </c>
       <c r="D3427" t="inlineStr">
         <is>
-          <t>TALLIS16</t>
+          <t>S.ALVES</t>
         </is>
       </c>
     </row>
     <row r="3428">
       <c r="A3428" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3428" t="n">
-        <v>3286</v>
+        <v>3583</v>
       </c>
       <c r="C3428" t="inlineStr">
         <is>
-          <t>VALERIA MAIA DA SILVA</t>
+          <t>TALLIS GUTTEMBERG GUIMARES BATISTA</t>
         </is>
       </c>
       <c r="D3428" t="inlineStr">
         <is>
-          <t>VMAIAS</t>
+          <t>TALLIS16</t>
         </is>
       </c>
     </row>
@@ -68998,156 +68998,156 @@
         </is>
       </c>
       <c r="B3429" t="n">
-        <v>3287</v>
+        <v>3286</v>
       </c>
       <c r="C3429" t="inlineStr">
         <is>
-          <t>ERIVELTON DA SILVA OLIVEIRA</t>
+          <t>VALERIA MAIA DA SILVA</t>
         </is>
       </c>
       <c r="D3429" t="inlineStr">
         <is>
-          <t>ESOLIVEIRA</t>
+          <t>VMAIAS</t>
         </is>
       </c>
     </row>
     <row r="3430">
       <c r="A3430" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3430" t="n">
-        <v>3307</v>
+        <v>3287</v>
       </c>
       <c r="C3430" t="inlineStr">
         <is>
-          <t>ADRIEL XERES BARROS MARTINS</t>
+          <t>ERIVELTON DA SILVA OLIVEIRA</t>
         </is>
       </c>
       <c r="D3430" t="inlineStr">
         <is>
-          <t>AXERES</t>
+          <t>ESOLIVEIRA</t>
         </is>
       </c>
     </row>
     <row r="3431">
       <c r="A3431" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3431" t="n">
-        <v>3308</v>
+        <v>3307</v>
       </c>
       <c r="C3431" t="inlineStr">
         <is>
-          <t>ELKZIEL JUVINO DA SILVA</t>
+          <t>ADRIEL XERES BARROS MARTINS</t>
         </is>
       </c>
       <c r="D3431" t="inlineStr">
         <is>
-          <t>EJUVINO</t>
+          <t>AXERES</t>
         </is>
       </c>
     </row>
     <row r="3432">
       <c r="A3432" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3432" t="n">
-        <v>940539</v>
+        <v>3308</v>
       </c>
       <c r="C3432" t="inlineStr">
         <is>
-          <t>EDSON ARAUJO - FL9</t>
+          <t>ELKZIEL JUVINO DA SILVA</t>
         </is>
       </c>
       <c r="D3432" t="inlineStr">
         <is>
-          <t>EDS</t>
+          <t>EJUVINO</t>
         </is>
       </c>
     </row>
     <row r="3433">
       <c r="A3433" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3433" t="n">
-        <v>940540</v>
+        <v>940539</v>
       </c>
       <c r="C3433" t="inlineStr">
         <is>
-          <t>EDSON ARAUJO - FL8</t>
+          <t>EDSON ARAUJO - FL9</t>
         </is>
       </c>
       <c r="D3433" t="inlineStr">
         <is>
-          <t>EDS8</t>
+          <t>EDS</t>
         </is>
       </c>
     </row>
     <row r="3434">
       <c r="A3434" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B3434" t="n">
-        <v>3328</v>
+        <v>940540</v>
       </c>
       <c r="C3434" t="inlineStr">
         <is>
-          <t>ALAN ARAUJO DA SILVA</t>
+          <t>EDSON ARAUJO - FL8</t>
         </is>
       </c>
       <c r="D3434" t="inlineStr">
         <is>
-          <t>ARSILVA</t>
+          <t>EDS8</t>
         </is>
       </c>
     </row>
     <row r="3435">
       <c r="A3435" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3435" t="n">
-        <v>3350</v>
+        <v>3328</v>
       </c>
       <c r="C3435" t="inlineStr">
         <is>
-          <t xml:space="preserve">EDER RODRIGUES DA SILVA </t>
+          <t>ALAN ARAUJO DA SILVA</t>
         </is>
       </c>
       <c r="D3435" t="inlineStr">
         <is>
-          <t>EDERS</t>
+          <t>ARSILVA</t>
         </is>
       </c>
     </row>
     <row r="3436">
       <c r="A3436" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3436" t="n">
-        <v>3373</v>
+        <v>3350</v>
       </c>
       <c r="C3436" t="inlineStr">
         <is>
-          <t xml:space="preserve">NATANAEL TAVARES DE SOUSA </t>
+          <t xml:space="preserve">EDER RODRIGUES DA SILVA </t>
         </is>
       </c>
       <c r="D3436" t="inlineStr">
         <is>
-          <t>NTSOUSA</t>
+          <t>EDERS</t>
         </is>
       </c>
     </row>
@@ -69158,156 +69158,156 @@
         </is>
       </c>
       <c r="B3437" t="n">
-        <v>3374</v>
+        <v>3373</v>
       </c>
       <c r="C3437" t="inlineStr">
         <is>
-          <t>REINALDO DA SILVA COSTA</t>
+          <t xml:space="preserve">NATANAEL TAVARES DE SOUSA </t>
         </is>
       </c>
       <c r="D3437" t="inlineStr">
         <is>
-          <t>RSCOSTA</t>
+          <t>NTSOUSA</t>
         </is>
       </c>
     </row>
     <row r="3438">
       <c r="A3438" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3438" t="n">
-        <v>3399</v>
+        <v>3374</v>
       </c>
       <c r="C3438" t="inlineStr">
         <is>
-          <t xml:space="preserve">RICARDO BARBOSA DOS SANTOS </t>
+          <t>REINALDO DA SILVA COSTA</t>
         </is>
       </c>
       <c r="D3438" t="inlineStr">
         <is>
-          <t>RICARDOSAN</t>
+          <t>RSCOSTA</t>
         </is>
       </c>
     </row>
     <row r="3439">
       <c r="A3439" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3439" t="n">
-        <v>3427</v>
+        <v>3399</v>
       </c>
       <c r="C3439" t="inlineStr">
         <is>
-          <t>ROQUE COMERCIO TEMPORARIO</t>
+          <t xml:space="preserve">RICARDO BARBOSA DOS SANTOS </t>
         </is>
       </c>
       <c r="D3439" t="inlineStr">
         <is>
-          <t>ROQUECOM</t>
+          <t>RICARDOSAN</t>
         </is>
       </c>
     </row>
     <row r="3440">
       <c r="A3440" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3440" t="n">
-        <v>3428</v>
+        <v>3427</v>
       </c>
       <c r="C3440" t="inlineStr">
         <is>
-          <t>ROQUE PLUS TEMPORARIO</t>
+          <t>ROQUE COMERCIO TEMPORARIO</t>
         </is>
       </c>
       <c r="D3440" t="inlineStr">
         <is>
-          <t>ROQUEPLUS</t>
+          <t>ROQUECOM</t>
         </is>
       </c>
     </row>
     <row r="3441">
       <c r="A3441" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3441" t="n">
-        <v>3432</v>
+        <v>3428</v>
       </c>
       <c r="C3441" t="inlineStr">
         <is>
-          <t>PATRICIA DOS SANTOS NONATO OLIVEIRA</t>
+          <t>ROQUE PLUS TEMPORARIO</t>
         </is>
       </c>
       <c r="D3441" t="inlineStr">
         <is>
-          <t>PATRICIAD</t>
+          <t>ROQUEPLUS</t>
         </is>
       </c>
     </row>
     <row r="3442">
       <c r="A3442" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3442" t="n">
-        <v>3448</v>
+        <v>3432</v>
       </c>
       <c r="C3442" t="inlineStr">
         <is>
-          <t xml:space="preserve">GABRIEL SOUZA CARVALHO </t>
+          <t>PATRICIA DOS SANTOS NONATO OLIVEIRA</t>
         </is>
       </c>
       <c r="D3442" t="inlineStr">
         <is>
-          <t>GABRIEL20</t>
+          <t>PATRICIAD</t>
         </is>
       </c>
     </row>
     <row r="3443">
       <c r="A3443" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3443" t="n">
-        <v>3465</v>
+        <v>3448</v>
       </c>
       <c r="C3443" t="inlineStr">
         <is>
-          <t>LUIZA MARIA BARRETO BARBOSA</t>
+          <t xml:space="preserve">GABRIEL SOUZA CARVALHO </t>
         </is>
       </c>
       <c r="D3443" t="inlineStr">
         <is>
-          <t>LUIZA.MARIA</t>
+          <t>GABRIEL20</t>
         </is>
       </c>
     </row>
     <row r="3444">
       <c r="A3444" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3444" t="n">
-        <v>3468</v>
+        <v>3465</v>
       </c>
       <c r="C3444" t="inlineStr">
         <is>
-          <t>KAWA ALMEIDA CAMPOS</t>
+          <t>LUIZA MARIA BARRETO BARBOSA</t>
         </is>
       </c>
       <c r="D3444" t="inlineStr">
         <is>
-          <t>KAWA</t>
+          <t>LUIZA.MARIA</t>
         </is>
       </c>
     </row>
@@ -69318,16 +69318,16 @@
         </is>
       </c>
       <c r="B3445" t="n">
-        <v>3476</v>
+        <v>3468</v>
       </c>
       <c r="C3445" t="inlineStr">
         <is>
-          <t xml:space="preserve"> FRANCISCA LEIDIANE M. MENDES NASCIMENTO</t>
+          <t>KAWA ALMEIDA CAMPOS</t>
         </is>
       </c>
       <c r="D3445" t="inlineStr">
         <is>
-          <t>FLEIDIANE</t>
+          <t>KAWA</t>
         </is>
       </c>
     </row>
@@ -69338,76 +69338,76 @@
         </is>
       </c>
       <c r="B3446" t="n">
-        <v>3477</v>
+        <v>3476</v>
       </c>
       <c r="C3446" t="inlineStr">
         <is>
-          <t>MARIA THAIS MARTINS PEREIRA SILVA</t>
+          <t xml:space="preserve"> FRANCISCA LEIDIANE M. MENDES NASCIMENTO</t>
         </is>
       </c>
       <c r="D3446" t="inlineStr">
         <is>
-          <t>MTHAIS</t>
+          <t>FLEIDIANE</t>
         </is>
       </c>
     </row>
     <row r="3447">
       <c r="A3447" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3447" t="n">
-        <v>3271</v>
+        <v>3477</v>
       </c>
       <c r="C3447" t="inlineStr">
         <is>
-          <t>DIEGO DE ARAUJO CALÁBRIA</t>
+          <t>MARIA THAIS MARTINS PEREIRA SILVA</t>
         </is>
       </c>
       <c r="D3447" t="inlineStr">
         <is>
-          <t>ARAUJOC</t>
+          <t>MTHAIS</t>
         </is>
       </c>
     </row>
     <row r="3448">
       <c r="A3448" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3448" t="n">
-        <v>3272</v>
+        <v>3271</v>
       </c>
       <c r="C3448" t="inlineStr">
         <is>
-          <t>ANNE BEATRIZ SILVA VIRGINO</t>
+          <t>DIEGO DE ARAUJO CALÁBRIA</t>
         </is>
       </c>
       <c r="D3448" t="inlineStr">
         <is>
-          <t>ABVIRGINIO</t>
+          <t>ARAUJOC</t>
         </is>
       </c>
     </row>
     <row r="3449">
       <c r="A3449" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3449" t="n">
-        <v>3293</v>
+        <v>3272</v>
       </c>
       <c r="C3449" t="inlineStr">
         <is>
-          <t xml:space="preserve">CARLOS ALBERTO VIRIATO SANTOS </t>
+          <t>ANNE BEATRIZ SILVA VIRGINO</t>
         </is>
       </c>
       <c r="D3449" t="inlineStr">
         <is>
-          <t>CVIRIATO</t>
+          <t>ABVIRGINIO</t>
         </is>
       </c>
     </row>
@@ -69418,16 +69418,16 @@
         </is>
       </c>
       <c r="B3450" t="n">
-        <v>3381</v>
+        <v>3293</v>
       </c>
       <c r="C3450" t="inlineStr">
         <is>
-          <t>ALAN CAIQUE SANTOS E SANTOS</t>
+          <t xml:space="preserve">CARLOS ALBERTO VIRIATO SANTOS </t>
         </is>
       </c>
       <c r="D3450" t="inlineStr">
         <is>
-          <t>ALANSANTOS</t>
+          <t>CVIRIATO</t>
         </is>
       </c>
     </row>
@@ -69438,116 +69438,116 @@
         </is>
       </c>
       <c r="B3451" t="n">
-        <v>3443</v>
+        <v>3381</v>
       </c>
       <c r="C3451" t="inlineStr">
         <is>
-          <t>SANON MOREIRA SOUZA</t>
+          <t>ALAN CAIQUE SANTOS E SANTOS</t>
         </is>
       </c>
       <c r="D3451" t="inlineStr">
         <is>
-          <t>SANON</t>
+          <t>ALANSANTOS</t>
         </is>
       </c>
     </row>
     <row r="3452">
       <c r="A3452" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3452" t="n">
-        <v>3516</v>
+        <v>3443</v>
       </c>
       <c r="C3452" t="inlineStr">
         <is>
-          <t>FRANCISCO RILDER TELES DE OLIVEIRA</t>
+          <t>SANON MOREIRA SOUZA</t>
         </is>
       </c>
       <c r="D3452" t="inlineStr">
         <is>
-          <t>RILDER</t>
+          <t>SANON</t>
         </is>
       </c>
     </row>
     <row r="3453">
       <c r="A3453" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3453" t="n">
-        <v>3519</v>
+        <v>3516</v>
       </c>
       <c r="C3453" t="inlineStr">
         <is>
-          <t>MARIA LUANA DE ALMEIDA BATISTA</t>
+          <t>FRANCISCO RILDER TELES DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D3453" t="inlineStr">
         <is>
-          <t>M.LUANA</t>
+          <t>RILDER</t>
         </is>
       </c>
     </row>
     <row r="3454">
       <c r="A3454" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3454" t="n">
-        <v>3540</v>
+        <v>3519</v>
       </c>
       <c r="C3454" t="inlineStr">
         <is>
-          <t>HELEN VITORIA OLIVEIRA DA ROCHA</t>
+          <t>MARIA LUANA DE ALMEIDA BATISTA</t>
         </is>
       </c>
       <c r="D3454" t="inlineStr">
         <is>
-          <t>H.VITORIA</t>
+          <t>M.LUANA</t>
         </is>
       </c>
     </row>
     <row r="3455">
       <c r="A3455" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B3455" t="n">
-        <v>3559</v>
+        <v>3540</v>
       </c>
       <c r="C3455" t="inlineStr">
         <is>
-          <t>ARKBERYS TELES DE SOUSA</t>
+          <t>HELEN VITORIA OLIVEIRA DA ROCHA</t>
         </is>
       </c>
       <c r="D3455" t="inlineStr">
         <is>
-          <t>ARKBERYS</t>
+          <t>H.VITORIA</t>
         </is>
       </c>
     </row>
     <row r="3456">
       <c r="A3456" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3456" t="n">
-        <v>3567</v>
+        <v>3559</v>
       </c>
       <c r="C3456" t="inlineStr">
         <is>
-          <t>PEDRO HENRIQUE VIEIRA DE LIMA</t>
+          <t>ARKBERYS TELES DE SOUSA</t>
         </is>
       </c>
       <c r="D3456" t="inlineStr">
         <is>
-          <t>P.LIMA</t>
+          <t>ARKBERYS</t>
         </is>
       </c>
     </row>
@@ -69558,76 +69558,76 @@
         </is>
       </c>
       <c r="B3457" t="n">
-        <v>3331</v>
+        <v>3567</v>
       </c>
       <c r="C3457" t="inlineStr">
         <is>
-          <t>LOUIZE VANIELLE RODRIGUES FARIAS</t>
+          <t>PEDRO HENRIQUE VIEIRA DE LIMA</t>
         </is>
       </c>
       <c r="D3457" t="inlineStr">
         <is>
-          <t>LVFARIAS</t>
+          <t>P.LIMA</t>
         </is>
       </c>
     </row>
     <row r="3458">
       <c r="A3458" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3458" t="n">
-        <v>3334</v>
+        <v>3331</v>
       </c>
       <c r="C3458" t="inlineStr">
         <is>
-          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+          <t>LOUIZE VANIELLE RODRIGUES FARIAS</t>
         </is>
       </c>
       <c r="D3458" t="inlineStr">
         <is>
-          <t>MTGASPAR</t>
+          <t>LVFARIAS</t>
         </is>
       </c>
     </row>
     <row r="3459">
       <c r="A3459" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3459" t="n">
-        <v>3345</v>
+        <v>3334</v>
       </c>
       <c r="C3459" t="inlineStr">
         <is>
-          <t>AURICÉLIA INACIO PEREIRA</t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
       <c r="D3459" t="inlineStr">
         <is>
-          <t>AIPEREIRA</t>
+          <t>MTGASPAR</t>
         </is>
       </c>
     </row>
     <row r="3460">
       <c r="A3460" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3460" t="n">
-        <v>3363</v>
+        <v>3345</v>
       </c>
       <c r="C3460" t="inlineStr">
         <is>
-          <t>IASMIN LEAL ALVES</t>
+          <t>AURICÉLIA INACIO PEREIRA</t>
         </is>
       </c>
       <c r="D3460" t="inlineStr">
         <is>
-          <t>ILALVES</t>
+          <t>AIPEREIRA</t>
         </is>
       </c>
     </row>
@@ -69638,196 +69638,196 @@
         </is>
       </c>
       <c r="B3461" t="n">
-        <v>3370</v>
+        <v>3363</v>
       </c>
       <c r="C3461" t="inlineStr">
         <is>
-          <t>CARLOS DIEGO ARAUJO ALMEIDA</t>
+          <t>IASMIN LEAL ALVES</t>
         </is>
       </c>
       <c r="D3461" t="inlineStr">
         <is>
-          <t>CDIEGO</t>
+          <t>ILALVES</t>
         </is>
       </c>
     </row>
     <row r="3462">
       <c r="A3462" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3462" t="n">
-        <v>3379</v>
+        <v>3370</v>
       </c>
       <c r="C3462" t="inlineStr">
         <is>
-          <t xml:space="preserve">MATHEUS EVANGELISTA FERREIRA </t>
+          <t>CARLOS DIEGO ARAUJO ALMEIDA</t>
         </is>
       </c>
       <c r="D3462" t="inlineStr">
         <is>
-          <t>MMFERREIRA</t>
+          <t>CDIEGO</t>
         </is>
       </c>
     </row>
     <row r="3463">
       <c r="A3463" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3463" t="n">
-        <v>3419</v>
+        <v>3379</v>
       </c>
       <c r="C3463" t="inlineStr">
         <is>
-          <t xml:space="preserve">DAVID EVANGELISTA SILVA </t>
+          <t xml:space="preserve">MATHEUS EVANGELISTA FERREIRA </t>
         </is>
       </c>
       <c r="D3463" t="inlineStr">
         <is>
-          <t>DAVID</t>
+          <t>MMFERREIRA</t>
         </is>
       </c>
     </row>
     <row r="3464">
       <c r="A3464" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3464" t="n">
-        <v>3423</v>
+        <v>3419</v>
       </c>
       <c r="C3464" t="inlineStr">
         <is>
-          <t>MARCIO JOSE TIAGO</t>
+          <t xml:space="preserve">DAVID EVANGELISTA SILVA </t>
         </is>
       </c>
       <c r="D3464" t="inlineStr">
         <is>
-          <t>MJTIAGO</t>
+          <t>DAVID</t>
         </is>
       </c>
     </row>
     <row r="3465">
       <c r="A3465" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3465" t="n">
-        <v>3453</v>
+        <v>3423</v>
       </c>
       <c r="C3465" t="inlineStr">
         <is>
-          <t xml:space="preserve">LAURIENE SILVA BARBOSA </t>
+          <t>MARCIO JOSE TIAGO</t>
         </is>
       </c>
       <c r="D3465" t="inlineStr">
         <is>
-          <t>LAURIENE</t>
+          <t>MJTIAGO</t>
         </is>
       </c>
     </row>
     <row r="3466">
       <c r="A3466" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3466" t="n">
-        <v>3478</v>
+        <v>3453</v>
       </c>
       <c r="C3466" t="inlineStr">
         <is>
-          <t>LEANDRO BRITO NOGUEIRA DE OLIVEIRA</t>
+          <t xml:space="preserve">LAURIENE SILVA BARBOSA </t>
         </is>
       </c>
       <c r="D3466" t="inlineStr">
         <is>
-          <t>LBNOGUEIRA</t>
+          <t>LAURIENE</t>
         </is>
       </c>
     </row>
     <row r="3467">
       <c r="A3467" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3467" t="n">
-        <v>3479</v>
+        <v>3478</v>
       </c>
       <c r="C3467" t="inlineStr">
         <is>
-          <t>ESDRAS ALESSANDRO SANTOS SANTANA</t>
+          <t>LEANDRO BRITO NOGUEIRA DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D3467" t="inlineStr">
         <is>
-          <t>EALESSANDRO</t>
+          <t>LBNOGUEIRA</t>
         </is>
       </c>
     </row>
     <row r="3468">
       <c r="A3468" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3468" t="n">
-        <v>3480</v>
+        <v>3479</v>
       </c>
       <c r="C3468" t="inlineStr">
         <is>
-          <t xml:space="preserve">LUCIMARA SOUSA LIMA </t>
+          <t>ESDRAS ALESSANDRO SANTOS SANTANA</t>
         </is>
       </c>
       <c r="D3468" t="inlineStr">
         <is>
-          <t>LUCIMARA</t>
+          <t>EALESSANDRO</t>
         </is>
       </c>
     </row>
     <row r="3469">
       <c r="A3469" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3469" t="n">
-        <v>3482</v>
+        <v>3480</v>
       </c>
       <c r="C3469" t="inlineStr">
         <is>
-          <t>DANIEL FERNANDES DINIZ HERACLIO</t>
+          <t xml:space="preserve">LUCIMARA SOUSA LIMA </t>
         </is>
       </c>
       <c r="D3469" t="inlineStr">
         <is>
-          <t>DFDINIZ</t>
+          <t>LUCIMARA</t>
         </is>
       </c>
     </row>
     <row r="3470">
       <c r="A3470" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3470" t="n">
-        <v>3518</v>
+        <v>3482</v>
       </c>
       <c r="C3470" t="inlineStr">
         <is>
-          <t>RAMYRA ALVES FELIX DA SILVA</t>
+          <t>DANIEL FERNANDES DINIZ HERACLIO</t>
         </is>
       </c>
       <c r="D3470" t="inlineStr">
         <is>
-          <t>RFELIX</t>
+          <t>DFDINIZ</t>
         </is>
       </c>
     </row>
@@ -69838,36 +69838,36 @@
         </is>
       </c>
       <c r="B3471" t="n">
-        <v>3534</v>
+        <v>3518</v>
       </c>
       <c r="C3471" t="inlineStr">
         <is>
-          <t xml:space="preserve">CAIO DE SOUZA VINHAS </t>
+          <t>RAMYRA ALVES FELIX DA SILVA</t>
         </is>
       </c>
       <c r="D3471" t="inlineStr">
         <is>
-          <t>CVINHAS</t>
+          <t>RFELIX</t>
         </is>
       </c>
     </row>
     <row r="3472">
       <c r="A3472" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3472" t="n">
-        <v>3535</v>
+        <v>3534</v>
       </c>
       <c r="C3472" t="inlineStr">
         <is>
-          <t>ROMARIO DE SOUSA SILVA</t>
+          <t xml:space="preserve">CAIO DE SOUZA VINHAS </t>
         </is>
       </c>
       <c r="D3472" t="inlineStr">
         <is>
-          <t>RSOUSAS</t>
+          <t>CVINHAS</t>
         </is>
       </c>
     </row>
@@ -69878,56 +69878,56 @@
         </is>
       </c>
       <c r="B3473" t="n">
-        <v>3536</v>
+        <v>3535</v>
       </c>
       <c r="C3473" t="inlineStr">
         <is>
-          <t>JHONATAS CARVALHO OLIVEIRA</t>
+          <t>ROMARIO DE SOUSA SILVA</t>
         </is>
       </c>
       <c r="D3473" t="inlineStr">
         <is>
-          <t>JHONATASC</t>
+          <t>RSOUSAS</t>
         </is>
       </c>
     </row>
     <row r="3474">
       <c r="A3474" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3474" t="n">
-        <v>940529</v>
+        <v>3536</v>
       </c>
       <c r="C3474" t="inlineStr">
         <is>
-          <t>EDGAR FELIX - FL9</t>
+          <t>JHONATAS CARVALHO OLIVEIRA</t>
         </is>
       </c>
       <c r="D3474" t="inlineStr">
         <is>
-          <t>EDGAR F</t>
+          <t>JHONATASC</t>
         </is>
       </c>
     </row>
     <row r="3475">
       <c r="A3475" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3475" t="n">
-        <v>3304</v>
+        <v>940529</v>
       </c>
       <c r="C3475" t="inlineStr">
         <is>
-          <t>JOACI GUILHERME GONÇALVES DA LUZ</t>
+          <t>EDGAR FELIX - FL9</t>
         </is>
       </c>
       <c r="D3475" t="inlineStr">
         <is>
-          <t>JLUZ</t>
+          <t>EDGAR F</t>
         </is>
       </c>
     </row>
@@ -69938,16 +69938,16 @@
         </is>
       </c>
       <c r="B3476" t="n">
-        <v>3305</v>
+        <v>3304</v>
       </c>
       <c r="C3476" t="inlineStr">
         <is>
-          <t>JOÃO VITOR DE ARAÚJO GONÇALVES</t>
+          <t>JOACI GUILHERME GONÇALVES DA LUZ</t>
         </is>
       </c>
       <c r="D3476" t="inlineStr">
         <is>
-          <t>JJVITOR</t>
+          <t>JLUZ</t>
         </is>
       </c>
     </row>
@@ -69958,36 +69958,36 @@
         </is>
       </c>
       <c r="B3477" t="n">
-        <v>3306</v>
+        <v>3305</v>
       </c>
       <c r="C3477" t="inlineStr">
         <is>
-          <t>WENDERSON MARCOS DOS SANTOS</t>
+          <t>JOÃO VITOR DE ARAÚJO GONÇALVES</t>
         </is>
       </c>
       <c r="D3477" t="inlineStr">
         <is>
-          <t>WWMARCOS</t>
+          <t>JJVITOR</t>
         </is>
       </c>
     </row>
     <row r="3478">
       <c r="A3478" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3478" t="n">
-        <v>3335</v>
+        <v>3306</v>
       </c>
       <c r="C3478" t="inlineStr">
         <is>
-          <t>EDILBERTO LEMOS DE LIMA</t>
+          <t>WENDERSON MARCOS DOS SANTOS</t>
         </is>
       </c>
       <c r="D3478" t="inlineStr">
         <is>
-          <t>ELEMOS</t>
+          <t>WWMARCOS</t>
         </is>
       </c>
     </row>
@@ -69998,136 +69998,136 @@
         </is>
       </c>
       <c r="B3479" t="n">
-        <v>3336</v>
+        <v>3335</v>
       </c>
       <c r="C3479" t="inlineStr">
         <is>
-          <t>EZEQUIEL SOUZA DO NASCIMENTO</t>
+          <t>EDILBERTO LEMOS DE LIMA</t>
         </is>
       </c>
       <c r="D3479" t="inlineStr">
         <is>
-          <t>ESNASCIMENTO</t>
+          <t>ELEMOS</t>
         </is>
       </c>
     </row>
     <row r="3480">
       <c r="A3480" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3480" t="n">
-        <v>3341</v>
+        <v>3336</v>
       </c>
       <c r="C3480" t="inlineStr">
         <is>
-          <t>ALCIONE MARIANO DE OLIVEIRA</t>
+          <t>EZEQUIEL SOUZA DO NASCIMENTO</t>
         </is>
       </c>
       <c r="D3480" t="inlineStr">
         <is>
-          <t>AMOLIVEIRA</t>
+          <t>ESNASCIMENTO</t>
         </is>
       </c>
     </row>
     <row r="3481">
       <c r="A3481" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3481" t="n">
-        <v>3401</v>
+        <v>3341</v>
       </c>
       <c r="C3481" t="inlineStr">
         <is>
-          <t xml:space="preserve">TULIO HENRIQUE DA SILVA CARVALHO </t>
+          <t>ALCIONE MARIANO DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D3481" t="inlineStr">
         <is>
-          <t>TULIO</t>
+          <t>AMOLIVEIRA</t>
         </is>
       </c>
     </row>
     <row r="3482">
       <c r="A3482" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3482" t="n">
-        <v>3411</v>
+        <v>3401</v>
       </c>
       <c r="C3482" t="inlineStr">
         <is>
-          <t>CONEXAO RUBYA DANILLA</t>
+          <t xml:space="preserve">TULIO HENRIQUE DA SILVA CARVALHO </t>
         </is>
       </c>
       <c r="D3482" t="inlineStr">
         <is>
-          <t>CONEXAORUBYA</t>
+          <t>TULIO</t>
         </is>
       </c>
     </row>
     <row r="3483">
       <c r="A3483" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3483" t="n">
-        <v>3412</v>
+        <v>3411</v>
       </c>
       <c r="C3483" t="inlineStr">
         <is>
-          <t>CONEXAO RAFAEL</t>
+          <t>CONEXAO RUBYA DANILLA</t>
         </is>
       </c>
       <c r="D3483" t="inlineStr">
         <is>
-          <t>CONEXAORAFAEL</t>
+          <t>CONEXAORUBYA</t>
         </is>
       </c>
     </row>
     <row r="3484">
       <c r="A3484" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3484" t="n">
-        <v>3558</v>
+        <v>3412</v>
       </c>
       <c r="C3484" t="inlineStr">
         <is>
-          <t>WALLYS QUEIROZ VIANA</t>
+          <t>CONEXAO RAFAEL</t>
         </is>
       </c>
       <c r="D3484" t="inlineStr">
         <is>
-          <t>WALLYS</t>
+          <t>CONEXAORAFAEL</t>
         </is>
       </c>
     </row>
     <row r="3485">
       <c r="A3485" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3485" t="n">
-        <v>3264</v>
+        <v>3558</v>
       </c>
       <c r="C3485" t="inlineStr">
         <is>
-          <t xml:space="preserve">WILTON CARLOS MACIEL DE ASSIS </t>
+          <t>WALLYS QUEIROZ VIANA</t>
         </is>
       </c>
       <c r="D3485" t="inlineStr">
         <is>
-          <t>WCMACIEL</t>
+          <t>WALLYS</t>
         </is>
       </c>
     </row>
@@ -70138,56 +70138,56 @@
         </is>
       </c>
       <c r="B3486" t="n">
-        <v>3340</v>
+        <v>3264</v>
       </c>
       <c r="C3486" t="inlineStr">
         <is>
-          <t>ROGELENO FARIAS FEIJÃO FILHO</t>
+          <t xml:space="preserve">WILTON CARLOS MACIEL DE ASSIS </t>
         </is>
       </c>
       <c r="D3486" t="inlineStr">
         <is>
-          <t>RFEIJAO</t>
+          <t>WCMACIEL</t>
         </is>
       </c>
     </row>
     <row r="3487">
       <c r="A3487" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3487" t="n">
-        <v>940550</v>
+        <v>3340</v>
       </c>
       <c r="C3487" t="inlineStr">
         <is>
-          <t>RAFAELE RIBEIRO CARNEIRO</t>
+          <t>ROGELENO FARIAS FEIJÃO FILHO</t>
         </is>
       </c>
       <c r="D3487" t="inlineStr">
         <is>
-          <t>RAFAELE</t>
+          <t>RFEIJAO</t>
         </is>
       </c>
     </row>
     <row r="3488">
       <c r="A3488" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>99</t>
         </is>
       </c>
       <c r="B3488" t="n">
-        <v>3377</v>
+        <v>940550</v>
       </c>
       <c r="C3488" t="inlineStr">
         <is>
-          <t xml:space="preserve"> ISALTINO BISPO DE OLIVEIRA JUNIOR</t>
+          <t>RAFAELE RIBEIRO CARNEIRO</t>
         </is>
       </c>
       <c r="D3488" t="inlineStr">
         <is>
-          <t>BJUNIOR</t>
+          <t>RAFAELE</t>
         </is>
       </c>
     </row>
@@ -70198,56 +70198,56 @@
         </is>
       </c>
       <c r="B3489" t="n">
-        <v>3425</v>
+        <v>3377</v>
       </c>
       <c r="C3489" t="inlineStr">
         <is>
-          <t xml:space="preserve"> CIRLANE ARAUJO SOUZA </t>
+          <t xml:space="preserve"> ISALTINO BISPO DE OLIVEIRA JUNIOR</t>
         </is>
       </c>
       <c r="D3489" t="inlineStr">
         <is>
-          <t>CIRLANES</t>
+          <t>BJUNIOR</t>
         </is>
       </c>
     </row>
     <row r="3490">
       <c r="A3490" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3490" t="n">
-        <v>3454</v>
+        <v>3425</v>
       </c>
       <c r="C3490" t="inlineStr">
         <is>
-          <t>ANTONIA SAMARA DE SOUZA SOARES</t>
+          <t xml:space="preserve"> CIRLANE ARAUJO SOUZA </t>
         </is>
       </c>
       <c r="D3490" t="inlineStr">
         <is>
-          <t>ANTSAMARA</t>
+          <t>CIRLANES</t>
         </is>
       </c>
     </row>
     <row r="3491">
       <c r="A3491" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3491" t="n">
-        <v>3491</v>
+        <v>3454</v>
       </c>
       <c r="C3491" t="inlineStr">
         <is>
-          <t>PEDRO JOSE DO NASCIMENTO NETO</t>
+          <t>ANTONIA SAMARA DE SOUZA SOARES</t>
         </is>
       </c>
       <c r="D3491" t="inlineStr">
         <is>
-          <t>P.JOSE</t>
+          <t>ANTSAMARA</t>
         </is>
       </c>
     </row>
@@ -70258,36 +70258,36 @@
         </is>
       </c>
       <c r="B3492" t="n">
-        <v>3492</v>
+        <v>3491</v>
       </c>
       <c r="C3492" t="inlineStr">
         <is>
-          <t>PAULA CARLA CALDAS MOTA</t>
+          <t>PEDRO JOSE DO NASCIMENTO NETO</t>
         </is>
       </c>
       <c r="D3492" t="inlineStr">
         <is>
-          <t>P.CARLA</t>
+          <t>P.JOSE</t>
         </is>
       </c>
     </row>
     <row r="3493">
       <c r="A3493" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3493" t="n">
-        <v>3542</v>
+        <v>3492</v>
       </c>
       <c r="C3493" t="inlineStr">
         <is>
-          <t>ANTONIA MILENA SOUSA ANDRADE</t>
+          <t>PAULA CARLA CALDAS MOTA</t>
         </is>
       </c>
       <c r="D3493" t="inlineStr">
         <is>
-          <t>A.MILENA</t>
+          <t>P.CARLA</t>
         </is>
       </c>
     </row>
@@ -70298,56 +70298,56 @@
         </is>
       </c>
       <c r="B3494" t="n">
-        <v>3547</v>
+        <v>3542</v>
       </c>
       <c r="C3494" t="inlineStr">
         <is>
-          <t xml:space="preserve">DAVI PEREIRA DA SILVA </t>
+          <t>ANTONIA MILENA SOUSA ANDRADE</t>
         </is>
       </c>
       <c r="D3494" t="inlineStr">
         <is>
-          <t>DPSILVA</t>
+          <t>A.MILENA</t>
         </is>
       </c>
     </row>
     <row r="3495">
       <c r="A3495" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3495" t="n">
-        <v>3552</v>
+        <v>3547</v>
       </c>
       <c r="C3495" t="inlineStr">
         <is>
-          <t>PAULO SERGIO MENDES DE OLIVEIRA</t>
+          <t xml:space="preserve">DAVI PEREIRA DA SILVA </t>
         </is>
       </c>
       <c r="D3495" t="inlineStr">
         <is>
-          <t>PSMENDES</t>
+          <t>DPSILVA</t>
         </is>
       </c>
     </row>
     <row r="3496">
       <c r="A3496" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3496" t="n">
-        <v>3294</v>
+        <v>3552</v>
       </c>
       <c r="C3496" t="inlineStr">
         <is>
-          <t>GLEICIANE MIRANDA DE MORAIS</t>
+          <t>PAULO SERGIO MENDES DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D3496" t="inlineStr">
         <is>
-          <t>GMIRANDA</t>
+          <t>PSMENDES</t>
         </is>
       </c>
     </row>
@@ -70358,176 +70358,176 @@
         </is>
       </c>
       <c r="B3497" t="n">
-        <v>3295</v>
+        <v>3294</v>
       </c>
       <c r="C3497" t="inlineStr">
         <is>
-          <t>MARIA ESTEFANNY DA SILVA MOURA</t>
+          <t>GLEICIANE MIRANDA DE MORAIS</t>
         </is>
       </c>
       <c r="D3497" t="inlineStr">
         <is>
-          <t>MESTEFANNY</t>
+          <t>GMIRANDA</t>
         </is>
       </c>
     </row>
     <row r="3498">
       <c r="A3498" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3498" t="n">
-        <v>3296</v>
+        <v>3295</v>
       </c>
       <c r="C3498" t="inlineStr">
         <is>
-          <t>PEDRO IAGO FONSECA EVANGELISTA</t>
+          <t>MARIA ESTEFANNY DA SILVA MOURA</t>
         </is>
       </c>
       <c r="D3498" t="inlineStr">
         <is>
-          <t>PIFONSECA</t>
+          <t>MESTEFANNY</t>
         </is>
       </c>
     </row>
     <row r="3499">
       <c r="A3499" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3499" t="n">
-        <v>940544</v>
+        <v>3296</v>
       </c>
       <c r="C3499" t="inlineStr">
         <is>
-          <t>LUTY LOG TRANSPORTES - FL8</t>
+          <t>PEDRO IAGO FONSECA EVANGELISTA</t>
         </is>
       </c>
       <c r="D3499" t="inlineStr">
         <is>
-          <t>LUTY LOG</t>
+          <t>PIFONSECA</t>
         </is>
       </c>
     </row>
     <row r="3500">
       <c r="A3500" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B3500" t="n">
-        <v>3380</v>
+        <v>940544</v>
       </c>
       <c r="C3500" t="inlineStr">
         <is>
-          <t>FRANCISCO MATHEUS RABELO DA COSTA</t>
+          <t>LUTY LOG TRANSPORTES - FL8</t>
         </is>
       </c>
       <c r="D3500" t="inlineStr">
         <is>
-          <t>FMATHEUS</t>
+          <t>LUTY LOG</t>
         </is>
       </c>
     </row>
     <row r="3501">
       <c r="A3501" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3501" t="n">
-        <v>3410</v>
+        <v>3380</v>
       </c>
       <c r="C3501" t="inlineStr">
         <is>
-          <t xml:space="preserve"> BRENO ALLAN DE JESUS</t>
+          <t>FRANCISCO MATHEUS RABELO DA COSTA</t>
         </is>
       </c>
       <c r="D3501" t="inlineStr">
         <is>
-          <t>JESUS</t>
+          <t>FMATHEUS</t>
         </is>
       </c>
     </row>
     <row r="3502">
       <c r="A3502" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3502" t="n">
-        <v>3444</v>
+        <v>3410</v>
       </c>
       <c r="C3502" t="inlineStr">
         <is>
-          <t>THIAGO COSTA SILVA</t>
+          <t xml:space="preserve"> BRENO ALLAN DE JESUS</t>
         </is>
       </c>
       <c r="D3502" t="inlineStr">
         <is>
-          <t>THIAGOC</t>
+          <t>JESUS</t>
         </is>
       </c>
     </row>
     <row r="3503">
       <c r="A3503" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3503" t="n">
-        <v>3456</v>
+        <v>3444</v>
       </c>
       <c r="C3503" t="inlineStr">
         <is>
-          <t>FELIPE BOTH MAZUCHINI</t>
+          <t>THIAGO COSTA SILVA</t>
         </is>
       </c>
       <c r="D3503" t="inlineStr">
         <is>
-          <t>FELIPEB</t>
+          <t>THIAGOC</t>
         </is>
       </c>
     </row>
     <row r="3504">
       <c r="A3504" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3504" t="n">
-        <v>3457</v>
+        <v>3456</v>
       </c>
       <c r="C3504" t="inlineStr">
         <is>
-          <t>FRANKLIN VIEIRA GOMES</t>
+          <t>FELIPE BOTH MAZUCHINI</t>
         </is>
       </c>
       <c r="D3504" t="inlineStr">
         <is>
-          <t>VIEIRAF</t>
+          <t>FELIPEB</t>
         </is>
       </c>
     </row>
     <row r="3505">
       <c r="A3505" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3505" t="n">
-        <v>3507</v>
+        <v>3457</v>
       </c>
       <c r="C3505" t="inlineStr">
         <is>
-          <t>KARINE TEODORA ALVES DE OLIVEIRA</t>
+          <t>FRANKLIN VIEIRA GOMES</t>
         </is>
       </c>
       <c r="D3505" t="inlineStr">
         <is>
-          <t>KOLIVEIRA</t>
+          <t>VIEIRAF</t>
         </is>
       </c>
     </row>
@@ -70538,14 +70538,34 @@
         </is>
       </c>
       <c r="B3506" t="n">
+        <v>3507</v>
+      </c>
+      <c r="C3506" t="inlineStr">
+        <is>
+          <t>KARINE TEODORA ALVES DE OLIVEIRA</t>
+        </is>
+      </c>
+      <c r="D3506" t="inlineStr">
+        <is>
+          <t>KOLIVEIRA</t>
+        </is>
+      </c>
+    </row>
+    <row r="3507">
+      <c r="A3507" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B3507" t="n">
         <v>3520</v>
       </c>
-      <c r="C3506" t="inlineStr">
+      <c r="C3507" t="inlineStr">
         <is>
           <t xml:space="preserve"> EMERSON FILIPE MELO DE AGUIAR</t>
         </is>
       </c>
-      <c r="D3506" t="inlineStr">
+      <c r="D3507" t="inlineStr">
         <is>
           <t>E.FILIPE</t>
         </is>

</xml_diff>

<commit_message>
chore(data): batch update intraday televendas - 08:03:16
</commit_message>
<xml_diff>
--- a/data/dim_televendas.xlsx
+++ b/data/dim_televendas.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3507"/>
+  <dimension ref="A1:D3508"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -67394,100 +67394,100 @@
     <row r="3349">
       <c r="A3349" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3349" t="n">
-        <v>3303</v>
+        <v>3595</v>
       </c>
       <c r="C3349" t="inlineStr">
         <is>
-          <t>DANIEL ALVES RODRIGUES</t>
+          <t>MIRLLENE PEREIRA RODRIGUES ROCHA</t>
         </is>
       </c>
       <c r="D3349" t="inlineStr">
         <is>
-          <t>DARODRIGUES</t>
+          <t>MIRLLENE</t>
         </is>
       </c>
     </row>
     <row r="3350">
       <c r="A3350" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3350" t="n">
-        <v>3316</v>
+        <v>3303</v>
       </c>
       <c r="C3350" t="inlineStr">
         <is>
-          <t xml:space="preserve">MARCELO PEREIRA BASTOS </t>
+          <t>DANIEL ALVES RODRIGUES</t>
         </is>
       </c>
       <c r="D3350" t="inlineStr">
         <is>
-          <t>MBASTOS</t>
+          <t>DARODRIGUES</t>
         </is>
       </c>
     </row>
     <row r="3351">
       <c r="A3351" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3351" t="n">
-        <v>3366</v>
+        <v>3316</v>
       </c>
       <c r="C3351" t="inlineStr">
         <is>
-          <t>MATEUS TEIXEIRA DA PAZ SILVA</t>
+          <t xml:space="preserve">MARCELO PEREIRA BASTOS </t>
         </is>
       </c>
       <c r="D3351" t="inlineStr">
         <is>
-          <t>PAZSILVA</t>
+          <t>MBASTOS</t>
         </is>
       </c>
     </row>
     <row r="3352">
       <c r="A3352" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3352" t="n">
-        <v>3393</v>
+        <v>3366</v>
       </c>
       <c r="C3352" t="inlineStr">
         <is>
-          <t xml:space="preserve">DAVID LUCAS RIBEIRO DOS SANTOS </t>
+          <t>MATEUS TEIXEIRA DA PAZ SILVA</t>
         </is>
       </c>
       <c r="D3352" t="inlineStr">
         <is>
-          <t>DLUCAS</t>
+          <t>PAZSILVA</t>
         </is>
       </c>
     </row>
     <row r="3353">
       <c r="A3353" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3353" t="n">
-        <v>3420</v>
+        <v>3393</v>
       </c>
       <c r="C3353" t="inlineStr">
         <is>
-          <t xml:space="preserve">CLAUDIO ROBERTO SILVA SOUZA </t>
+          <t xml:space="preserve">DAVID LUCAS RIBEIRO DOS SANTOS </t>
         </is>
       </c>
       <c r="D3353" t="inlineStr">
         <is>
-          <t>CLAUDIO21</t>
+          <t>DLUCAS</t>
         </is>
       </c>
     </row>
@@ -67498,16 +67498,16 @@
         </is>
       </c>
       <c r="B3354" t="n">
-        <v>3421</v>
+        <v>3420</v>
       </c>
       <c r="C3354" t="inlineStr">
         <is>
-          <t>WILSON PORTUGAL AZEVEDO FILHO</t>
+          <t xml:space="preserve">CLAUDIO ROBERTO SILVA SOUZA </t>
         </is>
       </c>
       <c r="D3354" t="inlineStr">
         <is>
-          <t>WILSONF</t>
+          <t>CLAUDIO21</t>
         </is>
       </c>
     </row>
@@ -67518,176 +67518,176 @@
         </is>
       </c>
       <c r="B3355" t="n">
-        <v>3439</v>
+        <v>3421</v>
       </c>
       <c r="C3355" t="inlineStr">
         <is>
-          <t>FERNANDA MASCARENHAS CEDRAZ</t>
+          <t>WILSON PORTUGAL AZEVEDO FILHO</t>
         </is>
       </c>
       <c r="D3355" t="inlineStr">
         <is>
-          <t>FERNANDAM</t>
+          <t>WILSONF</t>
         </is>
       </c>
     </row>
     <row r="3356">
       <c r="A3356" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3356" t="n">
-        <v>3455</v>
+        <v>3439</v>
       </c>
       <c r="C3356" t="inlineStr">
         <is>
-          <t xml:space="preserve">MARDONIO CUNHA BASILIO </t>
+          <t>FERNANDA MASCARENHAS CEDRAZ</t>
         </is>
       </c>
       <c r="D3356" t="inlineStr">
         <is>
-          <t>MARDONIO1</t>
+          <t>FERNANDAM</t>
         </is>
       </c>
     </row>
     <row r="3357">
       <c r="A3357" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3357" t="n">
-        <v>3508</v>
+        <v>3455</v>
       </c>
       <c r="C3357" t="inlineStr">
         <is>
-          <t>REBECA PIRES DE SOUZA MELO</t>
+          <t xml:space="preserve">MARDONIO CUNHA BASILIO </t>
         </is>
       </c>
       <c r="D3357" t="inlineStr">
         <is>
-          <t>RPMELO</t>
+          <t>MARDONIO1</t>
         </is>
       </c>
     </row>
     <row r="3358">
       <c r="A3358" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3358" t="n">
-        <v>3543</v>
+        <v>3508</v>
       </c>
       <c r="C3358" t="inlineStr">
         <is>
-          <t>JOAO GABRIEL BARBOSA FIRMINO</t>
+          <t>REBECA PIRES DE SOUZA MELO</t>
         </is>
       </c>
       <c r="D3358" t="inlineStr">
         <is>
-          <t>JOAOG</t>
+          <t>RPMELO</t>
         </is>
       </c>
     </row>
     <row r="3359">
       <c r="A3359" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3359" t="n">
-        <v>3580</v>
+        <v>3543</v>
       </c>
       <c r="C3359" t="inlineStr">
         <is>
-          <t>ALEXANDRE MARTINS CHAVES</t>
+          <t>JOAO GABRIEL BARBOSA FIRMINO</t>
         </is>
       </c>
       <c r="D3359" t="inlineStr">
         <is>
-          <t>MARTINS</t>
+          <t>JOAOG</t>
         </is>
       </c>
     </row>
     <row r="3360">
       <c r="A3360" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3360" t="n">
-        <v>3351</v>
+        <v>3580</v>
       </c>
       <c r="C3360" t="inlineStr">
         <is>
-          <t>HAWLLYSON DA SILVA COUTINHO</t>
+          <t>ALEXANDRE MARTINS CHAVES</t>
         </is>
       </c>
       <c r="D3360" t="inlineStr">
         <is>
-          <t>HCOUTINHO</t>
+          <t>MARTINS</t>
         </is>
       </c>
     </row>
     <row r="3361">
       <c r="A3361" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3361" t="n">
-        <v>940553</v>
+        <v>3351</v>
       </c>
       <c r="C3361" t="inlineStr">
         <is>
-          <t>LUTY TRANSPORTES- BA</t>
+          <t>HAWLLYSON DA SILVA COUTINHO</t>
         </is>
       </c>
       <c r="D3361" t="inlineStr">
         <is>
-          <t>LUTY TRANSPORTE</t>
+          <t>HCOUTINHO</t>
         </is>
       </c>
     </row>
     <row r="3362">
       <c r="A3362" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3362" t="n">
-        <v>3391</v>
+        <v>940553</v>
       </c>
       <c r="C3362" t="inlineStr">
         <is>
-          <t xml:space="preserve">NIKSON DA SILVA ALVES </t>
+          <t>LUTY TRANSPORTES- BA</t>
         </is>
       </c>
       <c r="D3362" t="inlineStr">
         <is>
-          <t>NIKSON</t>
+          <t>LUTY TRANSPORTE</t>
         </is>
       </c>
     </row>
     <row r="3363">
       <c r="A3363" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3363" t="n">
-        <v>3397</v>
+        <v>3391</v>
       </c>
       <c r="C3363" t="inlineStr">
         <is>
-          <t>EDILANE MENESES BALTAZAR</t>
+          <t xml:space="preserve">NIKSON DA SILVA ALVES </t>
         </is>
       </c>
       <c r="D3363" t="inlineStr">
         <is>
-          <t>EDILANE</t>
+          <t>NIKSON</t>
         </is>
       </c>
     </row>
@@ -67698,56 +67698,56 @@
         </is>
       </c>
       <c r="B3364" t="n">
-        <v>3398</v>
+        <v>3397</v>
       </c>
       <c r="C3364" t="inlineStr">
         <is>
-          <t>LUANA MARIA ROSIO DA SILVA</t>
+          <t>EDILANE MENESES BALTAZAR</t>
         </is>
       </c>
       <c r="D3364" t="inlineStr">
         <is>
-          <t>LUMARIA</t>
+          <t>EDILANE</t>
         </is>
       </c>
     </row>
     <row r="3365">
       <c r="A3365" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3365" t="n">
-        <v>3400</v>
+        <v>3398</v>
       </c>
       <c r="C3365" t="inlineStr">
         <is>
-          <t>ELILTON PINTO ROMEU</t>
+          <t>LUANA MARIA ROSIO DA SILVA</t>
         </is>
       </c>
       <c r="D3365" t="inlineStr">
         <is>
-          <t>ELILTON</t>
+          <t>LUMARIA</t>
         </is>
       </c>
     </row>
     <row r="3366">
       <c r="A3366" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3366" t="n">
-        <v>3406</v>
+        <v>3400</v>
       </c>
       <c r="C3366" t="inlineStr">
         <is>
-          <t>CONEXAO ALDA</t>
+          <t>ELILTON PINTO ROMEU</t>
         </is>
       </c>
       <c r="D3366" t="inlineStr">
         <is>
-          <t>CONEXAOALDA</t>
+          <t>ELILTON</t>
         </is>
       </c>
     </row>
@@ -67758,176 +67758,176 @@
         </is>
       </c>
       <c r="B3367" t="n">
-        <v>3407</v>
+        <v>3406</v>
       </c>
       <c r="C3367" t="inlineStr">
         <is>
-          <t>CONEXAO IRACEMA</t>
+          <t>CONEXAO ALDA</t>
         </is>
       </c>
       <c r="D3367" t="inlineStr">
         <is>
-          <t>CONEXAOIRACEMA</t>
+          <t>CONEXAOALDA</t>
         </is>
       </c>
     </row>
     <row r="3368">
       <c r="A3368" t="inlineStr">
         <is>
-          <t>9999</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3368" t="n">
-        <v>3408</v>
+        <v>3407</v>
       </c>
       <c r="C3368" t="inlineStr">
         <is>
-          <t>CONEXAO TAMILES</t>
+          <t>CONEXAO IRACEMA</t>
         </is>
       </c>
       <c r="D3368" t="inlineStr">
         <is>
-          <t>CONEXAOTAMILES</t>
+          <t>CONEXAOIRACEMA</t>
         </is>
       </c>
     </row>
     <row r="3369">
       <c r="A3369" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>9999</t>
         </is>
       </c>
       <c r="B3369" t="n">
-        <v>3414</v>
+        <v>3408</v>
       </c>
       <c r="C3369" t="inlineStr">
         <is>
-          <t>CONEXAO ADM PI MA</t>
+          <t>CONEXAO TAMILES</t>
         </is>
       </c>
       <c r="D3369" t="inlineStr">
         <is>
-          <t>CONEXAOPIMA</t>
+          <t>CONEXAOTAMILES</t>
         </is>
       </c>
     </row>
     <row r="3370">
       <c r="A3370" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3370" t="n">
-        <v>3524</v>
+        <v>3414</v>
       </c>
       <c r="C3370" t="inlineStr">
         <is>
-          <t>LUIS FELIPE DA SILVA SOUSA</t>
+          <t>CONEXAO ADM PI MA</t>
         </is>
       </c>
       <c r="D3370" t="inlineStr">
         <is>
-          <t>L.FELIPE</t>
+          <t>CONEXAOPIMA</t>
         </is>
       </c>
     </row>
     <row r="3371">
       <c r="A3371" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3371" t="n">
-        <v>3531</v>
+        <v>3524</v>
       </c>
       <c r="C3371" t="inlineStr">
         <is>
-          <t>LEICIANE COELHO SILVA</t>
+          <t>LUIS FELIPE DA SILVA SOUSA</t>
         </is>
       </c>
       <c r="D3371" t="inlineStr">
         <is>
-          <t>LEI.SILVA</t>
+          <t>L.FELIPE</t>
         </is>
       </c>
     </row>
     <row r="3372">
       <c r="A3372" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3372" t="n">
-        <v>3550</v>
+        <v>3531</v>
       </c>
       <c r="C3372" t="inlineStr">
         <is>
-          <t>IARGO GABRIEL SANTOS DE OLIVEIRA</t>
+          <t>LEICIANE COELHO SILVA</t>
         </is>
       </c>
       <c r="D3372" t="inlineStr">
         <is>
-          <t>IARGOG</t>
+          <t>LEI.SILVA</t>
         </is>
       </c>
     </row>
     <row r="3373">
       <c r="A3373" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3373" t="n">
-        <v>940567</v>
+        <v>3550</v>
       </c>
       <c r="C3373" t="inlineStr">
         <is>
-          <t>MS CARGAS E TRANSPORTES</t>
+          <t>IARGO GABRIEL SANTOS DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D3373" t="inlineStr">
         <is>
-          <t>ALAN BARBOSA</t>
+          <t>IARGOG</t>
         </is>
       </c>
     </row>
     <row r="3374">
       <c r="A3374" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3374" t="n">
-        <v>3560</v>
+        <v>940567</v>
       </c>
       <c r="C3374" t="inlineStr">
         <is>
-          <t>MARIA EDUARDA MELO DOS SANTOS</t>
+          <t>MS CARGAS E TRANSPORTES</t>
         </is>
       </c>
       <c r="D3374" t="inlineStr">
         <is>
-          <t>EDU.MELO</t>
+          <t>ALAN BARBOSA</t>
         </is>
       </c>
     </row>
     <row r="3375">
       <c r="A3375" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3375" t="n">
-        <v>3355</v>
+        <v>3560</v>
       </c>
       <c r="C3375" t="inlineStr">
         <is>
-          <t>HUGO MATHEUS DA COSTA FEITOSA</t>
+          <t>MARIA EDUARDA MELO DOS SANTOS</t>
         </is>
       </c>
       <c r="D3375" t="inlineStr">
         <is>
-          <t>HMFEITOSA</t>
+          <t>EDU.MELO</t>
         </is>
       </c>
     </row>
@@ -67938,96 +67938,96 @@
         </is>
       </c>
       <c r="B3376" t="n">
-        <v>3356</v>
+        <v>3355</v>
       </c>
       <c r="C3376" t="inlineStr">
         <is>
-          <t>BRENDA LIMA DE OLIVEIRA CUNHA</t>
+          <t>HUGO MATHEUS DA COSTA FEITOSA</t>
         </is>
       </c>
       <c r="D3376" t="inlineStr">
         <is>
-          <t>BLCUNHA</t>
+          <t>HMFEITOSA</t>
         </is>
       </c>
     </row>
     <row r="3377">
       <c r="A3377" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3377" t="n">
-        <v>3361</v>
+        <v>3356</v>
       </c>
       <c r="C3377" t="inlineStr">
         <is>
-          <t>WLADIA DE ARAUJO BASTOS</t>
+          <t>BRENDA LIMA DE OLIVEIRA CUNHA</t>
         </is>
       </c>
       <c r="D3377" t="inlineStr">
         <is>
-          <t>WABASTOS</t>
+          <t>BLCUNHA</t>
         </is>
       </c>
     </row>
     <row r="3378">
       <c r="A3378" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3378" t="n">
-        <v>3362</v>
+        <v>3361</v>
       </c>
       <c r="C3378" t="inlineStr">
         <is>
-          <t>CARLOS HENRIQUE MELO DA SILVA</t>
+          <t>WLADIA DE ARAUJO BASTOS</t>
         </is>
       </c>
       <c r="D3378" t="inlineStr">
         <is>
-          <t>CHMELO</t>
+          <t>WABASTOS</t>
         </is>
       </c>
     </row>
     <row r="3379">
       <c r="A3379" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3379" t="n">
-        <v>3375</v>
+        <v>3362</v>
       </c>
       <c r="C3379" t="inlineStr">
         <is>
-          <t>AFONSO DE SOUSA RAMOS FILHO</t>
+          <t>CARLOS HENRIQUE MELO DA SILVA</t>
         </is>
       </c>
       <c r="D3379" t="inlineStr">
         <is>
-          <t>AFILHO</t>
+          <t>CHMELO</t>
         </is>
       </c>
     </row>
     <row r="3380">
       <c r="A3380" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3380" t="n">
-        <v>3404</v>
+        <v>3375</v>
       </c>
       <c r="C3380" t="inlineStr">
         <is>
-          <t>NOVATO 4 COM</t>
+          <t>AFONSO DE SOUSA RAMOS FILHO</t>
         </is>
       </c>
       <c r="D3380" t="inlineStr">
         <is>
-          <t>NOVATO4COM</t>
+          <t>AFILHO</t>
         </is>
       </c>
     </row>
@@ -68038,176 +68038,176 @@
         </is>
       </c>
       <c r="B3381" t="n">
-        <v>3405</v>
+        <v>3404</v>
       </c>
       <c r="C3381" t="inlineStr">
         <is>
-          <t>NOVATO 5 COM</t>
+          <t>NOVATO 4 COM</t>
         </is>
       </c>
       <c r="D3381" t="inlineStr">
         <is>
-          <t>NOVATO5COM</t>
+          <t>NOVATO4COM</t>
         </is>
       </c>
     </row>
     <row r="3382">
       <c r="A3382" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3382" t="n">
-        <v>3447</v>
+        <v>3405</v>
       </c>
       <c r="C3382" t="inlineStr">
         <is>
-          <t>RAYSSA KEYCE LINHARES AQUINO</t>
+          <t>NOVATO 5 COM</t>
         </is>
       </c>
       <c r="D3382" t="inlineStr">
         <is>
-          <t>RAYSSAK</t>
+          <t>NOVATO5COM</t>
         </is>
       </c>
     </row>
     <row r="3383">
       <c r="A3383" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3383" t="n">
-        <v>940559</v>
+        <v>3447</v>
       </c>
       <c r="C3383" t="inlineStr">
         <is>
-          <t>WALLEF DE OLIVEIRA</t>
+          <t>RAYSSA KEYCE LINHARES AQUINO</t>
         </is>
       </c>
       <c r="D3383" t="inlineStr">
         <is>
-          <t>WALLEF</t>
+          <t>RAYSSAK</t>
         </is>
       </c>
     </row>
     <row r="3384">
       <c r="A3384" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>99</t>
         </is>
       </c>
       <c r="B3384" t="n">
-        <v>3489</v>
+        <v>940559</v>
       </c>
       <c r="C3384" t="inlineStr">
         <is>
-          <t>MARCELA KARINA PEREIRA VELOSO</t>
+          <t>WALLEF DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D3384" t="inlineStr">
         <is>
-          <t>MKARINA</t>
+          <t>WALLEF</t>
         </is>
       </c>
     </row>
     <row r="3385">
       <c r="A3385" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3385" t="n">
-        <v>3490</v>
+        <v>3489</v>
       </c>
       <c r="C3385" t="inlineStr">
         <is>
-          <t>JOSE MAILSON GOMES NUNES</t>
+          <t>MARCELA KARINA PEREIRA VELOSO</t>
         </is>
       </c>
       <c r="D3385" t="inlineStr">
         <is>
-          <t>J.MAILSON</t>
+          <t>MKARINA</t>
         </is>
       </c>
     </row>
     <row r="3386">
       <c r="A3386" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3386" t="n">
-        <v>3537</v>
+        <v>3490</v>
       </c>
       <c r="C3386" t="inlineStr">
         <is>
-          <t>ALDAIR PEDRO DA SILVA</t>
+          <t>JOSE MAILSON GOMES NUNES</t>
         </is>
       </c>
       <c r="D3386" t="inlineStr">
         <is>
-          <t>A.PEDRO</t>
+          <t>J.MAILSON</t>
         </is>
       </c>
     </row>
     <row r="3387">
       <c r="A3387" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3387" t="n">
-        <v>3549</v>
+        <v>3537</v>
       </c>
       <c r="C3387" t="inlineStr">
         <is>
-          <t xml:space="preserve">FERNANDA CAROLINE E CESAR SOUSA </t>
+          <t>ALDAIR PEDRO DA SILVA</t>
         </is>
       </c>
       <c r="D3387" t="inlineStr">
         <is>
-          <t>FCAROLINE</t>
+          <t>A.PEDRO</t>
         </is>
       </c>
     </row>
     <row r="3388">
       <c r="A3388" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3388" t="n">
-        <v>3581</v>
+        <v>3549</v>
       </c>
       <c r="C3388" t="inlineStr">
         <is>
-          <t xml:space="preserve">VALQUIRIO OLIVEIRA SOUSA </t>
+          <t xml:space="preserve">FERNANDA CAROLINE E CESAR SOUSA </t>
         </is>
       </c>
       <c r="D3388" t="inlineStr">
         <is>
-          <t>VALQUIRIO</t>
+          <t>FCAROLINE</t>
         </is>
       </c>
     </row>
     <row r="3389">
       <c r="A3389" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3389" t="n">
-        <v>3337</v>
+        <v>3581</v>
       </c>
       <c r="C3389" t="inlineStr">
         <is>
-          <t>WESLEY FONTES DE ALMEIDA</t>
+          <t xml:space="preserve">VALQUIRIO OLIVEIRA SOUSA </t>
         </is>
       </c>
       <c r="D3389" t="inlineStr">
         <is>
-          <t>WFALMEIDA</t>
+          <t>VALQUIRIO</t>
         </is>
       </c>
     </row>
@@ -68218,16 +68218,16 @@
         </is>
       </c>
       <c r="B3390" t="n">
-        <v>3338</v>
+        <v>3337</v>
       </c>
       <c r="C3390" t="inlineStr">
         <is>
-          <t>FRANCISCA SAMARA MENDES DE OLIVEIRA C</t>
+          <t>WESLEY FONTES DE ALMEIDA</t>
         </is>
       </c>
       <c r="D3390" t="inlineStr">
         <is>
-          <t>FSCUNHA</t>
+          <t>WFALMEIDA</t>
         </is>
       </c>
     </row>
@@ -68238,176 +68238,176 @@
         </is>
       </c>
       <c r="B3391" t="n">
-        <v>3339</v>
+        <v>3338</v>
       </c>
       <c r="C3391" t="inlineStr">
         <is>
-          <t>MAYARA THALYA DIAS DE ANDRADE</t>
+          <t>FRANCISCA SAMARA MENDES DE OLIVEIRA C</t>
         </is>
       </c>
       <c r="D3391" t="inlineStr">
         <is>
-          <t>MTANDRADE</t>
+          <t>FSCUNHA</t>
         </is>
       </c>
     </row>
     <row r="3392">
       <c r="A3392" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3392" t="n">
-        <v>3359</v>
+        <v>3339</v>
       </c>
       <c r="C3392" t="inlineStr">
         <is>
-          <t xml:space="preserve">EVANESSA DA SILVA E SILVA </t>
+          <t>MAYARA THALYA DIAS DE ANDRADE</t>
         </is>
       </c>
       <c r="D3392" t="inlineStr">
         <is>
-          <t>EVANESSAS</t>
+          <t>MTANDRADE</t>
         </is>
       </c>
     </row>
     <row r="3393">
       <c r="A3393" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3393" t="n">
-        <v>3360</v>
+        <v>3359</v>
       </c>
       <c r="C3393" t="inlineStr">
         <is>
-          <t>THIAGO DE CARVALHO ARAUJO</t>
+          <t xml:space="preserve">EVANESSA DA SILVA E SILVA </t>
         </is>
       </c>
       <c r="D3393" t="inlineStr">
         <is>
-          <t>TCARAUJO</t>
+          <t>EVANESSAS</t>
         </is>
       </c>
     </row>
     <row r="3394">
       <c r="A3394" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3394" t="n">
-        <v>3481</v>
+        <v>3360</v>
       </c>
       <c r="C3394" t="inlineStr">
         <is>
-          <t xml:space="preserve">EDSON DA PAZ LIMA </t>
+          <t>THIAGO DE CARVALHO ARAUJO</t>
         </is>
       </c>
       <c r="D3394" t="inlineStr">
         <is>
-          <t>EDPAZ</t>
+          <t>TCARAUJO</t>
         </is>
       </c>
     </row>
     <row r="3395">
       <c r="A3395" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3395" t="n">
-        <v>3494</v>
+        <v>3481</v>
       </c>
       <c r="C3395" t="inlineStr">
         <is>
-          <t>ANTONIO CRISTINA BRITO GOMES</t>
+          <t xml:space="preserve">EDSON DA PAZ LIMA </t>
         </is>
       </c>
       <c r="D3395" t="inlineStr">
         <is>
-          <t>CRIS.GOMES</t>
+          <t>EDPAZ</t>
         </is>
       </c>
     </row>
     <row r="3396">
       <c r="A3396" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3396" t="n">
-        <v>3498</v>
+        <v>3494</v>
       </c>
       <c r="C3396" t="inlineStr">
         <is>
-          <t>SILVESTRA COSTA NUNES</t>
+          <t>ANTONIO CRISTINA BRITO GOMES</t>
         </is>
       </c>
       <c r="D3396" t="inlineStr">
         <is>
-          <t>SCNUNES</t>
+          <t>CRIS.GOMES</t>
         </is>
       </c>
     </row>
     <row r="3397">
       <c r="A3397" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3397" t="n">
-        <v>940562</v>
+        <v>3498</v>
       </c>
       <c r="C3397" t="inlineStr">
         <is>
-          <t>FRANCISCO DAVID ASSUNCAO ALVES</t>
+          <t>SILVESTRA COSTA NUNES</t>
         </is>
       </c>
       <c r="D3397" t="inlineStr">
         <is>
-          <t>ASSUNÇÃO</t>
+          <t>SCNUNES</t>
         </is>
       </c>
     </row>
     <row r="3398">
       <c r="A3398" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>99</t>
         </is>
       </c>
       <c r="B3398" t="n">
-        <v>3513</v>
+        <v>940562</v>
       </c>
       <c r="C3398" t="inlineStr">
         <is>
-          <t>RENARA ANDRADE MATIAS</t>
+          <t>FRANCISCO DAVID ASSUNCAO ALVES</t>
         </is>
       </c>
       <c r="D3398" t="inlineStr">
         <is>
-          <t>R.ANDRADE</t>
+          <t>ASSUNÇÃO</t>
         </is>
       </c>
     </row>
     <row r="3399">
       <c r="A3399" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3399" t="n">
-        <v>3275</v>
+        <v>3513</v>
       </c>
       <c r="C3399" t="inlineStr">
         <is>
-          <t>MARIA APARECIDA COELHO SILVA</t>
+          <t>RENARA ANDRADE MATIAS</t>
         </is>
       </c>
       <c r="D3399" t="inlineStr">
         <is>
-          <t>MCOELHO</t>
+          <t>R.ANDRADE</t>
         </is>
       </c>
     </row>
@@ -68418,136 +68418,136 @@
         </is>
       </c>
       <c r="B3400" t="n">
-        <v>3276</v>
+        <v>3275</v>
       </c>
       <c r="C3400" t="inlineStr">
         <is>
-          <t xml:space="preserve">PEROLA DE JESUS AMORIM SOUSA </t>
+          <t>MARIA APARECIDA COELHO SILVA</t>
         </is>
       </c>
       <c r="D3400" t="inlineStr">
         <is>
-          <t>PJESUS</t>
+          <t>MCOELHO</t>
         </is>
       </c>
     </row>
     <row r="3401">
       <c r="A3401" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3401" t="n">
-        <v>3526</v>
+        <v>3276</v>
       </c>
       <c r="C3401" t="inlineStr">
         <is>
-          <t>JOYCE NAZARE CORREA</t>
+          <t xml:space="preserve">PEROLA DE JESUS AMORIM SOUSA </t>
         </is>
       </c>
       <c r="D3401" t="inlineStr">
         <is>
-          <t>J.NAZARE</t>
+          <t>PJESUS</t>
         </is>
       </c>
     </row>
     <row r="3402">
       <c r="A3402" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3402" t="n">
-        <v>3527</v>
+        <v>3526</v>
       </c>
       <c r="C3402" t="inlineStr">
         <is>
-          <t>GILVANA DA SILVA MONTELES</t>
+          <t>JOYCE NAZARE CORREA</t>
         </is>
       </c>
       <c r="D3402" t="inlineStr">
         <is>
-          <t>GIL.SILVA</t>
+          <t>J.NAZARE</t>
         </is>
       </c>
     </row>
     <row r="3403">
       <c r="A3403" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3403" t="n">
-        <v>3548</v>
+        <v>3527</v>
       </c>
       <c r="C3403" t="inlineStr">
         <is>
-          <t>JAMILLY MARIA HENRIQUE ARAUJO</t>
+          <t>GILVANA DA SILVA MONTELES</t>
         </is>
       </c>
       <c r="D3403" t="inlineStr">
         <is>
-          <t>JAMILLY</t>
+          <t>GIL.SILVA</t>
         </is>
       </c>
     </row>
     <row r="3404">
       <c r="A3404" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3404" t="n">
-        <v>3551</v>
+        <v>3548</v>
       </c>
       <c r="C3404" t="inlineStr">
         <is>
-          <t xml:space="preserve">VITOR MANOEL DA SILVA BARBOSA </t>
+          <t>JAMILLY MARIA HENRIQUE ARAUJO</t>
         </is>
       </c>
       <c r="D3404" t="inlineStr">
         <is>
-          <t>VMANOEL</t>
+          <t>JAMILLY</t>
         </is>
       </c>
     </row>
     <row r="3405">
       <c r="A3405" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3405" t="n">
-        <v>3588</v>
+        <v>3551</v>
       </c>
       <c r="C3405" t="inlineStr">
         <is>
-          <t>BRUNA RAISEYLLA SANTOS DE SALES</t>
+          <t xml:space="preserve">VITOR MANOEL DA SILVA BARBOSA </t>
         </is>
       </c>
       <c r="D3405" t="inlineStr">
         <is>
-          <t>BRU.SALES</t>
+          <t>VMANOEL</t>
         </is>
       </c>
     </row>
     <row r="3406">
       <c r="A3406" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3406" t="n">
-        <v>940525</v>
+        <v>3588</v>
       </c>
       <c r="C3406" t="inlineStr">
         <is>
-          <t>SANDUWELLINGTON</t>
+          <t>BRUNA RAISEYLLA SANTOS DE SALES</t>
         </is>
       </c>
       <c r="D3406" t="inlineStr">
         <is>
-          <t>SANDUWELLINGTON</t>
+          <t>BRU.SALES</t>
         </is>
       </c>
     </row>
@@ -68558,36 +68558,36 @@
         </is>
       </c>
       <c r="B3407" t="n">
-        <v>3369</v>
+        <v>940525</v>
       </c>
       <c r="C3407" t="inlineStr">
         <is>
-          <t xml:space="preserve">PRISCILA DOS SANTOS LOPES </t>
+          <t>SANDUWELLINGTON</t>
         </is>
       </c>
       <c r="D3407" t="inlineStr">
         <is>
-          <t>PSLOPES</t>
+          <t>SANDUWELLINGTON</t>
         </is>
       </c>
     </row>
     <row r="3408">
       <c r="A3408" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3408" t="n">
-        <v>3433</v>
+        <v>3369</v>
       </c>
       <c r="C3408" t="inlineStr">
         <is>
-          <t>BRUNO NUNES CRUZ</t>
+          <t xml:space="preserve">PRISCILA DOS SANTOS LOPES </t>
         </is>
       </c>
       <c r="D3408" t="inlineStr">
         <is>
-          <t>BRUNOCRUZ</t>
+          <t>PSLOPES</t>
         </is>
       </c>
     </row>
@@ -68598,36 +68598,36 @@
         </is>
       </c>
       <c r="B3409" t="n">
-        <v>3434</v>
+        <v>3433</v>
       </c>
       <c r="C3409" t="inlineStr">
         <is>
-          <t>ANA TERCIA DE LIMA SA CARVALHO SERAFIM</t>
+          <t>BRUNO NUNES CRUZ</t>
         </is>
       </c>
       <c r="D3409" t="inlineStr">
         <is>
-          <t>ANATER</t>
+          <t>BRUNOCRUZ</t>
         </is>
       </c>
     </row>
     <row r="3410">
       <c r="A3410" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3410" t="n">
-        <v>3502</v>
+        <v>3434</v>
       </c>
       <c r="C3410" t="inlineStr">
         <is>
-          <t>LUIZ FELIPE MACHADO BARRETO</t>
+          <t>ANA TERCIA DE LIMA SA CARVALHO SERAFIM</t>
         </is>
       </c>
       <c r="D3410" t="inlineStr">
         <is>
-          <t>LUIZ.FELIPE</t>
+          <t>ANATER</t>
         </is>
       </c>
     </row>
@@ -68638,36 +68638,36 @@
         </is>
       </c>
       <c r="B3411" t="n">
-        <v>3503</v>
+        <v>3502</v>
       </c>
       <c r="C3411" t="inlineStr">
         <is>
-          <t>FABIO OLIVEIRA SILVA</t>
+          <t>LUIZ FELIPE MACHADO BARRETO</t>
         </is>
       </c>
       <c r="D3411" t="inlineStr">
         <is>
-          <t>FOSILVA</t>
+          <t>LUIZ.FELIPE</t>
         </is>
       </c>
     </row>
     <row r="3412">
       <c r="A3412" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3412" t="n">
-        <v>3554</v>
+        <v>3503</v>
       </c>
       <c r="C3412" t="inlineStr">
         <is>
-          <t xml:space="preserve">MANOEL RIBEIRO DE SOUZA JUNIOR </t>
+          <t>FABIO OLIVEIRA SILVA</t>
         </is>
       </c>
       <c r="D3412" t="inlineStr">
         <is>
-          <t>MRJUNIOR</t>
+          <t>FOSILVA</t>
         </is>
       </c>
     </row>
@@ -68678,16 +68678,16 @@
         </is>
       </c>
       <c r="B3413" t="n">
-        <v>3568</v>
+        <v>3554</v>
       </c>
       <c r="C3413" t="inlineStr">
         <is>
-          <t xml:space="preserve">ANGELICA TORRES DA SILVA </t>
+          <t xml:space="preserve">MANOEL RIBEIRO DE SOUZA JUNIOR </t>
         </is>
       </c>
       <c r="D3413" t="inlineStr">
         <is>
-          <t>ANGEL.TORRES</t>
+          <t>MRJUNIOR</t>
         </is>
       </c>
     </row>
@@ -68698,56 +68698,56 @@
         </is>
       </c>
       <c r="B3414" t="n">
-        <v>3569</v>
+        <v>3568</v>
       </c>
       <c r="C3414" t="inlineStr">
         <is>
-          <t>LORENA DE LIMA MATOS</t>
+          <t xml:space="preserve">ANGELICA TORRES DA SILVA </t>
         </is>
       </c>
       <c r="D3414" t="inlineStr">
         <is>
-          <t>LORE.LIMA</t>
+          <t>ANGEL.TORRES</t>
         </is>
       </c>
     </row>
     <row r="3415">
       <c r="A3415" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3415" t="n">
-        <v>3576</v>
+        <v>3569</v>
       </c>
       <c r="C3415" t="inlineStr">
         <is>
-          <t>ANA BEATRIZ PARENTE CAVALCANTE</t>
+          <t>LORENA DE LIMA MATOS</t>
         </is>
       </c>
       <c r="D3415" t="inlineStr">
         <is>
-          <t>A.BEATRIZ</t>
+          <t>LORE.LIMA</t>
         </is>
       </c>
     </row>
     <row r="3416">
       <c r="A3416" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3416" t="n">
-        <v>940549</v>
+        <v>3576</v>
       </c>
       <c r="C3416" t="inlineStr">
         <is>
-          <t>EDILSON ARAUJO - FL9</t>
+          <t>ANA BEATRIZ PARENTE CAVALCANTE</t>
         </is>
       </c>
       <c r="D3416" t="inlineStr">
         <is>
-          <t>EDILSON</t>
+          <t>A.BEATRIZ</t>
         </is>
       </c>
     </row>
@@ -68758,36 +68758,36 @@
         </is>
       </c>
       <c r="B3417" t="n">
-        <v>3470</v>
+        <v>940549</v>
       </c>
       <c r="C3417" t="inlineStr">
         <is>
-          <t>DEBORA ALVES CARVALHO</t>
+          <t>EDILSON ARAUJO - FL9</t>
         </is>
       </c>
       <c r="D3417" t="inlineStr">
         <is>
-          <t>DEBORA.ALVES</t>
+          <t>EDILSON</t>
         </is>
       </c>
     </row>
     <row r="3418">
       <c r="A3418" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3418" t="n">
-        <v>3510</v>
+        <v>3470</v>
       </c>
       <c r="C3418" t="inlineStr">
         <is>
-          <t>CAMILA RODIGUES PINTO</t>
+          <t>DEBORA ALVES CARVALHO</t>
         </is>
       </c>
       <c r="D3418" t="inlineStr">
         <is>
-          <t>MILA.PINTO</t>
+          <t>DEBORA.ALVES</t>
         </is>
       </c>
     </row>
@@ -68798,96 +68798,96 @@
         </is>
       </c>
       <c r="B3419" t="n">
-        <v>3511</v>
+        <v>3510</v>
       </c>
       <c r="C3419" t="inlineStr">
         <is>
-          <t>JORGE HENRIQUE DOS SANTOS RODRIGUES</t>
+          <t>CAMILA RODIGUES PINTO</t>
         </is>
       </c>
       <c r="D3419" t="inlineStr">
         <is>
-          <t>J.HENRIQUE</t>
+          <t>MILA.PINTO</t>
         </is>
       </c>
     </row>
     <row r="3420">
       <c r="A3420" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3420" t="n">
-        <v>3561</v>
+        <v>3511</v>
       </c>
       <c r="C3420" t="inlineStr">
         <is>
-          <t>RONARIA PATRICIA VILARINDO DE ALMEIDA</t>
+          <t>JORGE HENRIQUE DOS SANTOS RODRIGUES</t>
         </is>
       </c>
       <c r="D3420" t="inlineStr">
         <is>
-          <t>RPATRICIA</t>
+          <t>J.HENRIQUE</t>
         </is>
       </c>
     </row>
     <row r="3421">
       <c r="A3421" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3421" t="n">
-        <v>3562</v>
+        <v>3561</v>
       </c>
       <c r="C3421" t="inlineStr">
         <is>
-          <t>LETICIA MARIA BENTO NOGUEIRA</t>
+          <t>RONARIA PATRICIA VILARINDO DE ALMEIDA</t>
         </is>
       </c>
       <c r="D3421" t="inlineStr">
         <is>
-          <t>LBENTO</t>
+          <t>RPATRICIA</t>
         </is>
       </c>
     </row>
     <row r="3422">
       <c r="A3422" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3422" t="n">
-        <v>3270</v>
+        <v>3562</v>
       </c>
       <c r="C3422" t="inlineStr">
         <is>
-          <t>ITANA NASCIMENTO SIMOES</t>
+          <t>LETICIA MARIA BENTO NOGUEIRA</t>
         </is>
       </c>
       <c r="D3422" t="inlineStr">
         <is>
-          <t>ISIMOES</t>
+          <t>LBENTO</t>
         </is>
       </c>
     </row>
     <row r="3423">
       <c r="A3423" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3423" t="n">
-        <v>3318</v>
+        <v>3270</v>
       </c>
       <c r="C3423" t="inlineStr">
         <is>
-          <t>LUAN MONTEIRO COSTA</t>
+          <t>ITANA NASCIMENTO SIMOES</t>
         </is>
       </c>
       <c r="D3423" t="inlineStr">
         <is>
-          <t>LMONTEIRO</t>
+          <t>ISIMOES</t>
         </is>
       </c>
     </row>
@@ -68898,36 +68898,36 @@
         </is>
       </c>
       <c r="B3424" t="n">
-        <v>3319</v>
+        <v>3318</v>
       </c>
       <c r="C3424" t="inlineStr">
         <is>
-          <t>MARIANA MACEDA DOS SANTOS</t>
+          <t>LUAN MONTEIRO COSTA</t>
         </is>
       </c>
       <c r="D3424" t="inlineStr">
         <is>
-          <t>MMACEDA</t>
+          <t>LMONTEIRO</t>
         </is>
       </c>
     </row>
     <row r="3425">
       <c r="A3425" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3425" t="n">
-        <v>3389</v>
+        <v>3319</v>
       </c>
       <c r="C3425" t="inlineStr">
         <is>
-          <t>TAMILES DE SANTANA AMORIM BISPO</t>
+          <t>MARIANA MACEDA DOS SANTOS</t>
         </is>
       </c>
       <c r="D3425" t="inlineStr">
         <is>
-          <t>TAMILES</t>
+          <t>MMACEDA</t>
         </is>
       </c>
     </row>
@@ -68938,76 +68938,76 @@
         </is>
       </c>
       <c r="B3426" t="n">
-        <v>3390</v>
+        <v>3389</v>
       </c>
       <c r="C3426" t="inlineStr">
         <is>
-          <t>IRACEMA DE ALMEIDA MOURA</t>
+          <t>TAMILES DE SANTANA AMORIM BISPO</t>
         </is>
       </c>
       <c r="D3426" t="inlineStr">
         <is>
-          <t>IRACEMA</t>
+          <t>TAMILES</t>
         </is>
       </c>
     </row>
     <row r="3427">
       <c r="A3427" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3427" t="n">
-        <v>3575</v>
+        <v>3390</v>
       </c>
       <c r="C3427" t="inlineStr">
         <is>
-          <t>SAMARA ALVES DA SILVA</t>
+          <t>IRACEMA DE ALMEIDA MOURA</t>
         </is>
       </c>
       <c r="D3427" t="inlineStr">
         <is>
-          <t>S.ALVES</t>
+          <t>IRACEMA</t>
         </is>
       </c>
     </row>
     <row r="3428">
       <c r="A3428" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3428" t="n">
-        <v>3583</v>
+        <v>3575</v>
       </c>
       <c r="C3428" t="inlineStr">
         <is>
-          <t>TALLIS GUTTEMBERG GUIMARES BATISTA</t>
+          <t>SAMARA ALVES DA SILVA</t>
         </is>
       </c>
       <c r="D3428" t="inlineStr">
         <is>
-          <t>TALLIS16</t>
+          <t>S.ALVES</t>
         </is>
       </c>
     </row>
     <row r="3429">
       <c r="A3429" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3429" t="n">
-        <v>3286</v>
+        <v>3583</v>
       </c>
       <c r="C3429" t="inlineStr">
         <is>
-          <t>VALERIA MAIA DA SILVA</t>
+          <t>TALLIS GUTTEMBERG GUIMARES BATISTA</t>
         </is>
       </c>
       <c r="D3429" t="inlineStr">
         <is>
-          <t>VMAIAS</t>
+          <t>TALLIS16</t>
         </is>
       </c>
     </row>
@@ -69018,156 +69018,156 @@
         </is>
       </c>
       <c r="B3430" t="n">
-        <v>3287</v>
+        <v>3286</v>
       </c>
       <c r="C3430" t="inlineStr">
         <is>
-          <t>ERIVELTON DA SILVA OLIVEIRA</t>
+          <t>VALERIA MAIA DA SILVA</t>
         </is>
       </c>
       <c r="D3430" t="inlineStr">
         <is>
-          <t>ESOLIVEIRA</t>
+          <t>VMAIAS</t>
         </is>
       </c>
     </row>
     <row r="3431">
       <c r="A3431" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3431" t="n">
-        <v>3307</v>
+        <v>3287</v>
       </c>
       <c r="C3431" t="inlineStr">
         <is>
-          <t>ADRIEL XERES BARROS MARTINS</t>
+          <t>ERIVELTON DA SILVA OLIVEIRA</t>
         </is>
       </c>
       <c r="D3431" t="inlineStr">
         <is>
-          <t>AXERES</t>
+          <t>ESOLIVEIRA</t>
         </is>
       </c>
     </row>
     <row r="3432">
       <c r="A3432" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3432" t="n">
-        <v>3308</v>
+        <v>3307</v>
       </c>
       <c r="C3432" t="inlineStr">
         <is>
-          <t>ELKZIEL JUVINO DA SILVA</t>
+          <t>ADRIEL XERES BARROS MARTINS</t>
         </is>
       </c>
       <c r="D3432" t="inlineStr">
         <is>
-          <t>EJUVINO</t>
+          <t>AXERES</t>
         </is>
       </c>
     </row>
     <row r="3433">
       <c r="A3433" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3433" t="n">
-        <v>940539</v>
+        <v>3308</v>
       </c>
       <c r="C3433" t="inlineStr">
         <is>
-          <t>EDSON ARAUJO - FL9</t>
+          <t>ELKZIEL JUVINO DA SILVA</t>
         </is>
       </c>
       <c r="D3433" t="inlineStr">
         <is>
-          <t>EDS</t>
+          <t>EJUVINO</t>
         </is>
       </c>
     </row>
     <row r="3434">
       <c r="A3434" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3434" t="n">
-        <v>940540</v>
+        <v>940539</v>
       </c>
       <c r="C3434" t="inlineStr">
         <is>
-          <t>EDSON ARAUJO - FL8</t>
+          <t>EDSON ARAUJO - FL9</t>
         </is>
       </c>
       <c r="D3434" t="inlineStr">
         <is>
-          <t>EDS8</t>
+          <t>EDS</t>
         </is>
       </c>
     </row>
     <row r="3435">
       <c r="A3435" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B3435" t="n">
-        <v>3328</v>
+        <v>940540</v>
       </c>
       <c r="C3435" t="inlineStr">
         <is>
-          <t>ALAN ARAUJO DA SILVA</t>
+          <t>EDSON ARAUJO - FL8</t>
         </is>
       </c>
       <c r="D3435" t="inlineStr">
         <is>
-          <t>ARSILVA</t>
+          <t>EDS8</t>
         </is>
       </c>
     </row>
     <row r="3436">
       <c r="A3436" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3436" t="n">
-        <v>3350</v>
+        <v>3328</v>
       </c>
       <c r="C3436" t="inlineStr">
         <is>
-          <t xml:space="preserve">EDER RODRIGUES DA SILVA </t>
+          <t>ALAN ARAUJO DA SILVA</t>
         </is>
       </c>
       <c r="D3436" t="inlineStr">
         <is>
-          <t>EDERS</t>
+          <t>ARSILVA</t>
         </is>
       </c>
     </row>
     <row r="3437">
       <c r="A3437" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3437" t="n">
-        <v>3373</v>
+        <v>3350</v>
       </c>
       <c r="C3437" t="inlineStr">
         <is>
-          <t xml:space="preserve">NATANAEL TAVARES DE SOUSA </t>
+          <t xml:space="preserve">EDER RODRIGUES DA SILVA </t>
         </is>
       </c>
       <c r="D3437" t="inlineStr">
         <is>
-          <t>NTSOUSA</t>
+          <t>EDERS</t>
         </is>
       </c>
     </row>
@@ -69178,156 +69178,156 @@
         </is>
       </c>
       <c r="B3438" t="n">
-        <v>3374</v>
+        <v>3373</v>
       </c>
       <c r="C3438" t="inlineStr">
         <is>
-          <t>REINALDO DA SILVA COSTA</t>
+          <t xml:space="preserve">NATANAEL TAVARES DE SOUSA </t>
         </is>
       </c>
       <c r="D3438" t="inlineStr">
         <is>
-          <t>RSCOSTA</t>
+          <t>NTSOUSA</t>
         </is>
       </c>
     </row>
     <row r="3439">
       <c r="A3439" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3439" t="n">
-        <v>3399</v>
+        <v>3374</v>
       </c>
       <c r="C3439" t="inlineStr">
         <is>
-          <t xml:space="preserve">RICARDO BARBOSA DOS SANTOS </t>
+          <t>REINALDO DA SILVA COSTA</t>
         </is>
       </c>
       <c r="D3439" t="inlineStr">
         <is>
-          <t>RICARDOSAN</t>
+          <t>RSCOSTA</t>
         </is>
       </c>
     </row>
     <row r="3440">
       <c r="A3440" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3440" t="n">
-        <v>3427</v>
+        <v>3399</v>
       </c>
       <c r="C3440" t="inlineStr">
         <is>
-          <t>ROQUE COMERCIO TEMPORARIO</t>
+          <t xml:space="preserve">RICARDO BARBOSA DOS SANTOS </t>
         </is>
       </c>
       <c r="D3440" t="inlineStr">
         <is>
-          <t>ROQUECOM</t>
+          <t>RICARDOSAN</t>
         </is>
       </c>
     </row>
     <row r="3441">
       <c r="A3441" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3441" t="n">
-        <v>3428</v>
+        <v>3427</v>
       </c>
       <c r="C3441" t="inlineStr">
         <is>
-          <t>ROQUE PLUS TEMPORARIO</t>
+          <t>ROQUE COMERCIO TEMPORARIO</t>
         </is>
       </c>
       <c r="D3441" t="inlineStr">
         <is>
-          <t>ROQUEPLUS</t>
+          <t>ROQUECOM</t>
         </is>
       </c>
     </row>
     <row r="3442">
       <c r="A3442" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3442" t="n">
-        <v>3432</v>
+        <v>3428</v>
       </c>
       <c r="C3442" t="inlineStr">
         <is>
-          <t>PATRICIA DOS SANTOS NONATO OLIVEIRA</t>
+          <t>ROQUE PLUS TEMPORARIO</t>
         </is>
       </c>
       <c r="D3442" t="inlineStr">
         <is>
-          <t>PATRICIAD</t>
+          <t>ROQUEPLUS</t>
         </is>
       </c>
     </row>
     <row r="3443">
       <c r="A3443" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3443" t="n">
-        <v>3448</v>
+        <v>3432</v>
       </c>
       <c r="C3443" t="inlineStr">
         <is>
-          <t xml:space="preserve">GABRIEL SOUZA CARVALHO </t>
+          <t>PATRICIA DOS SANTOS NONATO OLIVEIRA</t>
         </is>
       </c>
       <c r="D3443" t="inlineStr">
         <is>
-          <t>GABRIEL20</t>
+          <t>PATRICIAD</t>
         </is>
       </c>
     </row>
     <row r="3444">
       <c r="A3444" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3444" t="n">
-        <v>3465</v>
+        <v>3448</v>
       </c>
       <c r="C3444" t="inlineStr">
         <is>
-          <t>LUIZA MARIA BARRETO BARBOSA</t>
+          <t xml:space="preserve">GABRIEL SOUZA CARVALHO </t>
         </is>
       </c>
       <c r="D3444" t="inlineStr">
         <is>
-          <t>LUIZA.MARIA</t>
+          <t>GABRIEL20</t>
         </is>
       </c>
     </row>
     <row r="3445">
       <c r="A3445" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3445" t="n">
-        <v>3468</v>
+        <v>3465</v>
       </c>
       <c r="C3445" t="inlineStr">
         <is>
-          <t>KAWA ALMEIDA CAMPOS</t>
+          <t>LUIZA MARIA BARRETO BARBOSA</t>
         </is>
       </c>
       <c r="D3445" t="inlineStr">
         <is>
-          <t>KAWA</t>
+          <t>LUIZA.MARIA</t>
         </is>
       </c>
     </row>
@@ -69338,16 +69338,16 @@
         </is>
       </c>
       <c r="B3446" t="n">
-        <v>3476</v>
+        <v>3468</v>
       </c>
       <c r="C3446" t="inlineStr">
         <is>
-          <t xml:space="preserve"> FRANCISCA LEIDIANE M. MENDES NASCIMENTO</t>
+          <t>KAWA ALMEIDA CAMPOS</t>
         </is>
       </c>
       <c r="D3446" t="inlineStr">
         <is>
-          <t>FLEIDIANE</t>
+          <t>KAWA</t>
         </is>
       </c>
     </row>
@@ -69358,76 +69358,76 @@
         </is>
       </c>
       <c r="B3447" t="n">
-        <v>3477</v>
+        <v>3476</v>
       </c>
       <c r="C3447" t="inlineStr">
         <is>
-          <t>MARIA THAIS MARTINS PEREIRA SILVA</t>
+          <t xml:space="preserve"> FRANCISCA LEIDIANE M. MENDES NASCIMENTO</t>
         </is>
       </c>
       <c r="D3447" t="inlineStr">
         <is>
-          <t>MTHAIS</t>
+          <t>FLEIDIANE</t>
         </is>
       </c>
     </row>
     <row r="3448">
       <c r="A3448" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3448" t="n">
-        <v>3271</v>
+        <v>3477</v>
       </c>
       <c r="C3448" t="inlineStr">
         <is>
-          <t>DIEGO DE ARAUJO CALÁBRIA</t>
+          <t>MARIA THAIS MARTINS PEREIRA SILVA</t>
         </is>
       </c>
       <c r="D3448" t="inlineStr">
         <is>
-          <t>ARAUJOC</t>
+          <t>MTHAIS</t>
         </is>
       </c>
     </row>
     <row r="3449">
       <c r="A3449" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3449" t="n">
-        <v>3272</v>
+        <v>3271</v>
       </c>
       <c r="C3449" t="inlineStr">
         <is>
-          <t>ANNE BEATRIZ SILVA VIRGINO</t>
+          <t>DIEGO DE ARAUJO CALÁBRIA</t>
         </is>
       </c>
       <c r="D3449" t="inlineStr">
         <is>
-          <t>ABVIRGINIO</t>
+          <t>ARAUJOC</t>
         </is>
       </c>
     </row>
     <row r="3450">
       <c r="A3450" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3450" t="n">
-        <v>3293</v>
+        <v>3272</v>
       </c>
       <c r="C3450" t="inlineStr">
         <is>
-          <t xml:space="preserve">CARLOS ALBERTO VIRIATO SANTOS </t>
+          <t>ANNE BEATRIZ SILVA VIRGINO</t>
         </is>
       </c>
       <c r="D3450" t="inlineStr">
         <is>
-          <t>CVIRIATO</t>
+          <t>ABVIRGINIO</t>
         </is>
       </c>
     </row>
@@ -69438,16 +69438,16 @@
         </is>
       </c>
       <c r="B3451" t="n">
-        <v>3381</v>
+        <v>3293</v>
       </c>
       <c r="C3451" t="inlineStr">
         <is>
-          <t>ALAN CAIQUE SANTOS E SANTOS</t>
+          <t xml:space="preserve">CARLOS ALBERTO VIRIATO SANTOS </t>
         </is>
       </c>
       <c r="D3451" t="inlineStr">
         <is>
-          <t>ALANSANTOS</t>
+          <t>CVIRIATO</t>
         </is>
       </c>
     </row>
@@ -69458,116 +69458,116 @@
         </is>
       </c>
       <c r="B3452" t="n">
-        <v>3443</v>
+        <v>3381</v>
       </c>
       <c r="C3452" t="inlineStr">
         <is>
-          <t>SANON MOREIRA SOUZA</t>
+          <t>ALAN CAIQUE SANTOS E SANTOS</t>
         </is>
       </c>
       <c r="D3452" t="inlineStr">
         <is>
-          <t>SANON</t>
+          <t>ALANSANTOS</t>
         </is>
       </c>
     </row>
     <row r="3453">
       <c r="A3453" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3453" t="n">
-        <v>3516</v>
+        <v>3443</v>
       </c>
       <c r="C3453" t="inlineStr">
         <is>
-          <t>FRANCISCO RILDER TELES DE OLIVEIRA</t>
+          <t>SANON MOREIRA SOUZA</t>
         </is>
       </c>
       <c r="D3453" t="inlineStr">
         <is>
-          <t>RILDER</t>
+          <t>SANON</t>
         </is>
       </c>
     </row>
     <row r="3454">
       <c r="A3454" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3454" t="n">
-        <v>3519</v>
+        <v>3516</v>
       </c>
       <c r="C3454" t="inlineStr">
         <is>
-          <t>MARIA LUANA DE ALMEIDA BATISTA</t>
+          <t>FRANCISCO RILDER TELES DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D3454" t="inlineStr">
         <is>
-          <t>M.LUANA</t>
+          <t>RILDER</t>
         </is>
       </c>
     </row>
     <row r="3455">
       <c r="A3455" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3455" t="n">
-        <v>3540</v>
+        <v>3519</v>
       </c>
       <c r="C3455" t="inlineStr">
         <is>
-          <t>HELEN VITORIA OLIVEIRA DA ROCHA</t>
+          <t>MARIA LUANA DE ALMEIDA BATISTA</t>
         </is>
       </c>
       <c r="D3455" t="inlineStr">
         <is>
-          <t>H.VITORIA</t>
+          <t>M.LUANA</t>
         </is>
       </c>
     </row>
     <row r="3456">
       <c r="A3456" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B3456" t="n">
-        <v>3559</v>
+        <v>3540</v>
       </c>
       <c r="C3456" t="inlineStr">
         <is>
-          <t>ARKBERYS TELES DE SOUSA</t>
+          <t>HELEN VITORIA OLIVEIRA DA ROCHA</t>
         </is>
       </c>
       <c r="D3456" t="inlineStr">
         <is>
-          <t>ARKBERYS</t>
+          <t>H.VITORIA</t>
         </is>
       </c>
     </row>
     <row r="3457">
       <c r="A3457" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3457" t="n">
-        <v>3567</v>
+        <v>3559</v>
       </c>
       <c r="C3457" t="inlineStr">
         <is>
-          <t>PEDRO HENRIQUE VIEIRA DE LIMA</t>
+          <t>ARKBERYS TELES DE SOUSA</t>
         </is>
       </c>
       <c r="D3457" t="inlineStr">
         <is>
-          <t>P.LIMA</t>
+          <t>ARKBERYS</t>
         </is>
       </c>
     </row>
@@ -69578,76 +69578,76 @@
         </is>
       </c>
       <c r="B3458" t="n">
-        <v>3331</v>
+        <v>3567</v>
       </c>
       <c r="C3458" t="inlineStr">
         <is>
-          <t>LOUIZE VANIELLE RODRIGUES FARIAS</t>
+          <t>PEDRO HENRIQUE VIEIRA DE LIMA</t>
         </is>
       </c>
       <c r="D3458" t="inlineStr">
         <is>
-          <t>LVFARIAS</t>
+          <t>P.LIMA</t>
         </is>
       </c>
     </row>
     <row r="3459">
       <c r="A3459" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3459" t="n">
-        <v>3334</v>
+        <v>3331</v>
       </c>
       <c r="C3459" t="inlineStr">
         <is>
-          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+          <t>LOUIZE VANIELLE RODRIGUES FARIAS</t>
         </is>
       </c>
       <c r="D3459" t="inlineStr">
         <is>
-          <t>MTGASPAR</t>
+          <t>LVFARIAS</t>
         </is>
       </c>
     </row>
     <row r="3460">
       <c r="A3460" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3460" t="n">
-        <v>3345</v>
+        <v>3334</v>
       </c>
       <c r="C3460" t="inlineStr">
         <is>
-          <t>AURICÉLIA INACIO PEREIRA</t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
       <c r="D3460" t="inlineStr">
         <is>
-          <t>AIPEREIRA</t>
+          <t>MTGASPAR</t>
         </is>
       </c>
     </row>
     <row r="3461">
       <c r="A3461" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3461" t="n">
-        <v>3363</v>
+        <v>3345</v>
       </c>
       <c r="C3461" t="inlineStr">
         <is>
-          <t>IASMIN LEAL ALVES</t>
+          <t>AURICÉLIA INACIO PEREIRA</t>
         </is>
       </c>
       <c r="D3461" t="inlineStr">
         <is>
-          <t>ILALVES</t>
+          <t>AIPEREIRA</t>
         </is>
       </c>
     </row>
@@ -69658,196 +69658,196 @@
         </is>
       </c>
       <c r="B3462" t="n">
-        <v>3370</v>
+        <v>3363</v>
       </c>
       <c r="C3462" t="inlineStr">
         <is>
-          <t>CARLOS DIEGO ARAUJO ALMEIDA</t>
+          <t>IASMIN LEAL ALVES</t>
         </is>
       </c>
       <c r="D3462" t="inlineStr">
         <is>
-          <t>CDIEGO</t>
+          <t>ILALVES</t>
         </is>
       </c>
     </row>
     <row r="3463">
       <c r="A3463" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3463" t="n">
-        <v>3379</v>
+        <v>3370</v>
       </c>
       <c r="C3463" t="inlineStr">
         <is>
-          <t xml:space="preserve">MATHEUS EVANGELISTA FERREIRA </t>
+          <t>CARLOS DIEGO ARAUJO ALMEIDA</t>
         </is>
       </c>
       <c r="D3463" t="inlineStr">
         <is>
-          <t>MMFERREIRA</t>
+          <t>CDIEGO</t>
         </is>
       </c>
     </row>
     <row r="3464">
       <c r="A3464" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3464" t="n">
-        <v>3419</v>
+        <v>3379</v>
       </c>
       <c r="C3464" t="inlineStr">
         <is>
-          <t xml:space="preserve">DAVID EVANGELISTA SILVA </t>
+          <t xml:space="preserve">MATHEUS EVANGELISTA FERREIRA </t>
         </is>
       </c>
       <c r="D3464" t="inlineStr">
         <is>
-          <t>DAVID</t>
+          <t>MMFERREIRA</t>
         </is>
       </c>
     </row>
     <row r="3465">
       <c r="A3465" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3465" t="n">
-        <v>3423</v>
+        <v>3419</v>
       </c>
       <c r="C3465" t="inlineStr">
         <is>
-          <t>MARCIO JOSE TIAGO</t>
+          <t xml:space="preserve">DAVID EVANGELISTA SILVA </t>
         </is>
       </c>
       <c r="D3465" t="inlineStr">
         <is>
-          <t>MJTIAGO</t>
+          <t>DAVID</t>
         </is>
       </c>
     </row>
     <row r="3466">
       <c r="A3466" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3466" t="n">
-        <v>3453</v>
+        <v>3423</v>
       </c>
       <c r="C3466" t="inlineStr">
         <is>
-          <t xml:space="preserve">LAURIENE SILVA BARBOSA </t>
+          <t>MARCIO JOSE TIAGO</t>
         </is>
       </c>
       <c r="D3466" t="inlineStr">
         <is>
-          <t>LAURIENE</t>
+          <t>MJTIAGO</t>
         </is>
       </c>
     </row>
     <row r="3467">
       <c r="A3467" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3467" t="n">
-        <v>3478</v>
+        <v>3453</v>
       </c>
       <c r="C3467" t="inlineStr">
         <is>
-          <t>LEANDRO BRITO NOGUEIRA DE OLIVEIRA</t>
+          <t xml:space="preserve">LAURIENE SILVA BARBOSA </t>
         </is>
       </c>
       <c r="D3467" t="inlineStr">
         <is>
-          <t>LBNOGUEIRA</t>
+          <t>LAURIENE</t>
         </is>
       </c>
     </row>
     <row r="3468">
       <c r="A3468" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3468" t="n">
-        <v>3479</v>
+        <v>3478</v>
       </c>
       <c r="C3468" t="inlineStr">
         <is>
-          <t>ESDRAS ALESSANDRO SANTOS SANTANA</t>
+          <t>LEANDRO BRITO NOGUEIRA DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D3468" t="inlineStr">
         <is>
-          <t>EALESSANDRO</t>
+          <t>LBNOGUEIRA</t>
         </is>
       </c>
     </row>
     <row r="3469">
       <c r="A3469" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3469" t="n">
-        <v>3480</v>
+        <v>3479</v>
       </c>
       <c r="C3469" t="inlineStr">
         <is>
-          <t xml:space="preserve">LUCIMARA SOUSA LIMA </t>
+          <t>ESDRAS ALESSANDRO SANTOS SANTANA</t>
         </is>
       </c>
       <c r="D3469" t="inlineStr">
         <is>
-          <t>LUCIMARA</t>
+          <t>EALESSANDRO</t>
         </is>
       </c>
     </row>
     <row r="3470">
       <c r="A3470" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3470" t="n">
-        <v>3482</v>
+        <v>3480</v>
       </c>
       <c r="C3470" t="inlineStr">
         <is>
-          <t>DANIEL FERNANDES DINIZ HERACLIO</t>
+          <t xml:space="preserve">LUCIMARA SOUSA LIMA </t>
         </is>
       </c>
       <c r="D3470" t="inlineStr">
         <is>
-          <t>DFDINIZ</t>
+          <t>LUCIMARA</t>
         </is>
       </c>
     </row>
     <row r="3471">
       <c r="A3471" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3471" t="n">
-        <v>3518</v>
+        <v>3482</v>
       </c>
       <c r="C3471" t="inlineStr">
         <is>
-          <t>RAMYRA ALVES FELIX DA SILVA</t>
+          <t>DANIEL FERNANDES DINIZ HERACLIO</t>
         </is>
       </c>
       <c r="D3471" t="inlineStr">
         <is>
-          <t>RFELIX</t>
+          <t>DFDINIZ</t>
         </is>
       </c>
     </row>
@@ -69858,36 +69858,36 @@
         </is>
       </c>
       <c r="B3472" t="n">
-        <v>3534</v>
+        <v>3518</v>
       </c>
       <c r="C3472" t="inlineStr">
         <is>
-          <t xml:space="preserve">CAIO DE SOUZA VINHAS </t>
+          <t>RAMYRA ALVES FELIX DA SILVA</t>
         </is>
       </c>
       <c r="D3472" t="inlineStr">
         <is>
-          <t>CVINHAS</t>
+          <t>RFELIX</t>
         </is>
       </c>
     </row>
     <row r="3473">
       <c r="A3473" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3473" t="n">
-        <v>3535</v>
+        <v>3534</v>
       </c>
       <c r="C3473" t="inlineStr">
         <is>
-          <t>ROMARIO DE SOUSA SILVA</t>
+          <t xml:space="preserve">CAIO DE SOUZA VINHAS </t>
         </is>
       </c>
       <c r="D3473" t="inlineStr">
         <is>
-          <t>RSOUSAS</t>
+          <t>CVINHAS</t>
         </is>
       </c>
     </row>
@@ -69898,56 +69898,56 @@
         </is>
       </c>
       <c r="B3474" t="n">
-        <v>3536</v>
+        <v>3535</v>
       </c>
       <c r="C3474" t="inlineStr">
         <is>
-          <t>JHONATAS CARVALHO OLIVEIRA</t>
+          <t>ROMARIO DE SOUSA SILVA</t>
         </is>
       </c>
       <c r="D3474" t="inlineStr">
         <is>
-          <t>JHONATASC</t>
+          <t>RSOUSAS</t>
         </is>
       </c>
     </row>
     <row r="3475">
       <c r="A3475" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3475" t="n">
-        <v>940529</v>
+        <v>3536</v>
       </c>
       <c r="C3475" t="inlineStr">
         <is>
-          <t>EDGAR FELIX - FL9</t>
+          <t>JHONATAS CARVALHO OLIVEIRA</t>
         </is>
       </c>
       <c r="D3475" t="inlineStr">
         <is>
-          <t>EDGAR F</t>
+          <t>JHONATASC</t>
         </is>
       </c>
     </row>
     <row r="3476">
       <c r="A3476" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3476" t="n">
-        <v>3304</v>
+        <v>940529</v>
       </c>
       <c r="C3476" t="inlineStr">
         <is>
-          <t>JOACI GUILHERME GONÇALVES DA LUZ</t>
+          <t>EDGAR FELIX - FL9</t>
         </is>
       </c>
       <c r="D3476" t="inlineStr">
         <is>
-          <t>JLUZ</t>
+          <t>EDGAR F</t>
         </is>
       </c>
     </row>
@@ -69958,16 +69958,16 @@
         </is>
       </c>
       <c r="B3477" t="n">
-        <v>3305</v>
+        <v>3304</v>
       </c>
       <c r="C3477" t="inlineStr">
         <is>
-          <t>JOÃO VITOR DE ARAÚJO GONÇALVES</t>
+          <t>JOACI GUILHERME GONÇALVES DA LUZ</t>
         </is>
       </c>
       <c r="D3477" t="inlineStr">
         <is>
-          <t>JJVITOR</t>
+          <t>JLUZ</t>
         </is>
       </c>
     </row>
@@ -69978,36 +69978,36 @@
         </is>
       </c>
       <c r="B3478" t="n">
-        <v>3306</v>
+        <v>3305</v>
       </c>
       <c r="C3478" t="inlineStr">
         <is>
-          <t>WENDERSON MARCOS DOS SANTOS</t>
+          <t>JOÃO VITOR DE ARAÚJO GONÇALVES</t>
         </is>
       </c>
       <c r="D3478" t="inlineStr">
         <is>
-          <t>WWMARCOS</t>
+          <t>JJVITOR</t>
         </is>
       </c>
     </row>
     <row r="3479">
       <c r="A3479" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3479" t="n">
-        <v>3335</v>
+        <v>3306</v>
       </c>
       <c r="C3479" t="inlineStr">
         <is>
-          <t>EDILBERTO LEMOS DE LIMA</t>
+          <t>WENDERSON MARCOS DOS SANTOS</t>
         </is>
       </c>
       <c r="D3479" t="inlineStr">
         <is>
-          <t>ELEMOS</t>
+          <t>WWMARCOS</t>
         </is>
       </c>
     </row>
@@ -70018,136 +70018,136 @@
         </is>
       </c>
       <c r="B3480" t="n">
-        <v>3336</v>
+        <v>3335</v>
       </c>
       <c r="C3480" t="inlineStr">
         <is>
-          <t>EZEQUIEL SOUZA DO NASCIMENTO</t>
+          <t>EDILBERTO LEMOS DE LIMA</t>
         </is>
       </c>
       <c r="D3480" t="inlineStr">
         <is>
-          <t>ESNASCIMENTO</t>
+          <t>ELEMOS</t>
         </is>
       </c>
     </row>
     <row r="3481">
       <c r="A3481" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3481" t="n">
-        <v>3341</v>
+        <v>3336</v>
       </c>
       <c r="C3481" t="inlineStr">
         <is>
-          <t>ALCIONE MARIANO DE OLIVEIRA</t>
+          <t>EZEQUIEL SOUZA DO NASCIMENTO</t>
         </is>
       </c>
       <c r="D3481" t="inlineStr">
         <is>
-          <t>AMOLIVEIRA</t>
+          <t>ESNASCIMENTO</t>
         </is>
       </c>
     </row>
     <row r="3482">
       <c r="A3482" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3482" t="n">
-        <v>3401</v>
+        <v>3341</v>
       </c>
       <c r="C3482" t="inlineStr">
         <is>
-          <t xml:space="preserve">TULIO HENRIQUE DA SILVA CARVALHO </t>
+          <t>ALCIONE MARIANO DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D3482" t="inlineStr">
         <is>
-          <t>TULIO</t>
+          <t>AMOLIVEIRA</t>
         </is>
       </c>
     </row>
     <row r="3483">
       <c r="A3483" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3483" t="n">
-        <v>3411</v>
+        <v>3401</v>
       </c>
       <c r="C3483" t="inlineStr">
         <is>
-          <t>CONEXAO RUBYA DANILLA</t>
+          <t xml:space="preserve">TULIO HENRIQUE DA SILVA CARVALHO </t>
         </is>
       </c>
       <c r="D3483" t="inlineStr">
         <is>
-          <t>CONEXAORUBYA</t>
+          <t>TULIO</t>
         </is>
       </c>
     </row>
     <row r="3484">
       <c r="A3484" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3484" t="n">
-        <v>3412</v>
+        <v>3411</v>
       </c>
       <c r="C3484" t="inlineStr">
         <is>
-          <t>CONEXAO RAFAEL</t>
+          <t>CONEXAO RUBYA DANILLA</t>
         </is>
       </c>
       <c r="D3484" t="inlineStr">
         <is>
-          <t>CONEXAORAFAEL</t>
+          <t>CONEXAORUBYA</t>
         </is>
       </c>
     </row>
     <row r="3485">
       <c r="A3485" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3485" t="n">
-        <v>3558</v>
+        <v>3412</v>
       </c>
       <c r="C3485" t="inlineStr">
         <is>
-          <t>WALLYS QUEIROZ VIANA</t>
+          <t>CONEXAO RAFAEL</t>
         </is>
       </c>
       <c r="D3485" t="inlineStr">
         <is>
-          <t>WALLYS</t>
+          <t>CONEXAORAFAEL</t>
         </is>
       </c>
     </row>
     <row r="3486">
       <c r="A3486" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3486" t="n">
-        <v>3264</v>
+        <v>3558</v>
       </c>
       <c r="C3486" t="inlineStr">
         <is>
-          <t xml:space="preserve">WILTON CARLOS MACIEL DE ASSIS </t>
+          <t>WALLYS QUEIROZ VIANA</t>
         </is>
       </c>
       <c r="D3486" t="inlineStr">
         <is>
-          <t>WCMACIEL</t>
+          <t>WALLYS</t>
         </is>
       </c>
     </row>
@@ -70158,56 +70158,56 @@
         </is>
       </c>
       <c r="B3487" t="n">
-        <v>3340</v>
+        <v>3264</v>
       </c>
       <c r="C3487" t="inlineStr">
         <is>
-          <t>ROGELENO FARIAS FEIJÃO FILHO</t>
+          <t xml:space="preserve">WILTON CARLOS MACIEL DE ASSIS </t>
         </is>
       </c>
       <c r="D3487" t="inlineStr">
         <is>
-          <t>RFEIJAO</t>
+          <t>WCMACIEL</t>
         </is>
       </c>
     </row>
     <row r="3488">
       <c r="A3488" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3488" t="n">
-        <v>940550</v>
+        <v>3340</v>
       </c>
       <c r="C3488" t="inlineStr">
         <is>
-          <t>RAFAELE RIBEIRO CARNEIRO</t>
+          <t>ROGELENO FARIAS FEIJÃO FILHO</t>
         </is>
       </c>
       <c r="D3488" t="inlineStr">
         <is>
-          <t>RAFAELE</t>
+          <t>RFEIJAO</t>
         </is>
       </c>
     </row>
     <row r="3489">
       <c r="A3489" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>99</t>
         </is>
       </c>
       <c r="B3489" t="n">
-        <v>3377</v>
+        <v>940550</v>
       </c>
       <c r="C3489" t="inlineStr">
         <is>
-          <t xml:space="preserve"> ISALTINO BISPO DE OLIVEIRA JUNIOR</t>
+          <t>RAFAELE RIBEIRO CARNEIRO</t>
         </is>
       </c>
       <c r="D3489" t="inlineStr">
         <is>
-          <t>BJUNIOR</t>
+          <t>RAFAELE</t>
         </is>
       </c>
     </row>
@@ -70218,56 +70218,56 @@
         </is>
       </c>
       <c r="B3490" t="n">
-        <v>3425</v>
+        <v>3377</v>
       </c>
       <c r="C3490" t="inlineStr">
         <is>
-          <t xml:space="preserve"> CIRLANE ARAUJO SOUZA </t>
+          <t xml:space="preserve"> ISALTINO BISPO DE OLIVEIRA JUNIOR</t>
         </is>
       </c>
       <c r="D3490" t="inlineStr">
         <is>
-          <t>CIRLANES</t>
+          <t>BJUNIOR</t>
         </is>
       </c>
     </row>
     <row r="3491">
       <c r="A3491" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3491" t="n">
-        <v>3454</v>
+        <v>3425</v>
       </c>
       <c r="C3491" t="inlineStr">
         <is>
-          <t>ANTONIA SAMARA DE SOUZA SOARES</t>
+          <t xml:space="preserve"> CIRLANE ARAUJO SOUZA </t>
         </is>
       </c>
       <c r="D3491" t="inlineStr">
         <is>
-          <t>ANTSAMARA</t>
+          <t>CIRLANES</t>
         </is>
       </c>
     </row>
     <row r="3492">
       <c r="A3492" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3492" t="n">
-        <v>3491</v>
+        <v>3454</v>
       </c>
       <c r="C3492" t="inlineStr">
         <is>
-          <t>PEDRO JOSE DO NASCIMENTO NETO</t>
+          <t>ANTONIA SAMARA DE SOUZA SOARES</t>
         </is>
       </c>
       <c r="D3492" t="inlineStr">
         <is>
-          <t>P.JOSE</t>
+          <t>ANTSAMARA</t>
         </is>
       </c>
     </row>
@@ -70278,36 +70278,36 @@
         </is>
       </c>
       <c r="B3493" t="n">
-        <v>3492</v>
+        <v>3491</v>
       </c>
       <c r="C3493" t="inlineStr">
         <is>
-          <t>PAULA CARLA CALDAS MOTA</t>
+          <t>PEDRO JOSE DO NASCIMENTO NETO</t>
         </is>
       </c>
       <c r="D3493" t="inlineStr">
         <is>
-          <t>P.CARLA</t>
+          <t>P.JOSE</t>
         </is>
       </c>
     </row>
     <row r="3494">
       <c r="A3494" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3494" t="n">
-        <v>3542</v>
+        <v>3492</v>
       </c>
       <c r="C3494" t="inlineStr">
         <is>
-          <t>ANTONIA MILENA SOUSA ANDRADE</t>
+          <t>PAULA CARLA CALDAS MOTA</t>
         </is>
       </c>
       <c r="D3494" t="inlineStr">
         <is>
-          <t>A.MILENA</t>
+          <t>P.CARLA</t>
         </is>
       </c>
     </row>
@@ -70318,56 +70318,56 @@
         </is>
       </c>
       <c r="B3495" t="n">
-        <v>3547</v>
+        <v>3542</v>
       </c>
       <c r="C3495" t="inlineStr">
         <is>
-          <t xml:space="preserve">DAVI PEREIRA DA SILVA </t>
+          <t>ANTONIA MILENA SOUSA ANDRADE</t>
         </is>
       </c>
       <c r="D3495" t="inlineStr">
         <is>
-          <t>DPSILVA</t>
+          <t>A.MILENA</t>
         </is>
       </c>
     </row>
     <row r="3496">
       <c r="A3496" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3496" t="n">
-        <v>3552</v>
+        <v>3547</v>
       </c>
       <c r="C3496" t="inlineStr">
         <is>
-          <t>PAULO SERGIO MENDES DE OLIVEIRA</t>
+          <t xml:space="preserve">DAVI PEREIRA DA SILVA </t>
         </is>
       </c>
       <c r="D3496" t="inlineStr">
         <is>
-          <t>PSMENDES</t>
+          <t>DPSILVA</t>
         </is>
       </c>
     </row>
     <row r="3497">
       <c r="A3497" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3497" t="n">
-        <v>3294</v>
+        <v>3552</v>
       </c>
       <c r="C3497" t="inlineStr">
         <is>
-          <t>GLEICIANE MIRANDA DE MORAIS</t>
+          <t>PAULO SERGIO MENDES DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D3497" t="inlineStr">
         <is>
-          <t>GMIRANDA</t>
+          <t>PSMENDES</t>
         </is>
       </c>
     </row>
@@ -70378,176 +70378,176 @@
         </is>
       </c>
       <c r="B3498" t="n">
-        <v>3295</v>
+        <v>3294</v>
       </c>
       <c r="C3498" t="inlineStr">
         <is>
-          <t>MARIA ESTEFANNY DA SILVA MOURA</t>
+          <t>GLEICIANE MIRANDA DE MORAIS</t>
         </is>
       </c>
       <c r="D3498" t="inlineStr">
         <is>
-          <t>MESTEFANNY</t>
+          <t>GMIRANDA</t>
         </is>
       </c>
     </row>
     <row r="3499">
       <c r="A3499" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3499" t="n">
-        <v>3296</v>
+        <v>3295</v>
       </c>
       <c r="C3499" t="inlineStr">
         <is>
-          <t>PEDRO IAGO FONSECA EVANGELISTA</t>
+          <t>MARIA ESTEFANNY DA SILVA MOURA</t>
         </is>
       </c>
       <c r="D3499" t="inlineStr">
         <is>
-          <t>PIFONSECA</t>
+          <t>MESTEFANNY</t>
         </is>
       </c>
     </row>
     <row r="3500">
       <c r="A3500" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3500" t="n">
-        <v>940544</v>
+        <v>3296</v>
       </c>
       <c r="C3500" t="inlineStr">
         <is>
-          <t>LUTY LOG TRANSPORTES - FL8</t>
+          <t>PEDRO IAGO FONSECA EVANGELISTA</t>
         </is>
       </c>
       <c r="D3500" t="inlineStr">
         <is>
-          <t>LUTY LOG</t>
+          <t>PIFONSECA</t>
         </is>
       </c>
     </row>
     <row r="3501">
       <c r="A3501" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B3501" t="n">
-        <v>3380</v>
+        <v>940544</v>
       </c>
       <c r="C3501" t="inlineStr">
         <is>
-          <t>FRANCISCO MATHEUS RABELO DA COSTA</t>
+          <t>LUTY LOG TRANSPORTES - FL8</t>
         </is>
       </c>
       <c r="D3501" t="inlineStr">
         <is>
-          <t>FMATHEUS</t>
+          <t>LUTY LOG</t>
         </is>
       </c>
     </row>
     <row r="3502">
       <c r="A3502" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3502" t="n">
-        <v>3410</v>
+        <v>3380</v>
       </c>
       <c r="C3502" t="inlineStr">
         <is>
-          <t xml:space="preserve"> BRENO ALLAN DE JESUS</t>
+          <t>FRANCISCO MATHEUS RABELO DA COSTA</t>
         </is>
       </c>
       <c r="D3502" t="inlineStr">
         <is>
-          <t>JESUS</t>
+          <t>FMATHEUS</t>
         </is>
       </c>
     </row>
     <row r="3503">
       <c r="A3503" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3503" t="n">
-        <v>3444</v>
+        <v>3410</v>
       </c>
       <c r="C3503" t="inlineStr">
         <is>
-          <t>THIAGO COSTA SILVA</t>
+          <t xml:space="preserve"> BRENO ALLAN DE JESUS</t>
         </is>
       </c>
       <c r="D3503" t="inlineStr">
         <is>
-          <t>THIAGOC</t>
+          <t>JESUS</t>
         </is>
       </c>
     </row>
     <row r="3504">
       <c r="A3504" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3504" t="n">
-        <v>3456</v>
+        <v>3444</v>
       </c>
       <c r="C3504" t="inlineStr">
         <is>
-          <t>FELIPE BOTH MAZUCHINI</t>
+          <t>THIAGO COSTA SILVA</t>
         </is>
       </c>
       <c r="D3504" t="inlineStr">
         <is>
-          <t>FELIPEB</t>
+          <t>THIAGOC</t>
         </is>
       </c>
     </row>
     <row r="3505">
       <c r="A3505" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3505" t="n">
-        <v>3457</v>
+        <v>3456</v>
       </c>
       <c r="C3505" t="inlineStr">
         <is>
-          <t>FRANKLIN VIEIRA GOMES</t>
+          <t>FELIPE BOTH MAZUCHINI</t>
         </is>
       </c>
       <c r="D3505" t="inlineStr">
         <is>
-          <t>VIEIRAF</t>
+          <t>FELIPEB</t>
         </is>
       </c>
     </row>
     <row r="3506">
       <c r="A3506" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3506" t="n">
-        <v>3507</v>
+        <v>3457</v>
       </c>
       <c r="C3506" t="inlineStr">
         <is>
-          <t>KARINE TEODORA ALVES DE OLIVEIRA</t>
+          <t>FRANKLIN VIEIRA GOMES</t>
         </is>
       </c>
       <c r="D3506" t="inlineStr">
         <is>
-          <t>KOLIVEIRA</t>
+          <t>VIEIRAF</t>
         </is>
       </c>
     </row>
@@ -70558,14 +70558,34 @@
         </is>
       </c>
       <c r="B3507" t="n">
+        <v>3507</v>
+      </c>
+      <c r="C3507" t="inlineStr">
+        <is>
+          <t>KARINE TEODORA ALVES DE OLIVEIRA</t>
+        </is>
+      </c>
+      <c r="D3507" t="inlineStr">
+        <is>
+          <t>KOLIVEIRA</t>
+        </is>
+      </c>
+    </row>
+    <row r="3508">
+      <c r="A3508" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B3508" t="n">
         <v>3520</v>
       </c>
-      <c r="C3507" t="inlineStr">
+      <c r="C3508" t="inlineStr">
         <is>
           <t xml:space="preserve"> EMERSON FILIPE MELO DE AGUIAR</t>
         </is>
       </c>
-      <c r="D3507" t="inlineStr">
+      <c r="D3508" t="inlineStr">
         <is>
           <t>E.FILIPE</t>
         </is>

</xml_diff>

<commit_message>
chore(data): batch update intraday televendas - 08:02:48
</commit_message>
<xml_diff>
--- a/data/dim_televendas.xlsx
+++ b/data/dim_televendas.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3508"/>
+  <dimension ref="A1:D3509"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -66994,60 +66994,60 @@
     <row r="3329">
       <c r="A3329" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3329" t="n">
-        <v>3288</v>
+        <v>3597</v>
       </c>
       <c r="C3329" t="inlineStr">
         <is>
-          <t>ANA MARIA AMORIM MENDONÇA</t>
+          <t>YURI CAUAN DE JESUS COUTINHO</t>
         </is>
       </c>
       <c r="D3329" t="inlineStr">
         <is>
-          <t>AMENDONCA</t>
+          <t>YURI</t>
         </is>
       </c>
     </row>
     <row r="3330">
       <c r="A3330" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3330" t="n">
-        <v>3312</v>
+        <v>3288</v>
       </c>
       <c r="C3330" t="inlineStr">
         <is>
-          <t>AURIANA LIMA DE MORAES</t>
+          <t>ANA MARIA AMORIM MENDONÇA</t>
         </is>
       </c>
       <c r="D3330" t="inlineStr">
         <is>
-          <t>ALM</t>
+          <t>AMENDONCA</t>
         </is>
       </c>
     </row>
     <row r="3331">
       <c r="A3331" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3331" t="n">
-        <v>940547</v>
+        <v>3312</v>
       </c>
       <c r="C3331" t="inlineStr">
         <is>
-          <t>JM EXPRESS - AGRESTE</t>
+          <t>AURIANA LIMA DE MORAES</t>
         </is>
       </c>
       <c r="D3331" t="inlineStr">
         <is>
-          <t>J M A</t>
+          <t>ALM</t>
         </is>
       </c>
     </row>
@@ -67058,76 +67058,76 @@
         </is>
       </c>
       <c r="B3332" t="n">
-        <v>940548</v>
+        <v>940547</v>
       </c>
       <c r="C3332" t="inlineStr">
         <is>
-          <t>JM EXPRESS - SERTAO</t>
+          <t>JM EXPRESS - AGRESTE</t>
         </is>
       </c>
       <c r="D3332" t="inlineStr">
         <is>
-          <t>J M S</t>
+          <t>J M A</t>
         </is>
       </c>
     </row>
     <row r="3333">
       <c r="A3333" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3333" t="n">
-        <v>940551</v>
+        <v>940548</v>
       </c>
       <c r="C3333" t="inlineStr">
         <is>
-          <t>LUCAS PONTES NOBRE</t>
+          <t>JM EXPRESS - SERTAO</t>
         </is>
       </c>
       <c r="D3333" t="inlineStr">
         <is>
-          <t>PONTES</t>
+          <t>J M S</t>
         </is>
       </c>
     </row>
     <row r="3334">
       <c r="A3334" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>99</t>
         </is>
       </c>
       <c r="B3334" t="n">
-        <v>3382</v>
+        <v>940551</v>
       </c>
       <c r="C3334" t="inlineStr">
         <is>
-          <t>MARIA CASSILANIA SOUSA DO NASCIMENTO</t>
+          <t>LUCAS PONTES NOBRE</t>
         </is>
       </c>
       <c r="D3334" t="inlineStr">
         <is>
-          <t>MCASSILANIA</t>
+          <t>PONTES</t>
         </is>
       </c>
     </row>
     <row r="3335">
       <c r="A3335" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3335" t="n">
-        <v>3474</v>
+        <v>3382</v>
       </c>
       <c r="C3335" t="inlineStr">
         <is>
-          <t>MARCOS VINICIUS GONCALVES MIRANDA</t>
+          <t>MARIA CASSILANIA SOUSA DO NASCIMENTO</t>
         </is>
       </c>
       <c r="D3335" t="inlineStr">
         <is>
-          <t>MARCOS.VINICIUS</t>
+          <t>MCASSILANIA</t>
         </is>
       </c>
     </row>
@@ -67138,176 +67138,176 @@
         </is>
       </c>
       <c r="B3336" t="n">
-        <v>3523</v>
+        <v>3474</v>
       </c>
       <c r="C3336" t="inlineStr">
         <is>
-          <t>ORLANDO RICARDO SANTOS ANDRADE</t>
+          <t>MARCOS VINICIUS GONCALVES MIRANDA</t>
         </is>
       </c>
       <c r="D3336" t="inlineStr">
         <is>
-          <t>ORLANDOR</t>
+          <t>MARCOS.VINICIUS</t>
         </is>
       </c>
     </row>
     <row r="3337">
       <c r="A3337" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3337" t="n">
-        <v>3566</v>
+        <v>3523</v>
       </c>
       <c r="C3337" t="inlineStr">
         <is>
-          <t xml:space="preserve">WESLEY HENRIQUE ALVES DOS SANTOS </t>
+          <t>ORLANDO RICARDO SANTOS ANDRADE</t>
         </is>
       </c>
       <c r="D3337" t="inlineStr">
         <is>
-          <t>W.ALVES</t>
+          <t>ORLANDOR</t>
         </is>
       </c>
     </row>
     <row r="3338">
       <c r="A3338" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3338" t="n">
-        <v>3573</v>
+        <v>3566</v>
       </c>
       <c r="C3338" t="inlineStr">
         <is>
-          <t>GABRIEL DA SILVA MENDES</t>
+          <t xml:space="preserve">WESLEY HENRIQUE ALVES DOS SANTOS </t>
         </is>
       </c>
       <c r="D3338" t="inlineStr">
         <is>
-          <t>GMENDES</t>
+          <t>W.ALVES</t>
         </is>
       </c>
     </row>
     <row r="3339">
       <c r="A3339" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3339" t="n">
-        <v>940541</v>
+        <v>3573</v>
       </c>
       <c r="C3339" t="inlineStr">
         <is>
-          <t>JOSE AMSTERDA TEIXEIRA DE MENEZES</t>
+          <t>GABRIEL DA SILVA MENDES</t>
         </is>
       </c>
       <c r="D3339" t="inlineStr">
         <is>
-          <t>AMSTERDA</t>
+          <t>GMENDES</t>
         </is>
       </c>
     </row>
     <row r="3340">
       <c r="A3340" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>99</t>
         </is>
       </c>
       <c r="B3340" t="n">
-        <v>940554</v>
+        <v>940541</v>
       </c>
       <c r="C3340" t="inlineStr">
         <is>
-          <t>ALEXANDRE ALVES DE FREITAS</t>
+          <t>JOSE AMSTERDA TEIXEIRA DE MENEZES</t>
         </is>
       </c>
       <c r="D3340" t="inlineStr">
         <is>
-          <t>ALEXANDRE</t>
+          <t>AMSTERDA</t>
         </is>
       </c>
     </row>
     <row r="3341">
       <c r="A3341" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3341" t="n">
-        <v>3402</v>
+        <v>940554</v>
       </c>
       <c r="C3341" t="inlineStr">
         <is>
-          <t xml:space="preserve">VINICIUS GUEDES DA SILVA </t>
+          <t>ALEXANDRE ALVES DE FREITAS</t>
         </is>
       </c>
       <c r="D3341" t="inlineStr">
         <is>
-          <t>GUEDES5</t>
+          <t>ALEXANDRE</t>
         </is>
       </c>
     </row>
     <row r="3342">
       <c r="A3342" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3342" t="n">
-        <v>3467</v>
+        <v>3402</v>
       </c>
       <c r="C3342" t="inlineStr">
         <is>
-          <t>CILENE FERREIRA DA SILVA</t>
+          <t xml:space="preserve">VINICIUS GUEDES DA SILVA </t>
         </is>
       </c>
       <c r="D3342" t="inlineStr">
         <is>
-          <t>CILENE</t>
+          <t>GUEDES5</t>
         </is>
       </c>
     </row>
     <row r="3343">
       <c r="A3343" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3343" t="n">
-        <v>3495</v>
+        <v>3467</v>
       </c>
       <c r="C3343" t="inlineStr">
         <is>
-          <t>LUCILENE SANTOS DE MELO DAMASCENA</t>
+          <t>CILENE FERREIRA DA SILVA</t>
         </is>
       </c>
       <c r="D3343" t="inlineStr">
         <is>
-          <t>LUCILENE21</t>
+          <t>CILENE</t>
         </is>
       </c>
     </row>
     <row r="3344">
       <c r="A3344" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3344" t="n">
-        <v>3496</v>
+        <v>3495</v>
       </c>
       <c r="C3344" t="inlineStr">
         <is>
-          <t>JOAO PEDRO HENRIQUE ALVES DE ARAUJO</t>
+          <t>LUCILENE SANTOS DE MELO DAMASCENA</t>
         </is>
       </c>
       <c r="D3344" t="inlineStr">
         <is>
-          <t>JOAO.PEDRO</t>
+          <t>LUCILENE21</t>
         </is>
       </c>
     </row>
@@ -67318,16 +67318,16 @@
         </is>
       </c>
       <c r="B3345" t="n">
-        <v>3497</v>
+        <v>3496</v>
       </c>
       <c r="C3345" t="inlineStr">
         <is>
-          <t>ORLANDO MONTEIRO DE AMORIM</t>
+          <t>JOAO PEDRO HENRIQUE ALVES DE ARAUJO</t>
         </is>
       </c>
       <c r="D3345" t="inlineStr">
         <is>
-          <t>ORLANDO</t>
+          <t>JOAO.PEDRO</t>
         </is>
       </c>
     </row>
@@ -67338,176 +67338,176 @@
         </is>
       </c>
       <c r="B3346" t="n">
-        <v>3538</v>
+        <v>3497</v>
       </c>
       <c r="C3346" t="inlineStr">
         <is>
-          <t>PAULO HENRIQUE BENTO DA SILVA</t>
+          <t>ORLANDO MONTEIRO DE AMORIM</t>
         </is>
       </c>
       <c r="D3346" t="inlineStr">
         <is>
-          <t>P.BENTO</t>
+          <t>ORLANDO</t>
         </is>
       </c>
     </row>
     <row r="3347">
       <c r="A3347" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3347" t="n">
-        <v>3577</v>
+        <v>3538</v>
       </c>
       <c r="C3347" t="inlineStr">
         <is>
-          <t>NEGOCIACAO PI</t>
+          <t>PAULO HENRIQUE BENTO DA SILVA</t>
         </is>
       </c>
       <c r="D3347" t="inlineStr">
         <is>
-          <t>NEGOCIACAOPI</t>
+          <t>P.BENTO</t>
         </is>
       </c>
     </row>
     <row r="3348">
       <c r="A3348" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3348" t="n">
-        <v>3578</v>
+        <v>3577</v>
       </c>
       <c r="C3348" t="inlineStr">
         <is>
-          <t>NEGOCIACAO MA</t>
+          <t>NEGOCIACAO PI</t>
         </is>
       </c>
       <c r="D3348" t="inlineStr">
         <is>
-          <t>NEGOCIACAOMA</t>
+          <t>NEGOCIACAOPI</t>
         </is>
       </c>
     </row>
     <row r="3349">
       <c r="A3349" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3349" t="n">
-        <v>3595</v>
+        <v>3578</v>
       </c>
       <c r="C3349" t="inlineStr">
         <is>
-          <t>MIRLLENE PEREIRA RODRIGUES ROCHA</t>
+          <t>NEGOCIACAO MA</t>
         </is>
       </c>
       <c r="D3349" t="inlineStr">
         <is>
-          <t>MIRLLENE</t>
+          <t>NEGOCIACAOMA</t>
         </is>
       </c>
     </row>
     <row r="3350">
       <c r="A3350" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3350" t="n">
-        <v>3303</v>
+        <v>3595</v>
       </c>
       <c r="C3350" t="inlineStr">
         <is>
-          <t>DANIEL ALVES RODRIGUES</t>
+          <t>MIRLLENE PEREIRA RODRIGUES ROCHA</t>
         </is>
       </c>
       <c r="D3350" t="inlineStr">
         <is>
-          <t>DARODRIGUES</t>
+          <t>MIRLLENE</t>
         </is>
       </c>
     </row>
     <row r="3351">
       <c r="A3351" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3351" t="n">
-        <v>3316</v>
+        <v>3303</v>
       </c>
       <c r="C3351" t="inlineStr">
         <is>
-          <t xml:space="preserve">MARCELO PEREIRA BASTOS </t>
+          <t>DANIEL ALVES RODRIGUES</t>
         </is>
       </c>
       <c r="D3351" t="inlineStr">
         <is>
-          <t>MBASTOS</t>
+          <t>DARODRIGUES</t>
         </is>
       </c>
     </row>
     <row r="3352">
       <c r="A3352" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3352" t="n">
-        <v>3366</v>
+        <v>3316</v>
       </c>
       <c r="C3352" t="inlineStr">
         <is>
-          <t>MATEUS TEIXEIRA DA PAZ SILVA</t>
+          <t xml:space="preserve">MARCELO PEREIRA BASTOS </t>
         </is>
       </c>
       <c r="D3352" t="inlineStr">
         <is>
-          <t>PAZSILVA</t>
+          <t>MBASTOS</t>
         </is>
       </c>
     </row>
     <row r="3353">
       <c r="A3353" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3353" t="n">
-        <v>3393</v>
+        <v>3366</v>
       </c>
       <c r="C3353" t="inlineStr">
         <is>
-          <t xml:space="preserve">DAVID LUCAS RIBEIRO DOS SANTOS </t>
+          <t>MATEUS TEIXEIRA DA PAZ SILVA</t>
         </is>
       </c>
       <c r="D3353" t="inlineStr">
         <is>
-          <t>DLUCAS</t>
+          <t>PAZSILVA</t>
         </is>
       </c>
     </row>
     <row r="3354">
       <c r="A3354" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3354" t="n">
-        <v>3420</v>
+        <v>3393</v>
       </c>
       <c r="C3354" t="inlineStr">
         <is>
-          <t xml:space="preserve">CLAUDIO ROBERTO SILVA SOUZA </t>
+          <t xml:space="preserve">DAVID LUCAS RIBEIRO DOS SANTOS </t>
         </is>
       </c>
       <c r="D3354" t="inlineStr">
         <is>
-          <t>CLAUDIO21</t>
+          <t>DLUCAS</t>
         </is>
       </c>
     </row>
@@ -67518,16 +67518,16 @@
         </is>
       </c>
       <c r="B3355" t="n">
-        <v>3421</v>
+        <v>3420</v>
       </c>
       <c r="C3355" t="inlineStr">
         <is>
-          <t>WILSON PORTUGAL AZEVEDO FILHO</t>
+          <t xml:space="preserve">CLAUDIO ROBERTO SILVA SOUZA </t>
         </is>
       </c>
       <c r="D3355" t="inlineStr">
         <is>
-          <t>WILSONF</t>
+          <t>CLAUDIO21</t>
         </is>
       </c>
     </row>
@@ -67538,176 +67538,176 @@
         </is>
       </c>
       <c r="B3356" t="n">
-        <v>3439</v>
+        <v>3421</v>
       </c>
       <c r="C3356" t="inlineStr">
         <is>
-          <t>FERNANDA MASCARENHAS CEDRAZ</t>
+          <t>WILSON PORTUGAL AZEVEDO FILHO</t>
         </is>
       </c>
       <c r="D3356" t="inlineStr">
         <is>
-          <t>FERNANDAM</t>
+          <t>WILSONF</t>
         </is>
       </c>
     </row>
     <row r="3357">
       <c r="A3357" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3357" t="n">
-        <v>3455</v>
+        <v>3439</v>
       </c>
       <c r="C3357" t="inlineStr">
         <is>
-          <t xml:space="preserve">MARDONIO CUNHA BASILIO </t>
+          <t>FERNANDA MASCARENHAS CEDRAZ</t>
         </is>
       </c>
       <c r="D3357" t="inlineStr">
         <is>
-          <t>MARDONIO1</t>
+          <t>FERNANDAM</t>
         </is>
       </c>
     </row>
     <row r="3358">
       <c r="A3358" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3358" t="n">
-        <v>3508</v>
+        <v>3455</v>
       </c>
       <c r="C3358" t="inlineStr">
         <is>
-          <t>REBECA PIRES DE SOUZA MELO</t>
+          <t xml:space="preserve">MARDONIO CUNHA BASILIO </t>
         </is>
       </c>
       <c r="D3358" t="inlineStr">
         <is>
-          <t>RPMELO</t>
+          <t>MARDONIO1</t>
         </is>
       </c>
     </row>
     <row r="3359">
       <c r="A3359" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3359" t="n">
-        <v>3543</v>
+        <v>3508</v>
       </c>
       <c r="C3359" t="inlineStr">
         <is>
-          <t>JOAO GABRIEL BARBOSA FIRMINO</t>
+          <t>REBECA PIRES DE SOUZA MELO</t>
         </is>
       </c>
       <c r="D3359" t="inlineStr">
         <is>
-          <t>JOAOG</t>
+          <t>RPMELO</t>
         </is>
       </c>
     </row>
     <row r="3360">
       <c r="A3360" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3360" t="n">
-        <v>3580</v>
+        <v>3543</v>
       </c>
       <c r="C3360" t="inlineStr">
         <is>
-          <t>ALEXANDRE MARTINS CHAVES</t>
+          <t>JOAO GABRIEL BARBOSA FIRMINO</t>
         </is>
       </c>
       <c r="D3360" t="inlineStr">
         <is>
-          <t>MARTINS</t>
+          <t>JOAOG</t>
         </is>
       </c>
     </row>
     <row r="3361">
       <c r="A3361" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3361" t="n">
-        <v>3351</v>
+        <v>3580</v>
       </c>
       <c r="C3361" t="inlineStr">
         <is>
-          <t>HAWLLYSON DA SILVA COUTINHO</t>
+          <t>ALEXANDRE MARTINS CHAVES</t>
         </is>
       </c>
       <c r="D3361" t="inlineStr">
         <is>
-          <t>HCOUTINHO</t>
+          <t>MARTINS</t>
         </is>
       </c>
     </row>
     <row r="3362">
       <c r="A3362" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3362" t="n">
-        <v>940553</v>
+        <v>3351</v>
       </c>
       <c r="C3362" t="inlineStr">
         <is>
-          <t>LUTY TRANSPORTES- BA</t>
+          <t>HAWLLYSON DA SILVA COUTINHO</t>
         </is>
       </c>
       <c r="D3362" t="inlineStr">
         <is>
-          <t>LUTY TRANSPORTE</t>
+          <t>HCOUTINHO</t>
         </is>
       </c>
     </row>
     <row r="3363">
       <c r="A3363" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3363" t="n">
-        <v>3391</v>
+        <v>940553</v>
       </c>
       <c r="C3363" t="inlineStr">
         <is>
-          <t xml:space="preserve">NIKSON DA SILVA ALVES </t>
+          <t>LUTY TRANSPORTES- BA</t>
         </is>
       </c>
       <c r="D3363" t="inlineStr">
         <is>
-          <t>NIKSON</t>
+          <t>LUTY TRANSPORTE</t>
         </is>
       </c>
     </row>
     <row r="3364">
       <c r="A3364" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3364" t="n">
-        <v>3397</v>
+        <v>3391</v>
       </c>
       <c r="C3364" t="inlineStr">
         <is>
-          <t>EDILANE MENESES BALTAZAR</t>
+          <t xml:space="preserve">NIKSON DA SILVA ALVES </t>
         </is>
       </c>
       <c r="D3364" t="inlineStr">
         <is>
-          <t>EDILANE</t>
+          <t>NIKSON</t>
         </is>
       </c>
     </row>
@@ -67718,56 +67718,56 @@
         </is>
       </c>
       <c r="B3365" t="n">
-        <v>3398</v>
+        <v>3397</v>
       </c>
       <c r="C3365" t="inlineStr">
         <is>
-          <t>LUANA MARIA ROSIO DA SILVA</t>
+          <t>EDILANE MENESES BALTAZAR</t>
         </is>
       </c>
       <c r="D3365" t="inlineStr">
         <is>
-          <t>LUMARIA</t>
+          <t>EDILANE</t>
         </is>
       </c>
     </row>
     <row r="3366">
       <c r="A3366" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3366" t="n">
-        <v>3400</v>
+        <v>3398</v>
       </c>
       <c r="C3366" t="inlineStr">
         <is>
-          <t>ELILTON PINTO ROMEU</t>
+          <t>LUANA MARIA ROSIO DA SILVA</t>
         </is>
       </c>
       <c r="D3366" t="inlineStr">
         <is>
-          <t>ELILTON</t>
+          <t>LUMARIA</t>
         </is>
       </c>
     </row>
     <row r="3367">
       <c r="A3367" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3367" t="n">
-        <v>3406</v>
+        <v>3400</v>
       </c>
       <c r="C3367" t="inlineStr">
         <is>
-          <t>CONEXAO ALDA</t>
+          <t>ELILTON PINTO ROMEU</t>
         </is>
       </c>
       <c r="D3367" t="inlineStr">
         <is>
-          <t>CONEXAOALDA</t>
+          <t>ELILTON</t>
         </is>
       </c>
     </row>
@@ -67778,176 +67778,176 @@
         </is>
       </c>
       <c r="B3368" t="n">
-        <v>3407</v>
+        <v>3406</v>
       </c>
       <c r="C3368" t="inlineStr">
         <is>
-          <t>CONEXAO IRACEMA</t>
+          <t>CONEXAO ALDA</t>
         </is>
       </c>
       <c r="D3368" t="inlineStr">
         <is>
-          <t>CONEXAOIRACEMA</t>
+          <t>CONEXAOALDA</t>
         </is>
       </c>
     </row>
     <row r="3369">
       <c r="A3369" t="inlineStr">
         <is>
-          <t>9999</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3369" t="n">
-        <v>3408</v>
+        <v>3407</v>
       </c>
       <c r="C3369" t="inlineStr">
         <is>
-          <t>CONEXAO TAMILES</t>
+          <t>CONEXAO IRACEMA</t>
         </is>
       </c>
       <c r="D3369" t="inlineStr">
         <is>
-          <t>CONEXAOTAMILES</t>
+          <t>CONEXAOIRACEMA</t>
         </is>
       </c>
     </row>
     <row r="3370">
       <c r="A3370" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>9999</t>
         </is>
       </c>
       <c r="B3370" t="n">
-        <v>3414</v>
+        <v>3408</v>
       </c>
       <c r="C3370" t="inlineStr">
         <is>
-          <t>CONEXAO ADM PI MA</t>
+          <t>CONEXAO TAMILES</t>
         </is>
       </c>
       <c r="D3370" t="inlineStr">
         <is>
-          <t>CONEXAOPIMA</t>
+          <t>CONEXAOTAMILES</t>
         </is>
       </c>
     </row>
     <row r="3371">
       <c r="A3371" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3371" t="n">
-        <v>3524</v>
+        <v>3414</v>
       </c>
       <c r="C3371" t="inlineStr">
         <is>
-          <t>LUIS FELIPE DA SILVA SOUSA</t>
+          <t>CONEXAO ADM PI MA</t>
         </is>
       </c>
       <c r="D3371" t="inlineStr">
         <is>
-          <t>L.FELIPE</t>
+          <t>CONEXAOPIMA</t>
         </is>
       </c>
     </row>
     <row r="3372">
       <c r="A3372" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3372" t="n">
-        <v>3531</v>
+        <v>3524</v>
       </c>
       <c r="C3372" t="inlineStr">
         <is>
-          <t>LEICIANE COELHO SILVA</t>
+          <t>LUIS FELIPE DA SILVA SOUSA</t>
         </is>
       </c>
       <c r="D3372" t="inlineStr">
         <is>
-          <t>LEI.SILVA</t>
+          <t>L.FELIPE</t>
         </is>
       </c>
     </row>
     <row r="3373">
       <c r="A3373" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3373" t="n">
-        <v>3550</v>
+        <v>3531</v>
       </c>
       <c r="C3373" t="inlineStr">
         <is>
-          <t>IARGO GABRIEL SANTOS DE OLIVEIRA</t>
+          <t>LEICIANE COELHO SILVA</t>
         </is>
       </c>
       <c r="D3373" t="inlineStr">
         <is>
-          <t>IARGOG</t>
+          <t>LEI.SILVA</t>
         </is>
       </c>
     </row>
     <row r="3374">
       <c r="A3374" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3374" t="n">
-        <v>940567</v>
+        <v>3550</v>
       </c>
       <c r="C3374" t="inlineStr">
         <is>
-          <t>MS CARGAS E TRANSPORTES</t>
+          <t>IARGO GABRIEL SANTOS DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D3374" t="inlineStr">
         <is>
-          <t>ALAN BARBOSA</t>
+          <t>IARGOG</t>
         </is>
       </c>
     </row>
     <row r="3375">
       <c r="A3375" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3375" t="n">
-        <v>3560</v>
+        <v>940567</v>
       </c>
       <c r="C3375" t="inlineStr">
         <is>
-          <t>MARIA EDUARDA MELO DOS SANTOS</t>
+          <t>MS CARGAS E TRANSPORTES</t>
         </is>
       </c>
       <c r="D3375" t="inlineStr">
         <is>
-          <t>EDU.MELO</t>
+          <t>ALAN BARBOSA</t>
         </is>
       </c>
     </row>
     <row r="3376">
       <c r="A3376" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3376" t="n">
-        <v>3355</v>
+        <v>3560</v>
       </c>
       <c r="C3376" t="inlineStr">
         <is>
-          <t>HUGO MATHEUS DA COSTA FEITOSA</t>
+          <t>MARIA EDUARDA MELO DOS SANTOS</t>
         </is>
       </c>
       <c r="D3376" t="inlineStr">
         <is>
-          <t>HMFEITOSA</t>
+          <t>EDU.MELO</t>
         </is>
       </c>
     </row>
@@ -67958,96 +67958,96 @@
         </is>
       </c>
       <c r="B3377" t="n">
-        <v>3356</v>
+        <v>3355</v>
       </c>
       <c r="C3377" t="inlineStr">
         <is>
-          <t>BRENDA LIMA DE OLIVEIRA CUNHA</t>
+          <t>HUGO MATHEUS DA COSTA FEITOSA</t>
         </is>
       </c>
       <c r="D3377" t="inlineStr">
         <is>
-          <t>BLCUNHA</t>
+          <t>HMFEITOSA</t>
         </is>
       </c>
     </row>
     <row r="3378">
       <c r="A3378" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3378" t="n">
-        <v>3361</v>
+        <v>3356</v>
       </c>
       <c r="C3378" t="inlineStr">
         <is>
-          <t>WLADIA DE ARAUJO BASTOS</t>
+          <t>BRENDA LIMA DE OLIVEIRA CUNHA</t>
         </is>
       </c>
       <c r="D3378" t="inlineStr">
         <is>
-          <t>WABASTOS</t>
+          <t>BLCUNHA</t>
         </is>
       </c>
     </row>
     <row r="3379">
       <c r="A3379" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3379" t="n">
-        <v>3362</v>
+        <v>3361</v>
       </c>
       <c r="C3379" t="inlineStr">
         <is>
-          <t>CARLOS HENRIQUE MELO DA SILVA</t>
+          <t>WLADIA DE ARAUJO BASTOS</t>
         </is>
       </c>
       <c r="D3379" t="inlineStr">
         <is>
-          <t>CHMELO</t>
+          <t>WABASTOS</t>
         </is>
       </c>
     </row>
     <row r="3380">
       <c r="A3380" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3380" t="n">
-        <v>3375</v>
+        <v>3362</v>
       </c>
       <c r="C3380" t="inlineStr">
         <is>
-          <t>AFONSO DE SOUSA RAMOS FILHO</t>
+          <t>CARLOS HENRIQUE MELO DA SILVA</t>
         </is>
       </c>
       <c r="D3380" t="inlineStr">
         <is>
-          <t>AFILHO</t>
+          <t>CHMELO</t>
         </is>
       </c>
     </row>
     <row r="3381">
       <c r="A3381" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3381" t="n">
-        <v>3404</v>
+        <v>3375</v>
       </c>
       <c r="C3381" t="inlineStr">
         <is>
-          <t>NOVATO 4 COM</t>
+          <t>AFONSO DE SOUSA RAMOS FILHO</t>
         </is>
       </c>
       <c r="D3381" t="inlineStr">
         <is>
-          <t>NOVATO4COM</t>
+          <t>AFILHO</t>
         </is>
       </c>
     </row>
@@ -68058,176 +68058,176 @@
         </is>
       </c>
       <c r="B3382" t="n">
-        <v>3405</v>
+        <v>3404</v>
       </c>
       <c r="C3382" t="inlineStr">
         <is>
-          <t>NOVATO 5 COM</t>
+          <t>NOVATO 4 COM</t>
         </is>
       </c>
       <c r="D3382" t="inlineStr">
         <is>
-          <t>NOVATO5COM</t>
+          <t>NOVATO4COM</t>
         </is>
       </c>
     </row>
     <row r="3383">
       <c r="A3383" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3383" t="n">
-        <v>3447</v>
+        <v>3405</v>
       </c>
       <c r="C3383" t="inlineStr">
         <is>
-          <t>RAYSSA KEYCE LINHARES AQUINO</t>
+          <t>NOVATO 5 COM</t>
         </is>
       </c>
       <c r="D3383" t="inlineStr">
         <is>
-          <t>RAYSSAK</t>
+          <t>NOVATO5COM</t>
         </is>
       </c>
     </row>
     <row r="3384">
       <c r="A3384" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3384" t="n">
-        <v>940559</v>
+        <v>3447</v>
       </c>
       <c r="C3384" t="inlineStr">
         <is>
-          <t>WALLEF DE OLIVEIRA</t>
+          <t>RAYSSA KEYCE LINHARES AQUINO</t>
         </is>
       </c>
       <c r="D3384" t="inlineStr">
         <is>
-          <t>WALLEF</t>
+          <t>RAYSSAK</t>
         </is>
       </c>
     </row>
     <row r="3385">
       <c r="A3385" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>99</t>
         </is>
       </c>
       <c r="B3385" t="n">
-        <v>3489</v>
+        <v>940559</v>
       </c>
       <c r="C3385" t="inlineStr">
         <is>
-          <t>MARCELA KARINA PEREIRA VELOSO</t>
+          <t>WALLEF DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D3385" t="inlineStr">
         <is>
-          <t>MKARINA</t>
+          <t>WALLEF</t>
         </is>
       </c>
     </row>
     <row r="3386">
       <c r="A3386" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3386" t="n">
-        <v>3490</v>
+        <v>3489</v>
       </c>
       <c r="C3386" t="inlineStr">
         <is>
-          <t>JOSE MAILSON GOMES NUNES</t>
+          <t>MARCELA KARINA PEREIRA VELOSO</t>
         </is>
       </c>
       <c r="D3386" t="inlineStr">
         <is>
-          <t>J.MAILSON</t>
+          <t>MKARINA</t>
         </is>
       </c>
     </row>
     <row r="3387">
       <c r="A3387" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3387" t="n">
-        <v>3537</v>
+        <v>3490</v>
       </c>
       <c r="C3387" t="inlineStr">
         <is>
-          <t>ALDAIR PEDRO DA SILVA</t>
+          <t>JOSE MAILSON GOMES NUNES</t>
         </is>
       </c>
       <c r="D3387" t="inlineStr">
         <is>
-          <t>A.PEDRO</t>
+          <t>J.MAILSON</t>
         </is>
       </c>
     </row>
     <row r="3388">
       <c r="A3388" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3388" t="n">
-        <v>3549</v>
+        <v>3537</v>
       </c>
       <c r="C3388" t="inlineStr">
         <is>
-          <t xml:space="preserve">FERNANDA CAROLINE E CESAR SOUSA </t>
+          <t>ALDAIR PEDRO DA SILVA</t>
         </is>
       </c>
       <c r="D3388" t="inlineStr">
         <is>
-          <t>FCAROLINE</t>
+          <t>A.PEDRO</t>
         </is>
       </c>
     </row>
     <row r="3389">
       <c r="A3389" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3389" t="n">
-        <v>3581</v>
+        <v>3549</v>
       </c>
       <c r="C3389" t="inlineStr">
         <is>
-          <t xml:space="preserve">VALQUIRIO OLIVEIRA SOUSA </t>
+          <t xml:space="preserve">FERNANDA CAROLINE E CESAR SOUSA </t>
         </is>
       </c>
       <c r="D3389" t="inlineStr">
         <is>
-          <t>VALQUIRIO</t>
+          <t>FCAROLINE</t>
         </is>
       </c>
     </row>
     <row r="3390">
       <c r="A3390" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3390" t="n">
-        <v>3337</v>
+        <v>3581</v>
       </c>
       <c r="C3390" t="inlineStr">
         <is>
-          <t>WESLEY FONTES DE ALMEIDA</t>
+          <t xml:space="preserve">VALQUIRIO OLIVEIRA SOUSA </t>
         </is>
       </c>
       <c r="D3390" t="inlineStr">
         <is>
-          <t>WFALMEIDA</t>
+          <t>VALQUIRIO</t>
         </is>
       </c>
     </row>
@@ -68238,16 +68238,16 @@
         </is>
       </c>
       <c r="B3391" t="n">
-        <v>3338</v>
+        <v>3337</v>
       </c>
       <c r="C3391" t="inlineStr">
         <is>
-          <t>FRANCISCA SAMARA MENDES DE OLIVEIRA C</t>
+          <t>WESLEY FONTES DE ALMEIDA</t>
         </is>
       </c>
       <c r="D3391" t="inlineStr">
         <is>
-          <t>FSCUNHA</t>
+          <t>WFALMEIDA</t>
         </is>
       </c>
     </row>
@@ -68258,176 +68258,176 @@
         </is>
       </c>
       <c r="B3392" t="n">
-        <v>3339</v>
+        <v>3338</v>
       </c>
       <c r="C3392" t="inlineStr">
         <is>
-          <t>MAYARA THALYA DIAS DE ANDRADE</t>
+          <t>FRANCISCA SAMARA MENDES DE OLIVEIRA C</t>
         </is>
       </c>
       <c r="D3392" t="inlineStr">
         <is>
-          <t>MTANDRADE</t>
+          <t>FSCUNHA</t>
         </is>
       </c>
     </row>
     <row r="3393">
       <c r="A3393" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3393" t="n">
-        <v>3359</v>
+        <v>3339</v>
       </c>
       <c r="C3393" t="inlineStr">
         <is>
-          <t xml:space="preserve">EVANESSA DA SILVA E SILVA </t>
+          <t>MAYARA THALYA DIAS DE ANDRADE</t>
         </is>
       </c>
       <c r="D3393" t="inlineStr">
         <is>
-          <t>EVANESSAS</t>
+          <t>MTANDRADE</t>
         </is>
       </c>
     </row>
     <row r="3394">
       <c r="A3394" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3394" t="n">
-        <v>3360</v>
+        <v>3359</v>
       </c>
       <c r="C3394" t="inlineStr">
         <is>
-          <t>THIAGO DE CARVALHO ARAUJO</t>
+          <t xml:space="preserve">EVANESSA DA SILVA E SILVA </t>
         </is>
       </c>
       <c r="D3394" t="inlineStr">
         <is>
-          <t>TCARAUJO</t>
+          <t>EVANESSAS</t>
         </is>
       </c>
     </row>
     <row r="3395">
       <c r="A3395" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3395" t="n">
-        <v>3481</v>
+        <v>3360</v>
       </c>
       <c r="C3395" t="inlineStr">
         <is>
-          <t xml:space="preserve">EDSON DA PAZ LIMA </t>
+          <t>THIAGO DE CARVALHO ARAUJO</t>
         </is>
       </c>
       <c r="D3395" t="inlineStr">
         <is>
-          <t>EDPAZ</t>
+          <t>TCARAUJO</t>
         </is>
       </c>
     </row>
     <row r="3396">
       <c r="A3396" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3396" t="n">
-        <v>3494</v>
+        <v>3481</v>
       </c>
       <c r="C3396" t="inlineStr">
         <is>
-          <t>ANTONIO CRISTINA BRITO GOMES</t>
+          <t xml:space="preserve">EDSON DA PAZ LIMA </t>
         </is>
       </c>
       <c r="D3396" t="inlineStr">
         <is>
-          <t>CRIS.GOMES</t>
+          <t>EDPAZ</t>
         </is>
       </c>
     </row>
     <row r="3397">
       <c r="A3397" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3397" t="n">
-        <v>3498</v>
+        <v>3494</v>
       </c>
       <c r="C3397" t="inlineStr">
         <is>
-          <t>SILVESTRA COSTA NUNES</t>
+          <t>ANTONIO CRISTINA BRITO GOMES</t>
         </is>
       </c>
       <c r="D3397" t="inlineStr">
         <is>
-          <t>SCNUNES</t>
+          <t>CRIS.GOMES</t>
         </is>
       </c>
     </row>
     <row r="3398">
       <c r="A3398" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3398" t="n">
-        <v>940562</v>
+        <v>3498</v>
       </c>
       <c r="C3398" t="inlineStr">
         <is>
-          <t>FRANCISCO DAVID ASSUNCAO ALVES</t>
+          <t>SILVESTRA COSTA NUNES</t>
         </is>
       </c>
       <c r="D3398" t="inlineStr">
         <is>
-          <t>ASSUNÇÃO</t>
+          <t>SCNUNES</t>
         </is>
       </c>
     </row>
     <row r="3399">
       <c r="A3399" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>99</t>
         </is>
       </c>
       <c r="B3399" t="n">
-        <v>3513</v>
+        <v>940562</v>
       </c>
       <c r="C3399" t="inlineStr">
         <is>
-          <t>RENARA ANDRADE MATIAS</t>
+          <t>FRANCISCO DAVID ASSUNCAO ALVES</t>
         </is>
       </c>
       <c r="D3399" t="inlineStr">
         <is>
-          <t>R.ANDRADE</t>
+          <t>ASSUNÇÃO</t>
         </is>
       </c>
     </row>
     <row r="3400">
       <c r="A3400" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3400" t="n">
-        <v>3275</v>
+        <v>3513</v>
       </c>
       <c r="C3400" t="inlineStr">
         <is>
-          <t>MARIA APARECIDA COELHO SILVA</t>
+          <t>RENARA ANDRADE MATIAS</t>
         </is>
       </c>
       <c r="D3400" t="inlineStr">
         <is>
-          <t>MCOELHO</t>
+          <t>R.ANDRADE</t>
         </is>
       </c>
     </row>
@@ -68438,136 +68438,136 @@
         </is>
       </c>
       <c r="B3401" t="n">
-        <v>3276</v>
+        <v>3275</v>
       </c>
       <c r="C3401" t="inlineStr">
         <is>
-          <t xml:space="preserve">PEROLA DE JESUS AMORIM SOUSA </t>
+          <t>MARIA APARECIDA COELHO SILVA</t>
         </is>
       </c>
       <c r="D3401" t="inlineStr">
         <is>
-          <t>PJESUS</t>
+          <t>MCOELHO</t>
         </is>
       </c>
     </row>
     <row r="3402">
       <c r="A3402" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3402" t="n">
-        <v>3526</v>
+        <v>3276</v>
       </c>
       <c r="C3402" t="inlineStr">
         <is>
-          <t>JOYCE NAZARE CORREA</t>
+          <t xml:space="preserve">PEROLA DE JESUS AMORIM SOUSA </t>
         </is>
       </c>
       <c r="D3402" t="inlineStr">
         <is>
-          <t>J.NAZARE</t>
+          <t>PJESUS</t>
         </is>
       </c>
     </row>
     <row r="3403">
       <c r="A3403" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3403" t="n">
-        <v>3527</v>
+        <v>3526</v>
       </c>
       <c r="C3403" t="inlineStr">
         <is>
-          <t>GILVANA DA SILVA MONTELES</t>
+          <t>JOYCE NAZARE CORREA</t>
         </is>
       </c>
       <c r="D3403" t="inlineStr">
         <is>
-          <t>GIL.SILVA</t>
+          <t>J.NAZARE</t>
         </is>
       </c>
     </row>
     <row r="3404">
       <c r="A3404" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B3404" t="n">
-        <v>3548</v>
+        <v>3527</v>
       </c>
       <c r="C3404" t="inlineStr">
         <is>
-          <t>JAMILLY MARIA HENRIQUE ARAUJO</t>
+          <t>GILVANA DA SILVA MONTELES</t>
         </is>
       </c>
       <c r="D3404" t="inlineStr">
         <is>
-          <t>JAMILLY</t>
+          <t>GIL.SILVA</t>
         </is>
       </c>
     </row>
     <row r="3405">
       <c r="A3405" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3405" t="n">
-        <v>3551</v>
+        <v>3548</v>
       </c>
       <c r="C3405" t="inlineStr">
         <is>
-          <t xml:space="preserve">VITOR MANOEL DA SILVA BARBOSA </t>
+          <t>JAMILLY MARIA HENRIQUE ARAUJO</t>
         </is>
       </c>
       <c r="D3405" t="inlineStr">
         <is>
-          <t>VMANOEL</t>
+          <t>JAMILLY</t>
         </is>
       </c>
     </row>
     <row r="3406">
       <c r="A3406" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3406" t="n">
-        <v>3588</v>
+        <v>3551</v>
       </c>
       <c r="C3406" t="inlineStr">
         <is>
-          <t>BRUNA RAISEYLLA SANTOS DE SALES</t>
+          <t xml:space="preserve">VITOR MANOEL DA SILVA BARBOSA </t>
         </is>
       </c>
       <c r="D3406" t="inlineStr">
         <is>
-          <t>BRU.SALES</t>
+          <t>VMANOEL</t>
         </is>
       </c>
     </row>
     <row r="3407">
       <c r="A3407" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3407" t="n">
-        <v>940525</v>
+        <v>3588</v>
       </c>
       <c r="C3407" t="inlineStr">
         <is>
-          <t>SANDUWELLINGTON</t>
+          <t>BRUNA RAISEYLLA SANTOS DE SALES</t>
         </is>
       </c>
       <c r="D3407" t="inlineStr">
         <is>
-          <t>SANDUWELLINGTON</t>
+          <t>BRU.SALES</t>
         </is>
       </c>
     </row>
@@ -68578,36 +68578,36 @@
         </is>
       </c>
       <c r="B3408" t="n">
-        <v>3369</v>
+        <v>940525</v>
       </c>
       <c r="C3408" t="inlineStr">
         <is>
-          <t xml:space="preserve">PRISCILA DOS SANTOS LOPES </t>
+          <t>SANDUWELLINGTON</t>
         </is>
       </c>
       <c r="D3408" t="inlineStr">
         <is>
-          <t>PSLOPES</t>
+          <t>SANDUWELLINGTON</t>
         </is>
       </c>
     </row>
     <row r="3409">
       <c r="A3409" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3409" t="n">
-        <v>3433</v>
+        <v>3369</v>
       </c>
       <c r="C3409" t="inlineStr">
         <is>
-          <t>BRUNO NUNES CRUZ</t>
+          <t xml:space="preserve">PRISCILA DOS SANTOS LOPES </t>
         </is>
       </c>
       <c r="D3409" t="inlineStr">
         <is>
-          <t>BRUNOCRUZ</t>
+          <t>PSLOPES</t>
         </is>
       </c>
     </row>
@@ -68618,36 +68618,36 @@
         </is>
       </c>
       <c r="B3410" t="n">
-        <v>3434</v>
+        <v>3433</v>
       </c>
       <c r="C3410" t="inlineStr">
         <is>
-          <t>ANA TERCIA DE LIMA SA CARVALHO SERAFIM</t>
+          <t>BRUNO NUNES CRUZ</t>
         </is>
       </c>
       <c r="D3410" t="inlineStr">
         <is>
-          <t>ANATER</t>
+          <t>BRUNOCRUZ</t>
         </is>
       </c>
     </row>
     <row r="3411">
       <c r="A3411" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3411" t="n">
-        <v>3502</v>
+        <v>3434</v>
       </c>
       <c r="C3411" t="inlineStr">
         <is>
-          <t>LUIZ FELIPE MACHADO BARRETO</t>
+          <t>ANA TERCIA DE LIMA SA CARVALHO SERAFIM</t>
         </is>
       </c>
       <c r="D3411" t="inlineStr">
         <is>
-          <t>LUIZ.FELIPE</t>
+          <t>ANATER</t>
         </is>
       </c>
     </row>
@@ -68658,36 +68658,36 @@
         </is>
       </c>
       <c r="B3412" t="n">
-        <v>3503</v>
+        <v>3502</v>
       </c>
       <c r="C3412" t="inlineStr">
         <is>
-          <t>FABIO OLIVEIRA SILVA</t>
+          <t>LUIZ FELIPE MACHADO BARRETO</t>
         </is>
       </c>
       <c r="D3412" t="inlineStr">
         <is>
-          <t>FOSILVA</t>
+          <t>LUIZ.FELIPE</t>
         </is>
       </c>
     </row>
     <row r="3413">
       <c r="A3413" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3413" t="n">
-        <v>3554</v>
+        <v>3503</v>
       </c>
       <c r="C3413" t="inlineStr">
         <is>
-          <t xml:space="preserve">MANOEL RIBEIRO DE SOUZA JUNIOR </t>
+          <t>FABIO OLIVEIRA SILVA</t>
         </is>
       </c>
       <c r="D3413" t="inlineStr">
         <is>
-          <t>MRJUNIOR</t>
+          <t>FOSILVA</t>
         </is>
       </c>
     </row>
@@ -68698,16 +68698,16 @@
         </is>
       </c>
       <c r="B3414" t="n">
-        <v>3568</v>
+        <v>3554</v>
       </c>
       <c r="C3414" t="inlineStr">
         <is>
-          <t xml:space="preserve">ANGELICA TORRES DA SILVA </t>
+          <t xml:space="preserve">MANOEL RIBEIRO DE SOUZA JUNIOR </t>
         </is>
       </c>
       <c r="D3414" t="inlineStr">
         <is>
-          <t>ANGEL.TORRES</t>
+          <t>MRJUNIOR</t>
         </is>
       </c>
     </row>
@@ -68718,56 +68718,56 @@
         </is>
       </c>
       <c r="B3415" t="n">
-        <v>3569</v>
+        <v>3568</v>
       </c>
       <c r="C3415" t="inlineStr">
         <is>
-          <t>LORENA DE LIMA MATOS</t>
+          <t xml:space="preserve">ANGELICA TORRES DA SILVA </t>
         </is>
       </c>
       <c r="D3415" t="inlineStr">
         <is>
-          <t>LORE.LIMA</t>
+          <t>ANGEL.TORRES</t>
         </is>
       </c>
     </row>
     <row r="3416">
       <c r="A3416" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3416" t="n">
-        <v>3576</v>
+        <v>3569</v>
       </c>
       <c r="C3416" t="inlineStr">
         <is>
-          <t>ANA BEATRIZ PARENTE CAVALCANTE</t>
+          <t>LORENA DE LIMA MATOS</t>
         </is>
       </c>
       <c r="D3416" t="inlineStr">
         <is>
-          <t>A.BEATRIZ</t>
+          <t>LORE.LIMA</t>
         </is>
       </c>
     </row>
     <row r="3417">
       <c r="A3417" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3417" t="n">
-        <v>940549</v>
+        <v>3576</v>
       </c>
       <c r="C3417" t="inlineStr">
         <is>
-          <t>EDILSON ARAUJO - FL9</t>
+          <t>ANA BEATRIZ PARENTE CAVALCANTE</t>
         </is>
       </c>
       <c r="D3417" t="inlineStr">
         <is>
-          <t>EDILSON</t>
+          <t>A.BEATRIZ</t>
         </is>
       </c>
     </row>
@@ -68778,36 +68778,36 @@
         </is>
       </c>
       <c r="B3418" t="n">
-        <v>3470</v>
+        <v>940549</v>
       </c>
       <c r="C3418" t="inlineStr">
         <is>
-          <t>DEBORA ALVES CARVALHO</t>
+          <t>EDILSON ARAUJO - FL9</t>
         </is>
       </c>
       <c r="D3418" t="inlineStr">
         <is>
-          <t>DEBORA.ALVES</t>
+          <t>EDILSON</t>
         </is>
       </c>
     </row>
     <row r="3419">
       <c r="A3419" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3419" t="n">
-        <v>3510</v>
+        <v>3470</v>
       </c>
       <c r="C3419" t="inlineStr">
         <is>
-          <t>CAMILA RODIGUES PINTO</t>
+          <t>DEBORA ALVES CARVALHO</t>
         </is>
       </c>
       <c r="D3419" t="inlineStr">
         <is>
-          <t>MILA.PINTO</t>
+          <t>DEBORA.ALVES</t>
         </is>
       </c>
     </row>
@@ -68818,96 +68818,96 @@
         </is>
       </c>
       <c r="B3420" t="n">
-        <v>3511</v>
+        <v>3510</v>
       </c>
       <c r="C3420" t="inlineStr">
         <is>
-          <t>JORGE HENRIQUE DOS SANTOS RODRIGUES</t>
+          <t>CAMILA RODIGUES PINTO</t>
         </is>
       </c>
       <c r="D3420" t="inlineStr">
         <is>
-          <t>J.HENRIQUE</t>
+          <t>MILA.PINTO</t>
         </is>
       </c>
     </row>
     <row r="3421">
       <c r="A3421" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3421" t="n">
-        <v>3561</v>
+        <v>3511</v>
       </c>
       <c r="C3421" t="inlineStr">
         <is>
-          <t>RONARIA PATRICIA VILARINDO DE ALMEIDA</t>
+          <t>JORGE HENRIQUE DOS SANTOS RODRIGUES</t>
         </is>
       </c>
       <c r="D3421" t="inlineStr">
         <is>
-          <t>RPATRICIA</t>
+          <t>J.HENRIQUE</t>
         </is>
       </c>
     </row>
     <row r="3422">
       <c r="A3422" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3422" t="n">
-        <v>3562</v>
+        <v>3561</v>
       </c>
       <c r="C3422" t="inlineStr">
         <is>
-          <t>LETICIA MARIA BENTO NOGUEIRA</t>
+          <t>RONARIA PATRICIA VILARINDO DE ALMEIDA</t>
         </is>
       </c>
       <c r="D3422" t="inlineStr">
         <is>
-          <t>LBENTO</t>
+          <t>RPATRICIA</t>
         </is>
       </c>
     </row>
     <row r="3423">
       <c r="A3423" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3423" t="n">
-        <v>3270</v>
+        <v>3562</v>
       </c>
       <c r="C3423" t="inlineStr">
         <is>
-          <t>ITANA NASCIMENTO SIMOES</t>
+          <t>LETICIA MARIA BENTO NOGUEIRA</t>
         </is>
       </c>
       <c r="D3423" t="inlineStr">
         <is>
-          <t>ISIMOES</t>
+          <t>LBENTO</t>
         </is>
       </c>
     </row>
     <row r="3424">
       <c r="A3424" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3424" t="n">
-        <v>3318</v>
+        <v>3270</v>
       </c>
       <c r="C3424" t="inlineStr">
         <is>
-          <t>LUAN MONTEIRO COSTA</t>
+          <t>ITANA NASCIMENTO SIMOES</t>
         </is>
       </c>
       <c r="D3424" t="inlineStr">
         <is>
-          <t>LMONTEIRO</t>
+          <t>ISIMOES</t>
         </is>
       </c>
     </row>
@@ -68918,36 +68918,36 @@
         </is>
       </c>
       <c r="B3425" t="n">
-        <v>3319</v>
+        <v>3318</v>
       </c>
       <c r="C3425" t="inlineStr">
         <is>
-          <t>MARIANA MACEDA DOS SANTOS</t>
+          <t>LUAN MONTEIRO COSTA</t>
         </is>
       </c>
       <c r="D3425" t="inlineStr">
         <is>
-          <t>MMACEDA</t>
+          <t>LMONTEIRO</t>
         </is>
       </c>
     </row>
     <row r="3426">
       <c r="A3426" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3426" t="n">
-        <v>3389</v>
+        <v>3319</v>
       </c>
       <c r="C3426" t="inlineStr">
         <is>
-          <t>TAMILES DE SANTANA AMORIM BISPO</t>
+          <t>MARIANA MACEDA DOS SANTOS</t>
         </is>
       </c>
       <c r="D3426" t="inlineStr">
         <is>
-          <t>TAMILES</t>
+          <t>MMACEDA</t>
         </is>
       </c>
     </row>
@@ -68958,76 +68958,76 @@
         </is>
       </c>
       <c r="B3427" t="n">
-        <v>3390</v>
+        <v>3389</v>
       </c>
       <c r="C3427" t="inlineStr">
         <is>
-          <t>IRACEMA DE ALMEIDA MOURA</t>
+          <t>TAMILES DE SANTANA AMORIM BISPO</t>
         </is>
       </c>
       <c r="D3427" t="inlineStr">
         <is>
-          <t>IRACEMA</t>
+          <t>TAMILES</t>
         </is>
       </c>
     </row>
     <row r="3428">
       <c r="A3428" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3428" t="n">
-        <v>3575</v>
+        <v>3390</v>
       </c>
       <c r="C3428" t="inlineStr">
         <is>
-          <t>SAMARA ALVES DA SILVA</t>
+          <t>IRACEMA DE ALMEIDA MOURA</t>
         </is>
       </c>
       <c r="D3428" t="inlineStr">
         <is>
-          <t>S.ALVES</t>
+          <t>IRACEMA</t>
         </is>
       </c>
     </row>
     <row r="3429">
       <c r="A3429" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3429" t="n">
-        <v>3583</v>
+        <v>3575</v>
       </c>
       <c r="C3429" t="inlineStr">
         <is>
-          <t>TALLIS GUTTEMBERG GUIMARES BATISTA</t>
+          <t>SAMARA ALVES DA SILVA</t>
         </is>
       </c>
       <c r="D3429" t="inlineStr">
         <is>
-          <t>TALLIS16</t>
+          <t>S.ALVES</t>
         </is>
       </c>
     </row>
     <row r="3430">
       <c r="A3430" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3430" t="n">
-        <v>3286</v>
+        <v>3583</v>
       </c>
       <c r="C3430" t="inlineStr">
         <is>
-          <t>VALERIA MAIA DA SILVA</t>
+          <t>TALLIS GUTTEMBERG GUIMARES BATISTA</t>
         </is>
       </c>
       <c r="D3430" t="inlineStr">
         <is>
-          <t>VMAIAS</t>
+          <t>TALLIS16</t>
         </is>
       </c>
     </row>
@@ -69038,156 +69038,156 @@
         </is>
       </c>
       <c r="B3431" t="n">
-        <v>3287</v>
+        <v>3286</v>
       </c>
       <c r="C3431" t="inlineStr">
         <is>
-          <t>ERIVELTON DA SILVA OLIVEIRA</t>
+          <t>VALERIA MAIA DA SILVA</t>
         </is>
       </c>
       <c r="D3431" t="inlineStr">
         <is>
-          <t>ESOLIVEIRA</t>
+          <t>VMAIAS</t>
         </is>
       </c>
     </row>
     <row r="3432">
       <c r="A3432" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3432" t="n">
-        <v>3307</v>
+        <v>3287</v>
       </c>
       <c r="C3432" t="inlineStr">
         <is>
-          <t>ADRIEL XERES BARROS MARTINS</t>
+          <t>ERIVELTON DA SILVA OLIVEIRA</t>
         </is>
       </c>
       <c r="D3432" t="inlineStr">
         <is>
-          <t>AXERES</t>
+          <t>ESOLIVEIRA</t>
         </is>
       </c>
     </row>
     <row r="3433">
       <c r="A3433" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3433" t="n">
-        <v>3308</v>
+        <v>3307</v>
       </c>
       <c r="C3433" t="inlineStr">
         <is>
-          <t>ELKZIEL JUVINO DA SILVA</t>
+          <t>ADRIEL XERES BARROS MARTINS</t>
         </is>
       </c>
       <c r="D3433" t="inlineStr">
         <is>
-          <t>EJUVINO</t>
+          <t>AXERES</t>
         </is>
       </c>
     </row>
     <row r="3434">
       <c r="A3434" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3434" t="n">
-        <v>940539</v>
+        <v>3308</v>
       </c>
       <c r="C3434" t="inlineStr">
         <is>
-          <t>EDSON ARAUJO - FL9</t>
+          <t>ELKZIEL JUVINO DA SILVA</t>
         </is>
       </c>
       <c r="D3434" t="inlineStr">
         <is>
-          <t>EDS</t>
+          <t>EJUVINO</t>
         </is>
       </c>
     </row>
     <row r="3435">
       <c r="A3435" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3435" t="n">
-        <v>940540</v>
+        <v>940539</v>
       </c>
       <c r="C3435" t="inlineStr">
         <is>
-          <t>EDSON ARAUJO - FL8</t>
+          <t>EDSON ARAUJO - FL9</t>
         </is>
       </c>
       <c r="D3435" t="inlineStr">
         <is>
-          <t>EDS8</t>
+          <t>EDS</t>
         </is>
       </c>
     </row>
     <row r="3436">
       <c r="A3436" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B3436" t="n">
-        <v>3328</v>
+        <v>940540</v>
       </c>
       <c r="C3436" t="inlineStr">
         <is>
-          <t>ALAN ARAUJO DA SILVA</t>
+          <t>EDSON ARAUJO - FL8</t>
         </is>
       </c>
       <c r="D3436" t="inlineStr">
         <is>
-          <t>ARSILVA</t>
+          <t>EDS8</t>
         </is>
       </c>
     </row>
     <row r="3437">
       <c r="A3437" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3437" t="n">
-        <v>3350</v>
+        <v>3328</v>
       </c>
       <c r="C3437" t="inlineStr">
         <is>
-          <t xml:space="preserve">EDER RODRIGUES DA SILVA </t>
+          <t>ALAN ARAUJO DA SILVA</t>
         </is>
       </c>
       <c r="D3437" t="inlineStr">
         <is>
-          <t>EDERS</t>
+          <t>ARSILVA</t>
         </is>
       </c>
     </row>
     <row r="3438">
       <c r="A3438" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3438" t="n">
-        <v>3373</v>
+        <v>3350</v>
       </c>
       <c r="C3438" t="inlineStr">
         <is>
-          <t xml:space="preserve">NATANAEL TAVARES DE SOUSA </t>
+          <t xml:space="preserve">EDER RODRIGUES DA SILVA </t>
         </is>
       </c>
       <c r="D3438" t="inlineStr">
         <is>
-          <t>NTSOUSA</t>
+          <t>EDERS</t>
         </is>
       </c>
     </row>
@@ -69198,156 +69198,156 @@
         </is>
       </c>
       <c r="B3439" t="n">
-        <v>3374</v>
+        <v>3373</v>
       </c>
       <c r="C3439" t="inlineStr">
         <is>
-          <t>REINALDO DA SILVA COSTA</t>
+          <t xml:space="preserve">NATANAEL TAVARES DE SOUSA </t>
         </is>
       </c>
       <c r="D3439" t="inlineStr">
         <is>
-          <t>RSCOSTA</t>
+          <t>NTSOUSA</t>
         </is>
       </c>
     </row>
     <row r="3440">
       <c r="A3440" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3440" t="n">
-        <v>3399</v>
+        <v>3374</v>
       </c>
       <c r="C3440" t="inlineStr">
         <is>
-          <t xml:space="preserve">RICARDO BARBOSA DOS SANTOS </t>
+          <t>REINALDO DA SILVA COSTA</t>
         </is>
       </c>
       <c r="D3440" t="inlineStr">
         <is>
-          <t>RICARDOSAN</t>
+          <t>RSCOSTA</t>
         </is>
       </c>
     </row>
     <row r="3441">
       <c r="A3441" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3441" t="n">
-        <v>3427</v>
+        <v>3399</v>
       </c>
       <c r="C3441" t="inlineStr">
         <is>
-          <t>ROQUE COMERCIO TEMPORARIO</t>
+          <t xml:space="preserve">RICARDO BARBOSA DOS SANTOS </t>
         </is>
       </c>
       <c r="D3441" t="inlineStr">
         <is>
-          <t>ROQUECOM</t>
+          <t>RICARDOSAN</t>
         </is>
       </c>
     </row>
     <row r="3442">
       <c r="A3442" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3442" t="n">
-        <v>3428</v>
+        <v>3427</v>
       </c>
       <c r="C3442" t="inlineStr">
         <is>
-          <t>ROQUE PLUS TEMPORARIO</t>
+          <t>ROQUE COMERCIO TEMPORARIO</t>
         </is>
       </c>
       <c r="D3442" t="inlineStr">
         <is>
-          <t>ROQUEPLUS</t>
+          <t>ROQUECOM</t>
         </is>
       </c>
     </row>
     <row r="3443">
       <c r="A3443" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3443" t="n">
-        <v>3432</v>
+        <v>3428</v>
       </c>
       <c r="C3443" t="inlineStr">
         <is>
-          <t>PATRICIA DOS SANTOS NONATO OLIVEIRA</t>
+          <t>ROQUE PLUS TEMPORARIO</t>
         </is>
       </c>
       <c r="D3443" t="inlineStr">
         <is>
-          <t>PATRICIAD</t>
+          <t>ROQUEPLUS</t>
         </is>
       </c>
     </row>
     <row r="3444">
       <c r="A3444" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3444" t="n">
-        <v>3448</v>
+        <v>3432</v>
       </c>
       <c r="C3444" t="inlineStr">
         <is>
-          <t xml:space="preserve">GABRIEL SOUZA CARVALHO </t>
+          <t>PATRICIA DOS SANTOS NONATO OLIVEIRA</t>
         </is>
       </c>
       <c r="D3444" t="inlineStr">
         <is>
-          <t>GABRIEL20</t>
+          <t>PATRICIAD</t>
         </is>
       </c>
     </row>
     <row r="3445">
       <c r="A3445" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3445" t="n">
-        <v>3465</v>
+        <v>3448</v>
       </c>
       <c r="C3445" t="inlineStr">
         <is>
-          <t>LUIZA MARIA BARRETO BARBOSA</t>
+          <t xml:space="preserve">GABRIEL SOUZA CARVALHO </t>
         </is>
       </c>
       <c r="D3445" t="inlineStr">
         <is>
-          <t>LUIZA.MARIA</t>
+          <t>GABRIEL20</t>
         </is>
       </c>
     </row>
     <row r="3446">
       <c r="A3446" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3446" t="n">
-        <v>3468</v>
+        <v>3465</v>
       </c>
       <c r="C3446" t="inlineStr">
         <is>
-          <t>KAWA ALMEIDA CAMPOS</t>
+          <t>LUIZA MARIA BARRETO BARBOSA</t>
         </is>
       </c>
       <c r="D3446" t="inlineStr">
         <is>
-          <t>KAWA</t>
+          <t>LUIZA.MARIA</t>
         </is>
       </c>
     </row>
@@ -69358,16 +69358,16 @@
         </is>
       </c>
       <c r="B3447" t="n">
-        <v>3476</v>
+        <v>3468</v>
       </c>
       <c r="C3447" t="inlineStr">
         <is>
-          <t xml:space="preserve"> FRANCISCA LEIDIANE M. MENDES NASCIMENTO</t>
+          <t>KAWA ALMEIDA CAMPOS</t>
         </is>
       </c>
       <c r="D3447" t="inlineStr">
         <is>
-          <t>FLEIDIANE</t>
+          <t>KAWA</t>
         </is>
       </c>
     </row>
@@ -69378,76 +69378,76 @@
         </is>
       </c>
       <c r="B3448" t="n">
-        <v>3477</v>
+        <v>3476</v>
       </c>
       <c r="C3448" t="inlineStr">
         <is>
-          <t>MARIA THAIS MARTINS PEREIRA SILVA</t>
+          <t xml:space="preserve"> FRANCISCA LEIDIANE M. MENDES NASCIMENTO</t>
         </is>
       </c>
       <c r="D3448" t="inlineStr">
         <is>
-          <t>MTHAIS</t>
+          <t>FLEIDIANE</t>
         </is>
       </c>
     </row>
     <row r="3449">
       <c r="A3449" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3449" t="n">
-        <v>3271</v>
+        <v>3477</v>
       </c>
       <c r="C3449" t="inlineStr">
         <is>
-          <t>DIEGO DE ARAUJO CALÁBRIA</t>
+          <t>MARIA THAIS MARTINS PEREIRA SILVA</t>
         </is>
       </c>
       <c r="D3449" t="inlineStr">
         <is>
-          <t>ARAUJOC</t>
+          <t>MTHAIS</t>
         </is>
       </c>
     </row>
     <row r="3450">
       <c r="A3450" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3450" t="n">
-        <v>3272</v>
+        <v>3271</v>
       </c>
       <c r="C3450" t="inlineStr">
         <is>
-          <t>ANNE BEATRIZ SILVA VIRGINO</t>
+          <t>DIEGO DE ARAUJO CALÁBRIA</t>
         </is>
       </c>
       <c r="D3450" t="inlineStr">
         <is>
-          <t>ABVIRGINIO</t>
+          <t>ARAUJOC</t>
         </is>
       </c>
     </row>
     <row r="3451">
       <c r="A3451" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3451" t="n">
-        <v>3293</v>
+        <v>3272</v>
       </c>
       <c r="C3451" t="inlineStr">
         <is>
-          <t xml:space="preserve">CARLOS ALBERTO VIRIATO SANTOS </t>
+          <t>ANNE BEATRIZ SILVA VIRGINO</t>
         </is>
       </c>
       <c r="D3451" t="inlineStr">
         <is>
-          <t>CVIRIATO</t>
+          <t>ABVIRGINIO</t>
         </is>
       </c>
     </row>
@@ -69458,16 +69458,16 @@
         </is>
       </c>
       <c r="B3452" t="n">
-        <v>3381</v>
+        <v>3293</v>
       </c>
       <c r="C3452" t="inlineStr">
         <is>
-          <t>ALAN CAIQUE SANTOS E SANTOS</t>
+          <t xml:space="preserve">CARLOS ALBERTO VIRIATO SANTOS </t>
         </is>
       </c>
       <c r="D3452" t="inlineStr">
         <is>
-          <t>ALANSANTOS</t>
+          <t>CVIRIATO</t>
         </is>
       </c>
     </row>
@@ -69478,116 +69478,116 @@
         </is>
       </c>
       <c r="B3453" t="n">
-        <v>3443</v>
+        <v>3381</v>
       </c>
       <c r="C3453" t="inlineStr">
         <is>
-          <t>SANON MOREIRA SOUZA</t>
+          <t>ALAN CAIQUE SANTOS E SANTOS</t>
         </is>
       </c>
       <c r="D3453" t="inlineStr">
         <is>
-          <t>SANON</t>
+          <t>ALANSANTOS</t>
         </is>
       </c>
     </row>
     <row r="3454">
       <c r="A3454" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3454" t="n">
-        <v>3516</v>
+        <v>3443</v>
       </c>
       <c r="C3454" t="inlineStr">
         <is>
-          <t>FRANCISCO RILDER TELES DE OLIVEIRA</t>
+          <t>SANON MOREIRA SOUZA</t>
         </is>
       </c>
       <c r="D3454" t="inlineStr">
         <is>
-          <t>RILDER</t>
+          <t>SANON</t>
         </is>
       </c>
     </row>
     <row r="3455">
       <c r="A3455" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3455" t="n">
-        <v>3519</v>
+        <v>3516</v>
       </c>
       <c r="C3455" t="inlineStr">
         <is>
-          <t>MARIA LUANA DE ALMEIDA BATISTA</t>
+          <t>FRANCISCO RILDER TELES DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D3455" t="inlineStr">
         <is>
-          <t>M.LUANA</t>
+          <t>RILDER</t>
         </is>
       </c>
     </row>
     <row r="3456">
       <c r="A3456" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3456" t="n">
-        <v>3540</v>
+        <v>3519</v>
       </c>
       <c r="C3456" t="inlineStr">
         <is>
-          <t>HELEN VITORIA OLIVEIRA DA ROCHA</t>
+          <t>MARIA LUANA DE ALMEIDA BATISTA</t>
         </is>
       </c>
       <c r="D3456" t="inlineStr">
         <is>
-          <t>H.VITORIA</t>
+          <t>M.LUANA</t>
         </is>
       </c>
     </row>
     <row r="3457">
       <c r="A3457" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B3457" t="n">
-        <v>3559</v>
+        <v>3540</v>
       </c>
       <c r="C3457" t="inlineStr">
         <is>
-          <t>ARKBERYS TELES DE SOUSA</t>
+          <t>HELEN VITORIA OLIVEIRA DA ROCHA</t>
         </is>
       </c>
       <c r="D3457" t="inlineStr">
         <is>
-          <t>ARKBERYS</t>
+          <t>H.VITORIA</t>
         </is>
       </c>
     </row>
     <row r="3458">
       <c r="A3458" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3458" t="n">
-        <v>3567</v>
+        <v>3559</v>
       </c>
       <c r="C3458" t="inlineStr">
         <is>
-          <t>PEDRO HENRIQUE VIEIRA DE LIMA</t>
+          <t>ARKBERYS TELES DE SOUSA</t>
         </is>
       </c>
       <c r="D3458" t="inlineStr">
         <is>
-          <t>P.LIMA</t>
+          <t>ARKBERYS</t>
         </is>
       </c>
     </row>
@@ -69598,76 +69598,76 @@
         </is>
       </c>
       <c r="B3459" t="n">
-        <v>3331</v>
+        <v>3567</v>
       </c>
       <c r="C3459" t="inlineStr">
         <is>
-          <t>LOUIZE VANIELLE RODRIGUES FARIAS</t>
+          <t>PEDRO HENRIQUE VIEIRA DE LIMA</t>
         </is>
       </c>
       <c r="D3459" t="inlineStr">
         <is>
-          <t>LVFARIAS</t>
+          <t>P.LIMA</t>
         </is>
       </c>
     </row>
     <row r="3460">
       <c r="A3460" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3460" t="n">
-        <v>3334</v>
+        <v>3331</v>
       </c>
       <c r="C3460" t="inlineStr">
         <is>
-          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+          <t>LOUIZE VANIELLE RODRIGUES FARIAS</t>
         </is>
       </c>
       <c r="D3460" t="inlineStr">
         <is>
-          <t>MTGASPAR</t>
+          <t>LVFARIAS</t>
         </is>
       </c>
     </row>
     <row r="3461">
       <c r="A3461" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3461" t="n">
-        <v>3345</v>
+        <v>3334</v>
       </c>
       <c r="C3461" t="inlineStr">
         <is>
-          <t>AURICÉLIA INACIO PEREIRA</t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
       <c r="D3461" t="inlineStr">
         <is>
-          <t>AIPEREIRA</t>
+          <t>MTGASPAR</t>
         </is>
       </c>
     </row>
     <row r="3462">
       <c r="A3462" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3462" t="n">
-        <v>3363</v>
+        <v>3345</v>
       </c>
       <c r="C3462" t="inlineStr">
         <is>
-          <t>IASMIN LEAL ALVES</t>
+          <t>AURICÉLIA INACIO PEREIRA</t>
         </is>
       </c>
       <c r="D3462" t="inlineStr">
         <is>
-          <t>ILALVES</t>
+          <t>AIPEREIRA</t>
         </is>
       </c>
     </row>
@@ -69678,196 +69678,196 @@
         </is>
       </c>
       <c r="B3463" t="n">
-        <v>3370</v>
+        <v>3363</v>
       </c>
       <c r="C3463" t="inlineStr">
         <is>
-          <t>CARLOS DIEGO ARAUJO ALMEIDA</t>
+          <t>IASMIN LEAL ALVES</t>
         </is>
       </c>
       <c r="D3463" t="inlineStr">
         <is>
-          <t>CDIEGO</t>
+          <t>ILALVES</t>
         </is>
       </c>
     </row>
     <row r="3464">
       <c r="A3464" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3464" t="n">
-        <v>3379</v>
+        <v>3370</v>
       </c>
       <c r="C3464" t="inlineStr">
         <is>
-          <t xml:space="preserve">MATHEUS EVANGELISTA FERREIRA </t>
+          <t>CARLOS DIEGO ARAUJO ALMEIDA</t>
         </is>
       </c>
       <c r="D3464" t="inlineStr">
         <is>
-          <t>MMFERREIRA</t>
+          <t>CDIEGO</t>
         </is>
       </c>
     </row>
     <row r="3465">
       <c r="A3465" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3465" t="n">
-        <v>3419</v>
+        <v>3379</v>
       </c>
       <c r="C3465" t="inlineStr">
         <is>
-          <t xml:space="preserve">DAVID EVANGELISTA SILVA </t>
+          <t xml:space="preserve">MATHEUS EVANGELISTA FERREIRA </t>
         </is>
       </c>
       <c r="D3465" t="inlineStr">
         <is>
-          <t>DAVID</t>
+          <t>MMFERREIRA</t>
         </is>
       </c>
     </row>
     <row r="3466">
       <c r="A3466" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3466" t="n">
-        <v>3423</v>
+        <v>3419</v>
       </c>
       <c r="C3466" t="inlineStr">
         <is>
-          <t>MARCIO JOSE TIAGO</t>
+          <t xml:space="preserve">DAVID EVANGELISTA SILVA </t>
         </is>
       </c>
       <c r="D3466" t="inlineStr">
         <is>
-          <t>MJTIAGO</t>
+          <t>DAVID</t>
         </is>
       </c>
     </row>
     <row r="3467">
       <c r="A3467" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3467" t="n">
-        <v>3453</v>
+        <v>3423</v>
       </c>
       <c r="C3467" t="inlineStr">
         <is>
-          <t xml:space="preserve">LAURIENE SILVA BARBOSA </t>
+          <t>MARCIO JOSE TIAGO</t>
         </is>
       </c>
       <c r="D3467" t="inlineStr">
         <is>
-          <t>LAURIENE</t>
+          <t>MJTIAGO</t>
         </is>
       </c>
     </row>
     <row r="3468">
       <c r="A3468" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3468" t="n">
-        <v>3478</v>
+        <v>3453</v>
       </c>
       <c r="C3468" t="inlineStr">
         <is>
-          <t>LEANDRO BRITO NOGUEIRA DE OLIVEIRA</t>
+          <t xml:space="preserve">LAURIENE SILVA BARBOSA </t>
         </is>
       </c>
       <c r="D3468" t="inlineStr">
         <is>
-          <t>LBNOGUEIRA</t>
+          <t>LAURIENE</t>
         </is>
       </c>
     </row>
     <row r="3469">
       <c r="A3469" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3469" t="n">
-        <v>3479</v>
+        <v>3478</v>
       </c>
       <c r="C3469" t="inlineStr">
         <is>
-          <t>ESDRAS ALESSANDRO SANTOS SANTANA</t>
+          <t>LEANDRO BRITO NOGUEIRA DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D3469" t="inlineStr">
         <is>
-          <t>EALESSANDRO</t>
+          <t>LBNOGUEIRA</t>
         </is>
       </c>
     </row>
     <row r="3470">
       <c r="A3470" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3470" t="n">
-        <v>3480</v>
+        <v>3479</v>
       </c>
       <c r="C3470" t="inlineStr">
         <is>
-          <t xml:space="preserve">LUCIMARA SOUSA LIMA </t>
+          <t>ESDRAS ALESSANDRO SANTOS SANTANA</t>
         </is>
       </c>
       <c r="D3470" t="inlineStr">
         <is>
-          <t>LUCIMARA</t>
+          <t>EALESSANDRO</t>
         </is>
       </c>
     </row>
     <row r="3471">
       <c r="A3471" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3471" t="n">
-        <v>3482</v>
+        <v>3480</v>
       </c>
       <c r="C3471" t="inlineStr">
         <is>
-          <t>DANIEL FERNANDES DINIZ HERACLIO</t>
+          <t xml:space="preserve">LUCIMARA SOUSA LIMA </t>
         </is>
       </c>
       <c r="D3471" t="inlineStr">
         <is>
-          <t>DFDINIZ</t>
+          <t>LUCIMARA</t>
         </is>
       </c>
     </row>
     <row r="3472">
       <c r="A3472" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3472" t="n">
-        <v>3518</v>
+        <v>3482</v>
       </c>
       <c r="C3472" t="inlineStr">
         <is>
-          <t>RAMYRA ALVES FELIX DA SILVA</t>
+          <t>DANIEL FERNANDES DINIZ HERACLIO</t>
         </is>
       </c>
       <c r="D3472" t="inlineStr">
         <is>
-          <t>RFELIX</t>
+          <t>DFDINIZ</t>
         </is>
       </c>
     </row>
@@ -69878,36 +69878,36 @@
         </is>
       </c>
       <c r="B3473" t="n">
-        <v>3534</v>
+        <v>3518</v>
       </c>
       <c r="C3473" t="inlineStr">
         <is>
-          <t xml:space="preserve">CAIO DE SOUZA VINHAS </t>
+          <t>RAMYRA ALVES FELIX DA SILVA</t>
         </is>
       </c>
       <c r="D3473" t="inlineStr">
         <is>
-          <t>CVINHAS</t>
+          <t>RFELIX</t>
         </is>
       </c>
     </row>
     <row r="3474">
       <c r="A3474" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3474" t="n">
-        <v>3535</v>
+        <v>3534</v>
       </c>
       <c r="C3474" t="inlineStr">
         <is>
-          <t>ROMARIO DE SOUSA SILVA</t>
+          <t xml:space="preserve">CAIO DE SOUZA VINHAS </t>
         </is>
       </c>
       <c r="D3474" t="inlineStr">
         <is>
-          <t>RSOUSAS</t>
+          <t>CVINHAS</t>
         </is>
       </c>
     </row>
@@ -69918,56 +69918,56 @@
         </is>
       </c>
       <c r="B3475" t="n">
-        <v>3536</v>
+        <v>3535</v>
       </c>
       <c r="C3475" t="inlineStr">
         <is>
-          <t>JHONATAS CARVALHO OLIVEIRA</t>
+          <t>ROMARIO DE SOUSA SILVA</t>
         </is>
       </c>
       <c r="D3475" t="inlineStr">
         <is>
-          <t>JHONATASC</t>
+          <t>RSOUSAS</t>
         </is>
       </c>
     </row>
     <row r="3476">
       <c r="A3476" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3476" t="n">
-        <v>940529</v>
+        <v>3536</v>
       </c>
       <c r="C3476" t="inlineStr">
         <is>
-          <t>EDGAR FELIX - FL9</t>
+          <t>JHONATAS CARVALHO OLIVEIRA</t>
         </is>
       </c>
       <c r="D3476" t="inlineStr">
         <is>
-          <t>EDGAR F</t>
+          <t>JHONATASC</t>
         </is>
       </c>
     </row>
     <row r="3477">
       <c r="A3477" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3477" t="n">
-        <v>3304</v>
+        <v>940529</v>
       </c>
       <c r="C3477" t="inlineStr">
         <is>
-          <t>JOACI GUILHERME GONÇALVES DA LUZ</t>
+          <t>EDGAR FELIX - FL9</t>
         </is>
       </c>
       <c r="D3477" t="inlineStr">
         <is>
-          <t>JLUZ</t>
+          <t>EDGAR F</t>
         </is>
       </c>
     </row>
@@ -69978,16 +69978,16 @@
         </is>
       </c>
       <c r="B3478" t="n">
-        <v>3305</v>
+        <v>3304</v>
       </c>
       <c r="C3478" t="inlineStr">
         <is>
-          <t>JOÃO VITOR DE ARAÚJO GONÇALVES</t>
+          <t>JOACI GUILHERME GONÇALVES DA LUZ</t>
         </is>
       </c>
       <c r="D3478" t="inlineStr">
         <is>
-          <t>JJVITOR</t>
+          <t>JLUZ</t>
         </is>
       </c>
     </row>
@@ -69998,36 +69998,36 @@
         </is>
       </c>
       <c r="B3479" t="n">
-        <v>3306</v>
+        <v>3305</v>
       </c>
       <c r="C3479" t="inlineStr">
         <is>
-          <t>WENDERSON MARCOS DOS SANTOS</t>
+          <t>JOÃO VITOR DE ARAÚJO GONÇALVES</t>
         </is>
       </c>
       <c r="D3479" t="inlineStr">
         <is>
-          <t>WWMARCOS</t>
+          <t>JJVITOR</t>
         </is>
       </c>
     </row>
     <row r="3480">
       <c r="A3480" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3480" t="n">
-        <v>3335</v>
+        <v>3306</v>
       </c>
       <c r="C3480" t="inlineStr">
         <is>
-          <t>EDILBERTO LEMOS DE LIMA</t>
+          <t>WENDERSON MARCOS DOS SANTOS</t>
         </is>
       </c>
       <c r="D3480" t="inlineStr">
         <is>
-          <t>ELEMOS</t>
+          <t>WWMARCOS</t>
         </is>
       </c>
     </row>
@@ -70038,136 +70038,136 @@
         </is>
       </c>
       <c r="B3481" t="n">
-        <v>3336</v>
+        <v>3335</v>
       </c>
       <c r="C3481" t="inlineStr">
         <is>
-          <t>EZEQUIEL SOUZA DO NASCIMENTO</t>
+          <t>EDILBERTO LEMOS DE LIMA</t>
         </is>
       </c>
       <c r="D3481" t="inlineStr">
         <is>
-          <t>ESNASCIMENTO</t>
+          <t>ELEMOS</t>
         </is>
       </c>
     </row>
     <row r="3482">
       <c r="A3482" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3482" t="n">
-        <v>3341</v>
+        <v>3336</v>
       </c>
       <c r="C3482" t="inlineStr">
         <is>
-          <t>ALCIONE MARIANO DE OLIVEIRA</t>
+          <t>EZEQUIEL SOUZA DO NASCIMENTO</t>
         </is>
       </c>
       <c r="D3482" t="inlineStr">
         <is>
-          <t>AMOLIVEIRA</t>
+          <t>ESNASCIMENTO</t>
         </is>
       </c>
     </row>
     <row r="3483">
       <c r="A3483" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3483" t="n">
-        <v>3401</v>
+        <v>3341</v>
       </c>
       <c r="C3483" t="inlineStr">
         <is>
-          <t xml:space="preserve">TULIO HENRIQUE DA SILVA CARVALHO </t>
+          <t>ALCIONE MARIANO DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D3483" t="inlineStr">
         <is>
-          <t>TULIO</t>
+          <t>AMOLIVEIRA</t>
         </is>
       </c>
     </row>
     <row r="3484">
       <c r="A3484" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3484" t="n">
-        <v>3411</v>
+        <v>3401</v>
       </c>
       <c r="C3484" t="inlineStr">
         <is>
-          <t>CONEXAO RUBYA DANILLA</t>
+          <t xml:space="preserve">TULIO HENRIQUE DA SILVA CARVALHO </t>
         </is>
       </c>
       <c r="D3484" t="inlineStr">
         <is>
-          <t>CONEXAORUBYA</t>
+          <t>TULIO</t>
         </is>
       </c>
     </row>
     <row r="3485">
       <c r="A3485" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3485" t="n">
-        <v>3412</v>
+        <v>3411</v>
       </c>
       <c r="C3485" t="inlineStr">
         <is>
-          <t>CONEXAO RAFAEL</t>
+          <t>CONEXAO RUBYA DANILLA</t>
         </is>
       </c>
       <c r="D3485" t="inlineStr">
         <is>
-          <t>CONEXAORAFAEL</t>
+          <t>CONEXAORUBYA</t>
         </is>
       </c>
     </row>
     <row r="3486">
       <c r="A3486" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3486" t="n">
-        <v>3558</v>
+        <v>3412</v>
       </c>
       <c r="C3486" t="inlineStr">
         <is>
-          <t>WALLYS QUEIROZ VIANA</t>
+          <t>CONEXAO RAFAEL</t>
         </is>
       </c>
       <c r="D3486" t="inlineStr">
         <is>
-          <t>WALLYS</t>
+          <t>CONEXAORAFAEL</t>
         </is>
       </c>
     </row>
     <row r="3487">
       <c r="A3487" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3487" t="n">
-        <v>3264</v>
+        <v>3558</v>
       </c>
       <c r="C3487" t="inlineStr">
         <is>
-          <t xml:space="preserve">WILTON CARLOS MACIEL DE ASSIS </t>
+          <t>WALLYS QUEIROZ VIANA</t>
         </is>
       </c>
       <c r="D3487" t="inlineStr">
         <is>
-          <t>WCMACIEL</t>
+          <t>WALLYS</t>
         </is>
       </c>
     </row>
@@ -70178,56 +70178,56 @@
         </is>
       </c>
       <c r="B3488" t="n">
-        <v>3340</v>
+        <v>3264</v>
       </c>
       <c r="C3488" t="inlineStr">
         <is>
-          <t>ROGELENO FARIAS FEIJÃO FILHO</t>
+          <t xml:space="preserve">WILTON CARLOS MACIEL DE ASSIS </t>
         </is>
       </c>
       <c r="D3488" t="inlineStr">
         <is>
-          <t>RFEIJAO</t>
+          <t>WCMACIEL</t>
         </is>
       </c>
     </row>
     <row r="3489">
       <c r="A3489" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3489" t="n">
-        <v>940550</v>
+        <v>3340</v>
       </c>
       <c r="C3489" t="inlineStr">
         <is>
-          <t>RAFAELE RIBEIRO CARNEIRO</t>
+          <t>ROGELENO FARIAS FEIJÃO FILHO</t>
         </is>
       </c>
       <c r="D3489" t="inlineStr">
         <is>
-          <t>RAFAELE</t>
+          <t>RFEIJAO</t>
         </is>
       </c>
     </row>
     <row r="3490">
       <c r="A3490" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>99</t>
         </is>
       </c>
       <c r="B3490" t="n">
-        <v>3377</v>
+        <v>940550</v>
       </c>
       <c r="C3490" t="inlineStr">
         <is>
-          <t xml:space="preserve"> ISALTINO BISPO DE OLIVEIRA JUNIOR</t>
+          <t>RAFAELE RIBEIRO CARNEIRO</t>
         </is>
       </c>
       <c r="D3490" t="inlineStr">
         <is>
-          <t>BJUNIOR</t>
+          <t>RAFAELE</t>
         </is>
       </c>
     </row>
@@ -70238,56 +70238,56 @@
         </is>
       </c>
       <c r="B3491" t="n">
-        <v>3425</v>
+        <v>3377</v>
       </c>
       <c r="C3491" t="inlineStr">
         <is>
-          <t xml:space="preserve"> CIRLANE ARAUJO SOUZA </t>
+          <t xml:space="preserve"> ISALTINO BISPO DE OLIVEIRA JUNIOR</t>
         </is>
       </c>
       <c r="D3491" t="inlineStr">
         <is>
-          <t>CIRLANES</t>
+          <t>BJUNIOR</t>
         </is>
       </c>
     </row>
     <row r="3492">
       <c r="A3492" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3492" t="n">
-        <v>3454</v>
+        <v>3425</v>
       </c>
       <c r="C3492" t="inlineStr">
         <is>
-          <t>ANTONIA SAMARA DE SOUZA SOARES</t>
+          <t xml:space="preserve"> CIRLANE ARAUJO SOUZA </t>
         </is>
       </c>
       <c r="D3492" t="inlineStr">
         <is>
-          <t>ANTSAMARA</t>
+          <t>CIRLANES</t>
         </is>
       </c>
     </row>
     <row r="3493">
       <c r="A3493" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3493" t="n">
-        <v>3491</v>
+        <v>3454</v>
       </c>
       <c r="C3493" t="inlineStr">
         <is>
-          <t>PEDRO JOSE DO NASCIMENTO NETO</t>
+          <t>ANTONIA SAMARA DE SOUZA SOARES</t>
         </is>
       </c>
       <c r="D3493" t="inlineStr">
         <is>
-          <t>P.JOSE</t>
+          <t>ANTSAMARA</t>
         </is>
       </c>
     </row>
@@ -70298,36 +70298,36 @@
         </is>
       </c>
       <c r="B3494" t="n">
-        <v>3492</v>
+        <v>3491</v>
       </c>
       <c r="C3494" t="inlineStr">
         <is>
-          <t>PAULA CARLA CALDAS MOTA</t>
+          <t>PEDRO JOSE DO NASCIMENTO NETO</t>
         </is>
       </c>
       <c r="D3494" t="inlineStr">
         <is>
-          <t>P.CARLA</t>
+          <t>P.JOSE</t>
         </is>
       </c>
     </row>
     <row r="3495">
       <c r="A3495" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3495" t="n">
-        <v>3542</v>
+        <v>3492</v>
       </c>
       <c r="C3495" t="inlineStr">
         <is>
-          <t>ANTONIA MILENA SOUSA ANDRADE</t>
+          <t>PAULA CARLA CALDAS MOTA</t>
         </is>
       </c>
       <c r="D3495" t="inlineStr">
         <is>
-          <t>A.MILENA</t>
+          <t>P.CARLA</t>
         </is>
       </c>
     </row>
@@ -70338,56 +70338,56 @@
         </is>
       </c>
       <c r="B3496" t="n">
-        <v>3547</v>
+        <v>3542</v>
       </c>
       <c r="C3496" t="inlineStr">
         <is>
-          <t xml:space="preserve">DAVI PEREIRA DA SILVA </t>
+          <t>ANTONIA MILENA SOUSA ANDRADE</t>
         </is>
       </c>
       <c r="D3496" t="inlineStr">
         <is>
-          <t>DPSILVA</t>
+          <t>A.MILENA</t>
         </is>
       </c>
     </row>
     <row r="3497">
       <c r="A3497" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3497" t="n">
-        <v>3552</v>
+        <v>3547</v>
       </c>
       <c r="C3497" t="inlineStr">
         <is>
-          <t>PAULO SERGIO MENDES DE OLIVEIRA</t>
+          <t xml:space="preserve">DAVI PEREIRA DA SILVA </t>
         </is>
       </c>
       <c r="D3497" t="inlineStr">
         <is>
-          <t>PSMENDES</t>
+          <t>DPSILVA</t>
         </is>
       </c>
     </row>
     <row r="3498">
       <c r="A3498" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3498" t="n">
-        <v>3294</v>
+        <v>3552</v>
       </c>
       <c r="C3498" t="inlineStr">
         <is>
-          <t>GLEICIANE MIRANDA DE MORAIS</t>
+          <t>PAULO SERGIO MENDES DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D3498" t="inlineStr">
         <is>
-          <t>GMIRANDA</t>
+          <t>PSMENDES</t>
         </is>
       </c>
     </row>
@@ -70398,176 +70398,176 @@
         </is>
       </c>
       <c r="B3499" t="n">
-        <v>3295</v>
+        <v>3294</v>
       </c>
       <c r="C3499" t="inlineStr">
         <is>
-          <t>MARIA ESTEFANNY DA SILVA MOURA</t>
+          <t>GLEICIANE MIRANDA DE MORAIS</t>
         </is>
       </c>
       <c r="D3499" t="inlineStr">
         <is>
-          <t>MESTEFANNY</t>
+          <t>GMIRANDA</t>
         </is>
       </c>
     </row>
     <row r="3500">
       <c r="A3500" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3500" t="n">
-        <v>3296</v>
+        <v>3295</v>
       </c>
       <c r="C3500" t="inlineStr">
         <is>
-          <t>PEDRO IAGO FONSECA EVANGELISTA</t>
+          <t>MARIA ESTEFANNY DA SILVA MOURA</t>
         </is>
       </c>
       <c r="D3500" t="inlineStr">
         <is>
-          <t>PIFONSECA</t>
+          <t>MESTEFANNY</t>
         </is>
       </c>
     </row>
     <row r="3501">
       <c r="A3501" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3501" t="n">
-        <v>940544</v>
+        <v>3296</v>
       </c>
       <c r="C3501" t="inlineStr">
         <is>
-          <t>LUTY LOG TRANSPORTES - FL8</t>
+          <t>PEDRO IAGO FONSECA EVANGELISTA</t>
         </is>
       </c>
       <c r="D3501" t="inlineStr">
         <is>
-          <t>LUTY LOG</t>
+          <t>PIFONSECA</t>
         </is>
       </c>
     </row>
     <row r="3502">
       <c r="A3502" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B3502" t="n">
-        <v>3380</v>
+        <v>940544</v>
       </c>
       <c r="C3502" t="inlineStr">
         <is>
-          <t>FRANCISCO MATHEUS RABELO DA COSTA</t>
+          <t>LUTY LOG TRANSPORTES - FL8</t>
         </is>
       </c>
       <c r="D3502" t="inlineStr">
         <is>
-          <t>FMATHEUS</t>
+          <t>LUTY LOG</t>
         </is>
       </c>
     </row>
     <row r="3503">
       <c r="A3503" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3503" t="n">
-        <v>3410</v>
+        <v>3380</v>
       </c>
       <c r="C3503" t="inlineStr">
         <is>
-          <t xml:space="preserve"> BRENO ALLAN DE JESUS</t>
+          <t>FRANCISCO MATHEUS RABELO DA COSTA</t>
         </is>
       </c>
       <c r="D3503" t="inlineStr">
         <is>
-          <t>JESUS</t>
+          <t>FMATHEUS</t>
         </is>
       </c>
     </row>
     <row r="3504">
       <c r="A3504" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3504" t="n">
-        <v>3444</v>
+        <v>3410</v>
       </c>
       <c r="C3504" t="inlineStr">
         <is>
-          <t>THIAGO COSTA SILVA</t>
+          <t xml:space="preserve"> BRENO ALLAN DE JESUS</t>
         </is>
       </c>
       <c r="D3504" t="inlineStr">
         <is>
-          <t>THIAGOC</t>
+          <t>JESUS</t>
         </is>
       </c>
     </row>
     <row r="3505">
       <c r="A3505" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3505" t="n">
-        <v>3456</v>
+        <v>3444</v>
       </c>
       <c r="C3505" t="inlineStr">
         <is>
-          <t>FELIPE BOTH MAZUCHINI</t>
+          <t>THIAGO COSTA SILVA</t>
         </is>
       </c>
       <c r="D3505" t="inlineStr">
         <is>
-          <t>FELIPEB</t>
+          <t>THIAGOC</t>
         </is>
       </c>
     </row>
     <row r="3506">
       <c r="A3506" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3506" t="n">
-        <v>3457</v>
+        <v>3456</v>
       </c>
       <c r="C3506" t="inlineStr">
         <is>
-          <t>FRANKLIN VIEIRA GOMES</t>
+          <t>FELIPE BOTH MAZUCHINI</t>
         </is>
       </c>
       <c r="D3506" t="inlineStr">
         <is>
-          <t>VIEIRAF</t>
+          <t>FELIPEB</t>
         </is>
       </c>
     </row>
     <row r="3507">
       <c r="A3507" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3507" t="n">
-        <v>3507</v>
+        <v>3457</v>
       </c>
       <c r="C3507" t="inlineStr">
         <is>
-          <t>KARINE TEODORA ALVES DE OLIVEIRA</t>
+          <t>FRANKLIN VIEIRA GOMES</t>
         </is>
       </c>
       <c r="D3507" t="inlineStr">
         <is>
-          <t>KOLIVEIRA</t>
+          <t>VIEIRAF</t>
         </is>
       </c>
     </row>
@@ -70578,14 +70578,34 @@
         </is>
       </c>
       <c r="B3508" t="n">
+        <v>3507</v>
+      </c>
+      <c r="C3508" t="inlineStr">
+        <is>
+          <t>KARINE TEODORA ALVES DE OLIVEIRA</t>
+        </is>
+      </c>
+      <c r="D3508" t="inlineStr">
+        <is>
+          <t>KOLIVEIRA</t>
+        </is>
+      </c>
+    </row>
+    <row r="3509">
+      <c r="A3509" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B3509" t="n">
         <v>3520</v>
       </c>
-      <c r="C3508" t="inlineStr">
+      <c r="C3509" t="inlineStr">
         <is>
           <t xml:space="preserve"> EMERSON FILIPE MELO DE AGUIAR</t>
         </is>
       </c>
-      <c r="D3508" t="inlineStr">
+      <c r="D3509" t="inlineStr">
         <is>
           <t>E.FILIPE</t>
         </is>

</xml_diff>

<commit_message>
chore(data): batch update intraday televendas - 08:02:45
</commit_message>
<xml_diff>
--- a/data/dim_televendas.xlsx
+++ b/data/dim_televendas.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3511"/>
+  <dimension ref="A1:D3514"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -68614,80 +68614,80 @@
     <row r="3410">
       <c r="A3410" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9999</t>
         </is>
       </c>
       <c r="B3410" t="n">
-        <v>940525</v>
+        <v>3602</v>
       </c>
       <c r="C3410" t="inlineStr">
         <is>
-          <t>SANDUWELLINGTON</t>
+          <t>NEGOCIACOES CE</t>
         </is>
       </c>
       <c r="D3410" t="inlineStr">
         <is>
-          <t>SANDUWELLINGTON</t>
+          <t>NEGOCIACAOCE</t>
         </is>
       </c>
     </row>
     <row r="3411">
       <c r="A3411" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9999</t>
         </is>
       </c>
       <c r="B3411" t="n">
-        <v>3369</v>
+        <v>3603</v>
       </c>
       <c r="C3411" t="inlineStr">
         <is>
-          <t xml:space="preserve">PRISCILA DOS SANTOS LOPES </t>
+          <t>NEGOCIACAO PE</t>
         </is>
       </c>
       <c r="D3411" t="inlineStr">
         <is>
-          <t>PSLOPES</t>
+          <t>NEGOCIACAOPE</t>
         </is>
       </c>
     </row>
     <row r="3412">
       <c r="A3412" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>9999</t>
         </is>
       </c>
       <c r="B3412" t="n">
-        <v>3433</v>
+        <v>3604</v>
       </c>
       <c r="C3412" t="inlineStr">
         <is>
-          <t>BRUNO NUNES CRUZ</t>
+          <t>NEGOCIACAO BA</t>
         </is>
       </c>
       <c r="D3412" t="inlineStr">
         <is>
-          <t>BRUNOCRUZ</t>
+          <t>NEGOCIACAOBA</t>
         </is>
       </c>
     </row>
     <row r="3413">
       <c r="A3413" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3413" t="n">
-        <v>3434</v>
+        <v>940525</v>
       </c>
       <c r="C3413" t="inlineStr">
         <is>
-          <t>ANA TERCIA DE LIMA SA CARVALHO SERAFIM</t>
+          <t>SANDUWELLINGTON</t>
         </is>
       </c>
       <c r="D3413" t="inlineStr">
         <is>
-          <t>ANATER</t>
+          <t>SANDUWELLINGTON</t>
         </is>
       </c>
     </row>
@@ -68698,216 +68698,216 @@
         </is>
       </c>
       <c r="B3414" t="n">
-        <v>3502</v>
+        <v>3369</v>
       </c>
       <c r="C3414" t="inlineStr">
         <is>
-          <t>LUIZ FELIPE MACHADO BARRETO</t>
+          <t xml:space="preserve">PRISCILA DOS SANTOS LOPES </t>
         </is>
       </c>
       <c r="D3414" t="inlineStr">
         <is>
-          <t>LUIZ.FELIPE</t>
+          <t>PSLOPES</t>
         </is>
       </c>
     </row>
     <row r="3415">
       <c r="A3415" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3415" t="n">
-        <v>3503</v>
+        <v>3433</v>
       </c>
       <c r="C3415" t="inlineStr">
         <is>
-          <t>FABIO OLIVEIRA SILVA</t>
+          <t>BRUNO NUNES CRUZ</t>
         </is>
       </c>
       <c r="D3415" t="inlineStr">
         <is>
-          <t>FOSILVA</t>
+          <t>BRUNOCRUZ</t>
         </is>
       </c>
     </row>
     <row r="3416">
       <c r="A3416" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3416" t="n">
-        <v>3554</v>
+        <v>3434</v>
       </c>
       <c r="C3416" t="inlineStr">
         <is>
-          <t xml:space="preserve">MANOEL RIBEIRO DE SOUZA JUNIOR </t>
+          <t>ANA TERCIA DE LIMA SA CARVALHO SERAFIM</t>
         </is>
       </c>
       <c r="D3416" t="inlineStr">
         <is>
-          <t>MRJUNIOR</t>
+          <t>ANATER</t>
         </is>
       </c>
     </row>
     <row r="3417">
       <c r="A3417" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3417" t="n">
-        <v>3568</v>
+        <v>3502</v>
       </c>
       <c r="C3417" t="inlineStr">
         <is>
-          <t xml:space="preserve">ANGELICA TORRES DA SILVA </t>
+          <t>LUIZ FELIPE MACHADO BARRETO</t>
         </is>
       </c>
       <c r="D3417" t="inlineStr">
         <is>
-          <t>ANGEL.TORRES</t>
+          <t>LUIZ.FELIPE</t>
         </is>
       </c>
     </row>
     <row r="3418">
       <c r="A3418" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3418" t="n">
-        <v>3569</v>
+        <v>3503</v>
       </c>
       <c r="C3418" t="inlineStr">
         <is>
-          <t>LORENA DE LIMA MATOS</t>
+          <t>FABIO OLIVEIRA SILVA</t>
         </is>
       </c>
       <c r="D3418" t="inlineStr">
         <is>
-          <t>LORE.LIMA</t>
+          <t>FOSILVA</t>
         </is>
       </c>
     </row>
     <row r="3419">
       <c r="A3419" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3419" t="n">
-        <v>3576</v>
+        <v>3554</v>
       </c>
       <c r="C3419" t="inlineStr">
         <is>
-          <t>ANA BEATRIZ PARENTE CAVALCANTE</t>
+          <t xml:space="preserve">MANOEL RIBEIRO DE SOUZA JUNIOR </t>
         </is>
       </c>
       <c r="D3419" t="inlineStr">
         <is>
-          <t>A.BEATRIZ</t>
+          <t>MRJUNIOR</t>
         </is>
       </c>
     </row>
     <row r="3420">
       <c r="A3420" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3420" t="n">
-        <v>940549</v>
+        <v>3568</v>
       </c>
       <c r="C3420" t="inlineStr">
         <is>
-          <t>EDILSON ARAUJO - FL9</t>
+          <t xml:space="preserve">ANGELICA TORRES DA SILVA </t>
         </is>
       </c>
       <c r="D3420" t="inlineStr">
         <is>
-          <t>EDILSON</t>
+          <t>ANGEL.TORRES</t>
         </is>
       </c>
     </row>
     <row r="3421">
       <c r="A3421" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3421" t="n">
-        <v>3470</v>
+        <v>3569</v>
       </c>
       <c r="C3421" t="inlineStr">
         <is>
-          <t>DEBORA ALVES CARVALHO</t>
+          <t>LORENA DE LIMA MATOS</t>
         </is>
       </c>
       <c r="D3421" t="inlineStr">
         <is>
-          <t>DEBORA.ALVES</t>
+          <t>LORE.LIMA</t>
         </is>
       </c>
     </row>
     <row r="3422">
       <c r="A3422" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3422" t="n">
-        <v>3510</v>
+        <v>3576</v>
       </c>
       <c r="C3422" t="inlineStr">
         <is>
-          <t>CAMILA RODIGUES PINTO</t>
+          <t>ANA BEATRIZ PARENTE CAVALCANTE</t>
         </is>
       </c>
       <c r="D3422" t="inlineStr">
         <is>
-          <t>MILA.PINTO</t>
+          <t>A.BEATRIZ</t>
         </is>
       </c>
     </row>
     <row r="3423">
       <c r="A3423" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3423" t="n">
-        <v>3511</v>
+        <v>940549</v>
       </c>
       <c r="C3423" t="inlineStr">
         <is>
-          <t>JORGE HENRIQUE DOS SANTOS RODRIGUES</t>
+          <t>EDILSON ARAUJO - FL9</t>
         </is>
       </c>
       <c r="D3423" t="inlineStr">
         <is>
-          <t>J.HENRIQUE</t>
+          <t>EDILSON</t>
         </is>
       </c>
     </row>
     <row r="3424">
       <c r="A3424" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3424" t="n">
-        <v>3561</v>
+        <v>3470</v>
       </c>
       <c r="C3424" t="inlineStr">
         <is>
-          <t>RONARIA PATRICIA VILARINDO DE ALMEIDA</t>
+          <t>DEBORA ALVES CARVALHO</t>
         </is>
       </c>
       <c r="D3424" t="inlineStr">
         <is>
-          <t>RPATRICIA</t>
+          <t>DEBORA.ALVES</t>
         </is>
       </c>
     </row>
@@ -68918,76 +68918,76 @@
         </is>
       </c>
       <c r="B3425" t="n">
-        <v>3562</v>
+        <v>3510</v>
       </c>
       <c r="C3425" t="inlineStr">
         <is>
-          <t>LETICIA MARIA BENTO NOGUEIRA</t>
+          <t>CAMILA RODIGUES PINTO</t>
         </is>
       </c>
       <c r="D3425" t="inlineStr">
         <is>
-          <t>LBENTO</t>
+          <t>MILA.PINTO</t>
         </is>
       </c>
     </row>
     <row r="3426">
       <c r="A3426" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3426" t="n">
-        <v>3270</v>
+        <v>3511</v>
       </c>
       <c r="C3426" t="inlineStr">
         <is>
-          <t>ITANA NASCIMENTO SIMOES</t>
+          <t>JORGE HENRIQUE DOS SANTOS RODRIGUES</t>
         </is>
       </c>
       <c r="D3426" t="inlineStr">
         <is>
-          <t>ISIMOES</t>
+          <t>J.HENRIQUE</t>
         </is>
       </c>
     </row>
     <row r="3427">
       <c r="A3427" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3427" t="n">
-        <v>3318</v>
+        <v>3561</v>
       </c>
       <c r="C3427" t="inlineStr">
         <is>
-          <t>LUAN MONTEIRO COSTA</t>
+          <t>RONARIA PATRICIA VILARINDO DE ALMEIDA</t>
         </is>
       </c>
       <c r="D3427" t="inlineStr">
         <is>
-          <t>LMONTEIRO</t>
+          <t>RPATRICIA</t>
         </is>
       </c>
     </row>
     <row r="3428">
       <c r="A3428" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3428" t="n">
-        <v>3319</v>
+        <v>3562</v>
       </c>
       <c r="C3428" t="inlineStr">
         <is>
-          <t>MARIANA MACEDA DOS SANTOS</t>
+          <t>LETICIA MARIA BENTO NOGUEIRA</t>
         </is>
       </c>
       <c r="D3428" t="inlineStr">
         <is>
-          <t>MMACEDA</t>
+          <t>LBENTO</t>
         </is>
       </c>
     </row>
@@ -68998,96 +68998,96 @@
         </is>
       </c>
       <c r="B3429" t="n">
-        <v>3389</v>
+        <v>3270</v>
       </c>
       <c r="C3429" t="inlineStr">
         <is>
-          <t>TAMILES DE SANTANA AMORIM BISPO</t>
+          <t>ITANA NASCIMENTO SIMOES</t>
         </is>
       </c>
       <c r="D3429" t="inlineStr">
         <is>
-          <t>TAMILES</t>
+          <t>ISIMOES</t>
         </is>
       </c>
     </row>
     <row r="3430">
       <c r="A3430" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3430" t="n">
-        <v>3390</v>
+        <v>3318</v>
       </c>
       <c r="C3430" t="inlineStr">
         <is>
-          <t>IRACEMA DE ALMEIDA MOURA</t>
+          <t>LUAN MONTEIRO COSTA</t>
         </is>
       </c>
       <c r="D3430" t="inlineStr">
         <is>
-          <t>IRACEMA</t>
+          <t>LMONTEIRO</t>
         </is>
       </c>
     </row>
     <row r="3431">
       <c r="A3431" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3431" t="n">
-        <v>3575</v>
+        <v>3319</v>
       </c>
       <c r="C3431" t="inlineStr">
         <is>
-          <t>SAMARA ALVES DA SILVA</t>
+          <t>MARIANA MACEDA DOS SANTOS</t>
         </is>
       </c>
       <c r="D3431" t="inlineStr">
         <is>
-          <t>S.ALVES</t>
+          <t>MMACEDA</t>
         </is>
       </c>
     </row>
     <row r="3432">
       <c r="A3432" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3432" t="n">
-        <v>3583</v>
+        <v>3389</v>
       </c>
       <c r="C3432" t="inlineStr">
         <is>
-          <t>TALLIS GUTTEMBERG GUIMARES BATISTA</t>
+          <t>TAMILES DE SANTANA AMORIM BISPO</t>
         </is>
       </c>
       <c r="D3432" t="inlineStr">
         <is>
-          <t>TALLIS16</t>
+          <t>TAMILES</t>
         </is>
       </c>
     </row>
     <row r="3433">
       <c r="A3433" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3433" t="n">
-        <v>3286</v>
+        <v>3390</v>
       </c>
       <c r="C3433" t="inlineStr">
         <is>
-          <t>VALERIA MAIA DA SILVA</t>
+          <t>IRACEMA DE ALMEIDA MOURA</t>
         </is>
       </c>
       <c r="D3433" t="inlineStr">
         <is>
-          <t>VMAIAS</t>
+          <t>IRACEMA</t>
         </is>
       </c>
     </row>
@@ -69098,196 +69098,196 @@
         </is>
       </c>
       <c r="B3434" t="n">
-        <v>3287</v>
+        <v>3575</v>
       </c>
       <c r="C3434" t="inlineStr">
         <is>
-          <t>ERIVELTON DA SILVA OLIVEIRA</t>
+          <t>SAMARA ALVES DA SILVA</t>
         </is>
       </c>
       <c r="D3434" t="inlineStr">
         <is>
-          <t>ESOLIVEIRA</t>
+          <t>S.ALVES</t>
         </is>
       </c>
     </row>
     <row r="3435">
       <c r="A3435" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3435" t="n">
-        <v>3307</v>
+        <v>3583</v>
       </c>
       <c r="C3435" t="inlineStr">
         <is>
-          <t>ADRIEL XERES BARROS MARTINS</t>
+          <t>TALLIS GUTTEMBERG GUIMARES BATISTA</t>
         </is>
       </c>
       <c r="D3435" t="inlineStr">
         <is>
-          <t>AXERES</t>
+          <t>TALLIS16</t>
         </is>
       </c>
     </row>
     <row r="3436">
       <c r="A3436" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3436" t="n">
-        <v>3308</v>
+        <v>3286</v>
       </c>
       <c r="C3436" t="inlineStr">
         <is>
-          <t>ELKZIEL JUVINO DA SILVA</t>
+          <t>VALERIA MAIA DA SILVA</t>
         </is>
       </c>
       <c r="D3436" t="inlineStr">
         <is>
-          <t>EJUVINO</t>
+          <t>VMAIAS</t>
         </is>
       </c>
     </row>
     <row r="3437">
       <c r="A3437" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3437" t="n">
-        <v>940539</v>
+        <v>3287</v>
       </c>
       <c r="C3437" t="inlineStr">
         <is>
-          <t>EDSON ARAUJO - FL9</t>
+          <t>ERIVELTON DA SILVA OLIVEIRA</t>
         </is>
       </c>
       <c r="D3437" t="inlineStr">
         <is>
-          <t>EDS</t>
+          <t>ESOLIVEIRA</t>
         </is>
       </c>
     </row>
     <row r="3438">
       <c r="A3438" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3438" t="n">
-        <v>940540</v>
+        <v>3307</v>
       </c>
       <c r="C3438" t="inlineStr">
         <is>
-          <t>EDSON ARAUJO - FL8</t>
+          <t>ADRIEL XERES BARROS MARTINS</t>
         </is>
       </c>
       <c r="D3438" t="inlineStr">
         <is>
-          <t>EDS8</t>
+          <t>AXERES</t>
         </is>
       </c>
     </row>
     <row r="3439">
       <c r="A3439" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3439" t="n">
-        <v>3328</v>
+        <v>3308</v>
       </c>
       <c r="C3439" t="inlineStr">
         <is>
-          <t>ALAN ARAUJO DA SILVA</t>
+          <t>ELKZIEL JUVINO DA SILVA</t>
         </is>
       </c>
       <c r="D3439" t="inlineStr">
         <is>
-          <t>ARSILVA</t>
+          <t>EJUVINO</t>
         </is>
       </c>
     </row>
     <row r="3440">
       <c r="A3440" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3440" t="n">
-        <v>3350</v>
+        <v>940539</v>
       </c>
       <c r="C3440" t="inlineStr">
         <is>
-          <t xml:space="preserve">EDER RODRIGUES DA SILVA </t>
+          <t>EDSON ARAUJO - FL9</t>
         </is>
       </c>
       <c r="D3440" t="inlineStr">
         <is>
-          <t>EDERS</t>
+          <t>EDS</t>
         </is>
       </c>
     </row>
     <row r="3441">
       <c r="A3441" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B3441" t="n">
-        <v>3373</v>
+        <v>940540</v>
       </c>
       <c r="C3441" t="inlineStr">
         <is>
-          <t xml:space="preserve">NATANAEL TAVARES DE SOUSA </t>
+          <t>EDSON ARAUJO - FL8</t>
         </is>
       </c>
       <c r="D3441" t="inlineStr">
         <is>
-          <t>NTSOUSA</t>
+          <t>EDS8</t>
         </is>
       </c>
     </row>
     <row r="3442">
       <c r="A3442" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3442" t="n">
-        <v>3374</v>
+        <v>3328</v>
       </c>
       <c r="C3442" t="inlineStr">
         <is>
-          <t>REINALDO DA SILVA COSTA</t>
+          <t>ALAN ARAUJO DA SILVA</t>
         </is>
       </c>
       <c r="D3442" t="inlineStr">
         <is>
-          <t>RSCOSTA</t>
+          <t>ARSILVA</t>
         </is>
       </c>
     </row>
     <row r="3443">
       <c r="A3443" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3443" t="n">
-        <v>3399</v>
+        <v>3350</v>
       </c>
       <c r="C3443" t="inlineStr">
         <is>
-          <t xml:space="preserve">RICARDO BARBOSA DOS SANTOS </t>
+          <t xml:space="preserve">EDER RODRIGUES DA SILVA </t>
         </is>
       </c>
       <c r="D3443" t="inlineStr">
         <is>
-          <t>RICARDOSAN</t>
+          <t>EDERS</t>
         </is>
       </c>
     </row>
@@ -69298,36 +69298,36 @@
         </is>
       </c>
       <c r="B3444" t="n">
-        <v>3427</v>
+        <v>3373</v>
       </c>
       <c r="C3444" t="inlineStr">
         <is>
-          <t>ROQUE COMERCIO TEMPORARIO</t>
+          <t xml:space="preserve">NATANAEL TAVARES DE SOUSA </t>
         </is>
       </c>
       <c r="D3444" t="inlineStr">
         <is>
-          <t>ROQUECOM</t>
+          <t>NTSOUSA</t>
         </is>
       </c>
     </row>
     <row r="3445">
       <c r="A3445" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3445" t="n">
-        <v>3428</v>
+        <v>3374</v>
       </c>
       <c r="C3445" t="inlineStr">
         <is>
-          <t>ROQUE PLUS TEMPORARIO</t>
+          <t>REINALDO DA SILVA COSTA</t>
         </is>
       </c>
       <c r="D3445" t="inlineStr">
         <is>
-          <t>ROQUEPLUS</t>
+          <t>RSCOSTA</t>
         </is>
       </c>
     </row>
@@ -69338,76 +69338,76 @@
         </is>
       </c>
       <c r="B3446" t="n">
-        <v>3432</v>
+        <v>3399</v>
       </c>
       <c r="C3446" t="inlineStr">
         <is>
-          <t>PATRICIA DOS SANTOS NONATO OLIVEIRA</t>
+          <t xml:space="preserve">RICARDO BARBOSA DOS SANTOS </t>
         </is>
       </c>
       <c r="D3446" t="inlineStr">
         <is>
-          <t>PATRICIAD</t>
+          <t>RICARDOSAN</t>
         </is>
       </c>
     </row>
     <row r="3447">
       <c r="A3447" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3447" t="n">
-        <v>3448</v>
+        <v>3427</v>
       </c>
       <c r="C3447" t="inlineStr">
         <is>
-          <t xml:space="preserve">GABRIEL SOUZA CARVALHO </t>
+          <t>ROQUE COMERCIO TEMPORARIO</t>
         </is>
       </c>
       <c r="D3447" t="inlineStr">
         <is>
-          <t>GABRIEL20</t>
+          <t>ROQUECOM</t>
         </is>
       </c>
     </row>
     <row r="3448">
       <c r="A3448" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3448" t="n">
-        <v>3465</v>
+        <v>3428</v>
       </c>
       <c r="C3448" t="inlineStr">
         <is>
-          <t>LUIZA MARIA BARRETO BARBOSA</t>
+          <t>ROQUE PLUS TEMPORARIO</t>
         </is>
       </c>
       <c r="D3448" t="inlineStr">
         <is>
-          <t>LUIZA.MARIA</t>
+          <t>ROQUEPLUS</t>
         </is>
       </c>
     </row>
     <row r="3449">
       <c r="A3449" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3449" t="n">
-        <v>3468</v>
+        <v>3432</v>
       </c>
       <c r="C3449" t="inlineStr">
         <is>
-          <t>KAWA ALMEIDA CAMPOS</t>
+          <t>PATRICIA DOS SANTOS NONATO OLIVEIRA</t>
         </is>
       </c>
       <c r="D3449" t="inlineStr">
         <is>
-          <t>KAWA</t>
+          <t>PATRICIAD</t>
         </is>
       </c>
     </row>
@@ -69418,276 +69418,276 @@
         </is>
       </c>
       <c r="B3450" t="n">
-        <v>3476</v>
+        <v>3448</v>
       </c>
       <c r="C3450" t="inlineStr">
         <is>
-          <t xml:space="preserve"> FRANCISCA LEIDIANE M. MENDES NASCIMENTO</t>
+          <t xml:space="preserve">GABRIEL SOUZA CARVALHO </t>
         </is>
       </c>
       <c r="D3450" t="inlineStr">
         <is>
-          <t>FLEIDIANE</t>
+          <t>GABRIEL20</t>
         </is>
       </c>
     </row>
     <row r="3451">
       <c r="A3451" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3451" t="n">
-        <v>3477</v>
+        <v>3465</v>
       </c>
       <c r="C3451" t="inlineStr">
         <is>
-          <t>MARIA THAIS MARTINS PEREIRA SILVA</t>
+          <t>LUIZA MARIA BARRETO BARBOSA</t>
         </is>
       </c>
       <c r="D3451" t="inlineStr">
         <is>
-          <t>MTHAIS</t>
+          <t>LUIZA.MARIA</t>
         </is>
       </c>
     </row>
     <row r="3452">
       <c r="A3452" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3452" t="n">
-        <v>3271</v>
+        <v>3468</v>
       </c>
       <c r="C3452" t="inlineStr">
         <is>
-          <t>DIEGO DE ARAUJO CALÁBRIA</t>
+          <t>KAWA ALMEIDA CAMPOS</t>
         </is>
       </c>
       <c r="D3452" t="inlineStr">
         <is>
-          <t>ARAUJOC</t>
+          <t>KAWA</t>
         </is>
       </c>
     </row>
     <row r="3453">
       <c r="A3453" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3453" t="n">
-        <v>3272</v>
+        <v>3476</v>
       </c>
       <c r="C3453" t="inlineStr">
         <is>
-          <t>ANNE BEATRIZ SILVA VIRGINO</t>
+          <t xml:space="preserve"> FRANCISCA LEIDIANE M. MENDES NASCIMENTO</t>
         </is>
       </c>
       <c r="D3453" t="inlineStr">
         <is>
-          <t>ABVIRGINIO</t>
+          <t>FLEIDIANE</t>
         </is>
       </c>
     </row>
     <row r="3454">
       <c r="A3454" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3454" t="n">
-        <v>3293</v>
+        <v>3477</v>
       </c>
       <c r="C3454" t="inlineStr">
         <is>
-          <t xml:space="preserve">CARLOS ALBERTO VIRIATO SANTOS </t>
+          <t>MARIA THAIS MARTINS PEREIRA SILVA</t>
         </is>
       </c>
       <c r="D3454" t="inlineStr">
         <is>
-          <t>CVIRIATO</t>
+          <t>MTHAIS</t>
         </is>
       </c>
     </row>
     <row r="3455">
       <c r="A3455" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3455" t="n">
-        <v>3381</v>
+        <v>3271</v>
       </c>
       <c r="C3455" t="inlineStr">
         <is>
-          <t>ALAN CAIQUE SANTOS E SANTOS</t>
+          <t>DIEGO DE ARAUJO CALÁBRIA</t>
         </is>
       </c>
       <c r="D3455" t="inlineStr">
         <is>
-          <t>ALANSANTOS</t>
+          <t>ARAUJOC</t>
         </is>
       </c>
     </row>
     <row r="3456">
       <c r="A3456" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3456" t="n">
-        <v>3443</v>
+        <v>3272</v>
       </c>
       <c r="C3456" t="inlineStr">
         <is>
-          <t>SANON MOREIRA SOUZA</t>
+          <t>ANNE BEATRIZ SILVA VIRGINO</t>
         </is>
       </c>
       <c r="D3456" t="inlineStr">
         <is>
-          <t>SANON</t>
+          <t>ABVIRGINIO</t>
         </is>
       </c>
     </row>
     <row r="3457">
       <c r="A3457" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3457" t="n">
-        <v>3516</v>
+        <v>3293</v>
       </c>
       <c r="C3457" t="inlineStr">
         <is>
-          <t>FRANCISCO RILDER TELES DE OLIVEIRA</t>
+          <t xml:space="preserve">CARLOS ALBERTO VIRIATO SANTOS </t>
         </is>
       </c>
       <c r="D3457" t="inlineStr">
         <is>
-          <t>RILDER</t>
+          <t>CVIRIATO</t>
         </is>
       </c>
     </row>
     <row r="3458">
       <c r="A3458" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3458" t="n">
-        <v>3519</v>
+        <v>3381</v>
       </c>
       <c r="C3458" t="inlineStr">
         <is>
-          <t>MARIA LUANA DE ALMEIDA BATISTA</t>
+          <t>ALAN CAIQUE SANTOS E SANTOS</t>
         </is>
       </c>
       <c r="D3458" t="inlineStr">
         <is>
-          <t>M.LUANA</t>
+          <t>ALANSANTOS</t>
         </is>
       </c>
     </row>
     <row r="3459">
       <c r="A3459" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3459" t="n">
-        <v>3540</v>
+        <v>3443</v>
       </c>
       <c r="C3459" t="inlineStr">
         <is>
-          <t>HELEN VITORIA OLIVEIRA DA ROCHA</t>
+          <t>SANON MOREIRA SOUZA</t>
         </is>
       </c>
       <c r="D3459" t="inlineStr">
         <is>
-          <t>H.VITORIA</t>
+          <t>SANON</t>
         </is>
       </c>
     </row>
     <row r="3460">
       <c r="A3460" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3460" t="n">
-        <v>3559</v>
+        <v>3516</v>
       </c>
       <c r="C3460" t="inlineStr">
         <is>
-          <t>ARKBERYS TELES DE SOUSA</t>
+          <t>FRANCISCO RILDER TELES DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D3460" t="inlineStr">
         <is>
-          <t>ARKBERYS</t>
+          <t>RILDER</t>
         </is>
       </c>
     </row>
     <row r="3461">
       <c r="A3461" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3461" t="n">
-        <v>3567</v>
+        <v>3519</v>
       </c>
       <c r="C3461" t="inlineStr">
         <is>
-          <t>PEDRO HENRIQUE VIEIRA DE LIMA</t>
+          <t>MARIA LUANA DE ALMEIDA BATISTA</t>
         </is>
       </c>
       <c r="D3461" t="inlineStr">
         <is>
-          <t>P.LIMA</t>
+          <t>M.LUANA</t>
         </is>
       </c>
     </row>
     <row r="3462">
       <c r="A3462" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B3462" t="n">
-        <v>3331</v>
+        <v>3540</v>
       </c>
       <c r="C3462" t="inlineStr">
         <is>
-          <t>LOUIZE VANIELLE RODRIGUES FARIAS</t>
+          <t>HELEN VITORIA OLIVEIRA DA ROCHA</t>
         </is>
       </c>
       <c r="D3462" t="inlineStr">
         <is>
-          <t>LVFARIAS</t>
+          <t>H.VITORIA</t>
         </is>
       </c>
     </row>
     <row r="3463">
       <c r="A3463" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3463" t="n">
-        <v>3334</v>
+        <v>3559</v>
       </c>
       <c r="C3463" t="inlineStr">
         <is>
-          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
+          <t>ARKBERYS TELES DE SOUSA</t>
         </is>
       </c>
       <c r="D3463" t="inlineStr">
         <is>
-          <t>MTGASPAR</t>
+          <t>ARKBERYS</t>
         </is>
       </c>
     </row>
@@ -69698,176 +69698,176 @@
         </is>
       </c>
       <c r="B3464" t="n">
-        <v>3345</v>
+        <v>3567</v>
       </c>
       <c r="C3464" t="inlineStr">
         <is>
-          <t>AURICÉLIA INACIO PEREIRA</t>
+          <t>PEDRO HENRIQUE VIEIRA DE LIMA</t>
         </is>
       </c>
       <c r="D3464" t="inlineStr">
         <is>
-          <t>AIPEREIRA</t>
+          <t>P.LIMA</t>
         </is>
       </c>
     </row>
     <row r="3465">
       <c r="A3465" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3465" t="n">
-        <v>3363</v>
+        <v>3331</v>
       </c>
       <c r="C3465" t="inlineStr">
         <is>
-          <t>IASMIN LEAL ALVES</t>
+          <t>LOUIZE VANIELLE RODRIGUES FARIAS</t>
         </is>
       </c>
       <c r="D3465" t="inlineStr">
         <is>
-          <t>ILALVES</t>
+          <t>LVFARIAS</t>
         </is>
       </c>
     </row>
     <row r="3466">
       <c r="A3466" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3466" t="n">
-        <v>3370</v>
+        <v>3334</v>
       </c>
       <c r="C3466" t="inlineStr">
         <is>
-          <t>CARLOS DIEGO ARAUJO ALMEIDA</t>
+          <t>MATHEUS TEIXEIRA ALVES GASPAR</t>
         </is>
       </c>
       <c r="D3466" t="inlineStr">
         <is>
-          <t>CDIEGO</t>
+          <t>MTGASPAR</t>
         </is>
       </c>
     </row>
     <row r="3467">
       <c r="A3467" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3467" t="n">
-        <v>3379</v>
+        <v>3345</v>
       </c>
       <c r="C3467" t="inlineStr">
         <is>
-          <t xml:space="preserve">MATHEUS EVANGELISTA FERREIRA </t>
+          <t>AURICÉLIA INACIO PEREIRA</t>
         </is>
       </c>
       <c r="D3467" t="inlineStr">
         <is>
-          <t>MMFERREIRA</t>
+          <t>AIPEREIRA</t>
         </is>
       </c>
     </row>
     <row r="3468">
       <c r="A3468" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3468" t="n">
-        <v>3419</v>
+        <v>3363</v>
       </c>
       <c r="C3468" t="inlineStr">
         <is>
-          <t xml:space="preserve">DAVID EVANGELISTA SILVA </t>
+          <t>IASMIN LEAL ALVES</t>
         </is>
       </c>
       <c r="D3468" t="inlineStr">
         <is>
-          <t>DAVID</t>
+          <t>ILALVES</t>
         </is>
       </c>
     </row>
     <row r="3469">
       <c r="A3469" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3469" t="n">
-        <v>3423</v>
+        <v>3370</v>
       </c>
       <c r="C3469" t="inlineStr">
         <is>
-          <t>MARCIO JOSE TIAGO</t>
+          <t>CARLOS DIEGO ARAUJO ALMEIDA</t>
         </is>
       </c>
       <c r="D3469" t="inlineStr">
         <is>
-          <t>MJTIAGO</t>
+          <t>CDIEGO</t>
         </is>
       </c>
     </row>
     <row r="3470">
       <c r="A3470" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3470" t="n">
-        <v>3453</v>
+        <v>3379</v>
       </c>
       <c r="C3470" t="inlineStr">
         <is>
-          <t xml:space="preserve">LAURIENE SILVA BARBOSA </t>
+          <t xml:space="preserve">MATHEUS EVANGELISTA FERREIRA </t>
         </is>
       </c>
       <c r="D3470" t="inlineStr">
         <is>
-          <t>LAURIENE</t>
+          <t>MMFERREIRA</t>
         </is>
       </c>
     </row>
     <row r="3471">
       <c r="A3471" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3471" t="n">
-        <v>3478</v>
+        <v>3419</v>
       </c>
       <c r="C3471" t="inlineStr">
         <is>
-          <t>LEANDRO BRITO NOGUEIRA DE OLIVEIRA</t>
+          <t xml:space="preserve">DAVID EVANGELISTA SILVA </t>
         </is>
       </c>
       <c r="D3471" t="inlineStr">
         <is>
-          <t>LBNOGUEIRA</t>
+          <t>DAVID</t>
         </is>
       </c>
     </row>
     <row r="3472">
       <c r="A3472" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3472" t="n">
-        <v>3479</v>
+        <v>3423</v>
       </c>
       <c r="C3472" t="inlineStr">
         <is>
-          <t>ESDRAS ALESSANDRO SANTOS SANTANA</t>
+          <t>MARCIO JOSE TIAGO</t>
         </is>
       </c>
       <c r="D3472" t="inlineStr">
         <is>
-          <t>EALESSANDRO</t>
+          <t>MJTIAGO</t>
         </is>
       </c>
     </row>
@@ -69878,456 +69878,456 @@
         </is>
       </c>
       <c r="B3473" t="n">
-        <v>3480</v>
+        <v>3453</v>
       </c>
       <c r="C3473" t="inlineStr">
         <is>
-          <t xml:space="preserve">LUCIMARA SOUSA LIMA </t>
+          <t xml:space="preserve">LAURIENE SILVA BARBOSA </t>
         </is>
       </c>
       <c r="D3473" t="inlineStr">
         <is>
-          <t>LUCIMARA</t>
+          <t>LAURIENE</t>
         </is>
       </c>
     </row>
     <row r="3474">
       <c r="A3474" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3474" t="n">
-        <v>3482</v>
+        <v>3478</v>
       </c>
       <c r="C3474" t="inlineStr">
         <is>
-          <t>DANIEL FERNANDES DINIZ HERACLIO</t>
+          <t>LEANDRO BRITO NOGUEIRA DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D3474" t="inlineStr">
         <is>
-          <t>DFDINIZ</t>
+          <t>LBNOGUEIRA</t>
         </is>
       </c>
     </row>
     <row r="3475">
       <c r="A3475" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3475" t="n">
-        <v>3518</v>
+        <v>3479</v>
       </c>
       <c r="C3475" t="inlineStr">
         <is>
-          <t>RAMYRA ALVES FELIX DA SILVA</t>
+          <t>ESDRAS ALESSANDRO SANTOS SANTANA</t>
         </is>
       </c>
       <c r="D3475" t="inlineStr">
         <is>
-          <t>RFELIX</t>
+          <t>EALESSANDRO</t>
         </is>
       </c>
     </row>
     <row r="3476">
       <c r="A3476" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3476" t="n">
-        <v>3534</v>
+        <v>3480</v>
       </c>
       <c r="C3476" t="inlineStr">
         <is>
-          <t xml:space="preserve">CAIO DE SOUZA VINHAS </t>
+          <t xml:space="preserve">LUCIMARA SOUSA LIMA </t>
         </is>
       </c>
       <c r="D3476" t="inlineStr">
         <is>
-          <t>CVINHAS</t>
+          <t>LUCIMARA</t>
         </is>
       </c>
     </row>
     <row r="3477">
       <c r="A3477" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3477" t="n">
-        <v>3535</v>
+        <v>3482</v>
       </c>
       <c r="C3477" t="inlineStr">
         <is>
-          <t>ROMARIO DE SOUSA SILVA</t>
+          <t>DANIEL FERNANDES DINIZ HERACLIO</t>
         </is>
       </c>
       <c r="D3477" t="inlineStr">
         <is>
-          <t>RSOUSAS</t>
+          <t>DFDINIZ</t>
         </is>
       </c>
     </row>
     <row r="3478">
       <c r="A3478" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3478" t="n">
-        <v>3536</v>
+        <v>3518</v>
       </c>
       <c r="C3478" t="inlineStr">
         <is>
-          <t>JHONATAS CARVALHO OLIVEIRA</t>
+          <t>RAMYRA ALVES FELIX DA SILVA</t>
         </is>
       </c>
       <c r="D3478" t="inlineStr">
         <is>
-          <t>JHONATASC</t>
+          <t>RFELIX</t>
         </is>
       </c>
     </row>
     <row r="3479">
       <c r="A3479" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3479" t="n">
-        <v>940529</v>
+        <v>3534</v>
       </c>
       <c r="C3479" t="inlineStr">
         <is>
-          <t>EDGAR FELIX - FL9</t>
+          <t xml:space="preserve">CAIO DE SOUZA VINHAS </t>
         </is>
       </c>
       <c r="D3479" t="inlineStr">
         <is>
-          <t>EDGAR F</t>
+          <t>CVINHAS</t>
         </is>
       </c>
     </row>
     <row r="3480">
       <c r="A3480" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3480" t="n">
-        <v>3304</v>
+        <v>3535</v>
       </c>
       <c r="C3480" t="inlineStr">
         <is>
-          <t>JOACI GUILHERME GONÇALVES DA LUZ</t>
+          <t>ROMARIO DE SOUSA SILVA</t>
         </is>
       </c>
       <c r="D3480" t="inlineStr">
         <is>
-          <t>JLUZ</t>
+          <t>RSOUSAS</t>
         </is>
       </c>
     </row>
     <row r="3481">
       <c r="A3481" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3481" t="n">
-        <v>3305</v>
+        <v>3536</v>
       </c>
       <c r="C3481" t="inlineStr">
         <is>
-          <t>JOÃO VITOR DE ARAÚJO GONÇALVES</t>
+          <t>JHONATAS CARVALHO OLIVEIRA</t>
         </is>
       </c>
       <c r="D3481" t="inlineStr">
         <is>
-          <t>JJVITOR</t>
+          <t>JHONATASC</t>
         </is>
       </c>
     </row>
     <row r="3482">
       <c r="A3482" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3482" t="n">
-        <v>3306</v>
+        <v>940529</v>
       </c>
       <c r="C3482" t="inlineStr">
         <is>
-          <t>WENDERSON MARCOS DOS SANTOS</t>
+          <t>EDGAR FELIX - FL9</t>
         </is>
       </c>
       <c r="D3482" t="inlineStr">
         <is>
-          <t>WWMARCOS</t>
+          <t>EDGAR F</t>
         </is>
       </c>
     </row>
     <row r="3483">
       <c r="A3483" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3483" t="n">
-        <v>3335</v>
+        <v>3304</v>
       </c>
       <c r="C3483" t="inlineStr">
         <is>
-          <t>EDILBERTO LEMOS DE LIMA</t>
+          <t>JOACI GUILHERME GONÇALVES DA LUZ</t>
         </is>
       </c>
       <c r="D3483" t="inlineStr">
         <is>
-          <t>ELEMOS</t>
+          <t>JLUZ</t>
         </is>
       </c>
     </row>
     <row r="3484">
       <c r="A3484" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3484" t="n">
-        <v>3336</v>
+        <v>3305</v>
       </c>
       <c r="C3484" t="inlineStr">
         <is>
-          <t>EZEQUIEL SOUZA DO NASCIMENTO</t>
+          <t>JOÃO VITOR DE ARAÚJO GONÇALVES</t>
         </is>
       </c>
       <c r="D3484" t="inlineStr">
         <is>
-          <t>ESNASCIMENTO</t>
+          <t>JJVITOR</t>
         </is>
       </c>
     </row>
     <row r="3485">
       <c r="A3485" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3485" t="n">
-        <v>3341</v>
+        <v>3306</v>
       </c>
       <c r="C3485" t="inlineStr">
         <is>
-          <t>ALCIONE MARIANO DE OLIVEIRA</t>
+          <t>WENDERSON MARCOS DOS SANTOS</t>
         </is>
       </c>
       <c r="D3485" t="inlineStr">
         <is>
-          <t>AMOLIVEIRA</t>
+          <t>WWMARCOS</t>
         </is>
       </c>
     </row>
     <row r="3486">
       <c r="A3486" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3486" t="n">
-        <v>3401</v>
+        <v>3335</v>
       </c>
       <c r="C3486" t="inlineStr">
         <is>
-          <t xml:space="preserve">TULIO HENRIQUE DA SILVA CARVALHO </t>
+          <t>EDILBERTO LEMOS DE LIMA</t>
         </is>
       </c>
       <c r="D3486" t="inlineStr">
         <is>
-          <t>TULIO</t>
+          <t>ELEMOS</t>
         </is>
       </c>
     </row>
     <row r="3487">
       <c r="A3487" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3487" t="n">
-        <v>3411</v>
+        <v>3336</v>
       </c>
       <c r="C3487" t="inlineStr">
         <is>
-          <t>CONEXAO RUBYA DANILLA</t>
+          <t>EZEQUIEL SOUZA DO NASCIMENTO</t>
         </is>
       </c>
       <c r="D3487" t="inlineStr">
         <is>
-          <t>CONEXAORUBYA</t>
+          <t>ESNASCIMENTO</t>
         </is>
       </c>
     </row>
     <row r="3488">
       <c r="A3488" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B3488" t="n">
-        <v>3412</v>
+        <v>3341</v>
       </c>
       <c r="C3488" t="inlineStr">
         <is>
-          <t>CONEXAO RAFAEL</t>
+          <t>ALCIONE MARIANO DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D3488" t="inlineStr">
         <is>
-          <t>CONEXAORAFAEL</t>
+          <t>AMOLIVEIRA</t>
         </is>
       </c>
     </row>
     <row r="3489">
       <c r="A3489" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3489" t="n">
-        <v>3558</v>
+        <v>3401</v>
       </c>
       <c r="C3489" t="inlineStr">
         <is>
-          <t>WALLYS QUEIROZ VIANA</t>
+          <t xml:space="preserve">TULIO HENRIQUE DA SILVA CARVALHO </t>
         </is>
       </c>
       <c r="D3489" t="inlineStr">
         <is>
-          <t>WALLYS</t>
+          <t>TULIO</t>
         </is>
       </c>
     </row>
     <row r="3490">
       <c r="A3490" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B3490" t="n">
-        <v>3264</v>
+        <v>3411</v>
       </c>
       <c r="C3490" t="inlineStr">
         <is>
-          <t xml:space="preserve">WILTON CARLOS MACIEL DE ASSIS </t>
+          <t>CONEXAO RUBYA DANILLA</t>
         </is>
       </c>
       <c r="D3490" t="inlineStr">
         <is>
-          <t>WCMACIEL</t>
+          <t>CONEXAORUBYA</t>
         </is>
       </c>
     </row>
     <row r="3491">
       <c r="A3491" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3491" t="n">
-        <v>3340</v>
+        <v>3412</v>
       </c>
       <c r="C3491" t="inlineStr">
         <is>
-          <t>ROGELENO FARIAS FEIJÃO FILHO</t>
+          <t>CONEXAO RAFAEL</t>
         </is>
       </c>
       <c r="D3491" t="inlineStr">
         <is>
-          <t>RFEIJAO</t>
+          <t>CONEXAORAFAEL</t>
         </is>
       </c>
     </row>
     <row r="3492">
       <c r="A3492" t="inlineStr">
         <is>
-          <t>99</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B3492" t="n">
-        <v>940550</v>
+        <v>3558</v>
       </c>
       <c r="C3492" t="inlineStr">
         <is>
-          <t>RAFAELE RIBEIRO CARNEIRO</t>
+          <t>WALLYS QUEIROZ VIANA</t>
         </is>
       </c>
       <c r="D3492" t="inlineStr">
         <is>
-          <t>RAFAELE</t>
+          <t>WALLYS</t>
         </is>
       </c>
     </row>
     <row r="3493">
       <c r="A3493" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3493" t="n">
-        <v>3377</v>
+        <v>3264</v>
       </c>
       <c r="C3493" t="inlineStr">
         <is>
-          <t xml:space="preserve"> ISALTINO BISPO DE OLIVEIRA JUNIOR</t>
+          <t xml:space="preserve">WILTON CARLOS MACIEL DE ASSIS </t>
         </is>
       </c>
       <c r="D3493" t="inlineStr">
         <is>
-          <t>BJUNIOR</t>
+          <t>WCMACIEL</t>
         </is>
       </c>
     </row>
     <row r="3494">
       <c r="A3494" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B3494" t="n">
-        <v>3425</v>
+        <v>3340</v>
       </c>
       <c r="C3494" t="inlineStr">
         <is>
-          <t xml:space="preserve"> CIRLANE ARAUJO SOUZA </t>
+          <t>ROGELENO FARIAS FEIJÃO FILHO</t>
         </is>
       </c>
       <c r="D3494" t="inlineStr">
         <is>
-          <t>CIRLANES</t>
+          <t>RFEIJAO</t>
         </is>
       </c>
     </row>
     <row r="3495">
       <c r="A3495" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>99</t>
         </is>
       </c>
       <c r="B3495" t="n">
-        <v>3454</v>
+        <v>940550</v>
       </c>
       <c r="C3495" t="inlineStr">
         <is>
-          <t>ANTONIA SAMARA DE SOUZA SOARES</t>
+          <t>RAFAELE RIBEIRO CARNEIRO</t>
         </is>
       </c>
       <c r="D3495" t="inlineStr">
         <is>
-          <t>ANTSAMARA</t>
+          <t>RAFAELE</t>
         </is>
       </c>
     </row>
@@ -70338,16 +70338,16 @@
         </is>
       </c>
       <c r="B3496" t="n">
-        <v>3491</v>
+        <v>3377</v>
       </c>
       <c r="C3496" t="inlineStr">
         <is>
-          <t>PEDRO JOSE DO NASCIMENTO NETO</t>
+          <t xml:space="preserve"> ISALTINO BISPO DE OLIVEIRA JUNIOR</t>
         </is>
       </c>
       <c r="D3496" t="inlineStr">
         <is>
-          <t>P.JOSE</t>
+          <t>BJUNIOR</t>
         </is>
       </c>
     </row>
@@ -70358,76 +70358,76 @@
         </is>
       </c>
       <c r="B3497" t="n">
-        <v>3492</v>
+        <v>3425</v>
       </c>
       <c r="C3497" t="inlineStr">
         <is>
-          <t>PAULA CARLA CALDAS MOTA</t>
+          <t xml:space="preserve"> CIRLANE ARAUJO SOUZA </t>
         </is>
       </c>
       <c r="D3497" t="inlineStr">
         <is>
-          <t>P.CARLA</t>
+          <t>CIRLANES</t>
         </is>
       </c>
     </row>
     <row r="3498">
       <c r="A3498" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3498" t="n">
-        <v>3542</v>
+        <v>3454</v>
       </c>
       <c r="C3498" t="inlineStr">
         <is>
-          <t>ANTONIA MILENA SOUSA ANDRADE</t>
+          <t>ANTONIA SAMARA DE SOUZA SOARES</t>
         </is>
       </c>
       <c r="D3498" t="inlineStr">
         <is>
-          <t>A.MILENA</t>
+          <t>ANTSAMARA</t>
         </is>
       </c>
     </row>
     <row r="3499">
       <c r="A3499" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3499" t="n">
-        <v>3547</v>
+        <v>3491</v>
       </c>
       <c r="C3499" t="inlineStr">
         <is>
-          <t xml:space="preserve">DAVI PEREIRA DA SILVA </t>
+          <t>PEDRO JOSE DO NASCIMENTO NETO</t>
         </is>
       </c>
       <c r="D3499" t="inlineStr">
         <is>
-          <t>DPSILVA</t>
+          <t>P.JOSE</t>
         </is>
       </c>
     </row>
     <row r="3500">
       <c r="A3500" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3500" t="n">
-        <v>3552</v>
+        <v>3492</v>
       </c>
       <c r="C3500" t="inlineStr">
         <is>
-          <t>PAULO SERGIO MENDES DE OLIVEIRA</t>
+          <t>PAULA CARLA CALDAS MOTA</t>
         </is>
       </c>
       <c r="D3500" t="inlineStr">
         <is>
-          <t>PSMENDES</t>
+          <t>P.CARLA</t>
         </is>
       </c>
     </row>
@@ -70438,16 +70438,16 @@
         </is>
       </c>
       <c r="B3501" t="n">
-        <v>3294</v>
+        <v>3542</v>
       </c>
       <c r="C3501" t="inlineStr">
         <is>
-          <t>GLEICIANE MIRANDA DE MORAIS</t>
+          <t>ANTONIA MILENA SOUSA ANDRADE</t>
         </is>
       </c>
       <c r="D3501" t="inlineStr">
         <is>
-          <t>GMIRANDA</t>
+          <t>A.MILENA</t>
         </is>
       </c>
     </row>
@@ -70458,16 +70458,16 @@
         </is>
       </c>
       <c r="B3502" t="n">
-        <v>3295</v>
+        <v>3547</v>
       </c>
       <c r="C3502" t="inlineStr">
         <is>
-          <t>MARIA ESTEFANNY DA SILVA MOURA</t>
+          <t xml:space="preserve">DAVI PEREIRA DA SILVA </t>
         </is>
       </c>
       <c r="D3502" t="inlineStr">
         <is>
-          <t>MESTEFANNY</t>
+          <t>DPSILVA</t>
         </is>
       </c>
     </row>
@@ -70478,36 +70478,36 @@
         </is>
       </c>
       <c r="B3503" t="n">
-        <v>3296</v>
+        <v>3552</v>
       </c>
       <c r="C3503" t="inlineStr">
         <is>
-          <t>PEDRO IAGO FONSECA EVANGELISTA</t>
+          <t>PAULO SERGIO MENDES DE OLIVEIRA</t>
         </is>
       </c>
       <c r="D3503" t="inlineStr">
         <is>
-          <t>PIFONSECA</t>
+          <t>PSMENDES</t>
         </is>
       </c>
     </row>
     <row r="3504">
       <c r="A3504" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3504" t="n">
-        <v>940544</v>
+        <v>3294</v>
       </c>
       <c r="C3504" t="inlineStr">
         <is>
-          <t>LUTY LOG TRANSPORTES - FL8</t>
+          <t>GLEICIANE MIRANDA DE MORAIS</t>
         </is>
       </c>
       <c r="D3504" t="inlineStr">
         <is>
-          <t>LUTY LOG</t>
+          <t>GMIRANDA</t>
         </is>
       </c>
     </row>
@@ -70518,96 +70518,96 @@
         </is>
       </c>
       <c r="B3505" t="n">
-        <v>3380</v>
+        <v>3295</v>
       </c>
       <c r="C3505" t="inlineStr">
         <is>
-          <t>FRANCISCO MATHEUS RABELO DA COSTA</t>
+          <t>MARIA ESTEFANNY DA SILVA MOURA</t>
         </is>
       </c>
       <c r="D3505" t="inlineStr">
         <is>
-          <t>FMATHEUS</t>
+          <t>MESTEFANNY</t>
         </is>
       </c>
     </row>
     <row r="3506">
       <c r="A3506" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B3506" t="n">
-        <v>3410</v>
+        <v>3296</v>
       </c>
       <c r="C3506" t="inlineStr">
         <is>
-          <t xml:space="preserve"> BRENO ALLAN DE JESUS</t>
+          <t>PEDRO IAGO FONSECA EVANGELISTA</t>
         </is>
       </c>
       <c r="D3506" t="inlineStr">
         <is>
-          <t>JESUS</t>
+          <t>PIFONSECA</t>
         </is>
       </c>
     </row>
     <row r="3507">
       <c r="A3507" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B3507" t="n">
-        <v>3444</v>
+        <v>940544</v>
       </c>
       <c r="C3507" t="inlineStr">
         <is>
-          <t>THIAGO COSTA SILVA</t>
+          <t>LUTY LOG TRANSPORTES - FL8</t>
         </is>
       </c>
       <c r="D3507" t="inlineStr">
         <is>
-          <t>THIAGOC</t>
+          <t>LUTY LOG</t>
         </is>
       </c>
     </row>
     <row r="3508">
       <c r="A3508" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3508" t="n">
-        <v>3456</v>
+        <v>3380</v>
       </c>
       <c r="C3508" t="inlineStr">
         <is>
-          <t>FELIPE BOTH MAZUCHINI</t>
+          <t>FRANCISCO MATHEUS RABELO DA COSTA</t>
         </is>
       </c>
       <c r="D3508" t="inlineStr">
         <is>
-          <t>FELIPEB</t>
+          <t>FMATHEUS</t>
         </is>
       </c>
     </row>
     <row r="3509">
       <c r="A3509" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B3509" t="n">
-        <v>3457</v>
+        <v>3410</v>
       </c>
       <c r="C3509" t="inlineStr">
         <is>
-          <t>FRANKLIN VIEIRA GOMES</t>
+          <t xml:space="preserve"> BRENO ALLAN DE JESUS</t>
         </is>
       </c>
       <c r="D3509" t="inlineStr">
         <is>
-          <t>VIEIRAF</t>
+          <t>JESUS</t>
         </is>
       </c>
     </row>
@@ -70618,34 +70618,94 @@
         </is>
       </c>
       <c r="B3510" t="n">
-        <v>3507</v>
+        <v>3444</v>
       </c>
       <c r="C3510" t="inlineStr">
         <is>
-          <t>KARINE TEODORA ALVES DE OLIVEIRA</t>
+          <t>THIAGO COSTA SILVA</t>
         </is>
       </c>
       <c r="D3510" t="inlineStr">
         <is>
-          <t>KOLIVEIRA</t>
+          <t>THIAGOC</t>
         </is>
       </c>
     </row>
     <row r="3511">
       <c r="A3511" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B3511" t="n">
+        <v>3456</v>
+      </c>
+      <c r="C3511" t="inlineStr">
+        <is>
+          <t>FELIPE BOTH MAZUCHINI</t>
+        </is>
+      </c>
+      <c r="D3511" t="inlineStr">
+        <is>
+          <t>FELIPEB</t>
+        </is>
+      </c>
+    </row>
+    <row r="3512">
+      <c r="A3512" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="B3512" t="n">
+        <v>3457</v>
+      </c>
+      <c r="C3512" t="inlineStr">
+        <is>
+          <t>FRANKLIN VIEIRA GOMES</t>
+        </is>
+      </c>
+      <c r="D3512" t="inlineStr">
+        <is>
+          <t>VIEIRAF</t>
+        </is>
+      </c>
+    </row>
+    <row r="3513">
+      <c r="A3513" t="inlineStr">
+        <is>
           <t>5</t>
         </is>
       </c>
-      <c r="B3511" t="n">
+      <c r="B3513" t="n">
+        <v>3507</v>
+      </c>
+      <c r="C3513" t="inlineStr">
+        <is>
+          <t>KARINE TEODORA ALVES DE OLIVEIRA</t>
+        </is>
+      </c>
+      <c r="D3513" t="inlineStr">
+        <is>
+          <t>KOLIVEIRA</t>
+        </is>
+      </c>
+    </row>
+    <row r="3514">
+      <c r="A3514" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B3514" t="n">
         <v>3520</v>
       </c>
-      <c r="C3511" t="inlineStr">
+      <c r="C3514" t="inlineStr">
         <is>
           <t xml:space="preserve"> EMERSON FILIPE MELO DE AGUIAR</t>
         </is>
       </c>
-      <c r="D3511" t="inlineStr">
+      <c r="D3514" t="inlineStr">
         <is>
           <t>E.FILIPE</t>
         </is>

</xml_diff>